<commit_message>
Accuracy pass: fix dates, citations, initiative maths and budget scenarios
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V2NJtrYy3bzNxqKeiRXJfY
</commit_message>
<xml_diff>
--- a/operation_uptime/Operation_Uptime_Model.xlsx
+++ b/operation_uptime/Operation_Uptime_Model.xlsx
@@ -268,7 +268,7 @@
     <t xml:space="preserve">Days: interview → written offer</t>
   </si>
   <si>
-    <t xml:space="preserve">Tesla is known for fast decisions; assumes offer approval within 3 days (client to confirm).</t>
+    <t xml:space="preserve">Assumes offer approval within 3 working days of the interview (client to confirm; it is one of the asks).</t>
   </si>
   <si>
     <t xml:space="preserve">T5</t>
@@ -370,13 +370,13 @@
     <t xml:space="preserve">Offer → signed contract</t>
   </si>
   <si>
-    <t xml:space="preserve">Engpassberuf with counter-offers from energy/grid, rail, aerospace; Tesla shift work and IG Metall disputes are known. Tesla pays above Brandenburg trade median (€3,030/month, WSI https://www.lohnspiegel.de/gehaltsinfos/elektroniker_in_fuer_betriebstechnik_26252114.html) which helps.</t>
+    <t xml:space="preserve">Engpassberuf with counter-offers from energy/grid, rail, aerospace; Tesla shift work and IG Metall disputes are known. Acceptance improves if Tesla's offer beats the Brandenburg trade median (€3,030/month at 10 yrs, WSI https://www.lohnspiegel.de/gehaltsinfos/elektroniker_in_fuer_betriebstechnik_26252114.html); client to confirm pay band.</t>
   </si>
   <si>
     <t xml:space="preserve">AM</t>
   </si>
   <si>
-    <t xml:space="preserve">Bigger pool, fewer counter-offers; pay premium vs Brandenburg/Polish wages is strong for border commuters.</t>
+    <t xml:space="preserve">Bigger pool, fewer counter-offers; German pay vs Polish wages is a strong pull for border commuters.</t>
   </si>
   <si>
     <t xml:space="preserve">AA</t>
@@ -400,7 +400,7 @@
     <t xml:space="preserve">Reserve held back (share of total budget)</t>
   </si>
   <si>
-    <t xml:space="preserve">Covers ±30% error on the conversion that matters most (Part 1.4) for the cheapest channels; released from week 3 only on the rules in Part 4.</t>
+    <t xml:space="preserve">Buffer for estimate error: at €50k (incl. rounding) funds about half of the extra media a 30% miss on share qualified would need (Funnel F45 – F42). Beyond that the binding limit is assessment slots, not money. Released from week 3 only on the Tracker rules.</t>
   </si>
   <si>
     <t xml:space="preserve">B2</t>
@@ -535,7 +535,7 @@
     <t xml:space="preserve">people</t>
   </si>
   <si>
-    <t xml:space="preserve">≈7% of German employment is in Berlin+Brandenburg (BA statistics); assumed ~150–200k industrial electricians in DE, lower industrial density in the East → ~7,000 within 75 km of Grünheide. Order of magnitude only.</t>
+    <t xml:space="preserve">Berlin+Brandenburg hold roughly 7% of German employment (approx. 2.6M of ~35M employees subject to social insurance, from memory of BA figures); assumed ~150–200k industrial electricians in DE, lower industrial density in the East → ~7,000 within 75 km of Grünheide. Order of magnitude only.</t>
   </si>
   <si>
     <t xml:space="preserve">PSM</t>
@@ -955,7 +955,7 @@
     <t xml:space="preserve">I2: construction/Handwerk electricians (Elektroniker Energie- und Gebäudetechnik) within 75 km</t>
   </si>
   <si>
-    <t xml:space="preserve">Bauelektrik is a larger occupation than industrial electrics and is itself an Engpassberuf (BA Engpassanalyse https://statistik.arbeitsagentur.de/DE/Navigation/Statistiken/Interaktive-Statistiken/Fachkraeftebedarf/Engpassanalyse-Nav.html); Berlin construction boom → large local pool.</t>
+    <t xml:space="preserve">Bauelektrik is a larger occupation than industrial electrics and is itself an Engpassberuf (BA Engpassanalyse 2024: KldB 2621 Bauelektrik scores 2.7, threshold 2.0 – https://www.vbw-bayern.de/Redaktion/Frei-zugaengliche-Medien/Abteilungen-GS/Bildung/2025/Downloads/2024_BA-FK-Engpassanalyse.pdf); Berlin construction boom → large local pool.</t>
   </si>
   <si>
     <t xml:space="preserve">I2S</t>
@@ -1009,7 +1009,7 @@
     <t xml:space="preserve">I3: blended cost per application, Pracuj.pl + OLX Praca + Polish-geo Meta</t>
   </si>
   <si>
-    <t xml:space="preserve">Pracuj.pl 30-day ad 1,499 PLN ≈ €350 (https://dlafirm.pracuj.pl/cennik-uslug/pakiety-ogloszen) ÷ ~25 apps ≈ €14; PL Meta leads ~€8–10.</t>
+    <t xml:space="preserve">Pracuj.pl 30-day ad indicatively 1,499 PLN ≈ €350 (package page https://dlafirm.pracuj.pl/cennik-uslug/pakiety-ogloszen; exact price is quoted per role/location in their calculator) ÷ ~25 apps ≈ €14; PL Meta leads ~€8–10 (own estimate).</t>
   </si>
   <si>
     <t xml:space="preserve">I3Q</t>
@@ -1471,7 +1471,7 @@
     <t xml:space="preserve">≥15 qualified re-applicants + referrals across roles by day 14, ≥5 of them electricians</t>
   </si>
   <si>
-    <t xml:space="preserve">&lt;5 qualified by day 14 → stop re-contact waves (cost is tiny, so mostly a signal that the ATS data is stale); referral bonus stays live because it only costs on a hire</t>
+    <t xml:space="preserve">&lt;5 qualified by day 14 → stop re-contact waves (cost is tiny, so mostly a signal that the ATS data is stale); referral bonus stays live because it is paid only on a signed hire (from week 4)</t>
   </si>
   <si>
     <t xml:space="preserve">I2 Handwerk → Industrie</t>
@@ -2670,7 +2670,7 @@
       </c>
       <c r="C18" s="5" t="n">
         <f aca="false">Budget!H47</f>
-        <v>87.4362783297683</v>
+        <v>88.0409219542276</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6101,7 +6101,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
         <v>111</v>
       </c>
@@ -6124,7 +6124,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="2" t="s">
         <v>114</v>
       </c>
@@ -6227,7 +6227,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="2" t="s">
         <v>121</v>
       </c>
@@ -8258,7 +8258,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="129" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="129" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="2" t="s">
         <v>306</v>
       </c>
@@ -8396,7 +8396,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="135" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="135" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="2" t="s">
         <v>324</v>
       </c>
@@ -10558,8 +10558,8 @@
         <v>478</v>
       </c>
       <c r="B53" s="35" t="n">
-        <f aca="false">F10+F16*(Assumptions!$D$51+Assumptions!$D$52)</f>
-        <v>4402.45581875</v>
+        <f aca="false">F10</f>
+        <v>350</v>
       </c>
       <c r="C53" s="9" t="s">
         <v>479</v>
@@ -15088,7 +15088,7 @@
       </c>
       <c r="C45" s="35" t="n">
         <f aca="false">Scenarios!F4</f>
-        <v>49169.764891993</v>
+        <v>50000</v>
       </c>
       <c r="D45" s="26" t="n">
         <f aca="false">Scenarios!F39</f>
@@ -15112,7 +15112,7 @@
       </c>
       <c r="I45" s="35" t="n">
         <f aca="false">C45/H45</f>
-        <v>491.69764891993</v>
+        <v>500</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15122,11 +15122,11 @@
       </c>
       <c r="C46" s="35" t="n">
         <f aca="false">Scenarios!G4</f>
-        <v>41794.3001581941</v>
+        <v>42500</v>
       </c>
       <c r="D46" s="26" t="n">
         <f aca="false">Scenarios!G39</f>
-        <v>25.4545656012709</v>
+        <v>26.0544104668059</v>
       </c>
       <c r="E46" s="26" t="n">
         <f aca="false">Scenarios!G40</f>
@@ -15142,11 +15142,11 @@
       </c>
       <c r="H46" s="29" t="n">
         <f aca="false">SUM(D46:G46)</f>
-        <v>94.5366456012709</v>
+        <v>95.1364904668059</v>
       </c>
       <c r="I46" s="35" t="n">
         <f aca="false">C46/H46</f>
-        <v>442.096288612468</v>
+        <v>446.726590306888</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15156,7 +15156,7 @@
       </c>
       <c r="C47" s="35" t="n">
         <f aca="false">Scenarios!H4</f>
-        <v>34418.8354243951</v>
+        <v>35000</v>
       </c>
       <c r="D47" s="26" t="n">
         <f aca="false">Scenarios!H39</f>
@@ -15172,15 +15172,15 @@
       </c>
       <c r="G47" s="26" t="n">
         <f aca="false">Scenarios!H42</f>
-        <v>3.69112832976827</v>
+        <v>4.2957719542276</v>
       </c>
       <c r="H47" s="29" t="n">
         <f aca="false">SUM(D47:G47)</f>
-        <v>87.4362783297683</v>
+        <v>88.0409219542276</v>
       </c>
       <c r="I47" s="35" t="n">
         <f aca="false">C47/H47</f>
-        <v>393.644790033075</v>
+        <v>397.54240667989</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15190,11 +15190,11 @@
       </c>
       <c r="C48" s="35" t="n">
         <f aca="false">Scenarios!I4</f>
-        <v>24584.8824459965</v>
+        <v>25000</v>
       </c>
       <c r="D48" s="26" t="n">
         <f aca="false">Scenarios!I39</f>
-        <v>13.9630075154343</v>
+        <v>14.4171253636364</v>
       </c>
       <c r="E48" s="26" t="n">
         <f aca="false">Scenarios!I40</f>
@@ -15210,11 +15210,11 @@
       </c>
       <c r="H48" s="29" t="n">
         <f aca="false">SUM(D48:G48)</f>
-        <v>76.7261875154343</v>
+        <v>77.1803053636364</v>
       </c>
       <c r="I48" s="35" t="n">
         <f aca="false">C48/H48</f>
-        <v>320.423616005305</v>
+        <v>323.916831919906</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15299,20 +15299,20 @@
         <v>550</v>
       </c>
       <c r="F4" s="35" t="n">
-        <f aca="false">Budget!$C$11*F3</f>
-        <v>49169.764891993</v>
+        <f aca="false">Budget!$C$12*F3</f>
+        <v>50000</v>
       </c>
       <c r="G4" s="35" t="n">
-        <f aca="false">Budget!$C$11*G3</f>
-        <v>41794.3001581941</v>
+        <f aca="false">Budget!$C$12*G3</f>
+        <v>42500</v>
       </c>
       <c r="H4" s="35" t="n">
-        <f aca="false">Budget!$C$11*H3</f>
-        <v>34418.8354243951</v>
+        <f aca="false">Budget!$C$12*H3</f>
+        <v>35000</v>
       </c>
       <c r="I4" s="35" t="n">
-        <f aca="false">Budget!$C$11*I3</f>
-        <v>24584.8824459965</v>
+        <f aca="false">Budget!$C$12*I3</f>
+        <v>25000</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15321,19 +15321,19 @@
       </c>
       <c r="F5" s="35" t="n">
         <f aca="false">F4*(1-Assumptions!$D$48)-Budget!$C$6-Budget!$C$8</f>
-        <v>34486.5858724798</v>
+        <v>35192.2857142857</v>
       </c>
       <c r="G5" s="35" t="n">
         <f aca="false">G4*(1-Assumptions!$D$48)-Budget!$C$6-Budget!$C$8</f>
-        <v>28217.4408487507</v>
+        <v>28817.2857142857</v>
       </c>
       <c r="H5" s="35" t="n">
         <f aca="false">H4*(1-Assumptions!$D$48)-Budget!$C$6-Budget!$C$8</f>
-        <v>21948.2958250216</v>
+        <v>22442.2857142857</v>
       </c>
       <c r="I5" s="35" t="n">
         <f aca="false">I4*(1-Assumptions!$D$48)-Budget!$C$6-Budget!$C$8</f>
-        <v>13589.4357933827</v>
+        <v>13942.2857142857</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15346,15 +15346,15 @@
       </c>
       <c r="G6" s="35" t="n">
         <f aca="false">MAX(0,(Budget!$C$4+Budget!$C$5)-G5)</f>
-        <v>6269.14502372912</v>
+        <v>5669.30015819407</v>
       </c>
       <c r="H6" s="35" t="n">
         <f aca="false">MAX(0,(Budget!$C$4+Budget!$C$5)-H5)</f>
-        <v>12538.2900474582</v>
+        <v>12044.3001581941</v>
       </c>
       <c r="I6" s="35" t="n">
         <f aca="false">MAX(0,(Budget!$C$4+Budget!$C$5)-I5)</f>
-        <v>20897.150079097</v>
+        <v>20544.3001581941</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16131,7 +16131,7 @@
       </c>
       <c r="H21" s="26" t="n">
         <f aca="false">IF(C21&gt;0,E21*(1-L21/C21),E21)</f>
-        <v>0.927948329768269</v>
+        <v>1.5325919542276</v>
       </c>
       <c r="I21" s="26" t="n">
         <f aca="false">IF(C21&gt;0,E21*(1-M21/C21),E21)</f>
@@ -16147,7 +16147,7 @@
       </c>
       <c r="L21" s="35" t="n">
         <f aca="false">MIN(C21,MAX(0,H$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D21)))</f>
-        <v>3616.87227960109</v>
+        <v>3122.88239033693</v>
       </c>
       <c r="M21" s="35" t="n">
         <f aca="false">MIN(C21,MAX(0,I$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D21)))</f>
@@ -16721,7 +16721,7 @@
       </c>
       <c r="G32" s="26" t="n">
         <f aca="false">IF(C32&gt;0,E32*(1-K32/C32),E32)</f>
-        <v>1.70941560127088</v>
+        <v>2.30926046680593</v>
       </c>
       <c r="H32" s="26" t="n">
         <f aca="false">IF(C32&gt;0,E32*(1-L32/C32),E32)</f>
@@ -16737,7 +16737,7 @@
       </c>
       <c r="K32" s="35" t="n">
         <f aca="false">MIN(C32,MAX(0,G$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D32)))</f>
-        <v>2453.22502372912</v>
+        <v>1853.38015819407</v>
       </c>
       <c r="L32" s="35" t="n">
         <f aca="false">MIN(C32,MAX(0,H$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D32)))</f>
@@ -16945,7 +16945,7 @@
       </c>
       <c r="I36" s="26" t="n">
         <f aca="false">IF(C36&gt;0,E36*(1-M36/C36),E36)</f>
-        <v>1.80085751543425</v>
+        <v>2.25497536363637</v>
       </c>
       <c r="J36" s="35" t="n">
         <f aca="false">MIN(C36,MAX(0,F$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D36)))</f>
@@ -16961,7 +16961,7 @@
       </c>
       <c r="M36" s="35" t="n">
         <f aca="false">MIN(C36,MAX(0,I$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D36)))</f>
-        <v>7600.7323112399</v>
+        <v>7247.88239033693</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17033,7 +17033,7 @@
       </c>
       <c r="G39" s="26" t="n">
         <f aca="false">SUMIFS(G$8:G$37,$B$8:$B$37,$E39)</f>
-        <v>25.4545656012709</v>
+        <v>26.0544104668059</v>
       </c>
       <c r="H39" s="26" t="n">
         <f aca="false">SUMIFS(H$8:H$37,$B$8:$B$37,$E39)</f>
@@ -17041,7 +17041,7 @@
       </c>
       <c r="I39" s="26" t="n">
         <f aca="false">SUMIFS(I$8:I$37,$B$8:$B$37,$E39)</f>
-        <v>13.9630075154343</v>
+        <v>14.4171253636364</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17100,7 +17100,7 @@
       </c>
       <c r="H42" s="26" t="n">
         <f aca="false">SUMIFS(H$8:H$37,$B$8:$B$37,$E42)</f>
-        <v>3.69112832976827</v>
+        <v>4.2957719542276</v>
       </c>
       <c r="I42" s="26" t="n">
         <f aca="false">SUMIFS(I$8:I$37,$B$8:$B$37,$E42)</f>
@@ -17117,15 +17117,15 @@
       </c>
       <c r="G43" s="29" t="n">
         <f aca="false">SUM(G39:G42)</f>
-        <v>94.5366456012709</v>
+        <v>95.1364904668059</v>
       </c>
       <c r="H43" s="29" t="n">
         <f aca="false">SUM(H39:H42)</f>
-        <v>87.4362783297683</v>
+        <v>88.0409219542276</v>
       </c>
       <c r="I43" s="29" t="n">
         <f aca="false">SUM(I39:I42)</f>
-        <v>76.7261875154343</v>
+        <v>77.1803053636364</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17134,19 +17134,19 @@
       </c>
       <c r="F44" s="35" t="n">
         <f aca="false">F4/F43</f>
-        <v>491.69764891993</v>
+        <v>500</v>
       </c>
       <c r="G44" s="35" t="n">
         <f aca="false">G4/G43</f>
-        <v>442.096288612468</v>
+        <v>446.726590306888</v>
       </c>
       <c r="H44" s="35" t="n">
         <f aca="false">H4/H43</f>
-        <v>393.644790033075</v>
+        <v>397.54240667989</v>
       </c>
       <c r="I44" s="35" t="n">
         <f aca="false">I4/I43</f>
-        <v>320.423616005305</v>
+        <v>323.916831919906</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add model test suite (93 scenarios, oracle, edge cases, deck check) and fix bugs it found
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V2NJtrYy3bzNxqKeiRXJfY
</commit_message>
<xml_diff>
--- a/operation_uptime/Operation_Uptime_Model.xlsx
+++ b/operation_uptime/Operation_Uptime_Model.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1387" uniqueCount="751">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1389" uniqueCount="753">
   <si>
     <t xml:space="preserve">Operation Uptime — model summary (hypothetical Tesla Giga Berlin maintenance hiring)</t>
   </si>
@@ -877,7 +877,7 @@
     <t xml:space="preserve">qualified/wk</t>
   </si>
   <si>
-    <t xml:space="preserve">~80% of the 55 weekly slots; below this, slots would go unused.</t>
+    <t xml:space="preserve">~80% of the 55 weekly slots; below this, slots would go unused. Flagged automatically per week on the Weekly tab (col S).</t>
   </si>
   <si>
     <t xml:space="preserve">R8</t>
@@ -1705,7 +1705,7 @@
     <t xml:space="preserve">I2 Handwerk → Industrie</t>
   </si>
   <si>
-    <t xml:space="preserve">Fri 23 Oct – Fri 6 Nov (read Mon 9 Nov)</t>
+    <t xml:space="preserve">Fri 23 Oct – Thu 5 Nov (read Mon 9 Nov)</t>
   </si>
   <si>
     <t xml:space="preserve">Also kill at once if the client rejects the EGT profile. Week-4 quality check: ≥50% of the first 6 interviewed pass (kill below 40%). Money then moves to Meta, StepStone and programmatic electricians.</t>
@@ -2168,6 +2168,12 @@
   </si>
   <si>
     <t xml:space="preserve">Wk 9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wk 10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wk 11</t>
   </si>
   <si>
     <t xml:space="preserve">Weekly tracker — type actuals in the yellow cells; decisions and re-forecast update live</t>
@@ -3084,12 +3090,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>713</v>
+        <v>715</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>714</v>
+        <v>716</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3103,67 +3109,67 @@
         <v>288</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>715</v>
+        <v>717</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>716</v>
+        <v>718</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>717</v>
+        <v>719</v>
       </c>
       <c r="G4" s="12" t="s">
-        <v>718</v>
+        <v>720</v>
       </c>
       <c r="H4" s="12" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
       <c r="I4" s="12" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
       <c r="J4" s="12" t="s">
-        <v>721</v>
+        <v>723</v>
       </c>
       <c r="K4" s="12" t="s">
-        <v>722</v>
+        <v>724</v>
       </c>
       <c r="L4" s="12" t="s">
-        <v>723</v>
+        <v>725</v>
       </c>
       <c r="M4" s="12" t="s">
-        <v>724</v>
+        <v>726</v>
       </c>
       <c r="N4" s="12" t="s">
-        <v>725</v>
+        <v>727</v>
       </c>
       <c r="O4" s="12" t="s">
-        <v>726</v>
+        <v>728</v>
       </c>
       <c r="P4" s="12" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
       <c r="Q4" s="12" t="s">
-        <v>728</v>
+        <v>730</v>
       </c>
       <c r="R4" s="12" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
       <c r="S4" s="12" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="T4" s="12" t="s">
-        <v>731</v>
+        <v>733</v>
       </c>
       <c r="U4" s="12" t="s">
-        <v>732</v>
+        <v>734</v>
       </c>
       <c r="V4" s="12" t="s">
-        <v>733</v>
+        <v>735</v>
       </c>
       <c r="W4" s="12" t="s">
-        <v>734</v>
+        <v>736</v>
       </c>
       <c r="X4" s="12" t="s">
-        <v>735</v>
+        <v>737</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3225,7 +3231,7 @@
         <v>0.08</v>
       </c>
       <c r="V5" s="35" t="n">
-        <f aca="false">IF(Q5&gt;=Assumptions!$D$86,S5,D5)/U5</f>
+        <f aca="false">IF(U5&gt;0,IF(Q5&gt;=Assumptions!$D$86,S5,D5)/U5,0)</f>
         <v>0</v>
       </c>
       <c r="W5" s="45" t="str">
@@ -3296,7 +3302,7 @@
         <v>0.18</v>
       </c>
       <c r="V6" s="35" t="n">
-        <f aca="false">IF(Q6&gt;=Assumptions!$D$86,S6,D6)/U6</f>
+        <f aca="false">IF(U6&gt;0,IF(Q6&gt;=Assumptions!$D$86,S6,D6)/U6,0)</f>
         <v>0</v>
       </c>
       <c r="W6" s="45" t="str">
@@ -3367,7 +3373,7 @@
         <v>0.1</v>
       </c>
       <c r="V7" s="35" t="n">
-        <f aca="false">IF(Q7&gt;=Assumptions!$D$86,S7,D7)/U7</f>
+        <f aca="false">IF(U7&gt;0,IF(Q7&gt;=Assumptions!$D$86,S7,D7)/U7,0)</f>
         <v>0</v>
       </c>
       <c r="W7" s="45" t="str">
@@ -3438,7 +3444,7 @@
         <v>0.08</v>
       </c>
       <c r="V8" s="35" t="n">
-        <f aca="false">IF(Q8&gt;=Assumptions!$D$86,S8,D8)/U8</f>
+        <f aca="false">IF(U8&gt;0,IF(Q8&gt;=Assumptions!$D$86,S8,D8)/U8,0)</f>
         <v>0</v>
       </c>
       <c r="W8" s="45" t="str">
@@ -3509,7 +3515,7 @@
         <v>0.12</v>
       </c>
       <c r="V9" s="35" t="n">
-        <f aca="false">IF(Q9&gt;=Assumptions!$D$86,S9,D9)/U9</f>
+        <f aca="false">IF(U9&gt;0,IF(Q9&gt;=Assumptions!$D$86,S9,D9)/U9,0)</f>
         <v>476.190476190476</v>
       </c>
       <c r="W9" s="45" t="n">
@@ -3580,7 +3586,7 @@
         <v>0.22</v>
       </c>
       <c r="V10" s="35" t="n">
-        <f aca="false">IF(Q10&gt;=Assumptions!$D$86,S10,D10)/U10</f>
+        <f aca="false">IF(U10&gt;0,IF(Q10&gt;=Assumptions!$D$86,S10,D10)/U10,0)</f>
         <v>109.090909090909</v>
       </c>
       <c r="W10" s="45" t="n">
@@ -3651,7 +3657,7 @@
         <v>0.12</v>
       </c>
       <c r="V11" s="35" t="n">
-        <f aca="false">IF(Q11&gt;=Assumptions!$D$86,S11,D11)/U11</f>
+        <f aca="false">IF(U11&gt;0,IF(Q11&gt;=Assumptions!$D$86,S11,D11)/U11,0)</f>
         <v>375</v>
       </c>
       <c r="W11" s="45" t="n">
@@ -3722,7 +3728,7 @@
         <v>0.1</v>
       </c>
       <c r="V12" s="35" t="n">
-        <f aca="false">IF(Q12&gt;=Assumptions!$D$86,S12,D12)/U12</f>
+        <f aca="false">IF(U12&gt;0,IF(Q12&gt;=Assumptions!$D$86,S12,D12)/U12,0)</f>
         <v>425</v>
       </c>
       <c r="W12" s="45" t="n">
@@ -3793,7 +3799,7 @@
         <v>0.3</v>
       </c>
       <c r="V13" s="35" t="n">
-        <f aca="false">IF(Q13&gt;=Assumptions!$D$86,S13,D13)/U13</f>
+        <f aca="false">IF(U13&gt;0,IF(Q13&gt;=Assumptions!$D$86,S13,D13)/U13,0)</f>
         <v>322</v>
       </c>
       <c r="W13" s="45" t="n">
@@ -3864,7 +3870,7 @@
         <v>0.35</v>
       </c>
       <c r="V14" s="35" t="n">
-        <f aca="false">IF(Q14&gt;=Assumptions!$D$86,S14,D14)/U14</f>
+        <f aca="false">IF(U14&gt;0,IF(Q14&gt;=Assumptions!$D$86,S14,D14)/U14,0)</f>
         <v>165.6</v>
       </c>
       <c r="W14" s="45" t="n">
@@ -3935,7 +3941,7 @@
         <v>0.25</v>
       </c>
       <c r="V15" s="35" t="n">
-        <f aca="false">IF(Q15&gt;=Assumptions!$D$86,S15,D15)/U15</f>
+        <f aca="false">IF(U15&gt;0,IF(Q15&gt;=Assumptions!$D$86,S15,D15)/U15,0)</f>
         <v>386.4</v>
       </c>
       <c r="W15" s="45" t="n">
@@ -4006,7 +4012,7 @@
         <v>0.25</v>
       </c>
       <c r="V16" s="35" t="n">
-        <f aca="false">IF(Q16&gt;=Assumptions!$D$86,S16,D16)/U16</f>
+        <f aca="false">IF(U16&gt;0,IF(Q16&gt;=Assumptions!$D$86,S16,D16)/U16,0)</f>
         <v>386.4</v>
       </c>
       <c r="W16" s="45" t="n">
@@ -4077,7 +4083,7 @@
         <v>0.25</v>
       </c>
       <c r="V17" s="35" t="n">
-        <f aca="false">IF(Q17&gt;=Assumptions!$D$86,S17,D17)/U17</f>
+        <f aca="false">IF(U17&gt;0,IF(Q17&gt;=Assumptions!$D$86,S17,D17)/U17,0)</f>
         <v>175</v>
       </c>
       <c r="W17" s="45" t="n">
@@ -4148,7 +4154,7 @@
         <v>0.2</v>
       </c>
       <c r="V18" s="35" t="n">
-        <f aca="false">IF(Q18&gt;=Assumptions!$D$86,S18,D18)/U18</f>
+        <f aca="false">IF(U18&gt;0,IF(Q18&gt;=Assumptions!$D$86,S18,D18)/U18,0)</f>
         <v>218.75</v>
       </c>
       <c r="W18" s="45" t="n">
@@ -4219,7 +4225,7 @@
         <v>0.05</v>
       </c>
       <c r="V19" s="35" t="n">
-        <f aca="false">IF(Q19&gt;=Assumptions!$D$86,S19,D19)/U19</f>
+        <f aca="false">IF(U19&gt;0,IF(Q19&gt;=Assumptions!$D$86,S19,D19)/U19,0)</f>
         <v>360</v>
       </c>
       <c r="W19" s="45" t="n">
@@ -4290,7 +4296,7 @@
         <v>0.12</v>
       </c>
       <c r="V20" s="35" t="n">
-        <f aca="false">IF(Q20&gt;=Assumptions!$D$86,S20,D20)/U20</f>
+        <f aca="false">IF(U20&gt;0,IF(Q20&gt;=Assumptions!$D$86,S20,D20)/U20,0)</f>
         <v>100</v>
       </c>
       <c r="W20" s="45" t="n">
@@ -4361,7 +4367,7 @@
         <v>0.15</v>
       </c>
       <c r="V21" s="35" t="n">
-        <f aca="false">IF(Q21&gt;=Assumptions!$D$86,S21,D21)/U21</f>
+        <f aca="false">IF(U21&gt;0,IF(Q21&gt;=Assumptions!$D$86,S21,D21)/U21,0)</f>
         <v>209.52380952381</v>
       </c>
       <c r="W21" s="45" t="n">
@@ -4432,7 +4438,7 @@
         <v>0.25</v>
       </c>
       <c r="V22" s="35" t="n">
-        <f aca="false">IF(Q22&gt;=Assumptions!$D$86,S22,D22)/U22</f>
+        <f aca="false">IF(U22&gt;0,IF(Q22&gt;=Assumptions!$D$86,S22,D22)/U22,0)</f>
         <v>125.714285714286</v>
       </c>
       <c r="W22" s="45" t="n">
@@ -4503,7 +4509,7 @@
         <v>0.15</v>
       </c>
       <c r="V23" s="35" t="n">
-        <f aca="false">IF(Q23&gt;=Assumptions!$D$86,S23,D23)/U23</f>
+        <f aca="false">IF(U23&gt;0,IF(Q23&gt;=Assumptions!$D$86,S23,D23)/U23,0)</f>
         <v>209.52380952381</v>
       </c>
       <c r="W23" s="45" t="n">
@@ -4574,7 +4580,7 @@
         <v>0.12</v>
       </c>
       <c r="V24" s="35" t="n">
-        <f aca="false">IF(Q24&gt;=Assumptions!$D$86,S24,D24)/U24</f>
+        <f aca="false">IF(U24&gt;0,IF(Q24&gt;=Assumptions!$D$86,S24,D24)/U24,0)</f>
         <v>261.904761904762</v>
       </c>
       <c r="W24" s="45" t="n">
@@ -4645,7 +4651,7 @@
         <v>0.5</v>
       </c>
       <c r="V25" s="35" t="n">
-        <f aca="false">IF(Q25&gt;=Assumptions!$D$86,S25,D25)/U25</f>
+        <f aca="false">IF(U25&gt;0,IF(Q25&gt;=Assumptions!$D$86,S25,D25)/U25,0)</f>
         <v>8.33333333333333</v>
       </c>
       <c r="W25" s="45" t="n">
@@ -4716,7 +4722,7 @@
         <v>0.5</v>
       </c>
       <c r="V26" s="35" t="n">
-        <f aca="false">IF(Q26&gt;=Assumptions!$D$86,S26,D26)/U26</f>
+        <f aca="false">IF(U26&gt;0,IF(Q26&gt;=Assumptions!$D$86,S26,D26)/U26,0)</f>
         <v>8.33333333333333</v>
       </c>
       <c r="W26" s="45" t="n">
@@ -4787,7 +4793,7 @@
         <v>0.5</v>
       </c>
       <c r="V27" s="35" t="n">
-        <f aca="false">IF(Q27&gt;=Assumptions!$D$86,S27,D27)/U27</f>
+        <f aca="false">IF(U27&gt;0,IF(Q27&gt;=Assumptions!$D$86,S27,D27)/U27,0)</f>
         <v>8.33333333333333</v>
       </c>
       <c r="W27" s="45" t="n">
@@ -4858,7 +4864,7 @@
         <v>0.5</v>
       </c>
       <c r="V28" s="35" t="n">
-        <f aca="false">IF(Q28&gt;=Assumptions!$D$86,S28,D28)/U28</f>
+        <f aca="false">IF(U28&gt;0,IF(Q28&gt;=Assumptions!$D$86,S28,D28)/U28,0)</f>
         <v>8.33333333333333</v>
       </c>
       <c r="W28" s="45" t="n">
@@ -4929,7 +4935,7 @@
         <v>0.45</v>
       </c>
       <c r="V29" s="35" t="n">
-        <f aca="false">IF(Q29&gt;=Assumptions!$D$86,S29,D29)/U29</f>
+        <f aca="false">IF(U29&gt;0,IF(Q29&gt;=Assumptions!$D$86,S29,D29)/U29,0)</f>
         <v>370.0125</v>
       </c>
       <c r="W29" s="45" t="n">
@@ -5000,7 +5006,7 @@
         <v>0.45</v>
       </c>
       <c r="V30" s="35" t="n">
-        <f aca="false">IF(Q30&gt;=Assumptions!$D$86,S30,D30)/U30</f>
+        <f aca="false">IF(U30&gt;0,IF(Q30&gt;=Assumptions!$D$86,S30,D30)/U30,0)</f>
         <v>465.75</v>
       </c>
       <c r="W30" s="45" t="n">
@@ -5071,7 +5077,7 @@
         <v>0.45</v>
       </c>
       <c r="V31" s="35" t="n">
-        <f aca="false">IF(Q31&gt;=Assumptions!$D$86,S31,D31)/U31</f>
+        <f aca="false">IF(U31&gt;0,IF(Q31&gt;=Assumptions!$D$86,S31,D31)/U31,0)</f>
         <v>336.375</v>
       </c>
       <c r="W31" s="45" t="n">
@@ -5142,7 +5148,7 @@
         <v>0.45</v>
       </c>
       <c r="V32" s="35" t="n">
-        <f aca="false">IF(Q32&gt;=Assumptions!$D$86,S32,D32)/U32</f>
+        <f aca="false">IF(U32&gt;0,IF(Q32&gt;=Assumptions!$D$86,S32,D32)/U32,0)</f>
         <v>307.9125</v>
       </c>
       <c r="W32" s="45" t="n">
@@ -5213,7 +5219,7 @@
         <v>0.15</v>
       </c>
       <c r="V33" s="35" t="n">
-        <f aca="false">IF(Q33&gt;=Assumptions!$D$86,S33,D33)/U33</f>
+        <f aca="false">IF(U33&gt;0,IF(Q33&gt;=Assumptions!$D$86,S33,D33)/U33,0)</f>
         <v>200</v>
       </c>
       <c r="W33" s="45" t="n">
@@ -5284,7 +5290,7 @@
         <v>0.22</v>
       </c>
       <c r="V34" s="35" t="n">
-        <f aca="false">IF(Q34&gt;=Assumptions!$D$86,S34,D34)/U34</f>
+        <f aca="false">IF(U34&gt;0,IF(Q34&gt;=Assumptions!$D$86,S34,D34)/U34,0)</f>
         <v>88.6363636363636</v>
       </c>
       <c r="W34" s="45" t="n">
@@ -5351,7 +5357,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="22" t="s">
-        <v>736</v>
+        <v>738</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5360,46 +5366,46 @@
         <v>288</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>737</v>
+        <v>739</v>
       </c>
       <c r="D39" s="12" t="s">
-        <v>738</v>
+        <v>740</v>
       </c>
       <c r="E39" s="12" t="s">
-        <v>739</v>
+        <v>741</v>
       </c>
       <c r="F39" s="12" t="s">
-        <v>740</v>
+        <v>742</v>
       </c>
       <c r="G39" s="12" t="s">
-        <v>741</v>
+        <v>743</v>
       </c>
       <c r="H39" s="12" t="s">
-        <v>742</v>
+        <v>744</v>
       </c>
       <c r="I39" s="12" t="s">
-        <v>743</v>
+        <v>745</v>
       </c>
       <c r="J39" s="12" t="s">
-        <v>744</v>
+        <v>746</v>
       </c>
       <c r="K39" s="12" t="s">
-        <v>745</v>
+        <v>747</v>
       </c>
       <c r="L39" s="12" t="s">
-        <v>746</v>
+        <v>748</v>
       </c>
       <c r="M39" s="12" t="s">
-        <v>747</v>
+        <v>749</v>
       </c>
       <c r="N39" s="12" t="s">
-        <v>748</v>
+        <v>750</v>
       </c>
       <c r="O39" s="12" t="s">
         <v>49</v>
       </c>
       <c r="P39" s="12" t="s">
-        <v>749</v>
+        <v>751</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5428,7 +5434,7 @@
         <v>0.65</v>
       </c>
       <c r="L40" s="25" t="n">
-        <f aca="false">I40*Assumptions!$D$37*K40*Funnel!B5/(Funnel!O5*Funnel!G5)</f>
+        <f aca="false">IF(Funnel!O5*Funnel!G5&gt;0,I40*Assumptions!$D$37*K40*Budget!G21/(Funnel!O5*Funnel!G5),0)</f>
         <v>0.303789490642157</v>
       </c>
       <c r="M40" s="26" t="n">
@@ -5474,7 +5480,7 @@
         <v>0.75</v>
       </c>
       <c r="L41" s="25" t="n">
-        <f aca="false">I41*Assumptions!$D$38*K41*Funnel!B6/(Funnel!O6*Funnel!G6)</f>
+        <f aca="false">IF(Funnel!O6*Funnel!G6&gt;0,I41*Assumptions!$D$38*K41*Budget!G22/(Funnel!O6*Funnel!G6),0)</f>
         <v>0.427294347428975</v>
       </c>
       <c r="M41" s="26" t="n">
@@ -5520,7 +5526,7 @@
         <v>0.65</v>
       </c>
       <c r="L42" s="25" t="n">
-        <f aca="false">I42*Assumptions!$D$39*K42*Funnel!B7/(Funnel!O7*Funnel!G7)</f>
+        <f aca="false">IF(Funnel!O7*Funnel!G7&gt;0,I42*Assumptions!$D$39*K42*Budget!G23/(Funnel!O7*Funnel!G7),0)</f>
         <v>0.29879257155699</v>
       </c>
       <c r="M42" s="26" t="n">
@@ -5566,7 +5572,7 @@
         <v>0.7</v>
       </c>
       <c r="L43" s="25" t="n">
-        <f aca="false">I43*Assumptions!$D$40*K43*Funnel!B8/(Funnel!O8*Funnel!G8)</f>
+        <f aca="false">IF(Funnel!O8*Funnel!G8&gt;0,I43*Assumptions!$D$40*K43*Budget!G24/(Funnel!O8*Funnel!G8),0)</f>
         <v>0.274640123658854</v>
       </c>
       <c r="M43" s="26" t="n">
@@ -5629,7 +5635,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="9" t="s">
-        <v>750</v>
+        <v>752</v>
       </c>
       <c r="B46" s="9"/>
       <c r="C46" s="9"/>
@@ -9510,19 +9516,19 @@
         <v>0.0482625</v>
       </c>
       <c r="I5" s="26" t="n">
-        <f aca="false">B5/F5</f>
+        <f aca="false">IF(F5&gt;0,B5/F5,0)</f>
         <v>46.1538461538462</v>
       </c>
       <c r="J5" s="26" t="n">
-        <f aca="false">I5/E5</f>
+        <f aca="false">IF(E5&gt;0,I5/E5,0)</f>
         <v>51.2820512820513</v>
       </c>
       <c r="K5" s="26" t="n">
-        <f aca="false">J5/D5</f>
+        <f aca="false">IF(D5&gt;0,J5/D5,0)</f>
         <v>93.2400932400932</v>
       </c>
       <c r="L5" s="23" t="n">
-        <f aca="false">K5/C5</f>
+        <f aca="false">IF(C5&gt;0,K5/C5,0)</f>
         <v>621.600621600622</v>
       </c>
       <c r="M5" s="23" t="n">
@@ -9538,7 +9544,7 @@
         <v>98.7525932400932</v>
       </c>
       <c r="P5" s="25" t="n">
-        <f aca="false">O5/$B$22</f>
+        <f aca="false">IF($B$22&gt;0,O5/$B$22,0)</f>
         <v>0.306549069924901</v>
       </c>
     </row>
@@ -9575,19 +9581,19 @@
         <v>0.0891</v>
       </c>
       <c r="I6" s="26" t="n">
-        <f aca="false">B6/F6</f>
+        <f aca="false">IF(F6&gt;0,B6/F6,0)</f>
         <v>60</v>
       </c>
       <c r="J6" s="26" t="n">
-        <f aca="false">I6/E6</f>
+        <f aca="false">IF(E6&gt;0,I6/E6,0)</f>
         <v>66.6666666666667</v>
       </c>
       <c r="K6" s="26" t="n">
-        <f aca="false">J6/D6</f>
+        <f aca="false">IF(D6&gt;0,J6/D6,0)</f>
         <v>111.111111111111</v>
       </c>
       <c r="L6" s="23" t="n">
-        <f aca="false">K6/C6</f>
+        <f aca="false">IF(C6&gt;0,K6/C6,0)</f>
         <v>505.050505050505</v>
       </c>
       <c r="M6" s="23" t="n">
@@ -9603,7 +9609,7 @@
         <v>105.313820018365</v>
       </c>
       <c r="P6" s="25" t="n">
-        <f aca="false">O6/$B$22</f>
+        <f aca="false">IF($B$22&gt;0,O6/$B$22,0)</f>
         <v>0.326916514469427</v>
       </c>
     </row>
@@ -9640,19 +9646,19 @@
         <v>0.0351</v>
       </c>
       <c r="I7" s="26" t="n">
-        <f aca="false">B7/F7</f>
+        <f aca="false">IF(F7&gt;0,B7/F7,0)</f>
         <v>23.0769230769231</v>
       </c>
       <c r="J7" s="26" t="n">
-        <f aca="false">I7/E7</f>
+        <f aca="false">IF(E7&gt;0,I7/E7,0)</f>
         <v>25.6410256410256</v>
       </c>
       <c r="K7" s="26" t="n">
-        <f aca="false">J7/D7</f>
+        <f aca="false">IF(D7&gt;0,J7/D7,0)</f>
         <v>51.2820512820513</v>
       </c>
       <c r="L7" s="23" t="n">
-        <f aca="false">K7/C7</f>
+        <f aca="false">IF(C7&gt;0,K7/C7,0)</f>
         <v>427.350427350427</v>
       </c>
       <c r="M7" s="23" t="n">
@@ -9668,7 +9674,7 @@
         <v>50.2020512820513</v>
       </c>
       <c r="P7" s="25" t="n">
-        <f aca="false">O7/$B$22</f>
+        <f aca="false">IF($B$22&gt;0,O7/$B$22,0)</f>
         <v>0.155837853203707</v>
       </c>
     </row>
@@ -9705,19 +9711,19 @@
         <v>0.026775</v>
       </c>
       <c r="I8" s="26" t="n">
-        <f aca="false">B8/F8</f>
+        <f aca="false">IF(F8&gt;0,B8/F8,0)</f>
         <v>14.2857142857143</v>
       </c>
       <c r="J8" s="26" t="n">
-        <f aca="false">I8/E8</f>
+        <f aca="false">IF(E8&gt;0,I8/E8,0)</f>
         <v>16.8067226890756</v>
       </c>
       <c r="K8" s="26" t="n">
-        <f aca="false">J8/D8</f>
+        <f aca="false">IF(D8&gt;0,J8/D8,0)</f>
         <v>37.3482726423903</v>
       </c>
       <c r="L8" s="23" t="n">
-        <f aca="false">K8/C8</f>
+        <f aca="false">IF(C8&gt;0,K8/C8,0)</f>
         <v>373.482726423903</v>
       </c>
       <c r="M8" s="23" t="n">
@@ -9733,7 +9739,7 @@
         <v>36.4112856736898</v>
       </c>
       <c r="P8" s="25" t="n">
-        <f aca="false">O8/$B$22</f>
+        <f aca="false">IF($B$22&gt;0,O8/$B$22,0)</f>
         <v>0.113028381248704</v>
       </c>
     </row>
@@ -9746,7 +9752,7 @@
         <v>100</v>
       </c>
       <c r="G9" s="28" t="n">
-        <f aca="false">B9/K9</f>
+        <f aca="false">IF(K9&gt;0,B9/K9,0)</f>
         <v>0.341318446212476</v>
       </c>
       <c r="I9" s="29" t="n">
@@ -9770,7 +9776,7 @@
         <v>1610.75413506972</v>
       </c>
       <c r="N9" s="28" t="n">
-        <f aca="false">O9/M9</f>
+        <f aca="false">IF(M9&gt;0,O9/M9,0)</f>
         <v>0.180461899110145</v>
       </c>
       <c r="O9" s="29" t="n">
@@ -9778,7 +9784,7 @@
         <v>290.6797502142</v>
       </c>
       <c r="P9" s="28" t="n">
-        <f aca="false">O9/$B$22</f>
+        <f aca="false">IF($B$22&gt;0,O9/$B$22,0)</f>
         <v>0.90233181884674</v>
       </c>
     </row>
@@ -9869,7 +9875,7 @@
         <v>441</v>
       </c>
       <c r="B21" s="23" t="n">
-        <f aca="false">B17-B13+1</f>
+        <f aca="false">MAX(0,B17-B13+1)</f>
         <v>41</v>
       </c>
     </row>
@@ -9896,7 +9902,7 @@
         <v>11</v>
       </c>
       <c r="B24" s="33" t="n">
-        <f aca="false">B23/B22</f>
+        <f aca="false">IF(B22&gt;0,B23/B22,IF(B23&gt;0,9.99,0))</f>
         <v>0.90233181884674</v>
       </c>
       <c r="C24" s="22" t="str">
@@ -9909,7 +9915,7 @@
         <v>443</v>
       </c>
       <c r="B25" s="25" t="n">
-        <f aca="false">B9/O9</f>
+        <f aca="false">IF(O9&gt;0,Channels!U35/O9,0)</f>
         <v>0.344021212094447</v>
       </c>
     </row>
@@ -9982,7 +9988,7 @@
         <v>56.060915625</v>
       </c>
       <c r="E30" s="34" t="n">
-        <f aca="false">D30/B30</f>
+        <f aca="false">IF(B30&gt;0,D30/B30,0)</f>
         <v>1.8686971875</v>
       </c>
       <c r="F30" s="23" t="n">
@@ -10004,7 +10010,7 @@
         <v>457</v>
       </c>
       <c r="K30" s="34" t="n">
-        <f aca="false">(D30-SUMIFS(Channels!$N:$N,Channels!$A:$A,"I2-E",Channels!$C:$C,A30))/B30</f>
+        <f aca="false">IF(B30&gt;0,(D30-SUMIFS(Channels!$N:$N,Channels!$A:$A,"I2-E",Channels!$C:$C,A30))/B30,0)</f>
         <v>1.4825971875</v>
       </c>
     </row>
@@ -10025,7 +10031,7 @@
         <v>145.767375</v>
       </c>
       <c r="E31" s="34" t="n">
-        <f aca="false">D31/B31</f>
+        <f aca="false">IF(B31&gt;0,D31/B31,0)</f>
         <v>3.239275</v>
       </c>
       <c r="F31" s="23" t="n">
@@ -10047,7 +10053,7 @@
         <v>459</v>
       </c>
       <c r="K31" s="34" t="n">
-        <f aca="false">(D31-SUMIFS(Channels!$N:$N,Channels!$A:$A,"I2-E",Channels!$C:$C,A31))/B31</f>
+        <f aca="false">IF(B31&gt;0,(D31-SUMIFS(Channels!$N:$N,Channels!$A:$A,"I2-E",Channels!$C:$C,A31))/B31,0)</f>
         <v>3.239275</v>
       </c>
     </row>
@@ -10068,7 +10074,7 @@
         <v>29.9680875</v>
       </c>
       <c r="E32" s="34" t="n">
-        <f aca="false">D32/B32</f>
+        <f aca="false">IF(B32&gt;0,D32/B32,0)</f>
         <v>1.9978725</v>
       </c>
       <c r="F32" s="23" t="n">
@@ -10090,7 +10096,7 @@
         <v>459</v>
       </c>
       <c r="K32" s="34" t="n">
-        <f aca="false">(D32-SUMIFS(Channels!$N:$N,Channels!$A:$A,"I2-E",Channels!$C:$C,A32))/B32</f>
+        <f aca="false">IF(B32&gt;0,(D32-SUMIFS(Channels!$N:$N,Channels!$A:$A,"I2-E",Channels!$C:$C,A32))/B32,0)</f>
         <v>1.9978725</v>
       </c>
     </row>
@@ -10111,7 +10117,7 @@
         <v>17.55369</v>
       </c>
       <c r="E33" s="34" t="n">
-        <f aca="false">D33/B33</f>
+        <f aca="false">IF(B33&gt;0,D33/B33,0)</f>
         <v>1.755369</v>
       </c>
       <c r="F33" s="23" t="n">
@@ -10133,7 +10139,7 @@
         <v>459</v>
       </c>
       <c r="K33" s="34" t="n">
-        <f aca="false">(D33-SUMIFS(Channels!$N:$N,Channels!$A:$A,"I2-E",Channels!$C:$C,A33))/B33</f>
+        <f aca="false">IF(B33&gt;0,(D33-SUMIFS(Channels!$N:$N,Channels!$A:$A,"I2-E",Channels!$C:$C,A33))/B33,0)</f>
         <v>1.755369</v>
       </c>
     </row>
@@ -10224,11 +10230,11 @@
         <v>290.6797502142</v>
       </c>
       <c r="C42" s="24" t="n">
-        <f aca="false">B42/($B$22)</f>
+        <f aca="false">IF(($B$22)&gt;0,B42/($B$22),IF(B42&gt;0,9.99,0))</f>
         <v>0.90233181884674</v>
       </c>
       <c r="D42" s="32" t="n">
-        <f aca="false">MIN($B$9,$B$22/B42*$B$9,MIN(B5,D30*1)+MIN(B6,D31*1)+MIN(B7,D32*1)+MIN(B8,D33*1))</f>
+        <f aca="false">MIN($B$9,IF(B42&gt;0,$B$22/B42*$B$9,$B$9),MIN(B5,D30*1)+MIN(B6,D31*1)+MIN(B7,D32*1)+MIN(B8,D33*1))</f>
         <v>100</v>
       </c>
       <c r="E42" s="23" t="n">
@@ -10240,7 +10246,7 @@
         <v>38733.4681977991</v>
       </c>
       <c r="G42" s="24" t="n">
-        <f aca="false">F42/Budget!$C$7-1</f>
+        <f aca="false">IF(Budget!$C$7&gt;0,F42/Budget!$C$7-1,0)</f>
         <v>0</v>
       </c>
       <c r="H42" s="13" t="s">
@@ -10256,11 +10262,11 @@
         <v>415.256786020285</v>
       </c>
       <c r="C43" s="24" t="n">
-        <f aca="false">B43/($B$22)</f>
+        <f aca="false">IF(($B$22)&gt;0,B43/($B$22),IF(B43&gt;0,9.99,0))</f>
         <v>1.28904545549534</v>
       </c>
       <c r="D43" s="32" t="n">
-        <f aca="false">MIN($B$9,$B$22/B43*$B$9,MIN(B5,D30*(1-$B$40))+MIN(B6,D31*(1-$B$40))+MIN(B7,D32*(1-$B$40))+MIN(B8,D33*(1-$B$40)))</f>
+        <f aca="false">MIN($B$9,IF(B43&gt;0,$B$22/B43*$B$9,$B$9),MIN(B5,D30*(1-$B$40))+MIN(B6,D31*(1-$B$40))+MIN(B7,D32*(1-$B$40))+MIN(B8,D33*(1-$B$40)))</f>
         <v>77.5767833272977</v>
       </c>
       <c r="E43" s="23" t="n">
@@ -10272,7 +10278,7 @@
         <v>55333.5259968559</v>
       </c>
       <c r="G43" s="24" t="n">
-        <f aca="false">F43/Budget!$C$7-1</f>
+        <f aca="false">IF(Budget!$C$7&gt;0,F43/Budget!$C$7-1,0)</f>
         <v>0.428571428571429</v>
       </c>
       <c r="H43" s="13" t="s">
@@ -10288,11 +10294,11 @@
         <v>415.256786020285</v>
       </c>
       <c r="C44" s="24" t="n">
-        <f aca="false">B44/($B$22)</f>
+        <f aca="false">IF(($B$22)&gt;0,B44/($B$22),IF(B44&gt;0,9.99,0))</f>
         <v>1.28904545549534</v>
       </c>
       <c r="D44" s="32" t="n">
-        <f aca="false">MIN($B$9,$B$22/B44*$B$9,MIN(B5,D30*(1-$B$40))+MIN(B6,D31*(1-$B$40))+MIN(B7,D32*(1-$B$40))+MIN(B8,D33*(1-$B$40)))</f>
+        <f aca="false">MIN($B$9,IF(B44&gt;0,$B$22/B44*$B$9,$B$9),MIN(B5,D30*(1-$B$40))+MIN(B6,D31*(1-$B$40))+MIN(B7,D32*(1-$B$40))+MIN(B8,D33*(1-$B$40)))</f>
         <v>77.5767833272977</v>
       </c>
       <c r="E44" s="23" t="n">
@@ -10304,7 +10310,7 @@
         <v>55333.5259968559</v>
       </c>
       <c r="G44" s="24" t="n">
-        <f aca="false">F44/Budget!$C$7-1</f>
+        <f aca="false">IF(Budget!$C$7&gt;0,F44/Budget!$C$7-1,0)</f>
         <v>0.428571428571429</v>
       </c>
       <c r="H44" s="13" t="s">
@@ -10320,11 +10326,11 @@
         <v>290.6797502142</v>
       </c>
       <c r="C45" s="24" t="n">
-        <f aca="false">B45/($B$22)</f>
+        <f aca="false">IF(($B$22)&gt;0,B45/($B$22),IF(B45&gt;0,9.99,0))</f>
         <v>0.90233181884674</v>
       </c>
       <c r="D45" s="32" t="n">
-        <f aca="false">MIN($B$9,$B$22/B45*$B$9,MIN(B5,D30*(1-$B$40))+MIN(B6,D31*(1-$B$40))+MIN(B7,D32*(1-$B$40))+MIN(B8,D33*(1-$B$40)))</f>
+        <f aca="false">MIN($B$9,IF(B45&gt;0,$B$22/B45*$B$9,$B$9),MIN(B5,D30*(1-$B$40))+MIN(B6,D31*(1-$B$40))+MIN(B7,D32*(1-$B$40))+MIN(B8,D33*(1-$B$40)))</f>
         <v>100</v>
       </c>
       <c r="E45" s="23" t="n">
@@ -10336,7 +10342,7 @@
         <v>55333.5259968559</v>
       </c>
       <c r="G45" s="24" t="n">
-        <f aca="false">F45/Budget!$C$7-1</f>
+        <f aca="false">IF(Budget!$C$7&gt;0,F45/Budget!$C$7-1,0)</f>
         <v>0.428571428571429</v>
       </c>
       <c r="H45" s="13" t="s">
@@ -10352,11 +10358,11 @@
         <v>290.6797502142</v>
       </c>
       <c r="C46" s="24" t="n">
-        <f aca="false">B46/($B$22)</f>
+        <f aca="false">IF(($B$22)&gt;0,B46/($B$22),IF(B46&gt;0,9.99,0))</f>
         <v>0.90233181884674</v>
       </c>
       <c r="D46" s="32" t="n">
-        <f aca="false">MIN($B$9,$B$22/B46*$B$9,MIN(B5,D30*1)+MIN(B6,D31*1)+MIN(B7,D32*1)+MIN(B8,D33*1))</f>
+        <f aca="false">MIN($B$9,IF(B46&gt;0,$B$22/B46*$B$9,$B$9),MIN(B5,D30*1)+MIN(B6,D31*1)+MIN(B7,D32*1)+MIN(B8,D33*1))</f>
         <v>100</v>
       </c>
       <c r="E46" s="23" t="n">
@@ -10368,7 +10374,7 @@
         <v>50353.5086571388</v>
       </c>
       <c r="G46" s="24" t="n">
-        <f aca="false">F46/Budget!$C$7-1</f>
+        <f aca="false">IF(Budget!$C$7&gt;0,F46/Budget!$C$7-1,0)</f>
         <v>0.3</v>
       </c>
       <c r="H46" s="13" t="s">
@@ -10384,11 +10390,11 @@
         <v>290.6797502142</v>
       </c>
       <c r="C47" s="24" t="n">
-        <f aca="false">B47/($B$22*(1-$B$40))</f>
+        <f aca="false">IF(($B$22*(1-$B$40))&gt;0,B47/($B$22*(1-$B$40)),IF(B47&gt;0,9.99,0))</f>
         <v>1.28904545549534</v>
       </c>
       <c r="D47" s="32" t="n">
-        <f aca="false">MIN($B$9,$B$22*(1-$B$40)/B47*$B$9,MIN(B5,D30*1)+MIN(B6,D31*1)+MIN(B7,D32*1)+MIN(B8,D33*1))</f>
+        <f aca="false">MIN($B$9,IF(B47&gt;0,$B$22*(1-$B$40)/B47*$B$9,$B$9),MIN(B5,D30*1)+MIN(B6,D31*1)+MIN(B7,D32*1)+MIN(B8,D33*1))</f>
         <v>77.5767833272977</v>
       </c>
       <c r="E47" s="23" t="n">
@@ -10400,7 +10406,7 @@
         <v>38733.4681977991</v>
       </c>
       <c r="G47" s="24" t="n">
-        <f aca="false">F47/Budget!$C$7-1</f>
+        <f aca="false">IF(Budget!$C$7&gt;0,F47/Budget!$C$7-1,0)</f>
         <v>0</v>
       </c>
       <c r="H47" s="13" t="s">
@@ -10534,7 +10540,7 @@
         <v>53.7525932400932</v>
       </c>
       <c r="H5" s="24" t="n">
-        <f aca="false">G5/F5</f>
+        <f aca="false">IF(F5&gt;0,G5/F5,0)</f>
         <v>0.0943027951580583</v>
       </c>
       <c r="I5" s="23" t="n">
@@ -10542,7 +10548,7 @@
         <v>134.75</v>
       </c>
       <c r="J5" s="24" t="n">
-        <f aca="false">I5/F5</f>
+        <f aca="false">IF(F5&gt;0,I5/F5,0)</f>
         <v>0.23640350877193</v>
       </c>
       <c r="K5" s="2" t="str">
@@ -10579,7 +10585,7 @@
         <v>105.313820018365</v>
       </c>
       <c r="H6" s="24" t="n">
-        <f aca="false">G6/F6</f>
+        <f aca="false">IF(F6&gt;0,G6/F6,0)</f>
         <v>0.054850947926232</v>
       </c>
       <c r="I6" s="23" t="n">
@@ -10587,7 +10593,7 @@
         <v>409.75</v>
       </c>
       <c r="J6" s="24" t="n">
-        <f aca="false">I6/F6</f>
+        <f aca="false">IF(F6&gt;0,I6/F6,0)</f>
         <v>0.213411458333333</v>
       </c>
       <c r="K6" s="2" t="str">
@@ -10624,7 +10630,7 @@
         <v>50.2020512820513</v>
       </c>
       <c r="H7" s="24" t="n">
-        <f aca="false">G7/F7</f>
+        <f aca="false">IF(F7&gt;0,G7/F7,0)</f>
         <v>0.0912764568764569</v>
       </c>
       <c r="I7" s="23" t="n">
@@ -10632,7 +10638,7 @@
         <v>100.7</v>
       </c>
       <c r="J7" s="24" t="n">
-        <f aca="false">I7/F7</f>
+        <f aca="false">IF(F7&gt;0,I7/F7,0)</f>
         <v>0.183090909090909</v>
       </c>
       <c r="K7" s="2" t="str">
@@ -10669,7 +10675,7 @@
         <v>36.4112856736898</v>
       </c>
       <c r="H8" s="24" t="n">
-        <f aca="false">G8/F8</f>
+        <f aca="false">IF(F8&gt;0,G8/F8,0)</f>
         <v>0.165505843971317</v>
       </c>
       <c r="I8" s="23" t="n">
@@ -10677,7 +10683,7 @@
         <v>64.3</v>
       </c>
       <c r="J8" s="24" t="n">
-        <f aca="false">I8/F8</f>
+        <f aca="false">IF(F8&gt;0,I8/F8,0)</f>
         <v>0.292272727272727</v>
       </c>
       <c r="K8" s="2" t="str">
@@ -10916,19 +10922,19 @@
         <v>505</v>
       </c>
       <c r="B11" s="37" t="n">
-        <f aca="false">B10/B7</f>
+        <f aca="false">IF(B7&gt;0,B10/B7,0)</f>
         <v>4.16666666666667</v>
       </c>
       <c r="C11" s="37" t="n">
-        <f aca="false">C10/C7</f>
+        <f aca="false">IF(C7&gt;0,C10/C7,0)</f>
         <v>4.16666666666667</v>
       </c>
       <c r="D11" s="37" t="n">
-        <f aca="false">D10/D7</f>
+        <f aca="false">IF(D7&gt;0,D10/D7,0)</f>
         <v>4.16666666666667</v>
       </c>
       <c r="E11" s="37" t="n">
-        <f aca="false">E10/E7</f>
+        <f aca="false">IF(E7&gt;0,E10/E7,0)</f>
         <v>4.16666666666667</v>
       </c>
       <c r="G11" s="13" t="s">
@@ -11061,19 +11067,19 @@
         <v>512</v>
       </c>
       <c r="B17" s="37" t="n">
-        <f aca="false">B16/B13</f>
+        <f aca="false">IF(B13&gt;0,B16/B13,0)</f>
         <v>166.505625</v>
       </c>
       <c r="C17" s="37" t="n">
-        <f aca="false">C16/C13</f>
+        <f aca="false">IF(C13&gt;0,C16/C13,0)</f>
         <v>209.5875</v>
       </c>
       <c r="D17" s="37" t="n">
-        <f aca="false">D16/D13</f>
+        <f aca="false">IF(D13&gt;0,D16/D13,0)</f>
         <v>151.36875</v>
       </c>
       <c r="E17" s="37" t="n">
-        <f aca="false">E16/E13</f>
+        <f aca="false">IF(E13&gt;0,E16/E13,0)</f>
         <v>138.560625</v>
       </c>
       <c r="G17" s="13" t="s">
@@ -11135,23 +11141,23 @@
         <v>516</v>
       </c>
       <c r="B20" s="35" t="n">
-        <f aca="false">B19/B18</f>
+        <f aca="false">IF(B18&gt;0,B19/B18,0)</f>
         <v>495.49510278823</v>
       </c>
       <c r="C20" s="35" t="n">
-        <f aca="false">C19/C18</f>
+        <f aca="false">IF(C18&gt;0,C19/C18,0)</f>
         <v>438.795593384965</v>
       </c>
       <c r="D20" s="35" t="n">
-        <f aca="false">D19/D18</f>
+        <f aca="false">IF(D18&gt;0,D19/D18,0)</f>
         <v>399.860884810718</v>
       </c>
       <c r="E20" s="35" t="n">
-        <f aca="false">E19/E18</f>
+        <f aca="false">IF(E18&gt;0,E19/E18,0)</f>
         <v>444.036551818795</v>
       </c>
       <c r="F20" s="36" t="n">
-        <f aca="false">F19/F18</f>
+        <f aca="false">IF(F18&gt;0,F19/F18,0)</f>
         <v>450.47833548117</v>
       </c>
     </row>
@@ -11255,7 +11261,7 @@
         <v>528</v>
       </c>
       <c r="B34" s="35" t="n">
-        <f aca="false">(B32+B33)/B31</f>
+        <f aca="false">IF(B31&gt;0,(B32+B33)/B31,0)</f>
         <v>880.600880600881</v>
       </c>
     </row>
@@ -11350,7 +11356,7 @@
         <v>538</v>
       </c>
       <c r="B47" s="23" t="n">
-        <f aca="false">B43/B41/B39</f>
+        <f aca="false">IF(B41*B39&gt;0,B43/B41/B39,0)</f>
         <v>183.654729109275</v>
       </c>
     </row>
@@ -11359,7 +11365,7 @@
         <v>539</v>
       </c>
       <c r="B48" s="35" t="n">
-        <f aca="false">(B47*B38+B46)/B43</f>
+        <f aca="false">IF(B43&gt;0,(B47*B38+B46)/B43,0)</f>
         <v>221.181512090603</v>
       </c>
     </row>
@@ -11451,19 +11457,19 @@
         <v>558</v>
       </c>
       <c r="C54" s="24" t="n">
-        <f aca="false">(Assumptions!$D$55*4/7+Assumptions!$D$56+Assumptions!$D$57*4/7)</f>
-        <v>0.181428571428571</v>
+        <f aca="false">(Assumptions!$D$55*4/7+Assumptions!$D$56+Assumptions!$D$57*3/7)</f>
+        <v>0.152857142857143</v>
       </c>
       <c r="D54" s="35" t="n">
         <f aca="false">B33+SUMIFS(Channels!$X:$X,Channels!$A:$A,"I2-E")*C54</f>
-        <v>2832.85714285714</v>
+        <v>2575.71428571429</v>
       </c>
       <c r="E54" s="26" t="n">
         <f aca="false">SUMIFS(Channels!$V:$V,Channels!$A:$A,"I2-E")*C54</f>
-        <v>8.16428571428572</v>
+        <v>6.87857142857143</v>
       </c>
       <c r="F54" s="35" t="n">
-        <f aca="false">B27/B28</f>
+        <f aca="false">IF(B28&gt;0,B27/B28,0)</f>
         <v>200</v>
       </c>
       <c r="G54" s="23" t="n">
@@ -11506,7 +11512,7 @@
         <v>7.7432277318641</v>
       </c>
       <c r="F55" s="35" t="n">
-        <f aca="false">B38/B39</f>
+        <f aca="false">IF(B39&gt;0,B38/B39,0)</f>
         <v>88.6363636363636</v>
       </c>
       <c r="G55" s="23" t="n">
@@ -11714,7 +11720,7 @@
         <v/>
       </c>
       <c r="H5" s="37" t="n">
-        <f aca="false">IF(E5="CPC",F5/G5,IF(E5="Slot",F5/G5,F5))</f>
+        <f aca="false">IF(OR(E5="CPC",E5="Slot"),IF(N(G5)&gt;0,F5/G5,0),F5)</f>
         <v>0</v>
       </c>
       <c r="I5" s="24" t="n">
@@ -11722,7 +11728,7 @@
         <v>0.08</v>
       </c>
       <c r="J5" s="23" t="n">
-        <f aca="false">IF(E5="Slot",Assumptions!H112*G5,Assumptions!H112)</f>
+        <f aca="false">IF(AND(OR(E5="CPC",E5="Slot"),NOT(N(G5)&gt;0)),0,IF(E5="Slot",Assumptions!H112*G5,Assumptions!H112))</f>
         <v>150</v>
       </c>
       <c r="K5" s="26" t="n">
@@ -11754,11 +11760,11 @@
         <v>5E-006</v>
       </c>
       <c r="R5" s="23" t="n">
-        <f aca="false">COUNTIFS($C$5:$C$34,C5,$Q$5:$Q$34,"&lt;"&amp;Q5)+1</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C5)*($Q$5:$Q$34&lt;Q5))+1</f>
         <v>1</v>
       </c>
       <c r="S5" s="26" t="n">
-        <f aca="false">SUMIFS($AH$5:$AH$34,$C$5:$C$34,C5,$Q$5:$Q$34,"&lt;"&amp;Q5)</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C5)*($Q$5:$Q$34&lt;Q5)*$AH$5:$AH$34)</f>
         <v>0</v>
       </c>
       <c r="T5" s="26" t="n">
@@ -11778,7 +11784,7 @@
         <v>150</v>
       </c>
       <c r="X5" s="35" t="n">
-        <f aca="false">IF(E5="Slot",ROUNDUP(W5/G5,0)*F5,W5*H5)</f>
+        <f aca="false">IF(E5="Slot",IF(N(G5)&gt;0,ROUNDUP(W5/G5,0)*F5,0),W5*H5)</f>
         <v>0</v>
       </c>
       <c r="Y5" s="35" t="n">
@@ -11798,7 +11804,7 @@
         <v>0</v>
       </c>
       <c r="AC5" s="23" t="n">
-        <f aca="false">COUNTIF($Q$5:$Q$34,"&lt;"&amp;Q5)+1</f>
+        <f aca="false">SUMPRODUCT(--($Q$5:$Q$34&lt;Q5))+1</f>
         <v>1</v>
       </c>
       <c r="AD5" s="2" t="str">
@@ -11855,7 +11861,7 @@
         <v/>
       </c>
       <c r="H6" s="37" t="n">
-        <f aca="false">IF(E6="CPC",F6/G6,IF(E6="Slot",F6/G6,F6))</f>
+        <f aca="false">IF(OR(E6="CPC",E6="Slot"),IF(N(G6)&gt;0,F6/G6,0),F6)</f>
         <v>0</v>
       </c>
       <c r="I6" s="24" t="n">
@@ -11863,7 +11869,7 @@
         <v>0.18</v>
       </c>
       <c r="J6" s="23" t="n">
-        <f aca="false">IF(E6="Slot",Assumptions!H113*G6,Assumptions!H113)</f>
+        <f aca="false">IF(AND(OR(E6="CPC",E6="Slot"),NOT(N(G6)&gt;0)),0,IF(E6="Slot",Assumptions!H113*G6,Assumptions!H113))</f>
         <v>200</v>
       </c>
       <c r="K6" s="26" t="n">
@@ -11895,11 +11901,11 @@
         <v>6E-006</v>
       </c>
       <c r="R6" s="23" t="n">
-        <f aca="false">COUNTIFS($C$5:$C$34,C6,$Q$5:$Q$34,"&lt;"&amp;Q6)+1</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C6)*($Q$5:$Q$34&lt;Q6))+1</f>
         <v>1</v>
       </c>
       <c r="S6" s="26" t="n">
-        <f aca="false">SUMIFS($AH$5:$AH$34,$C$5:$C$34,C6,$Q$5:$Q$34,"&lt;"&amp;Q6)</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C6)*($Q$5:$Q$34&lt;Q6)*$AH$5:$AH$34)</f>
         <v>0</v>
       </c>
       <c r="T6" s="26" t="n">
@@ -11919,7 +11925,7 @@
         <v>200</v>
       </c>
       <c r="X6" s="35" t="n">
-        <f aca="false">IF(E6="Slot",ROUNDUP(W6/G6,0)*F6,W6*H6)</f>
+        <f aca="false">IF(E6="Slot",IF(N(G6)&gt;0,ROUNDUP(W6/G6,0)*F6,0),W6*H6)</f>
         <v>0</v>
       </c>
       <c r="Y6" s="35" t="n">
@@ -11939,7 +11945,7 @@
         <v>0</v>
       </c>
       <c r="AC6" s="23" t="n">
-        <f aca="false">COUNTIF($Q$5:$Q$34,"&lt;"&amp;Q6)+1</f>
+        <f aca="false">SUMPRODUCT(--($Q$5:$Q$34&lt;Q6))+1</f>
         <v>2</v>
       </c>
       <c r="AD6" s="2" t="str">
@@ -11996,7 +12002,7 @@
         <v/>
       </c>
       <c r="H7" s="37" t="n">
-        <f aca="false">IF(E7="CPC",F7/G7,IF(E7="Slot",F7/G7,F7))</f>
+        <f aca="false">IF(OR(E7="CPC",E7="Slot"),IF(N(G7)&gt;0,F7/G7,0),F7)</f>
         <v>0</v>
       </c>
       <c r="I7" s="24" t="n">
@@ -12004,7 +12010,7 @@
         <v>0.1</v>
       </c>
       <c r="J7" s="23" t="n">
-        <f aca="false">IF(E7="Slot",Assumptions!H114*G7,Assumptions!H114)</f>
+        <f aca="false">IF(AND(OR(E7="CPC",E7="Slot"),NOT(N(G7)&gt;0)),0,IF(E7="Slot",Assumptions!H114*G7,Assumptions!H114))</f>
         <v>80</v>
       </c>
       <c r="K7" s="26" t="n">
@@ -12036,11 +12042,11 @@
         <v>7E-006</v>
       </c>
       <c r="R7" s="23" t="n">
-        <f aca="false">COUNTIFS($C$5:$C$34,C7,$Q$5:$Q$34,"&lt;"&amp;Q7)+1</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C7)*($Q$5:$Q$34&lt;Q7))+1</f>
         <v>1</v>
       </c>
       <c r="S7" s="26" t="n">
-        <f aca="false">SUMIFS($AH$5:$AH$34,$C$5:$C$34,C7,$Q$5:$Q$34,"&lt;"&amp;Q7)</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C7)*($Q$5:$Q$34&lt;Q7)*$AH$5:$AH$34)</f>
         <v>0</v>
       </c>
       <c r="T7" s="26" t="n">
@@ -12060,7 +12066,7 @@
         <v>80</v>
       </c>
       <c r="X7" s="35" t="n">
-        <f aca="false">IF(E7="Slot",ROUNDUP(W7/G7,0)*F7,W7*H7)</f>
+        <f aca="false">IF(E7="Slot",IF(N(G7)&gt;0,ROUNDUP(W7/G7,0)*F7,0),W7*H7)</f>
         <v>0</v>
       </c>
       <c r="Y7" s="35" t="n">
@@ -12080,7 +12086,7 @@
         <v>0</v>
       </c>
       <c r="AC7" s="23" t="n">
-        <f aca="false">COUNTIF($Q$5:$Q$34,"&lt;"&amp;Q7)+1</f>
+        <f aca="false">SUMPRODUCT(--($Q$5:$Q$34&lt;Q7))+1</f>
         <v>3</v>
       </c>
       <c r="AD7" s="2" t="str">
@@ -12137,7 +12143,7 @@
         <v/>
       </c>
       <c r="H8" s="37" t="n">
-        <f aca="false">IF(E8="CPC",F8/G8,IF(E8="Slot",F8/G8,F8))</f>
+        <f aca="false">IF(OR(E8="CPC",E8="Slot"),IF(N(G8)&gt;0,F8/G8,0),F8)</f>
         <v>0</v>
       </c>
       <c r="I8" s="24" t="n">
@@ -12145,7 +12151,7 @@
         <v>0.08</v>
       </c>
       <c r="J8" s="23" t="n">
-        <f aca="false">IF(E8="Slot",Assumptions!H115*G8,Assumptions!H115)</f>
+        <f aca="false">IF(AND(OR(E8="CPC",E8="Slot"),NOT(N(G8)&gt;0)),0,IF(E8="Slot",Assumptions!H115*G8,Assumptions!H115))</f>
         <v>60</v>
       </c>
       <c r="K8" s="26" t="n">
@@ -12177,11 +12183,11 @@
         <v>8E-006</v>
       </c>
       <c r="R8" s="23" t="n">
-        <f aca="false">COUNTIFS($C$5:$C$34,C8,$Q$5:$Q$34,"&lt;"&amp;Q8)+1</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C8)*($Q$5:$Q$34&lt;Q8))+1</f>
         <v>1</v>
       </c>
       <c r="S8" s="26" t="n">
-        <f aca="false">SUMIFS($AH$5:$AH$34,$C$5:$C$34,C8,$Q$5:$Q$34,"&lt;"&amp;Q8)</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C8)*($Q$5:$Q$34&lt;Q8)*$AH$5:$AH$34)</f>
         <v>0</v>
       </c>
       <c r="T8" s="26" t="n">
@@ -12201,7 +12207,7 @@
         <v>60</v>
       </c>
       <c r="X8" s="35" t="n">
-        <f aca="false">IF(E8="Slot",ROUNDUP(W8/G8,0)*F8,W8*H8)</f>
+        <f aca="false">IF(E8="Slot",IF(N(G8)&gt;0,ROUNDUP(W8/G8,0)*F8,0),W8*H8)</f>
         <v>0</v>
       </c>
       <c r="Y8" s="35" t="n">
@@ -12221,7 +12227,7 @@
         <v>0</v>
       </c>
       <c r="AC8" s="23" t="n">
-        <f aca="false">COUNTIF($Q$5:$Q$34,"&lt;"&amp;Q8)+1</f>
+        <f aca="false">SUMPRODUCT(--($Q$5:$Q$34&lt;Q8))+1</f>
         <v>4</v>
       </c>
       <c r="AD8" s="2" t="str">
@@ -12278,7 +12284,7 @@
         <v>0.035</v>
       </c>
       <c r="H9" s="37" t="n">
-        <f aca="false">IF(E9="CPC",F9/G9,IF(E9="Slot",F9/G9,F9))</f>
+        <f aca="false">IF(OR(E9="CPC",E9="Slot"),IF(N(G9)&gt;0,F9/G9,0),F9)</f>
         <v>57.1428571428571</v>
       </c>
       <c r="I9" s="24" t="n">
@@ -12286,7 +12292,7 @@
         <v>0.12</v>
       </c>
       <c r="J9" s="23" t="n">
-        <f aca="false">IF(E9="Slot",Assumptions!H116*G9,Assumptions!H116)</f>
+        <f aca="false">IF(AND(OR(E9="CPC",E9="Slot"),NOT(N(G9)&gt;0)),0,IF(E9="Slot",Assumptions!H116*G9,Assumptions!H116))</f>
         <v>450</v>
       </c>
       <c r="K9" s="26" t="n">
@@ -12318,11 +12324,11 @@
         <v>1480.00148900148</v>
       </c>
       <c r="R9" s="23" t="n">
-        <f aca="false">COUNTIFS($C$5:$C$34,C9,$Q$5:$Q$34,"&lt;"&amp;Q9)+1</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C9)*($Q$5:$Q$34&lt;Q9))+1</f>
         <v>8</v>
       </c>
       <c r="S9" s="26" t="n">
-        <f aca="false">SUMIFS($AH$5:$AH$34,$C$5:$C$34,C9,$Q$5:$Q$34,"&lt;"&amp;Q9)</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C9)*($Q$5:$Q$34&lt;Q9)*$AH$5:$AH$34)</f>
         <v>36.864384375</v>
       </c>
       <c r="T9" s="26" t="n">
@@ -12342,7 +12348,7 @@
         <v>13.125</v>
       </c>
       <c r="X9" s="35" t="n">
-        <f aca="false">IF(E9="Slot",ROUNDUP(W9/G9,0)*F9,W9*H9)</f>
+        <f aca="false">IF(E9="Slot",IF(N(G9)&gt;0,ROUNDUP(W9/G9,0)*F9,0),W9*H9)</f>
         <v>750</v>
       </c>
       <c r="Y9" s="35" t="n">
@@ -12362,7 +12368,7 @@
         <v>1480.00148000148</v>
       </c>
       <c r="AC9" s="23" t="n">
-        <f aca="false">COUNTIF($Q$5:$Q$34,"&lt;"&amp;Q9)+1</f>
+        <f aca="false">SUMPRODUCT(--($Q$5:$Q$34&lt;Q9))+1</f>
         <v>29</v>
       </c>
       <c r="AD9" s="2" t="str">
@@ -12419,7 +12425,7 @@
         <v>0.05</v>
       </c>
       <c r="H10" s="37" t="n">
-        <f aca="false">IF(E10="CPC",F10/G10,IF(E10="Slot",F10/G10,F10))</f>
+        <f aca="false">IF(OR(E10="CPC",E10="Slot"),IF(N(G10)&gt;0,F10/G10,0),F10)</f>
         <v>24</v>
       </c>
       <c r="I10" s="24" t="n">
@@ -12427,7 +12433,7 @@
         <v>0.22</v>
       </c>
       <c r="J10" s="23" t="n">
-        <f aca="false">IF(E10="Slot",Assumptions!H117*G10,Assumptions!H117)</f>
+        <f aca="false">IF(AND(OR(E10="CPC",E10="Slot"),NOT(N(G10)&gt;0)),0,IF(E10="Slot",Assumptions!H117*G10,Assumptions!H117))</f>
         <v>600</v>
       </c>
       <c r="K10" s="26" t="n">
@@ -12459,11 +12465,11 @@
         <v>269.360279360269</v>
       </c>
       <c r="R10" s="23" t="n">
-        <f aca="false">COUNTIFS($C$5:$C$34,C10,$Q$5:$Q$34,"&lt;"&amp;Q10)+1</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C10)*($Q$5:$Q$34&lt;Q10))+1</f>
         <v>5</v>
       </c>
       <c r="S10" s="26" t="n">
-        <f aca="false">SUMIFS($AH$5:$AH$34,$C$5:$C$34,C10,$Q$5:$Q$34,"&lt;"&amp;Q10)</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C10)*($Q$5:$Q$34&lt;Q10)*$AH$5:$AH$34)</f>
         <v>62.226</v>
       </c>
       <c r="T10" s="26" t="n">
@@ -12483,7 +12489,7 @@
         <v>31.25</v>
       </c>
       <c r="X10" s="35" t="n">
-        <f aca="false">IF(E10="Slot",ROUNDUP(W10/G10,0)*F10,W10*H10)</f>
+        <f aca="false">IF(E10="Slot",IF(N(G10)&gt;0,ROUNDUP(W10/G10,0)*F10,0),W10*H10)</f>
         <v>750</v>
       </c>
       <c r="Y10" s="35" t="n">
@@ -12503,7 +12509,7 @@
         <v>269.360269360269</v>
       </c>
       <c r="AC10" s="23" t="n">
-        <f aca="false">COUNTIF($Q$5:$Q$34,"&lt;"&amp;Q10)+1</f>
+        <f aca="false">SUMPRODUCT(--($Q$5:$Q$34&lt;Q10))+1</f>
         <v>11</v>
       </c>
       <c r="AD10" s="2" t="str">
@@ -12560,7 +12566,7 @@
         <v>0.04</v>
       </c>
       <c r="H11" s="37" t="n">
-        <f aca="false">IF(E11="CPC",F11/G11,IF(E11="Slot",F11/G11,F11))</f>
+        <f aca="false">IF(OR(E11="CPC",E11="Slot"),IF(N(G11)&gt;0,F11/G11,0),F11)</f>
         <v>45</v>
       </c>
       <c r="I11" s="24" t="n">
@@ -12568,7 +12574,7 @@
         <v>0.12</v>
       </c>
       <c r="J11" s="23" t="n">
-        <f aca="false">IF(E11="Slot",Assumptions!H118*G11,Assumptions!H118)</f>
+        <f aca="false">IF(AND(OR(E11="CPC",E11="Slot"),NOT(N(G11)&gt;0)),0,IF(E11="Slot",Assumptions!H118*G11,Assumptions!H118))</f>
         <v>250</v>
       </c>
       <c r="K11" s="26" t="n">
@@ -12600,11 +12606,11 @@
         <v>1282.05129305128</v>
       </c>
       <c r="R11" s="23" t="n">
-        <f aca="false">COUNTIFS($C$5:$C$34,C11,$Q$5:$Q$34,"&lt;"&amp;Q11)+1</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C11)*($Q$5:$Q$34&lt;Q11))+1</f>
         <v>6</v>
       </c>
       <c r="S11" s="26" t="n">
-        <f aca="false">SUMIFS($AH$5:$AH$34,$C$5:$C$34,C11,$Q$5:$Q$34,"&lt;"&amp;Q11)</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C11)*($Q$5:$Q$34&lt;Q11)*$AH$5:$AH$34)</f>
         <v>16.698749025974</v>
       </c>
       <c r="T11" s="26" t="n">
@@ -12624,7 +12630,7 @@
         <v>16.6666666666667</v>
       </c>
       <c r="X11" s="35" t="n">
-        <f aca="false">IF(E11="Slot",ROUNDUP(W11/G11,0)*F11,W11*H11)</f>
+        <f aca="false">IF(E11="Slot",IF(N(G11)&gt;0,ROUNDUP(W11/G11,0)*F11,0),W11*H11)</f>
         <v>750</v>
       </c>
       <c r="Y11" s="35" t="n">
@@ -12644,7 +12650,7 @@
         <v>1282.05128205128</v>
       </c>
       <c r="AC11" s="23" t="n">
-        <f aca="false">COUNTIF($Q$5:$Q$34,"&lt;"&amp;Q11)+1</f>
+        <f aca="false">SUMPRODUCT(--($Q$5:$Q$34&lt;Q11))+1</f>
         <v>26</v>
       </c>
       <c r="AD11" s="2" t="str">
@@ -12701,7 +12707,7 @@
         <v>0.04</v>
       </c>
       <c r="H12" s="37" t="n">
-        <f aca="false">IF(E12="CPC",F12/G12,IF(E12="Slot",F12/G12,F12))</f>
+        <f aca="false">IF(OR(E12="CPC",E12="Slot"),IF(N(G12)&gt;0,F12/G12,0),F12)</f>
         <v>42.5</v>
       </c>
       <c r="I12" s="24" t="n">
@@ -12709,7 +12715,7 @@
         <v>0.1</v>
       </c>
       <c r="J12" s="23" t="n">
-        <f aca="false">IF(E12="Slot",Assumptions!H119*G12,Assumptions!H119)</f>
+        <f aca="false">IF(AND(OR(E12="CPC",E12="Slot"),NOT(N(G12)&gt;0)),0,IF(E12="Slot",Assumptions!H119*G12,Assumptions!H119))</f>
         <v>200</v>
       </c>
       <c r="K12" s="26" t="n">
@@ -12741,11 +12747,11 @@
         <v>1587.30159930159</v>
       </c>
       <c r="R12" s="23" t="n">
-        <f aca="false">COUNTIFS($C$5:$C$34,C12,$Q$5:$Q$34,"&lt;"&amp;Q12)+1</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C12)*($Q$5:$Q$34&lt;Q12))+1</f>
         <v>7</v>
       </c>
       <c r="S12" s="26" t="n">
-        <f aca="false">SUMIFS($AH$5:$AH$34,$C$5:$C$34,C12,$Q$5:$Q$34,"&lt;"&amp;Q12)</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C12)*($Q$5:$Q$34&lt;Q12)*$AH$5:$AH$34)</f>
         <v>10.5139513636364</v>
       </c>
       <c r="T12" s="26" t="n">
@@ -12765,7 +12771,7 @@
         <v>17.6470588235294</v>
       </c>
       <c r="X12" s="35" t="n">
-        <f aca="false">IF(E12="Slot",ROUNDUP(W12/G12,0)*F12,W12*H12)</f>
+        <f aca="false">IF(E12="Slot",IF(N(G12)&gt;0,ROUNDUP(W12/G12,0)*F12,0),W12*H12)</f>
         <v>750</v>
       </c>
       <c r="Y12" s="35" t="n">
@@ -12785,7 +12791,7 @@
         <v>1587.30158730159</v>
       </c>
       <c r="AC12" s="23" t="n">
-        <f aca="false">COUNTIF($Q$5:$Q$34,"&lt;"&amp;Q12)+1</f>
+        <f aca="false">SUMPRODUCT(--($Q$5:$Q$34&lt;Q12))+1</f>
         <v>30</v>
       </c>
       <c r="AD12" s="2" t="str">
@@ -12842,7 +12848,7 @@
         <v>15</v>
       </c>
       <c r="H13" s="37" t="n">
-        <f aca="false">IF(E13="CPC",F13/G13,IF(E13="Slot",F13/G13,F13))</f>
+        <f aca="false">IF(OR(E13="CPC",E13="Slot"),IF(N(G13)&gt;0,F13/G13,0),F13)</f>
         <v>96.6</v>
       </c>
       <c r="I13" s="24" t="n">
@@ -12850,7 +12856,7 @@
         <v>0.3</v>
       </c>
       <c r="J13" s="23" t="n">
-        <f aca="false">IF(E13="Slot",Assumptions!H120*G13,Assumptions!H120)</f>
+        <f aca="false">IF(AND(OR(E13="CPC",E13="Slot"),NOT(N(G13)&gt;0)),0,IF(E13="Slot",Assumptions!H120*G13,Assumptions!H120))</f>
         <v>45</v>
       </c>
       <c r="K13" s="26" t="n">
@@ -12882,11 +12888,11 @@
         <v>1000.777013777</v>
       </c>
       <c r="R13" s="23" t="n">
-        <f aca="false">COUNTIFS($C$5:$C$34,C13,$Q$5:$Q$34,"&lt;"&amp;Q13)+1</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C13)*($Q$5:$Q$34&lt;Q13))+1</f>
         <v>6</v>
       </c>
       <c r="S13" s="26" t="n">
-        <f aca="false">SUMIFS($AH$5:$AH$34,$C$5:$C$34,C13,$Q$5:$Q$34,"&lt;"&amp;Q13)</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C13)*($Q$5:$Q$34&lt;Q13)*$AH$5:$AH$34)</f>
         <v>26.756071875</v>
       </c>
       <c r="T13" s="26" t="n">
@@ -12906,7 +12912,7 @@
         <v>9.48086635586635</v>
       </c>
       <c r="X13" s="35" t="n">
-        <f aca="false">IF(E13="Slot",ROUNDUP(W13/G13,0)*F13,W13*H13)</f>
+        <f aca="false">IF(E13="Slot",IF(N(G13)&gt;0,ROUNDUP(W13/G13,0)*F13,0),W13*H13)</f>
         <v>1449</v>
       </c>
       <c r="Y13" s="35" t="n">
@@ -12926,7 +12932,7 @@
         <v>1583.36321262101</v>
       </c>
       <c r="AC13" s="23" t="n">
-        <f aca="false">COUNTIF($Q$5:$Q$34,"&lt;"&amp;Q13)+1</f>
+        <f aca="false">SUMPRODUCT(--($Q$5:$Q$34&lt;Q13))+1</f>
         <v>24</v>
       </c>
       <c r="AD13" s="2" t="str">
@@ -12983,7 +12989,7 @@
         <v>25</v>
       </c>
       <c r="H14" s="37" t="n">
-        <f aca="false">IF(E14="CPC",F14/G14,IF(E14="Slot",F14/G14,F14))</f>
+        <f aca="false">IF(OR(E14="CPC",E14="Slot"),IF(N(G14)&gt;0,F14/G14,0),F14)</f>
         <v>57.96</v>
       </c>
       <c r="I14" s="24" t="n">
@@ -12991,7 +12997,7 @@
         <v>0.35</v>
       </c>
       <c r="J14" s="23" t="n">
-        <f aca="false">IF(E14="Slot",Assumptions!H121*G14,Assumptions!H121)</f>
+        <f aca="false">IF(AND(OR(E14="CPC",E14="Slot"),NOT(N(G14)&gt;0)),0,IF(E14="Slot",Assumptions!H121*G14,Assumptions!H121))</f>
         <v>75</v>
       </c>
       <c r="K14" s="26" t="n">
@@ -13023,11 +13029,11 @@
         <v>408.888902888889</v>
       </c>
       <c r="R14" s="23" t="n">
-        <f aca="false">COUNTIFS($C$5:$C$34,C14,$Q$5:$Q$34,"&lt;"&amp;Q14)+1</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C14)*($Q$5:$Q$34&lt;Q14))+1</f>
         <v>7</v>
       </c>
       <c r="S14" s="26" t="n">
-        <f aca="false">SUMIFS($AH$5:$AH$34,$C$5:$C$34,C14,$Q$5:$Q$34,"&lt;"&amp;Q14)</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C14)*($Q$5:$Q$34&lt;Q14)*$AH$5:$AH$34)</f>
         <v>120.610431818182</v>
       </c>
       <c r="T14" s="26" t="n">
@@ -13047,7 +13053,7 @@
         <v>0</v>
       </c>
       <c r="X14" s="35" t="n">
-        <f aca="false">IF(E14="Slot",ROUNDUP(W14/G14,0)*F14,W14*H14)</f>
+        <f aca="false">IF(E14="Slot",IF(N(G14)&gt;0,ROUNDUP(W14/G14,0)*F14,0),W14*H14)</f>
         <v>0</v>
       </c>
       <c r="Y14" s="35" t="n">
@@ -13067,7 +13073,7 @@
         <v>–</v>
       </c>
       <c r="AC14" s="23" t="n">
-        <f aca="false">COUNTIF($Q$5:$Q$34,"&lt;"&amp;Q14)+1</f>
+        <f aca="false">SUMPRODUCT(--($Q$5:$Q$34&lt;Q14))+1</f>
         <v>13</v>
       </c>
       <c r="AD14" s="2" t="str">
@@ -13124,7 +13130,7 @@
         <v>15</v>
       </c>
       <c r="H15" s="37" t="n">
-        <f aca="false">IF(E15="CPC",F15/G15,IF(E15="Slot",F15/G15,F15))</f>
+        <f aca="false">IF(OR(E15="CPC",E15="Slot"),IF(N(G15)&gt;0,F15/G15,0),F15)</f>
         <v>96.6</v>
       </c>
       <c r="I15" s="24" t="n">
@@ -13132,7 +13138,7 @@
         <v>0.25</v>
       </c>
       <c r="J15" s="23" t="n">
-        <f aca="false">IF(E15="Slot",Assumptions!H122*G15,Assumptions!H122)</f>
+        <f aca="false">IF(AND(OR(E15="CPC",E15="Slot"),NOT(N(G15)&gt;0)),0,IF(E15="Slot",Assumptions!H122*G15,Assumptions!H122))</f>
         <v>30</v>
       </c>
       <c r="K15" s="26" t="n">
@@ -13164,11 +13170,11 @@
         <v>1321.02565602564</v>
       </c>
       <c r="R15" s="23" t="n">
-        <f aca="false">COUNTIFS($C$5:$C$34,C15,$Q$5:$Q$34,"&lt;"&amp;Q15)+1</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C15)*($Q$5:$Q$34&lt;Q15))+1</f>
         <v>7</v>
       </c>
       <c r="S15" s="26" t="n">
-        <f aca="false">SUMIFS($AH$5:$AH$34,$C$5:$C$34,C15,$Q$5:$Q$34,"&lt;"&amp;Q15)</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C15)*($Q$5:$Q$34&lt;Q15)*$AH$5:$AH$34)</f>
         <v>24.888749025974</v>
       </c>
       <c r="T15" s="26" t="n">
@@ -13188,7 +13194,7 @@
         <v>0</v>
       </c>
       <c r="X15" s="35" t="n">
-        <f aca="false">IF(E15="Slot",ROUNDUP(W15/G15,0)*F15,W15*H15)</f>
+        <f aca="false">IF(E15="Slot",IF(N(G15)&gt;0,ROUNDUP(W15/G15,0)*F15,0),W15*H15)</f>
         <v>0</v>
       </c>
       <c r="Y15" s="35" t="n">
@@ -13208,7 +13214,7 @@
         <v>–</v>
       </c>
       <c r="AC15" s="23" t="n">
-        <f aca="false">COUNTIF($Q$5:$Q$34,"&lt;"&amp;Q15)+1</f>
+        <f aca="false">SUMPRODUCT(--($Q$5:$Q$34&lt;Q15))+1</f>
         <v>27</v>
       </c>
       <c r="AD15" s="2" t="str">
@@ -13265,7 +13271,7 @@
         <v>15</v>
       </c>
       <c r="H16" s="37" t="n">
-        <f aca="false">IF(E16="CPC",F16/G16,IF(E16="Slot",F16/G16,F16))</f>
+        <f aca="false">IF(OR(E16="CPC",E16="Slot"),IF(N(G16)&gt;0,F16/G16,0),F16)</f>
         <v>96.6</v>
       </c>
       <c r="I16" s="24" t="n">
@@ -13273,7 +13279,7 @@
         <v>0.25</v>
       </c>
       <c r="J16" s="23" t="n">
-        <f aca="false">IF(E16="Slot",Assumptions!H123*G16,Assumptions!H123)</f>
+        <f aca="false">IF(AND(OR(E16="CPC",E16="Slot"),NOT(N(G16)&gt;0)),0,IF(E16="Slot",Assumptions!H123*G16,Assumptions!H123))</f>
         <v>30</v>
       </c>
       <c r="K16" s="26" t="n">
@@ -13305,11 +13311,11 @@
         <v>1443.13727090196</v>
       </c>
       <c r="R16" s="23" t="n">
-        <f aca="false">COUNTIFS($C$5:$C$34,C16,$Q$5:$Q$34,"&lt;"&amp;Q16)+1</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C16)*($Q$5:$Q$34&lt;Q16))+1</f>
         <v>6</v>
       </c>
       <c r="S16" s="26" t="n">
-        <f aca="false">SUMIFS($AH$5:$AH$34,$C$5:$C$34,C16,$Q$5:$Q$34,"&lt;"&amp;Q16)</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C16)*($Q$5:$Q$34&lt;Q16)*$AH$5:$AH$34)</f>
         <v>8.50582636363636</v>
       </c>
       <c r="T16" s="26" t="n">
@@ -13329,7 +13335,7 @@
         <v>0</v>
       </c>
       <c r="X16" s="35" t="n">
-        <f aca="false">IF(E16="Slot",ROUNDUP(W16/G16,0)*F16,W16*H16)</f>
+        <f aca="false">IF(E16="Slot",IF(N(G16)&gt;0,ROUNDUP(W16/G16,0)*F16,0),W16*H16)</f>
         <v>0</v>
       </c>
       <c r="Y16" s="35" t="n">
@@ -13349,7 +13355,7 @@
         <v>–</v>
       </c>
       <c r="AC16" s="23" t="n">
-        <f aca="false">COUNTIF($Q$5:$Q$34,"&lt;"&amp;Q16)+1</f>
+        <f aca="false">SUMPRODUCT(--($Q$5:$Q$34&lt;Q16))+1</f>
         <v>28</v>
       </c>
       <c r="AD16" s="2" t="str">
@@ -13406,7 +13412,7 @@
         <v>0.08</v>
       </c>
       <c r="H17" s="37" t="n">
-        <f aca="false">IF(E17="CPC",F17/G17,IF(E17="Slot",F17/G17,F17))</f>
+        <f aca="false">IF(OR(E17="CPC",E17="Slot"),IF(N(G17)&gt;0,F17/G17,0),F17)</f>
         <v>43.75</v>
       </c>
       <c r="I17" s="24" t="n">
@@ -13414,7 +13420,7 @@
         <v>0.25</v>
       </c>
       <c r="J17" s="23" t="n">
-        <f aca="false">IF(E17="Slot",Assumptions!H124*G17,Assumptions!H124)</f>
+        <f aca="false">IF(AND(OR(E17="CPC",E17="Slot"),NOT(N(G17)&gt;0)),0,IF(E17="Slot",Assumptions!H124*G17,Assumptions!H124))</f>
         <v>150</v>
       </c>
       <c r="K17" s="26" t="n">
@@ -13446,11 +13452,11 @@
         <v>598.290615290598</v>
       </c>
       <c r="R17" s="23" t="n">
-        <f aca="false">COUNTIFS($C$5:$C$34,C17,$Q$5:$Q$34,"&lt;"&amp;Q17)+1</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C17)*($Q$5:$Q$34&lt;Q17))+1</f>
         <v>3</v>
       </c>
       <c r="S17" s="26" t="n">
-        <f aca="false">SUMIFS($AH$5:$AH$34,$C$5:$C$34,C17,$Q$5:$Q$34,"&lt;"&amp;Q17)</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C17)*($Q$5:$Q$34&lt;Q17)*$AH$5:$AH$34)</f>
         <v>4.7619</v>
       </c>
       <c r="T17" s="26" t="n">
@@ -13470,7 +13476,7 @@
         <v>117.690023310023</v>
       </c>
       <c r="X17" s="35" t="n">
-        <f aca="false">IF(E17="Slot",ROUNDUP(W17/G17,0)*F17,W17*H17)</f>
+        <f aca="false">IF(E17="Slot",IF(N(G17)&gt;0,ROUNDUP(W17/G17,0)*F17,0),W17*H17)</f>
         <v>5148.93851981352</v>
       </c>
       <c r="Y17" s="35" t="n">
@@ -13490,7 +13496,7 @@
         <v>598.290598290598</v>
       </c>
       <c r="AC17" s="23" t="n">
-        <f aca="false">COUNTIF($Q$5:$Q$34,"&lt;"&amp;Q17)+1</f>
+        <f aca="false">SUMPRODUCT(--($Q$5:$Q$34&lt;Q17))+1</f>
         <v>14</v>
       </c>
       <c r="AD17" s="2" t="str">
@@ -13547,7 +13553,7 @@
         <v>0.08</v>
       </c>
       <c r="H18" s="37" t="n">
-        <f aca="false">IF(E18="CPC",F18/G18,IF(E18="Slot",F18/G18,F18))</f>
+        <f aca="false">IF(OR(E18="CPC",E18="Slot"),IF(N(G18)&gt;0,F18/G18,0),F18)</f>
         <v>43.75</v>
       </c>
       <c r="I18" s="24" t="n">
@@ -13555,7 +13561,7 @@
         <v>0.2</v>
       </c>
       <c r="J18" s="23" t="n">
-        <f aca="false">IF(E18="Slot",Assumptions!H125*G18,Assumptions!H125)</f>
+        <f aca="false">IF(AND(OR(E18="CPC",E18="Slot"),NOT(N(G18)&gt;0)),0,IF(E18="Slot",Assumptions!H125*G18,Assumptions!H125))</f>
         <v>100</v>
       </c>
       <c r="K18" s="26" t="n">
@@ -13587,11 +13593,11 @@
         <v>816.993482052288</v>
       </c>
       <c r="R18" s="23" t="n">
-        <f aca="false">COUNTIFS($C$5:$C$34,C18,$Q$5:$Q$34,"&lt;"&amp;Q18)+1</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C18)*($Q$5:$Q$34&lt;Q18))+1</f>
         <v>3</v>
       </c>
       <c r="S18" s="26" t="n">
-        <f aca="false">SUMIFS($AH$5:$AH$34,$C$5:$C$34,C18,$Q$5:$Q$34,"&lt;"&amp;Q18)</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C18)*($Q$5:$Q$34&lt;Q18)*$AH$5:$AH$34)</f>
         <v>2.76318</v>
       </c>
       <c r="T18" s="26" t="n">
@@ -13611,7 +13617,7 @@
         <v>100</v>
       </c>
       <c r="X18" s="35" t="n">
-        <f aca="false">IF(E18="Slot",ROUNDUP(W18/G18,0)*F18,W18*H18)</f>
+        <f aca="false">IF(E18="Slot",IF(N(G18)&gt;0,ROUNDUP(W18/G18,0)*F18,0),W18*H18)</f>
         <v>4375</v>
       </c>
       <c r="Y18" s="35" t="n">
@@ -13631,7 +13637,7 @@
         <v>816.993464052288</v>
       </c>
       <c r="AC18" s="23" t="n">
-        <f aca="false">COUNTIF($Q$5:$Q$34,"&lt;"&amp;Q18)+1</f>
+        <f aca="false">SUMPRODUCT(--($Q$5:$Q$34&lt;Q18))+1</f>
         <v>17</v>
       </c>
       <c r="AD18" s="2" t="str">
@@ -13688,7 +13694,7 @@
         <v>0</v>
       </c>
       <c r="H19" s="37" t="n">
-        <f aca="false">IF(E19="CPC",F19/G19,IF(E19="Slot",F19/G19,F19))</f>
+        <f aca="false">IF(OR(E19="CPC",E19="Slot"),IF(N(G19)&gt;0,F19/G19,0),F19)</f>
         <v>18</v>
       </c>
       <c r="I19" s="24" t="n">
@@ -13696,7 +13702,7 @@
         <v>0.05</v>
       </c>
       <c r="J19" s="23" t="n">
-        <f aca="false">IF(E19="Slot",Assumptions!H126*G19,Assumptions!H126)</f>
+        <f aca="false">IF(AND(OR(E19="CPC",E19="Slot"),NOT(N(G19)&gt;0)),0,IF(E19="Slot",Assumptions!H126*G19,Assumptions!H126))</f>
         <v>400</v>
       </c>
       <c r="K19" s="26" t="n">
@@ -13728,11 +13734,11 @@
         <v>1118.88113788112</v>
       </c>
       <c r="R19" s="23" t="n">
-        <f aca="false">COUNTIFS($C$5:$C$34,C19,$Q$5:$Q$34,"&lt;"&amp;Q19)+1</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C19)*($Q$5:$Q$34&lt;Q19))+1</f>
         <v>7</v>
       </c>
       <c r="S19" s="26" t="n">
-        <f aca="false">SUMIFS($AH$5:$AH$34,$C$5:$C$34,C19,$Q$5:$Q$34,"&lt;"&amp;Q19)</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C19)*($Q$5:$Q$34&lt;Q19)*$AH$5:$AH$34)</f>
         <v>31.099696875</v>
       </c>
       <c r="T19" s="26" t="n">
@@ -13752,7 +13758,7 @@
         <v>41.6666666666667</v>
       </c>
       <c r="X19" s="35" t="n">
-        <f aca="false">IF(E19="Slot",ROUNDUP(W19/G19,0)*F19,W19*H19)</f>
+        <f aca="false">IF(E19="Slot",IF(N(G19)&gt;0,ROUNDUP(W19/G19,0)*F19,0),W19*H19)</f>
         <v>750</v>
       </c>
       <c r="Y19" s="35" t="n">
@@ -13772,7 +13778,7 @@
         <v>1118.88111888112</v>
       </c>
       <c r="AC19" s="23" t="n">
-        <f aca="false">COUNTIF($Q$5:$Q$34,"&lt;"&amp;Q19)+1</f>
+        <f aca="false">SUMPRODUCT(--($Q$5:$Q$34&lt;Q19))+1</f>
         <v>25</v>
       </c>
       <c r="AD19" s="2" t="str">
@@ -13829,7 +13835,7 @@
         <v>0</v>
       </c>
       <c r="H20" s="37" t="n">
-        <f aca="false">IF(E20="CPC",F20/G20,IF(E20="Slot",F20/G20,F20))</f>
+        <f aca="false">IF(OR(E20="CPC",E20="Slot"),IF(N(G20)&gt;0,F20/G20,0),F20)</f>
         <v>12</v>
       </c>
       <c r="I20" s="24" t="n">
@@ -13837,7 +13843,7 @@
         <v>0.12</v>
       </c>
       <c r="J20" s="23" t="n">
-        <f aca="false">IF(E20="Slot",Assumptions!H127*G20,Assumptions!H127)</f>
+        <f aca="false">IF(AND(OR(E20="CPC",E20="Slot"),NOT(N(G20)&gt;0)),0,IF(E20="Slot",Assumptions!H127*G20,Assumptions!H127))</f>
         <v>500</v>
       </c>
       <c r="K20" s="26" t="n">
@@ -13869,11 +13875,11 @@
         <v>246.913600246914</v>
       </c>
       <c r="R20" s="23" t="n">
-        <f aca="false">COUNTIFS($C$5:$C$34,C20,$Q$5:$Q$34,"&lt;"&amp;Q20)+1</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C20)*($Q$5:$Q$34&lt;Q20))+1</f>
         <v>4</v>
       </c>
       <c r="S20" s="26" t="n">
-        <f aca="false">SUMIFS($AH$5:$AH$34,$C$5:$C$34,C20,$Q$5:$Q$34,"&lt;"&amp;Q20)</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C20)*($Q$5:$Q$34&lt;Q20)*$AH$5:$AH$34)</f>
         <v>40.9635</v>
       </c>
       <c r="T20" s="26" t="n">
@@ -13893,7 +13899,7 @@
         <v>62.5</v>
       </c>
       <c r="X20" s="35" t="n">
-        <f aca="false">IF(E20="Slot",ROUNDUP(W20/G20,0)*F20,W20*H20)</f>
+        <f aca="false">IF(E20="Slot",IF(N(G20)&gt;0,ROUNDUP(W20/G20,0)*F20,0),W20*H20)</f>
         <v>750</v>
       </c>
       <c r="Y20" s="35" t="n">
@@ -13913,7 +13919,7 @@
         <v>246.913580246914</v>
       </c>
       <c r="AC20" s="23" t="n">
-        <f aca="false">COUNTIF($Q$5:$Q$34,"&lt;"&amp;Q20)+1</f>
+        <f aca="false">SUMPRODUCT(--($Q$5:$Q$34&lt;Q20))+1</f>
         <v>10</v>
       </c>
       <c r="AD20" s="2" t="str">
@@ -13970,7 +13976,7 @@
         <v>0.07</v>
       </c>
       <c r="H21" s="37" t="n">
-        <f aca="false">IF(E21="CPC",F21/G21,IF(E21="Slot",F21/G21,F21))</f>
+        <f aca="false">IF(OR(E21="CPC",E21="Slot"),IF(N(G21)&gt;0,F21/G21,0),F21)</f>
         <v>31.4285714285714</v>
       </c>
       <c r="I21" s="24" t="n">
@@ -13978,7 +13984,7 @@
         <v>0.15</v>
       </c>
       <c r="J21" s="23" t="n">
-        <f aca="false">IF(E21="Slot",Assumptions!H128*G21,Assumptions!H128)</f>
+        <f aca="false">IF(AND(OR(E21="CPC",E21="Slot"),NOT(N(G21)&gt;0)),0,IF(E21="Slot",Assumptions!H128*G21,Assumptions!H128))</f>
         <v>80</v>
       </c>
       <c r="K21" s="26" t="n">
@@ -14010,11 +14016,11 @@
         <v>651.200672200651</v>
       </c>
       <c r="R21" s="23" t="n">
-        <f aca="false">COUNTIFS($C$5:$C$34,C21,$Q$5:$Q$34,"&lt;"&amp;Q21)+1</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C21)*($Q$5:$Q$34&lt;Q21))+1</f>
         <v>3</v>
       </c>
       <c r="S21" s="26" t="n">
-        <f aca="false">SUMIFS($AH$5:$AH$34,$C$5:$C$34,C21,$Q$5:$Q$34,"&lt;"&amp;Q21)</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C21)*($Q$5:$Q$34&lt;Q21)*$AH$5:$AH$34)</f>
         <v>8.30115</v>
       </c>
       <c r="T21" s="26" t="n">
@@ -14034,7 +14040,7 @@
         <v>80</v>
       </c>
       <c r="X21" s="35" t="n">
-        <f aca="false">IF(E21="Slot",ROUNDUP(W21/G21,0)*F21,W21*H21)</f>
+        <f aca="false">IF(E21="Slot",IF(N(G21)&gt;0,ROUNDUP(W21/G21,0)*F21,0),W21*H21)</f>
         <v>2514.28571428571</v>
       </c>
       <c r="Y21" s="35" t="n">
@@ -14054,7 +14060,7 @@
         <v>651.200651200651</v>
       </c>
       <c r="AC21" s="23" t="n">
-        <f aca="false">COUNTIF($Q$5:$Q$34,"&lt;"&amp;Q21)+1</f>
+        <f aca="false">SUMPRODUCT(--($Q$5:$Q$34&lt;Q21))+1</f>
         <v>15</v>
       </c>
       <c r="AD21" s="2" t="str">
@@ -14111,7 +14117,7 @@
         <v>0.07</v>
       </c>
       <c r="H22" s="37" t="n">
-        <f aca="false">IF(E22="CPC",F22/G22,IF(E22="Slot",F22/G22,F22))</f>
+        <f aca="false">IF(OR(E22="CPC",E22="Slot"),IF(N(G22)&gt;0,F22/G22,0),F22)</f>
         <v>31.4285714285714</v>
       </c>
       <c r="I22" s="24" t="n">
@@ -14119,7 +14125,7 @@
         <v>0.25</v>
       </c>
       <c r="J22" s="23" t="n">
-        <f aca="false">IF(E22="Slot",Assumptions!H129*G22,Assumptions!H129)</f>
+        <f aca="false">IF(AND(OR(E22="CPC",E22="Slot"),NOT(N(G22)&gt;0)),0,IF(E22="Slot",Assumptions!H129*G22,Assumptions!H129))</f>
         <v>100</v>
       </c>
       <c r="K22" s="26" t="n">
@@ -14151,11 +14157,11 @@
         <v>310.405665738977</v>
       </c>
       <c r="R22" s="23" t="n">
-        <f aca="false">COUNTIFS($C$5:$C$34,C22,$Q$5:$Q$34,"&lt;"&amp;Q22)+1</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C22)*($Q$5:$Q$34&lt;Q22))+1</f>
         <v>6</v>
       </c>
       <c r="S22" s="26" t="n">
-        <f aca="false">SUMIFS($AH$5:$AH$34,$C$5:$C$34,C22,$Q$5:$Q$34,"&lt;"&amp;Q22)</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C22)*($Q$5:$Q$34&lt;Q22)*$AH$5:$AH$34)</f>
         <v>112.901625</v>
       </c>
       <c r="T22" s="26" t="n">
@@ -14175,7 +14181,7 @@
         <v>23.8636363636364</v>
       </c>
       <c r="X22" s="35" t="n">
-        <f aca="false">IF(E22="Slot",ROUNDUP(W22/G22,0)*F22,W22*H22)</f>
+        <f aca="false">IF(E22="Slot",IF(N(G22)&gt;0,ROUNDUP(W22/G22,0)*F22,0),W22*H22)</f>
         <v>750</v>
       </c>
       <c r="Y22" s="35" t="n">
@@ -14195,7 +14201,7 @@
         <v>310.405643738977</v>
       </c>
       <c r="AC22" s="23" t="n">
-        <f aca="false">COUNTIF($Q$5:$Q$34,"&lt;"&amp;Q22)+1</f>
+        <f aca="false">SUMPRODUCT(--($Q$5:$Q$34&lt;Q22))+1</f>
         <v>12</v>
       </c>
       <c r="AD22" s="2" t="str">
@@ -14252,7 +14258,7 @@
         <v>0.07</v>
       </c>
       <c r="H23" s="37" t="n">
-        <f aca="false">IF(E23="CPC",F23/G23,IF(E23="Slot",F23/G23,F23))</f>
+        <f aca="false">IF(OR(E23="CPC",E23="Slot"),IF(N(G23)&gt;0,F23/G23,0),F23)</f>
         <v>31.4285714285714</v>
       </c>
       <c r="I23" s="24" t="n">
@@ -14260,7 +14266,7 @@
         <v>0.15</v>
       </c>
       <c r="J23" s="23" t="n">
-        <f aca="false">IF(E23="Slot",Assumptions!H130*G23,Assumptions!H130)</f>
+        <f aca="false">IF(AND(OR(E23="CPC",E23="Slot"),NOT(N(G23)&gt;0)),0,IF(E23="Slot",Assumptions!H130*G23,Assumptions!H130))</f>
         <v>40</v>
       </c>
       <c r="K23" s="26" t="n">
@@ -14292,11 +14298,11 @@
         <v>716.320739320716</v>
       </c>
       <c r="R23" s="23" t="n">
-        <f aca="false">COUNTIFS($C$5:$C$34,C23,$Q$5:$Q$34,"&lt;"&amp;Q23)+1</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C23)*($Q$5:$Q$34&lt;Q23))+1</f>
         <v>4</v>
       </c>
       <c r="S23" s="26" t="n">
-        <f aca="false">SUMIFS($AH$5:$AH$34,$C$5:$C$34,C23,$Q$5:$Q$34,"&lt;"&amp;Q23)</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C23)*($Q$5:$Q$34&lt;Q23)*$AH$5:$AH$34)</f>
         <v>14.4770785714286</v>
       </c>
       <c r="T23" s="26" t="n">
@@ -14316,7 +14322,7 @@
         <v>23.8636363636364</v>
       </c>
       <c r="X23" s="35" t="n">
-        <f aca="false">IF(E23="Slot",ROUNDUP(W23/G23,0)*F23,W23*H23)</f>
+        <f aca="false">IF(E23="Slot",IF(N(G23)&gt;0,ROUNDUP(W23/G23,0)*F23,0),W23*H23)</f>
         <v>750</v>
       </c>
       <c r="Y23" s="35" t="n">
@@ -14336,7 +14342,7 @@
         <v>716.320716320716</v>
       </c>
       <c r="AC23" s="23" t="n">
-        <f aca="false">COUNTIF($Q$5:$Q$34,"&lt;"&amp;Q23)+1</f>
+        <f aca="false">SUMPRODUCT(--($Q$5:$Q$34&lt;Q23))+1</f>
         <v>16</v>
       </c>
       <c r="AD23" s="2" t="str">
@@ -14393,7 +14399,7 @@
         <v>0.07</v>
       </c>
       <c r="H24" s="37" t="n">
-        <f aca="false">IF(E24="CPC",F24/G24,IF(E24="Slot",F24/G24,F24))</f>
+        <f aca="false">IF(OR(E24="CPC",E24="Slot"),IF(N(G24)&gt;0,F24/G24,0),F24)</f>
         <v>31.4285714285714</v>
       </c>
       <c r="I24" s="24" t="n">
@@ -14401,7 +14407,7 @@
         <v>0.12</v>
       </c>
       <c r="J24" s="23" t="n">
-        <f aca="false">IF(E24="Slot",Assumptions!H131*G24,Assumptions!H131)</f>
+        <f aca="false">IF(AND(OR(E24="CPC",E24="Slot"),NOT(N(G24)&gt;0)),0,IF(E24="Slot",Assumptions!H131*G24,Assumptions!H131))</f>
         <v>30</v>
       </c>
       <c r="K24" s="26" t="n">
@@ -14433,11 +14439,11 @@
         <v>978.169069395936</v>
       </c>
       <c r="R24" s="23" t="n">
-        <f aca="false">COUNTIFS($C$5:$C$34,C24,$Q$5:$Q$34,"&lt;"&amp;Q24)+1</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C24)*($Q$5:$Q$34&lt;Q24))+1</f>
         <v>4</v>
       </c>
       <c r="S24" s="26" t="n">
-        <f aca="false">SUMIFS($AH$5:$AH$34,$C$5:$C$34,C24,$Q$5:$Q$34,"&lt;"&amp;Q24)</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C24)*($Q$5:$Q$34&lt;Q24)*$AH$5:$AH$34)</f>
         <v>7.20018</v>
       </c>
       <c r="T24" s="26" t="n">
@@ -14457,7 +14463,7 @@
         <v>30</v>
       </c>
       <c r="X24" s="35" t="n">
-        <f aca="false">IF(E24="Slot",ROUNDUP(W24/G24,0)*F24,W24*H24)</f>
+        <f aca="false">IF(E24="Slot",IF(N(G24)&gt;0,ROUNDUP(W24/G24,0)*F24,0),W24*H24)</f>
         <v>942.857142857143</v>
       </c>
       <c r="Y24" s="35" t="n">
@@ -14477,7 +14483,7 @@
         <v>978.169045395936</v>
       </c>
       <c r="AC24" s="23" t="n">
-        <f aca="false">COUNTIF($Q$5:$Q$34,"&lt;"&amp;Q24)+1</f>
+        <f aca="false">SUMPRODUCT(--($Q$5:$Q$34&lt;Q24))+1</f>
         <v>19</v>
       </c>
       <c r="AD24" s="2" t="str">
@@ -14567,11 +14573,11 @@
         <v>22.5217866521964</v>
       </c>
       <c r="R25" s="23" t="n">
-        <f aca="false">COUNTIFS($C$5:$C$34,C25,$Q$5:$Q$34,"&lt;"&amp;Q25)+1</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C25)*($Q$5:$Q$34&lt;Q25))+1</f>
         <v>2</v>
       </c>
       <c r="S25" s="26" t="n">
-        <f aca="false">SUMIFS($AH$5:$AH$34,$C$5:$C$34,C25,$Q$5:$Q$34,"&lt;"&amp;Q25)</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C25)*($Q$5:$Q$34&lt;Q25)*$AH$5:$AH$34)</f>
         <v>3.861</v>
       </c>
       <c r="T25" s="26" t="n">
@@ -14591,7 +14597,7 @@
         <v>24</v>
       </c>
       <c r="X25" s="35" t="n">
-        <f aca="false">IF(E25="Slot",ROUNDUP(W25/G25,0)*F25,W25*H25)</f>
+        <f aca="false">IF(E25="Slot",IF(N(G25)&gt;0,ROUNDUP(W25/G25,0)*F25,0),W25*H25)</f>
         <v>100</v>
       </c>
       <c r="Y25" s="35" t="n">
@@ -14611,7 +14617,7 @@
         <v>22.5217616521964</v>
       </c>
       <c r="AC25" s="23" t="n">
-        <f aca="false">COUNTIF($Q$5:$Q$34,"&lt;"&amp;Q25)+1</f>
+        <f aca="false">SUMPRODUCT(--($Q$5:$Q$34&lt;Q25))+1</f>
         <v>6</v>
       </c>
       <c r="AD25" s="2" t="str">
@@ -14701,11 +14707,11 @@
         <v>17.8923144236894</v>
       </c>
       <c r="R26" s="23" t="n">
-        <f aca="false">COUNTIFS($C$5:$C$34,C26,$Q$5:$Q$34,"&lt;"&amp;Q26)+1</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C26)*($Q$5:$Q$34&lt;Q26))+1</f>
         <v>2</v>
       </c>
       <c r="S26" s="26" t="n">
-        <f aca="false">SUMIFS($AH$5:$AH$34,$C$5:$C$34,C26,$Q$5:$Q$34,"&lt;"&amp;Q26)</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C26)*($Q$5:$Q$34&lt;Q26)*$AH$5:$AH$34)</f>
         <v>14.58</v>
       </c>
       <c r="T26" s="26" t="n">
@@ -14725,7 +14731,7 @@
         <v>36</v>
       </c>
       <c r="X26" s="35" t="n">
-        <f aca="false">IF(E26="Slot",ROUNDUP(W26/G26,0)*F26,W26*H26)</f>
+        <f aca="false">IF(E26="Slot",IF(N(G26)&gt;0,ROUNDUP(W26/G26,0)*F26,0),W26*H26)</f>
         <v>150</v>
       </c>
       <c r="Y26" s="35" t="n">
@@ -14745,7 +14751,7 @@
         <v>17.8922884236894</v>
       </c>
       <c r="AC26" s="23" t="n">
-        <f aca="false">COUNTIF($Q$5:$Q$34,"&lt;"&amp;Q26)+1</f>
+        <f aca="false">SUMPRODUCT(--($Q$5:$Q$34&lt;Q26))+1</f>
         <v>5</v>
       </c>
       <c r="AD26" s="2" t="str">
@@ -14835,11 +14841,11 @@
         <v>24.7739648174161</v>
       </c>
       <c r="R27" s="23" t="n">
-        <f aca="false">COUNTIFS($C$5:$C$34,C27,$Q$5:$Q$34,"&lt;"&amp;Q27)+1</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C27)*($Q$5:$Q$34&lt;Q27))+1</f>
         <v>2</v>
       </c>
       <c r="S27" s="26" t="n">
-        <f aca="false">SUMIFS($AH$5:$AH$34,$C$5:$C$34,C27,$Q$5:$Q$34,"&lt;"&amp;Q27)</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C27)*($Q$5:$Q$34&lt;Q27)*$AH$5:$AH$34)</f>
         <v>2.34</v>
       </c>
       <c r="T27" s="26" t="n">
@@ -14859,7 +14865,7 @@
         <v>14.4</v>
       </c>
       <c r="X27" s="35" t="n">
-        <f aca="false">IF(E27="Slot",ROUNDUP(W27/G27,0)*F27,W27*H27)</f>
+        <f aca="false">IF(E27="Slot",IF(N(G27)&gt;0,ROUNDUP(W27/G27,0)*F27,0),W27*H27)</f>
         <v>60</v>
       </c>
       <c r="Y27" s="35" t="n">
@@ -14879,7 +14885,7 @@
         <v>24.7739378174161</v>
       </c>
       <c r="AC27" s="23" t="n">
-        <f aca="false">COUNTIF($Q$5:$Q$34,"&lt;"&amp;Q27)+1</f>
+        <f aca="false">SUMPRODUCT(--($Q$5:$Q$34&lt;Q27))+1</f>
         <v>7</v>
       </c>
       <c r="AD27" s="2" t="str">
@@ -14969,11 +14975,11 @@
         <v>27.0639936828915</v>
       </c>
       <c r="R28" s="23" t="n">
-        <f aca="false">COUNTIFS($C$5:$C$34,C28,$Q$5:$Q$34,"&lt;"&amp;Q28)+1</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C28)*($Q$5:$Q$34&lt;Q28))+1</f>
         <v>2</v>
       </c>
       <c r="S28" s="26" t="n">
-        <f aca="false">SUMIFS($AH$5:$AH$34,$C$5:$C$34,C28,$Q$5:$Q$34,"&lt;"&amp;Q28)</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C28)*($Q$5:$Q$34&lt;Q28)*$AH$5:$AH$34)</f>
         <v>1.2852</v>
       </c>
       <c r="T28" s="26" t="n">
@@ -14993,7 +14999,7 @@
         <v>9.6</v>
       </c>
       <c r="X28" s="35" t="n">
-        <f aca="false">IF(E28="Slot",ROUNDUP(W28/G28,0)*F28,W28*H28)</f>
+        <f aca="false">IF(E28="Slot",IF(N(G28)&gt;0,ROUNDUP(W28/G28,0)*F28,0),W28*H28)</f>
         <v>40</v>
       </c>
       <c r="Y28" s="35" t="n">
@@ -15013,7 +15019,7 @@
         <v>27.0639656828915</v>
       </c>
       <c r="AC28" s="23" t="n">
-        <f aca="false">COUNTIF($Q$5:$Q$34,"&lt;"&amp;Q28)+1</f>
+        <f aca="false">SUMPRODUCT(--($Q$5:$Q$34&lt;Q28))+1</f>
         <v>8</v>
       </c>
       <c r="AD28" s="2" t="str">
@@ -15103,11 +15109,11 @@
         <v>1000.000029</v>
       </c>
       <c r="R29" s="23" t="n">
-        <f aca="false">COUNTIFS($C$5:$C$34,C29,$Q$5:$Q$34,"&lt;"&amp;Q29)+1</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C29)*($Q$5:$Q$34&lt;Q29))+1</f>
         <v>5</v>
       </c>
       <c r="S29" s="26" t="n">
-        <f aca="false">SUMIFS($AH$5:$AH$34,$C$5:$C$34,C29,$Q$5:$Q$34,"&lt;"&amp;Q29)</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C29)*($Q$5:$Q$34&lt;Q29)*$AH$5:$AH$34)</f>
         <v>22.59343125</v>
       </c>
       <c r="T29" s="26" t="n">
@@ -15127,7 +15133,7 @@
         <v>25</v>
       </c>
       <c r="X29" s="35" t="n">
-        <f aca="false">IF(E29="Slot",ROUNDUP(W29/G29,0)*F29,W29*H29)</f>
+        <f aca="false">IF(E29="Slot",IF(N(G29)&gt;0,ROUNDUP(W29/G29,0)*F29,0),W29*H29)</f>
         <v>4162.640625</v>
       </c>
       <c r="Y29" s="35" t="n">
@@ -15147,7 +15153,7 @@
         <v>1000</v>
       </c>
       <c r="AC29" s="23" t="n">
-        <f aca="false">COUNTIF($Q$5:$Q$34,"&lt;"&amp;Q29)+1</f>
+        <f aca="false">SUMPRODUCT(--($Q$5:$Q$34&lt;Q29))+1</f>
         <v>20</v>
       </c>
       <c r="AD29" s="2" t="str">
@@ -15237,11 +15243,11 @@
         <v>1000.00003</v>
       </c>
       <c r="R30" s="23" t="n">
-        <f aca="false">COUNTIFS($C$5:$C$34,C30,$Q$5:$Q$34,"&lt;"&amp;Q30)+1</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C30)*($Q$5:$Q$34&lt;Q30))+1</f>
         <v>8</v>
       </c>
       <c r="S30" s="26" t="n">
-        <f aca="false">SUMIFS($AH$5:$AH$34,$C$5:$C$34,C30,$Q$5:$Q$34,"&lt;"&amp;Q30)</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C30)*($Q$5:$Q$34&lt;Q30)*$AH$5:$AH$34)</f>
         <v>131.241681818182</v>
       </c>
       <c r="T30" s="26" t="n">
@@ -15261,7 +15267,7 @@
         <v>0</v>
       </c>
       <c r="X30" s="35" t="n">
-        <f aca="false">IF(E30="Slot",ROUNDUP(W30/G30,0)*F30,W30*H30)</f>
+        <f aca="false">IF(E30="Slot",IF(N(G30)&gt;0,ROUNDUP(W30/G30,0)*F30,0),W30*H30)</f>
         <v>0</v>
       </c>
       <c r="Y30" s="35" t="n">
@@ -15281,7 +15287,7 @@
         <v>–</v>
       </c>
       <c r="AC30" s="23" t="n">
-        <f aca="false">COUNTIF($Q$5:$Q$34,"&lt;"&amp;Q30)+1</f>
+        <f aca="false">SUMPRODUCT(--($Q$5:$Q$34&lt;Q30))+1</f>
         <v>21</v>
       </c>
       <c r="AD30" s="2" t="str">
@@ -15371,11 +15377,11 @@
         <v>1000.000031</v>
       </c>
       <c r="R31" s="23" t="n">
-        <f aca="false">COUNTIFS($C$5:$C$34,C31,$Q$5:$Q$34,"&lt;"&amp;Q31)+1</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C31)*($Q$5:$Q$34&lt;Q31))+1</f>
         <v>5</v>
       </c>
       <c r="S31" s="26" t="n">
-        <f aca="false">SUMIFS($AH$5:$AH$34,$C$5:$C$34,C31,$Q$5:$Q$34,"&lt;"&amp;Q31)</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C31)*($Q$5:$Q$34&lt;Q31)*$AH$5:$AH$34)</f>
         <v>15.185061525974</v>
       </c>
       <c r="T31" s="26" t="n">
@@ -15395,7 +15401,7 @@
         <v>0</v>
       </c>
       <c r="X31" s="35" t="n">
-        <f aca="false">IF(E31="Slot",ROUNDUP(W31/G31,0)*F31,W31*H31)</f>
+        <f aca="false">IF(E31="Slot",IF(N(G31)&gt;0,ROUNDUP(W31/G31,0)*F31,0),W31*H31)</f>
         <v>0</v>
       </c>
       <c r="Y31" s="35" t="n">
@@ -15415,7 +15421,7 @@
         <v>–</v>
       </c>
       <c r="AC31" s="23" t="n">
-        <f aca="false">COUNTIF($Q$5:$Q$34,"&lt;"&amp;Q31)+1</f>
+        <f aca="false">SUMPRODUCT(--($Q$5:$Q$34&lt;Q31))+1</f>
         <v>22</v>
       </c>
       <c r="AD31" s="2" t="str">
@@ -15505,11 +15511,11 @@
         <v>1000.000032</v>
       </c>
       <c r="R32" s="23" t="n">
-        <f aca="false">COUNTIFS($C$5:$C$34,C32,$Q$5:$Q$34,"&lt;"&amp;Q32)+1</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C32)*($Q$5:$Q$34&lt;Q32))+1</f>
         <v>5</v>
       </c>
       <c r="S32" s="26" t="n">
-        <f aca="false">SUMIFS($AH$5:$AH$34,$C$5:$C$34,C32,$Q$5:$Q$34,"&lt;"&amp;Q32)</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C32)*($Q$5:$Q$34&lt;Q32)*$AH$5:$AH$34)</f>
         <v>7.39734136363636</v>
       </c>
       <c r="T32" s="26" t="n">
@@ -15529,7 +15535,7 @@
         <v>3.21462175852628</v>
       </c>
       <c r="X32" s="35" t="n">
-        <f aca="false">IF(E32="Slot",ROUNDUP(W32/G32,0)*F32,W32*H32)</f>
+        <f aca="false">IF(E32="Slot",IF(N(G32)&gt;0,ROUNDUP(W32/G32,0)*F32,0),W32*H32)</f>
         <v>445.42</v>
       </c>
       <c r="Y32" s="35" t="n">
@@ -15549,7 +15555,7 @@
         <v>1000</v>
       </c>
       <c r="AC32" s="23" t="n">
-        <f aca="false">COUNTIF($Q$5:$Q$34,"&lt;"&amp;Q32)+1</f>
+        <f aca="false">SUMPRODUCT(--($Q$5:$Q$34&lt;Q32))+1</f>
         <v>23</v>
       </c>
       <c r="AD32" s="2" t="str">
@@ -15639,11 +15645,11 @@
         <v>880.600913600881</v>
       </c>
       <c r="R33" s="23" t="n">
-        <f aca="false">COUNTIFS($C$5:$C$34,C33,$Q$5:$Q$34,"&lt;"&amp;Q33)+1</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C33)*($Q$5:$Q$34&lt;Q33))+1</f>
         <v>4</v>
       </c>
       <c r="S33" s="26" t="n">
-        <f aca="false">SUMIFS($AH$5:$AH$34,$C$5:$C$34,C33,$Q$5:$Q$34,"&lt;"&amp;Q33)</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C33)*($Q$5:$Q$34&lt;Q33)*$AH$5:$AH$34)</f>
         <v>11.01043125</v>
       </c>
       <c r="T33" s="26" t="n">
@@ -15663,7 +15669,7 @@
         <v>300</v>
       </c>
       <c r="X33" s="35" t="n">
-        <f aca="false">IF(E33="Slot",ROUNDUP(W33/G33,0)*F33,W33*H33)</f>
+        <f aca="false">IF(E33="Slot",IF(N(G33)&gt;0,ROUNDUP(W33/G33,0)*F33,0),W33*H33)</f>
         <v>9000</v>
       </c>
       <c r="Y33" s="35" t="n">
@@ -15683,7 +15689,7 @@
         <v>880.600880600881</v>
       </c>
       <c r="AC33" s="23" t="n">
-        <f aca="false">COUNTIF($Q$5:$Q$34,"&lt;"&amp;Q33)+1</f>
+        <f aca="false">SUMPRODUCT(--($Q$5:$Q$34&lt;Q33))+1</f>
         <v>18</v>
       </c>
       <c r="AD33" s="2" t="str">
@@ -15773,11 +15779,11 @@
         <v>221.181546090603</v>
       </c>
       <c r="R34" s="23" t="n">
-        <f aca="false">COUNTIFS($C$5:$C$34,C34,$Q$5:$Q$34,"&lt;"&amp;Q34)+1</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C34)*($Q$5:$Q$34&lt;Q34))+1</f>
         <v>3</v>
       </c>
       <c r="S34" s="26" t="n">
-        <f aca="false">SUMIFS($AH$5:$AH$34,$C$5:$C$34,C34,$Q$5:$Q$34,"&lt;"&amp;Q34)</f>
+        <f aca="false">SUMPRODUCT(($C$5:$C$34=C34)*($Q$5:$Q$34&lt;Q34)*$AH$5:$AH$34)</f>
         <v>22.9635</v>
       </c>
       <c r="T34" s="26" t="n">
@@ -15797,7 +15803,7 @@
         <v>140.785958761165</v>
       </c>
       <c r="X34" s="35" t="n">
-        <f aca="false">IF(E34="Slot",ROUNDUP(W34/G34,0)*F34,W34*H34)</f>
+        <f aca="false">IF(E34="Slot",IF(N(G34)&gt;0,ROUNDUP(W34/G34,0)*F34,0),W34*H34)</f>
         <v>2745.32619584272</v>
       </c>
       <c r="Y34" s="35" t="n">
@@ -15817,7 +15823,7 @@
         <v>227.948091296738</v>
       </c>
       <c r="AC34" s="23" t="n">
-        <f aca="false">COUNTIF($Q$5:$Q$34,"&lt;"&amp;Q34)+1</f>
+        <f aca="false">SUMPRODUCT(--($Q$5:$Q$34&lt;Q34))+1</f>
         <v>9</v>
       </c>
       <c r="AD34" s="2" t="str">
@@ -16087,7 +16093,7 @@
         <v>618</v>
       </c>
       <c r="C10" s="35" t="n">
-        <f aca="false">C9/(1-Assumptions!$D$48)*Assumptions!$D$48</f>
+        <f aca="false">IF(Assumptions!$D$48&lt;1,C9/(1-Assumptions!$D$48)*Assumptions!$D$48,0)</f>
         <v>6835.31791725867</v>
       </c>
     </row>
@@ -16123,7 +16129,7 @@
         <v>622</v>
       </c>
       <c r="C14" s="41" t="n">
-        <f aca="false">C9/C13</f>
+        <f aca="false">IF(C13&gt;0,C9/C13,0)</f>
         <v>387.334681977991</v>
       </c>
     </row>
@@ -16132,7 +16138,7 @@
         <v>623</v>
       </c>
       <c r="C15" s="35" t="n">
-        <f aca="false">C12/C13</f>
+        <f aca="false">IF(C13&gt;0,C12/C13,0)</f>
         <v>475</v>
       </c>
     </row>
@@ -16141,7 +16147,7 @@
         <v>624</v>
       </c>
       <c r="C16" s="24" t="n">
-        <f aca="false">Weekly!N5/C12</f>
+        <f aca="false">IF(C12&gt;0,Weekly!N5/C12,0)</f>
         <v>0.297811868076705</v>
       </c>
     </row>
@@ -16202,7 +16208,7 @@
         <v>30</v>
       </c>
       <c r="H21" s="35" t="n">
-        <f aca="false">F21/G21</f>
+        <f aca="false">IF(G21&gt;0,F21/G21,0)</f>
         <v>664.197544642857</v>
       </c>
       <c r="I21" s="26" t="n">
@@ -16235,7 +16241,7 @@
         <v>45</v>
       </c>
       <c r="H22" s="35" t="n">
-        <f aca="false">F22/G22</f>
+        <f aca="false">IF(G22&gt;0,F22/G22,0)</f>
         <v>123.229471018727</v>
       </c>
       <c r="I22" s="26" t="n">
@@ -16268,7 +16274,7 @@
         <v>15</v>
       </c>
       <c r="H23" s="35" t="n">
-        <f aca="false">F23/G23</f>
+        <f aca="false">IF(G23&gt;0,F23/G23,0)</f>
         <v>447.262567987568</v>
       </c>
       <c r="I23" s="26" t="n">
@@ -16301,7 +16307,7 @@
         <v>10</v>
       </c>
       <c r="H24" s="35" t="n">
-        <f aca="false">F24/G24</f>
+        <f aca="false">IF(G24&gt;0,F24/G24,0)</f>
         <v>655.327714285714</v>
       </c>
       <c r="I24" s="26" t="n">
@@ -16382,7 +16388,7 @@
         <v>0</v>
       </c>
       <c r="F29" s="24" t="n">
-        <f aca="false">C29/$C$9</f>
+        <f aca="false">IF($C$9&gt;0,C29/$C$9,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -16403,7 +16409,7 @@
         <v>689.872244283762</v>
       </c>
       <c r="F30" s="24" t="n">
-        <f aca="false">C30/$C$9</f>
+        <f aca="false">IF($C$9&gt;0,C30/$C$9,0)</f>
         <v>0.0774523981348633</v>
       </c>
     </row>
@@ -16424,7 +16430,7 @@
         <v>1583.36321262101</v>
       </c>
       <c r="F31" s="24" t="n">
-        <f aca="false">C31/$C$9</f>
+        <f aca="false">IF($C$9&gt;0,C31/$C$9,0)</f>
         <v>0.037409508299139</v>
       </c>
     </row>
@@ -16445,7 +16451,7 @@
         <v>682.177632696661</v>
       </c>
       <c r="F32" s="24" t="n">
-        <f aca="false">C32/$C$9</f>
+        <f aca="false">IF($C$9&gt;0,C32/$C$9,0)</f>
         <v>0.245883959349519</v>
       </c>
     </row>
@@ -16466,7 +16472,7 @@
         <v>404.551201011378</v>
       </c>
       <c r="F33" s="24" t="n">
-        <f aca="false">C33/$C$9</f>
+        <f aca="false">IF($C$9&gt;0,C33/$C$9,0)</f>
         <v>0.0387261990674316</v>
       </c>
     </row>
@@ -16487,7 +16493,7 @@
         <v>598.102911424966</v>
       </c>
       <c r="F34" s="24" t="n">
-        <f aca="false">C34/$C$9</f>
+        <f aca="false">IF($C$9&gt;0,C34/$C$9,0)</f>
         <v>0.127980867394274</v>
       </c>
     </row>
@@ -16508,7 +16514,7 @@
         <v>20.9285958167923</v>
       </c>
       <c r="F35" s="24" t="n">
-        <f aca="false">C35/$C$9</f>
+        <f aca="false">IF($C$9&gt;0,C35/$C$9,0)</f>
         <v>0.00903611311573405</v>
       </c>
     </row>
@@ -16529,7 +16535,7 @@
         <v>1000</v>
       </c>
       <c r="F36" s="24" t="n">
-        <f aca="false">C36/$C$9</f>
+        <f aca="false">IF($C$9&gt;0,C36/$C$9,0)</f>
         <v>0.118968448719029</v>
       </c>
     </row>
@@ -16550,7 +16556,7 @@
         <v>880.600880600881</v>
       </c>
       <c r="F37" s="24" t="n">
-        <f aca="false">C37/$C$9</f>
+        <f aca="false">IF($C$9&gt;0,C37/$C$9,0)</f>
         <v>0.263338153658535</v>
       </c>
     </row>
@@ -16571,7 +16577,7 @@
         <v>227.948091296738</v>
       </c>
       <c r="F38" s="24" t="n">
-        <f aca="false">C38/$C$9</f>
+        <f aca="false">IF($C$9&gt;0,C38/$C$9,0)</f>
         <v>0.0812043522614752</v>
       </c>
     </row>
@@ -16661,7 +16667,7 @@
         <v>100</v>
       </c>
       <c r="I45" s="35" t="n">
-        <f aca="false">C45/H45</f>
+        <f aca="false">IF(H45&gt;0,C45/H45,0)</f>
         <v>475</v>
       </c>
     </row>
@@ -16695,7 +16701,7 @@
         <v>96.8809299857171</v>
       </c>
       <c r="I46" s="35" t="n">
-        <f aca="false">C46/H46</f>
+        <f aca="false">IF(H46&gt;0,C46/H46,0)</f>
         <v>416.748683213016</v>
       </c>
     </row>
@@ -16729,7 +16735,7 @@
         <v>90.6720880966647</v>
       </c>
       <c r="I47" s="35" t="n">
-        <f aca="false">C47/H47</f>
+        <f aca="false">IF(H47&gt;0,C47/H47,0)</f>
         <v>366.706013922967</v>
       </c>
     </row>
@@ -16763,7 +16769,7 @@
         <v>80.2795630966647</v>
       </c>
       <c r="I48" s="35" t="n">
-        <f aca="false">C48/H48</f>
+        <f aca="false">IF(H48&gt;0,C48/H48,0)</f>
         <v>295.841171574422</v>
       </c>
     </row>
@@ -16995,19 +17001,19 @@
         <v>3.861</v>
       </c>
       <c r="J8" s="35" t="n">
-        <f aca="false">MIN(C8,MAX(0,F$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D8)))</f>
+        <f aca="false">MIN(C8,MAX(0,F$6-SUMPRODUCT(($D$8:$D$37&gt;D8)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="K8" s="35" t="n">
-        <f aca="false">MIN(C8,MAX(0,G$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D8)))</f>
+        <f aca="false">MIN(C8,MAX(0,G$6-SUMPRODUCT(($D$8:$D$37&gt;D8)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="L8" s="35" t="n">
-        <f aca="false">MIN(C8,MAX(0,H$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D8)))</f>
+        <f aca="false">MIN(C8,MAX(0,H$6-SUMPRODUCT(($D$8:$D$37&gt;D8)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="M8" s="35" t="n">
-        <f aca="false">MIN(C8,MAX(0,I$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D8)))</f>
+        <f aca="false">MIN(C8,MAX(0,I$6-SUMPRODUCT(($D$8:$D$37&gt;D8)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="N8" s="35" t="n">
@@ -17053,19 +17059,19 @@
         <v>14.58</v>
       </c>
       <c r="J9" s="35" t="n">
-        <f aca="false">MIN(C9,MAX(0,F$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D9)))</f>
+        <f aca="false">MIN(C9,MAX(0,F$6-SUMPRODUCT(($D$8:$D$37&gt;D9)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="K9" s="35" t="n">
-        <f aca="false">MIN(C9,MAX(0,G$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D9)))</f>
+        <f aca="false">MIN(C9,MAX(0,G$6-SUMPRODUCT(($D$8:$D$37&gt;D9)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="L9" s="35" t="n">
-        <f aca="false">MIN(C9,MAX(0,H$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D9)))</f>
+        <f aca="false">MIN(C9,MAX(0,H$6-SUMPRODUCT(($D$8:$D$37&gt;D9)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="M9" s="35" t="n">
-        <f aca="false">MIN(C9,MAX(0,I$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D9)))</f>
+        <f aca="false">MIN(C9,MAX(0,I$6-SUMPRODUCT(($D$8:$D$37&gt;D9)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="N9" s="35" t="n">
@@ -17111,19 +17117,19 @@
         <v>2.34</v>
       </c>
       <c r="J10" s="35" t="n">
-        <f aca="false">MIN(C10,MAX(0,F$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D10)))</f>
+        <f aca="false">MIN(C10,MAX(0,F$6-SUMPRODUCT(($D$8:$D$37&gt;D10)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="K10" s="35" t="n">
-        <f aca="false">MIN(C10,MAX(0,G$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D10)))</f>
+        <f aca="false">MIN(C10,MAX(0,G$6-SUMPRODUCT(($D$8:$D$37&gt;D10)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="L10" s="35" t="n">
-        <f aca="false">MIN(C10,MAX(0,H$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D10)))</f>
+        <f aca="false">MIN(C10,MAX(0,H$6-SUMPRODUCT(($D$8:$D$37&gt;D10)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="M10" s="35" t="n">
-        <f aca="false">MIN(C10,MAX(0,I$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D10)))</f>
+        <f aca="false">MIN(C10,MAX(0,I$6-SUMPRODUCT(($D$8:$D$37&gt;D10)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="N10" s="35" t="n">
@@ -17169,19 +17175,19 @@
         <v>1.2852</v>
       </c>
       <c r="J11" s="35" t="n">
-        <f aca="false">MIN(C11,MAX(0,F$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D11)))</f>
+        <f aca="false">MIN(C11,MAX(0,F$6-SUMPRODUCT(($D$8:$D$37&gt;D11)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="K11" s="35" t="n">
-        <f aca="false">MIN(C11,MAX(0,G$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D11)))</f>
+        <f aca="false">MIN(C11,MAX(0,G$6-SUMPRODUCT(($D$8:$D$37&gt;D11)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="L11" s="35" t="n">
-        <f aca="false">MIN(C11,MAX(0,H$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D11)))</f>
+        <f aca="false">MIN(C11,MAX(0,H$6-SUMPRODUCT(($D$8:$D$37&gt;D11)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="M11" s="35" t="n">
-        <f aca="false">MIN(C11,MAX(0,I$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D11)))</f>
+        <f aca="false">MIN(C11,MAX(0,I$6-SUMPRODUCT(($D$8:$D$37&gt;D11)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="N11" s="35" t="n">
@@ -17227,19 +17233,19 @@
         <v>0</v>
       </c>
       <c r="J12" s="35" t="n">
-        <f aca="false">MIN(C12,MAX(0,F$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D12)))</f>
+        <f aca="false">MIN(C12,MAX(0,F$6-SUMPRODUCT(($D$8:$D$37&gt;D12)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="K12" s="35" t="n">
-        <f aca="false">MIN(C12,MAX(0,G$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D12)))</f>
+        <f aca="false">MIN(C12,MAX(0,G$6-SUMPRODUCT(($D$8:$D$37&gt;D12)*$C$8:$C$37)))</f>
         <v>750</v>
       </c>
       <c r="L12" s="35" t="n">
-        <f aca="false">MIN(C12,MAX(0,H$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D12)))</f>
+        <f aca="false">MIN(C12,MAX(0,H$6-SUMPRODUCT(($D$8:$D$37&gt;D12)*$C$8:$C$37)))</f>
         <v>750</v>
       </c>
       <c r="M12" s="35" t="n">
-        <f aca="false">MIN(C12,MAX(0,I$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D12)))</f>
+        <f aca="false">MIN(C12,MAX(0,I$6-SUMPRODUCT(($D$8:$D$37&gt;D12)*$C$8:$C$37)))</f>
         <v>750</v>
       </c>
       <c r="N12" s="35" t="n">
@@ -17285,19 +17291,19 @@
         <v>2.784375</v>
       </c>
       <c r="J13" s="35" t="n">
-        <f aca="false">MIN(C13,MAX(0,F$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D13)))</f>
+        <f aca="false">MIN(C13,MAX(0,F$6-SUMPRODUCT(($D$8:$D$37&gt;D13)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="K13" s="35" t="n">
-        <f aca="false">MIN(C13,MAX(0,G$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D13)))</f>
+        <f aca="false">MIN(C13,MAX(0,G$6-SUMPRODUCT(($D$8:$D$37&gt;D13)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="L13" s="35" t="n">
-        <f aca="false">MIN(C13,MAX(0,H$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D13)))</f>
+        <f aca="false">MIN(C13,MAX(0,H$6-SUMPRODUCT(($D$8:$D$37&gt;D13)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="M13" s="35" t="n">
-        <f aca="false">MIN(C13,MAX(0,I$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D13)))</f>
+        <f aca="false">MIN(C13,MAX(0,I$6-SUMPRODUCT(($D$8:$D$37&gt;D13)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="N13" s="35" t="n">
@@ -17343,19 +17349,19 @@
         <v>0</v>
       </c>
       <c r="J14" s="35" t="n">
-        <f aca="false">MIN(C14,MAX(0,F$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D14)))</f>
+        <f aca="false">MIN(C14,MAX(0,F$6-SUMPRODUCT(($D$8:$D$37&gt;D14)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="K14" s="35" t="n">
-        <f aca="false">MIN(C14,MAX(0,G$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D14)))</f>
+        <f aca="false">MIN(C14,MAX(0,G$6-SUMPRODUCT(($D$8:$D$37&gt;D14)*$C$8:$C$37)))</f>
         <v>750</v>
       </c>
       <c r="L14" s="35" t="n">
-        <f aca="false">MIN(C14,MAX(0,H$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D14)))</f>
+        <f aca="false">MIN(C14,MAX(0,H$6-SUMPRODUCT(($D$8:$D$37&gt;D14)*$C$8:$C$37)))</f>
         <v>750</v>
       </c>
       <c r="M14" s="35" t="n">
-        <f aca="false">MIN(C14,MAX(0,I$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D14)))</f>
+        <f aca="false">MIN(C14,MAX(0,I$6-SUMPRODUCT(($D$8:$D$37&gt;D14)*$C$8:$C$37)))</f>
         <v>750</v>
       </c>
       <c r="N14" s="35" t="n">
@@ -17401,19 +17407,19 @@
         <v>0</v>
       </c>
       <c r="J15" s="35" t="n">
-        <f aca="false">MIN(C15,MAX(0,F$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D15)))</f>
+        <f aca="false">MIN(C15,MAX(0,F$6-SUMPRODUCT(($D$8:$D$37&gt;D15)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="K15" s="35" t="n">
-        <f aca="false">MIN(C15,MAX(0,G$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D15)))</f>
+        <f aca="false">MIN(C15,MAX(0,G$6-SUMPRODUCT(($D$8:$D$37&gt;D15)*$C$8:$C$37)))</f>
         <v>750</v>
       </c>
       <c r="L15" s="35" t="n">
-        <f aca="false">MIN(C15,MAX(0,H$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D15)))</f>
+        <f aca="false">MIN(C15,MAX(0,H$6-SUMPRODUCT(($D$8:$D$37&gt;D15)*$C$8:$C$37)))</f>
         <v>750</v>
       </c>
       <c r="M15" s="35" t="n">
-        <f aca="false">MIN(C15,MAX(0,I$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D15)))</f>
+        <f aca="false">MIN(C15,MAX(0,I$6-SUMPRODUCT(($D$8:$D$37&gt;D15)*$C$8:$C$37)))</f>
         <v>750</v>
       </c>
       <c r="N15" s="35" t="n">
@@ -17459,19 +17465,19 @@
         <v>0</v>
       </c>
       <c r="J16" s="35" t="n">
-        <f aca="false">MIN(C16,MAX(0,F$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D16)))</f>
+        <f aca="false">MIN(C16,MAX(0,F$6-SUMPRODUCT(($D$8:$D$37&gt;D16)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="K16" s="35" t="n">
-        <f aca="false">MIN(C16,MAX(0,G$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D16)))</f>
+        <f aca="false">MIN(C16,MAX(0,G$6-SUMPRODUCT(($D$8:$D$37&gt;D16)*$C$8:$C$37)))</f>
         <v>1449</v>
       </c>
       <c r="L16" s="35" t="n">
-        <f aca="false">MIN(C16,MAX(0,H$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D16)))</f>
+        <f aca="false">MIN(C16,MAX(0,H$6-SUMPRODUCT(($D$8:$D$37&gt;D16)*$C$8:$C$37)))</f>
         <v>1449</v>
       </c>
       <c r="M16" s="35" t="n">
-        <f aca="false">MIN(C16,MAX(0,I$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D16)))</f>
+        <f aca="false">MIN(C16,MAX(0,I$6-SUMPRODUCT(($D$8:$D$37&gt;D16)*$C$8:$C$37)))</f>
         <v>1449</v>
       </c>
       <c r="N16" s="35" t="n">
@@ -17517,19 +17523,19 @@
         <v>0</v>
       </c>
       <c r="J17" s="35" t="n">
-        <f aca="false">MIN(C17,MAX(0,F$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D17)))</f>
+        <f aca="false">MIN(C17,MAX(0,F$6-SUMPRODUCT(($D$8:$D$37&gt;D17)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="K17" s="35" t="n">
-        <f aca="false">MIN(C17,MAX(0,G$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D17)))</f>
+        <f aca="false">MIN(C17,MAX(0,G$6-SUMPRODUCT(($D$8:$D$37&gt;D17)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="L17" s="35" t="n">
-        <f aca="false">MIN(C17,MAX(0,H$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D17)))</f>
+        <f aca="false">MIN(C17,MAX(0,H$6-SUMPRODUCT(($D$8:$D$37&gt;D17)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="M17" s="35" t="n">
-        <f aca="false">MIN(C17,MAX(0,I$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D17)))</f>
+        <f aca="false">MIN(C17,MAX(0,I$6-SUMPRODUCT(($D$8:$D$37&gt;D17)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="N17" s="35" t="n">
@@ -17575,19 +17581,19 @@
         <v>0</v>
       </c>
       <c r="J18" s="35" t="n">
-        <f aca="false">MIN(C18,MAX(0,F$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D18)))</f>
+        <f aca="false">MIN(C18,MAX(0,F$6-SUMPRODUCT(($D$8:$D$37&gt;D18)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="K18" s="35" t="n">
-        <f aca="false">MIN(C18,MAX(0,G$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D18)))</f>
+        <f aca="false">MIN(C18,MAX(0,G$6-SUMPRODUCT(($D$8:$D$37&gt;D18)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="L18" s="35" t="n">
-        <f aca="false">MIN(C18,MAX(0,H$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D18)))</f>
+        <f aca="false">MIN(C18,MAX(0,H$6-SUMPRODUCT(($D$8:$D$37&gt;D18)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="M18" s="35" t="n">
-        <f aca="false">MIN(C18,MAX(0,I$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D18)))</f>
+        <f aca="false">MIN(C18,MAX(0,I$6-SUMPRODUCT(($D$8:$D$37&gt;D18)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="N18" s="35" t="n">
@@ -17633,19 +17639,19 @@
         <v>0</v>
       </c>
       <c r="J19" s="35" t="n">
-        <f aca="false">MIN(C19,MAX(0,F$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D19)))</f>
+        <f aca="false">MIN(C19,MAX(0,F$6-SUMPRODUCT(($D$8:$D$37&gt;D19)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="K19" s="35" t="n">
-        <f aca="false">MIN(C19,MAX(0,G$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D19)))</f>
+        <f aca="false">MIN(C19,MAX(0,G$6-SUMPRODUCT(($D$8:$D$37&gt;D19)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="L19" s="35" t="n">
-        <f aca="false">MIN(C19,MAX(0,H$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D19)))</f>
+        <f aca="false">MIN(C19,MAX(0,H$6-SUMPRODUCT(($D$8:$D$37&gt;D19)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="M19" s="35" t="n">
-        <f aca="false">MIN(C19,MAX(0,I$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D19)))</f>
+        <f aca="false">MIN(C19,MAX(0,I$6-SUMPRODUCT(($D$8:$D$37&gt;D19)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="N19" s="35" t="n">
@@ -17691,19 +17697,19 @@
         <v>8.60608295454545</v>
       </c>
       <c r="J20" s="35" t="n">
-        <f aca="false">MIN(C20,MAX(0,F$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D20)))</f>
+        <f aca="false">MIN(C20,MAX(0,F$6-SUMPRODUCT(($D$8:$D$37&gt;D20)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="K20" s="35" t="n">
-        <f aca="false">MIN(C20,MAX(0,G$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D20)))</f>
+        <f aca="false">MIN(C20,MAX(0,G$6-SUMPRODUCT(($D$8:$D$37&gt;D20)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="L20" s="35" t="n">
-        <f aca="false">MIN(C20,MAX(0,H$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D20)))</f>
+        <f aca="false">MIN(C20,MAX(0,H$6-SUMPRODUCT(($D$8:$D$37&gt;D20)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="M20" s="35" t="n">
-        <f aca="false">MIN(C20,MAX(0,I$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D20)))</f>
+        <f aca="false">MIN(C20,MAX(0,I$6-SUMPRODUCT(($D$8:$D$37&gt;D20)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="N20" s="35" t="n">
@@ -17749,19 +17755,19 @@
         <v>5.355</v>
       </c>
       <c r="J21" s="35" t="n">
-        <f aca="false">MIN(C21,MAX(0,F$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D21)))</f>
+        <f aca="false">MIN(C21,MAX(0,F$6-SUMPRODUCT(($D$8:$D$37&gt;D21)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="K21" s="35" t="n">
-        <f aca="false">MIN(C21,MAX(0,G$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D21)))</f>
+        <f aca="false">MIN(C21,MAX(0,G$6-SUMPRODUCT(($D$8:$D$37&gt;D21)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="L21" s="35" t="n">
-        <f aca="false">MIN(C21,MAX(0,H$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D21)))</f>
+        <f aca="false">MIN(C21,MAX(0,H$6-SUMPRODUCT(($D$8:$D$37&gt;D21)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="M21" s="35" t="n">
-        <f aca="false">MIN(C21,MAX(0,I$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D21)))</f>
+        <f aca="false">MIN(C21,MAX(0,I$6-SUMPRODUCT(($D$8:$D$37&gt;D21)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="N21" s="35" t="n">
@@ -17807,19 +17813,19 @@
         <v>0</v>
       </c>
       <c r="J22" s="35" t="n">
-        <f aca="false">MIN(C22,MAX(0,F$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D22)))</f>
+        <f aca="false">MIN(C22,MAX(0,F$6-SUMPRODUCT(($D$8:$D$37&gt;D22)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="K22" s="35" t="n">
-        <f aca="false">MIN(C22,MAX(0,G$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D22)))</f>
+        <f aca="false">MIN(C22,MAX(0,G$6-SUMPRODUCT(($D$8:$D$37&gt;D22)*$C$8:$C$37)))</f>
         <v>715.718197799099</v>
       </c>
       <c r="L22" s="35" t="n">
-        <f aca="false">MIN(C22,MAX(0,H$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D22)))</f>
+        <f aca="false">MIN(C22,MAX(0,H$6-SUMPRODUCT(($D$8:$D$37&gt;D22)*$C$8:$C$37)))</f>
         <v>750</v>
       </c>
       <c r="M22" s="35" t="n">
-        <f aca="false">MIN(C22,MAX(0,I$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D22)))</f>
+        <f aca="false">MIN(C22,MAX(0,I$6-SUMPRODUCT(($D$8:$D$37&gt;D22)*$C$8:$C$37)))</f>
         <v>750</v>
       </c>
       <c r="N22" s="35" t="n">
@@ -17865,19 +17871,19 @@
         <v>3.0375</v>
       </c>
       <c r="J23" s="35" t="n">
-        <f aca="false">MIN(C23,MAX(0,F$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D23)))</f>
+        <f aca="false">MIN(C23,MAX(0,F$6-SUMPRODUCT(($D$8:$D$37&gt;D23)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="K23" s="35" t="n">
-        <f aca="false">MIN(C23,MAX(0,G$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D23)))</f>
+        <f aca="false">MIN(C23,MAX(0,G$6-SUMPRODUCT(($D$8:$D$37&gt;D23)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="L23" s="35" t="n">
-        <f aca="false">MIN(C23,MAX(0,H$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D23)))</f>
+        <f aca="false">MIN(C23,MAX(0,H$6-SUMPRODUCT(($D$8:$D$37&gt;D23)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="M23" s="35" t="n">
-        <f aca="false">MIN(C23,MAX(0,I$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D23)))</f>
+        <f aca="false">MIN(C23,MAX(0,I$6-SUMPRODUCT(($D$8:$D$37&gt;D23)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="N23" s="35" t="n">
@@ -17923,19 +17929,19 @@
         <v>3.861</v>
       </c>
       <c r="J24" s="35" t="n">
-        <f aca="false">MIN(C24,MAX(0,F$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D24)))</f>
+        <f aca="false">MIN(C24,MAX(0,F$6-SUMPRODUCT(($D$8:$D$37&gt;D24)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="K24" s="35" t="n">
-        <f aca="false">MIN(C24,MAX(0,G$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D24)))</f>
+        <f aca="false">MIN(C24,MAX(0,G$6-SUMPRODUCT(($D$8:$D$37&gt;D24)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="L24" s="35" t="n">
-        <f aca="false">MIN(C24,MAX(0,H$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D24)))</f>
+        <f aca="false">MIN(C24,MAX(0,H$6-SUMPRODUCT(($D$8:$D$37&gt;D24)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="M24" s="35" t="n">
-        <f aca="false">MIN(C24,MAX(0,I$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D24)))</f>
+        <f aca="false">MIN(C24,MAX(0,I$6-SUMPRODUCT(($D$8:$D$37&gt;D24)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="N24" s="35" t="n">
@@ -17981,19 +17987,19 @@
         <v>2.41619318181818</v>
       </c>
       <c r="J25" s="35" t="n">
-        <f aca="false">MIN(C25,MAX(0,F$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D25)))</f>
+        <f aca="false">MIN(C25,MAX(0,F$6-SUMPRODUCT(($D$8:$D$37&gt;D25)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="K25" s="35" t="n">
-        <f aca="false">MIN(C25,MAX(0,G$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D25)))</f>
+        <f aca="false">MIN(C25,MAX(0,G$6-SUMPRODUCT(($D$8:$D$37&gt;D25)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="L25" s="35" t="n">
-        <f aca="false">MIN(C25,MAX(0,H$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D25)))</f>
+        <f aca="false">MIN(C25,MAX(0,H$6-SUMPRODUCT(($D$8:$D$37&gt;D25)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="M25" s="35" t="n">
-        <f aca="false">MIN(C25,MAX(0,I$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D25)))</f>
+        <f aca="false">MIN(C25,MAX(0,I$6-SUMPRODUCT(($D$8:$D$37&gt;D25)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="N25" s="35" t="n">
@@ -18039,19 +18045,19 @@
         <v>1.04701704545455</v>
       </c>
       <c r="J26" s="35" t="n">
-        <f aca="false">MIN(C26,MAX(0,F$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D26)))</f>
+        <f aca="false">MIN(C26,MAX(0,F$6-SUMPRODUCT(($D$8:$D$37&gt;D26)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="K26" s="35" t="n">
-        <f aca="false">MIN(C26,MAX(0,G$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D26)))</f>
+        <f aca="false">MIN(C26,MAX(0,G$6-SUMPRODUCT(($D$8:$D$37&gt;D26)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="L26" s="35" t="n">
-        <f aca="false">MIN(C26,MAX(0,H$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D26)))</f>
+        <f aca="false">MIN(C26,MAX(0,H$6-SUMPRODUCT(($D$8:$D$37&gt;D26)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="M26" s="35" t="n">
-        <f aca="false">MIN(C26,MAX(0,I$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D26)))</f>
+        <f aca="false">MIN(C26,MAX(0,I$6-SUMPRODUCT(($D$8:$D$37&gt;D26)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="N26" s="35" t="n">
@@ -18097,19 +18103,19 @@
         <v>0</v>
       </c>
       <c r="J27" s="35" t="n">
-        <f aca="false">MIN(C27,MAX(0,F$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D27)))</f>
+        <f aca="false">MIN(C27,MAX(0,F$6-SUMPRODUCT(($D$8:$D$37&gt;D27)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="K27" s="35" t="n">
-        <f aca="false">MIN(C27,MAX(0,G$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D27)))</f>
+        <f aca="false">MIN(C27,MAX(0,G$6-SUMPRODUCT(($D$8:$D$37&gt;D27)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="L27" s="35" t="n">
-        <f aca="false">MIN(C27,MAX(0,H$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D27)))</f>
+        <f aca="false">MIN(C27,MAX(0,H$6-SUMPRODUCT(($D$8:$D$37&gt;D27)*$C$8:$C$37)))</f>
         <v>942.857142857143</v>
       </c>
       <c r="M27" s="35" t="n">
-        <f aca="false">MIN(C27,MAX(0,I$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D27)))</f>
+        <f aca="false">MIN(C27,MAX(0,I$6-SUMPRODUCT(($D$8:$D$37&gt;D27)*$C$8:$C$37)))</f>
         <v>942.857142857143</v>
       </c>
       <c r="N27" s="35" t="n">
@@ -18155,19 +18161,19 @@
         <v>4.44015</v>
       </c>
       <c r="J28" s="35" t="n">
-        <f aca="false">MIN(C28,MAX(0,F$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D28)))</f>
+        <f aca="false">MIN(C28,MAX(0,F$6-SUMPRODUCT(($D$8:$D$37&gt;D28)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="K28" s="35" t="n">
-        <f aca="false">MIN(C28,MAX(0,G$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D28)))</f>
+        <f aca="false">MIN(C28,MAX(0,G$6-SUMPRODUCT(($D$8:$D$37&gt;D28)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="L28" s="35" t="n">
-        <f aca="false">MIN(C28,MAX(0,H$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D28)))</f>
+        <f aca="false">MIN(C28,MAX(0,H$6-SUMPRODUCT(($D$8:$D$37&gt;D28)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="M28" s="35" t="n">
-        <f aca="false">MIN(C28,MAX(0,I$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D28)))</f>
+        <f aca="false">MIN(C28,MAX(0,I$6-SUMPRODUCT(($D$8:$D$37&gt;D28)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="N28" s="35" t="n">
@@ -18213,19 +18219,19 @@
         <v>8.3835</v>
       </c>
       <c r="J29" s="35" t="n">
-        <f aca="false">MIN(C29,MAX(0,F$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D29)))</f>
+        <f aca="false">MIN(C29,MAX(0,F$6-SUMPRODUCT(($D$8:$D$37&gt;D29)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="K29" s="35" t="n">
-        <f aca="false">MIN(C29,MAX(0,G$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D29)))</f>
+        <f aca="false">MIN(C29,MAX(0,G$6-SUMPRODUCT(($D$8:$D$37&gt;D29)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="L29" s="35" t="n">
-        <f aca="false">MIN(C29,MAX(0,H$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D29)))</f>
+        <f aca="false">MIN(C29,MAX(0,H$6-SUMPRODUCT(($D$8:$D$37&gt;D29)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="M29" s="35" t="n">
-        <f aca="false">MIN(C29,MAX(0,I$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D29)))</f>
+        <f aca="false">MIN(C29,MAX(0,I$6-SUMPRODUCT(($D$8:$D$37&gt;D29)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="N29" s="35" t="n">
@@ -18271,19 +18277,19 @@
         <v>2.4219</v>
       </c>
       <c r="J30" s="35" t="n">
-        <f aca="false">MIN(C30,MAX(0,F$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D30)))</f>
+        <f aca="false">MIN(C30,MAX(0,F$6-SUMPRODUCT(($D$8:$D$37&gt;D30)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="K30" s="35" t="n">
-        <f aca="false">MIN(C30,MAX(0,G$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D30)))</f>
+        <f aca="false">MIN(C30,MAX(0,G$6-SUMPRODUCT(($D$8:$D$37&gt;D30)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="L30" s="35" t="n">
-        <f aca="false">MIN(C30,MAX(0,H$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D30)))</f>
+        <f aca="false">MIN(C30,MAX(0,H$6-SUMPRODUCT(($D$8:$D$37&gt;D30)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="M30" s="35" t="n">
-        <f aca="false">MIN(C30,MAX(0,I$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D30)))</f>
+        <f aca="false">MIN(C30,MAX(0,I$6-SUMPRODUCT(($D$8:$D$37&gt;D30)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="N30" s="35" t="n">
@@ -18329,19 +18335,19 @@
         <v>1.47798</v>
       </c>
       <c r="J31" s="35" t="n">
-        <f aca="false">MIN(C31,MAX(0,F$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D31)))</f>
+        <f aca="false">MIN(C31,MAX(0,F$6-SUMPRODUCT(($D$8:$D$37&gt;D31)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="K31" s="35" t="n">
-        <f aca="false">MIN(C31,MAX(0,G$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D31)))</f>
+        <f aca="false">MIN(C31,MAX(0,G$6-SUMPRODUCT(($D$8:$D$37&gt;D31)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="L31" s="35" t="n">
-        <f aca="false">MIN(C31,MAX(0,H$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D31)))</f>
+        <f aca="false">MIN(C31,MAX(0,H$6-SUMPRODUCT(($D$8:$D$37&gt;D31)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="M31" s="35" t="n">
-        <f aca="false">MIN(C31,MAX(0,I$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D31)))</f>
+        <f aca="false">MIN(C31,MAX(0,I$6-SUMPRODUCT(($D$8:$D$37&gt;D31)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="N31" s="35" t="n">
@@ -18387,19 +18393,19 @@
         <v>0</v>
       </c>
       <c r="J32" s="35" t="n">
-        <f aca="false">MIN(C32,MAX(0,F$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D32)))</f>
+        <f aca="false">MIN(C32,MAX(0,F$6-SUMPRODUCT(($D$8:$D$37&gt;D32)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="K32" s="35" t="n">
-        <f aca="false">MIN(C32,MAX(0,G$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D32)))</f>
+        <f aca="false">MIN(C32,MAX(0,G$6-SUMPRODUCT(($D$8:$D$37&gt;D32)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="L32" s="35" t="n">
-        <f aca="false">MIN(C32,MAX(0,H$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D32)))</f>
+        <f aca="false">MIN(C32,MAX(0,H$6-SUMPRODUCT(($D$8:$D$37&gt;D32)*$C$8:$C$37)))</f>
         <v>4162.640625</v>
       </c>
       <c r="M32" s="35" t="n">
-        <f aca="false">MIN(C32,MAX(0,I$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D32)))</f>
+        <f aca="false">MIN(C32,MAX(0,I$6-SUMPRODUCT(($D$8:$D$37&gt;D32)*$C$8:$C$37)))</f>
         <v>4162.640625</v>
       </c>
       <c r="N32" s="35" t="n">
@@ -18445,19 +18451,19 @@
         <v>0</v>
       </c>
       <c r="J33" s="35" t="n">
-        <f aca="false">MIN(C33,MAX(0,F$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D33)))</f>
+        <f aca="false">MIN(C33,MAX(0,F$6-SUMPRODUCT(($D$8:$D$37&gt;D33)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="K33" s="35" t="n">
-        <f aca="false">MIN(C33,MAX(0,G$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D33)))</f>
+        <f aca="false">MIN(C33,MAX(0,G$6-SUMPRODUCT(($D$8:$D$37&gt;D33)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="L33" s="35" t="n">
-        <f aca="false">MIN(C33,MAX(0,H$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D33)))</f>
+        <f aca="false">MIN(C33,MAX(0,H$6-SUMPRODUCT(($D$8:$D$37&gt;D33)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="M33" s="35" t="n">
-        <f aca="false">MIN(C33,MAX(0,I$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D33)))</f>
+        <f aca="false">MIN(C33,MAX(0,I$6-SUMPRODUCT(($D$8:$D$37&gt;D33)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="N33" s="35" t="n">
@@ -18503,19 +18509,19 @@
         <v>0</v>
       </c>
       <c r="J34" s="35" t="n">
-        <f aca="false">MIN(C34,MAX(0,F$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D34)))</f>
+        <f aca="false">MIN(C34,MAX(0,F$6-SUMPRODUCT(($D$8:$D$37&gt;D34)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="K34" s="35" t="n">
-        <f aca="false">MIN(C34,MAX(0,G$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D34)))</f>
+        <f aca="false">MIN(C34,MAX(0,G$6-SUMPRODUCT(($D$8:$D$37&gt;D34)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="L34" s="35" t="n">
-        <f aca="false">MIN(C34,MAX(0,H$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D34)))</f>
+        <f aca="false">MIN(C34,MAX(0,H$6-SUMPRODUCT(($D$8:$D$37&gt;D34)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="M34" s="35" t="n">
-        <f aca="false">MIN(C34,MAX(0,I$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D34)))</f>
+        <f aca="false">MIN(C34,MAX(0,I$6-SUMPRODUCT(($D$8:$D$37&gt;D34)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="N34" s="35" t="n">
@@ -18561,19 +18567,19 @@
         <v>0</v>
       </c>
       <c r="J35" s="35" t="n">
-        <f aca="false">MIN(C35,MAX(0,F$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D35)))</f>
+        <f aca="false">MIN(C35,MAX(0,F$6-SUMPRODUCT(($D$8:$D$37&gt;D35)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="K35" s="35" t="n">
-        <f aca="false">MIN(C35,MAX(0,G$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D35)))</f>
+        <f aca="false">MIN(C35,MAX(0,G$6-SUMPRODUCT(($D$8:$D$37&gt;D35)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="L35" s="35" t="n">
-        <f aca="false">MIN(C35,MAX(0,H$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D35)))</f>
+        <f aca="false">MIN(C35,MAX(0,H$6-SUMPRODUCT(($D$8:$D$37&gt;D35)*$C$8:$C$37)))</f>
         <v>445.42</v>
       </c>
       <c r="M35" s="35" t="n">
-        <f aca="false">MIN(C35,MAX(0,I$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D35)))</f>
+        <f aca="false">MIN(C35,MAX(0,I$6-SUMPRODUCT(($D$8:$D$37&gt;D35)*$C$8:$C$37)))</f>
         <v>445.42</v>
       </c>
       <c r="N35" s="35" t="n">
@@ -18619,19 +18625,19 @@
         <v>0.584233096664704</v>
       </c>
       <c r="J36" s="35" t="n">
-        <f aca="false">MIN(C36,MAX(0,F$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D36)))</f>
+        <f aca="false">MIN(C36,MAX(0,F$6-SUMPRODUCT(($D$8:$D$37&gt;D36)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="K36" s="35" t="n">
-        <f aca="false">MIN(C36,MAX(0,G$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D36)))</f>
+        <f aca="false">MIN(C36,MAX(0,G$6-SUMPRODUCT(($D$8:$D$37&gt;D36)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="L36" s="35" t="n">
-        <f aca="false">MIN(C36,MAX(0,H$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D36)))</f>
+        <f aca="false">MIN(C36,MAX(0,H$6-SUMPRODUCT(($D$8:$D$37&gt;D36)*$C$8:$C$37)))</f>
         <v>471.050429941955</v>
       </c>
       <c r="M36" s="35" t="n">
-        <f aca="false">MIN(C36,MAX(0,I$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D36)))</f>
+        <f aca="false">MIN(C36,MAX(0,I$6-SUMPRODUCT(($D$8:$D$37&gt;D36)*$C$8:$C$37)))</f>
         <v>8546.05042994196</v>
       </c>
       <c r="N36" s="35" t="n">
@@ -18677,19 +18683,19 @@
         <v>13.7984318181818</v>
       </c>
       <c r="J37" s="35" t="n">
-        <f aca="false">MIN(C37,MAX(0,F$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D37)))</f>
+        <f aca="false">MIN(C37,MAX(0,F$6-SUMPRODUCT(($D$8:$D$37&gt;D37)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="K37" s="35" t="n">
-        <f aca="false">MIN(C37,MAX(0,G$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D37)))</f>
+        <f aca="false">MIN(C37,MAX(0,G$6-SUMPRODUCT(($D$8:$D$37&gt;D37)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="L37" s="35" t="n">
-        <f aca="false">MIN(C37,MAX(0,H$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D37)))</f>
+        <f aca="false">MIN(C37,MAX(0,H$6-SUMPRODUCT(($D$8:$D$37&gt;D37)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="M37" s="35" t="n">
-        <f aca="false">MIN(C37,MAX(0,I$6-SUMIFS($C$8:$C$37,$D$8:$D$37,"&gt;"&amp;D37)))</f>
+        <f aca="false">MIN(C37,MAX(0,I$6-SUMPRODUCT(($D$8:$D$37&gt;D37)*$C$8:$C$37)))</f>
         <v>0</v>
       </c>
       <c r="N37" s="35" t="n">
@@ -18812,19 +18818,19 @@
         <v>629</v>
       </c>
       <c r="F44" s="35" t="n">
-        <f aca="false">F4/F43</f>
+        <f aca="false">IF(F43&gt;0,F4/F43,0)</f>
         <v>475</v>
       </c>
       <c r="G44" s="35" t="n">
-        <f aca="false">G4/G43</f>
+        <f aca="false">IF(G43&gt;0,G4/G43,0)</f>
         <v>416.748683213016</v>
       </c>
       <c r="H44" s="35" t="n">
-        <f aca="false">H4/H43</f>
+        <f aca="false">IF(H43&gt;0,H4/H43,0)</f>
         <v>366.706013922967</v>
       </c>
       <c r="I44" s="35" t="n">
-        <f aca="false">I4/I43</f>
+        <f aca="false">IF(I43&gt;0,I4/I43,0)</f>
         <v>295.841171574422</v>
       </c>
     </row>
@@ -18959,7 +18965,7 @@
         <v>0.03</v>
       </c>
       <c r="E4" s="24" t="n">
-        <f aca="false">IF(B4&lt;=Funnel!$B$20,D4,0)/SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14)</f>
+        <f aca="false">IF(SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14)&gt;0,IF(B4&lt;=Funnel!$B$20,D4,0)/SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14),0)</f>
         <v>0.0394736842105263</v>
       </c>
       <c r="F4" s="24" t="n">
@@ -19015,7 +19021,7 @@
         <v>0.998299142073115</v>
       </c>
       <c r="S4" s="2" t="str">
-        <f aca="false">IF(P4&gt;Q4+0.5,"OVER "&amp;Assumptions!$D$9&amp;"/wk – pace down",IF(R4&gt;Assumptions!$D$106,"Full",""))</f>
+        <f aca="false">IF(P4&gt;Q4+0.5,"OVER "&amp;Assumptions!$D$9&amp;"/wk – pace down",IF(R4&gt;Assumptions!$D$106,"Full",IF(AND(Q4&gt;=Assumptions!$D$107,P4&lt;Assumptions!$D$107),"Under "&amp;Assumptions!$D$107&amp;" – release reserve","")))</f>
         <v>Full</v>
       </c>
       <c r="T4" s="26" t="n">
@@ -19060,7 +19066,7 @@
         <v>0.05</v>
       </c>
       <c r="E5" s="24" t="n">
-        <f aca="false">IF(B5&lt;=Funnel!$B$20,D5,0)/SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14)</f>
+        <f aca="false">IF(SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14)&gt;0,IF(B5&lt;=Funnel!$B$20,D5,0)/SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14),0)</f>
         <v>0.0657894736842105</v>
       </c>
       <c r="F5" s="24" t="n">
@@ -19116,7 +19122,7 @@
         <v>0.993298679254963</v>
       </c>
       <c r="S5" s="2" t="str">
-        <f aca="false">IF(P5&gt;Q5+0.5,"OVER "&amp;Assumptions!$D$9&amp;"/wk – pace down",IF(R5&gt;Assumptions!$D$106,"Full",""))</f>
+        <f aca="false">IF(P5&gt;Q5+0.5,"OVER "&amp;Assumptions!$D$9&amp;"/wk – pace down",IF(R5&gt;Assumptions!$D$106,"Full",IF(AND(Q5&gt;=Assumptions!$D$107,P5&lt;Assumptions!$D$107),"Under "&amp;Assumptions!$D$107&amp;" – release reserve","")))</f>
         <v>Full</v>
       </c>
       <c r="T5" s="26" t="n">
@@ -19161,7 +19167,7 @@
         <v>0.2</v>
       </c>
       <c r="E6" s="24" t="n">
-        <f aca="false">IF(B6&lt;=Funnel!$B$20,D6,0)/SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14)</f>
+        <f aca="false">IF(SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14)&gt;0,IF(B6&lt;=Funnel!$B$20,D6,0)/SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14),0)</f>
         <v>0.263157894736842</v>
       </c>
       <c r="F6" s="24" t="n">
@@ -19217,7 +19223,7 @@
         <v>0.956789133298758</v>
       </c>
       <c r="S6" s="2" t="str">
-        <f aca="false">IF(P6&gt;Q6+0.5,"OVER "&amp;Assumptions!$D$9&amp;"/wk – pace down",IF(R6&gt;Assumptions!$D$106,"Full",""))</f>
+        <f aca="false">IF(P6&gt;Q6+0.5,"OVER "&amp;Assumptions!$D$9&amp;"/wk – pace down",IF(R6&gt;Assumptions!$D$106,"Full",IF(AND(Q6&gt;=Assumptions!$D$107,P6&lt;Assumptions!$D$107),"Under "&amp;Assumptions!$D$107&amp;" – release reserve","")))</f>
         <v>Full</v>
       </c>
       <c r="T6" s="26" t="n">
@@ -19262,7 +19268,7 @@
         <v>0.24</v>
       </c>
       <c r="E7" s="24" t="n">
-        <f aca="false">IF(B7&lt;=Funnel!$B$20,D7,0)/SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14)</f>
+        <f aca="false">IF(SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14)&gt;0,IF(B7&lt;=Funnel!$B$20,D7,0)/SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14),0)</f>
         <v>0.315789473684211</v>
       </c>
       <c r="F7" s="24" t="n">
@@ -19318,7 +19324,7 @@
         <v>0.9190560508676</v>
       </c>
       <c r="S7" s="2" t="str">
-        <f aca="false">IF(P7&gt;Q7+0.5,"OVER "&amp;Assumptions!$D$9&amp;"/wk – pace down",IF(R7&gt;Assumptions!$D$106,"Full",""))</f>
+        <f aca="false">IF(P7&gt;Q7+0.5,"OVER "&amp;Assumptions!$D$9&amp;"/wk – pace down",IF(R7&gt;Assumptions!$D$106,"Full",IF(AND(Q7&gt;=Assumptions!$D$107,P7&lt;Assumptions!$D$107),"Under "&amp;Assumptions!$D$107&amp;" – release reserve","")))</f>
         <v>Full</v>
       </c>
       <c r="T7" s="26" t="n">
@@ -19363,7 +19369,7 @@
         <v>0.24</v>
       </c>
       <c r="E8" s="24" t="n">
-        <f aca="false">IF(B8&lt;=Funnel!$B$20,D8,0)/SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14)</f>
+        <f aca="false">IF(SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14)&gt;0,IF(B8&lt;=Funnel!$B$20,D8,0)/SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14),0)</f>
         <v>0.315789473684211</v>
       </c>
       <c r="F8" s="24" t="n">
@@ -19419,7 +19425,7 @@
         <v>0.9190560508676</v>
       </c>
       <c r="S8" s="2" t="str">
-        <f aca="false">IF(P8&gt;Q8+0.5,"OVER "&amp;Assumptions!$D$9&amp;"/wk – pace down",IF(R8&gt;Assumptions!$D$106,"Full",""))</f>
+        <f aca="false">IF(P8&gt;Q8+0.5,"OVER "&amp;Assumptions!$D$9&amp;"/wk – pace down",IF(R8&gt;Assumptions!$D$106,"Full",IF(AND(Q8&gt;=Assumptions!$D$107,P8&lt;Assumptions!$D$107),"Under "&amp;Assumptions!$D$107&amp;" – release reserve","")))</f>
         <v>Full</v>
       </c>
       <c r="T8" s="26" t="n">
@@ -19464,7 +19470,7 @@
         <v>0.24</v>
       </c>
       <c r="E9" s="24" t="n">
-        <f aca="false">IF(B9&lt;=Funnel!$B$20,D9,0)/SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14)</f>
+        <f aca="false">IF(SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14)&gt;0,IF(B9&lt;=Funnel!$B$20,D9,0)/SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14),0)</f>
         <v>0</v>
       </c>
       <c r="F9" s="24" t="n">
@@ -19520,8 +19526,8 @@
         <v>0.783815637475472</v>
       </c>
       <c r="S9" s="2" t="str">
-        <f aca="false">IF(P9&gt;Q9+0.5,"OVER "&amp;Assumptions!$D$9&amp;"/wk – pace down",IF(R9&gt;Assumptions!$D$106,"Full",""))</f>
-        <v/>
+        <f aca="false">IF(P9&gt;Q9+0.5,"OVER "&amp;Assumptions!$D$9&amp;"/wk – pace down",IF(R9&gt;Assumptions!$D$106,"Full",IF(AND(Q9&gt;=Assumptions!$D$107,P9&lt;Assumptions!$D$107),"Under "&amp;Assumptions!$D$107&amp;" – release reserve","")))</f>
+        <v>Under 45 – release reserve</v>
       </c>
       <c r="T9" s="26" t="n">
         <f aca="false">$F$38*(F9*(Budget!$G$21+Budget!$G$22+Budget!$G$23-$F$29-$F$36)+IF(A9-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($X$4:$X$14,A9-ROUNDUP(Funnel!$B$15/7,0))*$F$29+INDEX($Y$4:$Y$14,A9-ROUNDUP(Funnel!$B$15/7,0))*$F$36,0))</f>
@@ -19565,7 +19571,7 @@
         <v>0</v>
       </c>
       <c r="E10" s="24" t="n">
-        <f aca="false">IF(B10&lt;=Funnel!$B$20,D10,0)/SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14)</f>
+        <f aca="false">IF(SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14)&gt;0,IF(B10&lt;=Funnel!$B$20,D10,0)/SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14),0)</f>
         <v>0</v>
       </c>
       <c r="F10" s="24" t="n">
@@ -19621,7 +19627,7 @@
         <v>0</v>
       </c>
       <c r="S10" s="2" t="str">
-        <f aca="false">IF(P10&gt;Q10+0.5,"OVER "&amp;Assumptions!$D$9&amp;"/wk – pace down",IF(R10&gt;Assumptions!$D$106,"Full",""))</f>
+        <f aca="false">IF(P10&gt;Q10+0.5,"OVER "&amp;Assumptions!$D$9&amp;"/wk – pace down",IF(R10&gt;Assumptions!$D$106,"Full",IF(AND(Q10&gt;=Assumptions!$D$107,P10&lt;Assumptions!$D$107),"Under "&amp;Assumptions!$D$107&amp;" – release reserve","")))</f>
         <v/>
       </c>
       <c r="T10" s="26" t="n">
@@ -19666,7 +19672,7 @@
         <v>0</v>
       </c>
       <c r="E11" s="24" t="n">
-        <f aca="false">IF(B11&lt;=Funnel!$B$20,D11,0)/SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14)</f>
+        <f aca="false">IF(SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14)&gt;0,IF(B11&lt;=Funnel!$B$20,D11,0)/SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14),0)</f>
         <v>0</v>
       </c>
       <c r="F11" s="24" t="n">
@@ -19722,7 +19728,7 @@
         <v>0</v>
       </c>
       <c r="S11" s="2" t="str">
-        <f aca="false">IF(P11&gt;Q11+0.5,"OVER "&amp;Assumptions!$D$9&amp;"/wk – pace down",IF(R11&gt;Assumptions!$D$106,"Full",""))</f>
+        <f aca="false">IF(P11&gt;Q11+0.5,"OVER "&amp;Assumptions!$D$9&amp;"/wk – pace down",IF(R11&gt;Assumptions!$D$106,"Full",IF(AND(Q11&gt;=Assumptions!$D$107,P11&lt;Assumptions!$D$107),"Under "&amp;Assumptions!$D$107&amp;" – release reserve","")))</f>
         <v/>
       </c>
       <c r="T11" s="26" t="n">
@@ -19767,7 +19773,7 @@
         <v>0</v>
       </c>
       <c r="E12" s="24" t="n">
-        <f aca="false">IF(B12&lt;=Funnel!$B$20,D12,0)/SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14)</f>
+        <f aca="false">IF(SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14)&gt;0,IF(B12&lt;=Funnel!$B$20,D12,0)/SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14),0)</f>
         <v>0</v>
       </c>
       <c r="F12" s="24" t="n">
@@ -19823,7 +19829,7 @@
         <v>0</v>
       </c>
       <c r="S12" s="2" t="str">
-        <f aca="false">IF(P12&gt;Q12+0.5,"OVER "&amp;Assumptions!$D$9&amp;"/wk – pace down",IF(R12&gt;Assumptions!$D$106,"Full",""))</f>
+        <f aca="false">IF(P12&gt;Q12+0.5,"OVER "&amp;Assumptions!$D$9&amp;"/wk – pace down",IF(R12&gt;Assumptions!$D$106,"Full",IF(AND(Q12&gt;=Assumptions!$D$107,P12&lt;Assumptions!$D$107),"Under "&amp;Assumptions!$D$107&amp;" – release reserve","")))</f>
         <v/>
       </c>
       <c r="T12" s="26" t="n">
@@ -19868,7 +19874,7 @@
         <v>0</v>
       </c>
       <c r="E13" s="24" t="n">
-        <f aca="false">IF(B13&lt;=Funnel!$B$20,D13,0)/SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14)</f>
+        <f aca="false">IF(SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14)&gt;0,IF(B13&lt;=Funnel!$B$20,D13,0)/SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14),0)</f>
         <v>0</v>
       </c>
       <c r="F13" s="24" t="n">
@@ -19924,7 +19930,7 @@
         <v>0</v>
       </c>
       <c r="S13" s="2" t="str">
-        <f aca="false">IF(P13&gt;Q13+0.5,"OVER "&amp;Assumptions!$D$9&amp;"/wk – pace down",IF(R13&gt;Assumptions!$D$106,"Full",""))</f>
+        <f aca="false">IF(P13&gt;Q13+0.5,"OVER "&amp;Assumptions!$D$9&amp;"/wk – pace down",IF(R13&gt;Assumptions!$D$106,"Full",IF(AND(Q13&gt;=Assumptions!$D$107,P13&lt;Assumptions!$D$107),"Under "&amp;Assumptions!$D$107&amp;" – release reserve","")))</f>
         <v/>
       </c>
       <c r="T13" s="26" t="n">
@@ -19969,7 +19975,7 @@
         <v>0</v>
       </c>
       <c r="E14" s="24" t="n">
-        <f aca="false">IF(B14&lt;=Funnel!$B$20,D14,0)/SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14)</f>
+        <f aca="false">IF(SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14)&gt;0,IF(B14&lt;=Funnel!$B$20,D14,0)/SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14),0)</f>
         <v>0</v>
       </c>
       <c r="F14" s="24" t="n">
@@ -20025,7 +20031,7 @@
         <v>0</v>
       </c>
       <c r="S14" s="2" t="str">
-        <f aca="false">IF(P14&gt;Q14+0.5,"OVER "&amp;Assumptions!$D$9&amp;"/wk – pace down",IF(R14&gt;Assumptions!$D$106,"Full",""))</f>
+        <f aca="false">IF(P14&gt;Q14+0.5,"OVER "&amp;Assumptions!$D$9&amp;"/wk – pace down",IF(R14&gt;Assumptions!$D$106,"Full",IF(AND(Q14&gt;=Assumptions!$D$107,P14&lt;Assumptions!$D$107),"Under "&amp;Assumptions!$D$107&amp;" – release reserve","")))</f>
         <v/>
       </c>
       <c r="T14" s="26" t="n">
@@ -20110,7 +20116,7 @@
         <v>322.142857142857</v>
       </c>
       <c r="S15" s="2" t="str">
-        <f aca="false">IF(OR(ABS(D15-1)&gt;0.001,ABS(Y15-1)&gt;0.001),"✗ shares must sum to 100%",IF(ABS(M15-Budget!C9)&gt;1,"✗ weeks ≠ planned spend",IF(ABS(P15-Funnel!O9)&gt;0.5,"✗ qualified ≠ plan",IF(ABS(V15-Budget!C13)&gt;0.5,"✗ signatures ≠ expected hires","✓ ties to plan"))))</f>
+        <f aca="false">IF(Funnel!B19&lt;Assumptions!$D$7,"✗ no application can sign by the deadline (Funnel B19 is before the campaign starts)",IF(AND(Budget!G24&gt;0,Funnel!B20&lt;Assumptions!$D$7),"✗ supervisors cannot apply in time (Funnel B20 is before the campaign starts)",IF(OR(ABS(D15-1)&gt;0.001,ABS(Y15-1)&gt;0.001),"✗ shares must sum to 100%",IF(ABS(M15-Budget!C9)&gt;1,"✗ weeks ≠ planned spend",IF(ABS(P15-Funnel!O9)&gt;0.5,"✗ qualified ≠ plan",IF(ABS(V15-Budget!C13)&gt;0.5,"✗ signatures ≠ expected hires","✓ ties to plan"))))))</f>
         <v>✓ ties to plan</v>
       </c>
       <c r="T15" s="29" t="n">
@@ -20367,7 +20373,7 @@
         <v>702</v>
       </c>
       <c r="F38" s="24" t="n">
-        <f aca="false">MIN(1,Funnel!B22/Funnel!B23)</f>
+        <f aca="false">IF(Funnel!B23&gt;0,MIN(1,Funnel!B22/Funnel!B23),1)</f>
         <v>1</v>
       </c>
     </row>
@@ -20409,6 +20415,12 @@
         <v>712</v>
       </c>
       <c r="L43" s="12" t="s">
+        <v>713</v>
+      </c>
+      <c r="M43" s="12" t="s">
+        <v>714</v>
+      </c>
+      <c r="N43" s="12" t="s">
         <v>432</v>
       </c>
     </row>
@@ -20453,8 +20465,16 @@
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B44,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B44,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$12+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B44,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B44,Channels!$C$5:$C$34,"Supervisors"))*$E$12+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B44)*$X$12</f>
         <v>0</v>
       </c>
-      <c r="L44" s="36" t="n">
-        <f aca="false">SUM(C44:K44)</f>
+      <c r="L44" s="35" t="n">
+        <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B44,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B44,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$13+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B44,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B44,Channels!$C$5:$C$34,"Supervisors"))*$E$13+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B44)*$X$13</f>
+        <v>0</v>
+      </c>
+      <c r="M44" s="35" t="n">
+        <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B44,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B44,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$14+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B44,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B44,Channels!$C$5:$C$34,"Supervisors"))*$E$14+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B44)*$X$14</f>
+        <v>0</v>
+      </c>
+      <c r="N44" s="36" t="n">
+        <f aca="false">SUM(C44:M44)</f>
         <v>0</v>
       </c>
     </row>
@@ -20499,8 +20519,16 @@
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$12+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"Supervisors"))*$E$12+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45)*$X$12</f>
         <v>0</v>
       </c>
-      <c r="L45" s="36" t="n">
-        <f aca="false">SUM(C45:K45)</f>
+      <c r="L45" s="35" t="n">
+        <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$13+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"Supervisors"))*$E$13+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45)*$X$13</f>
+        <v>0</v>
+      </c>
+      <c r="M45" s="35" t="n">
+        <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$14+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"Supervisors"))*$E$14+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45)*$X$14</f>
+        <v>0</v>
+      </c>
+      <c r="N45" s="36" t="n">
+        <f aca="false">SUM(C45:M45)</f>
         <v>3000</v>
       </c>
     </row>
@@ -20545,8 +20573,16 @@
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B46,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B46,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$12+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B46,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B46,Channels!$C$5:$C$34,"Supervisors"))*$E$12+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B46)*$X$12</f>
         <v>0</v>
       </c>
-      <c r="L46" s="36" t="n">
-        <f aca="false">SUM(C46:K46)</f>
+      <c r="L46" s="35" t="n">
+        <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B46,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B46,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$13+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B46,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B46,Channels!$C$5:$C$34,"Supervisors"))*$E$13+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B46)*$X$13</f>
+        <v>0</v>
+      </c>
+      <c r="M46" s="35" t="n">
+        <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B46,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B46,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$14+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B46,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B46,Channels!$C$5:$C$34,"Supervisors"))*$E$14+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B46)*$X$14</f>
+        <v>0</v>
+      </c>
+      <c r="N46" s="36" t="n">
+        <f aca="false">SUM(C46:M46)</f>
         <v>1449</v>
       </c>
     </row>
@@ -20591,8 +20627,16 @@
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$12+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"Supervisors"))*$E$12+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47)*$X$12</f>
         <v>0</v>
       </c>
-      <c r="L47" s="36" t="n">
-        <f aca="false">SUM(C47:K47)</f>
+      <c r="L47" s="35" t="n">
+        <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$13+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"Supervisors"))*$E$13+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47)*$X$13</f>
+        <v>0</v>
+      </c>
+      <c r="M47" s="35" t="n">
+        <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$14+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"Supervisors"))*$E$14+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47)*$X$14</f>
+        <v>0</v>
+      </c>
+      <c r="N47" s="36" t="n">
+        <f aca="false">SUM(C47:M47)</f>
         <v>9523.93851981352</v>
       </c>
     </row>
@@ -20637,8 +20681,16 @@
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B48,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B48,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$12+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B48,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B48,Channels!$C$5:$C$34,"Supervisors"))*$E$12+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B48)*$X$12</f>
         <v>0</v>
       </c>
-      <c r="L48" s="36" t="n">
-        <f aca="false">SUM(C48:K48)</f>
+      <c r="L48" s="35" t="n">
+        <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B48,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B48,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$13+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B48,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B48,Channels!$C$5:$C$34,"Supervisors"))*$E$13+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B48)*$X$13</f>
+        <v>0</v>
+      </c>
+      <c r="M48" s="35" t="n">
+        <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B48,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B48,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$14+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B48,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B48,Channels!$C$5:$C$34,"Supervisors"))*$E$14+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B48)*$X$14</f>
+        <v>0</v>
+      </c>
+      <c r="N48" s="36" t="n">
+        <f aca="false">SUM(C48:M48)</f>
         <v>1500</v>
       </c>
     </row>
@@ -20683,8 +20735,16 @@
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B49,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B49,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$12+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B49,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B49,Channels!$C$5:$C$34,"Supervisors"))*$E$12+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B49)*$X$12</f>
         <v>0</v>
       </c>
-      <c r="L49" s="36" t="n">
-        <f aca="false">SUM(C49:K49)</f>
+      <c r="L49" s="35" t="n">
+        <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B49,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B49,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$13+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B49,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B49,Channels!$C$5:$C$34,"Supervisors"))*$E$13+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B49)*$X$13</f>
+        <v>0</v>
+      </c>
+      <c r="M49" s="35" t="n">
+        <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B49,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B49,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$14+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B49,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B49,Channels!$C$5:$C$34,"Supervisors"))*$E$14+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B49)*$X$14</f>
+        <v>0</v>
+      </c>
+      <c r="N49" s="36" t="n">
+        <f aca="false">SUM(C49:M49)</f>
         <v>4957.14285714286</v>
       </c>
     </row>
@@ -20729,8 +20789,16 @@
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B50)*$Y$12</f>
         <v>0</v>
       </c>
-      <c r="L50" s="36" t="n">
-        <f aca="false">SUM(C50:K50)</f>
+      <c r="L50" s="35" t="n">
+        <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B50)*$Y$13</f>
+        <v>0</v>
+      </c>
+      <c r="M50" s="35" t="n">
+        <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B50)*$Y$14</f>
+        <v>0</v>
+      </c>
+      <c r="N50" s="36" t="n">
+        <f aca="false">SUM(C50:M50)</f>
         <v>350</v>
       </c>
     </row>
@@ -20775,8 +20843,16 @@
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B51,Channels!$C$5:$C$34,"&lt;&gt;Supervisors")*$F$12+SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B51,Channels!$C$5:$C$34,"Supervisors")*$G$12</f>
         <v>1139.69269736842</v>
       </c>
-      <c r="L51" s="36" t="n">
-        <f aca="false">SUM(C51:K51)</f>
+      <c r="L51" s="35" t="n">
+        <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B51,Channels!$C$5:$C$34,"&lt;&gt;Supervisors")*$F$13+SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B51,Channels!$C$5:$C$34,"Supervisors")*$G$13</f>
+        <v>0</v>
+      </c>
+      <c r="M51" s="35" t="n">
+        <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B51,Channels!$C$5:$C$34,"&lt;&gt;Supervisors")*$F$14+SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B51,Channels!$C$5:$C$34,"Supervisors")*$G$14</f>
+        <v>0</v>
+      </c>
+      <c r="N51" s="36" t="n">
+        <f aca="false">SUM(C51:M51)</f>
         <v>4608.060625</v>
       </c>
     </row>
@@ -20821,8 +20897,16 @@
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$12+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"Supervisors"))*$E$12+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52)*$X$12</f>
         <v>0</v>
       </c>
-      <c r="L52" s="36" t="n">
-        <f aca="false">SUM(C52:K52)</f>
+      <c r="L52" s="35" t="n">
+        <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$13+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"Supervisors"))*$E$13+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52)*$X$13</f>
+        <v>0</v>
+      </c>
+      <c r="M52" s="35" t="n">
+        <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$14+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"Supervisors"))*$E$14+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52)*$X$14</f>
+        <v>0</v>
+      </c>
+      <c r="N52" s="36" t="n">
+        <f aca="false">SUM(C52:M52)</f>
         <v>10200</v>
       </c>
     </row>
@@ -20867,8 +20951,16 @@
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$12+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"Supervisors"))*$E$12+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53)*$X$12</f>
         <v>0</v>
       </c>
-      <c r="L53" s="36" t="n">
-        <f aca="false">SUM(C53:K53)</f>
+      <c r="L53" s="35" t="n">
+        <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$13+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"Supervisors"))*$E$13+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53)*$X$13</f>
+        <v>0</v>
+      </c>
+      <c r="M53" s="35" t="n">
+        <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$14+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"Supervisors"))*$E$14+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53)*$X$14</f>
+        <v>0</v>
+      </c>
+      <c r="N53" s="36" t="n">
+        <f aca="false">SUM(C53:M53)</f>
         <v>3145.32619584272</v>
       </c>
     </row>
@@ -20914,12 +21006,20 @@
       </c>
       <c r="L54" s="36" t="n">
         <f aca="false">SUM(L44:L53)</f>
+        <v>0</v>
+      </c>
+      <c r="M54" s="36" t="n">
+        <f aca="false">SUM(M44:M53)</f>
+        <v>0</v>
+      </c>
+      <c r="N54" s="36" t="n">
+        <f aca="false">SUM(N44:N53)</f>
         <v>38733.4681977991</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B55" s="2" t="str">
-        <f aca="false">IF(ABS(L54-Budget!C9)&gt;1,"✗ matrix ≠ planned spend","✓ matrix ties to planned spend")</f>
+        <f aca="false">IF(ABS(N54-Budget!C9)&gt;1,"✗ matrix ≠ planned spend","✓ matrix ties to planned spend")</f>
         <v>✓ matrix ties to planned spend</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Cap budget scenarios by assessment capacity, flag invalid reserve, add 14 edge cases (107/107 pass), deck tweaks
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V2NJtrYy3bzNxqKeiRXJfY
</commit_message>
<xml_diff>
--- a/operation_uptime/Operation_Uptime_Model.xlsx
+++ b/operation_uptime/Operation_Uptime_Model.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1389" uniqueCount="753">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1396" uniqueCount="760">
   <si>
     <t xml:space="preserve">Operation Uptime — model summary (hypothetical Tesla Giga Berlin maintenance hiring)</t>
   </si>
@@ -1933,7 +1933,7 @@
     <t xml:space="preserve">Part 2.5 — What a smaller (or bigger) budget buys</t>
   </si>
   <si>
-    <t xml:space="preserve">Rule when money is cut: drop the most expensive cost-per-hire cells first (across roles), including their test tranches and set-up costs; keep the reserve at the same %. Detail on Scenarios tab.</t>
+    <t xml:space="preserve">Rule when money is cut: drop the most expensive cost-per-hire cells first (across roles), including their test tranches and set-up costs; keep the reserve at the same %. If assessment slots bind (Funnel B24 &gt; 100%), hires are capped by slots, and a cut can even raise hires because it removes low-conversion sources: then re-optimise for hires per assessment slot. Detail on Scenarios tab.</t>
   </si>
   <si>
     <t xml:space="preserve">Budget level</t>
@@ -1990,7 +1990,28 @@
     <t xml:space="preserve">Cut @L4</t>
   </si>
   <si>
+    <t xml:space="preserve">Qualified @L1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Qualified @L2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Qualified @L3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Qualified @L4</t>
+  </si>
+  <si>
     <t xml:space="preserve">Hires by role</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Qualified applicants (before capacity cap)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Capacity factor (assessment slots ÷ qualified, max 1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hires by role are scaled by the capacity factor: if a scenario's qualified applicants exceed the assessment slots, only the share that can be assessed turns into hires (same rule as Budget C13).</t>
   </si>
   <si>
     <t xml:space="preserve">Week-by-week plan: cash out, qualified flow vs 55/week, signatures</t>
@@ -3090,12 +3111,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>715</v>
+        <v>722</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>716</v>
+        <v>723</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3109,67 +3130,67 @@
         <v>288</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>717</v>
+        <v>724</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>718</v>
+        <v>725</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>719</v>
+        <v>726</v>
       </c>
       <c r="G4" s="12" t="s">
-        <v>720</v>
+        <v>727</v>
       </c>
       <c r="H4" s="12" t="s">
-        <v>721</v>
+        <v>728</v>
       </c>
       <c r="I4" s="12" t="s">
-        <v>722</v>
+        <v>729</v>
       </c>
       <c r="J4" s="12" t="s">
-        <v>723</v>
+        <v>730</v>
       </c>
       <c r="K4" s="12" t="s">
-        <v>724</v>
+        <v>731</v>
       </c>
       <c r="L4" s="12" t="s">
-        <v>725</v>
+        <v>732</v>
       </c>
       <c r="M4" s="12" t="s">
-        <v>726</v>
+        <v>733</v>
       </c>
       <c r="N4" s="12" t="s">
-        <v>727</v>
+        <v>734</v>
       </c>
       <c r="O4" s="12" t="s">
-        <v>728</v>
+        <v>735</v>
       </c>
       <c r="P4" s="12" t="s">
-        <v>729</v>
+        <v>736</v>
       </c>
       <c r="Q4" s="12" t="s">
-        <v>730</v>
+        <v>737</v>
       </c>
       <c r="R4" s="12" t="s">
-        <v>731</v>
+        <v>738</v>
       </c>
       <c r="S4" s="12" t="s">
-        <v>732</v>
+        <v>739</v>
       </c>
       <c r="T4" s="12" t="s">
-        <v>733</v>
+        <v>740</v>
       </c>
       <c r="U4" s="12" t="s">
-        <v>734</v>
+        <v>741</v>
       </c>
       <c r="V4" s="12" t="s">
-        <v>735</v>
+        <v>742</v>
       </c>
       <c r="W4" s="12" t="s">
-        <v>736</v>
+        <v>743</v>
       </c>
       <c r="X4" s="12" t="s">
-        <v>737</v>
+        <v>744</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5357,7 +5378,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="22" t="s">
-        <v>738</v>
+        <v>745</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5366,46 +5387,46 @@
         <v>288</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>739</v>
+        <v>746</v>
       </c>
       <c r="D39" s="12" t="s">
-        <v>740</v>
+        <v>747</v>
       </c>
       <c r="E39" s="12" t="s">
-        <v>741</v>
+        <v>748</v>
       </c>
       <c r="F39" s="12" t="s">
-        <v>742</v>
+        <v>749</v>
       </c>
       <c r="G39" s="12" t="s">
-        <v>743</v>
+        <v>750</v>
       </c>
       <c r="H39" s="12" t="s">
-        <v>744</v>
+        <v>751</v>
       </c>
       <c r="I39" s="12" t="s">
-        <v>745</v>
+        <v>752</v>
       </c>
       <c r="J39" s="12" t="s">
-        <v>746</v>
+        <v>753</v>
       </c>
       <c r="K39" s="12" t="s">
-        <v>747</v>
+        <v>754</v>
       </c>
       <c r="L39" s="12" t="s">
-        <v>748</v>
+        <v>755</v>
       </c>
       <c r="M39" s="12" t="s">
-        <v>749</v>
+        <v>756</v>
       </c>
       <c r="N39" s="12" t="s">
-        <v>750</v>
+        <v>757</v>
       </c>
       <c r="O39" s="12" t="s">
         <v>49</v>
       </c>
       <c r="P39" s="12" t="s">
-        <v>751</v>
+        <v>758</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5635,7 +5656,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="9" t="s">
-        <v>752</v>
+        <v>759</v>
       </c>
       <c r="B46" s="9"/>
       <c r="C46" s="9"/>
@@ -16596,7 +16617,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="2" t="str">
-        <f aca="false">IF(ABS(C39-C9)&lt;1,"✓ ties to planned spend","✗ check: channel totals ≠ planned spend")</f>
+        <f aca="false">IF(Assumptions!$D$48&gt;=1,"✗ reserve share must be below 100%",IF(ABS(C39-C9)&lt;1,"✓ ties to planned spend","✗ check: channel totals ≠ planned spend"))</f>
         <v>✓ ties to planned spend</v>
       </c>
     </row>
@@ -16816,7 +16837,7 @@
     <tabColor rgb="FF8EA9DB"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N44"/>
+  <dimension ref="A1:R49"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
@@ -16962,6 +16983,18 @@
       <c r="N7" s="12" t="s">
         <v>626</v>
       </c>
+      <c r="O7" s="12" t="s">
+        <v>653</v>
+      </c>
+      <c r="P7" s="12" t="s">
+        <v>654</v>
+      </c>
+      <c r="Q7" s="12" t="s">
+        <v>655</v>
+      </c>
+      <c r="R7" s="12" t="s">
+        <v>656</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="str">
@@ -17020,6 +17053,22 @@
         <f aca="false">Channels!X5</f>
         <v>0</v>
       </c>
+      <c r="O8" s="26" t="n">
+        <f aca="false">IF(E8&gt;0,F8*Channels!V5/E8,0)</f>
+        <v>12</v>
+      </c>
+      <c r="P8" s="26" t="n">
+        <f aca="false">IF(E8&gt;0,G8*Channels!V5/E8,0)</f>
+        <v>12</v>
+      </c>
+      <c r="Q8" s="26" t="n">
+        <f aca="false">IF(E8&gt;0,H8*Channels!V5/E8,0)</f>
+        <v>12</v>
+      </c>
+      <c r="R8" s="26" t="n">
+        <f aca="false">IF(E8&gt;0,I8*Channels!V5/E8,0)</f>
+        <v>12</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="str">
@@ -17078,6 +17127,22 @@
         <f aca="false">Channels!X6</f>
         <v>0</v>
       </c>
+      <c r="O9" s="26" t="n">
+        <f aca="false">IF(E9&gt;0,F9*Channels!V6/E9,0)</f>
+        <v>36</v>
+      </c>
+      <c r="P9" s="26" t="n">
+        <f aca="false">IF(E9&gt;0,G9*Channels!V6/E9,0)</f>
+        <v>36</v>
+      </c>
+      <c r="Q9" s="26" t="n">
+        <f aca="false">IF(E9&gt;0,H9*Channels!V6/E9,0)</f>
+        <v>36</v>
+      </c>
+      <c r="R9" s="26" t="n">
+        <f aca="false">IF(E9&gt;0,I9*Channels!V6/E9,0)</f>
+        <v>36</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="str">
@@ -17136,6 +17201,22 @@
         <f aca="false">Channels!X7</f>
         <v>0</v>
       </c>
+      <c r="O10" s="26" t="n">
+        <f aca="false">IF(E10&gt;0,F10*Channels!V7/E10,0)</f>
+        <v>8</v>
+      </c>
+      <c r="P10" s="26" t="n">
+        <f aca="false">IF(E10&gt;0,G10*Channels!V7/E10,0)</f>
+        <v>8</v>
+      </c>
+      <c r="Q10" s="26" t="n">
+        <f aca="false">IF(E10&gt;0,H10*Channels!V7/E10,0)</f>
+        <v>8</v>
+      </c>
+      <c r="R10" s="26" t="n">
+        <f aca="false">IF(E10&gt;0,I10*Channels!V7/E10,0)</f>
+        <v>8</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="str">
@@ -17194,6 +17275,22 @@
         <f aca="false">Channels!X8</f>
         <v>0</v>
       </c>
+      <c r="O11" s="26" t="n">
+        <f aca="false">IF(E11&gt;0,F11*Channels!V8/E11,0)</f>
+        <v>4.8</v>
+      </c>
+      <c r="P11" s="26" t="n">
+        <f aca="false">IF(E11&gt;0,G11*Channels!V8/E11,0)</f>
+        <v>4.8</v>
+      </c>
+      <c r="Q11" s="26" t="n">
+        <f aca="false">IF(E11&gt;0,H11*Channels!V8/E11,0)</f>
+        <v>4.8</v>
+      </c>
+      <c r="R11" s="26" t="n">
+        <f aca="false">IF(E11&gt;0,I11*Channels!V8/E11,0)</f>
+        <v>4.8</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="str">
@@ -17252,6 +17349,22 @@
         <f aca="false">Channels!X9</f>
         <v>750</v>
       </c>
+      <c r="O12" s="26" t="n">
+        <f aca="false">IF(E12&gt;0,F12*Channels!V9/E12,0)</f>
+        <v>1.575</v>
+      </c>
+      <c r="P12" s="26" t="n">
+        <f aca="false">IF(E12&gt;0,G12*Channels!V9/E12,0)</f>
+        <v>0</v>
+      </c>
+      <c r="Q12" s="26" t="n">
+        <f aca="false">IF(E12&gt;0,H12*Channels!V9/E12,0)</f>
+        <v>0</v>
+      </c>
+      <c r="R12" s="26" t="n">
+        <f aca="false">IF(E12&gt;0,I12*Channels!V9/E12,0)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="str">
@@ -17310,6 +17423,22 @@
         <f aca="false">Channels!X10</f>
         <v>750</v>
       </c>
+      <c r="O13" s="26" t="n">
+        <f aca="false">IF(E13&gt;0,F13*Channels!V10/E13,0)</f>
+        <v>6.875</v>
+      </c>
+      <c r="P13" s="26" t="n">
+        <f aca="false">IF(E13&gt;0,G13*Channels!V10/E13,0)</f>
+        <v>6.875</v>
+      </c>
+      <c r="Q13" s="26" t="n">
+        <f aca="false">IF(E13&gt;0,H13*Channels!V10/E13,0)</f>
+        <v>6.875</v>
+      </c>
+      <c r="R13" s="26" t="n">
+        <f aca="false">IF(E13&gt;0,I13*Channels!V10/E13,0)</f>
+        <v>6.875</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="str">
@@ -17368,6 +17497,22 @@
         <f aca="false">Channels!X11</f>
         <v>750</v>
       </c>
+      <c r="O14" s="26" t="n">
+        <f aca="false">IF(E14&gt;0,F14*Channels!V11/E14,0)</f>
+        <v>2</v>
+      </c>
+      <c r="P14" s="26" t="n">
+        <f aca="false">IF(E14&gt;0,G14*Channels!V11/E14,0)</f>
+        <v>0</v>
+      </c>
+      <c r="Q14" s="26" t="n">
+        <f aca="false">IF(E14&gt;0,H14*Channels!V11/E14,0)</f>
+        <v>0</v>
+      </c>
+      <c r="R14" s="26" t="n">
+        <f aca="false">IF(E14&gt;0,I14*Channels!V11/E14,0)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="str">
@@ -17426,6 +17571,22 @@
         <f aca="false">Channels!X12</f>
         <v>750</v>
       </c>
+      <c r="O15" s="26" t="n">
+        <f aca="false">IF(E15&gt;0,F15*Channels!V12/E15,0)</f>
+        <v>1.76470588235294</v>
+      </c>
+      <c r="P15" s="26" t="n">
+        <f aca="false">IF(E15&gt;0,G15*Channels!V12/E15,0)</f>
+        <v>0</v>
+      </c>
+      <c r="Q15" s="26" t="n">
+        <f aca="false">IF(E15&gt;0,H15*Channels!V12/E15,0)</f>
+        <v>0</v>
+      </c>
+      <c r="R15" s="26" t="n">
+        <f aca="false">IF(E15&gt;0,I15*Channels!V12/E15,0)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="str">
@@ -17484,6 +17645,22 @@
         <f aca="false">Channels!X13</f>
         <v>1449</v>
       </c>
+      <c r="O16" s="26" t="n">
+        <f aca="false">IF(E16&gt;0,F16*Channels!V13/E16,0)</f>
+        <v>2.8442599067599</v>
+      </c>
+      <c r="P16" s="26" t="n">
+        <f aca="false">IF(E16&gt;0,G16*Channels!V13/E16,0)</f>
+        <v>0</v>
+      </c>
+      <c r="Q16" s="26" t="n">
+        <f aca="false">IF(E16&gt;0,H16*Channels!V13/E16,0)</f>
+        <v>0</v>
+      </c>
+      <c r="R16" s="26" t="n">
+        <f aca="false">IF(E16&gt;0,I16*Channels!V13/E16,0)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="str">
@@ -17542,6 +17719,22 @@
         <f aca="false">Channels!X14</f>
         <v>0</v>
       </c>
+      <c r="O17" s="26" t="n">
+        <f aca="false">IF(E17&gt;0,F17*Channels!V14/E17,0)</f>
+        <v>0</v>
+      </c>
+      <c r="P17" s="26" t="n">
+        <f aca="false">IF(E17&gt;0,G17*Channels!V14/E17,0)</f>
+        <v>0</v>
+      </c>
+      <c r="Q17" s="26" t="n">
+        <f aca="false">IF(E17&gt;0,H17*Channels!V14/E17,0)</f>
+        <v>0</v>
+      </c>
+      <c r="R17" s="26" t="n">
+        <f aca="false">IF(E17&gt;0,I17*Channels!V14/E17,0)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="str">
@@ -17600,6 +17793,22 @@
         <f aca="false">Channels!X15</f>
         <v>0</v>
       </c>
+      <c r="O18" s="26" t="n">
+        <f aca="false">IF(E18&gt;0,F18*Channels!V15/E18,0)</f>
+        <v>0</v>
+      </c>
+      <c r="P18" s="26" t="n">
+        <f aca="false">IF(E18&gt;0,G18*Channels!V15/E18,0)</f>
+        <v>0</v>
+      </c>
+      <c r="Q18" s="26" t="n">
+        <f aca="false">IF(E18&gt;0,H18*Channels!V15/E18,0)</f>
+        <v>0</v>
+      </c>
+      <c r="R18" s="26" t="n">
+        <f aca="false">IF(E18&gt;0,I18*Channels!V15/E18,0)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="str">
@@ -17658,6 +17867,22 @@
         <f aca="false">Channels!X16</f>
         <v>0</v>
       </c>
+      <c r="O19" s="26" t="n">
+        <f aca="false">IF(E19&gt;0,F19*Channels!V16/E19,0)</f>
+        <v>0</v>
+      </c>
+      <c r="P19" s="26" t="n">
+        <f aca="false">IF(E19&gt;0,G19*Channels!V16/E19,0)</f>
+        <v>0</v>
+      </c>
+      <c r="Q19" s="26" t="n">
+        <f aca="false">IF(E19&gt;0,H19*Channels!V16/E19,0)</f>
+        <v>0</v>
+      </c>
+      <c r="R19" s="26" t="n">
+        <f aca="false">IF(E19&gt;0,I19*Channels!V16/E19,0)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="str">
@@ -17716,6 +17941,22 @@
         <f aca="false">Channels!X17</f>
         <v>5148.93851981352</v>
       </c>
+      <c r="O20" s="26" t="n">
+        <f aca="false">IF(E20&gt;0,F20*Channels!V17/E20,0)</f>
+        <v>29.4225058275058</v>
+      </c>
+      <c r="P20" s="26" t="n">
+        <f aca="false">IF(E20&gt;0,G20*Channels!V17/E20,0)</f>
+        <v>29.4225058275058</v>
+      </c>
+      <c r="Q20" s="26" t="n">
+        <f aca="false">IF(E20&gt;0,H20*Channels!V17/E20,0)</f>
+        <v>29.4225058275058</v>
+      </c>
+      <c r="R20" s="26" t="n">
+        <f aca="false">IF(E20&gt;0,I20*Channels!V17/E20,0)</f>
+        <v>29.4225058275058</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="str">
@@ -17774,6 +18015,22 @@
         <f aca="false">Channels!X18</f>
         <v>4375</v>
       </c>
+      <c r="O21" s="26" t="n">
+        <f aca="false">IF(E21&gt;0,F21*Channels!V18/E21,0)</f>
+        <v>20</v>
+      </c>
+      <c r="P21" s="26" t="n">
+        <f aca="false">IF(E21&gt;0,G21*Channels!V18/E21,0)</f>
+        <v>20</v>
+      </c>
+      <c r="Q21" s="26" t="n">
+        <f aca="false">IF(E21&gt;0,H21*Channels!V18/E21,0)</f>
+        <v>20</v>
+      </c>
+      <c r="R21" s="26" t="n">
+        <f aca="false">IF(E21&gt;0,I21*Channels!V18/E21,0)</f>
+        <v>20</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="str">
@@ -17832,6 +18089,22 @@
         <f aca="false">Channels!X19</f>
         <v>750</v>
       </c>
+      <c r="O22" s="26" t="n">
+        <f aca="false">IF(E22&gt;0,F22*Channels!V19/E22,0)</f>
+        <v>2.08333333333333</v>
+      </c>
+      <c r="P22" s="26" t="n">
+        <f aca="false">IF(E22&gt;0,G22*Channels!V19/E22,0)</f>
+        <v>0.0952272283358373</v>
+      </c>
+      <c r="Q22" s="26" t="n">
+        <f aca="false">IF(E22&gt;0,H22*Channels!V19/E22,0)</f>
+        <v>0</v>
+      </c>
+      <c r="R22" s="26" t="n">
+        <f aca="false">IF(E22&gt;0,I22*Channels!V19/E22,0)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="str">
@@ -17890,6 +18163,22 @@
         <f aca="false">Channels!X20</f>
         <v>750</v>
       </c>
+      <c r="O23" s="26" t="n">
+        <f aca="false">IF(E23&gt;0,F23*Channels!V20/E23,0)</f>
+        <v>7.5</v>
+      </c>
+      <c r="P23" s="26" t="n">
+        <f aca="false">IF(E23&gt;0,G23*Channels!V20/E23,0)</f>
+        <v>7.5</v>
+      </c>
+      <c r="Q23" s="26" t="n">
+        <f aca="false">IF(E23&gt;0,H23*Channels!V20/E23,0)</f>
+        <v>7.5</v>
+      </c>
+      <c r="R23" s="26" t="n">
+        <f aca="false">IF(E23&gt;0,I23*Channels!V20/E23,0)</f>
+        <v>7.5</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="str">
@@ -17948,6 +18237,22 @@
         <f aca="false">Channels!X21</f>
         <v>2514.28571428571</v>
       </c>
+      <c r="O24" s="26" t="n">
+        <f aca="false">IF(E24&gt;0,F24*Channels!V21/E24,0)</f>
+        <v>12</v>
+      </c>
+      <c r="P24" s="26" t="n">
+        <f aca="false">IF(E24&gt;0,G24*Channels!V21/E24,0)</f>
+        <v>12</v>
+      </c>
+      <c r="Q24" s="26" t="n">
+        <f aca="false">IF(E24&gt;0,H24*Channels!V21/E24,0)</f>
+        <v>12</v>
+      </c>
+      <c r="R24" s="26" t="n">
+        <f aca="false">IF(E24&gt;0,I24*Channels!V21/E24,0)</f>
+        <v>12</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="str">
@@ -18006,6 +18311,22 @@
         <f aca="false">Channels!X22</f>
         <v>750</v>
       </c>
+      <c r="O25" s="26" t="n">
+        <f aca="false">IF(E25&gt;0,F25*Channels!V22/E25,0)</f>
+        <v>5.96590909090909</v>
+      </c>
+      <c r="P25" s="26" t="n">
+        <f aca="false">IF(E25&gt;0,G25*Channels!V22/E25,0)</f>
+        <v>5.96590909090909</v>
+      </c>
+      <c r="Q25" s="26" t="n">
+        <f aca="false">IF(E25&gt;0,H25*Channels!V22/E25,0)</f>
+        <v>5.96590909090909</v>
+      </c>
+      <c r="R25" s="26" t="n">
+        <f aca="false">IF(E25&gt;0,I25*Channels!V22/E25,0)</f>
+        <v>5.96590909090909</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="str">
@@ -18064,6 +18385,22 @@
         <f aca="false">Channels!X23</f>
         <v>750</v>
       </c>
+      <c r="O26" s="26" t="n">
+        <f aca="false">IF(E26&gt;0,F26*Channels!V23/E26,0)</f>
+        <v>3.57954545454545</v>
+      </c>
+      <c r="P26" s="26" t="n">
+        <f aca="false">IF(E26&gt;0,G26*Channels!V23/E26,0)</f>
+        <v>3.57954545454545</v>
+      </c>
+      <c r="Q26" s="26" t="n">
+        <f aca="false">IF(E26&gt;0,H26*Channels!V23/E26,0)</f>
+        <v>3.57954545454545</v>
+      </c>
+      <c r="R26" s="26" t="n">
+        <f aca="false">IF(E26&gt;0,I26*Channels!V23/E26,0)</f>
+        <v>3.57954545454545</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="str">
@@ -18122,6 +18459,22 @@
         <f aca="false">Channels!X24</f>
         <v>942.857142857143</v>
       </c>
+      <c r="O27" s="26" t="n">
+        <f aca="false">IF(E27&gt;0,F27*Channels!V24/E27,0)</f>
+        <v>3.6</v>
+      </c>
+      <c r="P27" s="26" t="n">
+        <f aca="false">IF(E27&gt;0,G27*Channels!V24/E27,0)</f>
+        <v>3.6</v>
+      </c>
+      <c r="Q27" s="26" t="n">
+        <f aca="false">IF(E27&gt;0,H27*Channels!V24/E27,0)</f>
+        <v>0</v>
+      </c>
+      <c r="R27" s="26" t="n">
+        <f aca="false">IF(E27&gt;0,I27*Channels!V24/E27,0)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="str">
@@ -18180,6 +18533,22 @@
         <f aca="false">Channels!X25</f>
         <v>100</v>
       </c>
+      <c r="O28" s="26" t="n">
+        <f aca="false">IF(E28&gt;0,F28*Channels!V25/E28,0)</f>
+        <v>12</v>
+      </c>
+      <c r="P28" s="26" t="n">
+        <f aca="false">IF(E28&gt;0,G28*Channels!V25/E28,0)</f>
+        <v>12</v>
+      </c>
+      <c r="Q28" s="26" t="n">
+        <f aca="false">IF(E28&gt;0,H28*Channels!V25/E28,0)</f>
+        <v>12</v>
+      </c>
+      <c r="R28" s="26" t="n">
+        <f aca="false">IF(E28&gt;0,I28*Channels!V25/E28,0)</f>
+        <v>12</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="str">
@@ -18238,6 +18607,22 @@
         <f aca="false">Channels!X26</f>
         <v>150</v>
       </c>
+      <c r="O29" s="26" t="n">
+        <f aca="false">IF(E29&gt;0,F29*Channels!V26/E29,0)</f>
+        <v>18</v>
+      </c>
+      <c r="P29" s="26" t="n">
+        <f aca="false">IF(E29&gt;0,G29*Channels!V26/E29,0)</f>
+        <v>18</v>
+      </c>
+      <c r="Q29" s="26" t="n">
+        <f aca="false">IF(E29&gt;0,H29*Channels!V26/E29,0)</f>
+        <v>18</v>
+      </c>
+      <c r="R29" s="26" t="n">
+        <f aca="false">IF(E29&gt;0,I29*Channels!V26/E29,0)</f>
+        <v>18</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="str">
@@ -18296,6 +18681,22 @@
         <f aca="false">Channels!X27</f>
         <v>60</v>
       </c>
+      <c r="O30" s="26" t="n">
+        <f aca="false">IF(E30&gt;0,F30*Channels!V27/E30,0)</f>
+        <v>7.2</v>
+      </c>
+      <c r="P30" s="26" t="n">
+        <f aca="false">IF(E30&gt;0,G30*Channels!V27/E30,0)</f>
+        <v>7.2</v>
+      </c>
+      <c r="Q30" s="26" t="n">
+        <f aca="false">IF(E30&gt;0,H30*Channels!V27/E30,0)</f>
+        <v>7.2</v>
+      </c>
+      <c r="R30" s="26" t="n">
+        <f aca="false">IF(E30&gt;0,I30*Channels!V27/E30,0)</f>
+        <v>7.2</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="str">
@@ -18354,6 +18755,22 @@
         <f aca="false">Channels!X28</f>
         <v>40</v>
       </c>
+      <c r="O31" s="26" t="n">
+        <f aca="false">IF(E31&gt;0,F31*Channels!V28/E31,0)</f>
+        <v>4.8</v>
+      </c>
+      <c r="P31" s="26" t="n">
+        <f aca="false">IF(E31&gt;0,G31*Channels!V28/E31,0)</f>
+        <v>4.8</v>
+      </c>
+      <c r="Q31" s="26" t="n">
+        <f aca="false">IF(E31&gt;0,H31*Channels!V28/E31,0)</f>
+        <v>4.8</v>
+      </c>
+      <c r="R31" s="26" t="n">
+        <f aca="false">IF(E31&gt;0,I31*Channels!V28/E31,0)</f>
+        <v>4.8</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="str">
@@ -18412,6 +18829,22 @@
         <f aca="false">Channels!X29</f>
         <v>4162.640625</v>
       </c>
+      <c r="O32" s="26" t="n">
+        <f aca="false">IF(E32&gt;0,F32*Channels!V29/E32,0)</f>
+        <v>11.25</v>
+      </c>
+      <c r="P32" s="26" t="n">
+        <f aca="false">IF(E32&gt;0,G32*Channels!V29/E32,0)</f>
+        <v>11.25</v>
+      </c>
+      <c r="Q32" s="26" t="n">
+        <f aca="false">IF(E32&gt;0,H32*Channels!V29/E32,0)</f>
+        <v>0</v>
+      </c>
+      <c r="R32" s="26" t="n">
+        <f aca="false">IF(E32&gt;0,I32*Channels!V29/E32,0)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="str">
@@ -18470,6 +18903,22 @@
         <f aca="false">Channels!X30</f>
         <v>0</v>
       </c>
+      <c r="O33" s="26" t="n">
+        <f aca="false">IF(E33&gt;0,F33*Channels!V30/E33,0)</f>
+        <v>0</v>
+      </c>
+      <c r="P33" s="26" t="n">
+        <f aca="false">IF(E33&gt;0,G33*Channels!V30/E33,0)</f>
+        <v>0</v>
+      </c>
+      <c r="Q33" s="26" t="n">
+        <f aca="false">IF(E33&gt;0,H33*Channels!V30/E33,0)</f>
+        <v>0</v>
+      </c>
+      <c r="R33" s="26" t="n">
+        <f aca="false">IF(E33&gt;0,I33*Channels!V30/E33,0)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="str">
@@ -18528,6 +18977,22 @@
         <f aca="false">Channels!X31</f>
         <v>0</v>
       </c>
+      <c r="O34" s="26" t="n">
+        <f aca="false">IF(E34&gt;0,F34*Channels!V31/E34,0)</f>
+        <v>0</v>
+      </c>
+      <c r="P34" s="26" t="n">
+        <f aca="false">IF(E34&gt;0,G34*Channels!V31/E34,0)</f>
+        <v>0</v>
+      </c>
+      <c r="Q34" s="26" t="n">
+        <f aca="false">IF(E34&gt;0,H34*Channels!V31/E34,0)</f>
+        <v>0</v>
+      </c>
+      <c r="R34" s="26" t="n">
+        <f aca="false">IF(E34&gt;0,I34*Channels!V31/E34,0)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="str">
@@ -18586,6 +19051,22 @@
         <f aca="false">Channels!X32</f>
         <v>445.42</v>
       </c>
+      <c r="O35" s="26" t="n">
+        <f aca="false">IF(E35&gt;0,F35*Channels!V32/E35,0)</f>
+        <v>1.44657979133683</v>
+      </c>
+      <c r="P35" s="26" t="n">
+        <f aca="false">IF(E35&gt;0,G35*Channels!V32/E35,0)</f>
+        <v>1.44657979133683</v>
+      </c>
+      <c r="Q35" s="26" t="n">
+        <f aca="false">IF(E35&gt;0,H35*Channels!V32/E35,0)</f>
+        <v>0</v>
+      </c>
+      <c r="R35" s="26" t="n">
+        <f aca="false">IF(E35&gt;0,I35*Channels!V32/E35,0)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="str">
@@ -18644,6 +19125,22 @@
         <f aca="false">Channels!X33</f>
         <v>9000</v>
       </c>
+      <c r="O36" s="26" t="n">
+        <f aca="false">IF(E36&gt;0,F36*Channels!V33/E36,0)</f>
+        <v>45</v>
+      </c>
+      <c r="P36" s="26" t="n">
+        <f aca="false">IF(E36&gt;0,G36*Channels!V33/E36,0)</f>
+        <v>45</v>
+      </c>
+      <c r="Q36" s="26" t="n">
+        <f aca="false">IF(E36&gt;0,H36*Channels!V33/E36,0)</f>
+        <v>42.6447478502902</v>
+      </c>
+      <c r="R36" s="26" t="n">
+        <f aca="false">IF(E36&gt;0,I36*Channels!V33/E36,0)</f>
+        <v>2.26974785029022</v>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="str">
@@ -18702,10 +19199,26 @@
         <f aca="false">Channels!X34</f>
         <v>2745.32619584272</v>
       </c>
+      <c r="O37" s="26" t="n">
+        <f aca="false">IF(E37&gt;0,F37*Channels!V34/E37,0)</f>
+        <v>30.9729109274564</v>
+      </c>
+      <c r="P37" s="26" t="n">
+        <f aca="false">IF(E37&gt;0,G37*Channels!V34/E37,0)</f>
+        <v>30.9729109274564</v>
+      </c>
+      <c r="Q37" s="26" t="n">
+        <f aca="false">IF(E37&gt;0,H37*Channels!V34/E37,0)</f>
+        <v>30.9729109274564</v>
+      </c>
+      <c r="R37" s="26" t="n">
+        <f aca="false">IF(E37&gt;0,I37*Channels!V34/E37,0)</f>
+        <v>30.9729109274564</v>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E38" s="22" t="s">
-        <v>653</v>
+        <v>657</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18713,19 +19226,19 @@
         <v>50</v>
       </c>
       <c r="F39" s="26" t="n">
-        <f aca="false">SUMIFS(F$8:F$37,$B$8:$B$37,$E39)</f>
+        <f aca="false">SUMIFS(F$8:F$37,$B$8:$B$37,$E39)*F$47</f>
         <v>30</v>
       </c>
       <c r="G39" s="26" t="n">
-        <f aca="false">SUMIFS(G$8:G$37,$B$8:$B$37,$E39)</f>
+        <f aca="false">SUMIFS(G$8:G$37,$B$8:$B$37,$E39)*G$47</f>
         <v>27.9384299857171</v>
       </c>
       <c r="H39" s="26" t="n">
-        <f aca="false">SUMIFS(H$8:H$37,$B$8:$B$37,$E39)</f>
+        <f aca="false">SUMIFS(H$8:H$37,$B$8:$B$37,$E39)*H$47</f>
         <v>23.1389080966647</v>
       </c>
       <c r="I39" s="26" t="n">
-        <f aca="false">SUMIFS(I$8:I$37,$B$8:$B$37,$E39)</f>
+        <f aca="false">SUMIFS(I$8:I$37,$B$8:$B$37,$E39)*I$47</f>
         <v>12.7463830966647</v>
       </c>
     </row>
@@ -18734,19 +19247,19 @@
         <v>45</v>
       </c>
       <c r="F40" s="26" t="n">
-        <f aca="false">SUMIFS(F$8:F$37,$B$8:$B$37,$E40)</f>
+        <f aca="false">SUMIFS(F$8:F$37,$B$8:$B$37,$E40)*F$47</f>
         <v>45</v>
       </c>
       <c r="G40" s="26" t="n">
-        <f aca="false">SUMIFS(G$8:G$37,$B$8:$B$37,$E40)</f>
+        <f aca="false">SUMIFS(G$8:G$37,$B$8:$B$37,$E40)*G$47</f>
         <v>45</v>
       </c>
       <c r="H40" s="26" t="n">
-        <f aca="false">SUMIFS(H$8:H$37,$B$8:$B$37,$E40)</f>
+        <f aca="false">SUMIFS(H$8:H$37,$B$8:$B$37,$E40)*H$47</f>
         <v>45</v>
       </c>
       <c r="I40" s="26" t="n">
-        <f aca="false">SUMIFS(I$8:I$37,$B$8:$B$37,$E40)</f>
+        <f aca="false">SUMIFS(I$8:I$37,$B$8:$B$37,$E40)*I$47</f>
         <v>45</v>
       </c>
     </row>
@@ -18755,19 +19268,19 @@
         <v>55</v>
       </c>
       <c r="F41" s="26" t="n">
-        <f aca="false">SUMIFS(F$8:F$37,$B$8:$B$37,$E41)</f>
+        <f aca="false">SUMIFS(F$8:F$37,$B$8:$B$37,$E41)*F$47</f>
         <v>15</v>
       </c>
       <c r="G41" s="26" t="n">
-        <f aca="false">SUMIFS(G$8:G$37,$B$8:$B$37,$E41)</f>
+        <f aca="false">SUMIFS(G$8:G$37,$B$8:$B$37,$E41)*G$47</f>
         <v>14.415</v>
       </c>
       <c r="H41" s="26" t="n">
-        <f aca="false">SUMIFS(H$8:H$37,$B$8:$B$37,$E41)</f>
+        <f aca="false">SUMIFS(H$8:H$37,$B$8:$B$37,$E41)*H$47</f>
         <v>14.415</v>
       </c>
       <c r="I41" s="26" t="n">
-        <f aca="false">SUMIFS(I$8:I$37,$B$8:$B$37,$E41)</f>
+        <f aca="false">SUMIFS(I$8:I$37,$B$8:$B$37,$E41)*I$47</f>
         <v>14.415</v>
       </c>
     </row>
@@ -18776,19 +19289,19 @@
         <v>57</v>
       </c>
       <c r="F42" s="26" t="n">
-        <f aca="false">SUMIFS(F$8:F$37,$B$8:$B$37,$E42)</f>
+        <f aca="false">SUMIFS(F$8:F$37,$B$8:$B$37,$E42)*F$47</f>
         <v>10</v>
       </c>
       <c r="G42" s="26" t="n">
-        <f aca="false">SUMIFS(G$8:G$37,$B$8:$B$37,$E42)</f>
+        <f aca="false">SUMIFS(G$8:G$37,$B$8:$B$37,$E42)*G$47</f>
         <v>9.5275</v>
       </c>
       <c r="H42" s="26" t="n">
-        <f aca="false">SUMIFS(H$8:H$37,$B$8:$B$37,$E42)</f>
+        <f aca="false">SUMIFS(H$8:H$37,$B$8:$B$37,$E42)*H$47</f>
         <v>8.11818</v>
       </c>
       <c r="I42" s="26" t="n">
-        <f aca="false">SUMIFS(I$8:I$37,$B$8:$B$37,$E42)</f>
+        <f aca="false">SUMIFS(I$8:I$37,$B$8:$B$37,$E42)*I$47</f>
         <v>8.11818</v>
       </c>
     </row>
@@ -18832,6 +19345,53 @@
       <c r="I44" s="35" t="n">
         <f aca="false">IF(I43&gt;0,I4/I43,0)</f>
         <v>295.841171574422</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E46" s="2" t="s">
+        <v>658</v>
+      </c>
+      <c r="F46" s="26" t="n">
+        <f aca="false">SUM(O8:O37)</f>
+        <v>290.6797502142</v>
+      </c>
+      <c r="G46" s="26" t="n">
+        <f aca="false">SUM(P8:P37)</f>
+        <v>280.507678320089</v>
+      </c>
+      <c r="H46" s="26" t="n">
+        <f aca="false">SUM(Q8:Q37)</f>
+        <v>261.760619150707</v>
+      </c>
+      <c r="I46" s="26" t="n">
+        <f aca="false">SUM(R8:R37)</f>
+        <v>221.385619150707</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E47" s="2" t="s">
+        <v>659</v>
+      </c>
+      <c r="F47" s="24" t="n">
+        <f aca="false">IF(F46&gt;0,MIN(1,Funnel!$B$22/F46),1)</f>
+        <v>1</v>
+      </c>
+      <c r="G47" s="24" t="n">
+        <f aca="false">IF(G46&gt;0,MIN(1,Funnel!$B$22/G46),1)</f>
+        <v>1</v>
+      </c>
+      <c r="H47" s="24" t="n">
+        <f aca="false">IF(H46&gt;0,MIN(1,Funnel!$B$22/H46),1)</f>
+        <v>1</v>
+      </c>
+      <c r="I47" s="24" t="n">
+        <f aca="false">IF(I46&gt;0,MIN(1,Funnel!$B$22/I46),1)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="407.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="13" t="s">
+        <v>660</v>
       </c>
     </row>
   </sheetData>
@@ -18863,89 +19423,89 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>654</v>
+        <v>661</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>655</v>
+        <v>662</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
-        <v>656</v>
+        <v>663</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>657</v>
+        <v>664</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>658</v>
+        <v>665</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>659</v>
+        <v>666</v>
       </c>
       <c r="E3" s="12" t="s">
-        <v>660</v>
+        <v>667</v>
       </c>
       <c r="F3" s="12" t="s">
-        <v>661</v>
+        <v>668</v>
       </c>
       <c r="G3" s="12" t="s">
-        <v>662</v>
+        <v>669</v>
       </c>
       <c r="H3" s="12" t="s">
-        <v>663</v>
+        <v>670</v>
       </c>
       <c r="I3" s="12" t="s">
-        <v>664</v>
+        <v>671</v>
       </c>
       <c r="J3" s="12" t="s">
-        <v>665</v>
+        <v>672</v>
       </c>
       <c r="K3" s="12" t="s">
-        <v>666</v>
+        <v>673</v>
       </c>
       <c r="L3" s="12" t="s">
-        <v>667</v>
+        <v>674</v>
       </c>
       <c r="M3" s="12" t="s">
-        <v>668</v>
+        <v>675</v>
       </c>
       <c r="N3" s="12" t="s">
-        <v>669</v>
+        <v>676</v>
       </c>
       <c r="O3" s="12" t="s">
-        <v>670</v>
+        <v>677</v>
       </c>
       <c r="P3" s="12" t="s">
-        <v>671</v>
+        <v>678</v>
       </c>
       <c r="Q3" s="12" t="s">
-        <v>672</v>
+        <v>679</v>
       </c>
       <c r="R3" s="12" t="s">
-        <v>673</v>
+        <v>680</v>
       </c>
       <c r="S3" s="12" t="s">
-        <v>674</v>
+        <v>681</v>
       </c>
       <c r="T3" s="12" t="s">
-        <v>675</v>
+        <v>682</v>
       </c>
       <c r="U3" s="12" t="s">
-        <v>676</v>
+        <v>683</v>
       </c>
       <c r="V3" s="12" t="s">
-        <v>677</v>
+        <v>684</v>
       </c>
       <c r="W3" s="12" t="s">
-        <v>678</v>
+        <v>685</v>
       </c>
       <c r="X3" s="12" t="s">
-        <v>679</v>
+        <v>686</v>
       </c>
       <c r="Y3" s="12" t="s">
-        <v>680</v>
+        <v>687</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20116,7 +20676,7 @@
         <v>322.142857142857</v>
       </c>
       <c r="S15" s="2" t="str">
-        <f aca="false">IF(Funnel!B19&lt;Assumptions!$D$7,"✗ no application can sign by the deadline (Funnel B19 is before the campaign starts)",IF(AND(Budget!G24&gt;0,Funnel!B20&lt;Assumptions!$D$7),"✗ supervisors cannot apply in time (Funnel B20 is before the campaign starts)",IF(OR(ABS(D15-1)&gt;0.001,ABS(Y15-1)&gt;0.001),"✗ shares must sum to 100%",IF(ABS(M15-Budget!C9)&gt;1,"✗ weeks ≠ planned spend",IF(ABS(P15-Funnel!O9)&gt;0.5,"✗ qualified ≠ plan",IF(ABS(V15-Budget!C13)&gt;0.5,"✗ signatures ≠ expected hires","✓ ties to plan"))))))</f>
+        <f aca="false">IF(Assumptions!$D$48&gt;=1,"✗ reserve share must be below 100%",IF(Funnel!B19&lt;Assumptions!$D$7,"✗ no application can sign by the deadline (Funnel B19 is before the campaign starts)",IF(AND(Budget!G24&gt;0,Funnel!B20&lt;Assumptions!$D$7),"✗ supervisors cannot apply in time (Funnel B20 is before the campaign starts)",IF(OR(ABS(D15-1)&gt;0.001,ABS(Y15-1)&gt;0.001),"✗ shares must sum to 100%",IF(ABS(M15-Budget!C9)&gt;1,"✗ weeks ≠ planned spend",IF(ABS(P15-Funnel!O9)&gt;0.5,"✗ qualified ≠ plan",IF(ABS(V15-Budget!C13)&gt;0.5,"✗ signatures ≠ expected hires","✓ ties to plan")))))))</f>
         <v>✓ ties to plan</v>
       </c>
       <c r="T15" s="29" t="n">
@@ -20142,7 +20702,7 @@
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="B16" s="9"/>
       <c r="C16" s="9"/>
@@ -20194,12 +20754,12 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="22" t="s">
-        <v>682</v>
+        <v>689</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="2" t="s">
-        <v>683</v>
+        <v>690</v>
       </c>
       <c r="F19" s="35" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot",Channels!$B$5:$B$34,"&lt;&gt;I1b Employee referral sprint (bonus on hire)",Channels!$B$5:$B$34,"&lt;&gt;I1a Talent rediscovery (past applicants in ATS)")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
@@ -20208,7 +20768,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="2" t="s">
-        <v>684</v>
+        <v>691</v>
       </c>
       <c r="F20" s="35" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot",Channels!$B$5:$B$34,"&lt;&gt;I1b Employee referral sprint (bonus on hire)",Channels!$B$5:$B$34,"&lt;&gt;I1a Talent rediscovery (past applicants in ATS)")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$C$5:$C$34,"Supervisors")</f>
@@ -20217,7 +20777,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="2" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="F21" s="35" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$E$5:$E$34,"Slot")</f>
@@ -20226,7 +20786,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="2" t="s">
-        <v>686</v>
+        <v>693</v>
       </c>
       <c r="F22" s="35" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,"I1b Employee referral sprint (bonus on hire)",Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
@@ -20235,7 +20795,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="2" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F23" s="35" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,"I1b Employee referral sprint (bonus on hire)",Channels!$C$5:$C$34,"Supervisors")</f>
@@ -20244,7 +20804,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="2" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
       <c r="F24" s="35" t="n">
         <f aca="false">SUM(Channels!$Z$5:$Z$34)</f>
@@ -20253,7 +20813,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="2" t="s">
-        <v>689</v>
+        <v>696</v>
       </c>
       <c r="F25" s="26" t="n">
         <f aca="false">SUMIFS(Channels!$AF$5:$AF$34,Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
@@ -20262,7 +20822,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="2" t="s">
-        <v>690</v>
+        <v>697</v>
       </c>
       <c r="F26" s="26" t="n">
         <f aca="false">SUMIFS(Channels!$AF$5:$AF$34,Channels!$C$5:$C$34,"Supervisors")</f>
@@ -20271,7 +20831,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="2" t="s">
-        <v>691</v>
+        <v>698</v>
       </c>
       <c r="F27" s="26" t="n">
         <f aca="false">SUMIFS(Channels!$AE$5:$AE$34,Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
@@ -20280,7 +20840,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="2" t="s">
-        <v>692</v>
+        <v>699</v>
       </c>
       <c r="F28" s="26" t="n">
         <f aca="false">SUMIFS(Channels!$AE$5:$AE$34,Channels!$C$5:$C$34,"Supervisors")</f>
@@ -20289,7 +20849,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="2" t="s">
-        <v>693</v>
+        <v>700</v>
       </c>
       <c r="F29" s="26" t="n">
         <f aca="false">SUMIFS(Channels!$AG$5:$AG$34,Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
@@ -20298,7 +20858,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="2" t="s">
-        <v>694</v>
+        <v>701</v>
       </c>
       <c r="F30" s="26" t="n">
         <f aca="false">SUMIFS(Channels!$AG$5:$AG$34,Channels!$C$5:$C$34,"Supervisors")</f>
@@ -20307,7 +20867,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="2" t="s">
-        <v>695</v>
+        <v>702</v>
       </c>
       <c r="F31" s="35" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)")</f>
@@ -20316,7 +20876,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="2" t="s">
-        <v>696</v>
+        <v>703</v>
       </c>
       <c r="F32" s="26" t="n">
         <f aca="false">SUMIFS(Channels!$V$5:$V$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)",Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
@@ -20325,7 +20885,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="2" t="s">
-        <v>697</v>
+        <v>704</v>
       </c>
       <c r="F33" s="26" t="n">
         <f aca="false">SUMIFS(Channels!$V$5:$V$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)",Channels!$C$5:$C$34,"Supervisors")</f>
@@ -20334,7 +20894,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="2" t="s">
-        <v>698</v>
+        <v>705</v>
       </c>
       <c r="F34" s="26" t="n">
         <f aca="false">SUMIFS(Channels!$W$5:$W$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)",Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
@@ -20343,7 +20903,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="2" t="s">
-        <v>699</v>
+        <v>706</v>
       </c>
       <c r="F35" s="26" t="n">
         <f aca="false">SUMIFS(Channels!$W$5:$W$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)",Channels!$C$5:$C$34,"Supervisors")</f>
@@ -20352,7 +20912,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="2" t="s">
-        <v>700</v>
+        <v>707</v>
       </c>
       <c r="F36" s="26" t="n">
         <f aca="false">SUMIFS(Channels!$U$5:$U$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)",Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
@@ -20361,7 +20921,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="2" t="s">
-        <v>701</v>
+        <v>708</v>
       </c>
       <c r="F37" s="26" t="n">
         <f aca="false">SUMIFS(Channels!$U$5:$U$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)",Channels!$C$5:$C$34,"Supervisors")</f>
@@ -20370,7 +20930,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="2" t="s">
-        <v>702</v>
+        <v>709</v>
       </c>
       <c r="F38" s="24" t="n">
         <f aca="false">IF(Funnel!B23&gt;0,MIN(1,Funnel!B22/Funnel!B23),1)</f>
@@ -20379,7 +20939,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="22" t="s">
-        <v>703</v>
+        <v>710</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -20388,37 +20948,37 @@
         <v>287</v>
       </c>
       <c r="C43" s="12" t="s">
-        <v>704</v>
+        <v>711</v>
       </c>
       <c r="D43" s="12" t="s">
-        <v>705</v>
+        <v>712</v>
       </c>
       <c r="E43" s="12" t="s">
-        <v>706</v>
+        <v>713</v>
       </c>
       <c r="F43" s="12" t="s">
-        <v>707</v>
+        <v>714</v>
       </c>
       <c r="G43" s="12" t="s">
-        <v>708</v>
+        <v>715</v>
       </c>
       <c r="H43" s="12" t="s">
-        <v>709</v>
+        <v>716</v>
       </c>
       <c r="I43" s="12" t="s">
-        <v>710</v>
+        <v>717</v>
       </c>
       <c r="J43" s="12" t="s">
-        <v>711</v>
+        <v>718</v>
       </c>
       <c r="K43" s="12" t="s">
-        <v>712</v>
+        <v>719</v>
       </c>
       <c r="L43" s="12" t="s">
-        <v>713</v>
+        <v>720</v>
       </c>
       <c r="M43" s="12" t="s">
-        <v>714</v>
+        <v>721</v>
       </c>
       <c r="N43" s="12" t="s">
         <v>432</v>

</xml_diff>

<commit_message>
Skip tests for roles with no openings, explicit week-6 flag, guard edge divisions; 120/120 tests pass
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V2NJtrYy3bzNxqKeiRXJfY
</commit_message>
<xml_diff>
--- a/operation_uptime/Operation_Uptime_Model.xlsx
+++ b/operation_uptime/Operation_Uptime_Model.xlsx
@@ -1729,7 +1729,7 @@
     <t xml:space="preserve">Allocation logic: within each role, channels are filled in order of cost per hire (media at full capacity + fixed costs, ÷ hire capacity) up to their capacity until hires = openings. Polish cap enforced in hire capacity. Slots bought in whole 30-day ads.</t>
   </si>
   <si>
-    <t xml:space="preserve">Every paid CPC/CPA cell first gets a test tranche (B2) in weeks 1–2; its applicants and hires are counted (cols AE–AG). The allocation then fills only the remaining need (col T) from remaining capacity (col AH).</t>
+    <t xml:space="preserve">Every paid CPC/CPA cell for a role with openings first gets a test tranche (B2) in weeks 1–2; its applicants and hires are counted (cols AE–AG). The allocation then fills only the remaining need (col T) from remaining capacity (col AH).</t>
   </si>
   <si>
     <t xml:space="preserve">Type</t>
@@ -11813,7 +11813,7 @@
         <v>0</v>
       </c>
       <c r="Z5" s="35" t="n">
-        <f aca="false">IF(AND(D5="Channel",OR(E5="CPC",E5="CPA")),MIN(Assumptions!$D$49,J5*H5),0)</f>
+        <f aca="false">IF(AND(D5="Channel",OR(E5="CPC",E5="CPA"),INDEX(Funnel!$B$5:$B$8,MATCH(C5,Funnel!$A$5:$A$8,0))&gt;0),MIN(Assumptions!$D$49,J5*H5),0)</f>
         <v>0</v>
       </c>
       <c r="AA5" s="35" t="n">
@@ -11954,7 +11954,7 @@
         <v>0</v>
       </c>
       <c r="Z6" s="35" t="n">
-        <f aca="false">IF(AND(D6="Channel",OR(E6="CPC",E6="CPA")),MIN(Assumptions!$D$49,J6*H6),0)</f>
+        <f aca="false">IF(AND(D6="Channel",OR(E6="CPC",E6="CPA"),INDEX(Funnel!$B$5:$B$8,MATCH(C6,Funnel!$A$5:$A$8,0))&gt;0),MIN(Assumptions!$D$49,J6*H6),0)</f>
         <v>0</v>
       </c>
       <c r="AA6" s="35" t="n">
@@ -12095,7 +12095,7 @@
         <v>0</v>
       </c>
       <c r="Z7" s="35" t="n">
-        <f aca="false">IF(AND(D7="Channel",OR(E7="CPC",E7="CPA")),MIN(Assumptions!$D$49,J7*H7),0)</f>
+        <f aca="false">IF(AND(D7="Channel",OR(E7="CPC",E7="CPA"),INDEX(Funnel!$B$5:$B$8,MATCH(C7,Funnel!$A$5:$A$8,0))&gt;0),MIN(Assumptions!$D$49,J7*H7),0)</f>
         <v>0</v>
       </c>
       <c r="AA7" s="35" t="n">
@@ -12236,7 +12236,7 @@
         <v>0</v>
       </c>
       <c r="Z8" s="35" t="n">
-        <f aca="false">IF(AND(D8="Channel",OR(E8="CPC",E8="CPA")),MIN(Assumptions!$D$49,J8*H8),0)</f>
+        <f aca="false">IF(AND(D8="Channel",OR(E8="CPC",E8="CPA"),INDEX(Funnel!$B$5:$B$8,MATCH(C8,Funnel!$A$5:$A$8,0))&gt;0),MIN(Assumptions!$D$49,J8*H8),0)</f>
         <v>0</v>
       </c>
       <c r="AA8" s="35" t="n">
@@ -12377,7 +12377,7 @@
         <v>0</v>
       </c>
       <c r="Z9" s="35" t="n">
-        <f aca="false">IF(AND(D9="Channel",OR(E9="CPC",E9="CPA")),MIN(Assumptions!$D$49,J9*H9),0)</f>
+        <f aca="false">IF(AND(D9="Channel",OR(E9="CPC",E9="CPA"),INDEX(Funnel!$B$5:$B$8,MATCH(C9,Funnel!$A$5:$A$8,0))&gt;0),MIN(Assumptions!$D$49,J9*H9),0)</f>
         <v>750</v>
       </c>
       <c r="AA9" s="35" t="n">
@@ -12518,7 +12518,7 @@
         <v>0</v>
       </c>
       <c r="Z10" s="35" t="n">
-        <f aca="false">IF(AND(D10="Channel",OR(E10="CPC",E10="CPA")),MIN(Assumptions!$D$49,J10*H10),0)</f>
+        <f aca="false">IF(AND(D10="Channel",OR(E10="CPC",E10="CPA"),INDEX(Funnel!$B$5:$B$8,MATCH(C10,Funnel!$A$5:$A$8,0))&gt;0),MIN(Assumptions!$D$49,J10*H10),0)</f>
         <v>750</v>
       </c>
       <c r="AA10" s="35" t="n">
@@ -12659,7 +12659,7 @@
         <v>0</v>
       </c>
       <c r="Z11" s="35" t="n">
-        <f aca="false">IF(AND(D11="Channel",OR(E11="CPC",E11="CPA")),MIN(Assumptions!$D$49,J11*H11),0)</f>
+        <f aca="false">IF(AND(D11="Channel",OR(E11="CPC",E11="CPA"),INDEX(Funnel!$B$5:$B$8,MATCH(C11,Funnel!$A$5:$A$8,0))&gt;0),MIN(Assumptions!$D$49,J11*H11),0)</f>
         <v>750</v>
       </c>
       <c r="AA11" s="35" t="n">
@@ -12800,7 +12800,7 @@
         <v>0</v>
       </c>
       <c r="Z12" s="35" t="n">
-        <f aca="false">IF(AND(D12="Channel",OR(E12="CPC",E12="CPA")),MIN(Assumptions!$D$49,J12*H12),0)</f>
+        <f aca="false">IF(AND(D12="Channel",OR(E12="CPC",E12="CPA"),INDEX(Funnel!$B$5:$B$8,MATCH(C12,Funnel!$A$5:$A$8,0))&gt;0),MIN(Assumptions!$D$49,J12*H12),0)</f>
         <v>750</v>
       </c>
       <c r="AA12" s="35" t="n">
@@ -12941,7 +12941,7 @@
         <v>0</v>
       </c>
       <c r="Z13" s="35" t="n">
-        <f aca="false">IF(AND(D13="Channel",OR(E13="CPC",E13="CPA")),MIN(Assumptions!$D$49,J13*H13),0)</f>
+        <f aca="false">IF(AND(D13="Channel",OR(E13="CPC",E13="CPA"),INDEX(Funnel!$B$5:$B$8,MATCH(C13,Funnel!$A$5:$A$8,0))&gt;0),MIN(Assumptions!$D$49,J13*H13),0)</f>
         <v>0</v>
       </c>
       <c r="AA13" s="35" t="n">
@@ -13082,7 +13082,7 @@
         <v>0</v>
       </c>
       <c r="Z14" s="35" t="n">
-        <f aca="false">IF(AND(D14="Channel",OR(E14="CPC",E14="CPA")),MIN(Assumptions!$D$49,J14*H14),0)</f>
+        <f aca="false">IF(AND(D14="Channel",OR(E14="CPC",E14="CPA"),INDEX(Funnel!$B$5:$B$8,MATCH(C14,Funnel!$A$5:$A$8,0))&gt;0),MIN(Assumptions!$D$49,J14*H14),0)</f>
         <v>0</v>
       </c>
       <c r="AA14" s="35" t="n">
@@ -13223,7 +13223,7 @@
         <v>0</v>
       </c>
       <c r="Z15" s="35" t="n">
-        <f aca="false">IF(AND(D15="Channel",OR(E15="CPC",E15="CPA")),MIN(Assumptions!$D$49,J15*H15),0)</f>
+        <f aca="false">IF(AND(D15="Channel",OR(E15="CPC",E15="CPA"),INDEX(Funnel!$B$5:$B$8,MATCH(C15,Funnel!$A$5:$A$8,0))&gt;0),MIN(Assumptions!$D$49,J15*H15),0)</f>
         <v>0</v>
       </c>
       <c r="AA15" s="35" t="n">
@@ -13364,7 +13364,7 @@
         <v>0</v>
       </c>
       <c r="Z16" s="35" t="n">
-        <f aca="false">IF(AND(D16="Channel",OR(E16="CPC",E16="CPA")),MIN(Assumptions!$D$49,J16*H16),0)</f>
+        <f aca="false">IF(AND(D16="Channel",OR(E16="CPC",E16="CPA"),INDEX(Funnel!$B$5:$B$8,MATCH(C16,Funnel!$A$5:$A$8,0))&gt;0),MIN(Assumptions!$D$49,J16*H16),0)</f>
         <v>0</v>
       </c>
       <c r="AA16" s="35" t="n">
@@ -13505,7 +13505,7 @@
         <v>0</v>
       </c>
       <c r="Z17" s="35" t="n">
-        <f aca="false">IF(AND(D17="Channel",OR(E17="CPC",E17="CPA")),MIN(Assumptions!$D$49,J17*H17),0)</f>
+        <f aca="false">IF(AND(D17="Channel",OR(E17="CPC",E17="CPA"),INDEX(Funnel!$B$5:$B$8,MATCH(C17,Funnel!$A$5:$A$8,0))&gt;0),MIN(Assumptions!$D$49,J17*H17),0)</f>
         <v>750</v>
       </c>
       <c r="AA17" s="35" t="n">
@@ -13646,7 +13646,7 @@
         <v>0</v>
       </c>
       <c r="Z18" s="35" t="n">
-        <f aca="false">IF(AND(D18="Channel",OR(E18="CPC",E18="CPA")),MIN(Assumptions!$D$49,J18*H18),0)</f>
+        <f aca="false">IF(AND(D18="Channel",OR(E18="CPC",E18="CPA"),INDEX(Funnel!$B$5:$B$8,MATCH(C18,Funnel!$A$5:$A$8,0))&gt;0),MIN(Assumptions!$D$49,J18*H18),0)</f>
         <v>750</v>
       </c>
       <c r="AA18" s="35" t="n">
@@ -13787,7 +13787,7 @@
         <v>0</v>
       </c>
       <c r="Z19" s="35" t="n">
-        <f aca="false">IF(AND(D19="Channel",OR(E19="CPC",E19="CPA")),MIN(Assumptions!$D$49,J19*H19),0)</f>
+        <f aca="false">IF(AND(D19="Channel",OR(E19="CPC",E19="CPA"),INDEX(Funnel!$B$5:$B$8,MATCH(C19,Funnel!$A$5:$A$8,0))&gt;0),MIN(Assumptions!$D$49,J19*H19),0)</f>
         <v>750</v>
       </c>
       <c r="AA19" s="35" t="n">
@@ -13928,7 +13928,7 @@
         <v>0</v>
       </c>
       <c r="Z20" s="35" t="n">
-        <f aca="false">IF(AND(D20="Channel",OR(E20="CPC",E20="CPA")),MIN(Assumptions!$D$49,J20*H20),0)</f>
+        <f aca="false">IF(AND(D20="Channel",OR(E20="CPC",E20="CPA"),INDEX(Funnel!$B$5:$B$8,MATCH(C20,Funnel!$A$5:$A$8,0))&gt;0),MIN(Assumptions!$D$49,J20*H20),0)</f>
         <v>750</v>
       </c>
       <c r="AA20" s="35" t="n">
@@ -14069,7 +14069,7 @@
         <v>0</v>
       </c>
       <c r="Z21" s="35" t="n">
-        <f aca="false">IF(AND(D21="Channel",OR(E21="CPC",E21="CPA")),MIN(Assumptions!$D$49,J21*H21),0)</f>
+        <f aca="false">IF(AND(D21="Channel",OR(E21="CPC",E21="CPA"),INDEX(Funnel!$B$5:$B$8,MATCH(C21,Funnel!$A$5:$A$8,0))&gt;0),MIN(Assumptions!$D$49,J21*H21),0)</f>
         <v>750</v>
       </c>
       <c r="AA21" s="35" t="n">
@@ -14210,7 +14210,7 @@
         <v>0</v>
       </c>
       <c r="Z22" s="35" t="n">
-        <f aca="false">IF(AND(D22="Channel",OR(E22="CPC",E22="CPA")),MIN(Assumptions!$D$49,J22*H22),0)</f>
+        <f aca="false">IF(AND(D22="Channel",OR(E22="CPC",E22="CPA"),INDEX(Funnel!$B$5:$B$8,MATCH(C22,Funnel!$A$5:$A$8,0))&gt;0),MIN(Assumptions!$D$49,J22*H22),0)</f>
         <v>750</v>
       </c>
       <c r="AA22" s="35" t="n">
@@ -14351,7 +14351,7 @@
         <v>0</v>
       </c>
       <c r="Z23" s="35" t="n">
-        <f aca="false">IF(AND(D23="Channel",OR(E23="CPC",E23="CPA")),MIN(Assumptions!$D$49,J23*H23),0)</f>
+        <f aca="false">IF(AND(D23="Channel",OR(E23="CPC",E23="CPA"),INDEX(Funnel!$B$5:$B$8,MATCH(C23,Funnel!$A$5:$A$8,0))&gt;0),MIN(Assumptions!$D$49,J23*H23),0)</f>
         <v>750</v>
       </c>
       <c r="AA23" s="35" t="n">
@@ -14492,7 +14492,7 @@
         <v>0</v>
       </c>
       <c r="Z24" s="35" t="n">
-        <f aca="false">IF(AND(D24="Channel",OR(E24="CPC",E24="CPA")),MIN(Assumptions!$D$49,J24*H24),0)</f>
+        <f aca="false">IF(AND(D24="Channel",OR(E24="CPC",E24="CPA"),INDEX(Funnel!$B$5:$B$8,MATCH(C24,Funnel!$A$5:$A$8,0))&gt;0),MIN(Assumptions!$D$49,J24*H24),0)</f>
         <v>750</v>
       </c>
       <c r="AA24" s="35" t="n">
@@ -14626,7 +14626,7 @@
         <v>0</v>
       </c>
       <c r="Z25" s="35" t="n">
-        <f aca="false">IF(AND(D25="Channel",OR(E25="CPC",E25="CPA")),MIN(Assumptions!$D$49,J25*H25),0)</f>
+        <f aca="false">IF(AND(D25="Channel",OR(E25="CPC",E25="CPA"),INDEX(Funnel!$B$5:$B$8,MATCH(C25,Funnel!$A$5:$A$8,0))&gt;0),MIN(Assumptions!$D$49,J25*H25),0)</f>
         <v>0</v>
       </c>
       <c r="AA25" s="35" t="n">
@@ -14760,7 +14760,7 @@
         <v>0</v>
       </c>
       <c r="Z26" s="35" t="n">
-        <f aca="false">IF(AND(D26="Channel",OR(E26="CPC",E26="CPA")),MIN(Assumptions!$D$49,J26*H26),0)</f>
+        <f aca="false">IF(AND(D26="Channel",OR(E26="CPC",E26="CPA"),INDEX(Funnel!$B$5:$B$8,MATCH(C26,Funnel!$A$5:$A$8,0))&gt;0),MIN(Assumptions!$D$49,J26*H26),0)</f>
         <v>0</v>
       </c>
       <c r="AA26" s="35" t="n">
@@ -14894,7 +14894,7 @@
         <v>0</v>
       </c>
       <c r="Z27" s="35" t="n">
-        <f aca="false">IF(AND(D27="Channel",OR(E27="CPC",E27="CPA")),MIN(Assumptions!$D$49,J27*H27),0)</f>
+        <f aca="false">IF(AND(D27="Channel",OR(E27="CPC",E27="CPA"),INDEX(Funnel!$B$5:$B$8,MATCH(C27,Funnel!$A$5:$A$8,0))&gt;0),MIN(Assumptions!$D$49,J27*H27),0)</f>
         <v>0</v>
       </c>
       <c r="AA27" s="35" t="n">
@@ -15028,7 +15028,7 @@
         <v>0</v>
       </c>
       <c r="Z28" s="35" t="n">
-        <f aca="false">IF(AND(D28="Channel",OR(E28="CPC",E28="CPA")),MIN(Assumptions!$D$49,J28*H28),0)</f>
+        <f aca="false">IF(AND(D28="Channel",OR(E28="CPC",E28="CPA"),INDEX(Funnel!$B$5:$B$8,MATCH(C28,Funnel!$A$5:$A$8,0))&gt;0),MIN(Assumptions!$D$49,J28*H28),0)</f>
         <v>0</v>
       </c>
       <c r="AA28" s="35" t="n">
@@ -15162,7 +15162,7 @@
         <v>0</v>
       </c>
       <c r="Z29" s="35" t="n">
-        <f aca="false">IF(AND(D29="Channel",OR(E29="CPC",E29="CPA")),MIN(Assumptions!$D$49,J29*H29),0)</f>
+        <f aca="false">IF(AND(D29="Channel",OR(E29="CPC",E29="CPA"),INDEX(Funnel!$B$5:$B$8,MATCH(C29,Funnel!$A$5:$A$8,0))&gt;0),MIN(Assumptions!$D$49,J29*H29),0)</f>
         <v>0</v>
       </c>
       <c r="AA29" s="35" t="n">
@@ -15296,7 +15296,7 @@
         <v>0</v>
       </c>
       <c r="Z30" s="35" t="n">
-        <f aca="false">IF(AND(D30="Channel",OR(E30="CPC",E30="CPA")),MIN(Assumptions!$D$49,J30*H30),0)</f>
+        <f aca="false">IF(AND(D30="Channel",OR(E30="CPC",E30="CPA"),INDEX(Funnel!$B$5:$B$8,MATCH(C30,Funnel!$A$5:$A$8,0))&gt;0),MIN(Assumptions!$D$49,J30*H30),0)</f>
         <v>0</v>
       </c>
       <c r="AA30" s="35" t="n">
@@ -15430,7 +15430,7 @@
         <v>0</v>
       </c>
       <c r="Z31" s="35" t="n">
-        <f aca="false">IF(AND(D31="Channel",OR(E31="CPC",E31="CPA")),MIN(Assumptions!$D$49,J31*H31),0)</f>
+        <f aca="false">IF(AND(D31="Channel",OR(E31="CPC",E31="CPA"),INDEX(Funnel!$B$5:$B$8,MATCH(C31,Funnel!$A$5:$A$8,0))&gt;0),MIN(Assumptions!$D$49,J31*H31),0)</f>
         <v>0</v>
       </c>
       <c r="AA31" s="35" t="n">
@@ -15564,7 +15564,7 @@
         <v>0</v>
       </c>
       <c r="Z32" s="35" t="n">
-        <f aca="false">IF(AND(D32="Channel",OR(E32="CPC",E32="CPA")),MIN(Assumptions!$D$49,J32*H32),0)</f>
+        <f aca="false">IF(AND(D32="Channel",OR(E32="CPC",E32="CPA"),INDEX(Funnel!$B$5:$B$8,MATCH(C32,Funnel!$A$5:$A$8,0))&gt;0),MIN(Assumptions!$D$49,J32*H32),0)</f>
         <v>0</v>
       </c>
       <c r="AA32" s="35" t="n">
@@ -15698,7 +15698,7 @@
         <v>1200</v>
       </c>
       <c r="Z33" s="35" t="n">
-        <f aca="false">IF(AND(D33="Channel",OR(E33="CPC",E33="CPA")),MIN(Assumptions!$D$49,J33*H33),0)</f>
+        <f aca="false">IF(AND(D33="Channel",OR(E33="CPC",E33="CPA"),INDEX(Funnel!$B$5:$B$8,MATCH(C33,Funnel!$A$5:$A$8,0))&gt;0),MIN(Assumptions!$D$49,J33*H33),0)</f>
         <v>0</v>
       </c>
       <c r="AA33" s="35" t="n">
@@ -15832,7 +15832,7 @@
         <v>400</v>
       </c>
       <c r="Z34" s="35" t="n">
-        <f aca="false">IF(AND(D34="Channel",OR(E34="CPC",E34="CPA")),MIN(Assumptions!$D$49,J34*H34),0)</f>
+        <f aca="false">IF(AND(D34="Channel",OR(E34="CPC",E34="CPA"),INDEX(Funnel!$B$5:$B$8,MATCH(C34,Funnel!$A$5:$A$8,0))&gt;0),MIN(Assumptions!$D$49,J34*H34),0)</f>
         <v>0</v>
       </c>
       <c r="AA34" s="35" t="n">
@@ -15917,7 +15917,7 @@
         <v>38733.4681977991</v>
       </c>
       <c r="AB35" s="36" t="n">
-        <f aca="false">(X35+Y35)/U35</f>
+        <f aca="false">IF(U35&gt;0,(X35+Y35)/U35,0)</f>
         <v>387.334681977991</v>
       </c>
       <c r="AE35" s="27" t="n">
@@ -16132,7 +16132,7 @@
         <v>620</v>
       </c>
       <c r="C12" s="4" t="n">
-        <f aca="false">ROUNDUP(C11/Assumptions!$D$51,0)*Assumptions!$D$51</f>
+        <f aca="false">IF(Assumptions!$D$51&gt;0,ROUNDUP(C11/Assumptions!$D$51,0)*Assumptions!$D$51,C11)</f>
         <v>47500</v>
       </c>
     </row>
@@ -16361,7 +16361,7 @@
         <v>100</v>
       </c>
       <c r="H25" s="36" t="n">
-        <f aca="false">F25/G25</f>
+        <f aca="false">IF(G25&gt;0,F25/G25,0)</f>
         <v>387.334681977991</v>
       </c>
       <c r="I25" s="29" t="n">
@@ -20676,7 +20676,7 @@
         <v>322.142857142857</v>
       </c>
       <c r="S15" s="2" t="str">
-        <f aca="false">IF(Assumptions!$D$48&gt;=1,"✗ reserve share must be below 100%",IF(Funnel!B19&lt;Assumptions!$D$7,"✗ no application can sign by the deadline (Funnel B19 is before the campaign starts)",IF(AND(Budget!G24&gt;0,Funnel!B20&lt;Assumptions!$D$7),"✗ supervisors cannot apply in time (Funnel B20 is before the campaign starts)",IF(OR(ABS(D15-1)&gt;0.001,ABS(Y15-1)&gt;0.001),"✗ shares must sum to 100%",IF(ABS(M15-Budget!C9)&gt;1,"✗ weeks ≠ planned spend",IF(ABS(P15-Funnel!O9)&gt;0.5,"✗ qualified ≠ plan",IF(ABS(V15-Budget!C13)&gt;0.5,"✗ signatures ≠ expected hires","✓ ties to plan")))))))</f>
+        <f aca="false">IF(Assumptions!$D$48&gt;=1,"✗ reserve share must be below 100%",IF(Funnel!B19&lt;Assumptions!$D$7,"✗ no application can sign by the deadline (Funnel B19 is before the campaign starts)",IF(AND(Budget!G24&gt;0,Funnel!B20&lt;Assumptions!$D$7),"✗ supervisors cannot apply in time (Funnel B20 is before the campaign starts)",IF(OR(ABS(D15-1)&gt;0.001,ABS(Y15-1)&gt;0.001),"✗ shares must sum to 100%",IF(AND(F20&gt;0,ABS(E15-1)&gt;0.001),"✗ no spend share falls before the supervisor cut-off (Funnel B20): move weekly shares into weeks 1–5",IF(ABS(M15-Budget!C9)&gt;1,"✗ weeks ≠ planned spend",IF(ABS(P15-Funnel!O9)&gt;0.5,"✗ qualified ≠ plan",IF(ABS(V15-Budget!C13)&gt;0.5,"✗ signatures ≠ expected hires","✓ ties to plan"))))))))</f>
         <v>✓ ties to plan</v>
       </c>
       <c r="T15" s="29" t="n">

</xml_diff>

<commit_message>
Input check covers every numeric input; flags for spend after cut-off and late assessment start; tracker label fix; 148/148 tests pass
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V2NJtrYy3bzNxqKeiRXJfY
</commit_message>
<xml_diff>
--- a/operation_uptime/Operation_Uptime_Model.xlsx
+++ b/operation_uptime/Operation_Uptime_Model.xlsx
@@ -3067,7 +3067,7 @@
         <v>16</v>
       </c>
       <c r="C19" s="8" t="str">
-        <f aca="false">IF(((Assumptions!$D$10&lt;0)+(Assumptions!$D$10&gt;1)+(Assumptions!$D$54&lt;0)+(Assumptions!$D$54&gt;1)+(Assumptions!$D$50&lt;0)+(Assumptions!$D$50&gt;1)+(Assumptions!$D$52&lt;0)+(Assumptions!$D$52&gt;1)+(Assumptions!$D$53&lt;0)+(Assumptions!$D$53&gt;1)+(Assumptions!$D$66&lt;0)+(Assumptions!$D$66&gt;1)+(Assumptions!$D$139&lt;0)+(Assumptions!$D$139&gt;1)+(Assumptions!$D$140&lt;0)+(Assumptions!$D$140&gt;1)+(Assumptions!$D$145&lt;0)+(Assumptions!$D$145&gt;1)+(Assumptions!$D$150&lt;0)+(Assumptions!$D$150&gt;1)+(Assumptions!$D$152&lt;0)+(Assumptions!$D$152&gt;1)+(Assumptions!$D$156&lt;0)+(Assumptions!$D$156&gt;1)+(Assumptions!$D$97&lt;0)+(Assumptions!$D$97&gt;1)+(Assumptions!$D$98&lt;0)+(Assumptions!$D$98&gt;1)+(Assumptions!$D$99&lt;0)+(Assumptions!$D$99&gt;1)+(Assumptions!$D$93&lt;0)+(Assumptions!$D$93&gt;1)+(Assumptions!$D$95&lt;0)+(Assumptions!$D$95&gt;1)+(Assumptions!$D$92&lt;0)+(Assumptions!$D$92&gt;1)+(Assumptions!$D$29&lt;0)+(Assumptions!$D$29&gt;1)+(Assumptions!$D$30&lt;0)+(Assumptions!$D$30&gt;1)+(Assumptions!$D$31&lt;0)+(Assumptions!$D$31&gt;1)+(Assumptions!$D$32&lt;0)+(Assumptions!$D$32&gt;1)+(Assumptions!$D$33&lt;0)+(Assumptions!$D$33&gt;1)+(Assumptions!$D$34&lt;0)+(Assumptions!$D$34&gt;1)+(Assumptions!$D$35&lt;0)+(Assumptions!$D$35&gt;1)+(Assumptions!$D$36&lt;0)+(Assumptions!$D$36&gt;1)+(Assumptions!$D$37&lt;0)+(Assumptions!$D$37&gt;1)+(Assumptions!$D$38&lt;0)+(Assumptions!$D$38&gt;1)+(Assumptions!$D$39&lt;0)+(Assumptions!$D$39&gt;1)+(Assumptions!$D$40&lt;0)+(Assumptions!$D$40&gt;1)+(Assumptions!$D$41&lt;0)+(Assumptions!$D$41&gt;1)+(Assumptions!$D$42&lt;0)+(Assumptions!$D$42&gt;1)+(Assumptions!$D$43&lt;0)+(Assumptions!$D$43&gt;1)+(Assumptions!$D$44&lt;0)+(Assumptions!$D$44&gt;1)+(Assumptions!$D$55&lt;0)+(Assumptions!$D$55&gt;1)+(Assumptions!$D$56&lt;0)+(Assumptions!$D$56&gt;1)+(Assumptions!$D$57&lt;0)+(Assumptions!$D$57&gt;1)+(Assumptions!$D$58&lt;0)+(Assumptions!$D$58&gt;1)+(Assumptions!$D$59&lt;0)+(Assumptions!$D$59&gt;1)+(Assumptions!$D$60&lt;0)+(Assumptions!$D$60&gt;1)+(Assumptions!$D$61&lt;0)+(Assumptions!$D$61&gt;1)+(Assumptions!$D$62&lt;0)+(Assumptions!$D$62&gt;1)+(Assumptions!$D$63&lt;0)+(Assumptions!$D$63&gt;1)+(Assumptions!$D$64&lt;0)+(Assumptions!$D$64&gt;1)+(Assumptions!$D$65&lt;0)+(Assumptions!$D$65&gt;1)+(Assumptions!$D$74&lt;0)+(Assumptions!$D$74&gt;1)+(Assumptions!$D$75&lt;0)+(Assumptions!$D$75&gt;1)+(Assumptions!$D$76&lt;0)+(Assumptions!$D$76&gt;1)+(Assumptions!$D$77&lt;0)+(Assumptions!$D$77&gt;1))+((Assumptions!$D$9&lt;0)+(Assumptions!$D$11&lt;0)+(Assumptions!$D$12&lt;0)+(Assumptions!$D$13&lt;0)+(Assumptions!$D$14&lt;0)+(Assumptions!$D$49&lt;0)+(Assumptions!$D$51&lt;0)+(Assumptions!$D$19&lt;0)+(Assumptions!$D$21&lt;0)+(Assumptions!$D$22&lt;0)+(Assumptions!$D$23&lt;0)+(Assumptions!$D$24&lt;0)+(Assumptions!$D$25&lt;0)+(Assumptions!$D$85&lt;0)+(Assumptions!$D$86&lt;0)+(Assumptions!$D$90&lt;0)+(Assumptions!$D$108&lt;0)+(Assumptions!$D$91&lt;0)+(Assumptions!$D$107&lt;0)+(Assumptions!$D$146&lt;0)+(Assumptions!$D$147&lt;0)+(Assumptions!$D$149&lt;0)+(Assumptions!$D$151&lt;0)+(Assumptions!$D$154&lt;0)+(Assumptions!$D$155&lt;0)+(Assumptions!$D$159&lt;0)+(Assumptions!$D$160&lt;0)+(Assumptions!$D$161&lt;0)+(Assumptions!$D$148&lt;0)+(Assumptions!$D$153&lt;0)+(Assumptions!$D$158&lt;0)+(Assumptions!$D$94&lt;0)+(Assumptions!$D$96&lt;0)+(Assumptions!$D$135&lt;0)+(Assumptions!$D$136&lt;0)+(Assumptions!$D$137&lt;0)+(Assumptions!$D$138&lt;0)+(Assumptions!$D$141&lt;0)+(Assumptions!$D$142&lt;0)+(Assumptions!$D$143&lt;0)+(Assumptions!$D$144&lt;0)+(Assumptions!$D$70&lt;0)+(Assumptions!$D$71&lt;0)+(Assumptions!$D$72&lt;0)+(Assumptions!$D$73&lt;0)+(Assumptions!$D$78&lt;0)+(Assumptions!$D$79&lt;0)+(Assumptions!$D$80&lt;0)+(Assumptions!$D$81&lt;0))+SUMPRODUCT((Assumptions!$E$112:$E$131&lt;0)+(Assumptions!$G$112:$G$131&lt;0)+(Assumptions!$G$112:$G$131&gt;1)+(Assumptions!$H$112:$H$131&lt;0)+(Assumptions!$I$112:$I$131&lt;0)+(Assumptions!$J$112:$J$131&lt;0)+(Assumptions!$F$112:$F$131&lt;0)+((Assumptions!$D$112:$D$131="CPC")*(Assumptions!$F$112:$F$131&gt;1)))+(Assumptions!$D$48&lt;0)+(Assumptions!$D$48&gt;=1)+(Assumptions!$D$20&lt;Assumptions!$D$7)+(Assumptions!$D$20&gt;Assumptions!$D$8)=0,"✓ all inputs valid","✗ invalid input: "&amp;IF(((Assumptions!$D$10&lt;0)+(Assumptions!$D$10&gt;1)+(Assumptions!$D$54&lt;0)+(Assumptions!$D$54&gt;1)+(Assumptions!$D$50&lt;0)+(Assumptions!$D$50&gt;1)+(Assumptions!$D$52&lt;0)+(Assumptions!$D$52&gt;1)+(Assumptions!$D$53&lt;0)+(Assumptions!$D$53&gt;1)+(Assumptions!$D$66&lt;0)+(Assumptions!$D$66&gt;1)+(Assumptions!$D$139&lt;0)+(Assumptions!$D$139&gt;1)+(Assumptions!$D$140&lt;0)+(Assumptions!$D$140&gt;1)+(Assumptions!$D$145&lt;0)+(Assumptions!$D$145&gt;1)+(Assumptions!$D$150&lt;0)+(Assumptions!$D$150&gt;1)+(Assumptions!$D$152&lt;0)+(Assumptions!$D$152&gt;1)+(Assumptions!$D$156&lt;0)+(Assumptions!$D$156&gt;1)+(Assumptions!$D$97&lt;0)+(Assumptions!$D$97&gt;1)+(Assumptions!$D$98&lt;0)+(Assumptions!$D$98&gt;1)+(Assumptions!$D$99&lt;0)+(Assumptions!$D$99&gt;1)+(Assumptions!$D$93&lt;0)+(Assumptions!$D$93&gt;1)+(Assumptions!$D$95&lt;0)+(Assumptions!$D$95&gt;1)+(Assumptions!$D$92&lt;0)+(Assumptions!$D$92&gt;1)+(Assumptions!$D$29&lt;0)+(Assumptions!$D$29&gt;1)+(Assumptions!$D$30&lt;0)+(Assumptions!$D$30&gt;1)+(Assumptions!$D$31&lt;0)+(Assumptions!$D$31&gt;1)+(Assumptions!$D$32&lt;0)+(Assumptions!$D$32&gt;1)+(Assumptions!$D$33&lt;0)+(Assumptions!$D$33&gt;1)+(Assumptions!$D$34&lt;0)+(Assumptions!$D$34&gt;1)+(Assumptions!$D$35&lt;0)+(Assumptions!$D$35&gt;1)+(Assumptions!$D$36&lt;0)+(Assumptions!$D$36&gt;1)+(Assumptions!$D$37&lt;0)+(Assumptions!$D$37&gt;1)+(Assumptions!$D$38&lt;0)+(Assumptions!$D$38&gt;1)+(Assumptions!$D$39&lt;0)+(Assumptions!$D$39&gt;1)+(Assumptions!$D$40&lt;0)+(Assumptions!$D$40&gt;1)+(Assumptions!$D$41&lt;0)+(Assumptions!$D$41&gt;1)+(Assumptions!$D$42&lt;0)+(Assumptions!$D$42&gt;1)+(Assumptions!$D$43&lt;0)+(Assumptions!$D$43&gt;1)+(Assumptions!$D$44&lt;0)+(Assumptions!$D$44&gt;1)+(Assumptions!$D$55&lt;0)+(Assumptions!$D$55&gt;1)+(Assumptions!$D$56&lt;0)+(Assumptions!$D$56&gt;1)+(Assumptions!$D$57&lt;0)+(Assumptions!$D$57&gt;1)+(Assumptions!$D$58&lt;0)+(Assumptions!$D$58&gt;1)+(Assumptions!$D$59&lt;0)+(Assumptions!$D$59&gt;1)+(Assumptions!$D$60&lt;0)+(Assumptions!$D$60&gt;1)+(Assumptions!$D$61&lt;0)+(Assumptions!$D$61&gt;1)+(Assumptions!$D$62&lt;0)+(Assumptions!$D$62&gt;1)+(Assumptions!$D$63&lt;0)+(Assumptions!$D$63&gt;1)+(Assumptions!$D$64&lt;0)+(Assumptions!$D$64&gt;1)+(Assumptions!$D$65&lt;0)+(Assumptions!$D$65&gt;1)+(Assumptions!$D$74&lt;0)+(Assumptions!$D$74&gt;1)+(Assumptions!$D$75&lt;0)+(Assumptions!$D$75&gt;1)+(Assumptions!$D$76&lt;0)+(Assumptions!$D$76&gt;1)+(Assumptions!$D$77&lt;0)+(Assumptions!$D$77&gt;1))&gt;0,"a share/rate is outside 0–100%; ","")&amp;IF(((Assumptions!$D$9&lt;0)+(Assumptions!$D$11&lt;0)+(Assumptions!$D$12&lt;0)+(Assumptions!$D$13&lt;0)+(Assumptions!$D$14&lt;0)+(Assumptions!$D$49&lt;0)+(Assumptions!$D$51&lt;0)+(Assumptions!$D$19&lt;0)+(Assumptions!$D$21&lt;0)+(Assumptions!$D$22&lt;0)+(Assumptions!$D$23&lt;0)+(Assumptions!$D$24&lt;0)+(Assumptions!$D$25&lt;0)+(Assumptions!$D$85&lt;0)+(Assumptions!$D$86&lt;0)+(Assumptions!$D$90&lt;0)+(Assumptions!$D$108&lt;0)+(Assumptions!$D$91&lt;0)+(Assumptions!$D$107&lt;0)+(Assumptions!$D$146&lt;0)+(Assumptions!$D$147&lt;0)+(Assumptions!$D$149&lt;0)+(Assumptions!$D$151&lt;0)+(Assumptions!$D$154&lt;0)+(Assumptions!$D$155&lt;0)+(Assumptions!$D$159&lt;0)+(Assumptions!$D$160&lt;0)+(Assumptions!$D$161&lt;0)+(Assumptions!$D$148&lt;0)+(Assumptions!$D$153&lt;0)+(Assumptions!$D$158&lt;0)+(Assumptions!$D$94&lt;0)+(Assumptions!$D$96&lt;0)+(Assumptions!$D$135&lt;0)+(Assumptions!$D$136&lt;0)+(Assumptions!$D$137&lt;0)+(Assumptions!$D$138&lt;0)+(Assumptions!$D$141&lt;0)+(Assumptions!$D$142&lt;0)+(Assumptions!$D$143&lt;0)+(Assumptions!$D$144&lt;0)+(Assumptions!$D$70&lt;0)+(Assumptions!$D$71&lt;0)+(Assumptions!$D$72&lt;0)+(Assumptions!$D$73&lt;0)+(Assumptions!$D$78&lt;0)+(Assumptions!$D$79&lt;0)+(Assumptions!$D$80&lt;0)+(Assumptions!$D$81&lt;0))&gt;0,"a count, cost or day value is negative; ","")&amp;IF(SUMPRODUCT((Assumptions!$E$112:$E$131&lt;0)+(Assumptions!$G$112:$G$131&lt;0)+(Assumptions!$G$112:$G$131&gt;1)+(Assumptions!$H$112:$H$131&lt;0)+(Assumptions!$I$112:$I$131&lt;0)+(Assumptions!$J$112:$J$131&lt;0)+(Assumptions!$F$112:$F$131&lt;0)+((Assumptions!$D$112:$D$131="CPC")*(Assumptions!$F$112:$F$131&gt;1)))&gt;0,"a channel input (Assumptions §7) is out of range; ","")&amp;IF(OR(Assumptions!$D$48&lt;0,Assumptions!$D$48&gt;=1),"reserve share must be 0–99%; ","")&amp;IF(OR(Assumptions!$D$20&lt;Assumptions!$D$7,Assumptions!$D$20&gt;Assumptions!$D$8),"last signing date must fall inside the campaign; ",""))</f>
+        <f aca="false">IF(((Assumptions!$D$10&lt;0)+(Assumptions!$D$10&gt;1)+(Assumptions!$D$54&lt;0)+(Assumptions!$D$54&gt;1)+(Assumptions!$D$50&lt;0)+(Assumptions!$D$50&gt;1)+(Assumptions!$D$52&lt;0)+(Assumptions!$D$52&gt;1)+(Assumptions!$D$53&lt;0)+(Assumptions!$D$53&gt;1)+(Assumptions!$D$66&lt;0)+(Assumptions!$D$66&gt;1)+(Assumptions!$D$139&lt;0)+(Assumptions!$D$139&gt;1)+(Assumptions!$D$140&lt;0)+(Assumptions!$D$140&gt;1)+(Assumptions!$D$145&lt;0)+(Assumptions!$D$145&gt;1)+(Assumptions!$D$150&lt;0)+(Assumptions!$D$150&gt;1)+(Assumptions!$D$152&lt;0)+(Assumptions!$D$152&gt;1)+(Assumptions!$D$156&lt;0)+(Assumptions!$D$156&gt;1)+(Assumptions!$D$97&lt;0)+(Assumptions!$D$97&gt;1)+(Assumptions!$D$98&lt;0)+(Assumptions!$D$98&gt;1)+(Assumptions!$D$99&lt;0)+(Assumptions!$D$99&gt;1)+(Assumptions!$D$93&lt;0)+(Assumptions!$D$93&gt;1)+(Assumptions!$D$95&lt;0)+(Assumptions!$D$95&gt;1)+(Assumptions!$D$92&lt;0)+(Assumptions!$D$92&gt;1)+(Assumptions!$D$29&lt;0)+(Assumptions!$D$29&gt;1)+(Assumptions!$D$30&lt;0)+(Assumptions!$D$30&gt;1)+(Assumptions!$D$31&lt;0)+(Assumptions!$D$31&gt;1)+(Assumptions!$D$32&lt;0)+(Assumptions!$D$32&gt;1)+(Assumptions!$D$33&lt;0)+(Assumptions!$D$33&gt;1)+(Assumptions!$D$34&lt;0)+(Assumptions!$D$34&gt;1)+(Assumptions!$D$35&lt;0)+(Assumptions!$D$35&gt;1)+(Assumptions!$D$36&lt;0)+(Assumptions!$D$36&gt;1)+(Assumptions!$D$37&lt;0)+(Assumptions!$D$37&gt;1)+(Assumptions!$D$38&lt;0)+(Assumptions!$D$38&gt;1)+(Assumptions!$D$39&lt;0)+(Assumptions!$D$39&gt;1)+(Assumptions!$D$40&lt;0)+(Assumptions!$D$40&gt;1)+(Assumptions!$D$41&lt;0)+(Assumptions!$D$41&gt;1)+(Assumptions!$D$42&lt;0)+(Assumptions!$D$42&gt;1)+(Assumptions!$D$43&lt;0)+(Assumptions!$D$43&gt;1)+(Assumptions!$D$44&lt;0)+(Assumptions!$D$44&gt;1)+(Assumptions!$D$55&lt;0)+(Assumptions!$D$55&gt;1)+(Assumptions!$D$56&lt;0)+(Assumptions!$D$56&gt;1)+(Assumptions!$D$57&lt;0)+(Assumptions!$D$57&gt;1)+(Assumptions!$D$58&lt;0)+(Assumptions!$D$58&gt;1)+(Assumptions!$D$59&lt;0)+(Assumptions!$D$59&gt;1)+(Assumptions!$D$60&lt;0)+(Assumptions!$D$60&gt;1)+(Assumptions!$D$61&lt;0)+(Assumptions!$D$61&gt;1)+(Assumptions!$D$62&lt;0)+(Assumptions!$D$62&gt;1)+(Assumptions!$D$63&lt;0)+(Assumptions!$D$63&gt;1)+(Assumptions!$D$64&lt;0)+(Assumptions!$D$64&gt;1)+(Assumptions!$D$65&lt;0)+(Assumptions!$D$65&gt;1)+(Assumptions!$D$74&lt;0)+(Assumptions!$D$74&gt;1)+(Assumptions!$D$75&lt;0)+(Assumptions!$D$75&gt;1)+(Assumptions!$D$76&lt;0)+(Assumptions!$D$76&gt;1)+(Assumptions!$D$77&lt;0)+(Assumptions!$D$77&gt;1)+(Assumptions!$D$100&lt;0)+(Assumptions!$D$100&gt;1)+(Assumptions!$D$103&lt;0)+(Assumptions!$D$103&gt;1)+(Assumptions!$D$104&lt;0)+(Assumptions!$D$104&gt;1)+(Assumptions!$D$105&lt;0)+(Assumptions!$D$105&gt;1)+(Assumptions!$D$106&lt;0)+(Assumptions!$D$106&gt;1))+((Assumptions!$D$9&lt;0)+(Assumptions!$D$11&lt;0)+(Assumptions!$D$12&lt;0)+(Assumptions!$D$13&lt;0)+(Assumptions!$D$14&lt;0)+(Assumptions!$D$15&lt;0)+(Assumptions!$D$19&lt;0)+(Assumptions!$D$21&lt;0)+(Assumptions!$D$22&lt;0)+(Assumptions!$D$23&lt;0)+(Assumptions!$D$24&lt;0)+(Assumptions!$D$25&lt;0)+(Assumptions!$D$49&lt;0)+(Assumptions!$D$51&lt;0)+(Assumptions!$D$70&lt;0)+(Assumptions!$D$71&lt;0)+(Assumptions!$D$72&lt;0)+(Assumptions!$D$73&lt;0)+(Assumptions!$D$78&lt;0)+(Assumptions!$D$79&lt;0)+(Assumptions!$D$80&lt;0)+(Assumptions!$D$81&lt;0)+(Assumptions!$D$85&lt;0)+(Assumptions!$D$86&lt;0)+(Assumptions!$D$87&lt;0)+(Assumptions!$D$88&lt;0)+(Assumptions!$D$89&lt;0)+(Assumptions!$D$90&lt;0)+(Assumptions!$D$91&lt;0)+(Assumptions!$D$94&lt;0)+(Assumptions!$D$96&lt;0)+(Assumptions!$D$101&lt;0)+(Assumptions!$D$102&lt;0)+(Assumptions!$D$107&lt;0)+(Assumptions!$D$108&lt;0)+(Assumptions!$D$135&lt;0)+(Assumptions!$D$136&lt;0)+(Assumptions!$D$137&lt;0)+(Assumptions!$D$138&lt;0)+(Assumptions!$D$141&lt;0)+(Assumptions!$D$142&lt;0)+(Assumptions!$D$143&lt;0)+(Assumptions!$D$144&lt;0)+(Assumptions!$D$146&lt;0)+(Assumptions!$D$147&lt;0)+(Assumptions!$D$148&lt;0)+(Assumptions!$D$149&lt;0)+(Assumptions!$D$151&lt;0)+(Assumptions!$D$153&lt;0)+(Assumptions!$D$154&lt;0)+(Assumptions!$D$155&lt;0)+(Assumptions!$D$157&lt;0)+(Assumptions!$D$158&lt;0)+(Assumptions!$D$159&lt;0)+(Assumptions!$D$160&lt;0)+(Assumptions!$D$161&lt;0))+SUMPRODUCT((Assumptions!$E$112:$E$131&lt;0)+(Assumptions!$G$112:$G$131&lt;0)+(Assumptions!$G$112:$G$131&gt;1)+(Assumptions!$H$112:$H$131&lt;0)+(Assumptions!$I$112:$I$131&lt;0)+(Assumptions!$J$112:$J$131&lt;0)+(Assumptions!$F$112:$F$131&lt;0)+((Assumptions!$D$112:$D$131="CPC")*(Assumptions!$F$112:$F$131&gt;1)))+(Assumptions!$D$48&lt;0)+(Assumptions!$D$48&gt;=1)+(Assumptions!$D$20&lt;Assumptions!$D$7)+(Assumptions!$D$20&gt;Assumptions!$D$8)+(Assumptions!$D$8&lt;=Assumptions!$D$7)=0,"✓ all inputs valid","✗ invalid input: "&amp;IF(((Assumptions!$D$10&lt;0)+(Assumptions!$D$10&gt;1)+(Assumptions!$D$54&lt;0)+(Assumptions!$D$54&gt;1)+(Assumptions!$D$50&lt;0)+(Assumptions!$D$50&gt;1)+(Assumptions!$D$52&lt;0)+(Assumptions!$D$52&gt;1)+(Assumptions!$D$53&lt;0)+(Assumptions!$D$53&gt;1)+(Assumptions!$D$66&lt;0)+(Assumptions!$D$66&gt;1)+(Assumptions!$D$139&lt;0)+(Assumptions!$D$139&gt;1)+(Assumptions!$D$140&lt;0)+(Assumptions!$D$140&gt;1)+(Assumptions!$D$145&lt;0)+(Assumptions!$D$145&gt;1)+(Assumptions!$D$150&lt;0)+(Assumptions!$D$150&gt;1)+(Assumptions!$D$152&lt;0)+(Assumptions!$D$152&gt;1)+(Assumptions!$D$156&lt;0)+(Assumptions!$D$156&gt;1)+(Assumptions!$D$97&lt;0)+(Assumptions!$D$97&gt;1)+(Assumptions!$D$98&lt;0)+(Assumptions!$D$98&gt;1)+(Assumptions!$D$99&lt;0)+(Assumptions!$D$99&gt;1)+(Assumptions!$D$93&lt;0)+(Assumptions!$D$93&gt;1)+(Assumptions!$D$95&lt;0)+(Assumptions!$D$95&gt;1)+(Assumptions!$D$92&lt;0)+(Assumptions!$D$92&gt;1)+(Assumptions!$D$29&lt;0)+(Assumptions!$D$29&gt;1)+(Assumptions!$D$30&lt;0)+(Assumptions!$D$30&gt;1)+(Assumptions!$D$31&lt;0)+(Assumptions!$D$31&gt;1)+(Assumptions!$D$32&lt;0)+(Assumptions!$D$32&gt;1)+(Assumptions!$D$33&lt;0)+(Assumptions!$D$33&gt;1)+(Assumptions!$D$34&lt;0)+(Assumptions!$D$34&gt;1)+(Assumptions!$D$35&lt;0)+(Assumptions!$D$35&gt;1)+(Assumptions!$D$36&lt;0)+(Assumptions!$D$36&gt;1)+(Assumptions!$D$37&lt;0)+(Assumptions!$D$37&gt;1)+(Assumptions!$D$38&lt;0)+(Assumptions!$D$38&gt;1)+(Assumptions!$D$39&lt;0)+(Assumptions!$D$39&gt;1)+(Assumptions!$D$40&lt;0)+(Assumptions!$D$40&gt;1)+(Assumptions!$D$41&lt;0)+(Assumptions!$D$41&gt;1)+(Assumptions!$D$42&lt;0)+(Assumptions!$D$42&gt;1)+(Assumptions!$D$43&lt;0)+(Assumptions!$D$43&gt;1)+(Assumptions!$D$44&lt;0)+(Assumptions!$D$44&gt;1)+(Assumptions!$D$55&lt;0)+(Assumptions!$D$55&gt;1)+(Assumptions!$D$56&lt;0)+(Assumptions!$D$56&gt;1)+(Assumptions!$D$57&lt;0)+(Assumptions!$D$57&gt;1)+(Assumptions!$D$58&lt;0)+(Assumptions!$D$58&gt;1)+(Assumptions!$D$59&lt;0)+(Assumptions!$D$59&gt;1)+(Assumptions!$D$60&lt;0)+(Assumptions!$D$60&gt;1)+(Assumptions!$D$61&lt;0)+(Assumptions!$D$61&gt;1)+(Assumptions!$D$62&lt;0)+(Assumptions!$D$62&gt;1)+(Assumptions!$D$63&lt;0)+(Assumptions!$D$63&gt;1)+(Assumptions!$D$64&lt;0)+(Assumptions!$D$64&gt;1)+(Assumptions!$D$65&lt;0)+(Assumptions!$D$65&gt;1)+(Assumptions!$D$74&lt;0)+(Assumptions!$D$74&gt;1)+(Assumptions!$D$75&lt;0)+(Assumptions!$D$75&gt;1)+(Assumptions!$D$76&lt;0)+(Assumptions!$D$76&gt;1)+(Assumptions!$D$77&lt;0)+(Assumptions!$D$77&gt;1)+(Assumptions!$D$100&lt;0)+(Assumptions!$D$100&gt;1)+(Assumptions!$D$103&lt;0)+(Assumptions!$D$103&gt;1)+(Assumptions!$D$104&lt;0)+(Assumptions!$D$104&gt;1)+(Assumptions!$D$105&lt;0)+(Assumptions!$D$105&gt;1)+(Assumptions!$D$106&lt;0)+(Assumptions!$D$106&gt;1))&gt;0,"a share/rate is outside 0–100%; ","")&amp;IF(((Assumptions!$D$9&lt;0)+(Assumptions!$D$11&lt;0)+(Assumptions!$D$12&lt;0)+(Assumptions!$D$13&lt;0)+(Assumptions!$D$14&lt;0)+(Assumptions!$D$15&lt;0)+(Assumptions!$D$19&lt;0)+(Assumptions!$D$21&lt;0)+(Assumptions!$D$22&lt;0)+(Assumptions!$D$23&lt;0)+(Assumptions!$D$24&lt;0)+(Assumptions!$D$25&lt;0)+(Assumptions!$D$49&lt;0)+(Assumptions!$D$51&lt;0)+(Assumptions!$D$70&lt;0)+(Assumptions!$D$71&lt;0)+(Assumptions!$D$72&lt;0)+(Assumptions!$D$73&lt;0)+(Assumptions!$D$78&lt;0)+(Assumptions!$D$79&lt;0)+(Assumptions!$D$80&lt;0)+(Assumptions!$D$81&lt;0)+(Assumptions!$D$85&lt;0)+(Assumptions!$D$86&lt;0)+(Assumptions!$D$87&lt;0)+(Assumptions!$D$88&lt;0)+(Assumptions!$D$89&lt;0)+(Assumptions!$D$90&lt;0)+(Assumptions!$D$91&lt;0)+(Assumptions!$D$94&lt;0)+(Assumptions!$D$96&lt;0)+(Assumptions!$D$101&lt;0)+(Assumptions!$D$102&lt;0)+(Assumptions!$D$107&lt;0)+(Assumptions!$D$108&lt;0)+(Assumptions!$D$135&lt;0)+(Assumptions!$D$136&lt;0)+(Assumptions!$D$137&lt;0)+(Assumptions!$D$138&lt;0)+(Assumptions!$D$141&lt;0)+(Assumptions!$D$142&lt;0)+(Assumptions!$D$143&lt;0)+(Assumptions!$D$144&lt;0)+(Assumptions!$D$146&lt;0)+(Assumptions!$D$147&lt;0)+(Assumptions!$D$148&lt;0)+(Assumptions!$D$149&lt;0)+(Assumptions!$D$151&lt;0)+(Assumptions!$D$153&lt;0)+(Assumptions!$D$154&lt;0)+(Assumptions!$D$155&lt;0)+(Assumptions!$D$157&lt;0)+(Assumptions!$D$158&lt;0)+(Assumptions!$D$159&lt;0)+(Assumptions!$D$160&lt;0)+(Assumptions!$D$161&lt;0))&gt;0,"a count, cost or day value is negative; ","")&amp;IF(SUMPRODUCT((Assumptions!$E$112:$E$131&lt;0)+(Assumptions!$G$112:$G$131&lt;0)+(Assumptions!$G$112:$G$131&gt;1)+(Assumptions!$H$112:$H$131&lt;0)+(Assumptions!$I$112:$I$131&lt;0)+(Assumptions!$J$112:$J$131&lt;0)+(Assumptions!$F$112:$F$131&lt;0)+((Assumptions!$D$112:$D$131="CPC")*(Assumptions!$F$112:$F$131&gt;1)))&gt;0,"a channel input (Assumptions §7) is out of range; ","")&amp;IF(OR(Assumptions!$D$48&lt;0,Assumptions!$D$48&gt;=1),"reserve share must be 0–99%; ","")&amp;IF(OR(Assumptions!$D$20&lt;Assumptions!$D$7,Assumptions!$D$20&gt;Assumptions!$D$8),"last signing date must fall inside the campaign; ","")&amp;IF(Assumptions!$D$8&lt;=Assumptions!$D$7,"campaign end must be after its start; ",""))</f>
         <v>✓ all inputs valid</v>
       </c>
     </row>
@@ -3271,7 +3271,7 @@
         <v/>
       </c>
       <c r="X5" s="2" t="str">
-        <f aca="false">IF(F5=0,"Free – monitor quality",IF(AND(P5&lt;Assumptions!$D$85,Q5&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W5&gt;=Assumptions!$D$89,AND(R5=0,P5&gt;=Assumptions!$D$90,P5/F5&gt;=Assumptions!$D$91),AND(P5&gt;=Assumptions!$D$90,P5/F5&lt;Assumptions!$D$91,Q5&lt;Assumptions!$D$92*P5/D5)),"SWITCH OFF",IF(W5&gt;=Assumptions!$D$88,"CUT 50%",IF(W5&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD")))))</f>
+        <f aca="false">IF(D5=0,"Free – monitor quality",IF(F5=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P5&lt;Assumptions!$D$85,Q5&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W5&gt;=Assumptions!$D$89,AND(R5=0,P5&gt;=Assumptions!$D$90,P5/F5&gt;=Assumptions!$D$91),AND(P5&gt;=Assumptions!$D$90,P5/F5&lt;Assumptions!$D$91,Q5&lt;Assumptions!$D$92*P5/D5)),"SWITCH OFF",IF(W5&gt;=Assumptions!$D$88,"CUT 50%",IF(W5&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Free – monitor quality</v>
       </c>
     </row>
@@ -3342,7 +3342,7 @@
         <v/>
       </c>
       <c r="X6" s="2" t="str">
-        <f aca="false">IF(F6=0,"Free – monitor quality",IF(AND(P6&lt;Assumptions!$D$85,Q6&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W6&gt;=Assumptions!$D$89,AND(R6=0,P6&gt;=Assumptions!$D$90,P6/F6&gt;=Assumptions!$D$91),AND(P6&gt;=Assumptions!$D$90,P6/F6&lt;Assumptions!$D$91,Q6&lt;Assumptions!$D$92*P6/D6)),"SWITCH OFF",IF(W6&gt;=Assumptions!$D$88,"CUT 50%",IF(W6&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD")))))</f>
+        <f aca="false">IF(D6=0,"Free – monitor quality",IF(F6=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P6&lt;Assumptions!$D$85,Q6&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W6&gt;=Assumptions!$D$89,AND(R6=0,P6&gt;=Assumptions!$D$90,P6/F6&gt;=Assumptions!$D$91),AND(P6&gt;=Assumptions!$D$90,P6/F6&lt;Assumptions!$D$91,Q6&lt;Assumptions!$D$92*P6/D6)),"SWITCH OFF",IF(W6&gt;=Assumptions!$D$88,"CUT 50%",IF(W6&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Free – monitor quality</v>
       </c>
     </row>
@@ -3413,7 +3413,7 @@
         <v/>
       </c>
       <c r="X7" s="2" t="str">
-        <f aca="false">IF(F7=0,"Free – monitor quality",IF(AND(P7&lt;Assumptions!$D$85,Q7&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W7&gt;=Assumptions!$D$89,AND(R7=0,P7&gt;=Assumptions!$D$90,P7/F7&gt;=Assumptions!$D$91),AND(P7&gt;=Assumptions!$D$90,P7/F7&lt;Assumptions!$D$91,Q7&lt;Assumptions!$D$92*P7/D7)),"SWITCH OFF",IF(W7&gt;=Assumptions!$D$88,"CUT 50%",IF(W7&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD")))))</f>
+        <f aca="false">IF(D7=0,"Free – monitor quality",IF(F7=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P7&lt;Assumptions!$D$85,Q7&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W7&gt;=Assumptions!$D$89,AND(R7=0,P7&gt;=Assumptions!$D$90,P7/F7&gt;=Assumptions!$D$91),AND(P7&gt;=Assumptions!$D$90,P7/F7&lt;Assumptions!$D$91,Q7&lt;Assumptions!$D$92*P7/D7)),"SWITCH OFF",IF(W7&gt;=Assumptions!$D$88,"CUT 50%",IF(W7&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Free – monitor quality</v>
       </c>
     </row>
@@ -3484,7 +3484,7 @@
         <v/>
       </c>
       <c r="X8" s="2" t="str">
-        <f aca="false">IF(F8=0,"Free – monitor quality",IF(AND(P8&lt;Assumptions!$D$85,Q8&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W8&gt;=Assumptions!$D$89,AND(R8=0,P8&gt;=Assumptions!$D$90,P8/F8&gt;=Assumptions!$D$91),AND(P8&gt;=Assumptions!$D$90,P8/F8&lt;Assumptions!$D$91,Q8&lt;Assumptions!$D$92*P8/D8)),"SWITCH OFF",IF(W8&gt;=Assumptions!$D$88,"CUT 50%",IF(W8&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD")))))</f>
+        <f aca="false">IF(D8=0,"Free – monitor quality",IF(F8=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P8&lt;Assumptions!$D$85,Q8&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W8&gt;=Assumptions!$D$89,AND(R8=0,P8&gt;=Assumptions!$D$90,P8/F8&gt;=Assumptions!$D$91),AND(P8&gt;=Assumptions!$D$90,P8/F8&lt;Assumptions!$D$91,Q8&lt;Assumptions!$D$92*P8/D8)),"SWITCH OFF",IF(W8&gt;=Assumptions!$D$88,"CUT 50%",IF(W8&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Free – monitor quality</v>
       </c>
     </row>
@@ -3555,7 +3555,7 @@
         <v>1</v>
       </c>
       <c r="X9" s="2" t="str">
-        <f aca="false">IF(F9=0,"Free – monitor quality",IF(AND(P9&lt;Assumptions!$D$85,Q9&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W9&gt;=Assumptions!$D$89,AND(R9=0,P9&gt;=Assumptions!$D$90,P9/F9&gt;=Assumptions!$D$91),AND(P9&gt;=Assumptions!$D$90,P9/F9&lt;Assumptions!$D$91,Q9&lt;Assumptions!$D$92*P9/D9)),"SWITCH OFF",IF(W9&gt;=Assumptions!$D$88,"CUT 50%",IF(W9&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD")))))</f>
+        <f aca="false">IF(D9=0,"Free – monitor quality",IF(F9=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P9&lt;Assumptions!$D$85,Q9&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W9&gt;=Assumptions!$D$89,AND(R9=0,P9&gt;=Assumptions!$D$90,P9/F9&gt;=Assumptions!$D$91),AND(P9&gt;=Assumptions!$D$90,P9/F9&lt;Assumptions!$D$91,Q9&lt;Assumptions!$D$92*P9/D9)),"SWITCH OFF",IF(W9&gt;=Assumptions!$D$88,"CUT 50%",IF(W9&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
       </c>
     </row>
@@ -3626,7 +3626,7 @@
         <v>1</v>
       </c>
       <c r="X10" s="2" t="str">
-        <f aca="false">IF(F10=0,"Free – monitor quality",IF(AND(P10&lt;Assumptions!$D$85,Q10&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W10&gt;=Assumptions!$D$89,AND(R10=0,P10&gt;=Assumptions!$D$90,P10/F10&gt;=Assumptions!$D$91),AND(P10&gt;=Assumptions!$D$90,P10/F10&lt;Assumptions!$D$91,Q10&lt;Assumptions!$D$92*P10/D10)),"SWITCH OFF",IF(W10&gt;=Assumptions!$D$88,"CUT 50%",IF(W10&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD")))))</f>
+        <f aca="false">IF(D10=0,"Free – monitor quality",IF(F10=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P10&lt;Assumptions!$D$85,Q10&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W10&gt;=Assumptions!$D$89,AND(R10=0,P10&gt;=Assumptions!$D$90,P10/F10&gt;=Assumptions!$D$91),AND(P10&gt;=Assumptions!$D$90,P10/F10&lt;Assumptions!$D$91,Q10&lt;Assumptions!$D$92*P10/D10)),"SWITCH OFF",IF(W10&gt;=Assumptions!$D$88,"CUT 50%",IF(W10&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
       </c>
     </row>
@@ -3697,7 +3697,7 @@
         <v>1</v>
       </c>
       <c r="X11" s="2" t="str">
-        <f aca="false">IF(F11=0,"Free – monitor quality",IF(AND(P11&lt;Assumptions!$D$85,Q11&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W11&gt;=Assumptions!$D$89,AND(R11=0,P11&gt;=Assumptions!$D$90,P11/F11&gt;=Assumptions!$D$91),AND(P11&gt;=Assumptions!$D$90,P11/F11&lt;Assumptions!$D$91,Q11&lt;Assumptions!$D$92*P11/D11)),"SWITCH OFF",IF(W11&gt;=Assumptions!$D$88,"CUT 50%",IF(W11&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD")))))</f>
+        <f aca="false">IF(D11=0,"Free – monitor quality",IF(F11=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P11&lt;Assumptions!$D$85,Q11&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W11&gt;=Assumptions!$D$89,AND(R11=0,P11&gt;=Assumptions!$D$90,P11/F11&gt;=Assumptions!$D$91),AND(P11&gt;=Assumptions!$D$90,P11/F11&lt;Assumptions!$D$91,Q11&lt;Assumptions!$D$92*P11/D11)),"SWITCH OFF",IF(W11&gt;=Assumptions!$D$88,"CUT 50%",IF(W11&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
       </c>
     </row>
@@ -3768,7 +3768,7 @@
         <v>1</v>
       </c>
       <c r="X12" s="2" t="str">
-        <f aca="false">IF(F12=0,"Free – monitor quality",IF(AND(P12&lt;Assumptions!$D$85,Q12&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W12&gt;=Assumptions!$D$89,AND(R12=0,P12&gt;=Assumptions!$D$90,P12/F12&gt;=Assumptions!$D$91),AND(P12&gt;=Assumptions!$D$90,P12/F12&lt;Assumptions!$D$91,Q12&lt;Assumptions!$D$92*P12/D12)),"SWITCH OFF",IF(W12&gt;=Assumptions!$D$88,"CUT 50%",IF(W12&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD")))))</f>
+        <f aca="false">IF(D12=0,"Free – monitor quality",IF(F12=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P12&lt;Assumptions!$D$85,Q12&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W12&gt;=Assumptions!$D$89,AND(R12=0,P12&gt;=Assumptions!$D$90,P12/F12&gt;=Assumptions!$D$91),AND(P12&gt;=Assumptions!$D$90,P12/F12&lt;Assumptions!$D$91,Q12&lt;Assumptions!$D$92*P12/D12)),"SWITCH OFF",IF(W12&gt;=Assumptions!$D$88,"CUT 50%",IF(W12&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
       </c>
     </row>
@@ -3839,7 +3839,7 @@
         <v>1</v>
       </c>
       <c r="X13" s="2" t="str">
-        <f aca="false">IF(F13=0,"Free – monitor quality",IF(AND(P13&lt;Assumptions!$D$85,Q13&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W13&gt;=Assumptions!$D$89,AND(R13=0,P13&gt;=Assumptions!$D$90,P13/F13&gt;=Assumptions!$D$91),AND(P13&gt;=Assumptions!$D$90,P13/F13&lt;Assumptions!$D$91,Q13&lt;Assumptions!$D$92*P13/D13)),"SWITCH OFF",IF(W13&gt;=Assumptions!$D$88,"CUT 50%",IF(W13&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD")))))</f>
+        <f aca="false">IF(D13=0,"Free – monitor quality",IF(F13=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P13&lt;Assumptions!$D$85,Q13&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W13&gt;=Assumptions!$D$89,AND(R13=0,P13&gt;=Assumptions!$D$90,P13/F13&gt;=Assumptions!$D$91),AND(P13&gt;=Assumptions!$D$90,P13/F13&lt;Assumptions!$D$91,Q13&lt;Assumptions!$D$92*P13/D13)),"SWITCH OFF",IF(W13&gt;=Assumptions!$D$88,"CUT 50%",IF(W13&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
       </c>
     </row>
@@ -3910,7 +3910,7 @@
         <v>1</v>
       </c>
       <c r="X14" s="2" t="str">
-        <f aca="false">IF(F14=0,"Free – monitor quality",IF(AND(P14&lt;Assumptions!$D$85,Q14&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W14&gt;=Assumptions!$D$89,AND(R14=0,P14&gt;=Assumptions!$D$90,P14/F14&gt;=Assumptions!$D$91),AND(P14&gt;=Assumptions!$D$90,P14/F14&lt;Assumptions!$D$91,Q14&lt;Assumptions!$D$92*P14/D14)),"SWITCH OFF",IF(W14&gt;=Assumptions!$D$88,"CUT 50%",IF(W14&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD")))))</f>
+        <f aca="false">IF(D14=0,"Free – monitor quality",IF(F14=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P14&lt;Assumptions!$D$85,Q14&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W14&gt;=Assumptions!$D$89,AND(R14=0,P14&gt;=Assumptions!$D$90,P14/F14&gt;=Assumptions!$D$91),AND(P14&gt;=Assumptions!$D$90,P14/F14&lt;Assumptions!$D$91,Q14&lt;Assumptions!$D$92*P14/D14)),"SWITCH OFF",IF(W14&gt;=Assumptions!$D$88,"CUT 50%",IF(W14&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
       </c>
     </row>
@@ -3981,7 +3981,7 @@
         <v>1</v>
       </c>
       <c r="X15" s="2" t="str">
-        <f aca="false">IF(F15=0,"Free – monitor quality",IF(AND(P15&lt;Assumptions!$D$85,Q15&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W15&gt;=Assumptions!$D$89,AND(R15=0,P15&gt;=Assumptions!$D$90,P15/F15&gt;=Assumptions!$D$91),AND(P15&gt;=Assumptions!$D$90,P15/F15&lt;Assumptions!$D$91,Q15&lt;Assumptions!$D$92*P15/D15)),"SWITCH OFF",IF(W15&gt;=Assumptions!$D$88,"CUT 50%",IF(W15&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD")))))</f>
+        <f aca="false">IF(D15=0,"Free – monitor quality",IF(F15=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P15&lt;Assumptions!$D$85,Q15&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W15&gt;=Assumptions!$D$89,AND(R15=0,P15&gt;=Assumptions!$D$90,P15/F15&gt;=Assumptions!$D$91),AND(P15&gt;=Assumptions!$D$90,P15/F15&lt;Assumptions!$D$91,Q15&lt;Assumptions!$D$92*P15/D15)),"SWITCH OFF",IF(W15&gt;=Assumptions!$D$88,"CUT 50%",IF(W15&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
       </c>
     </row>
@@ -4052,7 +4052,7 @@
         <v>1</v>
       </c>
       <c r="X16" s="2" t="str">
-        <f aca="false">IF(F16=0,"Free – monitor quality",IF(AND(P16&lt;Assumptions!$D$85,Q16&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W16&gt;=Assumptions!$D$89,AND(R16=0,P16&gt;=Assumptions!$D$90,P16/F16&gt;=Assumptions!$D$91),AND(P16&gt;=Assumptions!$D$90,P16/F16&lt;Assumptions!$D$91,Q16&lt;Assumptions!$D$92*P16/D16)),"SWITCH OFF",IF(W16&gt;=Assumptions!$D$88,"CUT 50%",IF(W16&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD")))))</f>
+        <f aca="false">IF(D16=0,"Free – monitor quality",IF(F16=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P16&lt;Assumptions!$D$85,Q16&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W16&gt;=Assumptions!$D$89,AND(R16=0,P16&gt;=Assumptions!$D$90,P16/F16&gt;=Assumptions!$D$91),AND(P16&gt;=Assumptions!$D$90,P16/F16&lt;Assumptions!$D$91,Q16&lt;Assumptions!$D$92*P16/D16)),"SWITCH OFF",IF(W16&gt;=Assumptions!$D$88,"CUT 50%",IF(W16&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
       </c>
     </row>
@@ -4123,7 +4123,7 @@
         <v>1</v>
       </c>
       <c r="X17" s="2" t="str">
-        <f aca="false">IF(F17=0,"Free – monitor quality",IF(AND(P17&lt;Assumptions!$D$85,Q17&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W17&gt;=Assumptions!$D$89,AND(R17=0,P17&gt;=Assumptions!$D$90,P17/F17&gt;=Assumptions!$D$91),AND(P17&gt;=Assumptions!$D$90,P17/F17&lt;Assumptions!$D$91,Q17&lt;Assumptions!$D$92*P17/D17)),"SWITCH OFF",IF(W17&gt;=Assumptions!$D$88,"CUT 50%",IF(W17&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD")))))</f>
+        <f aca="false">IF(D17=0,"Free – monitor quality",IF(F17=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P17&lt;Assumptions!$D$85,Q17&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W17&gt;=Assumptions!$D$89,AND(R17=0,P17&gt;=Assumptions!$D$90,P17/F17&gt;=Assumptions!$D$91),AND(P17&gt;=Assumptions!$D$90,P17/F17&lt;Assumptions!$D$91,Q17&lt;Assumptions!$D$92*P17/D17)),"SWITCH OFF",IF(W17&gt;=Assumptions!$D$88,"CUT 50%",IF(W17&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
       </c>
     </row>
@@ -4194,7 +4194,7 @@
         <v>1</v>
       </c>
       <c r="X18" s="2" t="str">
-        <f aca="false">IF(F18=0,"Free – monitor quality",IF(AND(P18&lt;Assumptions!$D$85,Q18&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W18&gt;=Assumptions!$D$89,AND(R18=0,P18&gt;=Assumptions!$D$90,P18/F18&gt;=Assumptions!$D$91),AND(P18&gt;=Assumptions!$D$90,P18/F18&lt;Assumptions!$D$91,Q18&lt;Assumptions!$D$92*P18/D18)),"SWITCH OFF",IF(W18&gt;=Assumptions!$D$88,"CUT 50%",IF(W18&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD")))))</f>
+        <f aca="false">IF(D18=0,"Free – monitor quality",IF(F18=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P18&lt;Assumptions!$D$85,Q18&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W18&gt;=Assumptions!$D$89,AND(R18=0,P18&gt;=Assumptions!$D$90,P18/F18&gt;=Assumptions!$D$91),AND(P18&gt;=Assumptions!$D$90,P18/F18&lt;Assumptions!$D$91,Q18&lt;Assumptions!$D$92*P18/D18)),"SWITCH OFF",IF(W18&gt;=Assumptions!$D$88,"CUT 50%",IF(W18&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
       </c>
     </row>
@@ -4265,7 +4265,7 @@
         <v>1</v>
       </c>
       <c r="X19" s="2" t="str">
-        <f aca="false">IF(F19=0,"Free – monitor quality",IF(AND(P19&lt;Assumptions!$D$85,Q19&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W19&gt;=Assumptions!$D$89,AND(R19=0,P19&gt;=Assumptions!$D$90,P19/F19&gt;=Assumptions!$D$91),AND(P19&gt;=Assumptions!$D$90,P19/F19&lt;Assumptions!$D$91,Q19&lt;Assumptions!$D$92*P19/D19)),"SWITCH OFF",IF(W19&gt;=Assumptions!$D$88,"CUT 50%",IF(W19&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD")))))</f>
+        <f aca="false">IF(D19=0,"Free – monitor quality",IF(F19=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P19&lt;Assumptions!$D$85,Q19&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W19&gt;=Assumptions!$D$89,AND(R19=0,P19&gt;=Assumptions!$D$90,P19/F19&gt;=Assumptions!$D$91),AND(P19&gt;=Assumptions!$D$90,P19/F19&lt;Assumptions!$D$91,Q19&lt;Assumptions!$D$92*P19/D19)),"SWITCH OFF",IF(W19&gt;=Assumptions!$D$88,"CUT 50%",IF(W19&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
       </c>
     </row>
@@ -4336,7 +4336,7 @@
         <v>1</v>
       </c>
       <c r="X20" s="2" t="str">
-        <f aca="false">IF(F20=0,"Free – monitor quality",IF(AND(P20&lt;Assumptions!$D$85,Q20&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W20&gt;=Assumptions!$D$89,AND(R20=0,P20&gt;=Assumptions!$D$90,P20/F20&gt;=Assumptions!$D$91),AND(P20&gt;=Assumptions!$D$90,P20/F20&lt;Assumptions!$D$91,Q20&lt;Assumptions!$D$92*P20/D20)),"SWITCH OFF",IF(W20&gt;=Assumptions!$D$88,"CUT 50%",IF(W20&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD")))))</f>
+        <f aca="false">IF(D20=0,"Free – monitor quality",IF(F20=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P20&lt;Assumptions!$D$85,Q20&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W20&gt;=Assumptions!$D$89,AND(R20=0,P20&gt;=Assumptions!$D$90,P20/F20&gt;=Assumptions!$D$91),AND(P20&gt;=Assumptions!$D$90,P20/F20&lt;Assumptions!$D$91,Q20&lt;Assumptions!$D$92*P20/D20)),"SWITCH OFF",IF(W20&gt;=Assumptions!$D$88,"CUT 50%",IF(W20&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
       </c>
     </row>
@@ -4407,7 +4407,7 @@
         <v>1</v>
       </c>
       <c r="X21" s="2" t="str">
-        <f aca="false">IF(F21=0,"Free – monitor quality",IF(AND(P21&lt;Assumptions!$D$85,Q21&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W21&gt;=Assumptions!$D$89,AND(R21=0,P21&gt;=Assumptions!$D$90,P21/F21&gt;=Assumptions!$D$91),AND(P21&gt;=Assumptions!$D$90,P21/F21&lt;Assumptions!$D$91,Q21&lt;Assumptions!$D$92*P21/D21)),"SWITCH OFF",IF(W21&gt;=Assumptions!$D$88,"CUT 50%",IF(W21&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD")))))</f>
+        <f aca="false">IF(D21=0,"Free – monitor quality",IF(F21=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P21&lt;Assumptions!$D$85,Q21&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W21&gt;=Assumptions!$D$89,AND(R21=0,P21&gt;=Assumptions!$D$90,P21/F21&gt;=Assumptions!$D$91),AND(P21&gt;=Assumptions!$D$90,P21/F21&lt;Assumptions!$D$91,Q21&lt;Assumptions!$D$92*P21/D21)),"SWITCH OFF",IF(W21&gt;=Assumptions!$D$88,"CUT 50%",IF(W21&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
       </c>
     </row>
@@ -4478,7 +4478,7 @@
         <v>1</v>
       </c>
       <c r="X22" s="2" t="str">
-        <f aca="false">IF(F22=0,"Free – monitor quality",IF(AND(P22&lt;Assumptions!$D$85,Q22&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W22&gt;=Assumptions!$D$89,AND(R22=0,P22&gt;=Assumptions!$D$90,P22/F22&gt;=Assumptions!$D$91),AND(P22&gt;=Assumptions!$D$90,P22/F22&lt;Assumptions!$D$91,Q22&lt;Assumptions!$D$92*P22/D22)),"SWITCH OFF",IF(W22&gt;=Assumptions!$D$88,"CUT 50%",IF(W22&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD")))))</f>
+        <f aca="false">IF(D22=0,"Free – monitor quality",IF(F22=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P22&lt;Assumptions!$D$85,Q22&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W22&gt;=Assumptions!$D$89,AND(R22=0,P22&gt;=Assumptions!$D$90,P22/F22&gt;=Assumptions!$D$91),AND(P22&gt;=Assumptions!$D$90,P22/F22&lt;Assumptions!$D$91,Q22&lt;Assumptions!$D$92*P22/D22)),"SWITCH OFF",IF(W22&gt;=Assumptions!$D$88,"CUT 50%",IF(W22&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
       </c>
     </row>
@@ -4549,7 +4549,7 @@
         <v>1</v>
       </c>
       <c r="X23" s="2" t="str">
-        <f aca="false">IF(F23=0,"Free – monitor quality",IF(AND(P23&lt;Assumptions!$D$85,Q23&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W23&gt;=Assumptions!$D$89,AND(R23=0,P23&gt;=Assumptions!$D$90,P23/F23&gt;=Assumptions!$D$91),AND(P23&gt;=Assumptions!$D$90,P23/F23&lt;Assumptions!$D$91,Q23&lt;Assumptions!$D$92*P23/D23)),"SWITCH OFF",IF(W23&gt;=Assumptions!$D$88,"CUT 50%",IF(W23&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD")))))</f>
+        <f aca="false">IF(D23=0,"Free – monitor quality",IF(F23=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P23&lt;Assumptions!$D$85,Q23&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W23&gt;=Assumptions!$D$89,AND(R23=0,P23&gt;=Assumptions!$D$90,P23/F23&gt;=Assumptions!$D$91),AND(P23&gt;=Assumptions!$D$90,P23/F23&lt;Assumptions!$D$91,Q23&lt;Assumptions!$D$92*P23/D23)),"SWITCH OFF",IF(W23&gt;=Assumptions!$D$88,"CUT 50%",IF(W23&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
       </c>
     </row>
@@ -4620,7 +4620,7 @@
         <v>1</v>
       </c>
       <c r="X24" s="2" t="str">
-        <f aca="false">IF(F24=0,"Free – monitor quality",IF(AND(P24&lt;Assumptions!$D$85,Q24&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W24&gt;=Assumptions!$D$89,AND(R24=0,P24&gt;=Assumptions!$D$90,P24/F24&gt;=Assumptions!$D$91),AND(P24&gt;=Assumptions!$D$90,P24/F24&lt;Assumptions!$D$91,Q24&lt;Assumptions!$D$92*P24/D24)),"SWITCH OFF",IF(W24&gt;=Assumptions!$D$88,"CUT 50%",IF(W24&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD")))))</f>
+        <f aca="false">IF(D24=0,"Free – monitor quality",IF(F24=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P24&lt;Assumptions!$D$85,Q24&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W24&gt;=Assumptions!$D$89,AND(R24=0,P24&gt;=Assumptions!$D$90,P24/F24&gt;=Assumptions!$D$91),AND(P24&gt;=Assumptions!$D$90,P24/F24&lt;Assumptions!$D$91,Q24&lt;Assumptions!$D$92*P24/D24)),"SWITCH OFF",IF(W24&gt;=Assumptions!$D$88,"CUT 50%",IF(W24&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
       </c>
     </row>
@@ -4691,7 +4691,7 @@
         <v>1</v>
       </c>
       <c r="X25" s="2" t="str">
-        <f aca="false">IF(F25=0,"Free – monitor quality",IF(AND(P25&lt;Assumptions!$D$85,Q25&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W25&gt;=Assumptions!$D$89,AND(R25=0,P25&gt;=Assumptions!$D$90,P25/F25&gt;=Assumptions!$D$91),AND(P25&gt;=Assumptions!$D$90,P25/F25&lt;Assumptions!$D$91,Q25&lt;Assumptions!$D$92*P25/D25)),"SWITCH OFF",IF(W25&gt;=Assumptions!$D$88,"CUT 50%",IF(W25&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD")))))</f>
+        <f aca="false">IF(D25=0,"Free – monitor quality",IF(F25=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P25&lt;Assumptions!$D$85,Q25&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W25&gt;=Assumptions!$D$89,AND(R25=0,P25&gt;=Assumptions!$D$90,P25/F25&gt;=Assumptions!$D$91),AND(P25&gt;=Assumptions!$D$90,P25/F25&lt;Assumptions!$D$91,Q25&lt;Assumptions!$D$92*P25/D25)),"SWITCH OFF",IF(W25&gt;=Assumptions!$D$88,"CUT 50%",IF(W25&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
       </c>
     </row>
@@ -4762,7 +4762,7 @@
         <v>1</v>
       </c>
       <c r="X26" s="2" t="str">
-        <f aca="false">IF(F26=0,"Free – monitor quality",IF(AND(P26&lt;Assumptions!$D$85,Q26&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W26&gt;=Assumptions!$D$89,AND(R26=0,P26&gt;=Assumptions!$D$90,P26/F26&gt;=Assumptions!$D$91),AND(P26&gt;=Assumptions!$D$90,P26/F26&lt;Assumptions!$D$91,Q26&lt;Assumptions!$D$92*P26/D26)),"SWITCH OFF",IF(W26&gt;=Assumptions!$D$88,"CUT 50%",IF(W26&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD")))))</f>
+        <f aca="false">IF(D26=0,"Free – monitor quality",IF(F26=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P26&lt;Assumptions!$D$85,Q26&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W26&gt;=Assumptions!$D$89,AND(R26=0,P26&gt;=Assumptions!$D$90,P26/F26&gt;=Assumptions!$D$91),AND(P26&gt;=Assumptions!$D$90,P26/F26&lt;Assumptions!$D$91,Q26&lt;Assumptions!$D$92*P26/D26)),"SWITCH OFF",IF(W26&gt;=Assumptions!$D$88,"CUT 50%",IF(W26&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
       </c>
     </row>
@@ -4833,7 +4833,7 @@
         <v>1</v>
       </c>
       <c r="X27" s="2" t="str">
-        <f aca="false">IF(F27=0,"Free – monitor quality",IF(AND(P27&lt;Assumptions!$D$85,Q27&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W27&gt;=Assumptions!$D$89,AND(R27=0,P27&gt;=Assumptions!$D$90,P27/F27&gt;=Assumptions!$D$91),AND(P27&gt;=Assumptions!$D$90,P27/F27&lt;Assumptions!$D$91,Q27&lt;Assumptions!$D$92*P27/D27)),"SWITCH OFF",IF(W27&gt;=Assumptions!$D$88,"CUT 50%",IF(W27&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD")))))</f>
+        <f aca="false">IF(D27=0,"Free – monitor quality",IF(F27=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P27&lt;Assumptions!$D$85,Q27&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W27&gt;=Assumptions!$D$89,AND(R27=0,P27&gt;=Assumptions!$D$90,P27/F27&gt;=Assumptions!$D$91),AND(P27&gt;=Assumptions!$D$90,P27/F27&lt;Assumptions!$D$91,Q27&lt;Assumptions!$D$92*P27/D27)),"SWITCH OFF",IF(W27&gt;=Assumptions!$D$88,"CUT 50%",IF(W27&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
       </c>
     </row>
@@ -4904,7 +4904,7 @@
         <v>1</v>
       </c>
       <c r="X28" s="2" t="str">
-        <f aca="false">IF(F28=0,"Free – monitor quality",IF(AND(P28&lt;Assumptions!$D$85,Q28&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W28&gt;=Assumptions!$D$89,AND(R28=0,P28&gt;=Assumptions!$D$90,P28/F28&gt;=Assumptions!$D$91),AND(P28&gt;=Assumptions!$D$90,P28/F28&lt;Assumptions!$D$91,Q28&lt;Assumptions!$D$92*P28/D28)),"SWITCH OFF",IF(W28&gt;=Assumptions!$D$88,"CUT 50%",IF(W28&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD")))))</f>
+        <f aca="false">IF(D28=0,"Free – monitor quality",IF(F28=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P28&lt;Assumptions!$D$85,Q28&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W28&gt;=Assumptions!$D$89,AND(R28=0,P28&gt;=Assumptions!$D$90,P28/F28&gt;=Assumptions!$D$91),AND(P28&gt;=Assumptions!$D$90,P28/F28&lt;Assumptions!$D$91,Q28&lt;Assumptions!$D$92*P28/D28)),"SWITCH OFF",IF(W28&gt;=Assumptions!$D$88,"CUT 50%",IF(W28&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
       </c>
     </row>
@@ -4975,7 +4975,7 @@
         <v>1</v>
       </c>
       <c r="X29" s="2" t="str">
-        <f aca="false">IF(F29=0,"Free – monitor quality",IF(AND(P29&lt;Assumptions!$D$85,Q29&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W29&gt;=Assumptions!$D$89,AND(R29=0,P29&gt;=Assumptions!$D$90,P29/F29&gt;=Assumptions!$D$91),AND(P29&gt;=Assumptions!$D$90,P29/F29&lt;Assumptions!$D$91,Q29&lt;Assumptions!$D$92*P29/D29)),"SWITCH OFF",IF(W29&gt;=Assumptions!$D$88,"CUT 50%",IF(W29&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD")))))</f>
+        <f aca="false">IF(D29=0,"Free – monitor quality",IF(F29=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P29&lt;Assumptions!$D$85,Q29&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W29&gt;=Assumptions!$D$89,AND(R29=0,P29&gt;=Assumptions!$D$90,P29/F29&gt;=Assumptions!$D$91),AND(P29&gt;=Assumptions!$D$90,P29/F29&lt;Assumptions!$D$91,Q29&lt;Assumptions!$D$92*P29/D29)),"SWITCH OFF",IF(W29&gt;=Assumptions!$D$88,"CUT 50%",IF(W29&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
       </c>
     </row>
@@ -5046,7 +5046,7 @@
         <v>1</v>
       </c>
       <c r="X30" s="2" t="str">
-        <f aca="false">IF(F30=0,"Free – monitor quality",IF(AND(P30&lt;Assumptions!$D$85,Q30&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W30&gt;=Assumptions!$D$89,AND(R30=0,P30&gt;=Assumptions!$D$90,P30/F30&gt;=Assumptions!$D$91),AND(P30&gt;=Assumptions!$D$90,P30/F30&lt;Assumptions!$D$91,Q30&lt;Assumptions!$D$92*P30/D30)),"SWITCH OFF",IF(W30&gt;=Assumptions!$D$88,"CUT 50%",IF(W30&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD")))))</f>
+        <f aca="false">IF(D30=0,"Free – monitor quality",IF(F30=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P30&lt;Assumptions!$D$85,Q30&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W30&gt;=Assumptions!$D$89,AND(R30=0,P30&gt;=Assumptions!$D$90,P30/F30&gt;=Assumptions!$D$91),AND(P30&gt;=Assumptions!$D$90,P30/F30&lt;Assumptions!$D$91,Q30&lt;Assumptions!$D$92*P30/D30)),"SWITCH OFF",IF(W30&gt;=Assumptions!$D$88,"CUT 50%",IF(W30&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
       </c>
     </row>
@@ -5117,7 +5117,7 @@
         <v>1</v>
       </c>
       <c r="X31" s="2" t="str">
-        <f aca="false">IF(F31=0,"Free – monitor quality",IF(AND(P31&lt;Assumptions!$D$85,Q31&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W31&gt;=Assumptions!$D$89,AND(R31=0,P31&gt;=Assumptions!$D$90,P31/F31&gt;=Assumptions!$D$91),AND(P31&gt;=Assumptions!$D$90,P31/F31&lt;Assumptions!$D$91,Q31&lt;Assumptions!$D$92*P31/D31)),"SWITCH OFF",IF(W31&gt;=Assumptions!$D$88,"CUT 50%",IF(W31&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD")))))</f>
+        <f aca="false">IF(D31=0,"Free – monitor quality",IF(F31=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P31&lt;Assumptions!$D$85,Q31&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W31&gt;=Assumptions!$D$89,AND(R31=0,P31&gt;=Assumptions!$D$90,P31/F31&gt;=Assumptions!$D$91),AND(P31&gt;=Assumptions!$D$90,P31/F31&lt;Assumptions!$D$91,Q31&lt;Assumptions!$D$92*P31/D31)),"SWITCH OFF",IF(W31&gt;=Assumptions!$D$88,"CUT 50%",IF(W31&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
       </c>
     </row>
@@ -5188,7 +5188,7 @@
         <v>1</v>
       </c>
       <c r="X32" s="2" t="str">
-        <f aca="false">IF(F32=0,"Free – monitor quality",IF(AND(P32&lt;Assumptions!$D$85,Q32&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W32&gt;=Assumptions!$D$89,AND(R32=0,P32&gt;=Assumptions!$D$90,P32/F32&gt;=Assumptions!$D$91),AND(P32&gt;=Assumptions!$D$90,P32/F32&lt;Assumptions!$D$91,Q32&lt;Assumptions!$D$92*P32/D32)),"SWITCH OFF",IF(W32&gt;=Assumptions!$D$88,"CUT 50%",IF(W32&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD")))))</f>
+        <f aca="false">IF(D32=0,"Free – monitor quality",IF(F32=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P32&lt;Assumptions!$D$85,Q32&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W32&gt;=Assumptions!$D$89,AND(R32=0,P32&gt;=Assumptions!$D$90,P32/F32&gt;=Assumptions!$D$91),AND(P32&gt;=Assumptions!$D$90,P32/F32&lt;Assumptions!$D$91,Q32&lt;Assumptions!$D$92*P32/D32)),"SWITCH OFF",IF(W32&gt;=Assumptions!$D$88,"CUT 50%",IF(W32&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
         <v>1</v>
       </c>
       <c r="X33" s="2" t="str">
-        <f aca="false">IF(F33=0,"Free – monitor quality",IF(AND(P33&lt;Assumptions!$D$85,Q33&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W33&gt;=Assumptions!$D$89,AND(R33=0,P33&gt;=Assumptions!$D$90,P33/F33&gt;=Assumptions!$D$91),AND(P33&gt;=Assumptions!$D$90,P33/F33&lt;Assumptions!$D$91,Q33&lt;Assumptions!$D$92*P33/D33)),"SWITCH OFF",IF(W33&gt;=Assumptions!$D$88,"CUT 50%",IF(W33&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD")))))</f>
+        <f aca="false">IF(D33=0,"Free – monitor quality",IF(F33=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P33&lt;Assumptions!$D$85,Q33&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W33&gt;=Assumptions!$D$89,AND(R33=0,P33&gt;=Assumptions!$D$90,P33/F33&gt;=Assumptions!$D$91),AND(P33&gt;=Assumptions!$D$90,P33/F33&lt;Assumptions!$D$91,Q33&lt;Assumptions!$D$92*P33/D33)),"SWITCH OFF",IF(W33&gt;=Assumptions!$D$88,"CUT 50%",IF(W33&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
       </c>
     </row>
@@ -5330,7 +5330,7 @@
         <v>1</v>
       </c>
       <c r="X34" s="2" t="str">
-        <f aca="false">IF(F34=0,"Free – monitor quality",IF(AND(P34&lt;Assumptions!$D$85,Q34&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W34&gt;=Assumptions!$D$89,AND(R34=0,P34&gt;=Assumptions!$D$90,P34/F34&gt;=Assumptions!$D$91),AND(P34&gt;=Assumptions!$D$90,P34/F34&lt;Assumptions!$D$91,Q34&lt;Assumptions!$D$92*P34/D34)),"SWITCH OFF",IF(W34&gt;=Assumptions!$D$88,"CUT 50%",IF(W34&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD")))))</f>
+        <f aca="false">IF(D34=0,"Free – monitor quality",IF(F34=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P34&lt;Assumptions!$D$85,Q34&lt;Assumptions!$D$86),"Wait – too little data",IF(OR(W34&gt;=Assumptions!$D$89,AND(R34=0,P34&gt;=Assumptions!$D$90,P34/F34&gt;=Assumptions!$D$91),AND(P34&gt;=Assumptions!$D$90,P34/F34&lt;Assumptions!$D$91,Q34&lt;Assumptions!$D$92*P34/D34)),"SWITCH OFF",IF(W34&gt;=Assumptions!$D$88,"CUT 50%",IF(W34&lt;=Assumptions!$D$87,"ADD +"&amp;TEXT(Assumptions!$D$100,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
       </c>
     </row>
@@ -20724,7 +20724,7 @@
         <v>322.142857142857</v>
       </c>
       <c r="S15" s="2" t="str">
-        <f aca="false">IF(LEFT(Summary!$C$19,1)&lt;&gt;"✓",Summary!$C$19,IF(Assumptions!$D$48&gt;=1,"✗ reserve share must be below 100%",IF(Funnel!B19&lt;Assumptions!$D$7,"✗ no application can sign by the deadline (Funnel B19 is before the campaign starts)",IF(AND(Budget!G24&gt;0,Funnel!B20&lt;Assumptions!$D$7),"✗ supervisors cannot apply in time (Funnel B20 is before the campaign starts)",IF(OR(ABS(D15-1)&gt;0.001,ABS(Y15-1)&gt;0.001),"✗ shares must sum to 100%",IF(AND(F20&gt;0,ABS(E15-1)&gt;0.001),"✗ no spend share falls before the supervisor cut-off (Funnel B20): move weekly shares into weeks 1–5",IF(ABS(M15-Budget!C9)&gt;1,"✗ weeks ≠ planned spend",IF(ABS(P15-Funnel!O9)&gt;0.5,"✗ qualified ≠ plan",IF(ABS(V15-Budget!C13)&gt;0.5,"✗ signatures ≠ expected hires","✓ ties to plan")))))))))</f>
+        <f aca="false">IF(LEFT(Summary!$C$19,1)&lt;&gt;"✓",Summary!$C$19,IF(Assumptions!$D$48&gt;=1,"✗ reserve share must be below 100%",IF(Funnel!B19&lt;Assumptions!$D$7,"✗ no application can sign by the deadline (Funnel B19 is before the campaign starts)",IF(AND(Budget!G24&gt;0,Funnel!B20&lt;Assumptions!$D$7),"✗ supervisors cannot apply in time (Funnel B20 is before the campaign starts)",IF(Funnel!B13&gt;Funnel!B17,"✗ assessments start (Funnel B13) after the last useful assessment day (Funnel B17): no hire can sign in time",IF(SUMPRODUCT(($B$4:$B$14&gt;Funnel!$B$19)*$D$4:$D$14)&gt;0.0001,"✗ a spend share falls after the last useful application (Funnel B19): move shares into weeks 1–6",IF(OR(ABS(D15-1)&gt;0.001,ABS(Y15-1)&gt;0.001),"✗ shares must sum to 100%",IF(AND(F20&gt;0,ABS(E15-1)&gt;0.001),"✗ no spend share falls before the supervisor cut-off (Funnel B20): move weekly shares into weeks 1–5",IF(ABS(M15-Budget!C9)&gt;1,"✗ weeks ≠ planned spend",IF(ABS(P15-Funnel!O9)&gt;0.5,"✗ qualified ≠ plan",IF(ABS(V15-Budget!C13)&gt;0.5,"✗ signatures ≠ expected hires","✓ ties to plan")))))))))))</f>
         <v>✓ ties to plan</v>
       </c>
       <c r="T15" s="29" t="n">

</xml_diff>

<commit_message>
Fold calculation-helper columns and rows into collapsible groups
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V2NJtrYy3bzNxqKeiRXJfY
</commit_message>
<xml_diff>
--- a/operation_uptime/Operation_Uptime_Model.xlsx
+++ b/operation_uptime/Operation_Uptime_Model.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1396" uniqueCount="754">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1396" uniqueCount="755">
   <si>
     <t xml:space="preserve">Operation Uptime — model summary (hypothetical Tesla Giga Berlin maintenance hiring)</t>
   </si>
@@ -1935,6 +1935,9 @@
   </si>
   <si>
     <t xml:space="preserve">Savings needed €</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID (+ to expand)</t>
   </si>
   <si>
     <t xml:space="preserve">Total € (media + fixed)</t>
@@ -9035,15 +9038,19 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AI42"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="1"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="44"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="6" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="6" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="1" max="20" min="17" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="28" min="21" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="1" max="29" min="29" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="30" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="1" max="35" min="31" style="0" width="13"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13499,7 +13506,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:R102"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="1" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="50"/>
@@ -14370,61 +14377,61 @@
     </row>
     <row r="60" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="12" t="s">
-        <v>22</v>
+        <v>636</v>
       </c>
       <c r="B60" s="12" t="s">
         <v>289</v>
       </c>
       <c r="C60" s="12" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="D60" s="12" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="E60" s="12" t="s">
         <v>621</v>
       </c>
       <c r="F60" s="12" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="G60" s="12" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="H60" s="12" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="I60" s="12" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="J60" s="12" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="K60" s="12" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="L60" s="12" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="M60" s="12" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="N60" s="12" t="s">
         <v>619</v>
       </c>
       <c r="O60" s="12" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="P60" s="12" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="Q60" s="12" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="R60" s="12" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A61" s="2" t="str">
         <f aca="false">Channels!A5</f>
         <v>C01</v>
@@ -14498,7 +14505,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="62" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A62" s="2" t="str">
         <f aca="false">Channels!A6</f>
         <v>C02</v>
@@ -14572,7 +14579,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="63" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A63" s="2" t="str">
         <f aca="false">Channels!A7</f>
         <v>C03</v>
@@ -14646,7 +14653,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="64" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A64" s="2" t="str">
         <f aca="false">Channels!A8</f>
         <v>C04</v>
@@ -14720,7 +14727,7 @@
         <v>4.8</v>
       </c>
     </row>
-    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="65" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A65" s="2" t="str">
         <f aca="false">Channels!A9</f>
         <v>C05</v>
@@ -14794,7 +14801,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="66" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A66" s="2" t="str">
         <f aca="false">Channels!A10</f>
         <v>C06</v>
@@ -14868,7 +14875,7 @@
         <v>1.02484472049689</v>
       </c>
     </row>
-    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="67" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A67" s="2" t="str">
         <f aca="false">Channels!A11</f>
         <v>C07</v>
@@ -14942,7 +14949,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="68" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A68" s="2" t="str">
         <f aca="false">Channels!A12</f>
         <v>C08</v>
@@ -15016,7 +15023,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="69" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A69" s="2" t="str">
         <f aca="false">Channels!A13</f>
         <v>C09</v>
@@ -15090,7 +15097,7 @@
         <v>13.5</v>
       </c>
     </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="70" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A70" s="2" t="str">
         <f aca="false">Channels!A14</f>
         <v>C10</v>
@@ -15164,7 +15171,7 @@
         <v>12.8835134018277</v>
       </c>
     </row>
-    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="71" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A71" s="2" t="str">
         <f aca="false">Channels!A15</f>
         <v>C11</v>
@@ -15238,7 +15245,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="72" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A72" s="2" t="str">
         <f aca="false">Channels!A16</f>
         <v>C12</v>
@@ -15312,7 +15319,7 @@
         <v>7.5</v>
       </c>
     </row>
-    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="73" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A73" s="2" t="str">
         <f aca="false">Channels!A17</f>
         <v>C13</v>
@@ -15386,7 +15393,7 @@
         <v>30.2675550787611</v>
       </c>
     </row>
-    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="74" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A74" s="2" t="str">
         <f aca="false">Channels!A18</f>
         <v>C14</v>
@@ -15460,7 +15467,7 @@
         <v>17.3998206768484</v>
       </c>
     </row>
-    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="75" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A75" s="2" t="str">
         <f aca="false">Channels!A19</f>
         <v>C15</v>
@@ -15534,7 +15541,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="76" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A76" s="2" t="str">
         <f aca="false">Channels!A20</f>
         <v>C16</v>
@@ -15608,7 +15615,7 @@
         <v>1.07142857142857</v>
       </c>
     </row>
-    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="77" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A77" s="2" t="str">
         <f aca="false">Channels!A21</f>
         <v>C17</v>
@@ -15682,7 +15689,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="78" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A78" s="2" t="str">
         <f aca="false">Channels!A22</f>
         <v>C18</v>
@@ -15756,7 +15763,7 @@
         <v>1.04748603351955</v>
       </c>
     </row>
-    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="79" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A79" s="2" t="str">
         <f aca="false">Channels!A23</f>
         <v>C19</v>
@@ -15830,7 +15837,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="80" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A80" s="2" t="str">
         <f aca="false">Channels!A24</f>
         <v>C20</v>
@@ -15904,7 +15911,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="81" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A81" s="2" t="str">
         <f aca="false">Channels!A25</f>
         <v>I1a-E</v>
@@ -15978,7 +15985,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="82" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A82" s="2" t="str">
         <f aca="false">Channels!A26</f>
         <v>I1a-M</v>
@@ -16052,7 +16059,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="83" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A83" s="2" t="str">
         <f aca="false">Channels!A27</f>
         <v>I1a-A</v>
@@ -16126,7 +16133,7 @@
         <v>7.2</v>
       </c>
     </row>
-    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="84" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A84" s="2" t="str">
         <f aca="false">Channels!A28</f>
         <v>I1a-S</v>
@@ -16200,7 +16207,7 @@
         <v>4.8</v>
       </c>
     </row>
-    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="85" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A85" s="2" t="str">
         <f aca="false">Channels!A29</f>
         <v>I1b-E</v>
@@ -16274,7 +16281,7 @@
         <v>11.25</v>
       </c>
     </row>
-    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="86" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A86" s="2" t="str">
         <f aca="false">Channels!A30</f>
         <v>I1b-M</v>
@@ -16348,7 +16355,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="87" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A87" s="2" t="str">
         <f aca="false">Channels!A31</f>
         <v>I1b-A</v>
@@ -16422,7 +16429,7 @@
         <v>4.5</v>
       </c>
     </row>
-    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="88" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A88" s="2" t="str">
         <f aca="false">Channels!A32</f>
         <v>I1b-S</v>
@@ -16496,7 +16503,7 @@
         <v>3.6</v>
       </c>
     </row>
-    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="89" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A89" s="2" t="str">
         <f aca="false">Channels!A33</f>
         <v>I2-E</v>
@@ -16570,7 +16577,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="90" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
       <c r="A90" s="2" t="str">
         <f aca="false">Channels!A34</f>
         <v>I3-M</v>
@@ -16646,7 +16653,7 @@
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E91" s="24" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16777,7 +16784,7 @@
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E99" s="2" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="F99" s="28" t="n">
         <f aca="false">SUM(O61:O90)</f>
@@ -16798,7 +16805,7 @@
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E100" s="2" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="F100" s="26" t="n">
         <f aca="false">IF(F99&gt;0,MIN(1,Funnel!$B$22/F99),1)</f>
@@ -16819,7 +16826,7 @@
     </row>
     <row r="102" customFormat="false" ht="407.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="13" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
     </row>
   </sheetData>
@@ -16843,103 +16850,104 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Z55"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="1"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="7" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="7" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="1" max="26" min="24" style="0" width="12"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="E3" s="12" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="F3" s="12" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="G3" s="12" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="H3" s="12" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="I3" s="12" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="J3" s="12" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="K3" s="12" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="L3" s="12" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="M3" s="12" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="N3" s="12" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="O3" s="12" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="P3" s="12" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="Q3" s="12" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="R3" s="12" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="S3" s="12" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="T3" s="12" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="U3" s="12" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="V3" s="12" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="W3" s="12" t="s">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="X3" s="12" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="Y3" s="12" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="Z3" s="45" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18184,7 +18192,7 @@
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="B16" s="9"/>
       <c r="C16" s="9"/>
@@ -18236,12 +18244,12 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="24" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="2" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="F19" s="37" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot",Channels!$B$5:$B$34,"&lt;&gt;I1b Employee referral sprint (bonus on hire)",Channels!$B$5:$B$34,"&lt;&gt;I1a Talent rediscovery (past applicants in ATS)")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
@@ -18250,7 +18258,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="2" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="F20" s="37" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot",Channels!$B$5:$B$34,"&lt;&gt;I1b Employee referral sprint (bonus on hire)",Channels!$B$5:$B$34,"&lt;&gt;I1a Talent rediscovery (past applicants in ATS)")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$C$5:$C$34,"Supervisors")</f>
@@ -18259,7 +18267,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="2" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="F21" s="37" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$E$5:$E$34,"Slot")</f>
@@ -18268,7 +18276,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="2" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="F22" s="37" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,"I1b Employee referral sprint (bonus on hire)",Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
@@ -18277,7 +18285,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="2" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="F23" s="37" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,"I1b Employee referral sprint (bonus on hire)",Channels!$C$5:$C$34,"Supervisors")</f>
@@ -18286,7 +18294,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="2" t="s">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="F24" s="37" t="n">
         <f aca="false">SUM(Channels!$Z$5:$Z$34)</f>
@@ -18295,7 +18303,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="2" t="s">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="F25" s="28" t="n">
         <f aca="false">SUMIFS(Channels!$AF$5:$AF$34,Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
@@ -18304,7 +18312,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="2" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="F26" s="28" t="n">
         <f aca="false">SUMIFS(Channels!$AF$5:$AF$34,Channels!$C$5:$C$34,"Supervisors")</f>
@@ -18313,7 +18321,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="2" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="F27" s="28" t="n">
         <f aca="false">SUMIFS(Channels!$AE$5:$AE$34,Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
@@ -18322,7 +18330,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="2" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="F28" s="28" t="n">
         <f aca="false">SUMIFS(Channels!$AE$5:$AE$34,Channels!$C$5:$C$34,"Supervisors")</f>
@@ -18331,7 +18339,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="2" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="F29" s="28" t="n">
         <f aca="false">SUMIFS(Channels!$AG$5:$AG$34,Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
@@ -18340,7 +18348,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="2" t="s">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="F30" s="28" t="n">
         <f aca="false">SUMIFS(Channels!$AG$5:$AG$34,Channels!$C$5:$C$34,"Supervisors")</f>
@@ -18349,7 +18357,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="2" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="F31" s="37" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)")</f>
@@ -18358,7 +18366,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="2" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="F32" s="28" t="n">
         <f aca="false">SUMIFS(Channels!$V$5:$V$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)",Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
@@ -18367,7 +18375,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="2" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="F33" s="28" t="n">
         <f aca="false">SUMIFS(Channels!$V$5:$V$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)",Channels!$C$5:$C$34,"Supervisors")</f>
@@ -18376,7 +18384,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="2" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="F34" s="28" t="n">
         <f aca="false">SUMIFS(Channels!$W$5:$W$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)",Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
@@ -18385,7 +18393,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="2" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="F35" s="28" t="n">
         <f aca="false">SUMIFS(Channels!$W$5:$W$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)",Channels!$C$5:$C$34,"Supervisors")</f>
@@ -18394,7 +18402,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="2" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="F36" s="28" t="n">
         <f aca="false">SUMIFS(Channels!$U$5:$U$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)",Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
@@ -18403,7 +18411,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="2" t="s">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="F37" s="28" t="n">
         <f aca="false">SUMIFS(Channels!$U$5:$U$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)",Channels!$C$5:$C$34,"Supervisors")</f>
@@ -18412,7 +18420,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="2" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="F38" s="26" t="n">
         <f aca="false">IF(Funnel!B23&gt;0,MIN(1,Funnel!B22/Funnel!B23),1)</f>
@@ -18421,7 +18429,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="24" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18430,37 +18438,37 @@
         <v>288</v>
       </c>
       <c r="C43" s="12" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="D43" s="12" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="E43" s="12" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="F43" s="12" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="G43" s="12" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="H43" s="12" t="s">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="I43" s="12" t="s">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="J43" s="12" t="s">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="K43" s="12" t="s">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="L43" s="12" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="M43" s="12" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="N43" s="12" t="s">
         <v>426</v>
@@ -19098,12 +19106,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>716</v>
+        <v>717</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>717</v>
+        <v>718</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -19117,67 +19125,67 @@
         <v>289</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="G4" s="12" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="H4" s="12" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="I4" s="12" t="s">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="J4" s="12" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="K4" s="12" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="L4" s="12" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="M4" s="12" t="s">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="N4" s="12" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="O4" s="12" t="s">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="P4" s="12" t="s">
-        <v>730</v>
+        <v>731</v>
       </c>
       <c r="Q4" s="12" t="s">
-        <v>731</v>
+        <v>732</v>
       </c>
       <c r="R4" s="12" t="s">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="S4" s="12" t="s">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="T4" s="12" t="s">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="U4" s="12" t="s">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="V4" s="12" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="W4" s="12" t="s">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="X4" s="12" t="s">
-        <v>738</v>
+        <v>739</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21365,7 +21373,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="24" t="s">
-        <v>739</v>
+        <v>740</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -21374,46 +21382,46 @@
         <v>289</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="D39" s="12" t="s">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="E39" s="12" t="s">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="F39" s="12" t="s">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="G39" s="12" t="s">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="H39" s="12" t="s">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="I39" s="12" t="s">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="J39" s="12" t="s">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="K39" s="12" t="s">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="L39" s="12" t="s">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="M39" s="12" t="s">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="N39" s="12" t="s">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="O39" s="12" t="s">
         <v>49</v>
       </c>
       <c r="P39" s="12" t="s">
-        <v>752</v>
+        <v>753</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21643,7 +21651,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="9" t="s">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="B46" s="9"/>
       <c r="C46" s="9"/>

</xml_diff>

<commit_message>
Verify BMJ and NIST sources; F4 back to 90% from the verified source; clean full test run
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V2NJtrYy3bzNxqKeiRXJfY
</commit_message>
<xml_diff>
--- a/operation_uptime/Operation_Uptime_Model.xlsx
+++ b/operation_uptime/Operation_Uptime_Model.xlsx
@@ -644,7 +644,7 @@
     <t xml:space="preserve">apps</t>
   </si>
   <si>
-    <t xml:space="preserve">Statistics: at the plan share qualified (~25%), 30 applications give a standard error of √(0.25 × 0.75 ÷ 30) = 7.9 points (95% range ±15.5 points). n ≥ 30 is the usual minimum for reading a proportion; the Tracker also blends each read with the plan (R8), which narrows it further.</t>
+    <t xml:space="preserve">Statistics: NIST's rule for reading a proportion is min{Np, N(1 − p)} ≥ 5 (https://www.itl.nist.gov/div898/handbook/prc/section2/prc24.htm). At the planned share qualified of ~25%, N × 0.25 ≥ 5 needs N ≥ 20; 30 applications gives N × p = 7.5 and a standard error of √(0.25 × 0.75 ÷ 30) = 7.9 points.</t>
   </si>
   <si>
     <t xml:space="preserve">R3</t>
@@ -656,7 +656,7 @@
     <t xml:space="preserve">× plan</t>
   </si>
   <si>
-    <t xml:space="preserve">Statistics: one-sided 95% test (z = 1.645, the standard α = 5%). At the first judgement (30 applications, R2) the plan-blended share qualified (R8, equal weights) has a relative standard error of 16% (raw √(0.25 × 0.75 ÷ 30) = 7.9 points ÷ 25% = 32%, halved by the blend). Better than plan with 95% confidence = 1 − 1.645 × 0.16 = 0.74 → 0.75.</t>
+    <t xml:space="preserve">NIST/SEMATECH e-Handbook: 'in practice values of 0.1, 0.05, and 0.01 are common' for the significance level α (https://www.itl.nist.gov/div898/handbook/prc/section1/prc131.htm). One-sided test at α = 5% (z = 1.645). At the first judgement point (30 applications, R2) the plan-blended share qualified (R8, equal weights) has a relative standard error of 16% (raw √(0.25 × 0.75 ÷ 30) = 7.9 points ÷ 25% = 32%, halved by the blend). Better than plan with 95% confidence = 1 − 1.645 × 0.16 = 0.74 → 0.75.</t>
   </si>
   <si>
     <t xml:space="preserve">R4</t>
@@ -716,7 +716,7 @@
     <t xml:space="preserve">Initiatives</t>
   </si>
   <si>
-    <t xml:space="preserve">Statistics convention: 5% significance level (the standard α). Each bar is the Poisson quantile of the initiative's planned qualified in its 14-day window (Initiatives col G/I, CRITBINOM with n = 100,000). An initiative running at plan reaches the PASS bar with ≥95% probability; one far below plan does not.</t>
+    <t xml:space="preserve">NIST/SEMATECH e-Handbook: 'in practice values of 0.1, 0.05, and 0.01 are common' for the significance level α (https://www.itl.nist.gov/div898/handbook/prc/section1/prc131.htm). PASS uses α = 5%. Each bar is the Poisson quantile of the initiative's planned qualified in its 14-day window (Initiatives col G/I, CRITBINOM with n = 100,000). An initiative running at plan reaches the PASS bar with ≥95% probability.</t>
   </si>
   <si>
     <t xml:space="preserve">TP2</t>
@@ -734,7 +734,7 @@
     <t xml:space="preserve">Initiative test: KILL bar significance level (an on-plan initiative falls below the bar with less than this probability)</t>
   </si>
   <si>
-    <t xml:space="preserve">Statistics convention: 1% significance level (the standard 'strong evidence' α). Each bar is the Poisson quantile of the initiative's planned qualified in its 14-day window (Initiatives col G/I, CRITBINOM with n = 100,000). An initiative running at plan falls below the KILL bar with &lt;1% probability, so a result there means the mechanism is not working.</t>
+    <t xml:space="preserve">NIST/SEMATECH e-Handbook: 'in practice values of 0.1, 0.05, and 0.01 are common' for the significance level α (https://www.itl.nist.gov/div898/handbook/prc/section1/prc131.htm). KILL uses α = 1%, the strictest common level, because killing is irreversible. Each bar is the Poisson quantile of the initiative's planned qualified in its 14-day window (Initiatives col G/I, CRITBINOM with n = 100,000). An initiative running at plan falls below the KILL bar with &lt;1% probability.</t>
   </si>
   <si>
     <t xml:space="preserve">TK2</t>
@@ -791,7 +791,7 @@
     <t xml:space="preserve">interviews</t>
   </si>
   <si>
-    <t xml:space="preserve">Statistics: below 10 interviews one result moves the pass rate by more than 10 points (1 ÷ 10). 10 is the smallest sample with n × p ≥ 5 at the ~50% planned pass rate (normal-approximation rule).</t>
+    <t xml:space="preserve">Statistics: NIST's min{Np, N(1 − p)} ≥ 5 rule (https://www.itl.nist.gov/div898/handbook/prc/section2/prc24.htm) at the ~50% planned pass rate needs N ≥ 10 interviews.</t>
   </si>
   <si>
     <t xml:space="preserve">R10</t>
@@ -803,7 +803,7 @@
     <t xml:space="preserve">offers</t>
   </si>
   <si>
-    <t xml:space="preserve">Statistics: same rule as R9. At the ~70% planned acceptance, n × p ≥ 5 needs 5 ÷ 0.70 = 7.1 offers, so 7. Until then the planned acceptance rate is used.</t>
+    <t xml:space="preserve">Statistics: NIST's min{Np, N(1 − p)} ≥ 5 rule (https://www.itl.nist.gov/div898/handbook/prc/section2/prc24.htm) at the 70% planned acceptance: N × 0.70 ≥ 5 needs N ≥ 7.1 → 7 offers (N × 0.30 ≥ 5 would need 17, more offers than exist before the first check, so the Tracker blends with the plan until then).</t>
   </si>
   <si>
     <t xml:space="preserve">F1</t>
@@ -836,7 +836,7 @@
     <t xml:space="preserve">Funnel / Weekly</t>
   </si>
   <si>
-    <t xml:space="preserve">Published standard: occupancy above 85% leads to regular capacity crises (Bagust, Place &amp; Posnett, BMJ 1999, 'Dynamics of bed use in accommodating emergency admissions', https://www.bmj.com/content/319/7203/155), the origin of the widely used 85% utilisation rule. Queueing theory gives the same knee: waiting grows with ρ ÷ (1 − ρ), 5.7× at 85% (https://en.wikipedia.org/wiki/Kingman%27s_formula).</t>
+    <t xml:space="preserve">Bagust, Place &amp; Posnett, BMJ 1999;319:155 (abstract, https://pubmed.ncbi.nlm.nih.gov/10406748/): 'Risks are discernible when average bed occupancy rates exceed about 85%'. Same shape as queueing theory, where waiting grows with ρ ÷ (1 − ρ).</t>
   </si>
   <si>
     <t xml:space="preserve">F4</t>
@@ -848,7 +848,7 @@
     <t xml:space="preserve">Weekly</t>
   </si>
   <si>
-    <t xml:space="preserve">Derivation: a week is full when less than one day of assessments is spare: 1 − 1/7 = 86% (slots are counted per calendar day, 55 ÷ 7 = 7.9 a day).</t>
+    <t xml:space="preserve">Bagust, Place &amp; Posnett, BMJ 1999 (https://pubmed.ncbi.nlm.nih.gov/10406748/): 'regular bed shortages and periodic bed crises if average bed occupancy rises to 90% or more'. A week above 90% of its slots is therefore treated as full.</t>
   </si>
   <si>
     <t xml:space="preserve">R13</t>
@@ -860,7 +860,7 @@
     <t xml:space="preserve">qualified/wk</t>
   </si>
   <si>
-    <t xml:space="preserve">Derivation: = F4 × G3 = 0.86 × 55 = 47. A week forecast below 'full' has at least one day of slots spare, so reserve is released to the cheapest cells with capacity.</t>
+    <t xml:space="preserve">Derivation: = F4 × G3 = 0.90 × 55 = 49.5 → 50. A week forecast below 'full' has spare slots, so reserve is released to the cheapest cells with capacity.</t>
   </si>
   <si>
     <t xml:space="preserve">R8</t>
@@ -869,7 +869,7 @@
     <t xml:space="preserve">Weight given to plan when updating qualified share (pseudo-applications)</t>
   </si>
   <si>
-    <t xml:space="preserve">Derivation: beta-binomial (empirical-Bayes) update with a prior worth 30 applications = R2. At the first point a cell may be judged (30 applications), its own data and the plan count equally; after 90 applications the data carry 75% of the weight.</t>
+    <t xml:space="preserve">Derivation: beta-binomial update whose prior is worth exactly R2 = 30 applications, so at the first point a cell may be judged its own data and the plan carry equal weight; after 90 applications the data carry 75%.</t>
   </si>
   <si>
     <t xml:space="preserve">7. Channel × role inputs (Part 2.2). Basis: CPC → CPA = CPC ÷ click-to-apply rate; CPA = bought per application/lead; Slot = fixed-price 30-day ad → CPA = price ÷ apps per ad; Free = no media cost.</t>
@@ -1055,7 +1055,7 @@
     <t xml:space="preserve">records</t>
   </si>
   <si>
-    <t xml:space="preserve">Derivation: German practice keeps rejected applicants' data 6 months, or up to 1 year with talent-pool consent (Haufe: https://www.haufe.de/compliance/management-praxis/aufbewahrung-wie-lange-duerfen-bewerberdaten-gespeichert-werden_230130_261218.html), so the usable pool is ~1 year of runners-up. Maintenance share: maintenance and the campaign's trades (KldB 2513 Wartung/Instandhaltung 240,934 + 2625 124,699 + 2611 84,727 + 2612 49,171 + supervisors 2519/2619/2629 36,989 = 536,520) are 7.8% of all production occupations (KldB 21–29: 6,850,263) in Germany (BA, 31.12.2025, https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-d-0-202512-xlsx.xlsx?__blob=publicationFile). Maintenance hires a year ≈ 10,703 staff (https://electrek.co/2026/03/04/tesla-giga-berlin-ig-metall-union-vote-collapse/) × 7.8% × 12% turnover (IAB-Betriebspanel Brandenburg 2024) = 100. Qualified runners-up per hire = 1 ÷ 0.32 qualified → signed − 1 = 2.1. Pool = 100 × 2.1 = 211, split by this campaign's openings (30/45/15/10%). The client's day-1 ATS export replaces it.</t>
+    <t xml:space="preserve">Derivation: German practice keeps rejected applicants' data 6 months, or up to 1 year with talent-pool consent (Haufe: https://www.haufe.de/compliance/management-praxis/aufbewahrung-wie-lange-duerfen-bewerberdaten-gespeichert-werden_230130_261218.html), so the usable pool is ~1 year of runners-up. Maintenance share: the occupations this campaign hires from, KldB 2513 maintenance technicians (Wartung/Instandhaltung) 240,934 + 2625 industrial electricians 124,699 + 2611 mechatronics 84,727 + 2612 automation 49,171 + their supervisor codes 2519/2619/2629 36,989 = 536,520, are 7.8% of all production occupations (KldB 21–29: 6,850,263) in Germany (BA, 31.12.2025, https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-d-0-202512-xlsx.xlsx?__blob=publicationFile); 7.3% without the supervisor codes. Maintenance hires a year ≈ 10,703 staff (https://electrek.co/2026/03/04/tesla-giga-berlin-ig-metall-union-vote-collapse/) × 7.8% × 12% turnover (IAB-Betriebspanel Brandenburg 2024) = 100. Qualified runners-up per hire = 1 ÷ 0.32 qualified → signed − 1 = 2.1. Pool = 100 × 2.1 = 211, split by this campaign's openings (30/45/15/10%). The client's day-1 ATS export replaces it.</t>
   </si>
   <si>
     <t xml:space="preserve">I1RM</t>
@@ -4832,7 +4832,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="86" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="2" t="s">
         <v>202</v>
       </c>
@@ -4851,11 +4851,11 @@
       <c r="F86" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="G86" s="13" t="s">
+      <c r="G86" s="17" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="87" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="87" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="2" t="s">
         <v>206</v>
       </c>
@@ -4874,7 +4874,7 @@
       <c r="F87" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="G87" s="13" t="s">
+      <c r="G87" s="17" t="s">
         <v>209</v>
       </c>
     </row>
@@ -5012,7 +5012,7 @@
       <c r="F93" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="G93" s="13" t="s">
+      <c r="G93" s="17" t="s">
         <v>229</v>
       </c>
     </row>
@@ -5039,7 +5039,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="95" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="95" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="2" t="s">
         <v>233</v>
       </c>
@@ -5058,7 +5058,7 @@
       <c r="F95" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="G95" s="13" t="s">
+      <c r="G95" s="17" t="s">
         <v>235</v>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       <c r="F101" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="G101" s="13" t="s">
+      <c r="G101" s="17" t="s">
         <v>254</v>
       </c>
     </row>
@@ -5219,7 +5219,7 @@
       <c r="F102" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="G102" s="13" t="s">
+      <c r="G102" s="17" t="s">
         <v>258</v>
       </c>
     </row>
@@ -5303,15 +5303,15 @@
         <v>272</v>
       </c>
       <c r="D106" s="16" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="E106" s="2" t="s">
         <v>46</v>
       </c>
       <c r="F106" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="G106" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="G106" s="17" t="s">
         <v>273</v>
       </c>
     </row>
@@ -5326,7 +5326,7 @@
         <v>40</v>
       </c>
       <c r="D107" s="15" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="E107" s="2" t="s">
         <v>276</v>
@@ -6858,63 +6858,70 @@
     <hyperlink ref="G79" r:id="rId34" display="Derivation: national stock (BA, 31.12.2025, bo-heft Germany: https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-d-0-202512-xlsx.xlsx?__blob=publicationFile) × 92.8% living outside Berlin-Brandenburg × 2.6% changing Bundesland of work a year (IAB Kurzbericht 4/2000, https://doku.iab.de/kurzber/2000/kb0400.pdf) × 6/52 of a year × 11.9% of inter-state movers choosing Berlin or Brandenburg (Destatis Binnenwanderung 2025, https://www.destatis.de/DE/Themen/Gesellschaft-Umwelt/Bevoelkerung/Wanderungen/Tabellen/_tabellen-liste-nach-bundeslaendern-jahr.html). 84,727 × 0.928 × 0.026 × 6/52 × 0.119 = 28. Upper-bound rates used (the all-ages migration rate is 1.19%)."/>
     <hyperlink ref="G80" r:id="rId35" display="Derivation: national stock (BA, 31.12.2025, bo-heft Germany: https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-d-0-202512-xlsx.xlsx?__blob=publicationFile) × 92.8% living outside Berlin-Brandenburg × 2.6% changing Bundesland of work a year (IAB Kurzbericht 4/2000, https://doku.iab.de/kurzber/2000/kb0400.pdf) × 6/52 of a year × 11.9% of inter-state movers choosing Berlin or Brandenburg (Destatis Binnenwanderung 2025, https://www.destatis.de/DE/Themen/Gesellschaft-Umwelt/Bevoelkerung/Wanderungen/Tabellen/_tabellen-liste-nach-bundeslaendern-jahr.html). 49,171 × 0.928 × 0.026 × 6/52 × 0.119 = 16. Upper-bound rates used (the all-ages migration rate is 1.19%)."/>
     <hyperlink ref="G81" r:id="rId36" display="Derivation: national stock (BA, 31.12.2025, bo-heft Germany: https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-d-0-202512-xlsx.xlsx?__blob=publicationFile) × 92.8% living outside Berlin-Brandenburg × 2.6% changing Bundesland of work a year (IAB Kurzbericht 4/2000, https://doku.iab.de/kurzber/2000/kb0400.pdf) × 6/52 of a year × 11.9% of inter-state movers choosing Berlin or Brandenburg (Destatis Binnenwanderung 2025, https://www.destatis.de/DE/Themen/Gesellschaft-Umwelt/Bevoelkerung/Wanderungen/Tabellen/_tabellen-liste-nach-bundeslaendern-jahr.html). 10,746 × 0.928 × 0.026 × 6/52 × 0.119 = 4. Upper-bound rates used (the all-ages migration rate is 1.19%)."/>
-    <hyperlink ref="G88" r:id="rId37" display="Statistics: 1.5× plan is about three standard errors worse (see R3), so the cell is very likely worse than plan. Practice: 'turn off a Meta ad once it has spent 1.5x your target CPA without a single conversion' (https://sparkugc.com/resources/when-to-kill-a-meta-ad-cpa-rule); here the response is a 50% cut, the full stop comes at R5."/>
-    <hyperlink ref="G89" r:id="rId38" display="Practice: 'Pause if CPA over 2x target' (https://roaspig.com/blog/automated-rules-manage-meta-budgets/). At 2× plan the same money buys twice the qualified applicants in a cell running at plan."/>
-    <hyperlink ref="G90" r:id="rId39" display="Derivation: equal to the test tranche B2, so the decision falls when the test is spent. Combined with R11 = 3 expected qualified, this matches the practitioner rule 'Spent 3× your target CPA with zero purchases? Kill it' (https://coinis.com/blog/when-to-kill-meta-ads-decision-framework)."/>
-    <hyperlink ref="G91" r:id="rId40" display="Statistics: Poisson P(0 | mean 3) = e^−3 = 5%, so a cell that reaches its test spend with zero qualified is wrong at most 1 time in 20 (with mean 2 it would be 13.5%). Matches the '3× target CPA with zero conversions' practice (https://coinis.com/blog/when-to-kill-meta-ads-decision-framework). Cells expecting fewer than 3 are judged on applications (R12)."/>
-    <hyperlink ref="G96" r:id="rId41" display="Derivation: the same multiple as the channel switch-off rule R5 (2×, 'Pause if CPA over 2x target', https://roaspig.com/blog/automated-rules-manage-meta-budgets/)."/>
-    <hyperlink ref="G97" r:id="rId42" display="Derivation from Pin 2026 reply timing (50% of replies within 4 h, 74.8% within 24 h, 93.9% within 7 days) and replies by message step (43.8% / 33.7% / 15.7%) (https://www.pin.com/blog/recruiting-outreach-benchmark-report/). Waves go out on day 2 (Wed 21 Oct), day 7 (Mon 26 Oct) and day 14 (Mon 2 Nov): week 1 = 0.47 × 0.90 + 0.36 × 0.50 = 60%; week 2 = 0.47 × 0.07 + 0.36 × 0.47 + 0.17 × 0.50 = 29%; week 3 = the rest, 11%."/>
-    <hyperlink ref="G98" r:id="rId43" display="Derivation from Pin 2026 reply timing (50% of replies within 4 h, 74.8% within 24 h, 93.9% within 7 days) and replies by message step (43.8% / 33.7% / 15.7%) (https://www.pin.com/blog/recruiting-outreach-benchmark-report/). Waves go out on day 2 (Wed 21 Oct), day 7 (Mon 26 Oct) and day 14 (Mon 2 Nov): week 1 = 0.47 × 0.90 + 0.36 × 0.50 = 60%; week 2 = 0.47 × 0.07 + 0.36 × 0.47 + 0.17 × 0.50 = 29%; week 3 = the rest, 11%."/>
-    <hyperlink ref="G99" r:id="rId44" display="Derivation from Pin 2026 reply timing (50% of replies within 4 h, 74.8% within 24 h, 93.9% within 7 days) and replies by message step (43.8% / 33.7% / 15.7%) (https://www.pin.com/blog/recruiting-outreach-benchmark-report/). Waves go out on day 2 (Wed 21 Oct), day 7 (Mon 26 Oct) and day 14 (Mon 2 Nov): week 1 = 0.47 × 0.90 + 0.36 × 0.50 = 60%; week 2 = 0.47 × 0.07 + 0.36 × 0.47 + 0.17 × 0.50 = 29%; week 3 = the rest, 11%."/>
-    <hyperlink ref="G100" r:id="rId45" display="Practice: budget rules use +20% ('safe') to +30% ('aggressive') per step (https://roaspig.com/blog/automated-rules-manage-meta-budgets/); Meta warns that large budget edits restart the learning phase (https://www.facebook.com/business/help/112167992830700). +25% once a week also gives Google bidding the 1–2 conversion cycles it needs between changes (https://support.google.com/google-ads/answer/6268637)."/>
-    <hyperlink ref="G103" r:id="rId46" display="Display flag only (changes no number). No published standard for 'share of the reachable pool'. Above 1 in 4 of everyone reachable and open to a move, a 30% miss in response rates (the sensitivity test) cannot be absorbed from the same pool. Proxy: BA Engpassanalyse treats fewer than 2 job seekers per vacancy as the tightest band (https://statistik.arbeitsagentur.de/DE/Navigation/Statistiken/Interaktive-Statistiken/Fachkraeftebedarf/Engpassanalyse-Nav.html)."/>
-    <hyperlink ref="G105" r:id="rId47" display="Published standard: occupancy above 85% leads to regular capacity crises (Bagust, Place &amp; Posnett, BMJ 1999, 'Dynamics of bed use in accommodating emergency admissions', https://www.bmj.com/content/319/7203/155), the origin of the widely used 85% utilisation rule. Queueing theory gives the same knee: waiting grows with ρ ÷ (1 − ρ), 5.7× at 85% (https://en.wikipedia.org/wiki/Kingman%27s_formula)."/>
-    <hyperlink ref="L112" r:id="rId48" display="Free: BA Jobbörse posting is free (https://www.arbeitsagentur.de/faktor-a/mitarbeiter-finden/so-funktioniert-deutschlands-groesste-jobboerse); Google for Jobs is free. Channel quality index from IAB-Stellenerhebung 2025: share of hires where a channel was decisive ÷ share where it was used: job boards 21/57 = 0.37, own homepage 20/70 = 0.29, referrals 27/48 = 0.56 (https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/); scaled so these three average 1 → job boards 0.90, homepage 0.71, referrals 1.37. Social media 7/40 = 0.18 vs job boards 16/51 = 0.31 in 2021 (https://iab-forum.de/iab-stellenerhebung-1-2022-174-millionen-offene-stellen-am-arbeitsmarkt/) → 0.57 × 0.90 = 0.50. Share qualified = role baseline Q (25%) × 0.71 = 17.8%. Volume: openings × 27 applications per vacancy at firms with 250+ staff (IAB, https://iab-forum.de/iab-stellenerhebung-2-2026-fast-drei-von-vier-bewerbungen-sind-aus-betrieblicher-sicht-ungeeignet/) × 13% of applications via the careers page (CareerPlug 2025, https://www.careerplug.com/wp-content/uploads/2025/04/Recruiting-Metrics-Report.pdf) = 30 × 27 × 0.13 = 105. Downstream adjustment ×1.0 and fixed cost €0: no published evidence of a channel-specific effect once an applicant is qualified, and no set-up fee beyond the media price."/>
-    <hyperlink ref="L113" r:id="rId49" display="Free: BA Jobbörse posting is free (https://www.arbeitsagentur.de/faktor-a/mitarbeiter-finden/so-funktioniert-deutschlands-groesste-jobboerse); Google for Jobs is free. Channel quality index from IAB-Stellenerhebung 2025: share of hires where a channel was decisive ÷ share where it was used: job boards 21/57 = 0.37, own homepage 20/70 = 0.29, referrals 27/48 = 0.56 (https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/); scaled so these three average 1 → job boards 0.90, homepage 0.71, referrals 1.37. Social media 7/40 = 0.18 vs job boards 16/51 = 0.31 in 2021 (https://iab-forum.de/iab-stellenerhebung-1-2022-174-millionen-offene-stellen-am-arbeitsmarkt/) → 0.57 × 0.90 = 0.50. Share qualified = role baseline Q (25%) × 0.71 = 17.8%. Volume: openings × 27 applications per vacancy at firms with 250+ staff (IAB, https://iab-forum.de/iab-stellenerhebung-2-2026-fast-drei-von-vier-bewerbungen-sind-aus-betrieblicher-sicht-ungeeignet/) × 13% of applications via the careers page (CareerPlug 2025, https://www.careerplug.com/wp-content/uploads/2025/04/Recruiting-Metrics-Report.pdf) = 45 × 27 × 0.13 = 158. Downstream adjustment ×1.0 and fixed cost €0: no published evidence of a channel-specific effect once an applicant is qualified, and no set-up fee beyond the media price."/>
-    <hyperlink ref="L114" r:id="rId50" display="Free: BA Jobbörse posting is free (https://www.arbeitsagentur.de/faktor-a/mitarbeiter-finden/so-funktioniert-deutschlands-groesste-jobboerse); Google for Jobs is free. Channel quality index from IAB-Stellenerhebung 2025: share of hires where a channel was decisive ÷ share where it was used: job boards 21/57 = 0.37, own homepage 20/70 = 0.29, referrals 27/48 = 0.56 (https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/); scaled so these three average 1 → job boards 0.90, homepage 0.71, referrals 1.37. Social media 7/40 = 0.18 vs job boards 16/51 = 0.31 in 2021 (https://iab-forum.de/iab-stellenerhebung-1-2022-174-millionen-offene-stellen-am-arbeitsmarkt/) → 0.57 × 0.90 = 0.50. Share qualified = role baseline Q (25%) × 0.71 = 17.8%. Volume: openings × 27 applications per vacancy at firms with 250+ staff (IAB, https://iab-forum.de/iab-stellenerhebung-2-2026-fast-drei-von-vier-bewerbungen-sind-aus-betrieblicher-sicht-ungeeignet/) × 13% of applications via the careers page (CareerPlug 2025, https://www.careerplug.com/wp-content/uploads/2025/04/Recruiting-Metrics-Report.pdf) = 15 × 27 × 0.13 = 53. Downstream adjustment ×1.0 and fixed cost €0: no published evidence of a channel-specific effect once an applicant is qualified, and no set-up fee beyond the media price."/>
-    <hyperlink ref="L115" r:id="rId51" display="Free: BA Jobbörse posting is free (https://www.arbeitsagentur.de/faktor-a/mitarbeiter-finden/so-funktioniert-deutschlands-groesste-jobboerse); Google for Jobs is free. Channel quality index from IAB-Stellenerhebung 2025: share of hires where a channel was decisive ÷ share where it was used: job boards 21/57 = 0.37, own homepage 20/70 = 0.29, referrals 27/48 = 0.56 (https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/); scaled so these three average 1 → job boards 0.90, homepage 0.71, referrals 1.37. Social media 7/40 = 0.18 vs job boards 16/51 = 0.31 in 2021 (https://iab-forum.de/iab-stellenerhebung-1-2022-174-millionen-offene-stellen-am-arbeitsmarkt/) → 0.57 × 0.90 = 0.50. Share qualified = role baseline Q (23%) × 0.71 = 16.3%. Volume: openings × 27 applications per vacancy at firms with 250+ staff (IAB, https://iab-forum.de/iab-stellenerhebung-2-2026-fast-drei-von-vier-bewerbungen-sind-aus-betrieblicher-sicht-ungeeignet/) × 13% of applications via the careers page (CareerPlug 2025, https://www.careerplug.com/wp-content/uploads/2025/04/Recruiting-Metrics-Report.pdf) = 10 × 27 × 0.13 = 35. Downstream adjustment ×1.0 and fixed cost €0: no published evidence of a channel-specific effect once an applicant is qualified, and no set-up fee beyond the media price."/>
-    <hyperlink ref="L116" r:id="rId52" display="Indeed Germany bills per started application since 1 Mar 2024 (https://www.personalwirtschaft.de/?p=162207). DACH median cost per application on Indeed: €161 (TalentBait, 2,549 campaigns, 2024–26: https://www.talentbait.de/recruiting-kanaele-uebersicht/). Channel quality index from IAB-Stellenerhebung 2025: share of hires where a channel was decisive ÷ share where it was used: job boards 21/57 = 0.37, own homepage 20/70 = 0.29, referrals 27/48 = 0.56 (https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/); scaled so these three average 1 → job boards 0.90, homepage 0.71, referrals 1.37. Social media 7/40 = 0.18 vs job boards 16/51 = 0.31 in 2021 (https://iab-forum.de/iab-stellenerhebung-1-2022-174-millionen-offene-stellen-am-arbeitsmarkt/) → 0.57 × 0.90 = 0.50. Share qualified = role baseline Q (25%) × 0.90 = 22.5%. Volume cap: Indeed is used by 36% of skilled-worker job seekers ('Indeed mit einem Nutzungsgrad von 36 Prozent an der Spitze', Trendence 2023, n = 42,817, https://www.personalwirtschaft.de/?p=157882); the other programmatic boards overlap with it, so Indeed alone is used. Cap = reachable in-market qualified pool (Funnel pool check: 569) × 0.36 reach ÷ 22.5% qualified = 910 applications (channels overlap, so caps are not additive; the pool check shows the total against the pool). Downstream adjustment ×1.0 and fixed cost €0: no published evidence of a channel-specific effect once an applicant is qualified, and no set-up fee beyond the media price."/>
-    <hyperlink ref="L117" r:id="rId53" display="Indeed Germany bills per started application since 1 Mar 2024 (https://www.personalwirtschaft.de/?p=162207). DACH median cost per application on Indeed: €161 (TalentBait, 2,549 campaigns, 2024–26: https://www.talentbait.de/recruiting-kanaele-uebersicht/). Channel quality index from IAB-Stellenerhebung 2025: share of hires where a channel was decisive ÷ share where it was used: job boards 21/57 = 0.37, own homepage 20/70 = 0.29, referrals 27/48 = 0.56 (https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/); scaled so these three average 1 → job boards 0.90, homepage 0.71, referrals 1.37. Social media 7/40 = 0.18 vs job boards 16/51 = 0.31 in 2021 (https://iab-forum.de/iab-stellenerhebung-1-2022-174-millionen-offene-stellen-am-arbeitsmarkt/) → 0.57 × 0.90 = 0.50. Share qualified = role baseline Q (25%) × 0.90 = 22.5%. Volume cap: Indeed is used by 36% of skilled-worker job seekers ('Indeed mit einem Nutzungsgrad von 36 Prozent an der Spitze', Trendence 2023, n = 42,817, https://www.personalwirtschaft.de/?p=157882); the other programmatic boards overlap with it, so Indeed alone is used. Cap = reachable in-market qualified pool (Funnel pool check: 2,932) × 0.36 reach ÷ 22.5% qualified = 4,690 applications (channels overlap, so caps are not additive; the pool check shows the total against the pool). Downstream adjustment ×1.0 and fixed cost €0: no published evidence of a channel-specific effect once an applicant is qualified, and no set-up fee beyond the media price."/>
-    <hyperlink ref="L118" r:id="rId54" display="Indeed Germany bills per started application since 1 Mar 2024 (https://www.personalwirtschaft.de/?p=162207). DACH median cost per application on Indeed: €161 (TalentBait, 2,549 campaigns, 2024–26: https://www.talentbait.de/recruiting-kanaele-uebersicht/). Channel quality index from IAB-Stellenerhebung 2025: share of hires where a channel was decisive ÷ share where it was used: job boards 21/57 = 0.37, own homepage 20/70 = 0.29, referrals 27/48 = 0.56 (https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/); scaled so these three average 1 → job boards 0.90, homepage 0.71, referrals 1.37. Social media 7/40 = 0.18 vs job boards 16/51 = 0.31 in 2021 (https://iab-forum.de/iab-stellenerhebung-1-2022-174-millionen-offene-stellen-am-arbeitsmarkt/) → 0.57 × 0.90 = 0.50. Share qualified = role baseline Q (25%) × 0.90 = 22.5%. Volume cap: Indeed is used by 36% of skilled-worker job seekers ('Indeed mit einem Nutzungsgrad von 36 Prozent an der Spitze', Trendence 2023, n = 42,817, https://www.personalwirtschaft.de/?p=157882); the other programmatic boards overlap with it, so Indeed alone is used. Cap = reachable in-market qualified pool (Funnel pool check: 236) × 0.36 reach ÷ 22.5% qualified = 380 applications (channels overlap, so caps are not additive; the pool check shows the total against the pool). Downstream adjustment ×1.0 and fixed cost €0: no published evidence of a channel-specific effect once an applicant is qualified, and no set-up fee beyond the media price."/>
-    <hyperlink ref="L119" r:id="rId55" display="Indeed Germany bills per started application since 1 Mar 2024 (https://www.personalwirtschaft.de/?p=162207). DACH median cost per application on Indeed: €161 (TalentBait, 2,549 campaigns, 2024–26: https://www.talentbait.de/recruiting-kanaele-uebersicht/). Channel quality index from IAB-Stellenerhebung 2025: share of hires where a channel was decisive ÷ share where it was used: job boards 21/57 = 0.37, own homepage 20/70 = 0.29, referrals 27/48 = 0.56 (https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/); scaled so these three average 1 → job boards 0.90, homepage 0.71, referrals 1.37. Social media 7/40 = 0.18 vs job boards 16/51 = 0.31 in 2021 (https://iab-forum.de/iab-stellenerhebung-1-2022-174-millionen-offene-stellen-am-arbeitsmarkt/) → 0.57 × 0.90 = 0.50. Share qualified = role baseline Q (23%) × 0.90 = 20.7%. Volume cap: Indeed is used by 36% of skilled-worker job seekers ('Indeed mit einem Nutzungsgrad von 36 Prozent an der Spitze', Trendence 2023, n = 42,817, https://www.personalwirtschaft.de/?p=157882); the other programmatic boards overlap with it, so Indeed alone is used. Cap = reachable in-market qualified pool (Funnel pool check: 246) × 0.36 reach ÷ 20.7% qualified = 430 applications (channels overlap, so caps are not additive; the pool check shows the total against the pool). Downstream adjustment ×1.0 and fixed cost €0: no published evidence of a channel-specific effect once an applicant is qualified, and no set-up fee beyond the media price."/>
-    <hyperlink ref="L120" r:id="rId56" display="Price €1,449 per 30-day ad (official price list, https://www.stepstone.de/e-recruiting/stellenanzeige-aufgeben/). 12 applications per ad: StepStone Application Quality study 2025, 'durchschnittlich 12 Bewerbungen pro Stelle' (https://www.stepstone.de/e-recruiting/hr-wissen/recruiting/bewerberqualitaet-steigern/). Max ads = 30-day ads that fit the application window: 20 Oct–24 Nov = 36 days → 2 ads. Channel quality index from IAB-Stellenerhebung 2025: share of hires where a channel was decisive ÷ share where it was used: job boards 21/57 = 0.37, own homepage 20/70 = 0.29, referrals 27/48 = 0.56 (https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/); scaled so these three average 1 → job boards 0.90, homepage 0.71, referrals 1.37. Social media 7/40 = 0.18 vs job boards 16/51 = 0.31 in 2021 (https://iab-forum.de/iab-stellenerhebung-1-2022-174-millionen-offene-stellen-am-arbeitsmarkt/) → 0.57 × 0.90 = 0.50. Share qualified = role baseline Q (25%) × 0.90 = 22.5%.  Downstream adjustment ×1.0 and fixed cost €0: no published evidence of a channel-specific effect once an applicant is qualified, and no set-up fee beyond the media price."/>
-    <hyperlink ref="L121" r:id="rId57" display="Price €1,449 per 30-day ad (official price list, https://www.stepstone.de/e-recruiting/stellenanzeige-aufgeben/). 12 applications per ad: StepStone Application Quality study 2025, 'durchschnittlich 12 Bewerbungen pro Stelle' (https://www.stepstone.de/e-recruiting/hr-wissen/recruiting/bewerberqualitaet-steigern/). Max ads = 30-day ads that fit the application window: 20 Oct–24 Nov = 36 days → 2 ads. Channel quality index from IAB-Stellenerhebung 2025: share of hires where a channel was decisive ÷ share where it was used: job boards 21/57 = 0.37, own homepage 20/70 = 0.29, referrals 27/48 = 0.56 (https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/); scaled so these three average 1 → job boards 0.90, homepage 0.71, referrals 1.37. Social media 7/40 = 0.18 vs job boards 16/51 = 0.31 in 2021 (https://iab-forum.de/iab-stellenerhebung-1-2022-174-millionen-offene-stellen-am-arbeitsmarkt/) → 0.57 × 0.90 = 0.50. Share qualified = role baseline Q (25%) × 0.90 = 22.5%.  Downstream adjustment ×1.0 and fixed cost €0: no published evidence of a channel-specific effect once an applicant is qualified, and no set-up fee beyond the media price."/>
-    <hyperlink ref="L122" r:id="rId58" display="Price €1,449 per 30-day ad (official price list, https://www.stepstone.de/e-recruiting/stellenanzeige-aufgeben/). 12 applications per ad: StepStone Application Quality study 2025, 'durchschnittlich 12 Bewerbungen pro Stelle' (https://www.stepstone.de/e-recruiting/hr-wissen/recruiting/bewerberqualitaet-steigern/). Max ads = 30-day ads that fit the application window: 20 Oct–24 Nov = 36 days → 2 ads. Channel quality index from IAB-Stellenerhebung 2025: share of hires where a channel was decisive ÷ share where it was used: job boards 21/57 = 0.37, own homepage 20/70 = 0.29, referrals 27/48 = 0.56 (https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/); scaled so these three average 1 → job boards 0.90, homepage 0.71, referrals 1.37. Social media 7/40 = 0.18 vs job boards 16/51 = 0.31 in 2021 (https://iab-forum.de/iab-stellenerhebung-1-2022-174-millionen-offene-stellen-am-arbeitsmarkt/) → 0.57 × 0.90 = 0.50. Share qualified = role baseline Q (25%) × 0.90 = 22.5%.  Downstream adjustment ×1.0 and fixed cost €0: no published evidence of a channel-specific effect once an applicant is qualified, and no set-up fee beyond the media price."/>
-    <hyperlink ref="L123" r:id="rId59" display="Price €1,449 per 30-day ad (official price list, https://www.stepstone.de/e-recruiting/stellenanzeige-aufgeben/). 12 applications per ad: StepStone Application Quality study 2025, 'durchschnittlich 12 Bewerbungen pro Stelle' (https://www.stepstone.de/e-recruiting/hr-wissen/recruiting/bewerberqualitaet-steigern/). Max ads = 30-day ads that fit the application window: 20 Oct–17 Nov = 29 days → 1 ad. Channel quality index from IAB-Stellenerhebung 2025: share of hires where a channel was decisive ÷ share where it was used: job boards 21/57 = 0.37, own homepage 20/70 = 0.29, referrals 27/48 = 0.56 (https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/); scaled so these three average 1 → job boards 0.90, homepage 0.71, referrals 1.37. Social media 7/40 = 0.18 vs job boards 16/51 = 0.31 in 2021 (https://iab-forum.de/iab-stellenerhebung-1-2022-174-millionen-offene-stellen-am-arbeitsmarkt/) → 0.57 × 0.90 = 0.50. Share qualified = role baseline Q (23%) × 0.90 = 20.7%.  Downstream adjustment ×1.0 and fixed cost €0: no published evidence of a channel-specific effect once an applicant is qualified, and no set-up fee beyond the media price."/>
-    <hyperlink ref="L124" r:id="rId60" display="DACH median cost per application on LinkedIn: €96 (TalentBait 2024–26: https://www.talentbait.de/recruiting-kanaele-uebersicht/). LinkedIn job postings count as an online job board. Channel quality index from IAB-Stellenerhebung 2025: share of hires where a channel was decisive ÷ share where it was used: job boards 21/57 = 0.37, own homepage 20/70 = 0.29, referrals 27/48 = 0.56 (https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/); scaled so these three average 1 → job boards 0.90, homepage 0.71, referrals 1.37. Social media 7/40 = 0.18 vs job boards 16/51 = 0.31 in 2021 (https://iab-forum.de/iab-stellenerhebung-1-2022-174-millionen-offene-stellen-am-arbeitsmarkt/) → 0.57 × 0.90 = 0.50. Share qualified = role baseline Q (25%) × 0.90 = 22.5%. Volume cap: LinkedIn is used by 15% of skilled-worker job seekers ('Linkedin kommt mit 15 Prozent erst auf den siebten Rang', Trendence 2023, https://www.personalwirtschaft.de/?p=157882). Cap = reachable in-market qualified pool (Funnel pool check: 236) × 0.15 reach ÷ 22.5% qualified = 160 applications (channels overlap, so caps are not additive; the pool check shows the total against the pool). Downstream adjustment ×1.0 and fixed cost €0: no published evidence of a channel-specific effect once an applicant is qualified, and no set-up fee beyond the media price."/>
-    <hyperlink ref="L125" r:id="rId61" display="DACH median cost per application on LinkedIn: €96 (TalentBait 2024–26: https://www.talentbait.de/recruiting-kanaele-uebersicht/). LinkedIn job postings count as an online job board. Channel quality index from IAB-Stellenerhebung 2025: share of hires where a channel was decisive ÷ share where it was used: job boards 21/57 = 0.37, own homepage 20/70 = 0.29, referrals 27/48 = 0.56 (https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/); scaled so these three average 1 → job boards 0.90, homepage 0.71, referrals 1.37. Social media 7/40 = 0.18 vs job boards 16/51 = 0.31 in 2021 (https://iab-forum.de/iab-stellenerhebung-1-2022-174-millionen-offene-stellen-am-arbeitsmarkt/) → 0.57 × 0.90 = 0.50. Share qualified = role baseline Q (23%) × 0.90 = 20.7%. Volume cap: LinkedIn is used by 15% of skilled-worker job seekers ('Linkedin kommt mit 15 Prozent erst auf den siebten Rang', Trendence 2023, https://www.personalwirtschaft.de/?p=157882). Cap = reachable in-market qualified pool (Funnel pool check: 246) × 0.15 reach ÷ 20.7% qualified = 180 applications (channels overlap, so caps are not additive; the pool check shows the total against the pool). Downstream adjustment ×1.0 and fixed cost €0: no published evidence of a channel-specific effect once an applicant is qualified, and no set-up fee beyond the media price."/>
-    <hyperlink ref="L126" r:id="rId62" display="Social-recruiting cost per application for trades: €84 (TalentBait, 818 campaigns: https://www.talentbait.de/social-media-recruiting). Channel quality index from IAB-Stellenerhebung 2025: share of hires where a channel was decisive ÷ share where it was used: job boards 21/57 = 0.37, own homepage 20/70 = 0.29, referrals 27/48 = 0.56 (https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/); scaled so these three average 1 → job boards 0.90, homepage 0.71, referrals 1.37. Social media 7/40 = 0.18 vs job boards 16/51 = 0.31 in 2021 (https://iab-forum.de/iab-stellenerhebung-1-2022-174-millionen-offene-stellen-am-arbeitsmarkt/) → 0.57 × 0.90 = 0.50. Share qualified = role baseline Q (25%) × 0.50 = 12.5%. Volume: Redline (181 trade social campaigns, 2024–26) reports a median of 20 qualified applications per Elektroniker campaign (https://redline-grow.de/bewerbungen-pro-stelle); cap = 20 ÷ 12.5% = 160 applications. Downstream adjustment ×1.0 and fixed cost €0: no published evidence of a channel-specific effect once an applicant is qualified, and no set-up fee beyond the media price."/>
-    <hyperlink ref="L127" r:id="rId63" display="Social-recruiting cost per application for trades: €84 (TalentBait, 818 campaigns: https://www.talentbait.de/social-media-recruiting). Channel quality index from IAB-Stellenerhebung 2025: share of hires where a channel was decisive ÷ share where it was used: job boards 21/57 = 0.37, own homepage 20/70 = 0.29, referrals 27/48 = 0.56 (https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/); scaled so these three average 1 → job boards 0.90, homepage 0.71, referrals 1.37. Social media 7/40 = 0.18 vs job boards 16/51 = 0.31 in 2021 (https://iab-forum.de/iab-stellenerhebung-1-2022-174-millionen-offene-stellen-am-arbeitsmarkt/) → 0.57 × 0.90 = 0.50. Share qualified = role baseline Q (25%) × 0.50 = 12.5%. Volume: Redline (181 trade social campaigns, 2024–26) reports a median of 23 qualified applications per Kfz-Mechatroniker campaign (https://redline-grow.de/bewerbungen-pro-stelle); cap = 23 ÷ 12.5% = 180 applications. Downstream adjustment ×1.0 and fixed cost €0: no published evidence of a channel-specific effect once an applicant is qualified, and no set-up fee beyond the media price."/>
-    <hyperlink ref="L128" r:id="rId64" display="DACH median cost per application from Google Search: €179, 'little volume' (TalentBait 2024–26: https://www.talentbait.de/recruiting-kanaele-uebersicht/). Search ads land on the careers page, so the homepage index applies. Channel quality index from IAB-Stellenerhebung 2025: share of hires where a channel was decisive ÷ share where it was used: job boards 21/57 = 0.37, own homepage 20/70 = 0.29, referrals 27/48 = 0.56 (https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/); scaled so these three average 1 → job boards 0.90, homepage 0.71, referrals 1.37. Social media 7/40 = 0.18 vs job boards 16/51 = 0.31 in 2021 (https://iab-forum.de/iab-stellenerhebung-1-2022-174-millionen-offene-stellen-am-arbeitsmarkt/) → 0.57 × 0.90 = 0.50. Share qualified = role baseline Q (25%) × 0.71 = 17.8%. Volume cap: 10.5% of job seekers start their search on Google (softgarden 2020, n = 6,720, https://www.personalwirtschaft.de/news/recruiting/jeder-zehnte-nutzt-google-zur-jobsuche-97400/). Cap = reachable in-market qualified pool (Funnel pool check: 569) × 0.105 reach ÷ 17.8% qualified = 340 applications (channels overlap, so caps are not additive; the pool check shows the total against the pool). Downstream adjustment ×1.0 and fixed cost €0: no published evidence of a channel-specific effect once an applicant is qualified, and no set-up fee beyond the media price."/>
-    <hyperlink ref="L129" r:id="rId65" display="DACH median cost per application from Google Search: €179, 'little volume' (TalentBait 2024–26: https://www.talentbait.de/recruiting-kanaele-uebersicht/). Search ads land on the careers page, so the homepage index applies. Channel quality index from IAB-Stellenerhebung 2025: share of hires where a channel was decisive ÷ share where it was used: job boards 21/57 = 0.37, own homepage 20/70 = 0.29, referrals 27/48 = 0.56 (https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/); scaled so these three average 1 → job boards 0.90, homepage 0.71, referrals 1.37. Social media 7/40 = 0.18 vs job boards 16/51 = 0.31 in 2021 (https://iab-forum.de/iab-stellenerhebung-1-2022-174-millionen-offene-stellen-am-arbeitsmarkt/) → 0.57 × 0.90 = 0.50. Share qualified = role baseline Q (25%) × 0.71 = 17.8%. Volume cap: 10.5% of job seekers start their search on Google (softgarden 2020, n = 6,720, https://www.personalwirtschaft.de/news/recruiting/jeder-zehnte-nutzt-google-zur-jobsuche-97400/). Cap = reachable in-market qualified pool (Funnel pool check: 2,932) × 0.105 reach ÷ 17.8% qualified = 1,730 applications (channels overlap, so caps are not additive; the pool check shows the total against the pool). Downstream adjustment ×1.0 and fixed cost €0: no published evidence of a channel-specific effect once an applicant is qualified, and no set-up fee beyond the media price."/>
-    <hyperlink ref="L130" r:id="rId66" display="DACH median cost per application from Google Search: €179, 'little volume' (TalentBait 2024–26: https://www.talentbait.de/recruiting-kanaele-uebersicht/). Search ads land on the careers page, so the homepage index applies. Channel quality index from IAB-Stellenerhebung 2025: share of hires where a channel was decisive ÷ share where it was used: job boards 21/57 = 0.37, own homepage 20/70 = 0.29, referrals 27/48 = 0.56 (https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/); scaled so these three average 1 → job boards 0.90, homepage 0.71, referrals 1.37. Social media 7/40 = 0.18 vs job boards 16/51 = 0.31 in 2021 (https://iab-forum.de/iab-stellenerhebung-1-2022-174-millionen-offene-stellen-am-arbeitsmarkt/) → 0.57 × 0.90 = 0.50. Share qualified = role baseline Q (25%) × 0.71 = 17.8%. Volume cap: 10.5% of job seekers start their search on Google (softgarden 2020, n = 6,720, https://www.personalwirtschaft.de/news/recruiting/jeder-zehnte-nutzt-google-zur-jobsuche-97400/). Cap = reachable in-market qualified pool (Funnel pool check: 236) × 0.105 reach ÷ 17.8% qualified = 140 applications (channels overlap, so caps are not additive; the pool check shows the total against the pool). Downstream adjustment ×1.0 and fixed cost €0: no published evidence of a channel-specific effect once an applicant is qualified, and no set-up fee beyond the media price."/>
-    <hyperlink ref="L131" r:id="rId67" display="DACH median cost per application from Google Search: €179, 'little volume' (TalentBait 2024–26: https://www.talentbait.de/recruiting-kanaele-uebersicht/). Search ads land on the careers page, so the homepage index applies. Channel quality index from IAB-Stellenerhebung 2025: share of hires where a channel was decisive ÷ share where it was used: job boards 21/57 = 0.37, own homepage 20/70 = 0.29, referrals 27/48 = 0.56 (https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/); scaled so these three average 1 → job boards 0.90, homepage 0.71, referrals 1.37. Social media 7/40 = 0.18 vs job boards 16/51 = 0.31 in 2021 (https://iab-forum.de/iab-stellenerhebung-1-2022-174-millionen-offene-stellen-am-arbeitsmarkt/) → 0.57 × 0.90 = 0.50. Share qualified = role baseline Q (23%) × 0.71 = 16.3%. Volume cap: 10.5% of job seekers start their search on Google (softgarden 2020, n = 6,720, https://www.personalwirtschaft.de/news/recruiting/jeder-zehnte-nutzt-google-zur-jobsuche-97400/). Cap = reachable in-market qualified pool (Funnel pool check: 246) × 0.105 reach ÷ 16.3% qualified = 160 applications (channels overlap, so caps are not additive; the pool check shows the total against the pool). Downstream adjustment ×1.0 and fixed cost €0: no published evidence of a channel-specific effect once an applicant is qualified, and no set-up fee beyond the media price."/>
-    <hyperlink ref="G135" r:id="rId68" display="Derivation: German practice keeps rejected applicants' data 6 months, or up to 1 year with talent-pool consent (Haufe: https://www.haufe.de/compliance/management-praxis/aufbewahrung-wie-lange-duerfen-bewerberdaten-gespeichert-werden_230130_261218.html), so the usable pool is ~1 year of runners-up. Maintenance share: maintenance and the campaign's trades (KldB 2513 Wartung/Instandhaltung 240,934 + 2625 124,699 + 2611 84,727 + 2612 49,171 + supervisors 2519/2619/2629 36,989 = 536,520) are 7.8% of all production occupations (KldB 21–29: 6,850,263) in Germany (BA, 31.12.2025, https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-d-0-202512-xlsx.xlsx?__blob=publicationFile). Maintenance hires a year ≈ 10,703 staff (https://electrek.co/2026/03/04/tesla-giga-berlin-ig-metall-union-vote-collapse/) × 7.8% × 12% turnover (IAB-Betriebspanel Brandenburg 2024) = 100. Qualified runners-up per hire = 1 ÷ 0.32 qualified → signed − 1 = 2.1. Pool = 100 × 2.1 = 211, split by this campaign's openings (30/45/15/10%). The client's day-1 ATS export replaces it."/>
-    <hyperlink ref="G136" r:id="rId69" display="Derivation: German practice keeps rejected applicants' data 6 months, or up to 1 year with talent-pool consent (Haufe: https://www.haufe.de/compliance/management-praxis/aufbewahrung-wie-lange-duerfen-bewerberdaten-gespeichert-werden_230130_261218.html), so the usable pool is ~1 year of runners-up. Maintenance share: maintenance and the campaign's trades (KldB 2513 Wartung/Instandhaltung 240,934 + 2625 124,699 + 2611 84,727 + 2612 49,171 + supervisors 2519/2619/2629 36,989 = 536,520) are 7.8% of all production occupations (KldB 21–29: 6,850,263) in Germany (BA, 31.12.2025, https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-d-0-202512-xlsx.xlsx?__blob=publicationFile). Maintenance hires a year ≈ 10,703 staff (https://electrek.co/2026/03/04/tesla-giga-berlin-ig-metall-union-vote-collapse/) × 7.8% × 12% turnover (IAB-Betriebspanel Brandenburg 2024) = 100. Qualified runners-up per hire = 1 ÷ 0.32 qualified → signed − 1 = 2.1. Pool = 100 × 2.1 = 211, split by this campaign's openings (30/45/15/10%). The client's day-1 ATS export replaces it."/>
-    <hyperlink ref="G137" r:id="rId70" display="Derivation: German practice keeps rejected applicants' data 6 months, or up to 1 year with talent-pool consent (Haufe: https://www.haufe.de/compliance/management-praxis/aufbewahrung-wie-lange-duerfen-bewerberdaten-gespeichert-werden_230130_261218.html), so the usable pool is ~1 year of runners-up. Maintenance share: maintenance and the campaign's trades (KldB 2513 Wartung/Instandhaltung 240,934 + 2625 124,699 + 2611 84,727 + 2612 49,171 + supervisors 2519/2619/2629 36,989 = 536,520) are 7.8% of all production occupations (KldB 21–29: 6,850,263) in Germany (BA, 31.12.2025, https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-d-0-202512-xlsx.xlsx?__blob=publicationFile). Maintenance hires a year ≈ 10,703 staff (https://electrek.co/2026/03/04/tesla-giga-berlin-ig-metall-union-vote-collapse/) × 7.8% × 12% turnover (IAB-Betriebspanel Brandenburg 2024) = 100. Qualified runners-up per hire = 1 ÷ 0.32 qualified → signed − 1 = 2.1. Pool = 100 × 2.1 = 211, split by this campaign's openings (30/45/15/10%). The client's day-1 ATS export replaces it."/>
-    <hyperlink ref="G138" r:id="rId71" display="Derivation: German practice keeps rejected applicants' data 6 months, or up to 1 year with talent-pool consent (Haufe: https://www.haufe.de/compliance/management-praxis/aufbewahrung-wie-lange-duerfen-bewerberdaten-gespeichert-werden_230130_261218.html), so the usable pool is ~1 year of runners-up. Maintenance share: maintenance and the campaign's trades (KldB 2513 Wartung/Instandhaltung 240,934 + 2625 124,699 + 2611 84,727 + 2612 49,171 + supervisors 2519/2619/2629 36,989 = 536,520) are 7.8% of all production occupations (KldB 21–29: 6,850,263) in Germany (BA, 31.12.2025, https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-d-0-202512-xlsx.xlsx?__blob=publicationFile). Maintenance hires a year ≈ 10,703 staff (https://electrek.co/2026/03/04/tesla-giga-berlin-ig-metall-union-vote-collapse/) × 7.8% × 12% turnover (IAB-Betriebspanel Brandenburg 2024) = 100. Qualified runners-up per hire = 1 ÷ 0.32 qualified → signed − 1 = 2.1. Pool = 100 × 2.1 = 211, split by this campaign's openings (30/45/15/10%). The client's day-1 ATS export replaces it."/>
-    <hyperlink ref="G139" r:id="rId72" display="Derivation: geometric mean of the cold automated-email reply rate 4.96% (Pin 2026, https://www.pin.com/blog/recruiting-outreach-benchmark-report/) and the warm enterprise outreach reply rate 29% (Gem, https://www.gem.com/blog/2022-recruiting-benchmarks): √(4.96 × 29) = 12.0%. Past applicants are warm, but re-applying is a stricter step than replying."/>
-    <hyperlink ref="G140" r:id="rId73" display="These people met the hard requirements when they applied (that is how the export is filtered). Forrester: rediscovered candidates 'often remain a 70 percent or more match' (via SHRM, https://www.shrm.org/mena/topics-tools/news/technology/talent-rediscovery-tools-help-address-labor-shortages). 50% is set below that 70% because a match is not the same as meeting every requirement again (shifts, availability)."/>
-    <hyperlink ref="G141" r:id="rId74" display="Derivation: sized so referrals deliver 11% of hires, the CareerPlug 2025 benchmark (referrals 2% of applicants but 11% of hires, https://www.careerplug.com/wp-content/uploads/2025/04/Recruiting-Metrics-Report.pdf): 11 hires ÷ (45% qualified × 37% qualified → signed incl. ×1.15) = 66 applications, split by openings. Equals 0.6% of the plant's 10,703 staff referring someone in 6 weeks, far below the 20% quarterly participation that marks a healthy programme (https://www.pin.com/blog/employee-referral-program-guide)."/>
-    <hyperlink ref="G142" r:id="rId75" display="Derivation: sized so referrals deliver 11% of hires, the CareerPlug 2025 benchmark (referrals 2% of applicants but 11% of hires, https://www.careerplug.com/wp-content/uploads/2025/04/Recruiting-Metrics-Report.pdf): 11 hires ÷ (45% qualified × 37% qualified → signed incl. ×1.15) = 66 applications, split by openings. Equals 0.6% of the plant's 10,703 staff referring someone in 6 weeks, far below the 20% quarterly participation that marks a healthy programme (https://www.pin.com/blog/employee-referral-program-guide)."/>
-    <hyperlink ref="G143" r:id="rId76" display="Derivation: sized so referrals deliver 11% of hires, the CareerPlug 2025 benchmark (referrals 2% of applicants but 11% of hires, https://www.careerplug.com/wp-content/uploads/2025/04/Recruiting-Metrics-Report.pdf): 11 hires ÷ (45% qualified × 37% qualified → signed incl. ×1.15) = 66 applications, split by openings. Equals 0.6% of the plant's 10,703 staff referring someone in 6 weeks, far below the 20% quarterly participation that marks a healthy programme (https://www.pin.com/blog/employee-referral-program-guide)."/>
-    <hyperlink ref="G144" r:id="rId77" display="Derivation: sized so referrals deliver 11% of hires, the CareerPlug 2025 benchmark (referrals 2% of applicants but 11% of hires, https://www.careerplug.com/wp-content/uploads/2025/04/Recruiting-Metrics-Report.pdf): 11 hires ÷ (45% qualified × 37% qualified → signed incl. ×1.15) = 66 applications, split by openings. Equals 0.6% of the plant's 10,703 staff referring someone in 6 weeks, far below the 20% quarterly participation that marks a healthy programme (https://www.pin.com/blog/employee-referral-program-guide)."/>
-    <hyperlink ref="G145" r:id="rId78" display="Referred applicants convert to hires 4–11× better than average in US data (Breezy 2026: 'convert at 8%, which is 4x the rate of any major job board', https://breezy.hr/resources/hiring-reports/source-of-hire-report; Gem 2026: 11×) and 1.37× in German employer data (IAB 2025, decisive ÷ used, https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/). 45% = 1.6 × the IAB 28% baseline, inside that range and close to the German figure."/>
-    <hyperlink ref="G146" r:id="rId79" display="Three waves × 1 SMS at €0.075 net (seven.io price list, https://www.seven.io/en/prices/) to €0.112 (Twilio Germany, https://www.twilio.com/en-us/sms/pricing/de) = €0.23–0.34; e-mail is near zero → €0.30 per record."/>
-    <hyperlink ref="G147" r:id="rId80" display="German practice example: €1,000 per referral, €2,000 for hard-to-fill roles (IW Köln/KOFA, https://www.kofa.de/media/Publikationen/Handlungsempfehlungen/Mitarbeiter_werben_Mitarbeiter.pdf)."/>
-    <hyperlink ref="G148" r:id="rId81" display="Published uplift range: referred interviewees are ~40% more likely to get an offer (NY Fed Staff Report 568) and accept 2.7–7.3 points more often (Burks et al., QJE), summarised at https://www.metaview.ai/resources/blog/do-referred-candidates-interview-better. Acceptance alone gives ×1.07 (75.1 ÷ 70); ×1.15 adds a fraction of the offer uplift and stays at the low end of the range."/>
-    <hyperlink ref="G149" r:id="rId82" display="BA employment 31.12.2025, KldB 2621 Bauelektrik: Brandenburg 5,905, Berlin 6,204 (https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-12-0-202512-xlsx.xlsx?__blob=publicationFile (Brandenburg; -11- Berlin, -d- Germany)); ~75 km scaling ≈ 9,750. Bauelektrik is itself a shortage occupation (BA Engpassanalyse)."/>
-    <hyperlink ref="G150" r:id="rId83" display="Derivation: Redline (181 trade social campaigns) reports a mean of 29.5 qualified applications per Elektroniker campaign (https://redline-grow.de/fachkraeftemangel-handwerk) → 30 ÷ 25% qualified (I2Q) = 120 applications ÷ 10,000 construction electricians in reach = 1.2%."/>
-    <hyperlink ref="G151" r:id="rId84" display="Social-recruiting cost per application, trades (Handwerk) average €84 (TalentBait, 818 campaigns, vendor data, https://www.talentbait.de/social-media-recruiting)."/>
-    <hyperlink ref="G153" r:id="rId85" display="Derivation: construction electricians lack the PLC/automation part, so they face the automation pass rate instead of the electrician one: PA ÷ PE = 45% ÷ 50% = 0.9. Context: closing the PLC gap fully takes a 141-day course (WBS SPS-Techniker, https://www.wbstraining.de/potsdam-weiterbildung-sps-techniker-mit-hwk-abschluss), hence the in-house bridge."/>
-    <hyperlink ref="G154" r:id="rId86" display="Copywriting: €65/hour average freelance rate (freelancermap, https://www.freelancermap.de/freelancer/texterstellung) × ~11 h = €700. Quiz funnel: Perspective Grow €147–184/month (https://www.perspective.co/pricing) × 3 months ≈ €500. Total €1,200."/>
-    <hyperlink ref="G155" r:id="rId87" display="Pracuj.pl 30-day ad 1,499 PLN net ≈ €350 (official package page, https://dlafirm.pracuj.pl/cennik-uslug/pakiety-ogloszen) ÷ ~25 applications per ad (own estimate; no published figure) = €14."/>
-    <hyperlink ref="G156" r:id="rId88" display="Eurostat Adult Education Survey 2022, Poland, ages 25–64 with vocational upper-secondary education: 58.7% know a foreign language, of whom 23.6% at a good or proficient level → 58.7% × 23.6% = 13.9% ≈ 14% (https://ec.europa.eu/eurostat/api/dissemination/statistics/1.0/data/edat_aes_l23?geo=PL&amp;time=2022&amp;age=Y25-64). Language is the binding filter for this trade; the pre-screen call checks it."/>
-    <hyperlink ref="G157" r:id="rId89" display="Derivation: the applications needed to reach the 40% Polish cap (given): 18 hires ÷ (14% qualified × 37% qualified → signed) = 347 → 350. Reachable: about 2,000 Polish metal/machine-trade workers already commute into Brandenburg (IAB Regional 1/2020: 825 + 424 in 2019, https://doku.iab.de/regional/BB/2020/regional_bb_0120.pdf, × 1.59 growth of Polish commuters 2019–23, https://iab-forum.de/immer-mehr-menschen-pendeln-aus-osteuropa-nach-deutschland/); 350 is ~18% of that."/>
-    <hyperlink ref="G158" r:id="rId90" display="Derivation: ×1.0, i.e. no uplift, because no study quantifies one: Pin 2026 and Indeed describe pre-screening only qualitatively ('how selective your pre-interview screening is directly determines your interview-to-offer efficiency', https://www.pin.com/blog/recruitment-funnel-benchmarks; https://www.indeed.com/hire/c/info/what-is-a-phone-screen). The pre-screen's effect is already in I3Q."/>
-    <hyperlink ref="G159" r:id="rId91" display="'A phone screen normally lasts for 15 to 30 minutes' (Indeed, https://www.indeed.com/hire/c/info/what-is-a-phone-screen). 15 minutes = the bottom of the range, for a fixed checklist (certificate, language, shifts, commute)."/>
-    <hyperlink ref="G160" r:id="rId92" display="Freelance recruiter in Poland: 60–80 PLN net per hour, B2B (RocketJobs listing, https://rocketjobs.pl/oferta-pracy/intent-tech-recruiter-freelance--warszawa-hr-recruitment-9e0cdcee) → top of range 80 PLN ÷ 4.25 PLN/€ = €19 per hour."/>
-    <hyperlink ref="G161" r:id="rId93" display="German statutory translator fee: €1.95 per started 55 characters (§11 JVEG, https://www.buzer.de/11_JVEG.htm); ~6,000 characters × 2 languages ≈ €430."/>
+    <hyperlink ref="G86" r:id="rId37" display="Statistics: NIST's rule for reading a proportion is min{Np, N(1 − p)} ≥ 5 (https://www.itl.nist.gov/div898/handbook/prc/section2/prc24.htm). At the planned share qualified of ~25%, N × 0.25 ≥ 5 needs N ≥ 20; 30 applications gives N × p = 7.5 and a standard error of √(0.25 × 0.75 ÷ 30) = 7.9 points."/>
+    <hyperlink ref="G87" r:id="rId38" display="NIST/SEMATECH e-Handbook: 'in practice values of 0.1, 0.05, and 0.01 are common' for the significance level α (https://www.itl.nist.gov/div898/handbook/prc/section1/prc131.htm). One-sided test at α = 5% (z = 1.645). At the first judgement point (30 applications, R2) the plan-blended share qualified (R8, equal weights) has a relative standard error of 16% (raw √(0.25 × 0.75 ÷ 30) = 7.9 points ÷ 25% = 32%, halved by the blend). Better than plan with 95% confidence = 1 − 1.645 × 0.16 = 0.74 → 0.75."/>
+    <hyperlink ref="G88" r:id="rId39" display="Statistics: 1.5× plan is about three standard errors worse (see R3), so the cell is very likely worse than plan. Practice: 'turn off a Meta ad once it has spent 1.5x your target CPA without a single conversion' (https://sparkugc.com/resources/when-to-kill-a-meta-ad-cpa-rule); here the response is a 50% cut, the full stop comes at R5."/>
+    <hyperlink ref="G89" r:id="rId40" display="Practice: 'Pause if CPA over 2x target' (https://roaspig.com/blog/automated-rules-manage-meta-budgets/). At 2× plan the same money buys twice the qualified applicants in a cell running at plan."/>
+    <hyperlink ref="G90" r:id="rId41" display="Derivation: equal to the test tranche B2, so the decision falls when the test is spent. Combined with R11 = 3 expected qualified, this matches the practitioner rule 'Spent 3× your target CPA with zero purchases? Kill it' (https://coinis.com/blog/when-to-kill-meta-ads-decision-framework)."/>
+    <hyperlink ref="G91" r:id="rId42" display="Statistics: Poisson P(0 | mean 3) = e^−3 = 5%, so a cell that reaches its test spend with zero qualified is wrong at most 1 time in 20 (with mean 2 it would be 13.5%). Matches the '3× target CPA with zero conversions' practice (https://coinis.com/blog/when-to-kill-meta-ads-decision-framework). Cells expecting fewer than 3 are judged on applications (R12)."/>
+    <hyperlink ref="G93" r:id="rId43" display="NIST/SEMATECH e-Handbook: 'in practice values of 0.1, 0.05, and 0.01 are common' for the significance level α (https://www.itl.nist.gov/div898/handbook/prc/section1/prc131.htm). PASS uses α = 5%. Each bar is the Poisson quantile of the initiative's planned qualified in its 14-day window (Initiatives col G/I, CRITBINOM with n = 100,000). An initiative running at plan reaches the PASS bar with ≥95% probability."/>
+    <hyperlink ref="G95" r:id="rId44" display="NIST/SEMATECH e-Handbook: 'in practice values of 0.1, 0.05, and 0.01 are common' for the significance level α (https://www.itl.nist.gov/div898/handbook/prc/section1/prc131.htm). KILL uses α = 1%, the strictest common level, because killing is irreversible. Each bar is the Poisson quantile of the initiative's planned qualified in its 14-day window (Initiatives col G/I, CRITBINOM with n = 100,000). An initiative running at plan falls below the KILL bar with &lt;1% probability."/>
+    <hyperlink ref="G96" r:id="rId45" display="Derivation: the same multiple as the channel switch-off rule R5 (2×, 'Pause if CPA over 2x target', https://roaspig.com/blog/automated-rules-manage-meta-budgets/)."/>
+    <hyperlink ref="G97" r:id="rId46" display="Derivation from Pin 2026 reply timing (50% of replies within 4 h, 74.8% within 24 h, 93.9% within 7 days) and replies by message step (43.8% / 33.7% / 15.7%) (https://www.pin.com/blog/recruiting-outreach-benchmark-report/). Waves go out on day 2 (Wed 21 Oct), day 7 (Mon 26 Oct) and day 14 (Mon 2 Nov): week 1 = 0.47 × 0.90 + 0.36 × 0.50 = 60%; week 2 = 0.47 × 0.07 + 0.36 × 0.47 + 0.17 × 0.50 = 29%; week 3 = the rest, 11%."/>
+    <hyperlink ref="G98" r:id="rId47" display="Derivation from Pin 2026 reply timing (50% of replies within 4 h, 74.8% within 24 h, 93.9% within 7 days) and replies by message step (43.8% / 33.7% / 15.7%) (https://www.pin.com/blog/recruiting-outreach-benchmark-report/). Waves go out on day 2 (Wed 21 Oct), day 7 (Mon 26 Oct) and day 14 (Mon 2 Nov): week 1 = 0.47 × 0.90 + 0.36 × 0.50 = 60%; week 2 = 0.47 × 0.07 + 0.36 × 0.47 + 0.17 × 0.50 = 29%; week 3 = the rest, 11%."/>
+    <hyperlink ref="G99" r:id="rId48" display="Derivation from Pin 2026 reply timing (50% of replies within 4 h, 74.8% within 24 h, 93.9% within 7 days) and replies by message step (43.8% / 33.7% / 15.7%) (https://www.pin.com/blog/recruiting-outreach-benchmark-report/). Waves go out on day 2 (Wed 21 Oct), day 7 (Mon 26 Oct) and day 14 (Mon 2 Nov): week 1 = 0.47 × 0.90 + 0.36 × 0.50 = 60%; week 2 = 0.47 × 0.07 + 0.36 × 0.47 + 0.17 × 0.50 = 29%; week 3 = the rest, 11%."/>
+    <hyperlink ref="G100" r:id="rId49" display="Practice: budget rules use +20% ('safe') to +30% ('aggressive') per step (https://roaspig.com/blog/automated-rules-manage-meta-budgets/); Meta warns that large budget edits restart the learning phase (https://www.facebook.com/business/help/112167992830700). +25% once a week also gives Google bidding the 1–2 conversion cycles it needs between changes (https://support.google.com/google-ads/answer/6268637)."/>
+    <hyperlink ref="G101" r:id="rId50" display="Statistics: NIST's min{Np, N(1 − p)} ≥ 5 rule (https://www.itl.nist.gov/div898/handbook/prc/section2/prc24.htm) at the ~50% planned pass rate needs N ≥ 10 interviews."/>
+    <hyperlink ref="G102" r:id="rId51" display="Statistics: NIST's min{Np, N(1 − p)} ≥ 5 rule (https://www.itl.nist.gov/div898/handbook/prc/section2/prc24.htm) at the 70% planned acceptance: N × 0.70 ≥ 5 needs N ≥ 7.1 → 7 offers (N × 0.30 ≥ 5 would need 17, more offers than exist before the first check, so the Tracker blends with the plan until then)."/>
+    <hyperlink ref="G103" r:id="rId52" display="Display flag only (changes no number). No published standard for 'share of the reachable pool'. Above 1 in 4 of everyone reachable and open to a move, a 30% miss in response rates (the sensitivity test) cannot be absorbed from the same pool. Proxy: BA Engpassanalyse treats fewer than 2 job seekers per vacancy as the tightest band (https://statistik.arbeitsagentur.de/DE/Navigation/Statistiken/Interaktive-Statistiken/Fachkraeftebedarf/Engpassanalyse-Nav.html)."/>
+    <hyperlink ref="G105" r:id="rId53" display="Bagust, Place &amp; Posnett, BMJ 1999;319:155 (abstract, https://pubmed.ncbi.nlm.nih.gov/10406748/): 'Risks are discernible when average bed occupancy rates exceed about 85%'. Same shape as queueing theory, where waiting grows with ρ ÷ (1 − ρ)."/>
+    <hyperlink ref="G106" r:id="rId54" display="Bagust, Place &amp; Posnett, BMJ 1999 (https://pubmed.ncbi.nlm.nih.gov/10406748/): 'regular bed shortages and periodic bed crises if average bed occupancy rises to 90% or more'. A week above 90% of its slots is therefore treated as full."/>
+    <hyperlink ref="L112" r:id="rId55" display="Free: BA Jobbörse posting is free (https://www.arbeitsagentur.de/faktor-a/mitarbeiter-finden/so-funktioniert-deutschlands-groesste-jobboerse); Google for Jobs is free. Channel quality index from IAB-Stellenerhebung 2025: share of hires where a channel was decisive ÷ share where it was used: job boards 21/57 = 0.37, own homepage 20/70 = 0.29, referrals 27/48 = 0.56 (https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/); scaled so these three average 1 → job boards 0.90, homepage 0.71, referrals 1.37. Social media 7/40 = 0.18 vs job boards 16/51 = 0.31 in 2021 (https://iab-forum.de/iab-stellenerhebung-1-2022-174-millionen-offene-stellen-am-arbeitsmarkt/) → 0.57 × 0.90 = 0.50. Share qualified = role baseline Q (25%) × 0.71 = 17.8%. Volume: openings × 27 applications per vacancy at firms with 250+ staff (IAB, https://iab-forum.de/iab-stellenerhebung-2-2026-fast-drei-von-vier-bewerbungen-sind-aus-betrieblicher-sicht-ungeeignet/) × 13% of applications via the careers page (CareerPlug 2025, https://www.careerplug.com/wp-content/uploads/2025/04/Recruiting-Metrics-Report.pdf) = 30 × 27 × 0.13 = 105. Downstream adjustment ×1.0 and fixed cost €0: no published evidence of a channel-specific effect once an applicant is qualified, and no set-up fee beyond the media price."/>
+    <hyperlink ref="L113" r:id="rId56" display="Free: BA Jobbörse posting is free (https://www.arbeitsagentur.de/faktor-a/mitarbeiter-finden/so-funktioniert-deutschlands-groesste-jobboerse); Google for Jobs is free. Channel quality index from IAB-Stellenerhebung 2025: share of hires where a channel was decisive ÷ share where it was used: job boards 21/57 = 0.37, own homepage 20/70 = 0.29, referrals 27/48 = 0.56 (https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/); scaled so these three average 1 → job boards 0.90, homepage 0.71, referrals 1.37. Social media 7/40 = 0.18 vs job boards 16/51 = 0.31 in 2021 (https://iab-forum.de/iab-stellenerhebung-1-2022-174-millionen-offene-stellen-am-arbeitsmarkt/) → 0.57 × 0.90 = 0.50. Share qualified = role baseline Q (25%) × 0.71 = 17.8%. Volume: openings × 27 applications per vacancy at firms with 250+ staff (IAB, https://iab-forum.de/iab-stellenerhebung-2-2026-fast-drei-von-vier-bewerbungen-sind-aus-betrieblicher-sicht-ungeeignet/) × 13% of applications via the careers page (CareerPlug 2025, https://www.careerplug.com/wp-content/uploads/2025/04/Recruiting-Metrics-Report.pdf) = 45 × 27 × 0.13 = 158. Downstream adjustment ×1.0 and fixed cost €0: no published evidence of a channel-specific effect once an applicant is qualified, and no set-up fee beyond the media price."/>
+    <hyperlink ref="L114" r:id="rId57" display="Free: BA Jobbörse posting is free (https://www.arbeitsagentur.de/faktor-a/mitarbeiter-finden/so-funktioniert-deutschlands-groesste-jobboerse); Google for Jobs is free. Channel quality index from IAB-Stellenerhebung 2025: share of hires where a channel was decisive ÷ share where it was used: job boards 21/57 = 0.37, own homepage 20/70 = 0.29, referrals 27/48 = 0.56 (https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/); scaled so these three average 1 → job boards 0.90, homepage 0.71, referrals 1.37. Social media 7/40 = 0.18 vs job boards 16/51 = 0.31 in 2021 (https://iab-forum.de/iab-stellenerhebung-1-2022-174-millionen-offene-stellen-am-arbeitsmarkt/) → 0.57 × 0.90 = 0.50. Share qualified = role baseline Q (25%) × 0.71 = 17.8%. Volume: openings × 27 applications per vacancy at firms with 250+ staff (IAB, https://iab-forum.de/iab-stellenerhebung-2-2026-fast-drei-von-vier-bewerbungen-sind-aus-betrieblicher-sicht-ungeeignet/) × 13% of applications via the careers page (CareerPlug 2025, https://www.careerplug.com/wp-content/uploads/2025/04/Recruiting-Metrics-Report.pdf) = 15 × 27 × 0.13 = 53. Downstream adjustment ×1.0 and fixed cost €0: no published evidence of a channel-specific effect once an applicant is qualified, and no set-up fee beyond the media price."/>
+    <hyperlink ref="L115" r:id="rId58" display="Free: BA Jobbörse posting is free (https://www.arbeitsagentur.de/faktor-a/mitarbeiter-finden/so-funktioniert-deutschlands-groesste-jobboerse); Google for Jobs is free. Channel quality index from IAB-Stellenerhebung 2025: share of hires where a channel was decisive ÷ share where it was used: job boards 21/57 = 0.37, own homepage 20/70 = 0.29, referrals 27/48 = 0.56 (https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/); scaled so these three average 1 → job boards 0.90, homepage 0.71, referrals 1.37. Social media 7/40 = 0.18 vs job boards 16/51 = 0.31 in 2021 (https://iab-forum.de/iab-stellenerhebung-1-2022-174-millionen-offene-stellen-am-arbeitsmarkt/) → 0.57 × 0.90 = 0.50. Share qualified = role baseline Q (23%) × 0.71 = 16.3%. Volume: openings × 27 applications per vacancy at firms with 250+ staff (IAB, https://iab-forum.de/iab-stellenerhebung-2-2026-fast-drei-von-vier-bewerbungen-sind-aus-betrieblicher-sicht-ungeeignet/) × 13% of applications via the careers page (CareerPlug 2025, https://www.careerplug.com/wp-content/uploads/2025/04/Recruiting-Metrics-Report.pdf) = 10 × 27 × 0.13 = 35. Downstream adjustment ×1.0 and fixed cost €0: no published evidence of a channel-specific effect once an applicant is qualified, and no set-up fee beyond the media price."/>
+    <hyperlink ref="L116" r:id="rId59" display="Indeed Germany bills per started application since 1 Mar 2024 (https://www.personalwirtschaft.de/?p=162207). DACH median cost per application on Indeed: €161 (TalentBait, 2,549 campaigns, 2024–26: https://www.talentbait.de/recruiting-kanaele-uebersicht/). Channel quality index from IAB-Stellenerhebung 2025: share of hires where a channel was decisive ÷ share where it was used: job boards 21/57 = 0.37, own homepage 20/70 = 0.29, referrals 27/48 = 0.56 (https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/); scaled so these three average 1 → job boards 0.90, homepage 0.71, referrals 1.37. Social media 7/40 = 0.18 vs job boards 16/51 = 0.31 in 2021 (https://iab-forum.de/iab-stellenerhebung-1-2022-174-millionen-offene-stellen-am-arbeitsmarkt/) → 0.57 × 0.90 = 0.50. Share qualified = role baseline Q (25%) × 0.90 = 22.5%. Volume cap: Indeed is used by 36% of skilled-worker job seekers ('Indeed mit einem Nutzungsgrad von 36 Prozent an der Spitze', Trendence 2023, n = 42,817, https://www.personalwirtschaft.de/?p=157882); the other programmatic boards overlap with it, so Indeed alone is used. Cap = reachable in-market qualified pool (Funnel pool check: 569) × 0.36 reach ÷ 22.5% qualified = 910 applications (channels overlap, so caps are not additive; the pool check shows the total against the pool). Downstream adjustment ×1.0 and fixed cost €0: no published evidence of a channel-specific effect once an applicant is qualified, and no set-up fee beyond the media price."/>
+    <hyperlink ref="L117" r:id="rId60" display="Indeed Germany bills per started application since 1 Mar 2024 (https://www.personalwirtschaft.de/?p=162207). DACH median cost per application on Indeed: €161 (TalentBait, 2,549 campaigns, 2024–26: https://www.talentbait.de/recruiting-kanaele-uebersicht/). Channel quality index from IAB-Stellenerhebung 2025: share of hires where a channel was decisive ÷ share where it was used: job boards 21/57 = 0.37, own homepage 20/70 = 0.29, referrals 27/48 = 0.56 (https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/); scaled so these three average 1 → job boards 0.90, homepage 0.71, referrals 1.37. Social media 7/40 = 0.18 vs job boards 16/51 = 0.31 in 2021 (https://iab-forum.de/iab-stellenerhebung-1-2022-174-millionen-offene-stellen-am-arbeitsmarkt/) → 0.57 × 0.90 = 0.50. Share qualified = role baseline Q (25%) × 0.90 = 22.5%. Volume cap: Indeed is used by 36% of skilled-worker job seekers ('Indeed mit einem Nutzungsgrad von 36 Prozent an der Spitze', Trendence 2023, n = 42,817, https://www.personalwirtschaft.de/?p=157882); the other programmatic boards overlap with it, so Indeed alone is used. Cap = reachable in-market qualified pool (Funnel pool check: 2,932) × 0.36 reach ÷ 22.5% qualified = 4,690 applications (channels overlap, so caps are not additive; the pool check shows the total against the pool). Downstream adjustment ×1.0 and fixed cost €0: no published evidence of a channel-specific effect once an applicant is qualified, and no set-up fee beyond the media price."/>
+    <hyperlink ref="L118" r:id="rId61" display="Indeed Germany bills per started application since 1 Mar 2024 (https://www.personalwirtschaft.de/?p=162207). DACH median cost per application on Indeed: €161 (TalentBait, 2,549 campaigns, 2024–26: https://www.talentbait.de/recruiting-kanaele-uebersicht/). Channel quality index from IAB-Stellenerhebung 2025: share of hires where a channel was decisive ÷ share where it was used: job boards 21/57 = 0.37, own homepage 20/70 = 0.29, referrals 27/48 = 0.56 (https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/); scaled so these three average 1 → job boards 0.90, homepage 0.71, referrals 1.37. Social media 7/40 = 0.18 vs job boards 16/51 = 0.31 in 2021 (https://iab-forum.de/iab-stellenerhebung-1-2022-174-millionen-offene-stellen-am-arbeitsmarkt/) → 0.57 × 0.90 = 0.50. Share qualified = role baseline Q (25%) × 0.90 = 22.5%. Volume cap: Indeed is used by 36% of skilled-worker job seekers ('Indeed mit einem Nutzungsgrad von 36 Prozent an der Spitze', Trendence 2023, n = 42,817, https://www.personalwirtschaft.de/?p=157882); the other programmatic boards overlap with it, so Indeed alone is used. Cap = reachable in-market qualified pool (Funnel pool check: 236) × 0.36 reach ÷ 22.5% qualified = 380 applications (channels overlap, so caps are not additive; the pool check shows the total against the pool). Downstream adjustment ×1.0 and fixed cost €0: no published evidence of a channel-specific effect once an applicant is qualified, and no set-up fee beyond the media price."/>
+    <hyperlink ref="L119" r:id="rId62" display="Indeed Germany bills per started application since 1 Mar 2024 (https://www.personalwirtschaft.de/?p=162207). DACH median cost per application on Indeed: €161 (TalentBait, 2,549 campaigns, 2024–26: https://www.talentbait.de/recruiting-kanaele-uebersicht/). Channel quality index from IAB-Stellenerhebung 2025: share of hires where a channel was decisive ÷ share where it was used: job boards 21/57 = 0.37, own homepage 20/70 = 0.29, referrals 27/48 = 0.56 (https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/); scaled so these three average 1 → job boards 0.90, homepage 0.71, referrals 1.37. Social media 7/40 = 0.18 vs job boards 16/51 = 0.31 in 2021 (https://iab-forum.de/iab-stellenerhebung-1-2022-174-millionen-offene-stellen-am-arbeitsmarkt/) → 0.57 × 0.90 = 0.50. Share qualified = role baseline Q (23%) × 0.90 = 20.7%. Volume cap: Indeed is used by 36% of skilled-worker job seekers ('Indeed mit einem Nutzungsgrad von 36 Prozent an der Spitze', Trendence 2023, n = 42,817, https://www.personalwirtschaft.de/?p=157882); the other programmatic boards overlap with it, so Indeed alone is used. Cap = reachable in-market qualified pool (Funnel pool check: 246) × 0.36 reach ÷ 20.7% qualified = 430 applications (channels overlap, so caps are not additive; the pool check shows the total against the pool). Downstream adjustment ×1.0 and fixed cost €0: no published evidence of a channel-specific effect once an applicant is qualified, and no set-up fee beyond the media price."/>
+    <hyperlink ref="L120" r:id="rId63" display="Price €1,449 per 30-day ad (official price list, https://www.stepstone.de/e-recruiting/stellenanzeige-aufgeben/). 12 applications per ad: StepStone Application Quality study 2025, 'durchschnittlich 12 Bewerbungen pro Stelle' (https://www.stepstone.de/e-recruiting/hr-wissen/recruiting/bewerberqualitaet-steigern/). Max ads = 30-day ads that fit the application window: 20 Oct–24 Nov = 36 days → 2 ads. Channel quality index from IAB-Stellenerhebung 2025: share of hires where a channel was decisive ÷ share where it was used: job boards 21/57 = 0.37, own homepage 20/70 = 0.29, referrals 27/48 = 0.56 (https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/); scaled so these three average 1 → job boards 0.90, homepage 0.71, referrals 1.37. Social media 7/40 = 0.18 vs job boards 16/51 = 0.31 in 2021 (https://iab-forum.de/iab-stellenerhebung-1-2022-174-millionen-offene-stellen-am-arbeitsmarkt/) → 0.57 × 0.90 = 0.50. Share qualified = role baseline Q (25%) × 0.90 = 22.5%.  Downstream adjustment ×1.0 and fixed cost €0: no published evidence of a channel-specific effect once an applicant is qualified, and no set-up fee beyond the media price."/>
+    <hyperlink ref="L121" r:id="rId64" display="Price €1,449 per 30-day ad (official price list, https://www.stepstone.de/e-recruiting/stellenanzeige-aufgeben/). 12 applications per ad: StepStone Application Quality study 2025, 'durchschnittlich 12 Bewerbungen pro Stelle' (https://www.stepstone.de/e-recruiting/hr-wissen/recruiting/bewerberqualitaet-steigern/). Max ads = 30-day ads that fit the application window: 20 Oct–24 Nov = 36 days → 2 ads. Channel quality index from IAB-Stellenerhebung 2025: share of hires where a channel was decisive ÷ share where it was used: job boards 21/57 = 0.37, own homepage 20/70 = 0.29, referrals 27/48 = 0.56 (https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/); scaled so these three average 1 → job boards 0.90, homepage 0.71, referrals 1.37. Social media 7/40 = 0.18 vs job boards 16/51 = 0.31 in 2021 (https://iab-forum.de/iab-stellenerhebung-1-2022-174-millionen-offene-stellen-am-arbeitsmarkt/) → 0.57 × 0.90 = 0.50. Share qualified = role baseline Q (25%) × 0.90 = 22.5%.  Downstream adjustment ×1.0 and fixed cost €0: no published evidence of a channel-specific effect once an applicant is qualified, and no set-up fee beyond the media price."/>
+    <hyperlink ref="L122" r:id="rId65" display="Price €1,449 per 30-day ad (official price list, https://www.stepstone.de/e-recruiting/stellenanzeige-aufgeben/). 12 applications per ad: StepStone Application Quality study 2025, 'durchschnittlich 12 Bewerbungen pro Stelle' (https://www.stepstone.de/e-recruiting/hr-wissen/recruiting/bewerberqualitaet-steigern/). Max ads = 30-day ads that fit the application window: 20 Oct–24 Nov = 36 days → 2 ads. Channel quality index from IAB-Stellenerhebung 2025: share of hires where a channel was decisive ÷ share where it was used: job boards 21/57 = 0.37, own homepage 20/70 = 0.29, referrals 27/48 = 0.56 (https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/); scaled so these three average 1 → job boards 0.90, homepage 0.71, referrals 1.37. Social media 7/40 = 0.18 vs job boards 16/51 = 0.31 in 2021 (https://iab-forum.de/iab-stellenerhebung-1-2022-174-millionen-offene-stellen-am-arbeitsmarkt/) → 0.57 × 0.90 = 0.50. Share qualified = role baseline Q (25%) × 0.90 = 22.5%.  Downstream adjustment ×1.0 and fixed cost €0: no published evidence of a channel-specific effect once an applicant is qualified, and no set-up fee beyond the media price."/>
+    <hyperlink ref="L123" r:id="rId66" display="Price €1,449 per 30-day ad (official price list, https://www.stepstone.de/e-recruiting/stellenanzeige-aufgeben/). 12 applications per ad: StepStone Application Quality study 2025, 'durchschnittlich 12 Bewerbungen pro Stelle' (https://www.stepstone.de/e-recruiting/hr-wissen/recruiting/bewerberqualitaet-steigern/). Max ads = 30-day ads that fit the application window: 20 Oct–17 Nov = 29 days → 1 ad. Channel quality index from IAB-Stellenerhebung 2025: share of hires where a channel was decisive ÷ share where it was used: job boards 21/57 = 0.37, own homepage 20/70 = 0.29, referrals 27/48 = 0.56 (https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/); scaled so these three average 1 → job boards 0.90, homepage 0.71, referrals 1.37. Social media 7/40 = 0.18 vs job boards 16/51 = 0.31 in 2021 (https://iab-forum.de/iab-stellenerhebung-1-2022-174-millionen-offene-stellen-am-arbeitsmarkt/) → 0.57 × 0.90 = 0.50. Share qualified = role baseline Q (23%) × 0.90 = 20.7%.  Downstream adjustment ×1.0 and fixed cost €0: no published evidence of a channel-specific effect once an applicant is qualified, and no set-up fee beyond the media price."/>
+    <hyperlink ref="L124" r:id="rId67" display="DACH median cost per application on LinkedIn: €96 (TalentBait 2024–26: https://www.talentbait.de/recruiting-kanaele-uebersicht/). LinkedIn job postings count as an online job board. Channel quality index from IAB-Stellenerhebung 2025: share of hires where a channel was decisive ÷ share where it was used: job boards 21/57 = 0.37, own homepage 20/70 = 0.29, referrals 27/48 = 0.56 (https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/); scaled so these three average 1 → job boards 0.90, homepage 0.71, referrals 1.37. Social media 7/40 = 0.18 vs job boards 16/51 = 0.31 in 2021 (https://iab-forum.de/iab-stellenerhebung-1-2022-174-millionen-offene-stellen-am-arbeitsmarkt/) → 0.57 × 0.90 = 0.50. Share qualified = role baseline Q (25%) × 0.90 = 22.5%. Volume cap: LinkedIn is used by 15% of skilled-worker job seekers ('Linkedin kommt mit 15 Prozent erst auf den siebten Rang', Trendence 2023, https://www.personalwirtschaft.de/?p=157882). Cap = reachable in-market qualified pool (Funnel pool check: 236) × 0.15 reach ÷ 22.5% qualified = 160 applications (channels overlap, so caps are not additive; the pool check shows the total against the pool). Downstream adjustment ×1.0 and fixed cost €0: no published evidence of a channel-specific effect once an applicant is qualified, and no set-up fee beyond the media price."/>
+    <hyperlink ref="L125" r:id="rId68" display="DACH median cost per application on LinkedIn: €96 (TalentBait 2024–26: https://www.talentbait.de/recruiting-kanaele-uebersicht/). LinkedIn job postings count as an online job board. Channel quality index from IAB-Stellenerhebung 2025: share of hires where a channel was decisive ÷ share where it was used: job boards 21/57 = 0.37, own homepage 20/70 = 0.29, referrals 27/48 = 0.56 (https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/); scaled so these three average 1 → job boards 0.90, homepage 0.71, referrals 1.37. Social media 7/40 = 0.18 vs job boards 16/51 = 0.31 in 2021 (https://iab-forum.de/iab-stellenerhebung-1-2022-174-millionen-offene-stellen-am-arbeitsmarkt/) → 0.57 × 0.90 = 0.50. Share qualified = role baseline Q (23%) × 0.90 = 20.7%. Volume cap: LinkedIn is used by 15% of skilled-worker job seekers ('Linkedin kommt mit 15 Prozent erst auf den siebten Rang', Trendence 2023, https://www.personalwirtschaft.de/?p=157882). Cap = reachable in-market qualified pool (Funnel pool check: 246) × 0.15 reach ÷ 20.7% qualified = 180 applications (channels overlap, so caps are not additive; the pool check shows the total against the pool). Downstream adjustment ×1.0 and fixed cost €0: no published evidence of a channel-specific effect once an applicant is qualified, and no set-up fee beyond the media price."/>
+    <hyperlink ref="L126" r:id="rId69" display="Social-recruiting cost per application for trades: €84 (TalentBait, 818 campaigns: https://www.talentbait.de/social-media-recruiting). Channel quality index from IAB-Stellenerhebung 2025: share of hires where a channel was decisive ÷ share where it was used: job boards 21/57 = 0.37, own homepage 20/70 = 0.29, referrals 27/48 = 0.56 (https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/); scaled so these three average 1 → job boards 0.90, homepage 0.71, referrals 1.37. Social media 7/40 = 0.18 vs job boards 16/51 = 0.31 in 2021 (https://iab-forum.de/iab-stellenerhebung-1-2022-174-millionen-offene-stellen-am-arbeitsmarkt/) → 0.57 × 0.90 = 0.50. Share qualified = role baseline Q (25%) × 0.50 = 12.5%. Volume: Redline (181 trade social campaigns, 2024–26) reports a median of 20 qualified applications per Elektroniker campaign (https://redline-grow.de/bewerbungen-pro-stelle); cap = 20 ÷ 12.5% = 160 applications. Downstream adjustment ×1.0 and fixed cost €0: no published evidence of a channel-specific effect once an applicant is qualified, and no set-up fee beyond the media price."/>
+    <hyperlink ref="L127" r:id="rId70" display="Social-recruiting cost per application for trades: €84 (TalentBait, 818 campaigns: https://www.talentbait.de/social-media-recruiting). Channel quality index from IAB-Stellenerhebung 2025: share of hires where a channel was decisive ÷ share where it was used: job boards 21/57 = 0.37, own homepage 20/70 = 0.29, referrals 27/48 = 0.56 (https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/); scaled so these three average 1 → job boards 0.90, homepage 0.71, referrals 1.37. Social media 7/40 = 0.18 vs job boards 16/51 = 0.31 in 2021 (https://iab-forum.de/iab-stellenerhebung-1-2022-174-millionen-offene-stellen-am-arbeitsmarkt/) → 0.57 × 0.90 = 0.50. Share qualified = role baseline Q (25%) × 0.50 = 12.5%. Volume: Redline (181 trade social campaigns, 2024–26) reports a median of 23 qualified applications per Kfz-Mechatroniker campaign (https://redline-grow.de/bewerbungen-pro-stelle); cap = 23 ÷ 12.5% = 180 applications. Downstream adjustment ×1.0 and fixed cost €0: no published evidence of a channel-specific effect once an applicant is qualified, and no set-up fee beyond the media price."/>
+    <hyperlink ref="L128" r:id="rId71" display="DACH median cost per application from Google Search: €179, 'little volume' (TalentBait 2024–26: https://www.talentbait.de/recruiting-kanaele-uebersicht/). Search ads land on the careers page, so the homepage index applies. Channel quality index from IAB-Stellenerhebung 2025: share of hires where a channel was decisive ÷ share where it was used: job boards 21/57 = 0.37, own homepage 20/70 = 0.29, referrals 27/48 = 0.56 (https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/); scaled so these three average 1 → job boards 0.90, homepage 0.71, referrals 1.37. Social media 7/40 = 0.18 vs job boards 16/51 = 0.31 in 2021 (https://iab-forum.de/iab-stellenerhebung-1-2022-174-millionen-offene-stellen-am-arbeitsmarkt/) → 0.57 × 0.90 = 0.50. Share qualified = role baseline Q (25%) × 0.71 = 17.8%. Volume cap: 10.5% of job seekers start their search on Google (softgarden 2020, n = 6,720, https://www.personalwirtschaft.de/news/recruiting/jeder-zehnte-nutzt-google-zur-jobsuche-97400/). Cap = reachable in-market qualified pool (Funnel pool check: 569) × 0.105 reach ÷ 17.8% qualified = 340 applications (channels overlap, so caps are not additive; the pool check shows the total against the pool). Downstream adjustment ×1.0 and fixed cost €0: no published evidence of a channel-specific effect once an applicant is qualified, and no set-up fee beyond the media price."/>
+    <hyperlink ref="L129" r:id="rId72" display="DACH median cost per application from Google Search: €179, 'little volume' (TalentBait 2024–26: https://www.talentbait.de/recruiting-kanaele-uebersicht/). Search ads land on the careers page, so the homepage index applies. Channel quality index from IAB-Stellenerhebung 2025: share of hires where a channel was decisive ÷ share where it was used: job boards 21/57 = 0.37, own homepage 20/70 = 0.29, referrals 27/48 = 0.56 (https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/); scaled so these three average 1 → job boards 0.90, homepage 0.71, referrals 1.37. Social media 7/40 = 0.18 vs job boards 16/51 = 0.31 in 2021 (https://iab-forum.de/iab-stellenerhebung-1-2022-174-millionen-offene-stellen-am-arbeitsmarkt/) → 0.57 × 0.90 = 0.50. Share qualified = role baseline Q (25%) × 0.71 = 17.8%. Volume cap: 10.5% of job seekers start their search on Google (softgarden 2020, n = 6,720, https://www.personalwirtschaft.de/news/recruiting/jeder-zehnte-nutzt-google-zur-jobsuche-97400/). Cap = reachable in-market qualified pool (Funnel pool check: 2,932) × 0.105 reach ÷ 17.8% qualified = 1,730 applications (channels overlap, so caps are not additive; the pool check shows the total against the pool). Downstream adjustment ×1.0 and fixed cost €0: no published evidence of a channel-specific effect once an applicant is qualified, and no set-up fee beyond the media price."/>
+    <hyperlink ref="L130" r:id="rId73" display="DACH median cost per application from Google Search: €179, 'little volume' (TalentBait 2024–26: https://www.talentbait.de/recruiting-kanaele-uebersicht/). Search ads land on the careers page, so the homepage index applies. Channel quality index from IAB-Stellenerhebung 2025: share of hires where a channel was decisive ÷ share where it was used: job boards 21/57 = 0.37, own homepage 20/70 = 0.29, referrals 27/48 = 0.56 (https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/); scaled so these three average 1 → job boards 0.90, homepage 0.71, referrals 1.37. Social media 7/40 = 0.18 vs job boards 16/51 = 0.31 in 2021 (https://iab-forum.de/iab-stellenerhebung-1-2022-174-millionen-offene-stellen-am-arbeitsmarkt/) → 0.57 × 0.90 = 0.50. Share qualified = role baseline Q (25%) × 0.71 = 17.8%. Volume cap: 10.5% of job seekers start their search on Google (softgarden 2020, n = 6,720, https://www.personalwirtschaft.de/news/recruiting/jeder-zehnte-nutzt-google-zur-jobsuche-97400/). Cap = reachable in-market qualified pool (Funnel pool check: 236) × 0.105 reach ÷ 17.8% qualified = 140 applications (channels overlap, so caps are not additive; the pool check shows the total against the pool). Downstream adjustment ×1.0 and fixed cost €0: no published evidence of a channel-specific effect once an applicant is qualified, and no set-up fee beyond the media price."/>
+    <hyperlink ref="L131" r:id="rId74" display="DACH median cost per application from Google Search: €179, 'little volume' (TalentBait 2024–26: https://www.talentbait.de/recruiting-kanaele-uebersicht/). Search ads land on the careers page, so the homepage index applies. Channel quality index from IAB-Stellenerhebung 2025: share of hires where a channel was decisive ÷ share where it was used: job boards 21/57 = 0.37, own homepage 20/70 = 0.29, referrals 27/48 = 0.56 (https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/); scaled so these three average 1 → job boards 0.90, homepage 0.71, referrals 1.37. Social media 7/40 = 0.18 vs job boards 16/51 = 0.31 in 2021 (https://iab-forum.de/iab-stellenerhebung-1-2022-174-millionen-offene-stellen-am-arbeitsmarkt/) → 0.57 × 0.90 = 0.50. Share qualified = role baseline Q (23%) × 0.71 = 16.3%. Volume cap: 10.5% of job seekers start their search on Google (softgarden 2020, n = 6,720, https://www.personalwirtschaft.de/news/recruiting/jeder-zehnte-nutzt-google-zur-jobsuche-97400/). Cap = reachable in-market qualified pool (Funnel pool check: 246) × 0.105 reach ÷ 16.3% qualified = 160 applications (channels overlap, so caps are not additive; the pool check shows the total against the pool). Downstream adjustment ×1.0 and fixed cost €0: no published evidence of a channel-specific effect once an applicant is qualified, and no set-up fee beyond the media price."/>
+    <hyperlink ref="G135" r:id="rId75" display="Derivation: German practice keeps rejected applicants' data 6 months, or up to 1 year with talent-pool consent (Haufe: https://www.haufe.de/compliance/management-praxis/aufbewahrung-wie-lange-duerfen-bewerberdaten-gespeichert-werden_230130_261218.html), so the usable pool is ~1 year of runners-up. Maintenance share: the occupations this campaign hires from, KldB 2513 maintenance technicians (Wartung/Instandhaltung) 240,934 + 2625 industrial electricians 124,699 + 2611 mechatronics 84,727 + 2612 automation 49,171 + their supervisor codes 2519/2619/2629 36,989 = 536,520, are 7.8% of all production occupations (KldB 21–29: 6,850,263) in Germany (BA, 31.12.2025, https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-d-0-202512-xlsx.xlsx?__blob=publicationFile); 7.3% without the supervisor codes. Maintenance hires a year ≈ 10,703 staff (https://electrek.co/2026/03/04/tesla-giga-berlin-ig-metall-union-vote-collapse/) × 7.8% × 12% turnover (IAB-Betriebspanel Brandenburg 2024) = 100. Qualified runners-up per hire = 1 ÷ 0.32 qualified → signed − 1 = 2.1. Pool = 100 × 2.1 = 211, split by this campaign's openings (30/45/15/10%). The client's day-1 ATS export replaces it."/>
+    <hyperlink ref="G136" r:id="rId76" display="Derivation: German practice keeps rejected applicants' data 6 months, or up to 1 year with talent-pool consent (Haufe: https://www.haufe.de/compliance/management-praxis/aufbewahrung-wie-lange-duerfen-bewerberdaten-gespeichert-werden_230130_261218.html), so the usable pool is ~1 year of runners-up. Maintenance share: the occupations this campaign hires from, KldB 2513 maintenance technicians (Wartung/Instandhaltung) 240,934 + 2625 industrial electricians 124,699 + 2611 mechatronics 84,727 + 2612 automation 49,171 + their supervisor codes 2519/2619/2629 36,989 = 536,520, are 7.8% of all production occupations (KldB 21–29: 6,850,263) in Germany (BA, 31.12.2025, https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-d-0-202512-xlsx.xlsx?__blob=publicationFile); 7.3% without the supervisor codes. Maintenance hires a year ≈ 10,703 staff (https://electrek.co/2026/03/04/tesla-giga-berlin-ig-metall-union-vote-collapse/) × 7.8% × 12% turnover (IAB-Betriebspanel Brandenburg 2024) = 100. Qualified runners-up per hire = 1 ÷ 0.32 qualified → signed − 1 = 2.1. Pool = 100 × 2.1 = 211, split by this campaign's openings (30/45/15/10%). The client's day-1 ATS export replaces it."/>
+    <hyperlink ref="G137" r:id="rId77" display="Derivation: German practice keeps rejected applicants' data 6 months, or up to 1 year with talent-pool consent (Haufe: https://www.haufe.de/compliance/management-praxis/aufbewahrung-wie-lange-duerfen-bewerberdaten-gespeichert-werden_230130_261218.html), so the usable pool is ~1 year of runners-up. Maintenance share: the occupations this campaign hires from, KldB 2513 maintenance technicians (Wartung/Instandhaltung) 240,934 + 2625 industrial electricians 124,699 + 2611 mechatronics 84,727 + 2612 automation 49,171 + their supervisor codes 2519/2619/2629 36,989 = 536,520, are 7.8% of all production occupations (KldB 21–29: 6,850,263) in Germany (BA, 31.12.2025, https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-d-0-202512-xlsx.xlsx?__blob=publicationFile); 7.3% without the supervisor codes. Maintenance hires a year ≈ 10,703 staff (https://electrek.co/2026/03/04/tesla-giga-berlin-ig-metall-union-vote-collapse/) × 7.8% × 12% turnover (IAB-Betriebspanel Brandenburg 2024) = 100. Qualified runners-up per hire = 1 ÷ 0.32 qualified → signed − 1 = 2.1. Pool = 100 × 2.1 = 211, split by this campaign's openings (30/45/15/10%). The client's day-1 ATS export replaces it."/>
+    <hyperlink ref="G138" r:id="rId78" display="Derivation: German practice keeps rejected applicants' data 6 months, or up to 1 year with talent-pool consent (Haufe: https://www.haufe.de/compliance/management-praxis/aufbewahrung-wie-lange-duerfen-bewerberdaten-gespeichert-werden_230130_261218.html), so the usable pool is ~1 year of runners-up. Maintenance share: the occupations this campaign hires from, KldB 2513 maintenance technicians (Wartung/Instandhaltung) 240,934 + 2625 industrial electricians 124,699 + 2611 mechatronics 84,727 + 2612 automation 49,171 + their supervisor codes 2519/2619/2629 36,989 = 536,520, are 7.8% of all production occupations (KldB 21–29: 6,850,263) in Germany (BA, 31.12.2025, https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-d-0-202512-xlsx.xlsx?__blob=publicationFile); 7.3% without the supervisor codes. Maintenance hires a year ≈ 10,703 staff (https://electrek.co/2026/03/04/tesla-giga-berlin-ig-metall-union-vote-collapse/) × 7.8% × 12% turnover (IAB-Betriebspanel Brandenburg 2024) = 100. Qualified runners-up per hire = 1 ÷ 0.32 qualified → signed − 1 = 2.1. Pool = 100 × 2.1 = 211, split by this campaign's openings (30/45/15/10%). The client's day-1 ATS export replaces it."/>
+    <hyperlink ref="G139" r:id="rId79" display="Derivation: geometric mean of the cold automated-email reply rate 4.96% (Pin 2026, https://www.pin.com/blog/recruiting-outreach-benchmark-report/) and the warm enterprise outreach reply rate 29% (Gem, https://www.gem.com/blog/2022-recruiting-benchmarks): √(4.96 × 29) = 12.0%. Past applicants are warm, but re-applying is a stricter step than replying."/>
+    <hyperlink ref="G140" r:id="rId80" display="These people met the hard requirements when they applied (that is how the export is filtered). Forrester: rediscovered candidates 'often remain a 70 percent or more match' (via SHRM, https://www.shrm.org/mena/topics-tools/news/technology/talent-rediscovery-tools-help-address-labor-shortages). 50% is set below that 70% because a match is not the same as meeting every requirement again (shifts, availability)."/>
+    <hyperlink ref="G141" r:id="rId81" display="Derivation: sized so referrals deliver 11% of hires, the CareerPlug 2025 benchmark (referrals 2% of applicants but 11% of hires, https://www.careerplug.com/wp-content/uploads/2025/04/Recruiting-Metrics-Report.pdf): 11 hires ÷ (45% qualified × 37% qualified → signed incl. ×1.15) = 66 applications, split by openings. Equals 0.6% of the plant's 10,703 staff referring someone in 6 weeks, far below the 20% quarterly participation that marks a healthy programme (https://www.pin.com/blog/employee-referral-program-guide)."/>
+    <hyperlink ref="G142" r:id="rId82" display="Derivation: sized so referrals deliver 11% of hires, the CareerPlug 2025 benchmark (referrals 2% of applicants but 11% of hires, https://www.careerplug.com/wp-content/uploads/2025/04/Recruiting-Metrics-Report.pdf): 11 hires ÷ (45% qualified × 37% qualified → signed incl. ×1.15) = 66 applications, split by openings. Equals 0.6% of the plant's 10,703 staff referring someone in 6 weeks, far below the 20% quarterly participation that marks a healthy programme (https://www.pin.com/blog/employee-referral-program-guide)."/>
+    <hyperlink ref="G143" r:id="rId83" display="Derivation: sized so referrals deliver 11% of hires, the CareerPlug 2025 benchmark (referrals 2% of applicants but 11% of hires, https://www.careerplug.com/wp-content/uploads/2025/04/Recruiting-Metrics-Report.pdf): 11 hires ÷ (45% qualified × 37% qualified → signed incl. ×1.15) = 66 applications, split by openings. Equals 0.6% of the plant's 10,703 staff referring someone in 6 weeks, far below the 20% quarterly participation that marks a healthy programme (https://www.pin.com/blog/employee-referral-program-guide)."/>
+    <hyperlink ref="G144" r:id="rId84" display="Derivation: sized so referrals deliver 11% of hires, the CareerPlug 2025 benchmark (referrals 2% of applicants but 11% of hires, https://www.careerplug.com/wp-content/uploads/2025/04/Recruiting-Metrics-Report.pdf): 11 hires ÷ (45% qualified × 37% qualified → signed incl. ×1.15) = 66 applications, split by openings. Equals 0.6% of the plant's 10,703 staff referring someone in 6 weeks, far below the 20% quarterly participation that marks a healthy programme (https://www.pin.com/blog/employee-referral-program-guide)."/>
+    <hyperlink ref="G145" r:id="rId85" display="Referred applicants convert to hires 4–11× better than average in US data (Breezy 2026: 'convert at 8%, which is 4x the rate of any major job board', https://breezy.hr/resources/hiring-reports/source-of-hire-report; Gem 2026: 11×) and 1.37× in German employer data (IAB 2025, decisive ÷ used, https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/). 45% = 1.6 × the IAB 28% baseline, inside that range and close to the German figure."/>
+    <hyperlink ref="G146" r:id="rId86" display="Three waves × 1 SMS at €0.075 net (seven.io price list, https://www.seven.io/en/prices/) to €0.112 (Twilio Germany, https://www.twilio.com/en-us/sms/pricing/de) = €0.23–0.34; e-mail is near zero → €0.30 per record."/>
+    <hyperlink ref="G147" r:id="rId87" display="German practice example: €1,000 per referral, €2,000 for hard-to-fill roles (IW Köln/KOFA, https://www.kofa.de/media/Publikationen/Handlungsempfehlungen/Mitarbeiter_werben_Mitarbeiter.pdf)."/>
+    <hyperlink ref="G148" r:id="rId88" display="Published uplift range: referred interviewees are ~40% more likely to get an offer (NY Fed Staff Report 568) and accept 2.7–7.3 points more often (Burks et al., QJE), summarised at https://www.metaview.ai/resources/blog/do-referred-candidates-interview-better. Acceptance alone gives ×1.07 (75.1 ÷ 70); ×1.15 adds a fraction of the offer uplift and stays at the low end of the range."/>
+    <hyperlink ref="G149" r:id="rId89" display="BA employment 31.12.2025, KldB 2621 Bauelektrik: Brandenburg 5,905, Berlin 6,204 (https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-12-0-202512-xlsx.xlsx?__blob=publicationFile (Brandenburg; -11- Berlin, -d- Germany)); ~75 km scaling ≈ 9,750. Bauelektrik is itself a shortage occupation (BA Engpassanalyse)."/>
+    <hyperlink ref="G150" r:id="rId90" display="Derivation: Redline (181 trade social campaigns) reports a mean of 29.5 qualified applications per Elektroniker campaign (https://redline-grow.de/fachkraeftemangel-handwerk) → 30 ÷ 25% qualified (I2Q) = 120 applications ÷ 10,000 construction electricians in reach = 1.2%."/>
+    <hyperlink ref="G151" r:id="rId91" display="Social-recruiting cost per application, trades (Handwerk) average €84 (TalentBait, 818 campaigns, vendor data, https://www.talentbait.de/social-media-recruiting)."/>
+    <hyperlink ref="G153" r:id="rId92" display="Derivation: construction electricians lack the PLC/automation part, so they face the automation pass rate instead of the electrician one: PA ÷ PE = 45% ÷ 50% = 0.9. Context: closing the PLC gap fully takes a 141-day course (WBS SPS-Techniker, https://www.wbstraining.de/potsdam-weiterbildung-sps-techniker-mit-hwk-abschluss), hence the in-house bridge."/>
+    <hyperlink ref="G154" r:id="rId93" display="Copywriting: €65/hour average freelance rate (freelancermap, https://www.freelancermap.de/freelancer/texterstellung) × ~11 h = €700. Quiz funnel: Perspective Grow €147–184/month (https://www.perspective.co/pricing) × 3 months ≈ €500. Total €1,200."/>
+    <hyperlink ref="G155" r:id="rId94" display="Pracuj.pl 30-day ad 1,499 PLN net ≈ €350 (official package page, https://dlafirm.pracuj.pl/cennik-uslug/pakiety-ogloszen) ÷ ~25 applications per ad (own estimate; no published figure) = €14."/>
+    <hyperlink ref="G156" r:id="rId95" display="Eurostat Adult Education Survey 2022, Poland, ages 25–64 with vocational upper-secondary education: 58.7% know a foreign language, of whom 23.6% at a good or proficient level → 58.7% × 23.6% = 13.9% ≈ 14% (https://ec.europa.eu/eurostat/api/dissemination/statistics/1.0/data/edat_aes_l23?geo=PL&amp;time=2022&amp;age=Y25-64). Language is the binding filter for this trade; the pre-screen call checks it."/>
+    <hyperlink ref="G157" r:id="rId96" display="Derivation: the applications needed to reach the 40% Polish cap (given): 18 hires ÷ (14% qualified × 37% qualified → signed) = 347 → 350. Reachable: about 2,000 Polish metal/machine-trade workers already commute into Brandenburg (IAB Regional 1/2020: 825 + 424 in 2019, https://doku.iab.de/regional/BB/2020/regional_bb_0120.pdf, × 1.59 growth of Polish commuters 2019–23, https://iab-forum.de/immer-mehr-menschen-pendeln-aus-osteuropa-nach-deutschland/); 350 is ~18% of that."/>
+    <hyperlink ref="G158" r:id="rId97" display="Derivation: ×1.0, i.e. no uplift, because no study quantifies one: Pin 2026 and Indeed describe pre-screening only qualitatively ('how selective your pre-interview screening is directly determines your interview-to-offer efficiency', https://www.pin.com/blog/recruitment-funnel-benchmarks; https://www.indeed.com/hire/c/info/what-is-a-phone-screen). The pre-screen's effect is already in I3Q."/>
+    <hyperlink ref="G159" r:id="rId98" display="'A phone screen normally lasts for 15 to 30 minutes' (Indeed, https://www.indeed.com/hire/c/info/what-is-a-phone-screen). 15 minutes = the bottom of the range, for a fixed checklist (certificate, language, shifts, commute)."/>
+    <hyperlink ref="G160" r:id="rId99" display="Freelance recruiter in Poland: 60–80 PLN net per hour, B2B (RocketJobs listing, https://rocketjobs.pl/oferta-pracy/intent-tech-recruiter-freelance--warszawa-hr-recruitment-9e0cdcee) → top of range 80 PLN ÷ 4.25 PLN/€ = €19 per hour."/>
+    <hyperlink ref="G161" r:id="rId100" display="German statutory translator fee: €1.95 per started 55 characters (§11 JVEG, https://www.buzer.de/11_JVEG.htm); ~6,000 characters × 2 languages ≈ €430."/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Ready-to-share pass: explicit sensitivity tie-break, derived-input notes name their inputs, clean file metadata
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V2NJtrYy3bzNxqKeiRXJfY
</commit_message>
<xml_diff>
--- a/operation_uptime/Operation_Uptime_Model.xlsx
+++ b/operation_uptime/Operation_Uptime_Model.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1464" uniqueCount="759">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1463" uniqueCount="758">
   <si>
     <t xml:space="preserve">Operation Uptime — model summary (hypothetical Tesla Giga Berlin maintenance hiring)</t>
   </si>
@@ -1085,7 +1085,7 @@
     <t xml:space="preserve">records</t>
   </si>
   <si>
-    <t xml:space="preserve">Calculated: about one year of runners-up in the client's applicant system (data is kept up to a year with consent). Replaced by the real export on day 1.</t>
+    <t xml:space="preserve">Calculated: last year's maintenance hires (STAFF × MSH × TURN × this role's share) × qualified runners-up per hire (1 ÷ qualified→signed − 1). Replaced by the real export on day 1.</t>
   </si>
   <si>
     <t xml:space="preserve">I1RM</t>
@@ -1121,7 +1121,7 @@
     <t xml:space="preserve">I1: employee-referred applications over campaign</t>
   </si>
   <si>
-    <t xml:space="preserve">Calculated: sized so referrals give ~11% of this role's hires.</t>
+    <t xml:space="preserve">Calculated: referrals give REFSH (11%) of this role's hires: REFSH × openings ÷ (I1FQ × qualified→signed × I1A).</t>
   </si>
   <si>
     <t xml:space="preserve">I1FM</t>
@@ -1184,7 +1184,7 @@
     <t xml:space="preserve">I2: share who apply over the campaign (reachable × persuaded)</t>
   </si>
   <si>
-    <t xml:space="preserve">Calculated from Redline's average electrician campaign (~30 qualified).</t>
+    <t xml:space="preserve">Calculated: RD2 (Redline, ~30 qualified per electrician campaign) ÷ I2Q ÷ I2P.</t>
   </si>
   <si>
     <t xml:space="preserve">I2C</t>
@@ -1481,16 +1481,13 @@
     <t xml:space="preserve">Pure money: +30% media, no effect on hires if the money is there.</t>
   </si>
   <si>
-    <t xml:space="preserve">Recruiter capacity ×0.7 (≈38/week)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fewer slots: hires capped by capacity.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Most sensitive assumption (largest hire loss):</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Why it matters most: recruiter capacity, not money, is the binding limit. Anything that lowers hires per qualified applicant (pass or acceptance) can't be fixed by spending more; anything upstream (share qualified, CPA) can.</t>
+    <t xml:space="preserve">Recruiter capacity ×0.7 (≈38/week), given in the brief, shown for context</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fewer slots: hires capped by capacity. Not ranked: 55/week is given, not assumed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Most sensitive assumption (largest hire loss; capacity excluded as it is given):</t>
   </si>
   <si>
     <t xml:space="preserve">Talent-pool sanity check (Part 2.2): can the channels plausibly deliver the qualified applicants we plan?</t>
@@ -3566,7 +3563,7 @@
         <v>62</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>78</v>
@@ -8317,13 +8314,14 @@
         <v>486</v>
       </c>
       <c r="D49" s="8" t="str">
-        <f aca="false">INDEX(A43:A47,MATCH(MAX(E43:E47),E43:E47,0))</f>
+        <f aca="false">INDEX(A43:A46,MATCH(MAX(E43:E46),E43:E46,0))</f>
         <v>Qualified → signed (assessment pass rate) ×0.7</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="9" t="s">
-        <v>487</v>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="9" t="str">
+        <f aca="false">IF(AND(E43&gt;0,ROUND(E43,6)=ROUND(E44,6)),"Pass rate and acceptance tie ("&amp;TEXT(E43,"0")&amp;" hires lost each). I name the pass rate: it depends on this plant’s own test, so it is the least known, and it can only be read after interviews (week-2 check). Acceptance can be protected with fast offers. ","")&amp;"Why it matters: assessment capacity, not money, is the limit, so a lower pass rate or acceptance can’t be fixed by spending more; a lower share qualified or dearer clicks only cost money."</f>
+        <v>Pass rate and acceptance tie (29 hires lost each). I name the pass rate: it depends on this plant’s own test, so it is the least known, and it can only be read after interviews (week-2 check). Acceptance can be protected with fast offers. Why it matters: assessment capacity, not money, is the limit, so a lower pass rate or acceptance can’t be fixed by spending more; a lower share qualified or dearer clicks only cost money.</v>
       </c>
       <c r="B50" s="9"/>
       <c r="C50" s="9"/>
@@ -8345,7 +8343,7 @@
     </row>
     <row r="54" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="1" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8353,34 +8351,34 @@
         <v>305</v>
       </c>
       <c r="B57" s="12" t="s">
+        <v>488</v>
+      </c>
+      <c r="C57" s="12" t="s">
         <v>489</v>
       </c>
-      <c r="C57" s="12" t="s">
+      <c r="D57" s="12" t="s">
         <v>490</v>
       </c>
-      <c r="D57" s="12" t="s">
+      <c r="E57" s="12" t="s">
         <v>491</v>
       </c>
-      <c r="E57" s="12" t="s">
+      <c r="F57" s="12" t="s">
         <v>492</v>
       </c>
-      <c r="F57" s="12" t="s">
+      <c r="G57" s="12" t="s">
         <v>493</v>
       </c>
-      <c r="G57" s="12" t="s">
+      <c r="H57" s="12" t="s">
         <v>494</v>
       </c>
-      <c r="H57" s="12" t="s">
+      <c r="I57" s="12" t="s">
         <v>495</v>
       </c>
-      <c r="I57" s="12" t="s">
+      <c r="J57" s="12" t="s">
         <v>496</v>
       </c>
-      <c r="J57" s="12" t="s">
+      <c r="K57" s="12" t="s">
         <v>497</v>
-      </c>
-      <c r="K57" s="12" t="s">
-        <v>498</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8565,7 +8563,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="9" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="B63" s="9"/>
       <c r="C63" s="9"/>
@@ -8625,22 +8623,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="28" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="B4" s="12" t="s">
         <v>48</v>
@@ -8660,7 +8658,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="B5" s="29" t="n">
         <f aca="false">Assumptions!$D$150</f>
@@ -8685,7 +8683,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="B6" s="30" t="n">
         <f aca="false">Assumptions!$D$154</f>
@@ -8706,7 +8704,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="B7" s="32" t="n">
         <f aca="false">B5*B6</f>
@@ -8731,7 +8729,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="B8" s="30" t="n">
         <f aca="false">Assumptions!$D$155</f>
@@ -8752,7 +8750,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="B9" s="31" t="n">
         <f aca="false">Funnel!$G$5*Assumptions!$D$163</f>
@@ -8773,7 +8771,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="B10" s="41" t="n">
         <f aca="false">B5*Assumptions!$D$161</f>
@@ -8798,7 +8796,7 @@
     </row>
     <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="B11" s="43" t="n">
         <f aca="false">IF(B7&gt;0,B10/B7,0)</f>
@@ -8823,7 +8821,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="B12" s="32" t="n">
         <f aca="false">B7*B8*B9</f>
@@ -8848,7 +8846,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="B13" s="32" t="n">
         <f aca="false">Assumptions!$D$156</f>
@@ -8873,7 +8871,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="B14" s="30" t="n">
         <f aca="false">Assumptions!$D$160</f>
@@ -8894,7 +8892,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="B15" s="32" t="n">
         <f aca="false">B13*B14*B9</f>
@@ -8919,7 +8917,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="B16" s="41" t="n">
         <f aca="false">B15*Assumptions!$D$162</f>
@@ -8944,7 +8942,7 @@
     </row>
     <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="B17" s="43" t="n">
         <f aca="false">IF(B13&gt;0,B16/B13,0)</f>
@@ -8963,12 +8961,12 @@
         <v>123.165</v>
       </c>
       <c r="G17" s="13" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="B18" s="32" t="n">
         <f aca="false">B12+B15</f>
@@ -8993,7 +8991,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B19" s="41" t="n">
         <f aca="false">B10+B16</f>
@@ -9018,7 +9016,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="B20" s="41" t="n">
         <f aca="false">IF(B18&gt;0,B19/B18,0)</f>
@@ -9043,12 +9041,12 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="28" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="B24" s="29" t="n">
         <f aca="false">Assumptions!$D$164</f>
@@ -9057,7 +9055,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="B25" s="31" t="n">
         <f aca="false">Assumptions!$D$165</f>
@@ -9066,7 +9064,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="B26" s="29" t="n">
         <f aca="false">B24*B25</f>
@@ -9075,7 +9073,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="B27" s="41" t="n">
         <f aca="false">Assumptions!$D$166</f>
@@ -9084,7 +9082,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="B28" s="30" t="n">
         <f aca="false">Assumptions!$D$167</f>
@@ -9093,7 +9091,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="B29" s="32" t="n">
         <f aca="false">B26*B28</f>
@@ -9102,7 +9100,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="B30" s="31" t="n">
         <f aca="false">Funnel!$G$5*Assumptions!$D$168</f>
@@ -9111,7 +9109,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="B31" s="32" t="n">
         <f aca="false">B29*B30</f>
@@ -9120,7 +9118,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="B32" s="41" t="n">
         <f aca="false">B26*B27</f>
@@ -9129,7 +9127,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="B33" s="41" t="n">
         <f aca="false">Assumptions!$D$169</f>
@@ -9138,7 +9136,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="B34" s="41" t="n">
         <f aca="false">IF(B31&gt;0,(B32+B33)/B31,0)</f>
@@ -9147,12 +9145,12 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="28" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="B38" s="43" t="n">
         <f aca="false">B44+B45</f>
@@ -9161,7 +9159,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B39" s="30" t="n">
         <f aca="false">Assumptions!$D$171</f>
@@ -9170,7 +9168,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="B40" s="29" t="n">
         <f aca="false">Assumptions!$D$172</f>
@@ -9179,7 +9177,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="B41" s="31" t="n">
         <f aca="false">Funnel!$G$6*Assumptions!$D$173</f>
@@ -9188,7 +9186,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="2" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="B42" s="32" t="n">
         <f aca="false">Assumptions!$D$10*Assumptions!$D$12</f>
@@ -9197,7 +9195,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="B43" s="32" t="n">
         <f aca="false">MIN(B40*B39*B41,B42)</f>
@@ -9206,7 +9204,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="2" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="B44" s="43" t="n">
         <f aca="false">Assumptions!$D$170</f>
@@ -9215,7 +9213,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="2" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="B45" s="43" t="n">
         <f aca="false">Assumptions!$D$174/60*Assumptions!$D$175</f>
@@ -9224,7 +9222,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="2" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="B46" s="41" t="n">
         <f aca="false">Assumptions!$D$176</f>
@@ -9233,7 +9231,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="2" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="B47" s="29" t="n">
         <f aca="false">IF(B41*B39&gt;0,B43/B41/B39,0)</f>
@@ -9242,7 +9240,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="2" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="B48" s="41" t="n">
         <f aca="false">IF(B43&gt;0,(B47*B38+B46)/B43,0)</f>
@@ -9251,50 +9249,50 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="28" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="12" t="s">
+        <v>544</v>
+      </c>
+      <c r="B52" s="12" t="s">
         <v>545</v>
       </c>
-      <c r="B52" s="12" t="s">
+      <c r="C52" s="12" t="s">
         <v>546</v>
       </c>
-      <c r="C52" s="12" t="s">
+      <c r="D52" s="12" t="s">
         <v>547</v>
       </c>
-      <c r="D52" s="12" t="s">
+      <c r="E52" s="12" t="s">
         <v>548</v>
       </c>
-      <c r="E52" s="12" t="s">
+      <c r="F52" s="12" t="s">
         <v>549</v>
       </c>
-      <c r="F52" s="12" t="s">
+      <c r="G52" s="12" t="s">
         <v>550</v>
       </c>
-      <c r="G52" s="12" t="s">
+      <c r="H52" s="12" t="s">
         <v>551</v>
       </c>
-      <c r="H52" s="12" t="s">
+      <c r="I52" s="12" t="s">
         <v>552</v>
       </c>
-      <c r="I52" s="12" t="s">
+      <c r="J52" s="12" t="s">
         <v>553</v>
       </c>
-      <c r="J52" s="12" t="s">
+      <c r="K52" s="12" t="s">
         <v>554</v>
-      </c>
-      <c r="K52" s="12" t="s">
-        <v>555</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="28" t="s">
+        <v>555</v>
+      </c>
+      <c r="B53" s="13" t="s">
         <v>556</v>
-      </c>
-      <c r="B53" s="13" t="s">
-        <v>557</v>
       </c>
       <c r="C53" s="30" t="n">
         <f aca="false">(Assumptions!$D$93+Assumptions!$D$94)</f>
@@ -9309,32 +9307,32 @@
         <v>18.2469</v>
       </c>
       <c r="F53" s="2" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="G53" s="29" t="n">
         <f aca="false">MAX(1,ROUNDDOWN(E53*Assumptions!$D$89,0))</f>
         <v>10</v>
       </c>
       <c r="H53" s="2" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="I53" s="29" t="n">
         <f aca="false">MIN(G53,MAX(1,ROUNDUP(E53*Assumptions!$D$91,0)))</f>
         <v>6</v>
       </c>
       <c r="J53" s="2" t="s">
+        <v>558</v>
+      </c>
+      <c r="K53" s="13" t="s">
         <v>559</v>
-      </c>
-      <c r="K53" s="13" t="s">
-        <v>560</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="28" t="s">
+        <v>560</v>
+      </c>
+      <c r="B54" s="13" t="s">
         <v>561</v>
-      </c>
-      <c r="B54" s="13" t="s">
-        <v>562</v>
       </c>
       <c r="C54" s="30" t="n">
         <f aca="false">(Weekly!$D$4*4/7+Weekly!$D$5+Weekly!$D$6*3/7)</f>
@@ -9369,15 +9367,15 @@
         <v>670</v>
       </c>
       <c r="K54" s="13" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="28" t="s">
+        <v>563</v>
+      </c>
+      <c r="B55" s="13" t="s">
         <v>564</v>
-      </c>
-      <c r="B55" s="13" t="s">
-        <v>565</v>
       </c>
       <c r="C55" s="30" t="n">
         <f aca="false">(Weekly!$D$5+Weekly!$D$6)</f>
@@ -9412,12 +9410,12 @@
         <v>270</v>
       </c>
       <c r="K55" s="13" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="13" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
     </row>
   </sheetData>
@@ -9455,17 +9453,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="369.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="13" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="318.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="13" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9479,100 +9477,100 @@
         <v>305</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="E4" s="12" t="s">
         <v>306</v>
       </c>
       <c r="F4" s="12" t="s">
+        <v>571</v>
+      </c>
+      <c r="G4" s="12" t="s">
         <v>572</v>
       </c>
-      <c r="G4" s="12" t="s">
-        <v>573</v>
-      </c>
       <c r="H4" s="12" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="I4" s="12" t="s">
         <v>309</v>
       </c>
       <c r="J4" s="12" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="K4" s="12" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="L4" s="12" t="s">
         <v>426</v>
       </c>
       <c r="M4" s="12" t="s">
+        <v>574</v>
+      </c>
+      <c r="N4" s="12" t="s">
         <v>575</v>
       </c>
-      <c r="N4" s="12" t="s">
+      <c r="O4" s="12" t="s">
         <v>576</v>
       </c>
-      <c r="O4" s="12" t="s">
+      <c r="P4" s="12" t="s">
         <v>577</v>
       </c>
-      <c r="P4" s="12" t="s">
+      <c r="Q4" s="12" t="s">
         <v>578</v>
       </c>
-      <c r="Q4" s="12" t="s">
+      <c r="R4" s="12" t="s">
         <v>579</v>
       </c>
-      <c r="R4" s="12" t="s">
+      <c r="S4" s="12" t="s">
         <v>580</v>
       </c>
-      <c r="S4" s="12" t="s">
+      <c r="T4" s="12" t="s">
         <v>581</v>
       </c>
-      <c r="T4" s="12" t="s">
+      <c r="U4" s="12" t="s">
         <v>582</v>
       </c>
-      <c r="U4" s="12" t="s">
+      <c r="V4" s="12" t="s">
         <v>583</v>
       </c>
-      <c r="V4" s="12" t="s">
+      <c r="W4" s="12" t="s">
         <v>584</v>
       </c>
-      <c r="W4" s="12" t="s">
+      <c r="X4" s="12" t="s">
         <v>585</v>
       </c>
-      <c r="X4" s="12" t="s">
+      <c r="Y4" s="12" t="s">
         <v>586</v>
       </c>
-      <c r="Y4" s="12" t="s">
+      <c r="Z4" s="12" t="s">
         <v>587</v>
       </c>
-      <c r="Z4" s="12" t="s">
+      <c r="AA4" s="12" t="s">
         <v>588</v>
       </c>
-      <c r="AA4" s="12" t="s">
+      <c r="AB4" s="12" t="s">
         <v>589</v>
       </c>
-      <c r="AB4" s="12" t="s">
+      <c r="AC4" s="12" t="s">
         <v>590</v>
       </c>
-      <c r="AC4" s="12" t="s">
+      <c r="AD4" s="12" t="s">
         <v>591</v>
       </c>
-      <c r="AD4" s="12" t="s">
+      <c r="AE4" s="12" t="s">
         <v>592</v>
       </c>
-      <c r="AE4" s="12" t="s">
+      <c r="AF4" s="12" t="s">
         <v>593</v>
       </c>
-      <c r="AF4" s="12" t="s">
+      <c r="AG4" s="12" t="s">
         <v>594</v>
       </c>
-      <c r="AG4" s="12" t="s">
+      <c r="AH4" s="12" t="s">
         <v>595</v>
       </c>
-      <c r="AH4" s="12" t="s">
+      <c r="AI4" s="12" t="s">
         <v>596</v>
-      </c>
-      <c r="AI4" s="12" t="s">
-        <v>597</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12397,16 +12395,16 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
+        <v>597</v>
+      </c>
+      <c r="B25" s="2" t="s">
         <v>598</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>599</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>48</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>322</v>
@@ -12531,16 +12529,16 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>43</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>322</v>
@@ -12665,16 +12663,16 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>52</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>322</v>
@@ -12799,16 +12797,16 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>54</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>322</v>
@@ -12933,16 +12931,16 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
+        <v>602</v>
+      </c>
+      <c r="B29" s="2" t="s">
         <v>603</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>604</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>48</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>322</v>
@@ -13067,16 +13065,16 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>43</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>322</v>
@@ -13201,16 +13199,16 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>52</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>322</v>
@@ -13335,16 +13333,16 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>54</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="E32" s="2" t="s">
         <v>322</v>
@@ -13469,16 +13467,16 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
+        <v>607</v>
+      </c>
+      <c r="B33" s="2" t="s">
         <v>608</v>
-      </c>
-      <c r="B33" s="2" t="s">
-        <v>609</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>48</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>322</v>
@@ -13603,16 +13601,16 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
+        <v>609</v>
+      </c>
+      <c r="B34" s="2" t="s">
         <v>610</v>
-      </c>
-      <c r="B34" s="2" t="s">
-        <v>611</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>43</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="E34" s="2" t="s">
         <v>322</v>
@@ -13802,7 +13800,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="28" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13814,10 +13812,10 @@
         <v>47</v>
       </c>
       <c r="D38" s="12" t="s">
+        <v>612</v>
+      </c>
+      <c r="E38" s="12" t="s">
         <v>613</v>
-      </c>
-      <c r="E38" s="12" t="s">
-        <v>614</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13916,7 +13914,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13927,7 +13925,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="2" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="C4" s="41" t="n">
         <f aca="false">SUMIFS(Channels!X5:X34,Channels!D5:D34,"Channel")</f>
@@ -13936,7 +13934,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="C5" s="41" t="n">
         <f aca="false">SUMIFS(Channels!X5:X34,Channels!D5:D34,"Initiative")</f>
@@ -13945,7 +13943,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="2" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="C6" s="41" t="n">
         <f aca="false">Channels!Y35</f>
@@ -13954,7 +13952,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="2" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="C7" s="41" t="n">
         <f aca="false">C4+C5+C6</f>
@@ -13963,7 +13961,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="2" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="C8" s="41" t="n">
         <f aca="false">Channels!Z35</f>
@@ -13972,7 +13970,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="2" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="C9" s="41" t="n">
         <f aca="false">C7</f>
@@ -13981,7 +13979,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="2" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="C10" s="41" t="n">
         <f aca="false">IF(Assumptions!$D$48&lt;1,C9/(1-Assumptions!$D$48)*Assumptions!$D$48,0)</f>
@@ -13990,7 +13988,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="2" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="C11" s="41" t="n">
         <f aca="false">C9+C10</f>
@@ -13999,7 +13997,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="28" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="C12" s="4" t="n">
         <f aca="false">IF(Assumptions!$D$51&gt;0,ROUNDUP(C11/Assumptions!$D$51,0)*Assumptions!$D$51,C11)</f>
@@ -14008,7 +14006,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="2" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="C13" s="46" t="n">
         <f aca="false">MIN(Channels!U35,Funnel!B26)</f>
@@ -14017,7 +14015,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="2" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="C14" s="47" t="n">
         <f aca="false">IF(C13&gt;0,C9/C13,0)</f>
@@ -14026,7 +14024,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="2" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="C15" s="41" t="n">
         <f aca="false">IF(C13&gt;0,C12/C13,0)</f>
@@ -14035,7 +14033,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="2" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="C16" s="30" t="n">
         <f aca="false">IF(C12&gt;0,Weekly!N5/C12,0)</f>
@@ -14044,7 +14042,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="28" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14053,25 +14051,25 @@
         <v>305</v>
       </c>
       <c r="C20" s="12" t="s">
+        <v>629</v>
+      </c>
+      <c r="D20" s="12" t="s">
+        <v>586</v>
+      </c>
+      <c r="E20" s="12" t="s">
         <v>630</v>
       </c>
-      <c r="D20" s="12" t="s">
-        <v>587</v>
-      </c>
-      <c r="E20" s="12" t="s">
+      <c r="F20" s="12" t="s">
+        <v>588</v>
+      </c>
+      <c r="G20" s="12" t="s">
         <v>631</v>
       </c>
-      <c r="F20" s="12" t="s">
-        <v>589</v>
-      </c>
-      <c r="G20" s="12" t="s">
+      <c r="H20" s="12" t="s">
         <v>632</v>
       </c>
-      <c r="H20" s="12" t="s">
+      <c r="I20" s="12" t="s">
         <v>633</v>
-      </c>
-      <c r="I20" s="12" t="s">
-        <v>634</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14241,7 +14239,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="28" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14250,16 +14248,16 @@
         <v>304</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="D28" s="12" t="s">
+        <v>631</v>
+      </c>
+      <c r="E28" s="12" t="s">
         <v>632</v>
       </c>
-      <c r="E28" s="12" t="s">
-        <v>633</v>
-      </c>
       <c r="F28" s="12" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14390,7 +14388,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="2" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="C35" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$AA$5:$AA$34,Channels!$B$5:$B$34,B35)</f>
@@ -14411,7 +14409,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="2" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="C36" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$AA$5:$AA$34,Channels!$B$5:$B$34,B36)</f>
@@ -14432,7 +14430,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="2" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="C37" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$AA$5:$AA$34,Channels!$B$5:$B$34,B37)</f>
@@ -14453,7 +14451,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="2" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="C38" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$AA$5:$AA$34,Channels!$B$5:$B$34,B38)</f>
@@ -14493,7 +14491,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="28" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14505,10 +14503,10 @@
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="12"/>
       <c r="B44" s="12" t="s">
+        <v>637</v>
+      </c>
+      <c r="C44" s="12" t="s">
         <v>638</v>
-      </c>
-      <c r="C44" s="12" t="s">
-        <v>639</v>
       </c>
       <c r="D44" s="12" t="s">
         <v>48</v>
@@ -14523,10 +14521,10 @@
         <v>54</v>
       </c>
       <c r="H44" s="12" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="I44" s="12" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14599,17 +14597,17 @@
     </row>
     <row r="49" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="1" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="2" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E51" s="28" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="F51" s="48" t="n">
         <f aca="false">1</f>
@@ -14622,7 +14620,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E52" s="2" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="F52" s="41" t="n">
         <f aca="false">Budget!$C$12*F51</f>
@@ -14635,7 +14633,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E53" s="2" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="F53" s="41" t="n">
         <f aca="false">F52*(1-Assumptions!$D$48)</f>
@@ -14648,7 +14646,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E54" s="2" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="F54" s="41" t="n">
         <f aca="false">MAX(0,Budget!$C$9-F53)</f>
@@ -14661,44 +14659,44 @@
     </row>
     <row r="55" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="12" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="B55" s="12" t="s">
         <v>305</v>
       </c>
       <c r="C55" s="12" t="s">
+        <v>646</v>
+      </c>
+      <c r="D55" s="12" t="s">
         <v>647</v>
       </c>
-      <c r="D55" s="12" t="s">
+      <c r="E55" s="12" t="s">
+        <v>631</v>
+      </c>
+      <c r="F55" s="12" t="s">
         <v>648</v>
       </c>
-      <c r="E55" s="12" t="s">
-        <v>632</v>
-      </c>
-      <c r="F55" s="12" t="s">
+      <c r="G55" s="12" t="s">
         <v>649</v>
-      </c>
-      <c r="G55" s="12" t="s">
-        <v>650</v>
       </c>
       <c r="H55" s="12"/>
       <c r="I55" s="12"/>
       <c r="J55" s="12" t="s">
+        <v>650</v>
+      </c>
+      <c r="K55" s="12" t="s">
         <v>651</v>
-      </c>
-      <c r="K55" s="12" t="s">
-        <v>652</v>
       </c>
       <c r="L55" s="12"/>
       <c r="M55" s="12"/>
       <c r="N55" s="12" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="O55" s="12" t="s">
+        <v>652</v>
+      </c>
+      <c r="P55" s="12" t="s">
         <v>653</v>
-      </c>
-      <c r="P55" s="12" t="s">
-        <v>654</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
@@ -16203,7 +16201,7 @@
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E86" s="28" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16273,7 +16271,7 @@
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E92" s="2" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="F92" s="41" t="n">
         <f aca="false">IF(F91&gt;0,F52/F91,0)</f>
@@ -16286,7 +16284,7 @@
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E94" s="2" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="F94" s="32" t="n">
         <f aca="false">SUM(O56:O85)</f>
@@ -16299,7 +16297,7 @@
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E95" s="2" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="F95" s="30" t="n">
         <f aca="false">IF(F94&gt;0,MIN(1,Funnel!$B$22/F94),1)</f>
@@ -16312,7 +16310,7 @@
     </row>
     <row r="97" customFormat="false" ht="407.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="13" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
     </row>
   </sheetData>
@@ -16345,92 +16343,92 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="344" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="13" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
+        <v>660</v>
+      </c>
+      <c r="B3" s="12" t="s">
         <v>661</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="C3" s="12" t="s">
         <v>662</v>
       </c>
-      <c r="C3" s="12" t="s">
+      <c r="D3" s="12" t="s">
         <v>663</v>
       </c>
-      <c r="D3" s="12" t="s">
+      <c r="E3" s="12" t="s">
         <v>664</v>
       </c>
-      <c r="E3" s="12" t="s">
+      <c r="F3" s="12" t="s">
         <v>665</v>
       </c>
-      <c r="F3" s="12" t="s">
+      <c r="G3" s="12" t="s">
         <v>666</v>
       </c>
-      <c r="G3" s="12" t="s">
+      <c r="H3" s="12" t="s">
         <v>667</v>
       </c>
-      <c r="H3" s="12" t="s">
+      <c r="I3" s="12" t="s">
         <v>668</v>
       </c>
-      <c r="I3" s="12" t="s">
+      <c r="J3" s="12" t="s">
         <v>669</v>
       </c>
-      <c r="J3" s="12" t="s">
+      <c r="K3" s="12" t="s">
         <v>670</v>
       </c>
-      <c r="K3" s="12" t="s">
+      <c r="L3" s="12" t="s">
         <v>671</v>
       </c>
-      <c r="L3" s="12" t="s">
+      <c r="M3" s="12" t="s">
         <v>672</v>
       </c>
-      <c r="M3" s="12" t="s">
+      <c r="N3" s="12" t="s">
         <v>673</v>
       </c>
-      <c r="N3" s="12" t="s">
+      <c r="O3" s="12" t="s">
         <v>674</v>
       </c>
-      <c r="O3" s="12" t="s">
+      <c r="P3" s="12" t="s">
         <v>675</v>
       </c>
-      <c r="P3" s="12" t="s">
+      <c r="Q3" s="12" t="s">
         <v>676</v>
       </c>
-      <c r="Q3" s="12" t="s">
+      <c r="R3" s="12" t="s">
         <v>677</v>
       </c>
-      <c r="R3" s="12" t="s">
+      <c r="S3" s="12" t="s">
         <v>678</v>
       </c>
-      <c r="S3" s="12" t="s">
+      <c r="T3" s="12" t="s">
         <v>679</v>
       </c>
-      <c r="T3" s="12" t="s">
+      <c r="U3" s="12" t="s">
         <v>680</v>
       </c>
-      <c r="U3" s="12" t="s">
+      <c r="V3" s="12" t="s">
         <v>681</v>
       </c>
-      <c r="V3" s="12" t="s">
+      <c r="W3" s="12" t="s">
         <v>682</v>
       </c>
-      <c r="W3" s="12" t="s">
+      <c r="X3" s="12" t="s">
         <v>683</v>
       </c>
-      <c r="X3" s="12" t="s">
+      <c r="Y3" s="12" t="s">
         <v>684</v>
       </c>
-      <c r="Y3" s="12" t="s">
+      <c r="Z3" s="49" t="s">
         <v>685</v>
-      </c>
-      <c r="Z3" s="49" t="s">
-        <v>686</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17675,7 +17673,7 @@
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="B16" s="9"/>
       <c r="C16" s="9"/>
@@ -17727,12 +17725,12 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="28" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="2" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="F19" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot",Channels!$B$5:$B$34,"&lt;&gt;I1b Employee referral sprint (bonus on hire)",Channels!$B$5:$B$34,"&lt;&gt;I1a Talent rediscovery (past applicants in ATS)")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
@@ -17741,7 +17739,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="2" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="F20" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot",Channels!$B$5:$B$34,"&lt;&gt;I1b Employee referral sprint (bonus on hire)",Channels!$B$5:$B$34,"&lt;&gt;I1a Talent rediscovery (past applicants in ATS)")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$C$5:$C$34,"Supervisors")</f>
@@ -17750,7 +17748,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="2" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="F21" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$E$5:$E$34,"Slot")</f>
@@ -17759,7 +17757,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="2" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="F22" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,"I1b Employee referral sprint (bonus on hire)",Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
@@ -17768,7 +17766,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="2" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="F23" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,"I1b Employee referral sprint (bonus on hire)",Channels!$C$5:$C$34,"Supervisors")</f>
@@ -17777,7 +17775,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="2" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="F24" s="41" t="n">
         <f aca="false">SUM(Channels!$Z$5:$Z$34)</f>
@@ -17786,7 +17784,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="2" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="F25" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$AF$5:$AF$34,Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
@@ -17795,7 +17793,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="2" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="F26" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$AF$5:$AF$34,Channels!$C$5:$C$34,"Supervisors")</f>
@@ -17804,7 +17802,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="2" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="F27" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$AE$5:$AE$34,Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
@@ -17813,7 +17811,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="2" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="F28" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$AE$5:$AE$34,Channels!$C$5:$C$34,"Supervisors")</f>
@@ -17822,7 +17820,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="2" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="F29" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$AG$5:$AG$34,Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
@@ -17831,7 +17829,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="2" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="F30" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$AG$5:$AG$34,Channels!$C$5:$C$34,"Supervisors")</f>
@@ -17840,7 +17838,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="2" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="F31" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)")</f>
@@ -17849,7 +17847,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="2" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="F32" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$V$5:$V$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)",Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
@@ -17858,7 +17856,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="2" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="F33" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$V$5:$V$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)",Channels!$C$5:$C$34,"Supervisors")</f>
@@ -17867,7 +17865,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="2" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="F34" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$W$5:$W$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)",Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
@@ -17876,7 +17874,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="2" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="F35" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$W$5:$W$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)",Channels!$C$5:$C$34,"Supervisors")</f>
@@ -17885,7 +17883,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="2" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="F36" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$U$5:$U$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)",Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
@@ -17894,7 +17892,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="2" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="F37" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$U$5:$U$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)",Channels!$C$5:$C$34,"Supervisors")</f>
@@ -17903,7 +17901,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="2" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="F38" s="30" t="n">
         <f aca="false">IF(Funnel!B23&gt;0,MIN(1,Funnel!B22/Funnel!B23),1)</f>
@@ -17912,7 +17910,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="28" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17921,37 +17919,37 @@
         <v>304</v>
       </c>
       <c r="C43" s="12" t="s">
+        <v>709</v>
+      </c>
+      <c r="D43" s="12" t="s">
         <v>710</v>
       </c>
-      <c r="D43" s="12" t="s">
+      <c r="E43" s="12" t="s">
         <v>711</v>
       </c>
-      <c r="E43" s="12" t="s">
+      <c r="F43" s="12" t="s">
         <v>712</v>
       </c>
-      <c r="F43" s="12" t="s">
+      <c r="G43" s="12" t="s">
         <v>713</v>
       </c>
-      <c r="G43" s="12" t="s">
+      <c r="H43" s="12" t="s">
         <v>714</v>
       </c>
-      <c r="H43" s="12" t="s">
+      <c r="I43" s="12" t="s">
         <v>715</v>
       </c>
-      <c r="I43" s="12" t="s">
+      <c r="J43" s="12" t="s">
         <v>716</v>
       </c>
-      <c r="J43" s="12" t="s">
+      <c r="K43" s="12" t="s">
         <v>717</v>
       </c>
-      <c r="K43" s="12" t="s">
+      <c r="L43" s="12" t="s">
         <v>718</v>
       </c>
-      <c r="L43" s="12" t="s">
+      <c r="M43" s="12" t="s">
         <v>719</v>
-      </c>
-      <c r="M43" s="12" t="s">
-        <v>720</v>
       </c>
       <c r="N43" s="12" t="s">
         <v>436</v>
@@ -18589,12 +18587,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18608,67 +18606,67 @@
         <v>305</v>
       </c>
       <c r="D4" s="12" t="s">
+        <v>722</v>
+      </c>
+      <c r="E4" s="12" t="s">
         <v>723</v>
       </c>
-      <c r="E4" s="12" t="s">
+      <c r="F4" s="12" t="s">
         <v>724</v>
       </c>
-      <c r="F4" s="12" t="s">
+      <c r="G4" s="12" t="s">
         <v>725</v>
       </c>
-      <c r="G4" s="12" t="s">
+      <c r="H4" s="12" t="s">
         <v>726</v>
       </c>
-      <c r="H4" s="12" t="s">
+      <c r="I4" s="12" t="s">
         <v>727</v>
       </c>
-      <c r="I4" s="12" t="s">
+      <c r="J4" s="12" t="s">
         <v>728</v>
       </c>
-      <c r="J4" s="12" t="s">
+      <c r="K4" s="12" t="s">
         <v>729</v>
       </c>
-      <c r="K4" s="12" t="s">
+      <c r="L4" s="12" t="s">
         <v>730</v>
       </c>
-      <c r="L4" s="12" t="s">
+      <c r="M4" s="12" t="s">
         <v>731</v>
       </c>
-      <c r="M4" s="12" t="s">
+      <c r="N4" s="12" t="s">
         <v>732</v>
       </c>
-      <c r="N4" s="12" t="s">
+      <c r="O4" s="12" t="s">
         <v>733</v>
       </c>
-      <c r="O4" s="12" t="s">
+      <c r="P4" s="12" t="s">
         <v>734</v>
       </c>
-      <c r="P4" s="12" t="s">
+      <c r="Q4" s="12" t="s">
         <v>735</v>
       </c>
-      <c r="Q4" s="12" t="s">
+      <c r="R4" s="12" t="s">
         <v>736</v>
       </c>
-      <c r="R4" s="12" t="s">
+      <c r="S4" s="12" t="s">
         <v>737</v>
       </c>
-      <c r="S4" s="12" t="s">
+      <c r="T4" s="12" t="s">
         <v>738</v>
       </c>
-      <c r="T4" s="12" t="s">
+      <c r="U4" s="12" t="s">
         <v>739</v>
       </c>
-      <c r="U4" s="12" t="s">
+      <c r="V4" s="12" t="s">
         <v>740</v>
       </c>
-      <c r="V4" s="12" t="s">
+      <c r="W4" s="12" t="s">
         <v>741</v>
       </c>
-      <c r="W4" s="12" t="s">
+      <c r="X4" s="12" t="s">
         <v>742</v>
-      </c>
-      <c r="X4" s="12" t="s">
-        <v>743</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20856,7 +20854,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="28" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -20865,46 +20863,46 @@
         <v>305</v>
       </c>
       <c r="C39" s="12" t="s">
+        <v>744</v>
+      </c>
+      <c r="D39" s="12" t="s">
         <v>745</v>
       </c>
-      <c r="D39" s="12" t="s">
+      <c r="E39" s="12" t="s">
         <v>746</v>
       </c>
-      <c r="E39" s="12" t="s">
+      <c r="F39" s="12" t="s">
         <v>747</v>
       </c>
-      <c r="F39" s="12" t="s">
+      <c r="G39" s="12" t="s">
         <v>748</v>
       </c>
-      <c r="G39" s="12" t="s">
+      <c r="H39" s="12" t="s">
         <v>749</v>
       </c>
-      <c r="H39" s="12" t="s">
+      <c r="I39" s="12" t="s">
         <v>750</v>
       </c>
-      <c r="I39" s="12" t="s">
+      <c r="J39" s="12" t="s">
         <v>751</v>
       </c>
-      <c r="J39" s="12" t="s">
+      <c r="K39" s="12" t="s">
         <v>752</v>
       </c>
-      <c r="K39" s="12" t="s">
+      <c r="L39" s="12" t="s">
         <v>753</v>
       </c>
-      <c r="L39" s="12" t="s">
+      <c r="M39" s="12" t="s">
         <v>754</v>
       </c>
-      <c r="M39" s="12" t="s">
+      <c r="N39" s="12" t="s">
         <v>755</v>
-      </c>
-      <c r="N39" s="12" t="s">
-        <v>756</v>
       </c>
       <c r="O39" s="12" t="s">
         <v>47</v>
       </c>
       <c r="P39" s="12" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21134,7 +21132,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="9" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="B46" s="9"/>
       <c r="C46" s="9"/>

</xml_diff>

<commit_message>
Accuracy pass: final labels (I1M, I2F own estimates), Q&A sources verified, counts updated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V2NJtrYy3bzNxqKeiRXJfY
</commit_message>
<xml_diff>
--- a/operation_uptime/Operation_Uptime_Model.xlsx
+++ b/operation_uptime/Operation_Uptime_Model.xlsx
@@ -1169,7 +1169,7 @@
     <t xml:space="preserve">I1: messaging cost per contacted past applicant (email + SMS tool)</t>
   </si>
   <si>
-    <t xml:space="preserve">Three text messages at ~€0.08–0.11 each, plus email. https://www.seven.io/en/prices/</t>
+    <t xml:space="preserve">Three text messages at ~€0.075 each (seven.io) plus email, rounded up to €0.30. https://www.seven.io/en/prices/</t>
   </si>
   <si>
     <t xml:space="preserve">I1B</t>
@@ -6826,7 +6826,7 @@
         <v>119</v>
       </c>
       <c r="F161" s="2" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="G161" s="17" t="s">
         <v>380</v>
@@ -7012,7 +7012,7 @@
         <v>119</v>
       </c>
       <c r="F169" s="2" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="G169" s="17" t="s">
         <v>404</v>
@@ -7278,7 +7278,7 @@
     <hyperlink ref="G154" r:id="rId72" display="Cold outreach gets ~5% replies (Pin 2026); past applicants already know the employer, so I assume 12%. https://www.pin.com/blog/recruiting-outreach-benchmark-report/"/>
     <hyperlink ref="G155" r:id="rId73" display="They met the requirements once; I assume half still do (Forrester via SHRM: most remain a 70%+ match). https://www.shrm.org/mena/topics-tools/news/technology/talent-rediscovery-tools-help-address-labor-shortages"/>
     <hyperlink ref="G160" r:id="rId74" display="Referred applicants are better pre-filtered (IAB: referrals are the most decisive channel), so 45% qualify. https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/"/>
-    <hyperlink ref="G161" r:id="rId75" display="Three text messages at ~€0.08–0.11 each, plus email. https://www.seven.io/en/prices/"/>
+    <hyperlink ref="G161" r:id="rId75" display="Three text messages at ~€0.075 each (seven.io) plus email, rounded up to €0.30. https://www.seven.io/en/prices/"/>
     <hyperlink ref="G162" r:id="rId76" display="Most firms pay €501–1,000 per successful referral (Radancy survey, 335 firms worldwide). https://www.personalwirtschaft.de/?p=166393"/>
     <hyperlink ref="G163" r:id="rId77" display="Referred and known candidates pass and accept a little more often (+15%). https://www.metaview.ai/resources/blog/do-referred-candidates-interview-better"/>
     <hyperlink ref="G164" r:id="rId78" display="BA employment, KldB 2621 Bauelektrik: Berlin 6,204 + 60% of Brandenburg 5,905 (75 km radius, own scaling) ≈ 10,000. Berlin file: https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-11-0-202512-xlsx.xlsx?__blob=publicationFile https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-12-0-202512-xlsx.xlsx?__blob=publicationFile"/>

</xml_diff>

<commit_message>
Accuracy fixes from independent re-audit: supervisor pacing by useful days, first-assessment logic explained, cut advice consistent with the cut rule, media lower bound labelled
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V2NJtrYy3bzNxqKeiRXJfY
</commit_message>
<xml_diff>
--- a/operation_uptime/Operation_Uptime_Model.xlsx
+++ b/operation_uptime/Operation_Uptime_Model.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1463" uniqueCount="765">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1464" uniqueCount="766">
   <si>
     <t xml:space="preserve">Operation Uptime — model summary (hypothetical Tesla Giga Berlin maintenance hiring)</t>
   </si>
@@ -221,7 +221,7 @@
     <t xml:space="preserve">Own estimate</t>
   </si>
   <si>
-    <t xml:space="preserve">Re-applicants were screened before, so the first assessments can run on day 2.</t>
+    <t xml:space="preserve">At launch there is no queue, so the first applicants (and re-applicants) can be assessed within 2 days; the 6-day lag (T2) applies once the queue is full and sets the last useful date.</t>
   </si>
   <si>
     <t xml:space="preserve">T1</t>
@@ -1463,7 +1463,7 @@
     <t xml:space="preserve">Hires lost vs 100</t>
   </si>
   <si>
-    <t xml:space="preserve">Paid media needed (€, approx.)</t>
+    <t xml:space="preserve">Paid media needed (€, lower bound: same channels, caps ignored)</t>
   </si>
   <si>
     <t xml:space="preserve">Change in media</t>
@@ -2106,6 +2106,9 @@
   </si>
   <si>
     <t xml:space="preserve">Input share (Assumptions W1–W11)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Supervisor share before re-scaling (useful days only)</t>
   </si>
   <si>
     <t xml:space="preserve">Weak channels are cut from Mon 2 Nov; tests are judged by Mon 9 Nov; the reserve is released only from week 3, on the Tracker rules.</t>
@@ -3475,7 +3478,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
         <v>60</v>
       </c>
@@ -4198,7 +4201,7 @@
         <v>131</v>
       </c>
       <c r="D53" s="16" t="n">
-        <v>0.26</v>
+        <v>0.25</v>
       </c>
       <c r="E53" s="2" t="s">
         <v>44</v>
@@ -4244,7 +4247,7 @@
         <v>131</v>
       </c>
       <c r="D55" s="16" t="n">
-        <v>0.185</v>
+        <v>0.18</v>
       </c>
       <c r="E55" s="2" t="s">
         <v>44</v>
@@ -4267,7 +4270,7 @@
         <v>131</v>
       </c>
       <c r="D56" s="16" t="n">
-        <v>0.19</v>
+        <v>0.185</v>
       </c>
       <c r="E56" s="2" t="s">
         <v>44</v>
@@ -4290,7 +4293,7 @@
         <v>131</v>
       </c>
       <c r="D57" s="16" t="n">
-        <v>0.19</v>
+        <v>0.215</v>
       </c>
       <c r="E57" s="2" t="s">
         <v>44</v>
@@ -4313,7 +4316,7 @@
         <v>131</v>
       </c>
       <c r="D58" s="16" t="n">
-        <v>0.03</v>
+        <v>0.025</v>
       </c>
       <c r="E58" s="2" t="s">
         <v>44</v>
@@ -8057,8 +8060,8 @@
     </row>
     <row r="35" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="9" t="str">
-        <f aca="false">"Hardest role: "&amp;Summary!C16&amp;", the highest in column H. Why: industrial electricians are the scarcest trade in Brandenburg (KOFA 2026: 85.7% of vacancies have no suitable unemployed candidate vs 41.4% overall, https://www.kofa.de/media/Publikationen/Laendersteckbriefe/Brandenburg.pdf), and they have no Polish or foreign-trained route under the brief. Automation’s pool is tighter (column G: "&amp;TEXT(G32,"0%")&amp;" of reachable people vs "&amp;TEXT(G30,"0%")&amp;"), but it needs only "&amp;B32&amp;" hires and its last hire is cheaper, so it is watched in the weekly pool check rather than ranked hardest."</f>
-        <v>Hardest role: Electricians (last hire costs €2,272), the highest in column H. Why: industrial electricians are the scarcest trade in Brandenburg (KOFA 2026: 85.7% of vacancies have no suitable unemployed candidate vs 41.4% overall, https://www.kofa.de/media/Publikationen/Laendersteckbriefe/Brandenburg.pdf), and they have no Polish or foreign-trained route under the brief. Automation’s pool is tighter (column G: 22% of reachable people vs 12%), but it needs only 15 hires and its last hire is cheaper, so it is watched in the weekly pool check rather than ranked hardest.</v>
+        <f aca="false">"Hardest role: "&amp;Summary!C16&amp;", the highest in column H. Why: industrial electricians are the scarcest trade in Brandenburg (KOFA 2026: 85.7% of vacancies have no suitable unemployed candidate vs 41.4% overall, https://www.kofa.de/media/Publikationen/Laendersteckbriefe/Brandenburg.pdf), and they have no Polish or foreign-trained route under the brief. Automation’s pool and channel coverage are tighter (column G: "&amp;TEXT(G32,"0%")&amp;" of reachable people vs "&amp;TEXT(G30,"0%")&amp;"; column E: "&amp;TEXT(E32,"0.0")&amp;"× vs "&amp;TEXT(E30,"0.0")&amp;"×), but it needs only "&amp;B32&amp;" hires and its last hire is cheaper, so it is watched in the weekly pool check rather than ranked hardest."</f>
+        <v>Hardest role: Electricians (last hire costs €2,272), the highest in column H. Why: industrial electricians are the scarcest trade in Brandenburg (KOFA 2026: 85.7% of vacancies have no suitable unemployed candidate vs 41.4% overall, https://www.kofa.de/media/Publikationen/Laendersteckbriefe/Brandenburg.pdf), and they have no Polish or foreign-trained route under the brief. Automation’s pool and channel coverage are tighter (column G: 22% of reachable people vs 12%; column E: 3.2× vs 3.7×), but it needs only 15 hires and its last hire is cheaper, so it is watched in the weekly pool check rather than ranked hardest.</v>
       </c>
       <c r="B35" s="9"/>
       <c r="C35" s="9"/>
@@ -9321,7 +9324,7 @@
       </c>
       <c r="E53" s="32" t="n">
         <f aca="false">(SUMIFS(Channels!$V:$V,Channels!$A:$A,"I1a-E")+SUMIFS(Channels!$V:$V,Channels!$A:$A,"I1a-M")+SUMIFS(Channels!$V:$V,Channels!$A:$A,"I1a-A")+SUMIFS(Channels!$V:$V,Channels!$A:$A,"I1a-S"))*(Assumptions!$D$93+Assumptions!$D$94)+(SUMIFS(Channels!$V:$V,Channels!$A:$A,"I1b-E")+SUMIFS(Channels!$V:$V,Channels!$A:$A,"I1b-M")+SUMIFS(Channels!$V:$V,Channels!$A:$A,"I1b-A")+SUMIFS(Channels!$V:$V,Channels!$A:$A,"I1b-S"))*(Weekly!$D$4+Weekly!$D$5)</f>
-        <v>23.2959</v>
+        <v>22.9989</v>
       </c>
       <c r="F53" s="2" t="s">
         <v>564</v>
@@ -9353,15 +9356,15 @@
       </c>
       <c r="C54" s="30" t="n">
         <f aca="false">(Weekly!$D$4*4/7+Weekly!$D$5+Weekly!$D$6*3/7)</f>
-        <v>0.372857142857143</v>
+        <v>0.365</v>
       </c>
       <c r="D54" s="41" t="n">
         <f aca="false">B33+SUMIFS(Channels!$X:$X,Channels!$A:$A,"I2-E")*C54</f>
-        <v>4895.76</v>
+        <v>4817.88</v>
       </c>
       <c r="E54" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$V:$V,Channels!$A:$A,"I2-E")*C54</f>
-        <v>10.9992857142857</v>
+        <v>10.7675</v>
       </c>
       <c r="F54" s="41" t="n">
         <f aca="false">IF(B28&gt;0,B27/B28,0)</f>
@@ -9396,15 +9399,15 @@
       </c>
       <c r="C55" s="30" t="n">
         <f aca="false">(Weekly!$D$5+Weekly!$D$6)</f>
-        <v>0.33</v>
+        <v>0.325</v>
       </c>
       <c r="D55" s="41" t="n">
         <f aca="false">B46+SUMIFS(Channels!$X:$X,Channels!$A:$A,"I3-M")*C55</f>
-        <v>2542.85714285714</v>
+        <v>2510.38961038961</v>
       </c>
       <c r="E55" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$V:$V,Channels!$A:$A,"I3-M")*C55</f>
-        <v>16</v>
+        <v>15.7575757575758</v>
       </c>
       <c r="F55" s="41" t="n">
         <f aca="false">IF(B39&gt;0,B38/B39,0)</f>
@@ -14054,7 +14057,7 @@
       </c>
       <c r="C16" s="30" t="n">
         <f aca="false">IF(C12&gt;0,Weekly!N5/C12,0)</f>
-        <v>0.388897765857544</v>
+        <v>0.39201909828295</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16347,7 +16350,7 @@
     <tabColor rgb="FF8EA9DB"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Z55"/>
+  <dimension ref="A1:AA55"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="1"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
@@ -16447,6 +16450,9 @@
       <c r="Z3" s="49" t="s">
         <v>692</v>
       </c>
+      <c r="AA3" s="49" t="s">
+        <v>693</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="29" t="n">
@@ -16462,11 +16468,11 @@
       </c>
       <c r="D4" s="30" t="n">
         <f aca="false">IF(SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$19)*$Z$4:$Z$14)&gt;0,IF(B4&lt;=Funnel!$B$19,Z4,0)/SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$19)*$Z$4:$Z$14),0)</f>
-        <v>0.26</v>
+        <v>0.25</v>
       </c>
       <c r="E4" s="30" t="n">
-        <f aca="false">IF(SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14)&gt;0,IF(B4&lt;=Funnel!$B$20,D4,0)/SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14),0)</f>
-        <v>0.268041237113402</v>
+        <f aca="false">IF(SUM($AA$4:$AA$14)&gt;0,AA4/SUM($AA$4:$AA$14),0)</f>
+        <v>0.31616982836495</v>
       </c>
       <c r="F4" s="30" t="n">
         <f aca="false">IF(A4-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($D$4:$D$14,A4-ROUNDUP(Funnel!$B$15/7,0)),0)</f>
@@ -16478,7 +16484,7 @@
       </c>
       <c r="H4" s="41" t="n">
         <f aca="false">$F$19*D4+$F$20*E4+$F$31*Y4</f>
-        <v>19435.5174685318</v>
+        <v>19398.7108822494</v>
       </c>
       <c r="I4" s="41" t="n">
         <f aca="false">IF(A4=1,$F$21,0)</f>
@@ -16498,19 +16504,19 @@
       </c>
       <c r="M4" s="41" t="n">
         <f aca="false">SUM(H4:L4)</f>
-        <v>30431.5174685318</v>
+        <v>30394.7108822494</v>
       </c>
       <c r="N4" s="41" t="n">
         <f aca="false">SUM($M$4:M4)</f>
-        <v>30431.5174685318</v>
+        <v>30394.7108822494</v>
       </c>
       <c r="O4" s="29" t="n">
         <f aca="false">(Funnel!$M$5+Funnel!$M$6+Funnel!$M$7-$F$27-$F$34)*D4+(Funnel!$M$8-$F$28-$F$35)*E4+($F$27+$F$28)*X4+($F$34+$F$35)*Y4</f>
-        <v>407.148943758426</v>
+        <v>403.092612777087</v>
       </c>
       <c r="P4" s="29" t="n">
         <f aca="false">(Funnel!$O$5+Funnel!$O$6+Funnel!$O$7-$F$25-$F$32)*D4+(Funnel!$O$8-$F$26-$F$33)*E4+($F$25+$F$26)*X4+($F$32+$F$33)*Y4</f>
-        <v>86.3784848169698</v>
+        <v>85.6365349277805</v>
       </c>
       <c r="Q4" s="29" t="n">
         <f aca="false">Assumptions!$D$9*MAX(0,MIN(C4+Assumptions!$D$21,Funnel!$B$17)-MAX(IF(A4=1,Funnel!$B$13,B4+Assumptions!$D$21),Funnel!$B$13)+1)/7</f>
@@ -16518,7 +16524,7 @@
       </c>
       <c r="R4" s="30" t="n">
         <f aca="false">IF(Q4&gt;0,P4/Q4,IF(P4&gt;0,9.99,0))</f>
-        <v>0.999420485485601</v>
+        <v>0.990835941313163</v>
       </c>
       <c r="S4" s="2" t="str">
         <f aca="false">IF(P4&gt;Q4+0.5,"OVER "&amp;Assumptions!$D$9&amp;"/wk – pace down",IF(R4&gt;Assumptions!$D$102,"Full",IF(AND(Q4&gt;=Assumptions!$D$103,P4&lt;Assumptions!$D$103),"Under "&amp;Assumptions!$D$103&amp;" – release reserve","")))</f>
@@ -16550,7 +16556,11 @@
       </c>
       <c r="Z4" s="30" t="n">
         <f aca="false">Assumptions!$D$53</f>
-        <v>0.26</v>
+        <v>0.25</v>
+      </c>
+      <c r="AA4" s="30" t="n">
+        <f aca="false">D4*IF(MAX(0,MIN(C4,Funnel!$B$19)-B4+1)&gt;0,MAX(0,MIN(C4,Funnel!$B$20)-B4+1)/MAX(0,MIN(C4,Funnel!$B$19)-B4+1),0)</f>
+        <v>0.25</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16570,8 +16580,8 @@
         <v>0.145</v>
       </c>
       <c r="E5" s="30" t="n">
-        <f aca="false">IF(SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14)&gt;0,IF(B5&lt;=Funnel!$B$20,D5,0)/SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14),0)</f>
-        <v>0.149484536082474</v>
+        <f aca="false">IF(SUM($AA$4:$AA$14)&gt;0,AA5/SUM($AA$4:$AA$14),0)</f>
+        <v>0.183378500451671</v>
       </c>
       <c r="F5" s="30" t="n">
         <f aca="false">IF(A5-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($D$4:$D$14,A5-ROUNDUP(Funnel!$B$15/7,0)),0)</f>
@@ -16583,7 +16593,7 @@
       </c>
       <c r="H5" s="41" t="n">
         <f aca="false">$F$19*D5+$F$20*E5+$F$31*Y5</f>
-        <v>10836.2144343735</v>
+        <v>11247.5809117046</v>
       </c>
       <c r="I5" s="41" t="n">
         <f aca="false">IF(A5=1,$F$21,0)</f>
@@ -16603,19 +16613,19 @@
       </c>
       <c r="M5" s="41" t="n">
         <f aca="false">SUM(H5:L5)</f>
-        <v>16236.2144343735</v>
+        <v>16647.5809117046</v>
       </c>
       <c r="N5" s="47" t="n">
         <f aca="false">SUM($M$4:M5)</f>
-        <v>46667.7319029052</v>
+        <v>47042.291793954</v>
       </c>
       <c r="O5" s="29" t="n">
         <f aca="false">(Funnel!$M$5+Funnel!$M$6+Funnel!$M$7-$F$27-$F$34)*D5+(Funnel!$M$8-$F$28-$F$35)*E5+($F$27+$F$28)*X5+($F$34+$F$35)*Y5</f>
-        <v>251.894922700201</v>
+        <v>257.671324604645</v>
       </c>
       <c r="P5" s="29" t="n">
         <f aca="false">(Funnel!$O$5+Funnel!$O$6+Funnel!$O$7-$F$25-$F$32)*D5+(Funnel!$O$8-$F$26-$F$33)*E5+($F$25+$F$26)*X5+($F$32+$F$33)*Y5</f>
-        <v>52.2173348421763</v>
+        <v>53.435335317969</v>
       </c>
       <c r="Q5" s="29" t="n">
         <f aca="false">Assumptions!$D$9*MAX(0,MIN(C5+Assumptions!$D$21,Funnel!$B$17)-MAX(IF(A5=1,Funnel!$B$13,B5+Assumptions!$D$21),Funnel!$B$13)+1)/7</f>
@@ -16623,7 +16633,7 @@
       </c>
       <c r="R5" s="30" t="n">
         <f aca="false">IF(Q5&gt;0,P5/Q5,IF(P5&gt;0,9.99,0))</f>
-        <v>0.949406088039569</v>
+        <v>0.971551551235801</v>
       </c>
       <c r="S5" s="2" t="str">
         <f aca="false">IF(P5&gt;Q5+0.5,"OVER "&amp;Assumptions!$D$9&amp;"/wk – pace down",IF(R5&gt;Assumptions!$D$102,"Full",IF(AND(Q5&gt;=Assumptions!$D$103,P5&lt;Assumptions!$D$103),"Under "&amp;Assumptions!$D$103&amp;" – release reserve","")))</f>
@@ -16657,6 +16667,10 @@
         <f aca="false">Assumptions!$D$54</f>
         <v>0.145</v>
       </c>
+      <c r="AA5" s="30" t="n">
+        <f aca="false">D5*IF(MAX(0,MIN(C5,Funnel!$B$19)-B5+1)&gt;0,MAX(0,MIN(C5,Funnel!$B$20)-B5+1)/MAX(0,MIN(C5,Funnel!$B$19)-B5+1),0)</f>
+        <v>0.145</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="29" t="n">
@@ -16672,11 +16686,11 @@
       </c>
       <c r="D6" s="30" t="n">
         <f aca="false">IF(SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$19)*$Z$4:$Z$14)&gt;0,IF(B6&lt;=Funnel!$B$19,Z6,0)/SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$19)*$Z$4:$Z$14),0)</f>
-        <v>0.185</v>
+        <v>0.18</v>
       </c>
       <c r="E6" s="30" t="n">
-        <f aca="false">IF(SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14)&gt;0,IF(B6&lt;=Funnel!$B$20,D6,0)/SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14),0)</f>
-        <v>0.190721649484536</v>
+        <f aca="false">IF(SUM($AA$4:$AA$14)&gt;0,AA6/SUM($AA$4:$AA$14),0)</f>
+        <v>0.227642276422764</v>
       </c>
       <c r="F6" s="30" t="n">
         <f aca="false">IF(A6-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($D$4:$D$14,A6-ROUNDUP(Funnel!$B$15/7,0)),0)</f>
@@ -16688,7 +16702,7 @@
       </c>
       <c r="H6" s="41" t="n">
         <f aca="false">$F$19*D6+$F$20*E6+$F$31*Y6</f>
-        <v>13809.0569679937</v>
+        <v>13946.6892352196</v>
       </c>
       <c r="I6" s="41" t="n">
         <f aca="false">IF(A6=1,$F$21,0)</f>
@@ -16708,19 +16722,19 @@
       </c>
       <c r="M6" s="41" t="n">
         <f aca="false">SUM(H6:L6)</f>
-        <v>13809.0569679937</v>
+        <v>13946.6892352196</v>
       </c>
       <c r="N6" s="41" t="n">
         <f aca="false">SUM($M$4:M6)</f>
-        <v>60476.788870899</v>
+        <v>60988.9810291736</v>
       </c>
       <c r="O6" s="29" t="n">
         <f aca="false">(Funnel!$M$5+Funnel!$M$6+Funnel!$M$7-$F$27-$F$34)*D6+(Funnel!$M$8-$F$28-$F$35)*E6+($F$27+$F$28)*X6+($F$34+$F$35)*Y6</f>
-        <v>262.07462527929</v>
+        <v>262.237508786858</v>
       </c>
       <c r="P6" s="29" t="n">
         <f aca="false">(Funnel!$O$5+Funnel!$O$6+Funnel!$O$7-$F$25-$F$32)*D6+(Funnel!$O$8-$F$26-$F$33)*E6+($F$25+$F$26)*X6+($F$32+$F$33)*Y6</f>
-        <v>53.968688126149</v>
+        <v>54.0597133620274</v>
       </c>
       <c r="Q6" s="29" t="n">
         <f aca="false">Assumptions!$D$9*MAX(0,MIN(C6+Assumptions!$D$21,Funnel!$B$17)-MAX(IF(A6=1,Funnel!$B$13,B6+Assumptions!$D$21),Funnel!$B$13)+1)/7</f>
@@ -16728,7 +16742,7 @@
       </c>
       <c r="R6" s="30" t="n">
         <f aca="false">IF(Q6&gt;0,P6/Q6,IF(P6&gt;0,9.99,0))</f>
-        <v>0.981248875020891</v>
+        <v>0.98290387930959</v>
       </c>
       <c r="S6" s="2" t="str">
         <f aca="false">IF(P6&gt;Q6+0.5,"OVER "&amp;Assumptions!$D$9&amp;"/wk – pace down",IF(R6&gt;Assumptions!$D$102,"Full",IF(AND(Q6&gt;=Assumptions!$D$103,P6&lt;Assumptions!$D$103),"Under "&amp;Assumptions!$D$103&amp;" – release reserve","")))</f>
@@ -16760,7 +16774,11 @@
       </c>
       <c r="Z6" s="30" t="n">
         <f aca="false">Assumptions!$D$55</f>
-        <v>0.185</v>
+        <v>0.18</v>
+      </c>
+      <c r="AA6" s="30" t="n">
+        <f aca="false">D6*IF(MAX(0,MIN(C6,Funnel!$B$19)-B6+1)&gt;0,MAX(0,MIN(C6,Funnel!$B$20)-B6+1)/MAX(0,MIN(C6,Funnel!$B$19)-B6+1),0)</f>
+        <v>0.18</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16777,15 +16795,15 @@
       </c>
       <c r="D7" s="30" t="n">
         <f aca="false">IF(SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$19)*$Z$4:$Z$14)&gt;0,IF(B7&lt;=Funnel!$B$19,Z7,0)/SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$19)*$Z$4:$Z$14),0)</f>
-        <v>0.19</v>
+        <v>0.185</v>
       </c>
       <c r="E7" s="30" t="n">
-        <f aca="false">IF(SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14)&gt;0,IF(B7&lt;=Funnel!$B$20,D7,0)/SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14),0)</f>
-        <v>0.195876288659794</v>
+        <f aca="false">IF(SUM($AA$4:$AA$14)&gt;0,AA7/SUM($AA$4:$AA$14),0)</f>
+        <v>0.233965672990063</v>
       </c>
       <c r="F7" s="30" t="n">
         <f aca="false">IF(A7-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($D$4:$D$14,A7-ROUNDUP(Funnel!$B$15/7,0)),0)</f>
-        <v>0.26</v>
+        <v>0.25</v>
       </c>
       <c r="G7" s="30" t="n">
         <f aca="false">IF(A7-ROUNDUP(Funnel!$B$16/7,0)&gt;=1,INDEX($E$4:$E$14,A7-ROUNDUP(Funnel!$B$16/7,0)),0)</f>
@@ -16793,7 +16811,7 @@
       </c>
       <c r="H7" s="41" t="n">
         <f aca="false">$F$19*D7+$F$20*E7+$F$31*Y7</f>
-        <v>14175.1235346963</v>
+        <v>14326.9408528645</v>
       </c>
       <c r="I7" s="41" t="n">
         <f aca="false">IF(A7=1,$F$21,0)</f>
@@ -16801,7 +16819,7 @@
       </c>
       <c r="J7" s="41" t="n">
         <f aca="false">$F$22*F7+$F$23*G7</f>
-        <v>2566.00305</v>
+        <v>2467.310625</v>
       </c>
       <c r="K7" s="41" t="n">
         <f aca="false">IF(A7=1,Budget!$C$6,0)</f>
@@ -16813,19 +16831,19 @@
       </c>
       <c r="M7" s="41" t="n">
         <f aca="false">SUM(H7:L7)</f>
-        <v>16741.1265846963</v>
+        <v>16794.2514778646</v>
       </c>
       <c r="N7" s="41" t="n">
         <f aca="false">SUM($M$4:M7)</f>
-        <v>77217.9154555953</v>
+        <v>77783.2325070381</v>
       </c>
       <c r="O7" s="29" t="n">
         <f aca="false">(Funnel!$M$5+Funnel!$M$6+Funnel!$M$7-$F$27-$F$34)*D7+(Funnel!$M$8-$F$28-$F$35)*E7+($F$27+$F$28)*X7+($F$34+$F$35)*Y7</f>
-        <v>266.297247584136</v>
+        <v>266.659317364271</v>
       </c>
       <c r="P7" s="29" t="n">
         <f aca="false">(Funnel!$O$5+Funnel!$O$6+Funnel!$O$7-$F$25-$F$32)*D7+(Funnel!$O$8-$F$26-$F$33)*E7+($F$25+$F$26)*X7+($F$32+$F$33)*Y7</f>
-        <v>53.9970634809098</v>
+        <v>54.1300887331949</v>
       </c>
       <c r="Q7" s="29" t="n">
         <f aca="false">Assumptions!$D$9*MAX(0,MIN(C7+Assumptions!$D$21,Funnel!$B$17)-MAX(IF(A7=1,Funnel!$B$13,B7+Assumptions!$D$21),Funnel!$B$13)+1)/7</f>
@@ -16833,7 +16851,7 @@
       </c>
       <c r="R7" s="30" t="n">
         <f aca="false">IF(Q7&gt;0,P7/Q7,IF(P7&gt;0,9.99,0))</f>
-        <v>0.981764790561996</v>
+        <v>0.984183431512634</v>
       </c>
       <c r="S7" s="2" t="str">
         <f aca="false">IF(P7&gt;Q7+0.5,"OVER "&amp;Assumptions!$D$9&amp;"/wk – pace down",IF(R7&gt;Assumptions!$D$102,"Full",IF(AND(Q7&gt;=Assumptions!$D$103,P7&lt;Assumptions!$D$103),"Under "&amp;Assumptions!$D$103&amp;" – release reserve","")))</f>
@@ -16841,7 +16859,7 @@
       </c>
       <c r="T7" s="32" t="n">
         <f aca="false">$F$38*(F7*(Budget!$G$21+Budget!$G$22+Budget!$G$23-$F$29-$F$36)+IF(A7-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($X$4:$X$14,A7-ROUNDUP(Funnel!$B$15/7,0))*$F$29+INDEX($Y$4:$Y$14,A7-ROUNDUP(Funnel!$B$15/7,0))*$F$36,0))</f>
-        <v>25.1959660894661</v>
+        <v>24.3656358529994</v>
       </c>
       <c r="U7" s="32" t="n">
         <f aca="false">$F$38*(G7*(Budget!$G$24-$F$30-$F$37)+IF(A7-ROUNDUP(Funnel!$B$16/7,0)&gt;=1,INDEX($X$4:$X$14,A7-ROUNDUP(Funnel!$B$16/7,0))*$F$30+INDEX($Y$4:$Y$14,A7-ROUNDUP(Funnel!$B$16/7,0))*$F$37,0))</f>
@@ -16849,11 +16867,11 @@
       </c>
       <c r="V7" s="32" t="n">
         <f aca="false">T7+U7</f>
-        <v>25.1959660894661</v>
+        <v>24.3656358529994</v>
       </c>
       <c r="W7" s="32" t="n">
         <f aca="false">SUM($V$4:V7)</f>
-        <v>25.1959660894661</v>
+        <v>24.3656358529994</v>
       </c>
       <c r="X7" s="30" t="n">
         <f aca="false">IF(A7=1,Assumptions!$D$50,IF(A7=2,1-Assumptions!$D$50,0))</f>
@@ -16865,7 +16883,11 @@
       </c>
       <c r="Z7" s="30" t="n">
         <f aca="false">Assumptions!$D$56</f>
-        <v>0.19</v>
+        <v>0.185</v>
+      </c>
+      <c r="AA7" s="30" t="n">
+        <f aca="false">D7*IF(MAX(0,MIN(C7,Funnel!$B$19)-B7+1)&gt;0,MAX(0,MIN(C7,Funnel!$B$20)-B7+1)/MAX(0,MIN(C7,Funnel!$B$19)-B7+1),0)</f>
+        <v>0.185</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16882,11 +16904,11 @@
       </c>
       <c r="D8" s="30" t="n">
         <f aca="false">IF(SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$19)*$Z$4:$Z$14)&gt;0,IF(B8&lt;=Funnel!$B$19,Z8,0)/SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$19)*$Z$4:$Z$14),0)</f>
-        <v>0.19</v>
+        <v>0.215</v>
       </c>
       <c r="E8" s="30" t="n">
-        <f aca="false">IF(SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14)&gt;0,IF(B8&lt;=Funnel!$B$20,D8,0)/SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14),0)</f>
-        <v>0.195876288659794</v>
+        <f aca="false">IF(SUM($AA$4:$AA$14)&gt;0,AA8/SUM($AA$4:$AA$14),0)</f>
+        <v>0.038843721770551</v>
       </c>
       <c r="F8" s="30" t="n">
         <f aca="false">IF(A8-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($D$4:$D$14,A8-ROUNDUP(Funnel!$B$15/7,0)),0)</f>
@@ -16894,11 +16916,11 @@
       </c>
       <c r="G8" s="30" t="n">
         <f aca="false">IF(A8-ROUNDUP(Funnel!$B$16/7,0)&gt;=1,INDEX($E$4:$E$14,A8-ROUNDUP(Funnel!$B$16/7,0)),0)</f>
-        <v>0.268041237113402</v>
+        <v>0.31616982836495</v>
       </c>
       <c r="H8" s="41" t="n">
         <f aca="false">$F$19*D8+$F$20*E8+$F$31*Y8</f>
-        <v>14175.1235346963</v>
+        <v>13821.5824640265</v>
       </c>
       <c r="I8" s="41" t="n">
         <f aca="false">IF(A8=1,$F$21,0)</f>
@@ -16906,7 +16928,7 @@
       </c>
       <c r="J8" s="41" t="n">
         <f aca="false">$F$22*F8+$F$23*G8</f>
-        <v>1728.15985322165</v>
+        <v>1781.50967469512</v>
       </c>
       <c r="K8" s="41" t="n">
         <f aca="false">IF(A8=1,Budget!$C$6,0)</f>
@@ -16918,19 +16940,19 @@
       </c>
       <c r="M8" s="41" t="n">
         <f aca="false">SUM(H8:L8)</f>
-        <v>15903.2833879179</v>
+        <v>15603.0921387216</v>
       </c>
       <c r="N8" s="41" t="n">
         <f aca="false">SUM($M$4:M8)</f>
-        <v>93121.1988435132</v>
+        <v>93386.3246457597</v>
       </c>
       <c r="O8" s="29" t="n">
         <f aca="false">(Funnel!$M$5+Funnel!$M$6+Funnel!$M$7-$F$27-$F$34)*D8+(Funnel!$M$8-$F$28-$F$35)*E8+($F$27+$F$28)*X8+($F$34+$F$35)*Y8</f>
-        <v>266.297247584136</v>
+        <v>270.18156279478</v>
       </c>
       <c r="P8" s="29" t="n">
         <f aca="false">(Funnel!$O$5+Funnel!$O$6+Funnel!$O$7-$F$25-$F$32)*D8+(Funnel!$O$8-$F$26-$F$33)*E8+($F$25+$F$26)*X8+($F$32+$F$33)*Y8</f>
-        <v>53.9970634809098</v>
+        <v>54.5327026287834</v>
       </c>
       <c r="Q8" s="29" t="n">
         <f aca="false">Assumptions!$D$9*MAX(0,MIN(C8+Assumptions!$D$21,Funnel!$B$17)-MAX(IF(A8=1,Funnel!$B$13,B8+Assumptions!$D$21),Funnel!$B$13)+1)/7</f>
@@ -16938,7 +16960,7 @@
       </c>
       <c r="R8" s="30" t="n">
         <f aca="false">IF(Q8&gt;0,P8/Q8,IF(P8&gt;0,9.99,0))</f>
-        <v>0.981764790561996</v>
+        <v>0.991503684159698</v>
       </c>
       <c r="S8" s="2" t="str">
         <f aca="false">IF(P8&gt;Q8+0.5,"OVER "&amp;Assumptions!$D$9&amp;"/wk – pace down",IF(R8&gt;Assumptions!$D$102,"Full",IF(AND(Q8&gt;=Assumptions!$D$103,P8&lt;Assumptions!$D$103),"Under "&amp;Assumptions!$D$103&amp;" – release reserve","")))</f>
@@ -16950,15 +16972,15 @@
       </c>
       <c r="U8" s="32" t="n">
         <f aca="false">$F$38*(G8*(Budget!$G$24-$F$30-$F$37)+IF(A8-ROUNDUP(Funnel!$B$16/7,0)&gt;=1,INDEX($X$4:$X$14,A8-ROUNDUP(Funnel!$B$16/7,0))*$F$30+INDEX($Y$4:$Y$14,A8-ROUNDUP(Funnel!$B$16/7,0))*$F$37,0))</f>
-        <v>2.95742092928641</v>
+        <v>3.37600787400241</v>
       </c>
       <c r="V8" s="32" t="n">
         <f aca="false">T8+U8</f>
-        <v>17.9054816000512</v>
+        <v>18.3240685447672</v>
       </c>
       <c r="W8" s="32" t="n">
         <f aca="false">SUM($V$4:V8)</f>
-        <v>43.1014476895173</v>
+        <v>42.6897043977666</v>
       </c>
       <c r="X8" s="30" t="n">
         <f aca="false">IF(A8=1,Assumptions!$D$50,IF(A8=2,1-Assumptions!$D$50,0))</f>
@@ -16970,7 +16992,11 @@
       </c>
       <c r="Z8" s="30" t="n">
         <f aca="false">Assumptions!$D$57</f>
-        <v>0.19</v>
+        <v>0.215</v>
+      </c>
+      <c r="AA8" s="30" t="n">
+        <f aca="false">D8*IF(MAX(0,MIN(C8,Funnel!$B$19)-B8+1)&gt;0,MAX(0,MIN(C8,Funnel!$B$20)-B8+1)/MAX(0,MIN(C8,Funnel!$B$19)-B8+1),0)</f>
+        <v>0.0307142857142857</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16987,23 +17013,23 @@
       </c>
       <c r="D9" s="30" t="n">
         <f aca="false">IF(SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$19)*$Z$4:$Z$14)&gt;0,IF(B9&lt;=Funnel!$B$19,Z9,0)/SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$19)*$Z$4:$Z$14),0)</f>
-        <v>0.03</v>
+        <v>0.025</v>
       </c>
       <c r="E9" s="30" t="n">
-        <f aca="false">IF(SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14)&gt;0,IF(B9&lt;=Funnel!$B$20,D9,0)/SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14),0)</f>
+        <f aca="false">IF(SUM($AA$4:$AA$14)&gt;0,AA9/SUM($AA$4:$AA$14),0)</f>
         <v>0</v>
       </c>
       <c r="F9" s="30" t="n">
         <f aca="false">IF(A9-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($D$4:$D$14,A9-ROUNDUP(Funnel!$B$15/7,0)),0)</f>
-        <v>0.185</v>
+        <v>0.18</v>
       </c>
       <c r="G9" s="30" t="n">
         <f aca="false">IF(A9-ROUNDUP(Funnel!$B$16/7,0)&gt;=1,INDEX($E$4:$E$14,A9-ROUNDUP(Funnel!$B$16/7,0)),0)</f>
-        <v>0.149484536082474</v>
+        <v>0.183378500451671</v>
       </c>
       <c r="H9" s="41" t="n">
         <f aca="false">$F$19*D9+$F$20*E9+$F$31*Y9</f>
-        <v>1862.81043463839</v>
+        <v>1552.34202886533</v>
       </c>
       <c r="I9" s="41" t="n">
         <f aca="false">IF(A9=1,$F$21,0)</f>
@@ -17011,7 +17037,7 @@
       </c>
       <c r="J9" s="41" t="n">
         <f aca="false">$F$22*F9+$F$23*G9</f>
-        <v>1991.51122847938</v>
+        <v>1979.73596707317</v>
       </c>
       <c r="K9" s="41" t="n">
         <f aca="false">IF(A9=1,Budget!$C$6,0)</f>
@@ -17023,19 +17049,19 @@
       </c>
       <c r="M9" s="41" t="n">
         <f aca="false">SUM(H9:L9)</f>
-        <v>3854.32166311777</v>
+        <v>3532.0779959385</v>
       </c>
       <c r="N9" s="41" t="n">
         <f aca="false">SUM($M$4:M9)</f>
-        <v>96975.520506631</v>
+        <v>96918.4026416982</v>
       </c>
       <c r="O9" s="29" t="n">
         <f aca="false">(Funnel!$M$5+Funnel!$M$6+Funnel!$M$7-$F$27-$F$34)*D9+(Funnel!$M$8-$F$28-$F$35)*E9+($F$27+$F$28)*X9+($F$34+$F$35)*Y9</f>
-        <v>36.7760365287142</v>
+        <v>30.6466971072619</v>
       </c>
       <c r="P9" s="29" t="n">
         <f aca="false">(Funnel!$O$5+Funnel!$O$6+Funnel!$O$7-$F$25-$F$32)*D9+(Funnel!$O$8-$F$26-$F$33)*E9+($F$25+$F$26)*X9+($F$32+$F$33)*Y9</f>
-        <v>7.41444133584382</v>
+        <v>6.17870111320319</v>
       </c>
       <c r="Q9" s="29" t="n">
         <f aca="false">Assumptions!$D$9*MAX(0,MIN(C9+Assumptions!$D$21,Funnel!$B$17)-MAX(IF(A9=1,Funnel!$B$13,B9+Assumptions!$D$21),Funnel!$B$13)+1)/7</f>
@@ -17043,27 +17069,27 @@
       </c>
       <c r="R9" s="30" t="n">
         <f aca="false">IF(Q9&gt;0,P9/Q9,IF(P9&gt;0,9.99,0))</f>
-        <v>0.943656170016487</v>
+        <v>0.786380141680406</v>
       </c>
       <c r="S9" s="2" t="str">
         <f aca="false">IF(P9&gt;Q9+0.5,"OVER "&amp;Assumptions!$D$9&amp;"/wk – pace down",IF(R9&gt;Assumptions!$D$102,"Full",IF(AND(Q9&gt;=Assumptions!$D$103,P9&lt;Assumptions!$D$103),"Under "&amp;Assumptions!$D$103&amp;" – release reserve","")))</f>
-        <v>Full</v>
+        <v/>
       </c>
       <c r="T9" s="32" t="n">
         <f aca="false">$F$38*(F9*(Budget!$G$21+Budget!$G$22+Budget!$G$23-$F$29-$F$36)+IF(A9-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($X$4:$X$14,A9-ROUNDUP(Funnel!$B$15/7,0))*$F$29+INDEX($Y$4:$Y$14,A9-ROUNDUP(Funnel!$B$15/7,0))*$F$36,0))</f>
-        <v>15.8124335446341</v>
+        <v>15.3972684264007</v>
       </c>
       <c r="U9" s="32" t="n">
         <f aca="false">$F$38*(G9*(Budget!$G$24-$F$30-$F$37)+IF(A9-ROUNDUP(Funnel!$B$16/7,0)&gt;=1,INDEX($X$4:$X$14,A9-ROUNDUP(Funnel!$B$16/7,0))*$F$30+INDEX($Y$4:$Y$14,A9-ROUNDUP(Funnel!$B$16/7,0))*$F$37,0))</f>
-        <v>1.9188429513919</v>
+        <v>2.21362762346889</v>
       </c>
       <c r="V9" s="32" t="n">
         <f aca="false">T9+U9</f>
-        <v>17.731276496026</v>
+        <v>17.6108960498696</v>
       </c>
       <c r="W9" s="32" t="n">
         <f aca="false">SUM($V$4:V9)</f>
-        <v>60.8327241855433</v>
+        <v>60.3006004476362</v>
       </c>
       <c r="X9" s="30" t="n">
         <f aca="false">IF(A9=1,Assumptions!$D$50,IF(A9=2,1-Assumptions!$D$50,0))</f>
@@ -17075,7 +17101,11 @@
       </c>
       <c r="Z9" s="30" t="n">
         <f aca="false">Assumptions!$D$58</f>
-        <v>0.03</v>
+        <v>0.025</v>
+      </c>
+      <c r="AA9" s="30" t="n">
+        <f aca="false">D9*IF(MAX(0,MIN(C9,Funnel!$B$19)-B9+1)&gt;0,MAX(0,MIN(C9,Funnel!$B$20)-B9+1)/MAX(0,MIN(C9,Funnel!$B$19)-B9+1),0)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17095,16 +17125,16 @@
         <v>0</v>
       </c>
       <c r="E10" s="30" t="n">
-        <f aca="false">IF(SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14)&gt;0,IF(B10&lt;=Funnel!$B$20,D10,0)/SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14),0)</f>
+        <f aca="false">IF(SUM($AA$4:$AA$14)&gt;0,AA10/SUM($AA$4:$AA$14),0)</f>
         <v>0</v>
       </c>
       <c r="F10" s="30" t="n">
         <f aca="false">IF(A10-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($D$4:$D$14,A10-ROUNDUP(Funnel!$B$15/7,0)),0)</f>
-        <v>0.19</v>
+        <v>0.185</v>
       </c>
       <c r="G10" s="30" t="n">
         <f aca="false">IF(A10-ROUNDUP(Funnel!$B$16/7,0)&gt;=1,INDEX($E$4:$E$14,A10-ROUNDUP(Funnel!$B$16/7,0)),0)</f>
-        <v>0.190721649484536</v>
+        <v>0.227642276422764</v>
       </c>
       <c r="H10" s="41" t="n">
         <f aca="false">$F$19*D10+$F$20*E10+$F$31*Y10</f>
@@ -17116,7 +17146,7 @@
       </c>
       <c r="J10" s="41" t="n">
         <f aca="false">$F$22*F10+$F$23*G10</f>
-        <v>2086.56816262887</v>
+        <v>2078.14791128049</v>
       </c>
       <c r="K10" s="41" t="n">
         <f aca="false">IF(A10=1,Budget!$C$6,0)</f>
@@ -17128,11 +17158,11 @@
       </c>
       <c r="M10" s="41" t="n">
         <f aca="false">SUM(H10:L10)</f>
-        <v>2086.56816262887</v>
+        <v>2078.14791128049</v>
       </c>
       <c r="N10" s="41" t="n">
         <f aca="false">SUM($M$4:M10)</f>
-        <v>99062.0886692598</v>
+        <v>98996.5505529787</v>
       </c>
       <c r="O10" s="29" t="n">
         <f aca="false">(Funnel!$M$5+Funnel!$M$6+Funnel!$M$7-$F$27-$F$34)*D10+(Funnel!$M$8-$F$28-$F$35)*E10+($F$27+$F$28)*X10+($F$34+$F$35)*Y10</f>
@@ -17156,19 +17186,19 @@
       </c>
       <c r="T10" s="32" t="n">
         <f aca="false">$F$38*(F10*(Budget!$G$21+Budget!$G$22+Budget!$G$23-$F$29-$F$36)+IF(A10-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($X$4:$X$14,A10-ROUNDUP(Funnel!$B$15/7,0))*$F$29+INDEX($Y$4:$Y$14,A10-ROUNDUP(Funnel!$B$15/7,0))*$F$36,0))</f>
-        <v>15.7762744928675</v>
+        <v>15.3611093746341</v>
       </c>
       <c r="U10" s="32" t="n">
         <f aca="false">$F$38*(G10*(Budget!$G$24-$F$30-$F$37)+IF(A10-ROUNDUP(Funnel!$B$16/7,0)&gt;=1,INDEX($X$4:$X$14,A10-ROUNDUP(Funnel!$B$16/7,0))*$F$30+INDEX($Y$4:$Y$14,A10-ROUNDUP(Funnel!$B$16/7,0))*$F$37,0))</f>
-        <v>1.71656150314073</v>
+        <v>2.03766985111414</v>
       </c>
       <c r="V10" s="32" t="n">
         <f aca="false">T10+U10</f>
-        <v>17.4928359960082</v>
+        <v>17.3987792257482</v>
       </c>
       <c r="W10" s="32" t="n">
         <f aca="false">SUM($V$4:V10)</f>
-        <v>78.3255601815515</v>
+        <v>77.6993796733844</v>
       </c>
       <c r="X10" s="30" t="n">
         <f aca="false">IF(A10=1,Assumptions!$D$50,IF(A10=2,1-Assumptions!$D$50,0))</f>
@@ -17180,6 +17210,10 @@
       </c>
       <c r="Z10" s="30" t="n">
         <f aca="false">Assumptions!$D$59</f>
+        <v>0</v>
+      </c>
+      <c r="AA10" s="30" t="n">
+        <f aca="false">D10*IF(MAX(0,MIN(C10,Funnel!$B$19)-B10+1)&gt;0,MAX(0,MIN(C10,Funnel!$B$20)-B10+1)/MAX(0,MIN(C10,Funnel!$B$19)-B10+1),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -17200,16 +17234,16 @@
         <v>0</v>
       </c>
       <c r="E11" s="30" t="n">
-        <f aca="false">IF(SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14)&gt;0,IF(B11&lt;=Funnel!$B$20,D11,0)/SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14),0)</f>
+        <f aca="false">IF(SUM($AA$4:$AA$14)&gt;0,AA11/SUM($AA$4:$AA$14),0)</f>
         <v>0</v>
       </c>
       <c r="F11" s="30" t="n">
         <f aca="false">IF(A11-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($D$4:$D$14,A11-ROUNDUP(Funnel!$B$15/7,0)),0)</f>
-        <v>0.19</v>
+        <v>0.215</v>
       </c>
       <c r="G11" s="30" t="n">
         <f aca="false">IF(A11-ROUNDUP(Funnel!$B$16/7,0)&gt;=1,INDEX($E$4:$E$14,A11-ROUNDUP(Funnel!$B$16/7,0)),0)</f>
-        <v>0.195876288659794</v>
+        <v>0.233965672990063</v>
       </c>
       <c r="H11" s="41" t="n">
         <f aca="false">$F$19*D11+$F$20*E11+$F$31*Y11</f>
@@ -17221,7 +17255,7 @@
       </c>
       <c r="J11" s="41" t="n">
         <f aca="false">$F$22*F11+$F$23*G11</f>
-        <v>2092.28200283505</v>
+        <v>2381.23457652439</v>
       </c>
       <c r="K11" s="41" t="n">
         <f aca="false">IF(A11=1,Budget!$C$6,0)</f>
@@ -17233,11 +17267,11 @@
       </c>
       <c r="M11" s="41" t="n">
         <f aca="false">SUM(H11:L11)</f>
-        <v>2092.28200283505</v>
+        <v>2381.23457652439</v>
       </c>
       <c r="N11" s="41" t="n">
         <f aca="false">SUM($M$4:M11)</f>
-        <v>101154.370672095</v>
+        <v>101377.785129503</v>
       </c>
       <c r="O11" s="29" t="n">
         <f aca="false">(Funnel!$M$5+Funnel!$M$6+Funnel!$M$7-$F$27-$F$34)*D11+(Funnel!$M$8-$F$28-$F$35)*E11+($F$27+$F$28)*X11+($F$34+$F$35)*Y11</f>
@@ -17261,19 +17295,19 @@
       </c>
       <c r="T11" s="32" t="n">
         <f aca="false">$F$38*(F11*(Budget!$G$21+Budget!$G$22+Budget!$G$23-$F$29-$F$36)+IF(A11-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($X$4:$X$14,A11-ROUNDUP(Funnel!$B$15/7,0))*$F$29+INDEX($Y$4:$Y$14,A11-ROUNDUP(Funnel!$B$15/7,0))*$F$36,0))</f>
-        <v>15.7762744928675</v>
+        <v>17.8521000840342</v>
       </c>
       <c r="U11" s="32" t="n">
         <f aca="false">$F$38*(G11*(Budget!$G$24-$F$30-$F$37)+IF(A11-ROUNDUP(Funnel!$B$16/7,0)&gt;=1,INDEX($X$4:$X$14,A11-ROUNDUP(Funnel!$B$16/7,0))*$F$30+INDEX($Y$4:$Y$14,A11-ROUNDUP(Funnel!$B$16/7,0))*$F$37,0))</f>
-        <v>1.70358730809048</v>
+        <v>2.0348606447562</v>
       </c>
       <c r="V11" s="32" t="n">
         <f aca="false">T11+U11</f>
-        <v>17.4798618009579</v>
+        <v>19.8869607287904</v>
       </c>
       <c r="W11" s="32" t="n">
         <f aca="false">SUM($V$4:V11)</f>
-        <v>95.8054219825094</v>
+        <v>97.5863404021749</v>
       </c>
       <c r="X11" s="30" t="n">
         <f aca="false">IF(A11=1,Assumptions!$D$50,IF(A11=2,1-Assumptions!$D$50,0))</f>
@@ -17285,6 +17319,10 @@
       </c>
       <c r="Z11" s="30" t="n">
         <f aca="false">Assumptions!$D$60</f>
+        <v>0</v>
+      </c>
+      <c r="AA11" s="30" t="n">
+        <f aca="false">D11*IF(MAX(0,MIN(C11,Funnel!$B$19)-B11+1)&gt;0,MAX(0,MIN(C11,Funnel!$B$20)-B11+1)/MAX(0,MIN(C11,Funnel!$B$19)-B11+1),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -17305,16 +17343,16 @@
         <v>0</v>
       </c>
       <c r="E12" s="30" t="n">
-        <f aca="false">IF(SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14)&gt;0,IF(B12&lt;=Funnel!$B$20,D12,0)/SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14),0)</f>
+        <f aca="false">IF(SUM($AA$4:$AA$14)&gt;0,AA12/SUM($AA$4:$AA$14),0)</f>
         <v>0</v>
       </c>
       <c r="F12" s="30" t="n">
         <f aca="false">IF(A12-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($D$4:$D$14,A12-ROUNDUP(Funnel!$B$15/7,0)),0)</f>
-        <v>0.03</v>
+        <v>0.025</v>
       </c>
       <c r="G12" s="30" t="n">
         <f aca="false">IF(A12-ROUNDUP(Funnel!$B$16/7,0)&gt;=1,INDEX($E$4:$E$14,A12-ROUNDUP(Funnel!$B$16/7,0)),0)</f>
-        <v>0.195876288659794</v>
+        <v>0.038843721770551</v>
       </c>
       <c r="H12" s="41" t="n">
         <f aca="false">$F$19*D12+$F$20*E12+$F$31*Y12</f>
@@ -17326,7 +17364,7 @@
       </c>
       <c r="J12" s="41" t="n">
         <f aca="false">$F$22*F12+$F$23*G12</f>
-        <v>513.203202835052</v>
+        <v>289.788745426829</v>
       </c>
       <c r="K12" s="41" t="n">
         <f aca="false">IF(A12=1,Budget!$C$6,0)</f>
@@ -17338,7 +17376,7 @@
       </c>
       <c r="M12" s="41" t="n">
         <f aca="false">SUM(H12:L12)</f>
-        <v>513.203202835052</v>
+        <v>289.788745426829</v>
       </c>
       <c r="N12" s="41" t="n">
         <f aca="false">SUM($M$4:M12)</f>
@@ -17366,15 +17404,15 @@
       </c>
       <c r="T12" s="32" t="n">
         <f aca="false">$F$38*(F12*(Budget!$G$21+Budget!$G$22+Budget!$G$23-$F$29-$F$36)+IF(A12-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($X$4:$X$14,A12-ROUNDUP(Funnel!$B$15/7,0))*$F$29+INDEX($Y$4:$Y$14,A12-ROUNDUP(Funnel!$B$15/7,0))*$F$36,0))</f>
-        <v>2.49099070940012</v>
+        <v>2.07582559116677</v>
       </c>
       <c r="U12" s="32" t="n">
         <f aca="false">$F$38*(G12*(Budget!$G$24-$F$30-$F$37)+IF(A12-ROUNDUP(Funnel!$B$16/7,0)&gt;=1,INDEX($X$4:$X$14,A12-ROUNDUP(Funnel!$B$16/7,0))*$F$30+INDEX($Y$4:$Y$14,A12-ROUNDUP(Funnel!$B$16/7,0))*$F$37,0))</f>
-        <v>1.70358730809048</v>
+        <v>0.337834006658365</v>
       </c>
       <c r="V12" s="32" t="n">
         <f aca="false">T12+U12</f>
-        <v>4.1945780174906</v>
+        <v>2.41365959782514</v>
       </c>
       <c r="W12" s="32" t="n">
         <f aca="false">SUM($V$4:V12)</f>
@@ -17392,6 +17430,10 @@
         <f aca="false">Assumptions!$D$61</f>
         <v>0</v>
       </c>
+      <c r="AA12" s="30" t="n">
+        <f aca="false">D12*IF(MAX(0,MIN(C12,Funnel!$B$19)-B12+1)&gt;0,MAX(0,MIN(C12,Funnel!$B$20)-B12+1)/MAX(0,MIN(C12,Funnel!$B$19)-B12+1),0)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="29" t="n">
@@ -17410,7 +17452,7 @@
         <v>0</v>
       </c>
       <c r="E13" s="30" t="n">
-        <f aca="false">IF(SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14)&gt;0,IF(B13&lt;=Funnel!$B$20,D13,0)/SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14),0)</f>
+        <f aca="false">IF(SUM($AA$4:$AA$14)&gt;0,AA13/SUM($AA$4:$AA$14),0)</f>
         <v>0</v>
       </c>
       <c r="F13" s="30" t="n">
@@ -17497,6 +17539,10 @@
         <f aca="false">Assumptions!$D$62</f>
         <v>0</v>
       </c>
+      <c r="AA13" s="30" t="n">
+        <f aca="false">D13*IF(MAX(0,MIN(C13,Funnel!$B$19)-B13+1)&gt;0,MAX(0,MIN(C13,Funnel!$B$20)-B13+1)/MAX(0,MIN(C13,Funnel!$B$19)-B13+1),0)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="29" t="n">
@@ -17515,7 +17561,7 @@
         <v>0</v>
       </c>
       <c r="E14" s="30" t="n">
-        <f aca="false">IF(SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14)&gt;0,IF(B14&lt;=Funnel!$B$20,D14,0)/SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$20)*$D$4:$D$14),0)</f>
+        <f aca="false">IF(SUM($AA$4:$AA$14)&gt;0,AA14/SUM($AA$4:$AA$14),0)</f>
         <v>0</v>
       </c>
       <c r="F14" s="30" t="n">
@@ -17602,6 +17648,10 @@
         <f aca="false">Assumptions!$D$63</f>
         <v>0</v>
       </c>
+      <c r="AA14" s="30" t="n">
+        <f aca="false">D14*IF(MAX(0,MIN(C14,Funnel!$B$19)-B14+1)&gt;0,MAX(0,MIN(C14,Funnel!$B$20)-B14+1)/MAX(0,MIN(C14,Funnel!$B$19)-B14+1),0)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="28" t="s">
@@ -17690,7 +17740,7 @@
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="B16" s="9"/>
       <c r="C16" s="9"/>
@@ -17742,12 +17792,12 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="28" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="2" t="s">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="F19" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot",Channels!$B$5:$B$34,"&lt;&gt;I1b Employee referral sprint (bonus on hire)",Channels!$B$5:$B$34,"&lt;&gt;I1a Talent rediscovery (past applicants in ATS)")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
@@ -17756,7 +17806,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="2" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="F20" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot",Channels!$B$5:$B$34,"&lt;&gt;I1b Employee referral sprint (bonus on hire)",Channels!$B$5:$B$34,"&lt;&gt;I1a Talent rediscovery (past applicants in ATS)")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$C$5:$C$34,"Supervisors")</f>
@@ -17765,7 +17815,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="2" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="F21" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$E$5:$E$34,"Slot")</f>
@@ -17774,7 +17824,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="2" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="F22" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,"I1b Employee referral sprint (bonus on hire)",Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
@@ -17783,7 +17833,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="2" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="F23" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,"I1b Employee referral sprint (bonus on hire)",Channels!$C$5:$C$34,"Supervisors")</f>
@@ -17792,7 +17842,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="2" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="F24" s="41" t="n">
         <f aca="false">SUM(Channels!$Z$5:$Z$34)</f>
@@ -17801,7 +17851,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="2" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="F25" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$AF$5:$AF$34,Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
@@ -17810,7 +17860,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="2" t="s">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="F26" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$AF$5:$AF$34,Channels!$C$5:$C$34,"Supervisors")</f>
@@ -17819,7 +17869,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="2" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="F27" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$AE$5:$AE$34,Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
@@ -17828,7 +17878,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="2" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="F28" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$AE$5:$AE$34,Channels!$C$5:$C$34,"Supervisors")</f>
@@ -17837,7 +17887,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="2" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="F29" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$AG$5:$AG$34,Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
@@ -17846,7 +17896,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="2" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="F30" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$AG$5:$AG$34,Channels!$C$5:$C$34,"Supervisors")</f>
@@ -17855,7 +17905,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="2" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="F31" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)")</f>
@@ -17864,7 +17914,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="2" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="F32" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$V$5:$V$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)",Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
@@ -17873,7 +17923,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="2" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="F33" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$V$5:$V$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)",Channels!$C$5:$C$34,"Supervisors")</f>
@@ -17882,7 +17932,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="2" t="s">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="F34" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$W$5:$W$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)",Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
@@ -17891,7 +17941,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="2" t="s">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="F35" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$W$5:$W$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)",Channels!$C$5:$C$34,"Supervisors")</f>
@@ -17900,7 +17950,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="2" t="s">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="F36" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$U$5:$U$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)",Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
@@ -17909,7 +17959,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="2" t="s">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="F37" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$U$5:$U$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)",Channels!$C$5:$C$34,"Supervisors")</f>
@@ -17918,7 +17968,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="2" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="F38" s="30" t="n">
         <f aca="false">IF(Funnel!B23&gt;0,MIN(1,Funnel!B22/Funnel!B23),1)</f>
@@ -17927,7 +17977,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="28" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17936,37 +17986,37 @@
         <v>311</v>
       </c>
       <c r="C43" s="12" t="s">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="D43" s="12" t="s">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="E43" s="12" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="F43" s="12" t="s">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="G43" s="12" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="H43" s="12" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="I43" s="12" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="J43" s="12" t="s">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="K43" s="12" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="L43" s="12" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="M43" s="12" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="N43" s="12" t="s">
         <v>443</v>
@@ -18033,7 +18083,7 @@
       </c>
       <c r="C45" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$4+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"Supervisors"))*$E$4+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45)*$X$4+SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$E$5:$E$34,"Slot")+SUMIFS(Channels!$Y$5:$Y$34,Channels!$B$5:$B$34,$B45)</f>
-        <v>9569.17349428738</v>
+        <v>9247.28220604556</v>
       </c>
       <c r="D45" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$5+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"Supervisors"))*$E$5+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45)*$X$5</f>
@@ -18041,19 +18091,19 @@
       </c>
       <c r="E45" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$6+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"Supervisors"))*$E$6+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45)*$X$6</f>
-        <v>5954.98883247371</v>
+        <v>5794.0431883528</v>
       </c>
       <c r="F45" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$7+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"Supervisors"))*$E$7+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45)*$X$7</f>
-        <v>6115.93447659462</v>
+        <v>5954.98883247371</v>
       </c>
       <c r="G45" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$8+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"Supervisors"))*$E$8+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45)*$X$8</f>
-        <v>6115.93447659462</v>
+        <v>6920.66269719918</v>
       </c>
       <c r="H45" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$9+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"Supervisors"))*$E$9+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45)*$X$9</f>
-        <v>965.673864725467</v>
+        <v>804.728220604556</v>
       </c>
       <c r="I45" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$10+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"Supervisors"))*$E$10+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45)*$X$10</f>
@@ -18141,27 +18191,27 @@
       </c>
       <c r="C47" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$4+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"Supervisors"))*$E$4+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47)*$X$4+SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$E$5:$E$34,"Slot")+SUMIFS(Channels!$Y$5:$Y$34,Channels!$B$5:$B$34,$B47)</f>
-        <v>7362.93228593269</v>
+        <v>7812.07205282721</v>
       </c>
       <c r="D47" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$5+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"Supervisors"))*$E$5+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47)*$X$5</f>
-        <v>4671.63531330861</v>
+        <v>5083.00179063978</v>
       </c>
       <c r="E47" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$6+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"Supervisors"))*$E$6+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47)*$X$6</f>
-        <v>4812.08643422134</v>
+        <v>5192.69187803559</v>
       </c>
       <c r="F47" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$7+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"Supervisors"))*$E$7+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47)*$X$7</f>
-        <v>4942.14282433543</v>
+        <v>5336.93331909214</v>
       </c>
       <c r="G47" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$8+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"Supervisors"))*$E$8+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47)*$X$8</f>
-        <v>4942.14282433543</v>
+        <v>3373.73587072339</v>
       </c>
       <c r="H47" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$9+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"Supervisors"))*$E$9+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47)*$X$9</f>
-        <v>404.971375107729</v>
+        <v>337.476145923107</v>
       </c>
       <c r="I47" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$10+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"Supervisors"))*$E$10+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47)*$X$10</f>
@@ -18369,27 +18419,27 @@
       </c>
       <c r="F51" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B51,Channels!$C$5:$C$34,"&lt;&gt;Supervisors")*$F$7+SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B51,Channels!$C$5:$C$34,"Supervisors")*$G$7</f>
-        <v>2566.00305</v>
+        <v>2467.310625</v>
       </c>
       <c r="G51" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B51,Channels!$C$5:$C$34,"&lt;&gt;Supervisors")*$F$8+SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B51,Channels!$C$5:$C$34,"Supervisors")*$G$8</f>
-        <v>1728.15985322165</v>
+        <v>1781.50967469512</v>
       </c>
       <c r="H51" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B51,Channels!$C$5:$C$34,"&lt;&gt;Supervisors")*$F$9+SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B51,Channels!$C$5:$C$34,"Supervisors")*$G$9</f>
-        <v>1991.51122847938</v>
+        <v>1979.73596707317</v>
       </c>
       <c r="I51" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B51,Channels!$C$5:$C$34,"&lt;&gt;Supervisors")*$F$10+SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B51,Channels!$C$5:$C$34,"Supervisors")*$G$10</f>
-        <v>2086.56816262887</v>
+        <v>2078.14791128049</v>
       </c>
       <c r="J51" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B51,Channels!$C$5:$C$34,"&lt;&gt;Supervisors")*$F$11+SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B51,Channels!$C$5:$C$34,"Supervisors")*$G$11</f>
-        <v>2092.28200283505</v>
+        <v>2381.23457652439</v>
       </c>
       <c r="K51" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B51,Channels!$C$5:$C$34,"&lt;&gt;Supervisors")*$F$12+SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B51,Channels!$C$5:$C$34,"Supervisors")*$G$12</f>
-        <v>513.203202835052</v>
+        <v>289.788745426829</v>
       </c>
       <c r="L51" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B51,Channels!$C$5:$C$34,"&lt;&gt;Supervisors")*$F$13+SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B51,Channels!$C$5:$C$34,"Supervisors")*$G$13</f>
@@ -18411,7 +18461,7 @@
       </c>
       <c r="C52" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$4+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"Supervisors"))*$E$4+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52)*$X$4+SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52,Channels!$E$5:$E$34,"Slot")+SUMIFS(Channels!$Y$5:$Y$34,Channels!$B$5:$B$34,$B52)</f>
-        <v>3777.12</v>
+        <v>3678</v>
       </c>
       <c r="D52" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$5+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"Supervisors"))*$E$5+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52)*$X$5</f>
@@ -18419,19 +18469,19 @@
       </c>
       <c r="E52" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$6+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"Supervisors"))*$E$6+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52)*$X$6</f>
-        <v>1833.72</v>
+        <v>1784.16</v>
       </c>
       <c r="F52" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$7+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"Supervisors"))*$E$7+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52)*$X$7</f>
-        <v>1883.28</v>
+        <v>1833.72</v>
       </c>
       <c r="G52" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$8+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"Supervisors"))*$E$8+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52)*$X$8</f>
-        <v>1883.28</v>
+        <v>2131.08</v>
       </c>
       <c r="H52" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$9+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"Supervisors"))*$E$9+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52)*$X$9</f>
-        <v>297.36</v>
+        <v>247.8</v>
       </c>
       <c r="I52" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$10+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"Supervisors"))*$E$10+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52)*$X$10</f>
@@ -18465,7 +18515,7 @@
       </c>
       <c r="C53" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$4+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"Supervisors"))*$E$4+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53)*$X$4+SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53,Channels!$E$5:$E$34,"Slot")+SUMIFS(Channels!$Y$5:$Y$34,Channels!$B$5:$B$34,$B53)</f>
-        <v>2088.31168831169</v>
+        <v>2023.37662337662</v>
       </c>
       <c r="D53" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$5+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"Supervisors"))*$E$5+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53)*$X$5</f>
@@ -18473,19 +18523,19 @@
       </c>
       <c r="E53" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$6+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"Supervisors"))*$E$6+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53)*$X$6</f>
-        <v>1201.2987012987</v>
+        <v>1168.83116883117</v>
       </c>
       <c r="F53" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$7+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"Supervisors"))*$E$7+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53)*$X$7</f>
-        <v>1233.76623376623</v>
+        <v>1201.2987012987</v>
       </c>
       <c r="G53" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$8+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"Supervisors"))*$E$8+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53)*$X$8</f>
-        <v>1233.76623376623</v>
+        <v>1396.1038961039</v>
       </c>
       <c r="H53" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$9+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"Supervisors"))*$E$9+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53)*$X$9</f>
-        <v>194.805194805195</v>
+        <v>162.337662337662</v>
       </c>
       <c r="I53" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$10+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"Supervisors"))*$E$10+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53)*$X$10</f>
@@ -18518,39 +18568,39 @@
       </c>
       <c r="C54" s="42" t="n">
         <f aca="false">SUM(C44:C53)</f>
-        <v>30431.5174685318</v>
+        <v>30394.7108822494</v>
       </c>
       <c r="D54" s="42" t="n">
         <f aca="false">SUM(D44:D53)</f>
-        <v>16236.2144343735</v>
+        <v>16647.5809117046</v>
       </c>
       <c r="E54" s="42" t="n">
         <f aca="false">SUM(E44:E53)</f>
-        <v>13809.0569679937</v>
+        <v>13946.6892352196</v>
       </c>
       <c r="F54" s="42" t="n">
         <f aca="false">SUM(F44:F53)</f>
-        <v>16741.1265846963</v>
+        <v>16794.2514778646</v>
       </c>
       <c r="G54" s="42" t="n">
         <f aca="false">SUM(G44:G53)</f>
-        <v>15903.2833879179</v>
+        <v>15603.0921387216</v>
       </c>
       <c r="H54" s="42" t="n">
         <f aca="false">SUM(H44:H53)</f>
-        <v>3854.32166311777</v>
+        <v>3532.0779959385</v>
       </c>
       <c r="I54" s="42" t="n">
         <f aca="false">SUM(I44:I53)</f>
-        <v>2086.56816262887</v>
+        <v>2078.14791128049</v>
       </c>
       <c r="J54" s="42" t="n">
         <f aca="false">SUM(J44:J53)</f>
-        <v>2092.28200283505</v>
+        <v>2381.23457652439</v>
       </c>
       <c r="K54" s="42" t="n">
         <f aca="false">SUM(K44:K53)</f>
-        <v>513.203202835052</v>
+        <v>289.788745426829</v>
       </c>
       <c r="L54" s="42" t="n">
         <f aca="false">SUM(L44:L53)</f>
@@ -18604,12 +18654,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>727</v>
+        <v>728</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18623,67 +18673,67 @@
         <v>312</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>730</v>
+        <v>731</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>731</v>
+        <v>732</v>
       </c>
       <c r="G4" s="12" t="s">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="H4" s="12" t="s">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="I4" s="12" t="s">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="J4" s="12" t="s">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="K4" s="12" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="L4" s="12" t="s">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="M4" s="12" t="s">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="N4" s="12" t="s">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="O4" s="12" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="P4" s="12" t="s">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="Q4" s="12" t="s">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="R4" s="12" t="s">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="S4" s="12" t="s">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="T4" s="12" t="s">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="U4" s="12" t="s">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="V4" s="12" t="s">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="W4" s="12" t="s">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="X4" s="12" t="s">
-        <v>749</v>
+        <v>750</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20871,7 +20921,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="28" t="s">
-        <v>750</v>
+        <v>751</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -20880,46 +20930,46 @@
         <v>312</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="D39" s="12" t="s">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="E39" s="12" t="s">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="F39" s="12" t="s">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="G39" s="12" t="s">
-        <v>755</v>
+        <v>756</v>
       </c>
       <c r="H39" s="12" t="s">
-        <v>756</v>
+        <v>757</v>
       </c>
       <c r="I39" s="12" t="s">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="J39" s="12" t="s">
-        <v>758</v>
+        <v>759</v>
       </c>
       <c r="K39" s="12" t="s">
-        <v>759</v>
+        <v>760</v>
       </c>
       <c r="L39" s="12" t="s">
-        <v>760</v>
+        <v>761</v>
       </c>
       <c r="M39" s="12" t="s">
-        <v>761</v>
+        <v>762</v>
       </c>
       <c r="N39" s="12" t="s">
-        <v>762</v>
+        <v>763</v>
       </c>
       <c r="O39" s="12" t="s">
         <v>47</v>
       </c>
       <c r="P39" s="12" t="s">
-        <v>763</v>
+        <v>764</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21149,7 +21199,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="9" t="s">
-        <v>764</v>
+        <v>765</v>
       </c>
       <c r="B46" s="9"/>
       <c r="C46" s="9"/>

</xml_diff>

<commit_message>
Launch assumption labelled as own estimate with its tested downside (~92 hires if assessments start 26 Oct)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V2NJtrYy3bzNxqKeiRXJfY
</commit_message>
<xml_diff>
--- a/operation_uptime/Operation_Uptime_Model.xlsx
+++ b/operation_uptime/Operation_Uptime_Model.xlsx
@@ -221,7 +221,7 @@
     <t xml:space="preserve">Own estimate</t>
   </si>
   <si>
-    <t xml:space="preserve">At launch there is no queue, so the first applicants (and re-applicants) can be assessed within 2 days; the 6-day lag (T2) applies once the queue is full and sets the last useful date.</t>
+    <t xml:space="preserve">Own estimate, not sourced: at launch there is no queue, so the first applicants and re-applicants are assessed within 2 days (published review times are 5–10 days once a queue exists; T2 = 6 sets the cut-off). If first assessments slip to 26 Oct, hires fall to ~92 (model run); 100 would then need 60 a week.</t>
   </si>
   <si>
     <t xml:space="preserve">T1</t>
@@ -3478,7 +3478,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
         <v>60</v>
       </c>

</xml_diff>

<commit_message>
Score-driven fixes: 40% Polish cap enforced in budget scenarios, zero-qualified rule needs 30+ applications, signed hires by source in Tracker, slide 4 spend and cost per qualified, downsides on slides 3 and 7, source-note wording
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V2NJtrYy3bzNxqKeiRXJfY
</commit_message>
<xml_diff>
--- a/operation_uptime/Operation_Uptime_Model.xlsx
+++ b/operation_uptime/Operation_Uptime_Model.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1464" uniqueCount="766">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1467" uniqueCount="769">
   <si>
     <t xml:space="preserve">Operation Uptime — model summary (hypothetical Tesla Giga Berlin maintenance hiring)</t>
   </si>
@@ -221,7 +221,7 @@
     <t xml:space="preserve">Own estimate</t>
   </si>
   <si>
-    <t xml:space="preserve">Own estimate, not sourced: at launch there is no queue, so the first applicants and re-applicants are assessed within 2 days (published review times are 5–10 days once a queue exists; T2 = 6 sets the cut-off). If first assessments slip to 26 Oct, hires fall to ~92 (model run); 100 would then need 60 a week.</t>
+    <t xml:space="preserve">Own estimate, not sourced: at launch there is no queue, so the first applicants and re-applicants are assessed within 2 days (SmartRecruiters' 6-day median review, T2, applies once a queue exists and sets the cut-off). If first assessments slip to 26 Oct, hires fall to ~92 (model run); 100 would then need 60 a week.</t>
   </si>
   <si>
     <t xml:space="preserve">T1</t>
@@ -230,18 +230,18 @@
     <t xml:space="preserve">Last realistic contract-signing date</t>
   </si>
   <si>
+    <t xml:space="preserve">My choice: the last Friday before Christmas. Indeed job searches fall to 45% below the 1–15 Dec average over the holidays (Indeed Hiring Lab). https://hiringlab.indeed.com/de/blog/2025/02/17/der-stellenmarkt-startet-unausgewogen-in-das-neue-jahr/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Days: application → recruiter assessment of a qualified applicant</t>
+  </si>
+  <si>
     <t xml:space="preserve">Researched</t>
   </si>
   <si>
-    <t xml:space="preserve">Last Friday before Christmas; job searches hit a low ~45% below normal over the holidays (Indeed Hiring Lab). https://hiringlab.indeed.com/de/blog/2025/02/17/der-stellenmarkt-startet-unausgewogen-in-das-neue-jahr/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Days: application → recruiter assessment of a qualified applicant</t>
-  </si>
-  <si>
     <t xml:space="preserve">Global median: 6 days to review an application (SmartRecruiters 2025, Germany edition; German processes run longer, so this assumes the client keeps pace). https://ta.smartrecruiters.com/rs/664-NIC-529/images/Germany%20Recruiting%20Benchmarks%202025%20Report%20DE.pdf</t>
   </si>
   <si>
@@ -509,25 +509,25 @@
     <t xml:space="preserve">people</t>
   </si>
   <si>
-    <t xml:space="preserve">BA employment, KldB 2625 + 2622: Berlin 2,708 + 60% of Brandenburg 3,417 (75 km radius, own scaling) ≈ 4,800. Berlin file: https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-11-0-202512-xlsx.xlsx?__blob=publicationFile https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-12-0-202512-xlsx.xlsx?__blob=publicationFile</t>
+    <t xml:space="preserve">BA employment, KldB 2625 + 2622: Berlin 2,708 + 60% of Brandenburg 3,417 (own scaling: ~60% of Brandenburg lies within 75 km) ≈ 4,800. Berlin file: https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-11-0-202512-xlsx.xlsx?__blob=publicationFile https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-12-0-202512-xlsx.xlsx?__blob=publicationFile</t>
   </si>
   <si>
     <t xml:space="preserve">PSM</t>
   </si>
   <si>
-    <t xml:space="preserve">BA employment, KldB 2611 + 2510/2511/2513 (skilled level): Berlin 17,490 + 60% of Brandenburg 14,878 (75 km radius, own scaling) ≈ 26,400. Berlin file: https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-11-0-202512-xlsx.xlsx?__blob=publicationFile https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-12-0-202512-xlsx.xlsx?__blob=publicationFile</t>
+    <t xml:space="preserve">BA employment, KldB 2611 + 2510/2511/2513 (skilled level): Berlin 17,490 + 60% of Brandenburg 14,878 (own scaling: ~60% of Brandenburg lies within 75 km) ≈ 26,400. Berlin file: https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-11-0-202512-xlsx.xlsx?__blob=publicationFile https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-12-0-202512-xlsx.xlsx?__blob=publicationFile</t>
   </si>
   <si>
     <t xml:space="preserve">PSA</t>
   </si>
   <si>
-    <t xml:space="preserve">BA employment, KldB 2612: Berlin 1,254 + 60% of Brandenburg 1,206 (75 km radius, own scaling) ≈ 2,000. Berlin file: https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-11-0-202512-xlsx.xlsx?__blob=publicationFile https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-12-0-202512-xlsx.xlsx?__blob=publicationFile</t>
+    <t xml:space="preserve">BA employment, KldB 2612: Berlin 1,254 + 60% of Brandenburg 1,206 (own scaling: ~60% of Brandenburg lies within 75 km) ≈ 2,000. Berlin file: https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-11-0-202512-xlsx.xlsx?__blob=publicationFile https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-12-0-202512-xlsx.xlsx?__blob=publicationFile</t>
   </si>
   <si>
     <t xml:space="preserve">PSS</t>
   </si>
   <si>
-    <t xml:space="preserve">BA employment, supervisor codes 2519 + 2619 + 2629 + 2639: Berlin 1,494 + 60% of Brandenburg 1,209 (75 km radius, own scaling) ≈ 2,200. Berlin file: https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-11-0-202512-xlsx.xlsx?__blob=publicationFile https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-12-0-202512-xlsx.xlsx?__blob=publicationFile</t>
+    <t xml:space="preserve">BA employment, supervisor codes 2519 + 2619 + 2629 + 2639: Berlin 1,494 + 60% of Brandenburg 1,209 (own scaling: ~60% of Brandenburg lies within 75 km) ≈ 2,200. Berlin file: https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-11-0-202512-xlsx.xlsx?__blob=publicationFile https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-12-0-202512-xlsx.xlsx?__blob=publicationFile</t>
   </si>
   <si>
     <t xml:space="preserve">PIE</t>
@@ -623,7 +623,7 @@
     <t xml:space="preserve">R6</t>
   </si>
   <si>
-    <t xml:space="preserve">…or switch off when spend reaches this with zero qualified</t>
+    <t xml:space="preserve">…or switch off when spend reaches this and R2 applications brought zero qualified</t>
   </si>
   <si>
     <t xml:space="preserve">Test fully spent with zero qualified → switch off.</t>
@@ -800,7 +800,7 @@
     <t xml:space="preserve">×</t>
   </si>
   <si>
-    <t xml:space="preserve">Derived from IAB 2025: decisive ÷ used for job boards (21% ÷ 57%), relative to the average channel (0.41). https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/</t>
+    <t xml:space="preserve">Derived from IAB 2025: decisive ÷ used for job boards (21% ÷ 57% = 0.37) ÷ 0.41 = 0.90. Average = mean of decisive ÷ used over the three channels IAB reports (homepage 20/70, job boards 21/57, personal contacts 27/48) = 0.41. https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/</t>
   </si>
   <si>
     <t xml:space="preserve">CXH</t>
@@ -809,7 +809,7 @@
     <t xml:space="preserve">Channel quality index: own careers page (organic, Google Search ads)</t>
   </si>
   <si>
-    <t xml:space="preserve">Derived from IAB 2025: decisive ÷ used for the employer homepage (20% ÷ 70%), relative to the average channel (0.41). https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/</t>
+    <t xml:space="preserve">Derived from IAB 2025: decisive ÷ used for the employer homepage (20% ÷ 70% = 0.29) ÷ 0.41 = 0.70. Average = mean of decisive ÷ used over the three channels IAB reports (homepage 20/70, job boards 21/57, personal contacts 27/48) = 0.41. https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/</t>
   </si>
   <si>
     <t xml:space="preserve">CXS</t>
@@ -938,7 +938,7 @@
     <t xml:space="preserve">Maintenance trades as share of production occupations</t>
   </si>
   <si>
-    <t xml:space="preserve">BA employment: maintenance codes 2513 + 2625 + 2611 + 2612 + supervisors (536,520) ÷ production occupations 21–29 (6,850,263) = 7.8%. https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-d-0-202512-xlsx.xlsx?__blob=publicationFile</t>
+    <t xml:space="preserve">BA employment, Germany: maintenance codes 2513 + 2625 + 2611 + 2612 + supervisors 2519 + 2619 + 2629 (536,520) ÷ production occupations 21–29 (6,850,263) = 7.8%. https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-d-0-202512-xlsx.xlsx?__blob=publicationFile</t>
   </si>
   <si>
     <t xml:space="preserve">TURN</t>
@@ -1019,7 +1019,7 @@
     <t xml:space="preserve">CPA</t>
   </si>
   <si>
-    <t xml:space="preserve">Indeed's DACH median is €161 per application (TalentBait, 2,549 campaigns), used as the programmatic proxy. Volume capped by Indeed's reach. https://www.talentbait.de/recruiting-kanaele-uebersicht/</t>
+    <t xml:space="preserve">Indeed's CPA median is €161 in TalentBait's DACH 2024–26 dataset (2,549 channel-campaigns across all channels), used as the programmatic proxy. Volume capped by Indeed's reach. https://www.talentbait.de/recruiting-kanaele-uebersicht/</t>
   </si>
   <si>
     <t xml:space="preserve">C06</t>
@@ -1070,7 +1070,7 @@
     <t xml:space="preserve">Meta social (FB/IG lead ads, 75 km geo)</t>
   </si>
   <si>
-    <t xml:space="preserve">TalentBait's trades example: ~€84 per application for social ads; volume from Redline campaign data. https://www.talentbait.de/social-media-recruiting</t>
+    <t xml:space="preserve">Own estimate: TalentBait's example ad shows ~€84 per application for trades (its measured averages: €52 raw, €104 per qualified); volume from Redline campaign data. https://www.talentbait.de/social-media-recruiting</t>
   </si>
   <si>
     <t xml:space="preserve">C16</t>
@@ -1169,7 +1169,7 @@
     <t xml:space="preserve">I1: messaging cost per contacted past applicant (email + SMS tool)</t>
   </si>
   <si>
-    <t xml:space="preserve">Three text messages at ~€0.075 each (seven.io) plus email, rounded up to €0.30. https://www.seven.io/en/prices/</t>
+    <t xml:space="preserve">Three text messages at ~€0.075 each (seven.io price list, 2016 rates) plus email, rounded up to €0.30. https://www.seven.io/en/prices/</t>
   </si>
   <si>
     <t xml:space="preserve">I1B</t>
@@ -1196,7 +1196,7 @@
     <t xml:space="preserve">I2: construction/Handwerk electricians (Elektroniker Energie- und Gebäudetechnik) within 75 km</t>
   </si>
   <si>
-    <t xml:space="preserve">BA employment, KldB 2621 Bauelektrik: Berlin 6,204 + 60% of Brandenburg 5,905 (75 km radius, own scaling) ≈ 10,000. Berlin file: https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-11-0-202512-xlsx.xlsx?__blob=publicationFile https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-12-0-202512-xlsx.xlsx?__blob=publicationFile</t>
+    <t xml:space="preserve">BA employment, KldB 2621 Bauelektrik: Berlin 6,204 + 60% of Brandenburg 5,905 (own scaling: ~60% of Brandenburg lies within 75 km) ≈ 10,000. Berlin file: https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-11-0-202512-xlsx.xlsx?__blob=publicationFile https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-12-0-202512-xlsx.xlsx?__blob=publicationFile</t>
   </si>
   <si>
     <t xml:space="preserve">I2S</t>
@@ -1214,7 +1214,7 @@
     <t xml:space="preserve">I2: cost per application (Meta/Google + 6-question quiz funnel)</t>
   </si>
   <si>
-    <t xml:space="preserve">TalentBait's trades example shows ~€84 per application for social ads. https://www.talentbait.de/social-media-recruiting</t>
+    <t xml:space="preserve">Own estimate: TalentBait's example ad shows ~€84 per application for trades; its measured averages are €52 per raw application and €104 per qualified one. https://www.talentbait.de/social-media-recruiting</t>
   </si>
   <si>
     <t xml:space="preserve">I2Q</t>
@@ -1259,7 +1259,7 @@
     <t xml:space="preserve">I3: share qualified after Polish-language pre-screen call</t>
   </si>
   <si>
-    <t xml:space="preserve">Eurostat AES 2022, Poland, vocational upper-secondary: 58.7% know a foreign language × 23.6% of them good or proficient ≈ 14%. https://ec.europa.eu/eurostat/databrowser/view/edat_aes_l33/default/table</t>
+    <t xml:space="preserve">Eurostat AES 2022, Poland, ages 25–64, vocational upper-secondary: 58.7% know a foreign language (edat_aes_l23: 100 − 41.3%) × 23.6% of them good or proficient (edat_aes_l33) ≈ 14%. https://ec.europa.eu/eurostat/databrowser/view/edat_aes_l23/default/table https://ec.europa.eu/eurostat/databrowser/view/edat_aes_l33/default/table</t>
   </si>
   <si>
     <t xml:space="preserve">I3X</t>
@@ -2280,6 +2280,15 @@
   </si>
   <si>
     <t xml:space="preserve">Decision</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Signed to date (ATS source tag)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cost per hire to date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plan hires</t>
   </si>
   <si>
     <t xml:space="preserve">Role-level funnel actuals (cumulative) → re-forecast hires</t>
@@ -3000,7 +3009,7 @@
       </c>
       <c r="C5" s="4" t="n">
         <f aca="false">Budget!C12</f>
-        <v>120000</v>
+        <v>122500</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3009,7 +3018,7 @@
       </c>
       <c r="C6" s="4" t="n">
         <f aca="false">Budget!C9</f>
-        <v>101667.57387493</v>
+        <v>102255.847555873</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3018,7 +3027,7 @@
       </c>
       <c r="C7" s="4" t="n">
         <f aca="false">Budget!C12-Budget!C9</f>
-        <v>18332.4261250701</v>
+        <v>20244.1524441265</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3046,7 +3055,7 @@
       </c>
       <c r="C10" s="4" t="n">
         <f aca="false">Budget!C14</f>
-        <v>1016.6757387493</v>
+        <v>1022.55847555873</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3118,7 +3127,7 @@
       </c>
       <c r="C18" s="5" t="n">
         <f aca="false">Budget!H46</f>
-        <v>86.977613550255</v>
+        <v>87.0578063312124</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3518,18 +3527,18 @@
         <v>32</v>
       </c>
       <c r="F20" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="G20" s="17" t="s">
         <v>67</v>
-      </c>
-      <c r="G20" s="17" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B21" s="13" t="s">
         <v>69</v>
-      </c>
-      <c r="B21" s="13" t="s">
-        <v>70</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>31</v>
@@ -3541,7 +3550,7 @@
         <v>62</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="G21" s="17" t="s">
         <v>71</v>
@@ -3564,7 +3573,7 @@
         <v>62</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="G22" s="17" t="s">
         <v>74</v>
@@ -3690,7 +3699,7 @@
         <v>44</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="G29" s="17" t="s">
         <v>87</v>
@@ -3713,7 +3722,7 @@
         <v>44</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="G30" s="17" t="s">
         <v>87</v>
@@ -3736,7 +3745,7 @@
         <v>44</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="G31" s="17" t="s">
         <v>87</v>
@@ -3759,7 +3768,7 @@
         <v>44</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="G32" s="17" t="s">
         <v>87</v>
@@ -4517,7 +4526,7 @@
         <v>159</v>
       </c>
       <c r="F68" s="2" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="G68" s="17" t="s">
         <v>160</v>
@@ -4540,7 +4549,7 @@
         <v>159</v>
       </c>
       <c r="F69" s="2" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="G69" s="17" t="s">
         <v>162</v>
@@ -4563,7 +4572,7 @@
         <v>159</v>
       </c>
       <c r="F70" s="2" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="G70" s="17" t="s">
         <v>164</v>
@@ -4586,7 +4595,7 @@
         <v>159</v>
       </c>
       <c r="F71" s="2" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="G71" s="17" t="s">
         <v>166</v>
@@ -4609,7 +4618,7 @@
         <v>44</v>
       </c>
       <c r="F72" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="G72" s="17" t="s">
         <v>169</v>
@@ -4632,7 +4641,7 @@
         <v>44</v>
       </c>
       <c r="F73" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="G73" s="17" t="s">
         <v>169</v>
@@ -4655,7 +4664,7 @@
         <v>44</v>
       </c>
       <c r="F74" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="G74" s="17" t="s">
         <v>169</v>
@@ -4678,7 +4687,7 @@
         <v>44</v>
       </c>
       <c r="F75" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="G75" s="17" t="s">
         <v>169</v>
@@ -4919,7 +4928,7 @@
         <v>189</v>
       </c>
       <c r="F87" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="G87" s="17" t="s">
         <v>196</v>
@@ -5057,7 +5066,7 @@
         <v>44</v>
       </c>
       <c r="F93" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="G93" s="17" t="s">
         <v>216</v>
@@ -5080,7 +5089,7 @@
         <v>44</v>
       </c>
       <c r="F94" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="G94" s="17" t="s">
         <v>216</v>
@@ -5103,7 +5112,7 @@
         <v>44</v>
       </c>
       <c r="F95" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="G95" s="17" t="s">
         <v>216</v>
@@ -5241,7 +5250,7 @@
         <v>44</v>
       </c>
       <c r="F101" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="G101" s="17" t="s">
         <v>243</v>
@@ -5264,7 +5273,7 @@
         <v>44</v>
       </c>
       <c r="F102" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="G102" s="17" t="s">
         <v>247</v>
@@ -5344,7 +5353,7 @@
         <v>256</v>
       </c>
       <c r="F108" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="G108" s="17" t="s">
         <v>257</v>
@@ -5361,13 +5370,13 @@
         <v>255</v>
       </c>
       <c r="D109" s="20" t="n">
-        <v>0.71</v>
+        <v>0.7</v>
       </c>
       <c r="E109" s="2" t="s">
         <v>256</v>
       </c>
       <c r="F109" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="G109" s="17" t="s">
         <v>260</v>
@@ -5390,7 +5399,7 @@
         <v>256</v>
       </c>
       <c r="F110" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="G110" s="17" t="s">
         <v>263</v>
@@ -5413,7 +5422,7 @@
         <v>44</v>
       </c>
       <c r="F111" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="G111" s="17" t="s">
         <v>266</v>
@@ -5436,7 +5445,7 @@
         <v>44</v>
       </c>
       <c r="F112" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="G112" s="17" t="s">
         <v>269</v>
@@ -5459,7 +5468,7 @@
         <v>44</v>
       </c>
       <c r="F113" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="G113" s="17" t="s">
         <v>272</v>
@@ -5482,7 +5491,7 @@
         <v>186</v>
       </c>
       <c r="F114" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="G114" s="17" t="s">
         <v>276</v>
@@ -5505,7 +5514,7 @@
         <v>44</v>
       </c>
       <c r="F115" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="G115" s="17" t="s">
         <v>279</v>
@@ -5528,7 +5537,7 @@
         <v>283</v>
       </c>
       <c r="F116" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="G116" s="17" t="s">
         <v>284</v>
@@ -5551,7 +5560,7 @@
         <v>283</v>
       </c>
       <c r="F117" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="G117" s="17" t="s">
         <v>288</v>
@@ -5574,7 +5583,7 @@
         <v>283</v>
       </c>
       <c r="F118" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="G118" s="17" t="s">
         <v>292</v>
@@ -5597,7 +5606,7 @@
         <v>62</v>
       </c>
       <c r="F119" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="G119" s="17" t="s">
         <v>296</v>
@@ -5620,7 +5629,7 @@
         <v>159</v>
       </c>
       <c r="F120" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="G120" s="17" t="s">
         <v>300</v>
@@ -5643,7 +5652,7 @@
         <v>44</v>
       </c>
       <c r="F121" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="G121" s="17" t="s">
         <v>303</v>
@@ -5666,7 +5675,7 @@
         <v>44</v>
       </c>
       <c r="F122" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="G122" s="17" t="s">
         <v>306</v>
@@ -5689,7 +5698,7 @@
         <v>44</v>
       </c>
       <c r="F123" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="G123" s="17" t="s">
         <v>309</v>
@@ -5768,7 +5777,7 @@
       <c r="F127" s="24"/>
       <c r="G127" s="25" t="n">
         <f aca="false">Assumptions!$D$29*Assumptions!$D$109</f>
-        <v>0.1775</v>
+        <v>0.175</v>
       </c>
       <c r="H127" s="26" t="n">
         <f aca="false">ROUND(Assumptions!$D$11*Assumptions!$D$114*Assumptions!$D$115,0)</f>
@@ -5781,7 +5790,7 @@
         <v>0</v>
       </c>
       <c r="K127" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="L127" s="17" t="s">
         <v>323</v>
@@ -5806,7 +5815,7 @@
       <c r="F128" s="24"/>
       <c r="G128" s="25" t="n">
         <f aca="false">Assumptions!$D$30*Assumptions!$D$109</f>
-        <v>0.1775</v>
+        <v>0.175</v>
       </c>
       <c r="H128" s="26" t="n">
         <f aca="false">ROUND(Assumptions!$D$12*Assumptions!$D$114*Assumptions!$D$115,0)</f>
@@ -5819,7 +5828,7 @@
         <v>0</v>
       </c>
       <c r="K128" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="L128" s="17" t="s">
         <v>323</v>
@@ -5844,7 +5853,7 @@
       <c r="F129" s="24"/>
       <c r="G129" s="25" t="n">
         <f aca="false">Assumptions!$D$31*Assumptions!$D$109</f>
-        <v>0.1775</v>
+        <v>0.175</v>
       </c>
       <c r="H129" s="26" t="n">
         <f aca="false">ROUND(Assumptions!$D$13*Assumptions!$D$114*Assumptions!$D$115,0)</f>
@@ -5857,7 +5866,7 @@
         <v>0</v>
       </c>
       <c r="K129" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="L129" s="17" t="s">
         <v>323</v>
@@ -5882,7 +5891,7 @@
       <c r="F130" s="24"/>
       <c r="G130" s="25" t="n">
         <f aca="false">Assumptions!$D$32*Assumptions!$D$109</f>
-        <v>0.1633</v>
+        <v>0.161</v>
       </c>
       <c r="H130" s="26" t="n">
         <f aca="false">ROUND(Assumptions!$D$14*Assumptions!$D$114*Assumptions!$D$115,0)</f>
@@ -5895,7 +5904,7 @@
         <v>0</v>
       </c>
       <c r="K130" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="L130" s="17" t="s">
         <v>323</v>
@@ -5933,7 +5942,7 @@
         <v>0</v>
       </c>
       <c r="K131" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="L131" s="17" t="s">
         <v>330</v>
@@ -5971,7 +5980,7 @@
         <v>0</v>
       </c>
       <c r="K132" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="L132" s="17" t="s">
         <v>330</v>
@@ -6009,7 +6018,7 @@
         <v>0</v>
       </c>
       <c r="K133" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="L133" s="17" t="s">
         <v>330</v>
@@ -6047,7 +6056,7 @@
         <v>0</v>
       </c>
       <c r="K134" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="L134" s="17" t="s">
         <v>330</v>
@@ -6087,7 +6096,7 @@
         <v>0</v>
       </c>
       <c r="K135" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="L135" s="17" t="s">
         <v>337</v>
@@ -6127,7 +6136,7 @@
         <v>0</v>
       </c>
       <c r="K136" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="L136" s="17" t="s">
         <v>337</v>
@@ -6167,7 +6176,7 @@
         <v>0</v>
       </c>
       <c r="K137" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="L137" s="17" t="s">
         <v>337</v>
@@ -6207,7 +6216,7 @@
         <v>0</v>
       </c>
       <c r="K138" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="L138" s="17" t="s">
         <v>337</v>
@@ -6245,7 +6254,7 @@
         <v>0</v>
       </c>
       <c r="K139" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="L139" s="17" t="s">
         <v>343</v>
@@ -6283,7 +6292,7 @@
         <v>0</v>
       </c>
       <c r="K140" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="L140" s="17" t="s">
         <v>343</v>
@@ -6321,7 +6330,7 @@
         <v>0</v>
       </c>
       <c r="K141" s="2" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="L141" s="17" t="s">
         <v>347</v>
@@ -6359,7 +6368,7 @@
         <v>0</v>
       </c>
       <c r="K142" s="2" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="L142" s="17" t="s">
         <v>347</v>
@@ -6384,7 +6393,7 @@
       <c r="F143" s="24"/>
       <c r="G143" s="25" t="n">
         <f aca="false">Assumptions!$D$29*Assumptions!$D$109</f>
-        <v>0.1775</v>
+        <v>0.175</v>
       </c>
       <c r="H143" s="26" t="n">
         <f aca="false">IF(G143&gt;0,ROUND((Assumptions!$D$68*Assumptions!$D$72+Assumptions!$D$76)*Assumptions!$D$113/G143,-1),0)</f>
@@ -6397,7 +6406,7 @@
         <v>0</v>
       </c>
       <c r="K143" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="L143" s="17" t="s">
         <v>351</v>
@@ -6422,11 +6431,11 @@
       <c r="F144" s="24"/>
       <c r="G144" s="25" t="n">
         <f aca="false">Assumptions!$D$30*Assumptions!$D$109</f>
-        <v>0.1775</v>
+        <v>0.175</v>
       </c>
       <c r="H144" s="26" t="n">
         <f aca="false">IF(G144&gt;0,ROUND((Assumptions!$D$69*Assumptions!$D$73+Assumptions!$D$77)*Assumptions!$D$113/G144,-1),0)</f>
-        <v>1730</v>
+        <v>1760</v>
       </c>
       <c r="I144" s="20" t="n">
         <v>1</v>
@@ -6435,7 +6444,7 @@
         <v>0</v>
       </c>
       <c r="K144" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="L144" s="17" t="s">
         <v>351</v>
@@ -6460,7 +6469,7 @@
       <c r="F145" s="24"/>
       <c r="G145" s="25" t="n">
         <f aca="false">Assumptions!$D$31*Assumptions!$D$109</f>
-        <v>0.1775</v>
+        <v>0.175</v>
       </c>
       <c r="H145" s="26" t="n">
         <f aca="false">IF(G145&gt;0,ROUND((Assumptions!$D$70*Assumptions!$D$74+Assumptions!$D$78)*Assumptions!$D$113/G145,-1),0)</f>
@@ -6473,7 +6482,7 @@
         <v>0</v>
       </c>
       <c r="K145" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="L145" s="17" t="s">
         <v>351</v>
@@ -6498,7 +6507,7 @@
       <c r="F146" s="24"/>
       <c r="G146" s="25" t="n">
         <f aca="false">Assumptions!$D$32*Assumptions!$D$109</f>
-        <v>0.1633</v>
+        <v>0.161</v>
       </c>
       <c r="H146" s="26" t="n">
         <f aca="false">IF(G146&gt;0,ROUND((Assumptions!$D$71*Assumptions!$D$75+Assumptions!$D$79)*Assumptions!$D$113/G146,-1),0)</f>
@@ -6511,7 +6520,7 @@
         <v>0</v>
       </c>
       <c r="K146" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="L146" s="17" t="s">
         <v>351</v>
@@ -6852,7 +6861,7 @@
         <v>119</v>
       </c>
       <c r="F162" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="G162" s="17" t="s">
         <v>383</v>
@@ -6945,7 +6954,7 @@
         <v>119</v>
       </c>
       <c r="F166" s="2" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="G166" s="17" t="s">
         <v>395</v>
@@ -7061,7 +7070,7 @@
         <v>44</v>
       </c>
       <c r="F171" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="G171" s="17" t="s">
         <v>410</v>
@@ -7131,7 +7140,7 @@
         <v>419</v>
       </c>
       <c r="F174" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="G174" s="17" t="s">
         <v>420</v>
@@ -7154,7 +7163,7 @@
         <v>119</v>
       </c>
       <c r="F175" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="G175" s="17" t="s">
         <v>423</v>
@@ -7209,7 +7218,7 @@
   <hyperlinks>
     <hyperlink ref="G10" r:id="rId1" display="From the brief. Polish hires need no work permit (EU free movement) and are insured and taxed in Germany. https://www.make-it-in-germany.com/en/working-in-germany/information-eu-citizens/print"/>
     <hyperlink ref="G15" r:id="rId2" display="From the brief, so I plan no foreign-trained electricians. Worth raising: for employees the trade is not legally regulated, which could open this route. https://www.anerkennung-in-deutschland.de/en/interest/finder/profession/62/profile"/>
-    <hyperlink ref="G20" r:id="rId3" display="Last Friday before Christmas; job searches hit a low ~45% below normal over the holidays (Indeed Hiring Lab). https://hiringlab.indeed.com/de/blog/2025/02/17/der-stellenmarkt-startet-unausgewogen-in-das-neue-jahr/"/>
+    <hyperlink ref="G20" r:id="rId3" display="My choice: the last Friday before Christmas. Indeed job searches fall to 45% below the 1–15 Dec average over the holidays (Indeed Hiring Lab). https://hiringlab.indeed.com/de/blog/2025/02/17/der-stellenmarkt-startet-unausgewogen-in-das-neue-jahr/"/>
     <hyperlink ref="G21" r:id="rId4" display="Global median: 6 days to review an application (SmartRecruiters 2025, Germany edition; German processes run longer, so this assumes the client keeps pace). https://ta.smartrecruiters.com/rs/664-NIC-529/images/Germany%20Recruiting%20Benchmarks%202025%20Report%20DE.pdf"/>
     <hyperlink ref="G22" r:id="rId5" display="Global median: 14 days from application to interview, minus the 6 above (SmartRecruiters 2025, Germany edition). https://ta.smartrecruiters.com/rs/664-NIC-529/images/Germany%20Recruiting%20Benchmarks%202025%20Report%20DE.pdf"/>
     <hyperlink ref="G24" r:id="rId6" display="One-week offer validity; candidates take ~9 days on average to decide (NACE 2025). https://www.naceweb.org/talent-acquisition/trends-and-predictions/employers-make-more-offers-as-student-acceptance-rate-rises-response-time-shortens"/>
@@ -7226,10 +7235,10 @@
     <hyperlink ref="G43" r:id="rId17" display="Königsteiner 2022: 47% accepted vs 14% declined after an offer → ~77% acceptance. I use 70–75%: shift work and competing offers. https://www.lebensmittelzeitung.net/handel/karriere/rekrutierung-bewerber-sagen-haeufiger-ab-166449"/>
     <hyperlink ref="G44" r:id="rId18" display="Königsteiner 2022: 47% accepted vs 14% declined after an offer → ~77% acceptance. I use 70–75%: shift work and competing offers. https://www.lebensmittelzeitung.net/handel/karriere/rekrutierung-bewerber-sagen-haeufiger-ab-166449"/>
     <hyperlink ref="G48" r:id="rId19" display="15% buffer, in the 10–20% range used for risky projects; released only on results. https://mastt.com/blogs/construction-contingency"/>
-    <hyperlink ref="G68" r:id="rId20" display="BA employment, KldB 2625 + 2622: Berlin 2,708 + 60% of Brandenburg 3,417 (75 km radius, own scaling) ≈ 4,800. Berlin file: https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-11-0-202512-xlsx.xlsx?__blob=publicationFile https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-12-0-202512-xlsx.xlsx?__blob=publicationFile"/>
-    <hyperlink ref="G69" r:id="rId21" display="BA employment, KldB 2611 + 2510/2511/2513 (skilled level): Berlin 17,490 + 60% of Brandenburg 14,878 (75 km radius, own scaling) ≈ 26,400. Berlin file: https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-11-0-202512-xlsx.xlsx?__blob=publicationFile https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-12-0-202512-xlsx.xlsx?__blob=publicationFile"/>
-    <hyperlink ref="G70" r:id="rId22" display="BA employment, KldB 2612: Berlin 1,254 + 60% of Brandenburg 1,206 (75 km radius, own scaling) ≈ 2,000. Berlin file: https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-11-0-202512-xlsx.xlsx?__blob=publicationFile https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-12-0-202512-xlsx.xlsx?__blob=publicationFile"/>
-    <hyperlink ref="G71" r:id="rId23" display="BA employment, supervisor codes 2519 + 2619 + 2629 + 2639: Berlin 1,494 + 60% of Brandenburg 1,209 (75 km radius, own scaling) ≈ 2,200. Berlin file: https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-11-0-202512-xlsx.xlsx?__blob=publicationFile https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-12-0-202512-xlsx.xlsx?__blob=publicationFile"/>
+    <hyperlink ref="G68" r:id="rId20" display="BA employment, KldB 2625 + 2622: Berlin 2,708 + 60% of Brandenburg 3,417 (own scaling: ~60% of Brandenburg lies within 75 km) ≈ 4,800. Berlin file: https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-11-0-202512-xlsx.xlsx?__blob=publicationFile https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-12-0-202512-xlsx.xlsx?__blob=publicationFile"/>
+    <hyperlink ref="G69" r:id="rId21" display="BA employment, KldB 2611 + 2510/2511/2513 (skilled level): Berlin 17,490 + 60% of Brandenburg 14,878 (own scaling: ~60% of Brandenburg lies within 75 km) ≈ 26,400. Berlin file: https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-11-0-202512-xlsx.xlsx?__blob=publicationFile https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-12-0-202512-xlsx.xlsx?__blob=publicationFile"/>
+    <hyperlink ref="G70" r:id="rId22" display="BA employment, KldB 2612: Berlin 1,254 + 60% of Brandenburg 1,206 (own scaling: ~60% of Brandenburg lies within 75 km) ≈ 2,000. Berlin file: https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-11-0-202512-xlsx.xlsx?__blob=publicationFile https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-12-0-202512-xlsx.xlsx?__blob=publicationFile"/>
+    <hyperlink ref="G71" r:id="rId23" display="BA employment, supervisor codes 2519 + 2619 + 2629 + 2639: Berlin 1,494 + 60% of Brandenburg 1,209 (own scaling: ~60% of Brandenburg lies within 75 km) ≈ 2,200. Berlin file: https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-11-0-202512-xlsx.xlsx?__blob=publicationFile https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-12-0-202512-xlsx.xlsx?__blob=publicationFile"/>
     <hyperlink ref="G72" r:id="rId24" display="Gallup 2024: active job search is 3% / 10% / 23% for high / low / no engagement; weighted by the 9% / 78% / 13% shares ≈ 11%. https://gallup.com/file/de/657716/Engagement-Index-Deutschland-Report-2024.pdf"/>
     <hyperlink ref="G73" r:id="rId25" display="Gallup 2024: active job search is 3% / 10% / 23% for high / low / no engagement; weighted by the 9% / 78% / 13% shares ≈ 11%. https://gallup.com/file/de/657716/Engagement-Index-Deutschland-Report-2024.pdf"/>
     <hyperlink ref="G74" r:id="rId26" display="Gallup 2024: active job search is 3% / 10% / 23% for high / low / no engagement; weighted by the 9% / 78% / 13% shares ≈ 11%. https://gallup.com/file/de/657716/Engagement-Index-Deutschland-Report-2024.pdf"/>
@@ -7242,8 +7251,8 @@
     <hyperlink ref="G96" r:id="rId33" display="Between the common +20% and +30% scale-up rules (roaspig). https://roaspig.com/blog/automated-rules-manage-meta-budgets/"/>
     <hyperlink ref="G101" r:id="rId34" display="Risk rises once capacity is more than 85% used (Bagust et al., BMJ 1999). https://pubmed.ncbi.nlm.nih.gov/10406748/"/>
     <hyperlink ref="G102" r:id="rId35" display="Above 90% use, shortages become regular (same study), so the week counts as full. https://pubmed.ncbi.nlm.nih.gov/10406748/"/>
-    <hyperlink ref="G108" r:id="rId36" display="Derived from IAB 2025: decisive ÷ used for job boards (21% ÷ 57%), relative to the average channel (0.41). https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/"/>
-    <hyperlink ref="G109" r:id="rId37" display="Derived from IAB 2025: decisive ÷ used for the employer homepage (20% ÷ 70%), relative to the average channel (0.41). https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/"/>
+    <hyperlink ref="G108" r:id="rId36" display="Derived from IAB 2025: decisive ÷ used for job boards (21% ÷ 57% = 0.37) ÷ 0.41 = 0.90. Average = mean of decisive ÷ used over the three channels IAB reports (homepage 20/70, job boards 21/57, personal contacts 27/48) = 0.41. https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/"/>
+    <hyperlink ref="G109" r:id="rId37" display="Derived from IAB 2025: decisive ÷ used for the employer homepage (20% ÷ 70% = 0.29) ÷ 0.41 = 0.70. Average = mean of decisive ÷ used over the three channels IAB reports (homepage 20/70, job boards 21/57, personal contacts 27/48) = 0.41. https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/"/>
     <hyperlink ref="G110" r:id="rId38" display="Derived from IAB data (2022): social media was used for 42% of filled jobs but decisive for 1 in 14; (7.1% ÷ 42%) ÷ 0.41 ≈ 0.41. https://ohn.haendlerbund.de/themen/unternehmen-maerkte/139538-social-media-whatsapp-mitarbeitersuche-immer-wichtiger"/>
     <hyperlink ref="G111" r:id="rId39" display="36% of skilled-worker job seekers use Indeed (Trendence 2023). https://www.personalwirtschaft.de/?p=157882"/>
     <hyperlink ref="G112" r:id="rId40" display="15% of skilled-worker job seekers use LinkedIn (Trendence 2023). https://www.personalwirtschaft.de/?p=157882"/>
@@ -7255,25 +7264,25 @@
     <hyperlink ref="G118" r:id="rId46" display="Redline 2024–26: mean 29.5 qualified applications per Elektroniker campaign (11 campaigns). https://redline-grow.de/bewerbungen-pro-stelle"/>
     <hyperlink ref="G119" r:id="rId47" display="A StepStone ad runs 30 days. https://www.stepstone.de/e-recruiting/stellenanzeige-aufgeben/"/>
     <hyperlink ref="G120" r:id="rId48" display="Plant headcount (Electrek, March 2026). https://electrek.co/2026/03/04/tesla-giga-berlin-ig-metall-union-vote-collapse/"/>
-    <hyperlink ref="G121" r:id="rId49" display="BA employment: maintenance codes 2513 + 2625 + 2611 + 2612 + supervisors (536,520) ÷ production occupations 21–29 (6,850,263) = 7.8%. https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-d-0-202512-xlsx.xlsx?__blob=publicationFile"/>
+    <hyperlink ref="G121" r:id="rId49" display="BA employment, Germany: maintenance codes 2513 + 2625 + 2611 + 2612 + supervisors 2519 + 2619 + 2629 (536,520) ÷ production occupations 21–29 (6,850,263) = 7.8%. https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-d-0-202512-xlsx.xlsx?__blob=publicationFile"/>
     <hyperlink ref="G122" r:id="rId50" display="IAB-Betriebspanel Brandenburg: ~6% of jobs ended in the first half of 2024 → ~12% a year. https://mweke.brandenburg.de/media/bb1.a.3814.de/Betriebspanel%20Brandenburg%202024%20-%20final.pdf"/>
     <hyperlink ref="G123" r:id="rId51" display="Referrals bring ~11% of hires (CareerPlug 2025). https://www.careerplug.com/wp-content/uploads/2025/04/Recruiting-Metrics-Report.pdf"/>
     <hyperlink ref="L127" r:id="rId52" display="Free listings (careers site, BA Jobbörse, Google for Jobs). Volume: ~27 applications per vacancy, 13% via the careers page. https://www.arbeitsagentur.de/faktor-a/mitarbeiter-finden/so-funktioniert-deutschlands-groesste-jobboerse"/>
     <hyperlink ref="L128" r:id="rId53" display="Free listings (careers site, BA Jobbörse, Google for Jobs). Volume: ~27 applications per vacancy, 13% via the careers page. https://www.arbeitsagentur.de/faktor-a/mitarbeiter-finden/so-funktioniert-deutschlands-groesste-jobboerse"/>
     <hyperlink ref="L129" r:id="rId54" display="Free listings (careers site, BA Jobbörse, Google for Jobs). Volume: ~27 applications per vacancy, 13% via the careers page. https://www.arbeitsagentur.de/faktor-a/mitarbeiter-finden/so-funktioniert-deutschlands-groesste-jobboerse"/>
     <hyperlink ref="L130" r:id="rId55" display="Free listings (careers site, BA Jobbörse, Google for Jobs). Volume: ~27 applications per vacancy, 13% via the careers page. https://www.arbeitsagentur.de/faktor-a/mitarbeiter-finden/so-funktioniert-deutschlands-groesste-jobboerse"/>
-    <hyperlink ref="L131" r:id="rId56" display="Indeed's DACH median is €161 per application (TalentBait, 2,549 campaigns), used as the programmatic proxy. Volume capped by Indeed's reach. https://www.talentbait.de/recruiting-kanaele-uebersicht/"/>
-    <hyperlink ref="L132" r:id="rId57" display="Indeed's DACH median is €161 per application (TalentBait, 2,549 campaigns), used as the programmatic proxy. Volume capped by Indeed's reach. https://www.talentbait.de/recruiting-kanaele-uebersicht/"/>
-    <hyperlink ref="L133" r:id="rId58" display="Indeed's DACH median is €161 per application (TalentBait, 2,549 campaigns), used as the programmatic proxy. Volume capped by Indeed's reach. https://www.talentbait.de/recruiting-kanaele-uebersicht/"/>
-    <hyperlink ref="L134" r:id="rId59" display="Indeed's DACH median is €161 per application (TalentBait, 2,549 campaigns), used as the programmatic proxy. Volume capped by Indeed's reach. https://www.talentbait.de/recruiting-kanaele-uebersicht/"/>
+    <hyperlink ref="L131" r:id="rId56" display="Indeed's CPA median is €161 in TalentBait's DACH 2024–26 dataset (2,549 channel-campaigns across all channels), used as the programmatic proxy. Volume capped by Indeed's reach. https://www.talentbait.de/recruiting-kanaele-uebersicht/"/>
+    <hyperlink ref="L132" r:id="rId57" display="Indeed's CPA median is €161 in TalentBait's DACH 2024–26 dataset (2,549 channel-campaigns across all channels), used as the programmatic proxy. Volume capped by Indeed's reach. https://www.talentbait.de/recruiting-kanaele-uebersicht/"/>
+    <hyperlink ref="L133" r:id="rId58" display="Indeed's CPA median is €161 in TalentBait's DACH 2024–26 dataset (2,549 channel-campaigns across all channels), used as the programmatic proxy. Volume capped by Indeed's reach. https://www.talentbait.de/recruiting-kanaele-uebersicht/"/>
+    <hyperlink ref="L134" r:id="rId59" display="Indeed's CPA median is €161 in TalentBait's DACH 2024–26 dataset (2,549 channel-campaigns across all channels), used as the programmatic proxy. Volume capped by Indeed's reach. https://www.talentbait.de/recruiting-kanaele-uebersicht/"/>
     <hyperlink ref="L135" r:id="rId60" display="From €1,449 per 30-day ad (StepStone price list); HR teams get ~12 applications per vacancy on average (StepStone), used as applications per ad. https://www.stepstone.de/e-recruiting/stellenanzeige-aufgeben/ https://www.stepstone.de/e-recruiting/hr-wissen/recruiting/bewerberqualitaet-steigern"/>
     <hyperlink ref="L136" r:id="rId61" display="From €1,449 per 30-day ad (StepStone price list); HR teams get ~12 applications per vacancy on average (StepStone), used as applications per ad. https://www.stepstone.de/e-recruiting/stellenanzeige-aufgeben/ https://www.stepstone.de/e-recruiting/hr-wissen/recruiting/bewerberqualitaet-steigern"/>
     <hyperlink ref="L137" r:id="rId62" display="From €1,449 per 30-day ad (StepStone price list); HR teams get ~12 applications per vacancy on average (StepStone), used as applications per ad. https://www.stepstone.de/e-recruiting/stellenanzeige-aufgeben/ https://www.stepstone.de/e-recruiting/hr-wissen/recruiting/bewerberqualitaet-steigern"/>
     <hyperlink ref="L138" r:id="rId63" display="From €1,449 per 30-day ad (StepStone price list); HR teams get ~12 applications per vacancy on average (StepStone), used as applications per ad. https://www.stepstone.de/e-recruiting/stellenanzeige-aufgeben/ https://www.stepstone.de/e-recruiting/hr-wissen/recruiting/bewerberqualitaet-steigern"/>
     <hyperlink ref="L139" r:id="rId64" display="DACH median €96 per application (TalentBait). Used only for automation and supervisors. https://www.talentbait.de/recruiting-kanaele-uebersicht/"/>
     <hyperlink ref="L140" r:id="rId65" display="DACH median €96 per application (TalentBait). Used only for automation and supervisors. https://www.talentbait.de/recruiting-kanaele-uebersicht/"/>
-    <hyperlink ref="L141" r:id="rId66" display="TalentBait's trades example: ~€84 per application for social ads; volume from Redline campaign data. https://www.talentbait.de/social-media-recruiting"/>
-    <hyperlink ref="L142" r:id="rId67" display="TalentBait's trades example: ~€84 per application for social ads; volume from Redline campaign data. https://www.talentbait.de/social-media-recruiting"/>
+    <hyperlink ref="L141" r:id="rId66" display="Own estimate: TalentBait's example ad shows ~€84 per application for trades (its measured averages: €52 raw, €104 per qualified); volume from Redline campaign data. https://www.talentbait.de/social-media-recruiting"/>
+    <hyperlink ref="L142" r:id="rId67" display="Own estimate: TalentBait's example ad shows ~€84 per application for trades (its measured averages: €52 raw, €104 per qualified); volume from Redline campaign data. https://www.talentbait.de/social-media-recruiting"/>
     <hyperlink ref="L143" r:id="rId68" display="Google Search ads ~€179 per application, low volume (TalentBait). https://www.talentbait.de/recruiting-kanaele-uebersicht/"/>
     <hyperlink ref="L144" r:id="rId69" display="Google Search ads ~€179 per application, low volume (TalentBait). https://www.talentbait.de/recruiting-kanaele-uebersicht/"/>
     <hyperlink ref="L145" r:id="rId70" display="Google Search ads ~€179 per application, low volume (TalentBait). https://www.talentbait.de/recruiting-kanaele-uebersicht/"/>
@@ -7281,14 +7290,14 @@
     <hyperlink ref="G154" r:id="rId72" display="Cold outreach gets ~5% replies (Pin 2026); past applicants already know the employer, so I assume 12%. https://www.pin.com/blog/recruiting-outreach-benchmark-report/"/>
     <hyperlink ref="G155" r:id="rId73" display="They met the requirements once; I assume half still do (Forrester via SHRM: most remain a 70%+ match). https://www.shrm.org/mena/topics-tools/news/technology/talent-rediscovery-tools-help-address-labor-shortages"/>
     <hyperlink ref="G160" r:id="rId74" display="Referred applicants are better pre-filtered (IAB: referrals are the most decisive channel), so 45% qualify. https://iab-forum.de/online-medien-sind-bei-der-personalsuche-auf-dem-vormarsch/"/>
-    <hyperlink ref="G161" r:id="rId75" display="Three text messages at ~€0.075 each (seven.io) plus email, rounded up to €0.30. https://www.seven.io/en/prices/"/>
+    <hyperlink ref="G161" r:id="rId75" display="Three text messages at ~€0.075 each (seven.io price list, 2016 rates) plus email, rounded up to €0.30. https://www.seven.io/en/prices/"/>
     <hyperlink ref="G162" r:id="rId76" display="Most firms pay €501–1,000 per successful referral (Radancy survey, 335 firms worldwide). https://www.personalwirtschaft.de/?p=166393"/>
     <hyperlink ref="G163" r:id="rId77" display="Referred and known candidates pass and accept a little more often (+15%). https://www.metaview.ai/resources/blog/do-referred-candidates-interview-better"/>
-    <hyperlink ref="G164" r:id="rId78" display="BA employment, KldB 2621 Bauelektrik: Berlin 6,204 + 60% of Brandenburg 5,905 (75 km radius, own scaling) ≈ 10,000. Berlin file: https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-11-0-202512-xlsx.xlsx?__blob=publicationFile https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-12-0-202512-xlsx.xlsx?__blob=publicationFile"/>
-    <hyperlink ref="G166" r:id="rId79" display="TalentBait's trades example shows ~€84 per application for social ads. https://www.talentbait.de/social-media-recruiting"/>
+    <hyperlink ref="G164" r:id="rId78" display="BA employment, KldB 2621 Bauelektrik: Berlin 6,204 + 60% of Brandenburg 5,905 (own scaling: ~60% of Brandenburg lies within 75 km) ≈ 10,000. Berlin file: https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-11-0-202512-xlsx.xlsx?__blob=publicationFile https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-12-0-202512-xlsx.xlsx?__blob=publicationFile"/>
+    <hyperlink ref="G166" r:id="rId79" display="Own estimate: TalentBait's example ad shows ~€84 per application for trades; its measured averages are €52 per raw application and €104 per qualified one. https://www.talentbait.de/social-media-recruiting"/>
     <hyperlink ref="G169" r:id="rId80" display="Copywriter (~11 hours at €65) plus a quiz tool for 3 months. https://www.freelancermap.de/freelancer/texterstellung"/>
     <hyperlink ref="G170" r:id="rId81" display="Pracuj.pl ad price divided by expected applications, blended with OLX and Meta. https://dlafirm.pracuj.pl/cennik-uslug/pakiety-ogloszen"/>
-    <hyperlink ref="G171" r:id="rId82" display="Eurostat AES 2022, Poland, vocational upper-secondary: 58.7% know a foreign language × 23.6% of them good or proficient ≈ 14%. https://ec.europa.eu/eurostat/databrowser/view/edat_aes_l33/default/table"/>
+    <hyperlink ref="G171" r:id="rId82" display="Eurostat AES 2022, Poland, ages 25–64, vocational upper-secondary: 58.7% know a foreign language (edat_aes_l23: 100 − 41.3%) × 23.6% of them good or proficient (edat_aes_l33) ≈ 14%. https://ec.europa.eu/eurostat/databrowser/view/edat_aes_l23/default/table https://ec.europa.eu/eurostat/databrowser/view/edat_aes_l33/default/table"/>
     <hyperlink ref="G174" r:id="rId83" display="Phone screens take 15–30 minutes (Indeed); a checklist call takes 15. https://www.indeed.com/hire/c/info/what-is-a-phone-screen"/>
     <hyperlink ref="G175" r:id="rId84" display="Polish freelance recruiters charge ~€14–19 an hour. https://rocketjobs.pl/oferta-pracy/intent-tech-recruiter-freelance--warszawa-hr-recruitment-9e0cdcee"/>
     <hyperlink ref="G176" r:id="rId85" display="Translation at the German statutory rate per line (JVEG). https://www.gesetze-im-internet.de/jveg/__11.html"/>
@@ -7429,11 +7438,11 @@
       </c>
       <c r="M5" s="29" t="n">
         <f aca="false">SUMIFS(Channels!$W:$W,Channels!$C:$C,A5)</f>
-        <v>413.059411486506</v>
+        <v>414.272633087996</v>
       </c>
       <c r="N5" s="31" t="n">
         <f aca="false">IF(M5&gt;0,O5/M5,0)</f>
-        <v>0.233024820549912</v>
+        <v>0.232342393753174</v>
       </c>
       <c r="O5" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$V:$V,Channels!$C:$C,A5)</f>
@@ -7494,11 +7503,11 @@
       </c>
       <c r="M6" s="29" t="n">
         <f aca="false">SUMIFS(Channels!$W:$W,Channels!$C:$C,A6)</f>
-        <v>660.667213314308</v>
+        <v>662.469323804687</v>
       </c>
       <c r="N6" s="31" t="n">
         <f aca="false">IF(M6&gt;0,O6/M6,0)</f>
-        <v>0.179777532195495</v>
+        <v>0.179288484680294</v>
       </c>
       <c r="O6" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$V:$V,Channels!$C:$C,A6)</f>
@@ -7559,11 +7568,11 @@
       </c>
       <c r="M7" s="29" t="n">
         <f aca="false">SUMIFS(Channels!$W:$W,Channels!$C:$C,A7)</f>
-        <v>225.835890028541</v>
+        <v>226.471333852253</v>
       </c>
       <c r="N7" s="31" t="n">
         <f aca="false">IF(M7&gt;0,O7/M7,0)</f>
-        <v>0.229483245127705</v>
+        <v>0.228839350342959</v>
       </c>
       <c r="O7" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$V:$V,Channels!$C:$C,A7)</f>
@@ -7624,11 +7633,11 @@
       </c>
       <c r="M8" s="29" t="n">
         <f aca="false">SUMIFS(Channels!$W:$W,Channels!$C:$C,A8)</f>
-        <v>190.926508605547</v>
+        <v>191.361952429259</v>
       </c>
       <c r="N8" s="31" t="n">
         <f aca="false">IF(M8&gt;0,O8/M8,0)</f>
-        <v>0.215377670827498</v>
+        <v>0.2148875792741</v>
       </c>
       <c r="O8" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$V:$V,Channels!$C:$C,A8)</f>
@@ -7669,11 +7678,11 @@
       </c>
       <c r="M9" s="33" t="n">
         <f aca="false">SUM(M5:M8)</f>
-        <v>1490.4890234349</v>
+        <v>1494.57524317419</v>
       </c>
       <c r="N9" s="34" t="n">
         <f aca="false">IF(M9&gt;0,O9/M9,0)</f>
-        <v>0.206625524402199</v>
+        <v>0.206060603164336</v>
       </c>
       <c r="O9" s="35" t="n">
         <f aca="false">SUM(O5:O8)</f>
@@ -7884,11 +7893,11 @@
       </c>
       <c r="D30" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$N:$N,Channels!$C:$C,A30)</f>
-        <v>110.5720875</v>
+        <v>110.22165</v>
       </c>
       <c r="E30" s="40" t="n">
         <f aca="false">IF(B30&gt;0,D30/B30,0)</f>
-        <v>3.68573625</v>
+        <v>3.674055</v>
       </c>
       <c r="F30" s="29" t="n">
         <f aca="false">Funnel!F58</f>
@@ -7910,11 +7919,11 @@
       </c>
       <c r="K30" s="40" t="n">
         <f aca="false">IF(B30&gt;0,(D30-SUMIFS(Channels!$N:$N,Channels!$A:$A,"I2-E",Channels!$C:$C,A30))/B30,0)</f>
-        <v>3.40696125</v>
+        <v>3.39528</v>
       </c>
       <c r="L30" s="40" t="n">
         <f aca="false">IF(B30&gt;0,K30,1000000000)</f>
-        <v>3.40696125</v>
+        <v>3.39528</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7931,11 +7940,11 @@
       </c>
       <c r="D31" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$N:$N,Channels!$C:$C,A31)</f>
-        <v>551.49330375</v>
+        <v>551.69006625</v>
       </c>
       <c r="E31" s="40" t="n">
         <f aca="false">IF(B31&gt;0,D31/B31,0)</f>
-        <v>12.25540675</v>
+        <v>12.25977925</v>
       </c>
       <c r="F31" s="29" t="n">
         <f aca="false">Funnel!F59</f>
@@ -7957,11 +7966,11 @@
       </c>
       <c r="K31" s="40" t="n">
         <f aca="false">IF(B31&gt;0,(D31-SUMIFS(Channels!$N:$N,Channels!$A:$A,"I2-E",Channels!$C:$C,A31))/B31,0)</f>
-        <v>12.25540675</v>
+        <v>12.25977925</v>
       </c>
       <c r="L31" s="40" t="n">
         <f aca="false">IF(B31&gt;0,K31,1000000000)</f>
-        <v>12.25540675</v>
+        <v>12.25977925</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7978,11 +7987,11 @@
       </c>
       <c r="D32" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$N:$N,Channels!$C:$C,A32)</f>
-        <v>48.045312</v>
+        <v>47.90852325</v>
       </c>
       <c r="E32" s="40" t="n">
         <f aca="false">IF(B32&gt;0,D32/B32,0)</f>
-        <v>3.2030208</v>
+        <v>3.19390155</v>
       </c>
       <c r="F32" s="29" t="n">
         <f aca="false">Funnel!F60</f>
@@ -8004,11 +8013,11 @@
       </c>
       <c r="K32" s="40" t="n">
         <f aca="false">IF(B32&gt;0,(D32-SUMIFS(Channels!$N:$N,Channels!$A:$A,"I2-E",Channels!$C:$C,A32))/B32,0)</f>
-        <v>3.2030208</v>
+        <v>3.19390155</v>
       </c>
       <c r="L32" s="40" t="n">
         <f aca="false">IF(B32&gt;0,K32,1000000000)</f>
-        <v>3.2030208</v>
+        <v>3.19390155</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8025,11 +8034,11 @@
       </c>
       <c r="D33" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$N:$N,Channels!$C:$C,A33)</f>
-        <v>39.856194</v>
+        <v>39.749451</v>
       </c>
       <c r="E33" s="40" t="n">
         <f aca="false">IF(B33&gt;0,D33/B33,0)</f>
-        <v>3.9856194</v>
+        <v>3.9749451</v>
       </c>
       <c r="F33" s="29" t="n">
         <f aca="false">Funnel!F61</f>
@@ -8051,11 +8060,11 @@
       </c>
       <c r="K33" s="40" t="n">
         <f aca="false">IF(B33&gt;0,(D33-SUMIFS(Channels!$N:$N,Channels!$A:$A,"I2-E",Channels!$C:$C,A33))/B33,0)</f>
-        <v>3.9856194</v>
+        <v>3.9749451</v>
       </c>
       <c r="L33" s="40" t="n">
         <f aca="false">IF(B33&gt;0,K33,1000000000)</f>
-        <v>3.9856194</v>
+        <v>3.9749451</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8159,7 +8168,7 @@
       </c>
       <c r="F42" s="41" t="n">
         <f aca="false">Budget!$C$7*1</f>
-        <v>101667.57387493</v>
+        <v>102255.847555873</v>
       </c>
       <c r="G42" s="30" t="n">
         <f aca="false">IF(Budget!$C$7&gt;0,F42/Budget!$C$7-1,0)</f>
@@ -8191,7 +8200,7 @@
       </c>
       <c r="F43" s="41" t="n">
         <f aca="false">Budget!$C$7*1/(1-$B$40)</f>
-        <v>145239.3912499</v>
+        <v>146079.782222676</v>
       </c>
       <c r="G43" s="30" t="n">
         <f aca="false">IF(Budget!$C$7&gt;0,F43/Budget!$C$7-1,0)</f>
@@ -8223,7 +8232,7 @@
       </c>
       <c r="F44" s="41" t="n">
         <f aca="false">Budget!$C$7*1/(1-$B$40)</f>
-        <v>145239.3912499</v>
+        <v>146079.782222676</v>
       </c>
       <c r="G44" s="30" t="n">
         <f aca="false">IF(Budget!$C$7&gt;0,F44/Budget!$C$7-1,0)</f>
@@ -8255,7 +8264,7 @@
       </c>
       <c r="F45" s="41" t="n">
         <f aca="false">Budget!$C$7*1/(1-$B$40)</f>
-        <v>145239.3912499</v>
+        <v>146079.782222676</v>
       </c>
       <c r="G45" s="30" t="n">
         <f aca="false">IF(Budget!$C$7&gt;0,F45/Budget!$C$7-1,0)</f>
@@ -8287,7 +8296,7 @@
       </c>
       <c r="F46" s="41" t="n">
         <f aca="false">Budget!$C$7*(1+$B$40)</f>
-        <v>132167.846037409</v>
+        <v>132932.601822636</v>
       </c>
       <c r="G46" s="30" t="n">
         <f aca="false">IF(Budget!$C$7&gt;0,F46/Budget!$C$7-1,0)</f>
@@ -8319,7 +8328,7 @@
       </c>
       <c r="F47" s="41" t="n">
         <f aca="false">Budget!$C$7*1</f>
-        <v>101667.57387493</v>
+        <v>102255.847555873</v>
       </c>
       <c r="G47" s="30" t="n">
         <f aca="false">IF(Budget!$C$7&gt;0,F47/Budget!$C$7-1,0)</f>
@@ -8435,11 +8444,11 @@
       </c>
       <c r="I58" s="29" t="n">
         <f aca="false">SUMIFS(Channels!$K:$K,Channels!$C:$C,A58)-SUMIFS(Channels!$K:$K,Channels!$A:$A,"I2-E",Channels!$C:$C,A58)</f>
-        <v>322.5375</v>
+        <v>321.425</v>
       </c>
       <c r="J58" s="30" t="n">
         <f aca="false">IF(F58&gt;0,I58/F58,0)</f>
-        <v>0.566849736379613</v>
+        <v>0.564894551845343</v>
       </c>
       <c r="K58" s="2" t="str">
         <f aca="false">IF(H58&gt;Assumptions!$D$99,"Very hard",IF(H58&gt;Assumptions!$D$100,"Tight","Comfortable"))</f>
@@ -8480,11 +8489,11 @@
       </c>
       <c r="I59" s="29" t="n">
         <f aca="false">SUMIFS(Channels!$K:$K,Channels!$C:$C,A59)-SUMIFS(Channels!$K:$K,Channels!$A:$A,"I2-E",Channels!$C:$C,A59)</f>
-        <v>1483.58</v>
+        <v>1484.11</v>
       </c>
       <c r="J59" s="30" t="n">
         <f aca="false">IF(F59&gt;0,I59/F59,0)</f>
-        <v>0.505995907230559</v>
+        <v>0.506176671214188</v>
       </c>
       <c r="K59" s="2" t="str">
         <f aca="false">IF(H59&gt;Assumptions!$D$99,"Very hard",IF(H59&gt;Assumptions!$D$100,"Tight","Comfortable"))</f>
@@ -8525,11 +8534,11 @@
       </c>
       <c r="I60" s="29" t="n">
         <f aca="false">SUMIFS(Channels!$K:$K,Channels!$C:$C,A60)-SUMIFS(Channels!$K:$K,Channels!$A:$A,"I2-E",Channels!$C:$C,A60)</f>
-        <v>168.3875</v>
+        <v>167.905</v>
       </c>
       <c r="J60" s="30" t="n">
         <f aca="false">IF(F60&gt;0,I60/F60,0)</f>
-        <v>0.713506355932203</v>
+        <v>0.71146186440678</v>
       </c>
       <c r="K60" s="2" t="str">
         <f aca="false">IF(H60&gt;Assumptions!$D$99,"Very hard",IF(H60&gt;Assumptions!$D$100,"Tight","Comfortable"))</f>
@@ -8570,11 +8579,11 @@
       </c>
       <c r="I61" s="29" t="n">
         <f aca="false">SUMIFS(Channels!$K:$K,Channels!$C:$C,A61)-SUMIFS(Channels!$K:$K,Channels!$A:$A,"I2-E",Channels!$C:$C,A61)</f>
-        <v>166.5675</v>
+        <v>166.119</v>
       </c>
       <c r="J61" s="30" t="n">
         <f aca="false">IF(F61&gt;0,I61/F61,0)</f>
-        <v>0.677103658536586</v>
+        <v>0.675280487804878</v>
       </c>
       <c r="K61" s="2" t="str">
         <f aca="false">IF(H61&gt;Assumptions!$D$99,"Very hard",IF(H61&gt;Assumptions!$D$100,"Tight","Comfortable"))</f>
@@ -9267,6 +9276,29 @@
         <v>382.972582972583</v>
       </c>
     </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="9" t="str">
+        <f aca="false">"Polish supply check: the plan needs "&amp;TEXT(B47,"0")&amp;" applications ("&amp;TEXT(B47*B39,"0")&amp;" qualified). ~1,700 Polish workers in machine, metal and building trades already commute to Brandenburg (IAB-Regional 1/2020, https://doku.iab.de/regional/BB/2020/regional_bb_0120.pdf); the ads also reach border-town workers who do not commute yet. Test bar below decides by 9 Nov; if it fails, the budget rises to the no-corridor case (see deck slide 7)."</f>
+        <v>Polish supply check: the plan needs 346 applications (48 qualified). ~1,700 Polish workers in machine, metal and building trades already commute to Brandenburg (IAB-Regional 1/2020, https://doku.iab.de/regional/BB/2020/regional_bb_0120.pdf); the ads also reach border-town workers who do not commute yet. Test bar below decides by 9 Nov; if it fails, the budget rises to the no-corridor case (see deck slide 7).</v>
+      </c>
+      <c r="B49" s="9"/>
+      <c r="C49" s="9"/>
+      <c r="D49" s="9"/>
+      <c r="E49" s="9"/>
+      <c r="F49" s="9"/>
+      <c r="G49" s="9"/>
+      <c r="H49" s="9"/>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="9"/>
+      <c r="B50" s="9"/>
+      <c r="C50" s="9"/>
+      <c r="D50" s="9"/>
+      <c r="E50" s="9"/>
+      <c r="F50" s="9"/>
+      <c r="G50" s="9"/>
+      <c r="H50" s="9"/>
+    </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="28" t="s">
         <v>550</v>
@@ -9439,6 +9471,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A49:H50"/>
+  </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -9627,7 +9662,7 @@
       </c>
       <c r="I5" s="30" t="n">
         <f aca="false">Assumptions!G127</f>
-        <v>0.1775</v>
+        <v>0.175</v>
       </c>
       <c r="J5" s="29" t="n">
         <f aca="false">IF(AND(OR(E5="CPC",E5="Slot"),NOT(N(G5)&gt;0)),0,IF(E5="Slot",Assumptions!H127*G5,Assumptions!H127))</f>
@@ -9635,7 +9670,7 @@
       </c>
       <c r="K5" s="32" t="n">
         <f aca="false">J5*I5</f>
-        <v>18.6375</v>
+        <v>18.375</v>
       </c>
       <c r="L5" s="31" t="n">
         <f aca="false">INDEX(Funnel!$G$5:$G$8,MATCH(C5,Funnel!$A$5:$A$8,0))*M5</f>
@@ -9647,7 +9682,7 @@
       </c>
       <c r="N5" s="32" t="n">
         <f aca="false">K5*L5</f>
-        <v>5.8708125</v>
+        <v>5.788125</v>
       </c>
       <c r="O5" s="41" t="n">
         <f aca="false">IF(I5&gt;0,H5/I5,0)</f>
@@ -9671,15 +9706,15 @@
       </c>
       <c r="T5" s="32" t="n">
         <f aca="false">INDEX(Funnel!$B$5:$B$8,MATCH(C5,Funnel!$A$5:$A$8,0))-SUMIFS($AG$5:$AG$34,$C$5:$C$34,C5)</f>
-        <v>29.1472854551251</v>
+        <v>29.1505850361307</v>
       </c>
       <c r="U5" s="46" t="n">
         <f aca="false">AG5+AI5</f>
-        <v>5.8708125</v>
+        <v>5.788125</v>
       </c>
       <c r="V5" s="32" t="n">
         <f aca="false">IF(L5&gt;0,U5/L5,0)</f>
-        <v>18.6375</v>
+        <v>18.375</v>
       </c>
       <c r="W5" s="29" t="n">
         <f aca="false">IF(I5&gt;0,V5/I5,0)</f>
@@ -9727,11 +9762,11 @@
       </c>
       <c r="AH5" s="32" t="n">
         <f aca="false">MAX(0,N5-AG5)</f>
-        <v>5.8708125</v>
+        <v>5.788125</v>
       </c>
       <c r="AI5" s="32" t="n">
         <f aca="false">MIN(AH5,MAX(0,T5-S5))</f>
-        <v>5.8708125</v>
+        <v>5.788125</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9768,7 +9803,7 @@
       </c>
       <c r="I6" s="30" t="n">
         <f aca="false">Assumptions!G128</f>
-        <v>0.1775</v>
+        <v>0.175</v>
       </c>
       <c r="J6" s="29" t="n">
         <f aca="false">IF(AND(OR(E6="CPC",E6="Slot"),NOT(N(G6)&gt;0)),0,IF(E6="Slot",Assumptions!H128*G6,Assumptions!H128))</f>
@@ -9776,7 +9811,7 @@
       </c>
       <c r="K6" s="32" t="n">
         <f aca="false">J6*I6</f>
-        <v>28.045</v>
+        <v>27.65</v>
       </c>
       <c r="L6" s="31" t="n">
         <f aca="false">INDEX(Funnel!$G$5:$G$8,MATCH(C6,Funnel!$A$5:$A$8,0))*M6</f>
@@ -9788,7 +9823,7 @@
       </c>
       <c r="N6" s="32" t="n">
         <f aca="false">K6*L6</f>
-        <v>10.41170625</v>
+        <v>10.2650625</v>
       </c>
       <c r="O6" s="41" t="n">
         <f aca="false">IF(I6&gt;0,H6/I6,0)</f>
@@ -9812,15 +9847,15 @@
       </c>
       <c r="T6" s="32" t="n">
         <f aca="false">INDEX(Funnel!$B$5:$B$8,MATCH(C6,Funnel!$A$5:$A$8,0))-SUMIFS($AG$5:$AG$34,$C$5:$C$34,C6)</f>
-        <v>43.9950150006831</v>
+        <v>43.9989037925826</v>
       </c>
       <c r="U6" s="46" t="n">
         <f aca="false">AG6+AI6</f>
-        <v>10.41170625</v>
+        <v>10.2650625</v>
       </c>
       <c r="V6" s="32" t="n">
         <f aca="false">IF(L6&gt;0,U6/L6,0)</f>
-        <v>28.045</v>
+        <v>27.65</v>
       </c>
       <c r="W6" s="29" t="n">
         <f aca="false">IF(I6&gt;0,V6/I6,0)</f>
@@ -9868,11 +9903,11 @@
       </c>
       <c r="AH6" s="32" t="n">
         <f aca="false">MAX(0,N6-AG6)</f>
-        <v>10.41170625</v>
+        <v>10.2650625</v>
       </c>
       <c r="AI6" s="32" t="n">
         <f aca="false">MIN(AH6,MAX(0,T6-S6))</f>
-        <v>10.41170625</v>
+        <v>10.2650625</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9909,7 +9944,7 @@
       </c>
       <c r="I7" s="30" t="n">
         <f aca="false">Assumptions!G129</f>
-        <v>0.1775</v>
+        <v>0.175</v>
       </c>
       <c r="J7" s="29" t="n">
         <f aca="false">IF(AND(OR(E7="CPC",E7="Slot"),NOT(N(G7)&gt;0)),0,IF(E7="Slot",Assumptions!H129*G7,Assumptions!H129))</f>
@@ -9917,7 +9952,7 @@
       </c>
       <c r="K7" s="32" t="n">
         <f aca="false">J7*I7</f>
-        <v>9.4075</v>
+        <v>9.275</v>
       </c>
       <c r="L7" s="31" t="n">
         <f aca="false">INDEX(Funnel!$G$5:$G$8,MATCH(C7,Funnel!$A$5:$A$8,0))*M7</f>
@@ -9929,7 +9964,7 @@
       </c>
       <c r="N7" s="32" t="n">
         <f aca="false">K7*L7</f>
-        <v>2.66702625</v>
+        <v>2.6294625</v>
       </c>
       <c r="O7" s="41" t="n">
         <f aca="false">IF(I7&gt;0,H7/I7,0)</f>
@@ -9953,15 +9988,15 @@
       </c>
       <c r="T7" s="32" t="n">
         <f aca="false">INDEX(Funnel!$B$5:$B$8,MATCH(C7,Funnel!$A$5:$A$8,0))-SUMIFS($AG$5:$AG$34,$C$5:$C$34,C7)</f>
-        <v>13.9936701908626</v>
+        <v>13.9966398137676</v>
       </c>
       <c r="U7" s="46" t="n">
         <f aca="false">AG7+AI7</f>
-        <v>2.66702625</v>
+        <v>2.6294625</v>
       </c>
       <c r="V7" s="32" t="n">
         <f aca="false">IF(L7&gt;0,U7/L7,0)</f>
-        <v>9.4075</v>
+        <v>9.275</v>
       </c>
       <c r="W7" s="29" t="n">
         <f aca="false">IF(I7&gt;0,V7/I7,0)</f>
@@ -10009,11 +10044,11 @@
       </c>
       <c r="AH7" s="32" t="n">
         <f aca="false">MAX(0,N7-AG7)</f>
-        <v>2.66702625</v>
+        <v>2.6294625</v>
       </c>
       <c r="AI7" s="32" t="n">
         <f aca="false">MIN(AH7,MAX(0,T7-S7))</f>
-        <v>2.66702625</v>
+        <v>2.6294625</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10050,7 +10085,7 @@
       </c>
       <c r="I8" s="30" t="n">
         <f aca="false">Assumptions!G130</f>
-        <v>0.1633</v>
+        <v>0.161</v>
       </c>
       <c r="J8" s="29" t="n">
         <f aca="false">IF(AND(OR(E8="CPC",E8="Slot"),NOT(N(G8)&gt;0)),0,IF(E8="Slot",Assumptions!H130*G8,Assumptions!H130))</f>
@@ -10058,7 +10093,7 @@
       </c>
       <c r="K8" s="32" t="n">
         <f aca="false">J8*I8</f>
-        <v>5.7155</v>
+        <v>5.635</v>
       </c>
       <c r="L8" s="31" t="n">
         <f aca="false">INDEX(Funnel!$G$5:$G$8,MATCH(C8,Funnel!$A$5:$A$8,0))*M8</f>
@@ -10070,7 +10105,7 @@
       </c>
       <c r="N8" s="32" t="n">
         <f aca="false">K8*L8</f>
-        <v>1.360289</v>
+        <v>1.34113</v>
       </c>
       <c r="O8" s="41" t="n">
         <f aca="false">IF(I8&gt;0,H8/I8,0)</f>
@@ -10094,15 +10129,15 @@
       </c>
       <c r="T8" s="32" t="n">
         <f aca="false">INDEX(Funnel!$B$5:$B$8,MATCH(C8,Funnel!$A$5:$A$8,0))-SUMIFS($AG$5:$AG$34,$C$5:$C$34,C8)</f>
-        <v>9.2227655202514</v>
+        <v>9.22505909567039</v>
       </c>
       <c r="U8" s="46" t="n">
         <f aca="false">AG8+AI8</f>
-        <v>1.360289</v>
+        <v>1.34113</v>
       </c>
       <c r="V8" s="32" t="n">
         <f aca="false">IF(L8&gt;0,U8/L8,0)</f>
-        <v>5.7155</v>
+        <v>5.635</v>
       </c>
       <c r="W8" s="29" t="n">
         <f aca="false">IF(I8&gt;0,V8/I8,0)</f>
@@ -10150,11 +10185,11 @@
       </c>
       <c r="AH8" s="32" t="n">
         <f aca="false">MAX(0,N8-AG8)</f>
-        <v>1.360289</v>
+        <v>1.34113</v>
       </c>
       <c r="AI8" s="32" t="n">
         <f aca="false">MIN(AH8,MAX(0,T8-S8))</f>
-        <v>1.360289</v>
+        <v>1.34113</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10231,27 +10266,27 @@
       </c>
       <c r="S9" s="32" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$34=C9)*($Q$5:$Q$34&lt;Q9)*$AH$5:$AH$34)</f>
-        <v>20.6080875</v>
+        <v>20.5254</v>
       </c>
       <c r="T9" s="32" t="n">
         <f aca="false">INDEX(Funnel!$B$5:$B$8,MATCH(C9,Funnel!$A$5:$A$8,0))-SUMIFS($AG$5:$AG$34,$C$5:$C$34,C9)</f>
-        <v>29.1472854551251</v>
+        <v>29.1505850361307</v>
       </c>
       <c r="U9" s="46" t="n">
         <f aca="false">AG9+AI9</f>
-        <v>8.86936099860335</v>
+        <v>8.95534807960894</v>
       </c>
       <c r="V9" s="32" t="n">
         <f aca="false">IF(L9&gt;0,U9/L9,0)</f>
-        <v>28.1567015828678</v>
+        <v>28.429676443203</v>
       </c>
       <c r="W9" s="29" t="n">
         <f aca="false">IF(I9&gt;0,V9/I9,0)</f>
-        <v>125.140895923857</v>
+        <v>126.354117525347</v>
       </c>
       <c r="X9" s="41" t="n">
         <f aca="false">IF(E9="Slot",IF(N(G9)&gt;0,ROUNDUP(W9/G9,0)*MAX(0,F9),0),W9*H9)</f>
-        <v>20147.6842437409</v>
+        <v>20343.0129215808</v>
       </c>
       <c r="Y9" s="41" t="n">
         <f aca="false">IF(U9&gt;0,Assumptions!J131,0)</f>
@@ -10263,11 +10298,11 @@
       </c>
       <c r="AA9" s="41" t="n">
         <f aca="false">X9+Y9</f>
-        <v>20147.6842437409</v>
+        <v>20343.0129215808</v>
       </c>
       <c r="AB9" s="41" t="n">
         <f aca="false">IF(U9&gt;0,(X9+Y9)/U9,"–")</f>
-        <v>2271.60493827161</v>
+        <v>2271.6049382716</v>
       </c>
       <c r="AC9" s="29" t="n">
         <f aca="false">SUMPRODUCT(--($Q$5:$Q$34&lt;Q9))+1</f>
@@ -10295,7 +10330,7 @@
       </c>
       <c r="AI9" s="32" t="n">
         <f aca="false">MIN(AH9,MAX(0,T9-S9))</f>
-        <v>8.53919795512509</v>
+        <v>8.62518503613068</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10372,27 +10407,27 @@
       </c>
       <c r="S10" s="32" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$34=C10)*($Q$5:$Q$34&lt;Q10)*$AH$5:$AH$34)</f>
-        <v>37.35846</v>
+        <v>37.21181625</v>
       </c>
       <c r="T10" s="32" t="n">
         <f aca="false">INDEX(Funnel!$B$5:$B$8,MATCH(C10,Funnel!$A$5:$A$8,0))-SUMIFS($AG$5:$AG$34,$C$5:$C$34,C10)</f>
-        <v>43.9950150006831</v>
+        <v>43.9989037925826</v>
       </c>
       <c r="U10" s="46" t="n">
         <f aca="false">AG10+AI10</f>
-        <v>7.0256757304968</v>
+        <v>7.17620827239625</v>
       </c>
       <c r="V10" s="32" t="n">
         <f aca="false">IF(L10&gt;0,U10/L10,0)</f>
-        <v>18.9243790720453</v>
+        <v>19.3298539323805</v>
       </c>
       <c r="W10" s="29" t="n">
         <f aca="false">IF(I10&gt;0,V10/I10,0)</f>
-        <v>84.1083514313123</v>
+        <v>85.9104619216909</v>
       </c>
       <c r="X10" s="41" t="n">
         <f aca="false">IF(E10="Slot",IF(N(G10)&gt;0,ROUNDUP(W10/G10,0)*MAX(0,F10),0),W10*H10)</f>
-        <v>13541.4445804413</v>
+        <v>13831.5843693922</v>
       </c>
       <c r="Y10" s="41" t="n">
         <f aca="false">IF(U10&gt;0,Assumptions!J132,0)</f>
@@ -10404,7 +10439,7 @@
       </c>
       <c r="AA10" s="41" t="n">
         <f aca="false">X10+Y10</f>
-        <v>13541.4445804413</v>
+        <v>13831.5843693922</v>
       </c>
       <c r="AB10" s="41" t="n">
         <f aca="false">IF(U10&gt;0,(X10+Y10)/U10,"–")</f>
@@ -10436,7 +10471,7 @@
       </c>
       <c r="AI10" s="32" t="n">
         <f aca="false">MIN(AH10,MAX(0,T10-S10))</f>
-        <v>6.63655500068314</v>
+        <v>6.78708754258258</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10513,11 +10548,11 @@
       </c>
       <c r="S11" s="32" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$34=C11)*($Q$5:$Q$34&lt;Q11)*$AH$5:$AH$34)</f>
-        <v>16.26274715625</v>
+        <v>16.22518340625</v>
       </c>
       <c r="T11" s="32" t="n">
         <f aca="false">INDEX(Funnel!$B$5:$B$8,MATCH(C11,Funnel!$A$5:$A$8,0))-SUMIFS($AG$5:$AG$34,$C$5:$C$34,C11)</f>
-        <v>13.9936701908626</v>
+        <v>13.9966398137676</v>
       </c>
       <c r="U11" s="46" t="n">
         <f aca="false">AG11+AI11</f>
@@ -10654,11 +10689,11 @@
       </c>
       <c r="S12" s="32" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$34=C12)*($Q$5:$Q$34&lt;Q12)*$AH$5:$AH$34)</f>
-        <v>12.068459375</v>
+        <v>12.049300375</v>
       </c>
       <c r="T12" s="32" t="n">
         <f aca="false">INDEX(Funnel!$B$5:$B$8,MATCH(C12,Funnel!$A$5:$A$8,0))-SUMIFS($AG$5:$AG$34,$C$5:$C$34,C12)</f>
-        <v>9.2227655202514</v>
+        <v>9.22505909567039</v>
       </c>
       <c r="U12" s="46" t="n">
         <f aca="false">AG12+AI12</f>
@@ -10795,11 +10830,11 @@
       </c>
       <c r="S13" s="32" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$34=C13)*($Q$5:$Q$34&lt;Q13)*$AH$5:$AH$34)</f>
-        <v>18.9070875</v>
+        <v>18.8244</v>
       </c>
       <c r="T13" s="32" t="n">
         <f aca="false">INDEX(Funnel!$B$5:$B$8,MATCH(C13,Funnel!$A$5:$A$8,0))-SUMIFS($AG$5:$AG$34,$C$5:$C$34,C13)</f>
-        <v>29.1472854551251</v>
+        <v>29.1505850361307</v>
       </c>
       <c r="U13" s="46" t="n">
         <f aca="false">AG13+AI13</f>
@@ -10936,11 +10971,11 @@
       </c>
       <c r="S14" s="32" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$34=C14)*($Q$5:$Q$34&lt;Q14)*$AH$5:$AH$34)</f>
-        <v>35.35371</v>
+        <v>35.20706625</v>
       </c>
       <c r="T14" s="32" t="n">
         <f aca="false">INDEX(Funnel!$B$5:$B$8,MATCH(C14,Funnel!$A$5:$A$8,0))-SUMIFS($AG$5:$AG$34,$C$5:$C$34,C14)</f>
-        <v>43.9950150006831</v>
+        <v>43.9989037925826</v>
       </c>
       <c r="U14" s="46" t="n">
         <f aca="false">AG14+AI14</f>
@@ -11077,11 +11112,11 @@
       </c>
       <c r="S15" s="32" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$34=C15)*($Q$5:$Q$34&lt;Q15)*$AH$5:$AH$34)</f>
-        <v>14.73184715625</v>
+        <v>14.69428340625</v>
       </c>
       <c r="T15" s="32" t="n">
         <f aca="false">INDEX(Funnel!$B$5:$B$8,MATCH(C15,Funnel!$A$5:$A$8,0))-SUMIFS($AG$5:$AG$34,$C$5:$C$34,C15)</f>
-        <v>13.9936701908626</v>
+        <v>13.9966398137676</v>
       </c>
       <c r="U15" s="46" t="n">
         <f aca="false">AG15+AI15</f>
@@ -11218,11 +11253,11 @@
       </c>
       <c r="S16" s="32" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$34=C16)*($Q$5:$Q$34&lt;Q16)*$AH$5:$AH$34)</f>
-        <v>11.477267375</v>
+        <v>11.458108375</v>
       </c>
       <c r="T16" s="32" t="n">
         <f aca="false">INDEX(Funnel!$B$5:$B$8,MATCH(C16,Funnel!$A$5:$A$8,0))-SUMIFS($AG$5:$AG$34,$C$5:$C$34,C16)</f>
-        <v>9.2227655202514</v>
+        <v>9.22505909567039</v>
       </c>
       <c r="U16" s="46" t="n">
         <f aca="false">AG16+AI16</f>
@@ -11359,27 +11394,27 @@
       </c>
       <c r="S17" s="32" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$34=C17)*($Q$5:$Q$34&lt;Q17)*$AH$5:$AH$34)</f>
-        <v>5.024187</v>
+        <v>4.98662325</v>
       </c>
       <c r="T17" s="32" t="n">
         <f aca="false">INDEX(Funnel!$B$5:$B$8,MATCH(C17,Funnel!$A$5:$A$8,0))-SUMIFS($AG$5:$AG$34,$C$5:$C$34,C17)</f>
-        <v>13.9936701908626</v>
+        <v>13.9966398137676</v>
       </c>
       <c r="U17" s="46" t="n">
         <f aca="false">AG17+AI17</f>
-        <v>9.46782303461258</v>
+        <v>9.50835640751761</v>
       </c>
       <c r="V17" s="32" t="n">
         <f aca="false">IF(L17&gt;0,U17/L17,0)</f>
-        <v>33.3962011802913</v>
+        <v>33.5391760406265</v>
       </c>
       <c r="W17" s="29" t="n">
         <f aca="false">IF(I17&gt;0,V17/I17,0)</f>
-        <v>148.427560801295</v>
+        <v>149.063004625007</v>
       </c>
       <c r="X17" s="41" t="n">
         <f aca="false">IF(E17="Slot",IF(N(G17)&gt;0,ROUNDUP(W17/G17,0)*MAX(0,F17),0),W17*H17)</f>
-        <v>14249.0458369243</v>
+        <v>14310.0484440006</v>
       </c>
       <c r="Y17" s="41" t="n">
         <f aca="false">IF(U17&gt;0,Assumptions!J139,0)</f>
@@ -11391,7 +11426,7 @@
       </c>
       <c r="AA17" s="41" t="n">
         <f aca="false">X17+Y17</f>
-        <v>14249.0458369243</v>
+        <v>14310.0484440006</v>
       </c>
       <c r="AB17" s="41" t="n">
         <f aca="false">IF(U17&gt;0,(X17+Y17)/U17,"–")</f>
@@ -11423,7 +11458,7 @@
       </c>
       <c r="AI17" s="32" t="n">
         <f aca="false">MIN(AH17,MAX(0,T17-S17))</f>
-        <v>8.96948319086258</v>
+        <v>9.01001656376761</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11500,27 +11535,27 @@
       </c>
       <c r="S18" s="32" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$34=C18)*($Q$5:$Q$34&lt;Q18)*$AH$5:$AH$34)</f>
-        <v>2.994278</v>
+        <v>2.975119</v>
       </c>
       <c r="T18" s="32" t="n">
         <f aca="false">INDEX(Funnel!$B$5:$B$8,MATCH(C18,Funnel!$A$5:$A$8,0))-SUMIFS($AG$5:$AG$34,$C$5:$C$34,C18)</f>
-        <v>9.2227655202514</v>
+        <v>9.22505909567039</v>
       </c>
       <c r="U18" s="46" t="n">
         <f aca="false">AG18+AI18</f>
-        <v>6.6133781452514</v>
+        <v>6.63483072067039</v>
       </c>
       <c r="V18" s="32" t="n">
         <f aca="false">IF(L18&gt;0,U18/L18,0)</f>
-        <v>27.7873031313084</v>
+        <v>27.8774400028168</v>
       </c>
       <c r="W18" s="29" t="n">
         <f aca="false">IF(I18&gt;0,V18/I18,0)</f>
-        <v>134.238179378301</v>
+        <v>134.673623202013</v>
       </c>
       <c r="X18" s="41" t="n">
         <f aca="false">IF(E18="Slot",IF(N(G18)&gt;0,ROUNDUP(W18/G18,0)*MAX(0,F18),0),W18*H18)</f>
-        <v>12886.8652203169</v>
+        <v>12928.6678273933</v>
       </c>
       <c r="Y18" s="41" t="n">
         <f aca="false">IF(U18&gt;0,Assumptions!J140,0)</f>
@@ -11532,7 +11567,7 @@
       </c>
       <c r="AA18" s="41" t="n">
         <f aca="false">X18+Y18</f>
-        <v>12886.8652203169</v>
+        <v>12928.6678273933</v>
       </c>
       <c r="AB18" s="41" t="n">
         <f aca="false">IF(U18&gt;0,(X18+Y18)/U18,"–")</f>
@@ -11564,7 +11599,7 @@
       </c>
       <c r="AI18" s="32" t="n">
         <f aca="false">MIN(AH18,MAX(0,T18-S18))</f>
-        <v>6.2284875202514</v>
+        <v>6.24994009567039</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11641,11 +11676,11 @@
       </c>
       <c r="S19" s="32" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$34=C19)*($Q$5:$Q$34&lt;Q19)*$AH$5:$AH$34)</f>
-        <v>84.7741744565217</v>
+        <v>84.6914869565217</v>
       </c>
       <c r="T19" s="32" t="n">
         <f aca="false">INDEX(Funnel!$B$5:$B$8,MATCH(C19,Funnel!$A$5:$A$8,0))-SUMIFS($AG$5:$AG$34,$C$5:$C$34,C19)</f>
-        <v>29.1472854551251</v>
+        <v>29.1505850361307</v>
       </c>
       <c r="U19" s="46" t="n">
         <f aca="false">AG19+AI19</f>
@@ -11782,11 +11817,11 @@
       </c>
       <c r="S20" s="32" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$34=C20)*($Q$5:$Q$34&lt;Q20)*$AH$5:$AH$34)</f>
-        <v>428.730901770186</v>
+        <v>428.584258020186</v>
       </c>
       <c r="T20" s="32" t="n">
         <f aca="false">INDEX(Funnel!$B$5:$B$8,MATCH(C20,Funnel!$A$5:$A$8,0))-SUMIFS($AG$5:$AG$34,$C$5:$C$34,C20)</f>
-        <v>43.9950150006831</v>
+        <v>43.9989037925826</v>
       </c>
       <c r="U20" s="46" t="n">
         <f aca="false">AG20+AI20</f>
@@ -11883,7 +11918,7 @@
       </c>
       <c r="I21" s="30" t="n">
         <f aca="false">Assumptions!G143</f>
-        <v>0.1775</v>
+        <v>0.175</v>
       </c>
       <c r="J21" s="29" t="n">
         <f aca="false">IF(AND(OR(E21="CPC",E21="Slot"),NOT(N(G21)&gt;0)),0,IF(E21="Slot",Assumptions!H143*G21,Assumptions!H143))</f>
@@ -11891,7 +11926,7 @@
       </c>
       <c r="K21" s="32" t="n">
         <f aca="false">J21*I21</f>
-        <v>60.35</v>
+        <v>59.5</v>
       </c>
       <c r="L21" s="31" t="n">
         <f aca="false">INDEX(Funnel!$G$5:$G$8,MATCH(C21,Funnel!$A$5:$A$8,0))*M21</f>
@@ -11903,19 +11938,19 @@
       </c>
       <c r="N21" s="32" t="n">
         <f aca="false">K21*L21</f>
-        <v>19.01025</v>
+        <v>18.7425</v>
       </c>
       <c r="O21" s="41" t="n">
         <f aca="false">IF(I21&gt;0,H21/I21,0)</f>
-        <v>1008.45070422535</v>
+        <v>1022.85714285714</v>
       </c>
       <c r="P21" s="41" t="n">
         <f aca="false">IF(N21&gt;0,(N21/L21/I21*H21+Assumptions!J143)/N21,0)</f>
-        <v>3201.43080706461</v>
+        <v>3247.16553287982</v>
       </c>
       <c r="Q21" s="45" t="n">
         <f aca="false">P21+ROW()/1000000</f>
-        <v>3201.43082806461</v>
+        <v>3247.16555387982</v>
       </c>
       <c r="R21" s="29" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$34=C21)*($Q$5:$Q$34&lt;Q21))+1</f>
@@ -11923,19 +11958,19 @@
       </c>
       <c r="S21" s="32" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$34=C21)*($Q$5:$Q$34&lt;Q21)*$AH$5:$AH$34)</f>
-        <v>90.9433932065217</v>
+        <v>90.8607057065217</v>
       </c>
       <c r="T21" s="32" t="n">
         <f aca="false">INDEX(Funnel!$B$5:$B$8,MATCH(C21,Funnel!$A$5:$A$8,0))-SUMIFS($AG$5:$AG$34,$C$5:$C$34,C21)</f>
-        <v>29.1472854551251</v>
+        <v>29.1505850361307</v>
       </c>
       <c r="U21" s="46" t="n">
         <f aca="false">AG21+AI21</f>
-        <v>0.234270251396648</v>
+        <v>0.230970670391061</v>
       </c>
       <c r="V21" s="32" t="n">
         <f aca="false">IF(L21&gt;0,U21/L21,0)</f>
-        <v>0.743715083798883</v>
+        <v>0.733240223463687</v>
       </c>
       <c r="W21" s="29" t="n">
         <f aca="false">IF(I21&gt;0,V21/I21,0)</f>
@@ -11959,7 +11994,7 @@
       </c>
       <c r="AB21" s="41" t="n">
         <f aca="false">IF(U21&gt;0,(X21+Y21)/U21,"–")</f>
-        <v>3201.43080706461</v>
+        <v>3247.16553287982</v>
       </c>
       <c r="AC21" s="29" t="n">
         <f aca="false">SUMPRODUCT(--($Q$5:$Q$34&lt;Q21))+1</f>
@@ -11975,15 +12010,15 @@
       </c>
       <c r="AF21" s="32" t="n">
         <f aca="false">AE21*I21</f>
-        <v>0.743715083798883</v>
+        <v>0.733240223463687</v>
       </c>
       <c r="AG21" s="32" t="n">
         <f aca="false">AF21*L21</f>
-        <v>0.234270251396648</v>
+        <v>0.230970670391061</v>
       </c>
       <c r="AH21" s="32" t="n">
         <f aca="false">MAX(0,N21-AG21)</f>
-        <v>18.7759797486034</v>
+        <v>18.5115293296089</v>
       </c>
       <c r="AI21" s="32" t="n">
         <f aca="false">MIN(AH21,MAX(0,T21-S21))</f>
@@ -12024,15 +12059,15 @@
       </c>
       <c r="I22" s="30" t="n">
         <f aca="false">Assumptions!G144</f>
-        <v>0.1775</v>
+        <v>0.175</v>
       </c>
       <c r="J22" s="29" t="n">
         <f aca="false">IF(AND(OR(E22="CPC",E22="Slot"),NOT(N(G22)&gt;0)),0,IF(E22="Slot",Assumptions!H144*G22,Assumptions!H144))</f>
-        <v>1730</v>
+        <v>1760</v>
       </c>
       <c r="K22" s="32" t="n">
         <f aca="false">J22*I22</f>
-        <v>307.075</v>
+        <v>308</v>
       </c>
       <c r="L22" s="31" t="n">
         <f aca="false">INDEX(Funnel!$G$5:$G$8,MATCH(C22,Funnel!$A$5:$A$8,0))*M22</f>
@@ -12044,19 +12079,19 @@
       </c>
       <c r="N22" s="32" t="n">
         <f aca="false">K22*L22</f>
-        <v>114.00159375</v>
+        <v>114.345</v>
       </c>
       <c r="O22" s="41" t="n">
         <f aca="false">IF(I22&gt;0,H22/I22,0)</f>
-        <v>1008.45070422535</v>
+        <v>1022.85714285714</v>
       </c>
       <c r="P22" s="41" t="n">
         <f aca="false">IF(N22&gt;0,(N22/L22/I22*H22+Assumptions!J144)/N22,0)</f>
-        <v>2716.36553326694</v>
+        <v>2755.17075517076</v>
       </c>
       <c r="Q22" s="45" t="n">
         <f aca="false">P22+ROW()/1000000</f>
-        <v>2716.36555526694</v>
+        <v>2755.17077717076</v>
       </c>
       <c r="R22" s="29" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$34=C22)*($Q$5:$Q$34&lt;Q22))+1</f>
@@ -12064,19 +12099,19 @@
       </c>
       <c r="S22" s="32" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$34=C22)*($Q$5:$Q$34&lt;Q22)*$AH$5:$AH$34)</f>
-        <v>436.762829225544</v>
+        <v>436.616185475544</v>
       </c>
       <c r="T22" s="32" t="n">
         <f aca="false">INDEX(Funnel!$B$5:$B$8,MATCH(C22,Funnel!$A$5:$A$8,0))-SUMIFS($AG$5:$AG$34,$C$5:$C$34,C22)</f>
-        <v>43.9950150006831</v>
+        <v>43.9989037925826</v>
       </c>
       <c r="U22" s="46" t="n">
         <f aca="false">AG22+AI22</f>
-        <v>0.276104224860335</v>
+        <v>0.272215432960894</v>
       </c>
       <c r="V22" s="32" t="n">
         <f aca="false">IF(L22&gt;0,U22/L22,0)</f>
-        <v>0.743715083798883</v>
+        <v>0.733240223463687</v>
       </c>
       <c r="W22" s="29" t="n">
         <f aca="false">IF(I22&gt;0,V22/I22,0)</f>
@@ -12100,7 +12135,7 @@
       </c>
       <c r="AB22" s="41" t="n">
         <f aca="false">IF(U22&gt;0,(X22+Y22)/U22,"–")</f>
-        <v>2716.36553326694</v>
+        <v>2755.17075517076</v>
       </c>
       <c r="AC22" s="29" t="n">
         <f aca="false">SUMPRODUCT(--($Q$5:$Q$34&lt;Q22))+1</f>
@@ -12116,15 +12151,15 @@
       </c>
       <c r="AF22" s="32" t="n">
         <f aca="false">AE22*I22</f>
-        <v>0.743715083798883</v>
+        <v>0.733240223463687</v>
       </c>
       <c r="AG22" s="32" t="n">
         <f aca="false">AF22*L22</f>
-        <v>0.276104224860335</v>
+        <v>0.272215432960894</v>
       </c>
       <c r="AH22" s="32" t="n">
         <f aca="false">MAX(0,N22-AG22)</f>
-        <v>113.72548952514</v>
+        <v>114.072784567039</v>
       </c>
       <c r="AI22" s="32" t="n">
         <f aca="false">MIN(AH22,MAX(0,T22-S22))</f>
@@ -12165,7 +12200,7 @@
       </c>
       <c r="I23" s="30" t="n">
         <f aca="false">Assumptions!G145</f>
-        <v>0.1775</v>
+        <v>0.175</v>
       </c>
       <c r="J23" s="29" t="n">
         <f aca="false">IF(AND(OR(E23="CPC",E23="Slot"),NOT(N(G23)&gt;0)),0,IF(E23="Slot",Assumptions!H145*G23,Assumptions!H145))</f>
@@ -12173,7 +12208,7 @@
       </c>
       <c r="K23" s="32" t="n">
         <f aca="false">J23*I23</f>
-        <v>24.85</v>
+        <v>24.5</v>
       </c>
       <c r="L23" s="31" t="n">
         <f aca="false">INDEX(Funnel!$G$5:$G$8,MATCH(C23,Funnel!$A$5:$A$8,0))*M23</f>
@@ -12185,19 +12220,19 @@
       </c>
       <c r="N23" s="32" t="n">
         <f aca="false">K23*L23</f>
-        <v>7.044975</v>
+        <v>6.94575</v>
       </c>
       <c r="O23" s="41" t="n">
         <f aca="false">IF(I23&gt;0,H23/I23,0)</f>
-        <v>1008.45070422535</v>
+        <v>1022.85714285714</v>
       </c>
       <c r="P23" s="41" t="n">
         <f aca="false">IF(N23&gt;0,(N23/L23/I23*H23+Assumptions!J145)/N23,0)</f>
-        <v>3557.1453411829</v>
+        <v>3607.9617031998</v>
       </c>
       <c r="Q23" s="45" t="n">
         <f aca="false">P23+ROW()/1000000</f>
-        <v>3557.1453641829</v>
+        <v>3607.9617261998</v>
       </c>
       <c r="R23" s="29" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$34=C23)*($Q$5:$Q$34&lt;Q23))+1</f>
@@ -12205,19 +12240,19 @@
       </c>
       <c r="S23" s="32" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$34=C23)*($Q$5:$Q$34&lt;Q23)*$AH$5:$AH$34)</f>
-        <v>40.2048504171196</v>
+        <v>40.1672866671196</v>
       </c>
       <c r="T23" s="32" t="n">
         <f aca="false">INDEX(Funnel!$B$5:$B$8,MATCH(C23,Funnel!$A$5:$A$8,0))-SUMIFS($AG$5:$AG$34,$C$5:$C$34,C23)</f>
-        <v>13.9936701908626</v>
+        <v>13.9966398137676</v>
       </c>
       <c r="U23" s="46" t="n">
         <f aca="false">AG23+AI23</f>
-        <v>0.210843226256983</v>
+        <v>0.207873603351955</v>
       </c>
       <c r="V23" s="32" t="n">
         <f aca="false">IF(L23&gt;0,U23/L23,0)</f>
-        <v>0.743715083798883</v>
+        <v>0.733240223463687</v>
       </c>
       <c r="W23" s="29" t="n">
         <f aca="false">IF(I23&gt;0,V23/I23,0)</f>
@@ -12241,7 +12276,7 @@
       </c>
       <c r="AB23" s="41" t="n">
         <f aca="false">IF(U23&gt;0,(X23+Y23)/U23,"–")</f>
-        <v>3557.1453411829</v>
+        <v>3607.9617031998</v>
       </c>
       <c r="AC23" s="29" t="n">
         <f aca="false">SUMPRODUCT(--($Q$5:$Q$34&lt;Q23))+1</f>
@@ -12257,15 +12292,15 @@
       </c>
       <c r="AF23" s="32" t="n">
         <f aca="false">AE23*I23</f>
-        <v>0.743715083798883</v>
+        <v>0.733240223463687</v>
       </c>
       <c r="AG23" s="32" t="n">
         <f aca="false">AF23*L23</f>
-        <v>0.210843226256983</v>
+        <v>0.207873603351955</v>
       </c>
       <c r="AH23" s="32" t="n">
         <f aca="false">MAX(0,N23-AG23)</f>
-        <v>6.83413177374302</v>
+        <v>6.73787639664804</v>
       </c>
       <c r="AI23" s="32" t="n">
         <f aca="false">MIN(AH23,MAX(0,T23-S23))</f>
@@ -12306,7 +12341,7 @@
       </c>
       <c r="I24" s="30" t="n">
         <f aca="false">Assumptions!G146</f>
-        <v>0.1633</v>
+        <v>0.161</v>
       </c>
       <c r="J24" s="29" t="n">
         <f aca="false">IF(AND(OR(E24="CPC",E24="Slot"),NOT(N(G24)&gt;0)),0,IF(E24="Slot",Assumptions!H146*G24,Assumptions!H146))</f>
@@ -12314,7 +12349,7 @@
       </c>
       <c r="K24" s="32" t="n">
         <f aca="false">J24*I24</f>
-        <v>26.128</v>
+        <v>25.76</v>
       </c>
       <c r="L24" s="31" t="n">
         <f aca="false">INDEX(Funnel!$G$5:$G$8,MATCH(C24,Funnel!$A$5:$A$8,0))*M24</f>
@@ -12326,19 +12361,19 @@
       </c>
       <c r="N24" s="32" t="n">
         <f aca="false">K24*L24</f>
-        <v>6.218464</v>
+        <v>6.13088</v>
       </c>
       <c r="O24" s="41" t="n">
         <f aca="false">IF(I24&gt;0,H24/I24,0)</f>
-        <v>1096.14206981017</v>
+        <v>1111.80124223602</v>
       </c>
       <c r="P24" s="41" t="n">
         <f aca="false">IF(N24&gt;0,(N24/L24/I24*H24+Assumptions!J146)/N24,0)</f>
-        <v>4605.63894878221</v>
+        <v>4671.43379090767</v>
       </c>
       <c r="Q24" s="45" t="n">
         <f aca="false">P24+ROW()/1000000</f>
-        <v>4605.63897278221</v>
+        <v>4671.43381490767</v>
       </c>
       <c r="R24" s="29" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$34=C24)*($Q$5:$Q$34&lt;Q24))+1</f>
@@ -12346,19 +12381,19 @@
       </c>
       <c r="S24" s="32" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$34=C24)*($Q$5:$Q$34&lt;Q24)*$AH$5:$AH$34)</f>
-        <v>33.023339375</v>
+        <v>33.004180375</v>
       </c>
       <c r="T24" s="32" t="n">
         <f aca="false">INDEX(Funnel!$B$5:$B$8,MATCH(C24,Funnel!$A$5:$A$8,0))-SUMIFS($AG$5:$AG$34,$C$5:$C$34,C24)</f>
-        <v>9.2227655202514</v>
+        <v>9.22505909567039</v>
       </c>
       <c r="U24" s="46" t="n">
         <f aca="false">AG24+AI24</f>
-        <v>0.162843854748603</v>
+        <v>0.160550279329609</v>
       </c>
       <c r="V24" s="32" t="n">
         <f aca="false">IF(L24&gt;0,U24/L24,0)</f>
-        <v>0.684217877094972</v>
+        <v>0.674581005586592</v>
       </c>
       <c r="W24" s="29" t="n">
         <f aca="false">IF(I24&gt;0,V24/I24,0)</f>
@@ -12382,7 +12417,7 @@
       </c>
       <c r="AB24" s="41" t="n">
         <f aca="false">IF(U24&gt;0,(X24+Y24)/U24,"–")</f>
-        <v>4605.63894878221</v>
+        <v>4671.43379090767</v>
       </c>
       <c r="AC24" s="29" t="n">
         <f aca="false">SUMPRODUCT(--($Q$5:$Q$34&lt;Q24))+1</f>
@@ -12398,15 +12433,15 @@
       </c>
       <c r="AF24" s="32" t="n">
         <f aca="false">AE24*I24</f>
-        <v>0.684217877094972</v>
+        <v>0.674581005586592</v>
       </c>
       <c r="AG24" s="32" t="n">
         <f aca="false">AF24*L24</f>
-        <v>0.162843854748603</v>
+        <v>0.160550279329609</v>
       </c>
       <c r="AH24" s="32" t="n">
         <f aca="false">MAX(0,N24-AG24)</f>
-        <v>6.0556201452514</v>
+        <v>5.97032972067039</v>
       </c>
       <c r="AI24" s="32" t="n">
         <f aca="false">MIN(AH24,MAX(0,T24-S24))</f>
@@ -12480,11 +12515,11 @@
       </c>
       <c r="S25" s="32" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$34=C25)*($Q$5:$Q$34&lt;Q25)*$AH$5:$AH$34)</f>
-        <v>5.8708125</v>
+        <v>5.788125</v>
       </c>
       <c r="T25" s="32" t="n">
         <f aca="false">INDEX(Funnel!$B$5:$B$8,MATCH(C25,Funnel!$A$5:$A$8,0))-SUMIFS($AG$5:$AG$34,$C$5:$C$34,C25)</f>
-        <v>29.1472854551251</v>
+        <v>29.1505850361307</v>
       </c>
       <c r="U25" s="46" t="n">
         <f aca="false">AG25+AI25</f>
@@ -12614,11 +12649,11 @@
       </c>
       <c r="S26" s="32" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$34=C26)*($Q$5:$Q$34&lt;Q26)*$AH$5:$AH$34)</f>
-        <v>10.41170625</v>
+        <v>10.2650625</v>
       </c>
       <c r="T26" s="32" t="n">
         <f aca="false">INDEX(Funnel!$B$5:$B$8,MATCH(C26,Funnel!$A$5:$A$8,0))-SUMIFS($AG$5:$AG$34,$C$5:$C$34,C26)</f>
-        <v>43.9950150006831</v>
+        <v>43.9989037925826</v>
       </c>
       <c r="U26" s="46" t="n">
         <f aca="false">AG26+AI26</f>
@@ -12748,11 +12783,11 @@
       </c>
       <c r="S27" s="32" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$34=C27)*($Q$5:$Q$34&lt;Q27)*$AH$5:$AH$34)</f>
-        <v>2.66702625</v>
+        <v>2.6294625</v>
       </c>
       <c r="T27" s="32" t="n">
         <f aca="false">INDEX(Funnel!$B$5:$B$8,MATCH(C27,Funnel!$A$5:$A$8,0))-SUMIFS($AG$5:$AG$34,$C$5:$C$34,C27)</f>
-        <v>13.9936701908626</v>
+        <v>13.9966398137676</v>
       </c>
       <c r="U27" s="46" t="n">
         <f aca="false">AG27+AI27</f>
@@ -12882,11 +12917,11 @@
       </c>
       <c r="S28" s="32" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$34=C28)*($Q$5:$Q$34&lt;Q28)*$AH$5:$AH$34)</f>
-        <v>1.360289</v>
+        <v>1.34113</v>
       </c>
       <c r="T28" s="32" t="n">
         <f aca="false">INDEX(Funnel!$B$5:$B$8,MATCH(C28,Funnel!$A$5:$A$8,0))-SUMIFS($AG$5:$AG$34,$C$5:$C$34,C28)</f>
-        <v>9.2227655202514</v>
+        <v>9.22505909567039</v>
       </c>
       <c r="U28" s="46" t="n">
         <f aca="false">AG28+AI28</f>
@@ -13016,11 +13051,11 @@
       </c>
       <c r="S29" s="32" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$34=C29)*($Q$5:$Q$34&lt;Q29)*$AH$5:$AH$34)</f>
-        <v>7.2835875</v>
+        <v>7.2009</v>
       </c>
       <c r="T29" s="32" t="n">
         <f aca="false">INDEX(Funnel!$B$5:$B$8,MATCH(C29,Funnel!$A$5:$A$8,0))-SUMIFS($AG$5:$AG$34,$C$5:$C$34,C29)</f>
-        <v>29.1472854551251</v>
+        <v>29.1505850361307</v>
       </c>
       <c r="U29" s="46" t="n">
         <f aca="false">AG29+AI29</f>
@@ -13150,11 +13185,11 @@
       </c>
       <c r="S30" s="32" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$34=C30)*($Q$5:$Q$34&lt;Q30)*$AH$5:$AH$34)</f>
-        <v>30.35854125</v>
+        <v>30.2118975</v>
       </c>
       <c r="T30" s="32" t="n">
         <f aca="false">INDEX(Funnel!$B$5:$B$8,MATCH(C30,Funnel!$A$5:$A$8,0))-SUMIFS($AG$5:$AG$34,$C$5:$C$34,C30)</f>
-        <v>43.9950150006831</v>
+        <v>43.9989037925826</v>
       </c>
       <c r="U30" s="46" t="n">
         <f aca="false">AG30+AI30</f>
@@ -13284,11 +13319,11 @@
       </c>
       <c r="S31" s="32" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$34=C31)*($Q$5:$Q$34&lt;Q31)*$AH$5:$AH$34)</f>
-        <v>3.41036325</v>
+        <v>3.3727995</v>
       </c>
       <c r="T31" s="32" t="n">
         <f aca="false">INDEX(Funnel!$B$5:$B$8,MATCH(C31,Funnel!$A$5:$A$8,0))-SUMIFS($AG$5:$AG$34,$C$5:$C$34,C31)</f>
-        <v>13.9936701908626</v>
+        <v>13.9966398137676</v>
       </c>
       <c r="U31" s="46" t="n">
         <f aca="false">AG31+AI31</f>
@@ -13418,11 +13453,11 @@
       </c>
       <c r="S32" s="32" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$34=C32)*($Q$5:$Q$34&lt;Q32)*$AH$5:$AH$34)</f>
-        <v>1.885793</v>
+        <v>1.866634</v>
       </c>
       <c r="T32" s="32" t="n">
         <f aca="false">INDEX(Funnel!$B$5:$B$8,MATCH(C32,Funnel!$A$5:$A$8,0))-SUMIFS($AG$5:$AG$34,$C$5:$C$34,C32)</f>
-        <v>9.2227655202514</v>
+        <v>9.22505909567039</v>
       </c>
       <c r="U32" s="46" t="n">
         <f aca="false">AG32+AI32</f>
@@ -13552,11 +13587,11 @@
       </c>
       <c r="S33" s="32" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$34=C33)*($Q$5:$Q$34&lt;Q33)*$AH$5:$AH$34)</f>
-        <v>10.5438375</v>
+        <v>10.46115</v>
       </c>
       <c r="T33" s="32" t="n">
         <f aca="false">INDEX(Funnel!$B$5:$B$8,MATCH(C33,Funnel!$A$5:$A$8,0))-SUMIFS($AG$5:$AG$34,$C$5:$C$34,C33)</f>
-        <v>29.1472854551251</v>
+        <v>29.1505850361307</v>
       </c>
       <c r="U33" s="46" t="n">
         <f aca="false">AG33+AI33</f>
@@ -13686,11 +13721,11 @@
       </c>
       <c r="S34" s="32" t="n">
         <f aca="false">SUMPRODUCT(($C$5:$C$34=C34)*($Q$5:$Q$34&lt;Q34)*$AH$5:$AH$34)</f>
-        <v>12.35854125</v>
+        <v>12.2118975</v>
       </c>
       <c r="T34" s="32" t="n">
         <f aca="false">INDEX(Funnel!$B$5:$B$8,MATCH(C34,Funnel!$A$5:$A$8,0))-SUMIFS($AG$5:$AG$34,$C$5:$C$34,C34)</f>
-        <v>43.9950150006831</v>
+        <v>43.9989037925826</v>
       </c>
       <c r="U34" s="46" t="n">
         <f aca="false">AG34+AI34</f>
@@ -13759,15 +13794,15 @@
       </c>
       <c r="J35" s="33" t="n">
         <f aca="false">SUM(J5:J34)</f>
-        <v>10534.32</v>
+        <v>10564.32</v>
       </c>
       <c r="K35" s="35" t="n">
         <f aca="false">SUM(K5:K34)</f>
-        <v>2170.5725</v>
+        <v>2169.059</v>
       </c>
       <c r="N35" s="35" t="n">
         <f aca="false">SUM(N5:N34)</f>
-        <v>749.96689725</v>
+        <v>749.5696905</v>
       </c>
       <c r="U35" s="35" t="n">
         <f aca="false">SUM(U5:U34)</f>
@@ -13779,11 +13814,11 @@
       </c>
       <c r="W35" s="33" t="n">
         <f aca="false">SUM(W5:W34)</f>
-        <v>1490.4890234349</v>
+        <v>1494.57524317419</v>
       </c>
       <c r="X35" s="42" t="n">
         <f aca="false">SUM(X5:X34)</f>
-        <v>100067.57387493</v>
+        <v>100655.847555873</v>
       </c>
       <c r="Y35" s="42" t="n">
         <f aca="false">SUM(Y5:Y34)</f>
@@ -13795,11 +13830,11 @@
       </c>
       <c r="AA35" s="42" t="n">
         <f aca="false">SUM(AA5:AA34)</f>
-        <v>101667.57387493</v>
+        <v>102255.847555873</v>
       </c>
       <c r="AB35" s="42" t="n">
         <f aca="false">IF(U35&gt;0,(X35+Y35)/U35,0)</f>
-        <v>1016.6757387493</v>
+        <v>1022.55847555873</v>
       </c>
       <c r="AE35" s="33" t="n">
         <f aca="false">SUM(AE5:AE34)</f>
@@ -13807,15 +13842,15 @@
       </c>
       <c r="AF35" s="35" t="n">
         <f aca="false">SUM(AF5:AF34)</f>
-        <v>12.2294159235227</v>
+        <v>12.1883544710087</v>
       </c>
       <c r="AG35" s="35" t="n">
         <f aca="false">SUM(AG5:AG34)</f>
-        <v>3.64126383307779</v>
+        <v>3.62881226184874</v>
       </c>
       <c r="AI35" s="35" t="n">
         <f aca="false">SUM(AI5:AI34)</f>
-        <v>96.3587361669222</v>
+        <v>96.3711877381513</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13949,7 +13984,7 @@
       </c>
       <c r="C4" s="41" t="n">
         <f aca="false">SUMIFS(Channels!X5:X34,Channels!D5:D34,"Channel")</f>
-        <v>72621.0398814234</v>
+        <v>73209.313562367</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13976,7 +14011,7 @@
       </c>
       <c r="C7" s="41" t="n">
         <f aca="false">C4+C5+C6</f>
-        <v>101667.57387493</v>
+        <v>102255.847555873</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13994,7 +14029,7 @@
       </c>
       <c r="C9" s="41" t="n">
         <f aca="false">C7</f>
-        <v>101667.57387493</v>
+        <v>102255.847555873</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14003,7 +14038,7 @@
       </c>
       <c r="C10" s="41" t="n">
         <f aca="false">IF(Assumptions!$D$48&lt;1,C9/(1-Assumptions!$D$48)*Assumptions!$D$48,0)</f>
-        <v>17941.3365661641</v>
+        <v>18045.1495686836</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14012,7 +14047,7 @@
       </c>
       <c r="C11" s="41" t="n">
         <f aca="false">C9+C10</f>
-        <v>119608.910441094</v>
+        <v>120300.997124557</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14021,7 +14056,7 @@
       </c>
       <c r="C12" s="4" t="n">
         <f aca="false">IF(Assumptions!$D$51&gt;0,ROUNDUP(C11/Assumptions!$D$51,0)*Assumptions!$D$51,C11)</f>
-        <v>120000</v>
+        <v>122500</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14039,7 +14074,7 @@
       </c>
       <c r="C14" s="47" t="n">
         <f aca="false">IF(C13&gt;0,C9/C13,0)</f>
-        <v>1016.6757387493</v>
+        <v>1022.55847555873</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14048,7 +14083,7 @@
       </c>
       <c r="C15" s="41" t="n">
         <f aca="false">IF(C13&gt;0,C12/C13,0)</f>
-        <v>1200</v>
+        <v>1225</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14057,7 +14092,7 @@
       </c>
       <c r="C16" s="30" t="n">
         <f aca="false">IF(C12&gt;0,Weekly!N5/C12,0)</f>
-        <v>0.39201909828295</v>
+        <v>0.385951267678667</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14098,7 +14133,7 @@
       </c>
       <c r="C21" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$C$5:$C$34,B21)</f>
-        <v>37737.434243741</v>
+        <v>37932.7629215808</v>
       </c>
       <c r="D21" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$Y$5:$Y$34,Channels!$C$5:$C$34,B21)</f>
@@ -14110,7 +14145,7 @@
       </c>
       <c r="F21" s="41" t="n">
         <f aca="false">C21+D21</f>
-        <v>38937.434243741</v>
+        <v>39132.7629215808</v>
       </c>
       <c r="G21" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$U$5:$U$34,Channels!$C$5:$C$34,B21)</f>
@@ -14118,7 +14153,7 @@
       </c>
       <c r="H21" s="41" t="n">
         <f aca="false">IF(G21&gt;0,F21/G21,0)</f>
-        <v>1297.91447479137</v>
+        <v>1304.42543071936</v>
       </c>
       <c r="I21" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$V$5:$V$34,Channels!$C$5:$C$34,B21)</f>
@@ -14131,7 +14166,7 @@
       </c>
       <c r="C22" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$C$5:$C$34,B22)</f>
-        <v>29450.9198239478</v>
+        <v>29741.0596128987</v>
       </c>
       <c r="D22" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$Y$5:$Y$34,Channels!$C$5:$C$34,B22)</f>
@@ -14143,7 +14178,7 @@
       </c>
       <c r="F22" s="41" t="n">
         <f aca="false">C22+D22</f>
-        <v>29850.9198239478</v>
+        <v>30141.0596128987</v>
       </c>
       <c r="G22" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$U$5:$U$34,Channels!$C$5:$C$34,B22)</f>
@@ -14151,7 +14186,7 @@
       </c>
       <c r="H22" s="41" t="n">
         <f aca="false">IF(G22&gt;0,F22/G22,0)</f>
-        <v>663.353773865506</v>
+        <v>669.801324731083</v>
       </c>
       <c r="I22" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$V$5:$V$34,Channels!$C$5:$C$34,B22)</f>
@@ -14164,7 +14199,7 @@
       </c>
       <c r="C23" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$C$5:$C$34,B23)</f>
-        <v>17374.2695869243</v>
+        <v>17435.2721940006</v>
       </c>
       <c r="D23" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$Y$5:$Y$34,Channels!$C$5:$C$34,B23)</f>
@@ -14176,7 +14211,7 @@
       </c>
       <c r="F23" s="41" t="n">
         <f aca="false">C23+D23</f>
-        <v>17374.2695869243</v>
+        <v>17435.2721940006</v>
       </c>
       <c r="G23" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$U$5:$U$34,Channels!$C$5:$C$34,B23)</f>
@@ -14184,7 +14219,7 @@
       </c>
       <c r="H23" s="41" t="n">
         <f aca="false">IF(G23&gt;0,F23/G23,0)</f>
-        <v>1158.28463912829</v>
+        <v>1162.35147960004</v>
       </c>
       <c r="I23" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$V$5:$V$34,Channels!$C$5:$C$34,B23)</f>
@@ -14197,7 +14232,7 @@
       </c>
       <c r="C24" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$C$5:$C$34,B24)</f>
-        <v>15504.9502203169</v>
+        <v>15546.7528273933</v>
       </c>
       <c r="D24" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$Y$5:$Y$34,Channels!$C$5:$C$34,B24)</f>
@@ -14209,7 +14244,7 @@
       </c>
       <c r="F24" s="41" t="n">
         <f aca="false">C24+D24</f>
-        <v>15504.9502203169</v>
+        <v>15546.7528273933</v>
       </c>
       <c r="G24" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$U$5:$U$34,Channels!$C$5:$C$34,B24)</f>
@@ -14217,7 +14252,7 @@
       </c>
       <c r="H24" s="41" t="n">
         <f aca="false">IF(G24&gt;0,F24/G24,0)</f>
-        <v>1550.49502203169</v>
+        <v>1554.67528273933</v>
       </c>
       <c r="I24" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$V$5:$V$34,Channels!$C$5:$C$34,B24)</f>
@@ -14230,7 +14265,7 @@
       </c>
       <c r="C25" s="42" t="n">
         <f aca="false">SUM(C21:C24)</f>
-        <v>100067.57387493</v>
+        <v>100655.847555873</v>
       </c>
       <c r="D25" s="42" t="n">
         <f aca="false">SUM(D21:D24)</f>
@@ -14242,7 +14277,7 @@
       </c>
       <c r="F25" s="42" t="n">
         <f aca="false">SUM(F21:F24)</f>
-        <v>101667.57387493</v>
+        <v>102255.847555873</v>
       </c>
       <c r="G25" s="35" t="n">
         <f aca="false">SUM(G21:G24)</f>
@@ -14250,7 +14285,7 @@
       </c>
       <c r="H25" s="42" t="n">
         <f aca="false">IF(G25&gt;0,F25/G25,0)</f>
-        <v>1016.6757387493</v>
+        <v>1022.55847555873</v>
       </c>
       <c r="I25" s="35" t="n">
         <f aca="false">SUM(I21:I24)</f>
@@ -14290,7 +14325,7 @@
       </c>
       <c r="D29" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$U$5:$U$34,Channels!$B$5:$B$34,B29)</f>
-        <v>20.309834</v>
+        <v>20.02378</v>
       </c>
       <c r="E29" s="41" t="n">
         <f aca="false">IF(D29&gt;0,C29/D29,"–")</f>
@@ -14307,19 +14342,19 @@
       </c>
       <c r="C30" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$AA$5:$AA$34,Channels!$B$5:$B$34,B30)</f>
-        <v>35189.1288241822</v>
+        <v>35674.597290973</v>
       </c>
       <c r="D30" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$U$5:$U$34,Channels!$B$5:$B$34,B30)</f>
-        <v>16.4216834682306</v>
+        <v>16.6582030911356</v>
       </c>
       <c r="E30" s="41" t="n">
         <f aca="false">IF(D30&gt;0,C30/D30,"–")</f>
-        <v>2142.8453965916</v>
+        <v>2141.56335445068</v>
       </c>
       <c r="F30" s="30" t="n">
         <f aca="false">IF($C$9&gt;0,C30/$C$9,0)</f>
-        <v>0.346119490049713</v>
+        <v>0.348875865230887</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14340,7 +14375,7 @@
       </c>
       <c r="F31" s="30" t="n">
         <f aca="false">IF($C$9&gt;0,C31/$C$9,0)</f>
-        <v>0.0570093273508244</v>
+        <v>0.0566813550377451</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14349,19 +14384,19 @@
       </c>
       <c r="C32" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$AA$5:$AA$34,Channels!$B$5:$B$34,B32)</f>
-        <v>27135.9110572412</v>
+        <v>27238.7162713939</v>
       </c>
       <c r="D32" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$U$5:$U$34,Channels!$B$5:$B$34,B32)</f>
-        <v>16.081201179864</v>
+        <v>16.143187128188</v>
       </c>
       <c r="E32" s="41" t="n">
         <f aca="false">IF(D32&gt;0,C32/D32,"–")</f>
-        <v>1687.43060631686</v>
+        <v>1687.31961384699</v>
       </c>
       <c r="F32" s="30" t="n">
         <f aca="false">IF($C$9&gt;0,C32/$C$9,0)</f>
-        <v>0.266908218844914</v>
+        <v>0.266378079322167</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14382,7 +14417,7 @@
       </c>
       <c r="F33" s="30" t="n">
         <f aca="false">IF($C$9&gt;0,C33/$C$9,0)</f>
-        <v>0.0147539667056999</v>
+        <v>0.0146690877426876</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14395,15 +14430,15 @@
       </c>
       <c r="D34" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$U$5:$U$34,Channels!$B$5:$B$34,B34)</f>
-        <v>0.88406155726257</v>
+        <v>0.87160998603352</v>
       </c>
       <c r="E34" s="41" t="n">
         <f aca="false">IF(D34&gt;0,C34/D34,"–")</f>
-        <v>3393.4288572498</v>
+        <v>3441.90641235337</v>
       </c>
       <c r="F34" s="30" t="n">
         <f aca="false">IF($C$9&gt;0,C34/$C$9,0)</f>
-        <v>0.0295079334113998</v>
+        <v>0.0293381754853753</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14424,7 +14459,7 @@
       </c>
       <c r="F35" s="30" t="n">
         <f aca="false">IF($C$9&gt;0,C35/$C$9,0)</f>
-        <v>0.000622617394980535</v>
+        <v>0.000619035502741419</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14445,7 +14480,7 @@
       </c>
       <c r="F36" s="30" t="n">
         <f aca="false">IF($C$9&gt;0,C36/$C$9,0)</f>
-        <v>0.107976684026164</v>
+        <v>0.107355498608543</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14466,7 +14501,7 @@
       </c>
       <c r="F37" s="30" t="n">
         <f aca="false">IF($C$9&gt;0,C37/$C$9,0)</f>
-        <v>0.109297385355825</v>
+        <v>0.10866860199783</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14487,7 +14522,7 @@
       </c>
       <c r="F38" s="30" t="n">
         <f aca="false">IF($C$9&gt;0,C38/$C$9,0)</f>
-        <v>0.0678043768604805</v>
+        <v>0.0674143010720225</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14496,7 +14531,7 @@
       </c>
       <c r="C39" s="42" t="n">
         <f aca="false">SUM(C29:C38)</f>
-        <v>101667.57387493</v>
+        <v>102255.847555873</v>
       </c>
       <c r="D39" s="35" t="n">
         <f aca="false">SUM(D29:D38)</f>
@@ -14554,7 +14589,7 @@
       </c>
       <c r="C45" s="41" t="n">
         <f aca="false">Budget!F52</f>
-        <v>120000</v>
+        <v>122500</v>
       </c>
       <c r="D45" s="32" t="n">
         <f aca="false">Budget!F87</f>
@@ -14578,7 +14613,7 @@
       </c>
       <c r="I45" s="41" t="n">
         <f aca="false">IF(H45&gt;0,C45/H45,0)</f>
-        <v>1200</v>
+        <v>1225</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14588,31 +14623,31 @@
       </c>
       <c r="C46" s="41" t="n">
         <f aca="false">Budget!G52</f>
-        <v>84000</v>
+        <v>85750</v>
       </c>
       <c r="D46" s="32" t="n">
         <f aca="false">Budget!G87</f>
-        <v>20.6080875</v>
+        <v>20.5254</v>
       </c>
       <c r="E46" s="32" t="n">
         <f aca="false">Budget!G88</f>
-        <v>44.3841357304968</v>
+        <v>43.9800408706604</v>
       </c>
       <c r="F46" s="32" t="n">
         <f aca="false">Budget!G89</f>
-        <v>14.4920100346126</v>
+        <v>14.4949796575176</v>
       </c>
       <c r="G46" s="32" t="n">
         <f aca="false">Budget!G90</f>
-        <v>7.4933802851456</v>
+        <v>8.05738580303432</v>
       </c>
       <c r="H46" s="35" t="n">
         <f aca="false">SUM(D46:G46)</f>
-        <v>86.977613550255</v>
+        <v>87.0578063312124</v>
       </c>
       <c r="I46" s="41" t="n">
         <f aca="false">IF(H46&gt;0,C46/H46,0)</f>
-        <v>965.765747889432</v>
+        <v>984.977724728822</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14644,11 +14679,11 @@
       </c>
       <c r="F52" s="41" t="n">
         <f aca="false">Budget!$C$12*F51</f>
-        <v>120000</v>
+        <v>122500</v>
       </c>
       <c r="G52" s="41" t="n">
         <f aca="false">Budget!$C$12*G51</f>
-        <v>84000</v>
+        <v>85750</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14657,11 +14692,11 @@
       </c>
       <c r="F53" s="41" t="n">
         <f aca="false">F52*(1-Assumptions!$D$48)</f>
-        <v>102000</v>
+        <v>104125</v>
       </c>
       <c r="G53" s="41" t="n">
         <f aca="false">G52*(1-Assumptions!$D$48)</f>
-        <v>71400</v>
+        <v>72887.5</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14674,7 +14709,7 @@
       </c>
       <c r="G54" s="41" t="n">
         <f aca="false">MAX(0,Budget!$C$9-G53)</f>
-        <v>30267.5738749299</v>
+        <v>29368.3475558735</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14738,15 +14773,15 @@
       </c>
       <c r="E56" s="32" t="n">
         <f aca="false">Channels!U5</f>
-        <v>5.8708125</v>
+        <v>5.788125</v>
       </c>
       <c r="F56" s="32" t="n">
         <f aca="false">IF(N56&gt;0,E56*MAX(0,N56-MIN(J56,N56))/N56,IF(C56&gt;0,E56*(1-J56/C56),E56))</f>
-        <v>5.8708125</v>
+        <v>5.788125</v>
       </c>
       <c r="G56" s="32" t="n">
         <f aca="false">IF(N56&gt;0,E56*MAX(0,N56-MIN(K56,N56))/N56,IF(C56&gt;0,E56*(1-K56/C56),E56))</f>
-        <v>5.8708125</v>
+        <v>5.788125</v>
       </c>
       <c r="J56" s="41" t="n">
         <f aca="false">MIN(C56,MAX(0,F$54-SUMPRODUCT(($D$56:$D$85&gt;D56)*$C$56:$C$85)))</f>
@@ -14762,11 +14797,11 @@
       </c>
       <c r="O56" s="32" t="n">
         <f aca="false">IF(E56&gt;0,F56*Channels!V5/E56,0)</f>
-        <v>18.6375</v>
+        <v>18.375</v>
       </c>
       <c r="P56" s="32" t="n">
         <f aca="false">IF(E56&gt;0,G56*Channels!V5/E56,0)</f>
-        <v>18.6375</v>
+        <v>18.375</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
@@ -14788,15 +14823,15 @@
       </c>
       <c r="E57" s="32" t="n">
         <f aca="false">Channels!U6</f>
-        <v>10.41170625</v>
+        <v>10.2650625</v>
       </c>
       <c r="F57" s="32" t="n">
         <f aca="false">IF(N57&gt;0,E57*MAX(0,N57-MIN(J57,N57))/N57,IF(C57&gt;0,E57*(1-J57/C57),E57))</f>
-        <v>10.41170625</v>
+        <v>10.2650625</v>
       </c>
       <c r="G57" s="32" t="n">
         <f aca="false">IF(N57&gt;0,E57*MAX(0,N57-MIN(K57,N57))/N57,IF(C57&gt;0,E57*(1-K57/C57),E57))</f>
-        <v>10.41170625</v>
+        <v>10.2650625</v>
       </c>
       <c r="J57" s="41" t="n">
         <f aca="false">MIN(C57,MAX(0,F$54-SUMPRODUCT(($D$56:$D$85&gt;D57)*$C$56:$C$85)))</f>
@@ -14812,11 +14847,11 @@
       </c>
       <c r="O57" s="32" t="n">
         <f aca="false">IF(E57&gt;0,F57*Channels!V6/E57,0)</f>
-        <v>28.045</v>
+        <v>27.65</v>
       </c>
       <c r="P57" s="32" t="n">
         <f aca="false">IF(E57&gt;0,G57*Channels!V6/E57,0)</f>
-        <v>28.045</v>
+        <v>27.65</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
@@ -14838,15 +14873,15 @@
       </c>
       <c r="E58" s="32" t="n">
         <f aca="false">Channels!U7</f>
-        <v>2.66702625</v>
+        <v>2.6294625</v>
       </c>
       <c r="F58" s="32" t="n">
         <f aca="false">IF(N58&gt;0,E58*MAX(0,N58-MIN(J58,N58))/N58,IF(C58&gt;0,E58*(1-J58/C58),E58))</f>
-        <v>2.66702625</v>
+        <v>2.6294625</v>
       </c>
       <c r="G58" s="32" t="n">
         <f aca="false">IF(N58&gt;0,E58*MAX(0,N58-MIN(K58,N58))/N58,IF(C58&gt;0,E58*(1-K58/C58),E58))</f>
-        <v>2.66702625</v>
+        <v>2.6294625</v>
       </c>
       <c r="J58" s="41" t="n">
         <f aca="false">MIN(C58,MAX(0,F$54-SUMPRODUCT(($D$56:$D$85&gt;D58)*$C$56:$C$85)))</f>
@@ -14862,11 +14897,11 @@
       </c>
       <c r="O58" s="32" t="n">
         <f aca="false">IF(E58&gt;0,F58*Channels!V7/E58,0)</f>
-        <v>9.4075</v>
+        <v>9.275</v>
       </c>
       <c r="P58" s="32" t="n">
         <f aca="false">IF(E58&gt;0,G58*Channels!V7/E58,0)</f>
-        <v>9.4075</v>
+        <v>9.275</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
@@ -14888,15 +14923,15 @@
       </c>
       <c r="E59" s="32" t="n">
         <f aca="false">Channels!U8</f>
-        <v>1.360289</v>
+        <v>1.34113</v>
       </c>
       <c r="F59" s="32" t="n">
         <f aca="false">IF(N59&gt;0,E59*MAX(0,N59-MIN(J59,N59))/N59,IF(C59&gt;0,E59*(1-J59/C59),E59))</f>
-        <v>1.360289</v>
+        <v>1.34113</v>
       </c>
       <c r="G59" s="32" t="n">
         <f aca="false">IF(N59&gt;0,E59*MAX(0,N59-MIN(K59,N59))/N59,IF(C59&gt;0,E59*(1-K59/C59),E59))</f>
-        <v>1.360289</v>
+        <v>1.34113</v>
       </c>
       <c r="J59" s="41" t="n">
         <f aca="false">MIN(C59,MAX(0,F$54-SUMPRODUCT(($D$56:$D$85&gt;D59)*$C$56:$C$85)))</f>
@@ -14912,11 +14947,11 @@
       </c>
       <c r="O59" s="32" t="n">
         <f aca="false">IF(E59&gt;0,F59*Channels!V8/E59,0)</f>
-        <v>5.7155</v>
+        <v>5.635</v>
       </c>
       <c r="P59" s="32" t="n">
         <f aca="false">IF(E59&gt;0,G59*Channels!V8/E59,0)</f>
-        <v>5.7155</v>
+        <v>5.635</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
@@ -14930,19 +14965,19 @@
       </c>
       <c r="C60" s="41" t="n">
         <f aca="false">Channels!AA9</f>
-        <v>20147.6842437409</v>
+        <v>20343.0129215808</v>
       </c>
       <c r="D60" s="45" t="n">
         <f aca="false">IF(ISNUMBER(Channels!AB9),Channels!AB9,0)+ROW()/1000000</f>
-        <v>2271.60499827161</v>
+        <v>2271.6049982716</v>
       </c>
       <c r="E60" s="32" t="n">
         <f aca="false">Channels!U9</f>
-        <v>8.86936099860335</v>
+        <v>8.95534807960894</v>
       </c>
       <c r="F60" s="32" t="n">
         <f aca="false">IF(N60&gt;0,E60*MAX(0,N60-MIN(J60,N60))/N60,IF(C60&gt;0,E60*(1-J60/C60),E60))</f>
-        <v>8.86936099860335</v>
+        <v>8.95534807960894</v>
       </c>
       <c r="G60" s="32" t="n">
         <f aca="false">IF(N60&gt;0,E60*MAX(0,N60-MIN(K60,N60))/N60,IF(C60&gt;0,E60*(1-K60/C60),E60))</f>
@@ -14954,15 +14989,15 @@
       </c>
       <c r="K60" s="41" t="n">
         <f aca="false">MIN(C60,MAX(0,G$54-SUMPRODUCT(($D$56:$D$85&gt;D60)*$C$56:$C$85)))</f>
-        <v>20147.6842437409</v>
+        <v>20343.0129215808</v>
       </c>
       <c r="N60" s="41" t="n">
         <f aca="false">Channels!X9</f>
-        <v>20147.6842437409</v>
+        <v>20343.0129215808</v>
       </c>
       <c r="O60" s="32" t="n">
         <f aca="false">IF(E60&gt;0,F60*Channels!V9/E60,0)</f>
-        <v>28.1567015828678</v>
+        <v>28.429676443203</v>
       </c>
       <c r="P60" s="32" t="n">
         <f aca="false">IF(E60&gt;0,G60*Channels!V9/E60,0)</f>
@@ -14980,7 +15015,7 @@
       </c>
       <c r="C61" s="41" t="n">
         <f aca="false">Channels!AA10</f>
-        <v>13541.4445804413</v>
+        <v>13831.5843693922</v>
       </c>
       <c r="D61" s="45" t="n">
         <f aca="false">IF(ISNUMBER(Channels!AB10),Channels!AB10,0)+ROW()/1000000</f>
@@ -14988,15 +15023,15 @@
       </c>
       <c r="E61" s="32" t="n">
         <f aca="false">Channels!U10</f>
-        <v>7.0256757304968</v>
+        <v>7.17620827239625</v>
       </c>
       <c r="F61" s="32" t="n">
         <f aca="false">IF(N61&gt;0,E61*MAX(0,N61-MIN(J61,N61))/N61,IF(C61&gt;0,E61*(1-J61/C61),E61))</f>
-        <v>7.0256757304968</v>
+        <v>7.17620827239625</v>
       </c>
       <c r="G61" s="32" t="n">
         <f aca="false">IF(N61&gt;0,E61*MAX(0,N61-MIN(K61,N61))/N61,IF(C61&gt;0,E61*(1-K61/C61),E61))</f>
-        <v>7.0256757304968</v>
+        <v>7.17620827239625</v>
       </c>
       <c r="J61" s="41" t="n">
         <f aca="false">MIN(C61,MAX(0,F$54-SUMPRODUCT(($D$56:$D$85&gt;D61)*$C$56:$C$85)))</f>
@@ -15008,15 +15043,15 @@
       </c>
       <c r="N61" s="41" t="n">
         <f aca="false">Channels!X10</f>
-        <v>13541.4445804413</v>
+        <v>13831.5843693922</v>
       </c>
       <c r="O61" s="32" t="n">
         <f aca="false">IF(E61&gt;0,F61*Channels!V10/E61,0)</f>
-        <v>18.9243790720453</v>
+        <v>19.3298539323805</v>
       </c>
       <c r="P61" s="32" t="n">
         <f aca="false">IF(E61&gt;0,G61*Channels!V10/E61,0)</f>
-        <v>18.9243790720453</v>
+        <v>19.3298539323805</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
@@ -15330,7 +15365,7 @@
       </c>
       <c r="C68" s="41" t="n">
         <f aca="false">Channels!AA17</f>
-        <v>14249.0458369243</v>
+        <v>14310.0484440006</v>
       </c>
       <c r="D68" s="45" t="n">
         <f aca="false">IF(ISNUMBER(Channels!AB17),Channels!AB17,0)+ROW()/1000000</f>
@@ -15338,15 +15373,15 @@
       </c>
       <c r="E68" s="32" t="n">
         <f aca="false">Channels!U17</f>
-        <v>9.46782303461258</v>
+        <v>9.50835640751761</v>
       </c>
       <c r="F68" s="32" t="n">
         <f aca="false">IF(N68&gt;0,E68*MAX(0,N68-MIN(J68,N68))/N68,IF(C68&gt;0,E68*(1-J68/C68),E68))</f>
-        <v>9.46782303461258</v>
+        <v>9.50835640751761</v>
       </c>
       <c r="G68" s="32" t="n">
         <f aca="false">IF(N68&gt;0,E68*MAX(0,N68-MIN(K68,N68))/N68,IF(C68&gt;0,E68*(1-K68/C68),E68))</f>
-        <v>9.46782303461258</v>
+        <v>9.50835640751761</v>
       </c>
       <c r="J68" s="41" t="n">
         <f aca="false">MIN(C68,MAX(0,F$54-SUMPRODUCT(($D$56:$D$85&gt;D68)*$C$56:$C$85)))</f>
@@ -15358,15 +15393,15 @@
       </c>
       <c r="N68" s="41" t="n">
         <f aca="false">Channels!X17</f>
-        <v>14249.0458369243</v>
+        <v>14310.0484440006</v>
       </c>
       <c r="O68" s="32" t="n">
         <f aca="false">IF(E68&gt;0,F68*Channels!V17/E68,0)</f>
-        <v>33.3962011802913</v>
+        <v>33.5391760406265</v>
       </c>
       <c r="P68" s="32" t="n">
         <f aca="false">IF(E68&gt;0,G68*Channels!V17/E68,0)</f>
-        <v>33.3962011802913</v>
+        <v>33.5391760406265</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
@@ -15380,7 +15415,7 @@
       </c>
       <c r="C69" s="41" t="n">
         <f aca="false">Channels!AA18</f>
-        <v>12886.8652203169</v>
+        <v>12928.6678273933</v>
       </c>
       <c r="D69" s="45" t="n">
         <f aca="false">IF(ISNUMBER(Channels!AB18),Channels!AB18,0)+ROW()/1000000</f>
@@ -15388,15 +15423,15 @@
       </c>
       <c r="E69" s="32" t="n">
         <f aca="false">Channels!U18</f>
-        <v>6.6133781452514</v>
+        <v>6.63483072067039</v>
       </c>
       <c r="F69" s="32" t="n">
         <f aca="false">IF(N69&gt;0,E69*MAX(0,N69-MIN(J69,N69))/N69,IF(C69&gt;0,E69*(1-J69/C69),E69))</f>
-        <v>6.6133781452514</v>
+        <v>6.63483072067039</v>
       </c>
       <c r="G69" s="32" t="n">
         <f aca="false">IF(N69&gt;0,E69*MAX(0,N69-MIN(K69,N69))/N69,IF(C69&gt;0,E69*(1-K69/C69),E69))</f>
-        <v>4.4991022851456</v>
+        <v>5.08226680303432</v>
       </c>
       <c r="J69" s="41" t="n">
         <f aca="false">MIN(C69,MAX(0,F$54-SUMPRODUCT(($D$56:$D$85&gt;D69)*$C$56:$C$85)))</f>
@@ -15404,19 +15439,19 @@
       </c>
       <c r="K69" s="41" t="n">
         <f aca="false">MIN(C69,MAX(0,G$54-SUMPRODUCT(($D$56:$D$85&gt;D69)*$C$56:$C$85)))</f>
-        <v>4119.88963118899</v>
+        <v>3025.33463429267</v>
       </c>
       <c r="N69" s="41" t="n">
         <f aca="false">Channels!X18</f>
-        <v>12886.8652203169</v>
+        <v>12928.6678273933</v>
       </c>
       <c r="O69" s="32" t="n">
         <f aca="false">IF(E69&gt;0,F69*Channels!V18/E69,0)</f>
-        <v>27.7873031313084</v>
+        <v>27.8774400028168</v>
       </c>
       <c r="P69" s="32" t="n">
         <f aca="false">IF(E69&gt;0,G69*Channels!V18/E69,0)</f>
-        <v>18.9037911140571</v>
+        <v>21.3540621976232</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
@@ -15534,15 +15569,15 @@
       </c>
       <c r="D72" s="45" t="n">
         <f aca="false">IF(ISNUMBER(Channels!AB21),Channels!AB21,0)+ROW()/1000000</f>
-        <v>3201.43087906461</v>
+        <v>3247.16560487982</v>
       </c>
       <c r="E72" s="32" t="n">
         <f aca="false">Channels!U21</f>
-        <v>0.234270251396648</v>
+        <v>0.230970670391061</v>
       </c>
       <c r="F72" s="32" t="n">
         <f aca="false">IF(N72&gt;0,E72*MAX(0,N72-MIN(J72,N72))/N72,IF(C72&gt;0,E72*(1-J72/C72),E72))</f>
-        <v>0.234270251396648</v>
+        <v>0.230970670391061</v>
       </c>
       <c r="G72" s="32" t="n">
         <f aca="false">IF(N72&gt;0,E72*MAX(0,N72-MIN(K72,N72))/N72,IF(C72&gt;0,E72*(1-K72/C72),E72))</f>
@@ -15562,7 +15597,7 @@
       </c>
       <c r="O72" s="32" t="n">
         <f aca="false">IF(E72&gt;0,F72*Channels!V21/E72,0)</f>
-        <v>0.743715083798883</v>
+        <v>0.733240223463687</v>
       </c>
       <c r="P72" s="32" t="n">
         <f aca="false">IF(E72&gt;0,G72*Channels!V21/E72,0)</f>
@@ -15584,15 +15619,15 @@
       </c>
       <c r="D73" s="45" t="n">
         <f aca="false">IF(ISNUMBER(Channels!AB22),Channels!AB22,0)+ROW()/1000000</f>
-        <v>2716.36560626694</v>
+        <v>2755.17082817076</v>
       </c>
       <c r="E73" s="32" t="n">
         <f aca="false">Channels!U22</f>
-        <v>0.276104224860335</v>
+        <v>0.272215432960894</v>
       </c>
       <c r="F73" s="32" t="n">
         <f aca="false">IF(N73&gt;0,E73*MAX(0,N73-MIN(J73,N73))/N73,IF(C73&gt;0,E73*(1-J73/C73),E73))</f>
-        <v>0.276104224860335</v>
+        <v>0.272215432960894</v>
       </c>
       <c r="G73" s="32" t="n">
         <f aca="false">IF(N73&gt;0,E73*MAX(0,N73-MIN(K73,N73))/N73,IF(C73&gt;0,E73*(1-K73/C73),E73))</f>
@@ -15612,7 +15647,7 @@
       </c>
       <c r="O73" s="32" t="n">
         <f aca="false">IF(E73&gt;0,F73*Channels!V22/E73,0)</f>
-        <v>0.743715083798883</v>
+        <v>0.733240223463687</v>
       </c>
       <c r="P73" s="32" t="n">
         <f aca="false">IF(E73&gt;0,G73*Channels!V22/E73,0)</f>
@@ -15634,15 +15669,15 @@
       </c>
       <c r="D74" s="45" t="n">
         <f aca="false">IF(ISNUMBER(Channels!AB23),Channels!AB23,0)+ROW()/1000000</f>
-        <v>3557.1454151829</v>
+        <v>3607.9617771998</v>
       </c>
       <c r="E74" s="32" t="n">
         <f aca="false">Channels!U23</f>
-        <v>0.210843226256983</v>
+        <v>0.207873603351955</v>
       </c>
       <c r="F74" s="32" t="n">
         <f aca="false">IF(N74&gt;0,E74*MAX(0,N74-MIN(J74,N74))/N74,IF(C74&gt;0,E74*(1-J74/C74),E74))</f>
-        <v>0.210843226256983</v>
+        <v>0.207873603351955</v>
       </c>
       <c r="G74" s="32" t="n">
         <f aca="false">IF(N74&gt;0,E74*MAX(0,N74-MIN(K74,N74))/N74,IF(C74&gt;0,E74*(1-K74/C74),E74))</f>
@@ -15662,7 +15697,7 @@
       </c>
       <c r="O74" s="32" t="n">
         <f aca="false">IF(E74&gt;0,F74*Channels!V23/E74,0)</f>
-        <v>0.743715083798883</v>
+        <v>0.733240223463687</v>
       </c>
       <c r="P74" s="32" t="n">
         <f aca="false">IF(E74&gt;0,G74*Channels!V23/E74,0)</f>
@@ -15684,15 +15719,15 @@
       </c>
       <c r="D75" s="45" t="n">
         <f aca="false">IF(ISNUMBER(Channels!AB24),Channels!AB24,0)+ROW()/1000000</f>
-        <v>4605.63902378221</v>
+        <v>4671.43386590767</v>
       </c>
       <c r="E75" s="32" t="n">
         <f aca="false">Channels!U24</f>
-        <v>0.162843854748603</v>
+        <v>0.160550279329609</v>
       </c>
       <c r="F75" s="32" t="n">
         <f aca="false">IF(N75&gt;0,E75*MAX(0,N75-MIN(J75,N75))/N75,IF(C75&gt;0,E75*(1-J75/C75),E75))</f>
-        <v>0.162843854748603</v>
+        <v>0.160550279329609</v>
       </c>
       <c r="G75" s="32" t="n">
         <f aca="false">IF(N75&gt;0,E75*MAX(0,N75-MIN(K75,N75))/N75,IF(C75&gt;0,E75*(1-K75/C75),E75))</f>
@@ -15712,7 +15747,7 @@
       </c>
       <c r="O75" s="32" t="n">
         <f aca="false">IF(E75&gt;0,F75*Channels!V24/E75,0)</f>
-        <v>0.684217877094972</v>
+        <v>0.674581005586592</v>
       </c>
       <c r="P75" s="32" t="n">
         <f aca="false">IF(E75&gt;0,G75*Channels!V24/E75,0)</f>
@@ -16191,12 +16226,12 @@
         <v>18</v>
       </c>
       <c r="F85" s="32" t="n">
-        <f aca="false">IF(N85&gt;0,E85*MAX(0,N85-MIN(J85,N85))/N85,IF(C85&gt;0,E85*(1-J85/C85),E85))</f>
+        <f aca="false">IF(Assumptions!$D$10&gt;=1,IF(N85&gt;0,E85*MAX(0,N85-MIN(J85,N85))/N85,IF(C85&gt;0,E85*(1-J85/C85),E85)),MIN(IF(N85&gt;0,E85*MAX(0,N85-MIN(J85,N85))/N85,IF(C85&gt;0,E85*(1-J85/C85),E85)),Assumptions!$D$10/(1-Assumptions!$D$10)*SUMIFS(F$56:F$84,$B$56:$B$84,"Mechatronics")))</f>
         <v>18</v>
       </c>
       <c r="G85" s="32" t="n">
-        <f aca="false">IF(N85&gt;0,E85*MAX(0,N85-MIN(K85,N85))/N85,IF(C85&gt;0,E85*(1-K85/C85),E85))</f>
-        <v>18</v>
+        <f aca="false">IF(Assumptions!$D$10&gt;=1,IF(N85&gt;0,E85*MAX(0,N85-MIN(K85,N85))/N85,IF(C85&gt;0,E85*(1-K85/C85),E85)),MIN(IF(N85&gt;0,E85*MAX(0,N85-MIN(K85,N85))/N85,IF(C85&gt;0,E85*(1-K85/C85),E85)),Assumptions!$D$10/(1-Assumptions!$D$10)*SUMIFS(G$56:G$84,$B$56:$B$84,"Mechatronics")))</f>
+        <v>17.5920163482642</v>
       </c>
       <c r="J85" s="41" t="n">
         <f aca="false">MIN(C85,MAX(0,F$54-SUMPRODUCT(($D$56:$D$85&gt;D85)*$C$56:$C$85)))</f>
@@ -16216,7 +16251,7 @@
       </c>
       <c r="P85" s="32" t="n">
         <f aca="false">IF(E85&gt;0,G85*Channels!V34/E85,0)</f>
-        <v>48.4848484848485</v>
+        <v>47.385902621587</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16234,7 +16269,7 @@
       </c>
       <c r="G87" s="32" t="n">
         <f aca="false">SUMIFS(G$56:G$85,$B$56:$B$85,$E87)*G$95</f>
-        <v>20.6080875</v>
+        <v>20.5254</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16247,7 +16282,7 @@
       </c>
       <c r="G88" s="32" t="n">
         <f aca="false">SUMIFS(G$56:G$85,$B$56:$B$85,$E88)*G$95</f>
-        <v>44.3841357304968</v>
+        <v>43.9800408706604</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16260,7 +16295,7 @@
       </c>
       <c r="G89" s="32" t="n">
         <f aca="false">SUMIFS(G$56:G$85,$B$56:$B$85,$E89)*G$95</f>
-        <v>14.4920100346126</v>
+        <v>14.4949796575176</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16273,7 +16308,7 @@
       </c>
       <c r="G90" s="32" t="n">
         <f aca="false">SUMIFS(G$56:G$85,$B$56:$B$85,$E90)*G$95</f>
-        <v>7.4933802851456</v>
+        <v>8.05738580303432</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16286,7 +16321,7 @@
       </c>
       <c r="G91" s="35" t="n">
         <f aca="false">SUM(G87:G90)</f>
-        <v>86.977613550255</v>
+        <v>87.0578063312124</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16295,11 +16330,11 @@
       </c>
       <c r="F92" s="41" t="n">
         <f aca="false">IF(F91&gt;0,F52/F91,0)</f>
-        <v>1200</v>
+        <v>1225</v>
       </c>
       <c r="G92" s="41" t="n">
         <f aca="false">IF(G91&gt;0,G52/G91,0)</f>
-        <v>965.765747889432</v>
+        <v>984.977724728822</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16312,7 +16347,7 @@
       </c>
       <c r="G94" s="32" t="n">
         <f aca="false">SUM(P56:P85)</f>
-        <v>264.174719851242</v>
+        <v>265.203994792217</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16484,7 +16519,7 @@
       </c>
       <c r="H4" s="41" t="n">
         <f aca="false">$F$19*D4+$F$20*E4+$F$31*Y4</f>
-        <v>19398.7108822494</v>
+        <v>19548.5453738207</v>
       </c>
       <c r="I4" s="41" t="n">
         <f aca="false">IF(A4=1,$F$21,0)</f>
@@ -16504,19 +16539,19 @@
       </c>
       <c r="M4" s="41" t="n">
         <f aca="false">SUM(H4:L4)</f>
-        <v>30394.7108822494</v>
+        <v>30544.5453738207</v>
       </c>
       <c r="N4" s="41" t="n">
         <f aca="false">SUM($M$4:M4)</f>
-        <v>30394.7108822494</v>
+        <v>30544.5453738207</v>
       </c>
       <c r="O4" s="29" t="n">
         <f aca="false">(Funnel!$M$5+Funnel!$M$6+Funnel!$M$7-$F$27-$F$34)*D4+(Funnel!$M$8-$F$28-$F$35)*E4+($F$27+$F$28)*X4+($F$34+$F$35)*Y4</f>
-        <v>403.092612777087</v>
+        <v>404.142980954988</v>
       </c>
       <c r="P4" s="29" t="n">
         <f aca="false">(Funnel!$O$5+Funnel!$O$6+Funnel!$O$7-$F$25-$F$32)*D4+(Funnel!$O$8-$F$26-$F$33)*E4+($F$25+$F$26)*X4+($F$32+$F$33)*Y4</f>
-        <v>85.6365349277805</v>
+        <v>85.6310133800371</v>
       </c>
       <c r="Q4" s="29" t="n">
         <f aca="false">Assumptions!$D$9*MAX(0,MIN(C4+Assumptions!$D$21,Funnel!$B$17)-MAX(IF(A4=1,Funnel!$B$13,B4+Assumptions!$D$21),Funnel!$B$13)+1)/7</f>
@@ -16524,7 +16559,7 @@
       </c>
       <c r="R4" s="30" t="n">
         <f aca="false">IF(Q4&gt;0,P4/Q4,IF(P4&gt;0,9.99,0))</f>
-        <v>0.990835941313163</v>
+        <v>0.990772055636793</v>
       </c>
       <c r="S4" s="2" t="str">
         <f aca="false">IF(P4&gt;Q4+0.5,"OVER "&amp;Assumptions!$D$9&amp;"/wk – pace down",IF(R4&gt;Assumptions!$D$102,"Full",IF(AND(Q4&gt;=Assumptions!$D$103,P4&lt;Assumptions!$D$103),"Under "&amp;Assumptions!$D$103&amp;" – release reserve","")))</f>
@@ -16593,7 +16628,7 @@
       </c>
       <c r="H5" s="41" t="n">
         <f aca="false">$F$19*D5+$F$20*E5+$F$31*Y5</f>
-        <v>11247.5809117046</v>
+        <v>11334.484916816</v>
       </c>
       <c r="I5" s="41" t="n">
         <f aca="false">IF(A5=1,$F$21,0)</f>
@@ -16613,19 +16648,19 @@
       </c>
       <c r="M5" s="41" t="n">
         <f aca="false">SUM(H5:L5)</f>
-        <v>16647.5809117046</v>
+        <v>16734.484916816</v>
       </c>
       <c r="N5" s="47" t="n">
         <f aca="false">SUM($M$4:M5)</f>
-        <v>47042.291793954</v>
+        <v>47279.0302906367</v>
       </c>
       <c r="O5" s="29" t="n">
         <f aca="false">(Funnel!$M$5+Funnel!$M$6+Funnel!$M$7-$F$27-$F$34)*D5+(Funnel!$M$8-$F$28-$F$35)*E5+($F$27+$F$28)*X5+($F$34+$F$35)*Y5</f>
-        <v>257.671324604645</v>
+        <v>258.280538147827</v>
       </c>
       <c r="P5" s="29" t="n">
         <f aca="false">(Funnel!$O$5+Funnel!$O$6+Funnel!$O$7-$F$25-$F$32)*D5+(Funnel!$O$8-$F$26-$F$33)*E5+($F$25+$F$26)*X5+($F$32+$F$33)*Y5</f>
-        <v>53.435335317969</v>
+        <v>53.4170222057527</v>
       </c>
       <c r="Q5" s="29" t="n">
         <f aca="false">Assumptions!$D$9*MAX(0,MIN(C5+Assumptions!$D$21,Funnel!$B$17)-MAX(IF(A5=1,Funnel!$B$13,B5+Assumptions!$D$21),Funnel!$B$13)+1)/7</f>
@@ -16633,7 +16668,7 @@
       </c>
       <c r="R5" s="30" t="n">
         <f aca="false">IF(Q5&gt;0,P5/Q5,IF(P5&gt;0,9.99,0))</f>
-        <v>0.971551551235801</v>
+        <v>0.97121858555914</v>
       </c>
       <c r="S5" s="2" t="str">
         <f aca="false">IF(P5&gt;Q5+0.5,"OVER "&amp;Assumptions!$D$9&amp;"/wk – pace down",IF(R5&gt;Assumptions!$D$102,"Full",IF(AND(Q5&gt;=Assumptions!$D$103,P5&lt;Assumptions!$D$103),"Under "&amp;Assumptions!$D$103&amp;" – release reserve","")))</f>
@@ -16702,7 +16737,7 @@
       </c>
       <c r="H6" s="41" t="n">
         <f aca="false">$F$19*D6+$F$20*E6+$F$31*Y6</f>
-        <v>13946.6892352196</v>
+        <v>14054.5700691509</v>
       </c>
       <c r="I6" s="41" t="n">
         <f aca="false">IF(A6=1,$F$21,0)</f>
@@ -16722,19 +16757,19 @@
       </c>
       <c r="M6" s="41" t="n">
         <f aca="false">SUM(H6:L6)</f>
-        <v>13946.6892352196</v>
+        <v>14054.5700691509</v>
       </c>
       <c r="N6" s="41" t="n">
         <f aca="false">SUM($M$4:M6)</f>
-        <v>60988.9810291736</v>
+        <v>61333.6003597877</v>
       </c>
       <c r="O6" s="29" t="n">
         <f aca="false">(Funnel!$M$5+Funnel!$M$6+Funnel!$M$7-$F$27-$F$34)*D6+(Funnel!$M$8-$F$28-$F$35)*E6+($F$27+$F$28)*X6+($F$34+$F$35)*Y6</f>
-        <v>262.237508786858</v>
+        <v>262.993773874947</v>
       </c>
       <c r="P6" s="29" t="n">
         <f aca="false">(Funnel!$O$5+Funnel!$O$6+Funnel!$O$7-$F$25-$F$32)*D6+(Funnel!$O$8-$F$26-$F$33)*E6+($F$25+$F$26)*X6+($F$32+$F$33)*Y6</f>
-        <v>54.0597133620274</v>
+        <v>54.0675635459762</v>
       </c>
       <c r="Q6" s="29" t="n">
         <f aca="false">Assumptions!$D$9*MAX(0,MIN(C6+Assumptions!$D$21,Funnel!$B$17)-MAX(IF(A6=1,Funnel!$B$13,B6+Assumptions!$D$21),Funnel!$B$13)+1)/7</f>
@@ -16742,7 +16777,7 @@
       </c>
       <c r="R6" s="30" t="n">
         <f aca="false">IF(Q6&gt;0,P6/Q6,IF(P6&gt;0,9.99,0))</f>
-        <v>0.98290387930959</v>
+        <v>0.98304660992684</v>
       </c>
       <c r="S6" s="2" t="str">
         <f aca="false">IF(P6&gt;Q6+0.5,"OVER "&amp;Assumptions!$D$9&amp;"/wk – pace down",IF(R6&gt;Assumptions!$D$102,"Full",IF(AND(Q6&gt;=Assumptions!$D$103,P6&lt;Assumptions!$D$103),"Under "&amp;Assumptions!$D$103&amp;" – release reserve","")))</f>
@@ -16811,7 +16846,7 @@
       </c>
       <c r="H7" s="41" t="n">
         <f aca="false">$F$19*D7+$F$20*E7+$F$31*Y7</f>
-        <v>14326.9408528645</v>
+        <v>14437.8183766273</v>
       </c>
       <c r="I7" s="41" t="n">
         <f aca="false">IF(A7=1,$F$21,0)</f>
@@ -16831,19 +16866,19 @@
       </c>
       <c r="M7" s="41" t="n">
         <f aca="false">SUM(H7:L7)</f>
-        <v>16794.2514778646</v>
+        <v>16905.1290016273</v>
       </c>
       <c r="N7" s="41" t="n">
         <f aca="false">SUM($M$4:M7)</f>
-        <v>77783.2325070381</v>
+        <v>78238.729361415</v>
       </c>
       <c r="O7" s="29" t="n">
         <f aca="false">(Funnel!$M$5+Funnel!$M$6+Funnel!$M$7-$F$27-$F$34)*D7+(Funnel!$M$8-$F$28-$F$35)*E7+($F$27+$F$28)*X7+($F$34+$F$35)*Y7</f>
-        <v>266.659317364271</v>
+        <v>267.436589815917</v>
       </c>
       <c r="P7" s="29" t="n">
         <f aca="false">(Funnel!$O$5+Funnel!$O$6+Funnel!$O$7-$F$25-$F$32)*D7+(Funnel!$O$8-$F$26-$F$33)*E7+($F$25+$F$26)*X7+($F$32+$F$33)*Y7</f>
-        <v>54.1300887331949</v>
+        <v>54.1381569778089</v>
       </c>
       <c r="Q7" s="29" t="n">
         <f aca="false">Assumptions!$D$9*MAX(0,MIN(C7+Assumptions!$D$21,Funnel!$B$17)-MAX(IF(A7=1,Funnel!$B$13,B7+Assumptions!$D$21),Funnel!$B$13)+1)/7</f>
@@ -16851,7 +16886,7 @@
       </c>
       <c r="R7" s="30" t="n">
         <f aca="false">IF(Q7&gt;0,P7/Q7,IF(P7&gt;0,9.99,0))</f>
-        <v>0.984183431512634</v>
+        <v>0.984330126869253</v>
       </c>
       <c r="S7" s="2" t="str">
         <f aca="false">IF(P7&gt;Q7+0.5,"OVER "&amp;Assumptions!$D$9&amp;"/wk – pace down",IF(R7&gt;Assumptions!$D$102,"Full",IF(AND(Q7&gt;=Assumptions!$D$103,P7&lt;Assumptions!$D$103),"Under "&amp;Assumptions!$D$103&amp;" – release reserve","")))</f>
@@ -16859,7 +16894,7 @@
       </c>
       <c r="T7" s="32" t="n">
         <f aca="false">$F$38*(F7*(Budget!$G$21+Budget!$G$22+Budget!$G$23-$F$29-$F$36)+IF(A7-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($X$4:$X$14,A7-ROUNDUP(Funnel!$B$15/7,0))*$F$29+INDEX($Y$4:$Y$14,A7-ROUNDUP(Funnel!$B$15/7,0))*$F$36,0))</f>
-        <v>24.3656358529994</v>
+        <v>24.3641121536279</v>
       </c>
       <c r="U7" s="32" t="n">
         <f aca="false">$F$38*(G7*(Budget!$G$24-$F$30-$F$37)+IF(A7-ROUNDUP(Funnel!$B$16/7,0)&gt;=1,INDEX($X$4:$X$14,A7-ROUNDUP(Funnel!$B$16/7,0))*$F$30+INDEX($Y$4:$Y$14,A7-ROUNDUP(Funnel!$B$16/7,0))*$F$37,0))</f>
@@ -16867,11 +16902,11 @@
       </c>
       <c r="V7" s="32" t="n">
         <f aca="false">T7+U7</f>
-        <v>24.3656358529994</v>
+        <v>24.3641121536279</v>
       </c>
       <c r="W7" s="32" t="n">
         <f aca="false">SUM($V$4:V7)</f>
-        <v>24.3656358529994</v>
+        <v>24.3641121536279</v>
       </c>
       <c r="X7" s="30" t="n">
         <f aca="false">IF(A7=1,Assumptions!$D$50,IF(A7=2,1-Assumptions!$D$50,0))</f>
@@ -16920,7 +16955,7 @@
       </c>
       <c r="H8" s="41" t="n">
         <f aca="false">$F$19*D8+$F$20*E8+$F$31*Y8</f>
-        <v>13821.5824640265</v>
+        <v>13940.6975137465</v>
       </c>
       <c r="I8" s="41" t="n">
         <f aca="false">IF(A8=1,$F$21,0)</f>
@@ -16940,19 +16975,19 @@
       </c>
       <c r="M8" s="41" t="n">
         <f aca="false">SUM(H8:L8)</f>
-        <v>15603.0921387216</v>
+        <v>15722.2071884416</v>
       </c>
       <c r="N8" s="41" t="n">
         <f aca="false">SUM($M$4:M8)</f>
-        <v>93386.3246457597</v>
+        <v>93960.9365498566</v>
       </c>
       <c r="O8" s="29" t="n">
         <f aca="false">(Funnel!$M$5+Funnel!$M$6+Funnel!$M$7-$F$27-$F$34)*D8+(Funnel!$M$8-$F$28-$F$35)*E8+($F$27+$F$28)*X8+($F$34+$F$35)*Y8</f>
-        <v>270.18156279478</v>
+        <v>270.983393875365</v>
       </c>
       <c r="P8" s="29" t="n">
         <f aca="false">(Funnel!$O$5+Funnel!$O$6+Funnel!$O$7-$F$25-$F$32)*D8+(Funnel!$O$8-$F$26-$F$33)*E8+($F$25+$F$26)*X8+($F$32+$F$33)*Y8</f>
-        <v>54.5327026287834</v>
+        <v>54.5398332456552</v>
       </c>
       <c r="Q8" s="29" t="n">
         <f aca="false">Assumptions!$D$9*MAX(0,MIN(C8+Assumptions!$D$21,Funnel!$B$17)-MAX(IF(A8=1,Funnel!$B$13,B8+Assumptions!$D$21),Funnel!$B$13)+1)/7</f>
@@ -16960,7 +16995,7 @@
       </c>
       <c r="R8" s="30" t="n">
         <f aca="false">IF(Q8&gt;0,P8/Q8,IF(P8&gt;0,9.99,0))</f>
-        <v>0.991503684159698</v>
+        <v>0.991633331739186</v>
       </c>
       <c r="S8" s="2" t="str">
         <f aca="false">IF(P8&gt;Q8+0.5,"OVER "&amp;Assumptions!$D$9&amp;"/wk – pace down",IF(R8&gt;Assumptions!$D$102,"Full",IF(AND(Q8&gt;=Assumptions!$D$103,P8&lt;Assumptions!$D$103),"Under "&amp;Assumptions!$D$103&amp;" – release reserve","")))</f>
@@ -16968,19 +17003,19 @@
       </c>
       <c r="T8" s="32" t="n">
         <f aca="false">$F$38*(F8*(Budget!$G$21+Budget!$G$22+Budget!$G$23-$F$29-$F$36)+IF(A8-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($X$4:$X$14,A8-ROUNDUP(Funnel!$B$15/7,0))*$F$29+INDEX($Y$4:$Y$14,A8-ROUNDUP(Funnel!$B$15/7,0))*$F$36,0))</f>
-        <v>14.9480606707648</v>
+        <v>14.9434387826712</v>
       </c>
       <c r="U8" s="32" t="n">
         <f aca="false">$F$38*(G8*(Budget!$G$24-$F$30-$F$37)+IF(A8-ROUNDUP(Funnel!$B$16/7,0)&gt;=1,INDEX($X$4:$X$14,A8-ROUNDUP(Funnel!$B$16/7,0))*$F$30+INDEX($Y$4:$Y$14,A8-ROUNDUP(Funnel!$B$16/7,0))*$F$37,0))</f>
-        <v>3.37600787400241</v>
+        <v>3.37581560318138</v>
       </c>
       <c r="V8" s="32" t="n">
         <f aca="false">T8+U8</f>
-        <v>18.3240685447672</v>
+        <v>18.3192543858526</v>
       </c>
       <c r="W8" s="32" t="n">
         <f aca="false">SUM($V$4:V8)</f>
-        <v>42.6897043977666</v>
+        <v>42.6833665394805</v>
       </c>
       <c r="X8" s="30" t="n">
         <f aca="false">IF(A8=1,Assumptions!$D$50,IF(A8=2,1-Assumptions!$D$50,0))</f>
@@ -17029,7 +17064,7 @@
       </c>
       <c r="H9" s="41" t="n">
         <f aca="false">$F$19*D9+$F$20*E9+$F$31*Y9</f>
-        <v>1552.34202886533</v>
+        <v>1566.003805712</v>
       </c>
       <c r="I9" s="41" t="n">
         <f aca="false">IF(A9=1,$F$21,0)</f>
@@ -17049,19 +17084,19 @@
       </c>
       <c r="M9" s="41" t="n">
         <f aca="false">SUM(H9:L9)</f>
-        <v>3532.0779959385</v>
+        <v>3545.73977278518</v>
       </c>
       <c r="N9" s="41" t="n">
         <f aca="false">SUM($M$4:M9)</f>
-        <v>96918.4026416982</v>
+        <v>97506.6763226418</v>
       </c>
       <c r="O9" s="29" t="n">
         <f aca="false">(Funnel!$M$5+Funnel!$M$6+Funnel!$M$7-$F$27-$F$34)*D9+(Funnel!$M$8-$F$28-$F$35)*E9+($F$27+$F$28)*X9+($F$34+$F$35)*Y9</f>
-        <v>30.6466971072619</v>
+        <v>30.7379665051514</v>
       </c>
       <c r="P9" s="29" t="n">
         <f aca="false">(Funnel!$O$5+Funnel!$O$6+Funnel!$O$7-$F$25-$F$32)*D9+(Funnel!$O$8-$F$26-$F$33)*E9+($F$25+$F$26)*X9+($F$32+$F$33)*Y9</f>
-        <v>6.17870111320319</v>
+        <v>6.17948672772832</v>
       </c>
       <c r="Q9" s="29" t="n">
         <f aca="false">Assumptions!$D$9*MAX(0,MIN(C9+Assumptions!$D$21,Funnel!$B$17)-MAX(IF(A9=1,Funnel!$B$13,B9+Assumptions!$D$21),Funnel!$B$13)+1)/7</f>
@@ -17069,7 +17104,7 @@
       </c>
       <c r="R9" s="30" t="n">
         <f aca="false">IF(Q9&gt;0,P9/Q9,IF(P9&gt;0,9.99,0))</f>
-        <v>0.786380141680406</v>
+        <v>0.786480128983605</v>
       </c>
       <c r="S9" s="2" t="str">
         <f aca="false">IF(P9&gt;Q9+0.5,"OVER "&amp;Assumptions!$D$9&amp;"/wk – pace down",IF(R9&gt;Assumptions!$D$102,"Full",IF(AND(Q9&gt;=Assumptions!$D$103,P9&lt;Assumptions!$D$103),"Under "&amp;Assumptions!$D$103&amp;" – release reserve","")))</f>
@@ -17077,19 +17112,19 @@
       </c>
       <c r="T9" s="32" t="n">
         <f aca="false">$F$38*(F9*(Budget!$G$21+Budget!$G$22+Budget!$G$23-$F$29-$F$36)+IF(A9-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($X$4:$X$14,A9-ROUNDUP(Funnel!$B$15/7,0))*$F$29+INDEX($Y$4:$Y$14,A9-ROUNDUP(Funnel!$B$15/7,0))*$F$36,0))</f>
-        <v>15.3972684264007</v>
+        <v>15.3990968656466</v>
       </c>
       <c r="U9" s="32" t="n">
         <f aca="false">$F$38*(G9*(Budget!$G$24-$F$30-$F$37)+IF(A9-ROUNDUP(Funnel!$B$16/7,0)&gt;=1,INDEX($X$4:$X$14,A9-ROUNDUP(Funnel!$B$16/7,0))*$F$30+INDEX($Y$4:$Y$14,A9-ROUNDUP(Funnel!$B$16/7,0))*$F$37,0))</f>
-        <v>2.21362762346889</v>
+        <v>2.2126720706385</v>
       </c>
       <c r="V9" s="32" t="n">
         <f aca="false">T9+U9</f>
-        <v>17.6108960498696</v>
+        <v>17.6117689362851</v>
       </c>
       <c r="W9" s="32" t="n">
         <f aca="false">SUM($V$4:V9)</f>
-        <v>60.3006004476362</v>
+        <v>60.2951354757655</v>
       </c>
       <c r="X9" s="30" t="n">
         <f aca="false">IF(A9=1,Assumptions!$D$50,IF(A9=2,1-Assumptions!$D$50,0))</f>
@@ -17162,7 +17197,7 @@
       </c>
       <c r="N10" s="41" t="n">
         <f aca="false">SUM($M$4:M10)</f>
-        <v>98996.5505529787</v>
+        <v>99584.8242339222</v>
       </c>
       <c r="O10" s="29" t="n">
         <f aca="false">(Funnel!$M$5+Funnel!$M$6+Funnel!$M$7-$F$27-$F$34)*D10+(Funnel!$M$8-$F$28-$F$35)*E10+($F$27+$F$28)*X10+($F$34+$F$35)*Y10</f>
@@ -17186,19 +17221,19 @@
       </c>
       <c r="T10" s="32" t="n">
         <f aca="false">$F$38*(F10*(Budget!$G$21+Budget!$G$22+Budget!$G$23-$F$29-$F$36)+IF(A10-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($X$4:$X$14,A10-ROUNDUP(Funnel!$B$15/7,0))*$F$29+INDEX($Y$4:$Y$14,A10-ROUNDUP(Funnel!$B$15/7,0))*$F$36,0))</f>
-        <v>15.3611093746341</v>
+        <v>15.362988603859</v>
       </c>
       <c r="U10" s="32" t="n">
         <f aca="false">$F$38*(G10*(Budget!$G$24-$F$30-$F$37)+IF(A10-ROUNDUP(Funnel!$B$16/7,0)&gt;=1,INDEX($X$4:$X$14,A10-ROUNDUP(Funnel!$B$16/7,0))*$F$30+INDEX($Y$4:$Y$14,A10-ROUNDUP(Funnel!$B$16/7,0))*$F$37,0))</f>
-        <v>2.03766985111414</v>
+        <v>2.03819196584367</v>
       </c>
       <c r="V10" s="32" t="n">
         <f aca="false">T10+U10</f>
-        <v>17.3987792257482</v>
+        <v>17.4011805697026</v>
       </c>
       <c r="W10" s="32" t="n">
         <f aca="false">SUM($V$4:V10)</f>
-        <v>77.6993796733844</v>
+        <v>77.6963160454681</v>
       </c>
       <c r="X10" s="30" t="n">
         <f aca="false">IF(A10=1,Assumptions!$D$50,IF(A10=2,1-Assumptions!$D$50,0))</f>
@@ -17271,7 +17306,7 @@
       </c>
       <c r="N11" s="41" t="n">
         <f aca="false">SUM($M$4:M11)</f>
-        <v>101377.785129503</v>
+        <v>101966.058810447</v>
       </c>
       <c r="O11" s="29" t="n">
         <f aca="false">(Funnel!$M$5+Funnel!$M$6+Funnel!$M$7-$F$27-$F$34)*D11+(Funnel!$M$8-$F$28-$F$35)*E11+($F$27+$F$28)*X11+($F$34+$F$35)*Y11</f>
@@ -17295,19 +17330,19 @@
       </c>
       <c r="T11" s="32" t="n">
         <f aca="false">$F$38*(F11*(Budget!$G$21+Budget!$G$22+Budget!$G$23-$F$29-$F$36)+IF(A11-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($X$4:$X$14,A11-ROUNDUP(Funnel!$B$15/7,0))*$F$29+INDEX($Y$4:$Y$14,A11-ROUNDUP(Funnel!$B$15/7,0))*$F$36,0))</f>
-        <v>17.8521000840342</v>
+        <v>17.8542840531334</v>
       </c>
       <c r="U11" s="32" t="n">
         <f aca="false">$F$38*(G11*(Budget!$G$24-$F$30-$F$37)+IF(A11-ROUNDUP(Funnel!$B$16/7,0)&gt;=1,INDEX($X$4:$X$14,A11-ROUNDUP(Funnel!$B$16/7,0))*$F$30+INDEX($Y$4:$Y$14,A11-ROUNDUP(Funnel!$B$16/7,0))*$F$37,0))</f>
-        <v>2.0348606447562</v>
+        <v>2.03539726267266</v>
       </c>
       <c r="V11" s="32" t="n">
         <f aca="false">T11+U11</f>
-        <v>19.8869607287904</v>
+        <v>19.889681315806</v>
       </c>
       <c r="W11" s="32" t="n">
         <f aca="false">SUM($V$4:V11)</f>
-        <v>97.5863404021749</v>
+        <v>97.5859973612742</v>
       </c>
       <c r="X11" s="30" t="n">
         <f aca="false">IF(A11=1,Assumptions!$D$50,IF(A11=2,1-Assumptions!$D$50,0))</f>
@@ -17380,7 +17415,7 @@
       </c>
       <c r="N12" s="41" t="n">
         <f aca="false">SUM($M$4:M12)</f>
-        <v>101667.57387493</v>
+        <v>102255.847555873</v>
       </c>
       <c r="O12" s="29" t="n">
         <f aca="false">(Funnel!$M$5+Funnel!$M$6+Funnel!$M$7-$F$27-$F$34)*D12+(Funnel!$M$8-$F$28-$F$35)*E12+($F$27+$F$28)*X12+($F$34+$F$35)*Y12</f>
@@ -17404,15 +17439,15 @@
       </c>
       <c r="T12" s="32" t="n">
         <f aca="false">$F$38*(F12*(Budget!$G$21+Budget!$G$22+Budget!$G$23-$F$29-$F$36)+IF(A12-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($X$4:$X$14,A12-ROUNDUP(Funnel!$B$15/7,0))*$F$29+INDEX($Y$4:$Y$14,A12-ROUNDUP(Funnel!$B$15/7,0))*$F$36,0))</f>
-        <v>2.07582559116677</v>
+        <v>2.07607954106202</v>
       </c>
       <c r="U12" s="32" t="n">
         <f aca="false">$F$38*(G12*(Budget!$G$24-$F$30-$F$37)+IF(A12-ROUNDUP(Funnel!$B$16/7,0)&gt;=1,INDEX($X$4:$X$14,A12-ROUNDUP(Funnel!$B$16/7,0))*$F$30+INDEX($Y$4:$Y$14,A12-ROUNDUP(Funnel!$B$16/7,0))*$F$37,0))</f>
-        <v>0.337834006658365</v>
+        <v>0.3379230976638</v>
       </c>
       <c r="V12" s="32" t="n">
         <f aca="false">T12+U12</f>
-        <v>2.41365959782514</v>
+        <v>2.41400263872582</v>
       </c>
       <c r="W12" s="32" t="n">
         <f aca="false">SUM($V$4:V12)</f>
@@ -17489,7 +17524,7 @@
       </c>
       <c r="N13" s="41" t="n">
         <f aca="false">SUM($M$4:M13)</f>
-        <v>101667.57387493</v>
+        <v>102255.847555873</v>
       </c>
       <c r="O13" s="29" t="n">
         <f aca="false">(Funnel!$M$5+Funnel!$M$6+Funnel!$M$7-$F$27-$F$34)*D13+(Funnel!$M$8-$F$28-$F$35)*E13+($F$27+$F$28)*X13+($F$34+$F$35)*Y13</f>
@@ -17598,7 +17633,7 @@
       </c>
       <c r="N14" s="41" t="n">
         <f aca="false">SUM($M$4:M14)</f>
-        <v>101667.57387493</v>
+        <v>102255.847555873</v>
       </c>
       <c r="O14" s="29" t="n">
         <f aca="false">(Funnel!$M$5+Funnel!$M$6+Funnel!$M$7-$F$27-$F$34)*D14+(Funnel!$M$8-$F$28-$F$35)*E14+($F$27+$F$28)*X14+($F$34+$F$35)*Y14</f>
@@ -17675,7 +17710,7 @@
       </c>
       <c r="H15" s="42" t="n">
         <f aca="false">SUM(H4:H14)</f>
-        <v>74293.8463749299</v>
+        <v>74882.1200558735</v>
       </c>
       <c r="I15" s="42" t="n">
         <f aca="false">SUM(I4:I14)</f>
@@ -17695,11 +17730,11 @@
       </c>
       <c r="M15" s="42" t="n">
         <f aca="false">SUM(M4:M14)</f>
-        <v>101667.57387493</v>
+        <v>102255.847555873</v>
       </c>
       <c r="O15" s="35" t="n">
         <f aca="false">SUM(O4:O14)</f>
-        <v>1490.4890234349</v>
+        <v>1494.5752431742</v>
       </c>
       <c r="P15" s="35" t="n">
         <f aca="false">SUM(P4:P14)</f>
@@ -17801,7 +17836,7 @@
       </c>
       <c r="F19" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot",Channels!$B$5:$B$34,"&lt;&gt;I1b Employee referral sprint (bonus on hire)",Channels!$B$5:$B$34,"&lt;&gt;I1a Talent rediscovery (past applicants in ATS)")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
-        <v>62093.681154613</v>
+        <v>62640.1522284802</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17810,7 +17845,7 @@
       </c>
       <c r="F20" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot",Channels!$B$5:$B$34,"&lt;&gt;I1b Employee referral sprint (bonus on hire)",Channels!$B$5:$B$34,"&lt;&gt;I1a Talent rediscovery (past applicants in ATS)")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$C$5:$C$34,"Supervisors")</f>
-        <v>12136.8652203169</v>
+        <v>12178.6678273933</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17855,7 +17890,7 @@
       </c>
       <c r="F25" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$AF$5:$AF$34,Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
-        <v>8.96372483214199</v>
+        <v>8.9323002511364</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17864,7 +17899,7 @@
       </c>
       <c r="F26" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$AF$5:$AF$34,Channels!$C$5:$C$34,"Supervisors")</f>
-        <v>3.26569109138069</v>
+        <v>3.25605421987231</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17891,7 +17926,7 @@
       </c>
       <c r="F29" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$AG$5:$AG$34,Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
-        <v>2.86402935332918</v>
+        <v>2.85387135751913</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17900,7 +17935,7 @@
       </c>
       <c r="F30" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$AG$5:$AG$34,Channels!$C$5:$C$34,"Supervisors")</f>
-        <v>0.777234479748603</v>
+        <v>0.774940904329609</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18083,27 +18118,27 @@
       </c>
       <c r="C45" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$4+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"Supervisors"))*$E$4+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45)*$X$4+SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$E$5:$E$34,"Slot")+SUMIFS(Channels!$Y$5:$Y$34,Channels!$B$5:$B$34,$B45)</f>
-        <v>9247.28220604556</v>
+        <v>9368.64932274326</v>
       </c>
       <c r="D45" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$5+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"Supervisors"))*$E$5+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45)*$X$5</f>
-        <v>6467.42367950642</v>
+        <v>6537.81660719109</v>
       </c>
       <c r="E45" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$6+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"Supervisors"))*$E$6+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45)*$X$6</f>
-        <v>5794.0431883528</v>
+        <v>5881.42751237515</v>
       </c>
       <c r="F45" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$7+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"Supervisors"))*$E$7+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45)*$X$7</f>
-        <v>5954.98883247371</v>
+        <v>6044.80049883001</v>
       </c>
       <c r="G45" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$8+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"Supervisors"))*$E$8+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45)*$X$8</f>
-        <v>6920.66269719918</v>
+        <v>7025.0384175592</v>
       </c>
       <c r="H45" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$9+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"Supervisors"))*$E$9+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45)*$X$9</f>
-        <v>804.728220604556</v>
+        <v>816.864932274326</v>
       </c>
       <c r="I45" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$10+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"Supervisors"))*$E$10+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45)*$X$10</f>
@@ -18127,7 +18162,7 @@
       </c>
       <c r="N45" s="42" t="n">
         <f aca="false">SUM(C45:M45)</f>
-        <v>35189.1288241822</v>
+        <v>35674.597290973</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18191,27 +18226,27 @@
       </c>
       <c r="C47" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$4+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"Supervisors"))*$E$4+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47)*$X$4+SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$E$5:$E$34,"Slot")+SUMIFS(Channels!$Y$5:$Y$34,Channels!$B$5:$B$34,$B47)</f>
-        <v>7812.07205282721</v>
+        <v>7840.53942770084</v>
       </c>
       <c r="D47" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$5+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"Supervisors"))*$E$5+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47)*$X$5</f>
-        <v>5083.00179063978</v>
+        <v>5099.51286806649</v>
       </c>
       <c r="E47" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$6+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"Supervisors"))*$E$6+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47)*$X$6</f>
-        <v>5192.69187803559</v>
+        <v>5213.1883879446</v>
       </c>
       <c r="F47" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$7+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"Supervisors"))*$E$7+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47)*$X$7</f>
-        <v>5336.93331909214</v>
+        <v>5357.99917649862</v>
       </c>
       <c r="G47" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$8+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"Supervisors"))*$E$8+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47)*$X$8</f>
-        <v>3373.73587072339</v>
+        <v>3388.47520008336</v>
       </c>
       <c r="H47" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$9+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"Supervisors"))*$E$9+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47)*$X$9</f>
-        <v>337.476145923107</v>
+        <v>339.001211100016</v>
       </c>
       <c r="I47" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$10+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"Supervisors"))*$E$10+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47)*$X$10</f>
@@ -18235,7 +18270,7 @@
       </c>
       <c r="N47" s="42" t="n">
         <f aca="false">SUM(C47:M47)</f>
-        <v>27135.9110572412</v>
+        <v>27238.7162713939</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18568,27 +18603,27 @@
       </c>
       <c r="C54" s="42" t="n">
         <f aca="false">SUM(C44:C53)</f>
-        <v>30394.7108822494</v>
+        <v>30544.5453738207</v>
       </c>
       <c r="D54" s="42" t="n">
         <f aca="false">SUM(D44:D53)</f>
-        <v>16647.5809117046</v>
+        <v>16734.484916816</v>
       </c>
       <c r="E54" s="42" t="n">
         <f aca="false">SUM(E44:E53)</f>
-        <v>13946.6892352196</v>
+        <v>14054.5700691509</v>
       </c>
       <c r="F54" s="42" t="n">
         <f aca="false">SUM(F44:F53)</f>
-        <v>16794.2514778646</v>
+        <v>16905.1290016273</v>
       </c>
       <c r="G54" s="42" t="n">
         <f aca="false">SUM(G44:G53)</f>
-        <v>15603.0921387216</v>
+        <v>15722.2071884416</v>
       </c>
       <c r="H54" s="42" t="n">
         <f aca="false">SUM(H44:H53)</f>
-        <v>3532.0779959385</v>
+        <v>3545.73977278518</v>
       </c>
       <c r="I54" s="42" t="n">
         <f aca="false">SUM(I44:I53)</f>
@@ -18612,7 +18647,7 @@
       </c>
       <c r="N54" s="42" t="n">
         <f aca="false">SUM(N44:N53)</f>
-        <v>101667.57387493</v>
+        <v>102255.847555873</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18641,15 +18676,15 @@
     <tabColor rgb="FF70AD47"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:X48"/>
+  <dimension ref="A1:AA48"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="40"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="4" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="27" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="4" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="25" style="0" width="10"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18735,6 +18770,15 @@
       <c r="X4" s="12" t="s">
         <v>750</v>
       </c>
+      <c r="Y4" s="12" t="s">
+        <v>751</v>
+      </c>
+      <c r="Z4" s="12" t="s">
+        <v>752</v>
+      </c>
+      <c r="AA4" s="12" t="s">
+        <v>753</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="str">
@@ -18755,7 +18799,7 @@
       </c>
       <c r="E5" s="30" t="n">
         <f aca="false">Channels!I5</f>
-        <v>0.1775</v>
+        <v>0.175</v>
       </c>
       <c r="F5" s="41" t="n">
         <f aca="false">Channels!O5</f>
@@ -18792,7 +18836,7 @@
       </c>
       <c r="U5" s="30" t="n">
         <f aca="false">IF(AND(OR(P5&gt;=Assumptions!$D$83,Q5&gt;=Assumptions!$D$84),R5&gt;0),R5/Q5,E5)</f>
-        <v>0.1775</v>
+        <v>0.175</v>
       </c>
       <c r="V5" s="41" t="n">
         <f aca="false">IF(U5&gt;0,IF(AND(OR(P5&gt;=Assumptions!$D$83,Q5&gt;=Assumptions!$D$84),Q5&gt;0),S5,D5)/U5,0)</f>
@@ -18803,8 +18847,17 @@
         <v/>
       </c>
       <c r="X5" s="2" t="str">
-        <f aca="false">IF(D5=0,"Free – monitor quality",IF(F5=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P5&lt;Assumptions!$D$83,Q5&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W5&gt;=Assumptions!$D$87,AND(R5=0,P5&gt;=Assumptions!$D$88)),"SWITCH OFF",IF(W5&gt;=Assumptions!$D$86,"CUT 50%",IF(W5&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
+        <f aca="false">IF(D5=0,"Free – monitor quality",IF(F5=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P5&lt;Assumptions!$D$83,Q5&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W5&gt;=Assumptions!$D$87,AND(R5=0,P5&gt;=Assumptions!$D$88,Q5&gt;=Assumptions!$D$84)),"SWITCH OFF",IF(W5&gt;=Assumptions!$D$86,"CUT 50%",IF(W5&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Free – monitor quality</v>
+      </c>
+      <c r="Y5" s="15"/>
+      <c r="Z5" s="41" t="str">
+        <f aca="false">IF(Y5&gt;0,P5/Y5,"")</f>
+        <v/>
+      </c>
+      <c r="AA5" s="32" t="n">
+        <f aca="false">Channels!U5</f>
+        <v>5.788125</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18826,7 +18879,7 @@
       </c>
       <c r="E6" s="30" t="n">
         <f aca="false">Channels!I6</f>
-        <v>0.1775</v>
+        <v>0.175</v>
       </c>
       <c r="F6" s="41" t="n">
         <f aca="false">Channels!O6</f>
@@ -18863,7 +18916,7 @@
       </c>
       <c r="U6" s="30" t="n">
         <f aca="false">IF(AND(OR(P6&gt;=Assumptions!$D$83,Q6&gt;=Assumptions!$D$84),R6&gt;0),R6/Q6,E6)</f>
-        <v>0.1775</v>
+        <v>0.175</v>
       </c>
       <c r="V6" s="41" t="n">
         <f aca="false">IF(U6&gt;0,IF(AND(OR(P6&gt;=Assumptions!$D$83,Q6&gt;=Assumptions!$D$84),Q6&gt;0),S6,D6)/U6,0)</f>
@@ -18874,8 +18927,17 @@
         <v/>
       </c>
       <c r="X6" s="2" t="str">
-        <f aca="false">IF(D6=0,"Free – monitor quality",IF(F6=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P6&lt;Assumptions!$D$83,Q6&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W6&gt;=Assumptions!$D$87,AND(R6=0,P6&gt;=Assumptions!$D$88)),"SWITCH OFF",IF(W6&gt;=Assumptions!$D$86,"CUT 50%",IF(W6&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
+        <f aca="false">IF(D6=0,"Free – monitor quality",IF(F6=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P6&lt;Assumptions!$D$83,Q6&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W6&gt;=Assumptions!$D$87,AND(R6=0,P6&gt;=Assumptions!$D$88,Q6&gt;=Assumptions!$D$84)),"SWITCH OFF",IF(W6&gt;=Assumptions!$D$86,"CUT 50%",IF(W6&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Free – monitor quality</v>
+      </c>
+      <c r="Y6" s="15"/>
+      <c r="Z6" s="41" t="str">
+        <f aca="false">IF(Y6&gt;0,P6/Y6,"")</f>
+        <v/>
+      </c>
+      <c r="AA6" s="32" t="n">
+        <f aca="false">Channels!U6</f>
+        <v>10.2650625</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18897,7 +18959,7 @@
       </c>
       <c r="E7" s="30" t="n">
         <f aca="false">Channels!I7</f>
-        <v>0.1775</v>
+        <v>0.175</v>
       </c>
       <c r="F7" s="41" t="n">
         <f aca="false">Channels!O7</f>
@@ -18934,7 +18996,7 @@
       </c>
       <c r="U7" s="30" t="n">
         <f aca="false">IF(AND(OR(P7&gt;=Assumptions!$D$83,Q7&gt;=Assumptions!$D$84),R7&gt;0),R7/Q7,E7)</f>
-        <v>0.1775</v>
+        <v>0.175</v>
       </c>
       <c r="V7" s="41" t="n">
         <f aca="false">IF(U7&gt;0,IF(AND(OR(P7&gt;=Assumptions!$D$83,Q7&gt;=Assumptions!$D$84),Q7&gt;0),S7,D7)/U7,0)</f>
@@ -18945,8 +19007,17 @@
         <v/>
       </c>
       <c r="X7" s="2" t="str">
-        <f aca="false">IF(D7=0,"Free – monitor quality",IF(F7=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P7&lt;Assumptions!$D$83,Q7&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W7&gt;=Assumptions!$D$87,AND(R7=0,P7&gt;=Assumptions!$D$88)),"SWITCH OFF",IF(W7&gt;=Assumptions!$D$86,"CUT 50%",IF(W7&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
+        <f aca="false">IF(D7=0,"Free – monitor quality",IF(F7=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P7&lt;Assumptions!$D$83,Q7&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W7&gt;=Assumptions!$D$87,AND(R7=0,P7&gt;=Assumptions!$D$88,Q7&gt;=Assumptions!$D$84)),"SWITCH OFF",IF(W7&gt;=Assumptions!$D$86,"CUT 50%",IF(W7&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Free – monitor quality</v>
+      </c>
+      <c r="Y7" s="15"/>
+      <c r="Z7" s="41" t="str">
+        <f aca="false">IF(Y7&gt;0,P7/Y7,"")</f>
+        <v/>
+      </c>
+      <c r="AA7" s="32" t="n">
+        <f aca="false">Channels!U7</f>
+        <v>2.6294625</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18968,7 +19039,7 @@
       </c>
       <c r="E8" s="30" t="n">
         <f aca="false">Channels!I8</f>
-        <v>0.1633</v>
+        <v>0.161</v>
       </c>
       <c r="F8" s="41" t="n">
         <f aca="false">Channels!O8</f>
@@ -19005,7 +19076,7 @@
       </c>
       <c r="U8" s="30" t="n">
         <f aca="false">IF(AND(OR(P8&gt;=Assumptions!$D$83,Q8&gt;=Assumptions!$D$84),R8&gt;0),R8/Q8,E8)</f>
-        <v>0.1633</v>
+        <v>0.161</v>
       </c>
       <c r="V8" s="41" t="n">
         <f aca="false">IF(U8&gt;0,IF(AND(OR(P8&gt;=Assumptions!$D$83,Q8&gt;=Assumptions!$D$84),Q8&gt;0),S8,D8)/U8,0)</f>
@@ -19016,8 +19087,17 @@
         <v/>
       </c>
       <c r="X8" s="2" t="str">
-        <f aca="false">IF(D8=0,"Free – monitor quality",IF(F8=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P8&lt;Assumptions!$D$83,Q8&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W8&gt;=Assumptions!$D$87,AND(R8=0,P8&gt;=Assumptions!$D$88)),"SWITCH OFF",IF(W8&gt;=Assumptions!$D$86,"CUT 50%",IF(W8&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
+        <f aca="false">IF(D8=0,"Free – monitor quality",IF(F8=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P8&lt;Assumptions!$D$83,Q8&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W8&gt;=Assumptions!$D$87,AND(R8=0,P8&gt;=Assumptions!$D$88,Q8&gt;=Assumptions!$D$84)),"SWITCH OFF",IF(W8&gt;=Assumptions!$D$86,"CUT 50%",IF(W8&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Free – monitor quality</v>
+      </c>
+      <c r="Y8" s="15"/>
+      <c r="Z8" s="41" t="str">
+        <f aca="false">IF(Y8&gt;0,P8/Y8,"")</f>
+        <v/>
+      </c>
+      <c r="AA8" s="32" t="n">
+        <f aca="false">Channels!U8</f>
+        <v>1.34113</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19087,8 +19167,17 @@
         <v>1</v>
       </c>
       <c r="X9" s="2" t="str">
-        <f aca="false">IF(D9=0,"Free – monitor quality",IF(F9=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P9&lt;Assumptions!$D$83,Q9&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W9&gt;=Assumptions!$D$87,AND(R9=0,P9&gt;=Assumptions!$D$88)),"SWITCH OFF",IF(W9&gt;=Assumptions!$D$86,"CUT 50%",IF(W9&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
+        <f aca="false">IF(D9=0,"Free – monitor quality",IF(F9=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P9&lt;Assumptions!$D$83,Q9&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W9&gt;=Assumptions!$D$87,AND(R9=0,P9&gt;=Assumptions!$D$88,Q9&gt;=Assumptions!$D$84)),"SWITCH OFF",IF(W9&gt;=Assumptions!$D$86,"CUT 50%",IF(W9&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
+      </c>
+      <c r="Y9" s="15"/>
+      <c r="Z9" s="41" t="str">
+        <f aca="false">IF(Y9&gt;0,P9/Y9,"")</f>
+        <v/>
+      </c>
+      <c r="AA9" s="32" t="n">
+        <f aca="false">Channels!U9</f>
+        <v>8.95534807960894</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19158,8 +19247,17 @@
         <v>1</v>
       </c>
       <c r="X10" s="2" t="str">
-        <f aca="false">IF(D10=0,"Free – monitor quality",IF(F10=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P10&lt;Assumptions!$D$83,Q10&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W10&gt;=Assumptions!$D$87,AND(R10=0,P10&gt;=Assumptions!$D$88)),"SWITCH OFF",IF(W10&gt;=Assumptions!$D$86,"CUT 50%",IF(W10&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
+        <f aca="false">IF(D10=0,"Free – monitor quality",IF(F10=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P10&lt;Assumptions!$D$83,Q10&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W10&gt;=Assumptions!$D$87,AND(R10=0,P10&gt;=Assumptions!$D$88,Q10&gt;=Assumptions!$D$84)),"SWITCH OFF",IF(W10&gt;=Assumptions!$D$86,"CUT 50%",IF(W10&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
+      </c>
+      <c r="Y10" s="15"/>
+      <c r="Z10" s="41" t="str">
+        <f aca="false">IF(Y10&gt;0,P10/Y10,"")</f>
+        <v/>
+      </c>
+      <c r="AA10" s="32" t="n">
+        <f aca="false">Channels!U10</f>
+        <v>7.17620827239625</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19229,8 +19327,17 @@
         <v>1</v>
       </c>
       <c r="X11" s="2" t="str">
-        <f aca="false">IF(D11=0,"Free – monitor quality",IF(F11=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P11&lt;Assumptions!$D$83,Q11&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W11&gt;=Assumptions!$D$87,AND(R11=0,P11&gt;=Assumptions!$D$88)),"SWITCH OFF",IF(W11&gt;=Assumptions!$D$86,"CUT 50%",IF(W11&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
+        <f aca="false">IF(D11=0,"Free – monitor quality",IF(F11=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P11&lt;Assumptions!$D$83,Q11&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W11&gt;=Assumptions!$D$87,AND(R11=0,P11&gt;=Assumptions!$D$88,Q11&gt;=Assumptions!$D$84)),"SWITCH OFF",IF(W11&gt;=Assumptions!$D$86,"CUT 50%",IF(W11&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
+      </c>
+      <c r="Y11" s="15"/>
+      <c r="Z11" s="41" t="str">
+        <f aca="false">IF(Y11&gt;0,P11/Y11,"")</f>
+        <v/>
+      </c>
+      <c r="AA11" s="32" t="n">
+        <f aca="false">Channels!U11</f>
+        <v>0.297146739130435</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19300,8 +19407,17 @@
         <v>1</v>
       </c>
       <c r="X12" s="2" t="str">
-        <f aca="false">IF(D12=0,"Free – monitor quality",IF(F12=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P12&lt;Assumptions!$D$83,Q12&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W12&gt;=Assumptions!$D$87,AND(R12=0,P12&gt;=Assumptions!$D$88)),"SWITCH OFF",IF(W12&gt;=Assumptions!$D$86,"CUT 50%",IF(W12&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
+        <f aca="false">IF(D12=0,"Free – monitor quality",IF(F12=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P12&lt;Assumptions!$D$83,Q12&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W12&gt;=Assumptions!$D$87,AND(R12=0,P12&gt;=Assumptions!$D$88,Q12&gt;=Assumptions!$D$84)),"SWITCH OFF",IF(W12&gt;=Assumptions!$D$86,"CUT 50%",IF(W12&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
+      </c>
+      <c r="Y12" s="15"/>
+      <c r="Z12" s="41" t="str">
+        <f aca="false">IF(Y12&gt;0,P12/Y12,"")</f>
+        <v/>
+      </c>
+      <c r="AA12" s="32" t="n">
+        <f aca="false">Channels!U12</f>
+        <v>0.2295</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19371,8 +19487,17 @@
         <v>1</v>
       </c>
       <c r="X13" s="2" t="str">
-        <f aca="false">IF(D13=0,"Free – monitor quality",IF(F13=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P13&lt;Assumptions!$D$83,Q13&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W13&gt;=Assumptions!$D$87,AND(R13=0,P13&gt;=Assumptions!$D$88)),"SWITCH OFF",IF(W13&gt;=Assumptions!$D$86,"CUT 50%",IF(W13&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
+        <f aca="false">IF(D13=0,"Free – monitor quality",IF(F13=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P13&lt;Assumptions!$D$83,Q13&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W13&gt;=Assumptions!$D$87,AND(R13=0,P13&gt;=Assumptions!$D$88,Q13&gt;=Assumptions!$D$84)),"SWITCH OFF",IF(W13&gt;=Assumptions!$D$86,"CUT 50%",IF(W13&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
+      </c>
+      <c r="Y13" s="15"/>
+      <c r="Z13" s="41" t="str">
+        <f aca="false">IF(Y13&gt;0,P13/Y13,"")</f>
+        <v/>
+      </c>
+      <c r="AA13" s="32" t="n">
+        <f aca="false">Channels!U13</f>
+        <v>1.701</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19442,8 +19567,17 @@
         <v>1</v>
       </c>
       <c r="X14" s="2" t="str">
-        <f aca="false">IF(D14=0,"Free – monitor quality",IF(F14=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P14&lt;Assumptions!$D$83,Q14&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W14&gt;=Assumptions!$D$87,AND(R14=0,P14&gt;=Assumptions!$D$88)),"SWITCH OFF",IF(W14&gt;=Assumptions!$D$86,"CUT 50%",IF(W14&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
+        <f aca="false">IF(D14=0,"Free – monitor quality",IF(F14=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P14&lt;Assumptions!$D$83,Q14&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W14&gt;=Assumptions!$D$87,AND(R14=0,P14&gt;=Assumptions!$D$88,Q14&gt;=Assumptions!$D$84)),"SWITCH OFF",IF(W14&gt;=Assumptions!$D$86,"CUT 50%",IF(W14&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
+      </c>
+      <c r="Y14" s="15"/>
+      <c r="Z14" s="41" t="str">
+        <f aca="false">IF(Y14&gt;0,P14/Y14,"")</f>
+        <v/>
+      </c>
+      <c r="AA14" s="32" t="n">
+        <f aca="false">Channels!U14</f>
+        <v>2.00475</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19513,8 +19647,17 @@
         <v>1</v>
       </c>
       <c r="X15" s="2" t="str">
-        <f aca="false">IF(D15=0,"Free – monitor quality",IF(F15=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P15&lt;Assumptions!$D$83,Q15&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W15&gt;=Assumptions!$D$87,AND(R15=0,P15&gt;=Assumptions!$D$88)),"SWITCH OFF",IF(W15&gt;=Assumptions!$D$86,"CUT 50%",IF(W15&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
+        <f aca="false">IF(D15=0,"Free – monitor quality",IF(F15=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P15&lt;Assumptions!$D$83,Q15&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W15&gt;=Assumptions!$D$87,AND(R15=0,P15&gt;=Assumptions!$D$88,Q15&gt;=Assumptions!$D$84)),"SWITCH OFF",IF(W15&gt;=Assumptions!$D$86,"CUT 50%",IF(W15&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
+      </c>
+      <c r="Y15" s="15"/>
+      <c r="Z15" s="41" t="str">
+        <f aca="false">IF(Y15&gt;0,P15/Y15,"")</f>
+        <v/>
+      </c>
+      <c r="AA15" s="32" t="n">
+        <f aca="false">Channels!U15</f>
+        <v>0</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19584,8 +19727,17 @@
         <v>1</v>
       </c>
       <c r="X16" s="2" t="str">
-        <f aca="false">IF(D16=0,"Free – monitor quality",IF(F16=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P16&lt;Assumptions!$D$83,Q16&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W16&gt;=Assumptions!$D$87,AND(R16=0,P16&gt;=Assumptions!$D$88)),"SWITCH OFF",IF(W16&gt;=Assumptions!$D$86,"CUT 50%",IF(W16&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
+        <f aca="false">IF(D16=0,"Free – monitor quality",IF(F16=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P16&lt;Assumptions!$D$83,Q16&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W16&gt;=Assumptions!$D$87,AND(R16=0,P16&gt;=Assumptions!$D$88,Q16&gt;=Assumptions!$D$84)),"SWITCH OFF",IF(W16&gt;=Assumptions!$D$86,"CUT 50%",IF(W16&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
+      </c>
+      <c r="Y16" s="15"/>
+      <c r="Z16" s="41" t="str">
+        <f aca="false">IF(Y16&gt;0,P16/Y16,"")</f>
+        <v/>
+      </c>
+      <c r="AA16" s="32" t="n">
+        <f aca="false">Channels!U16</f>
+        <v>0</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19655,8 +19807,17 @@
         <v>1</v>
       </c>
       <c r="X17" s="2" t="str">
-        <f aca="false">IF(D17=0,"Free – monitor quality",IF(F17=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P17&lt;Assumptions!$D$83,Q17&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W17&gt;=Assumptions!$D$87,AND(R17=0,P17&gt;=Assumptions!$D$88)),"SWITCH OFF",IF(W17&gt;=Assumptions!$D$86,"CUT 50%",IF(W17&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
+        <f aca="false">IF(D17=0,"Free – monitor quality",IF(F17=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P17&lt;Assumptions!$D$83,Q17&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W17&gt;=Assumptions!$D$87,AND(R17=0,P17&gt;=Assumptions!$D$88,Q17&gt;=Assumptions!$D$84)),"SWITCH OFF",IF(W17&gt;=Assumptions!$D$86,"CUT 50%",IF(W17&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
+      </c>
+      <c r="Y17" s="15"/>
+      <c r="Z17" s="41" t="str">
+        <f aca="false">IF(Y17&gt;0,P17/Y17,"")</f>
+        <v/>
+      </c>
+      <c r="AA17" s="32" t="n">
+        <f aca="false">Channels!U17</f>
+        <v>9.50835640751761</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19726,8 +19887,17 @@
         <v>1</v>
       </c>
       <c r="X18" s="2" t="str">
-        <f aca="false">IF(D18=0,"Free – monitor quality",IF(F18=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P18&lt;Assumptions!$D$83,Q18&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W18&gt;=Assumptions!$D$87,AND(R18=0,P18&gt;=Assumptions!$D$88)),"SWITCH OFF",IF(W18&gt;=Assumptions!$D$86,"CUT 50%",IF(W18&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
+        <f aca="false">IF(D18=0,"Free – monitor quality",IF(F18=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P18&lt;Assumptions!$D$83,Q18&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W18&gt;=Assumptions!$D$87,AND(R18=0,P18&gt;=Assumptions!$D$88,Q18&gt;=Assumptions!$D$84)),"SWITCH OFF",IF(W18&gt;=Assumptions!$D$86,"CUT 50%",IF(W18&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
+      </c>
+      <c r="Y18" s="15"/>
+      <c r="Z18" s="41" t="str">
+        <f aca="false">IF(Y18&gt;0,P18/Y18,"")</f>
+        <v/>
+      </c>
+      <c r="AA18" s="32" t="n">
+        <f aca="false">Channels!U18</f>
+        <v>6.63483072067039</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19797,8 +19967,17 @@
         <v>1</v>
       </c>
       <c r="X19" s="2" t="str">
-        <f aca="false">IF(D19=0,"Free – monitor quality",IF(F19=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P19&lt;Assumptions!$D$83,Q19&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W19&gt;=Assumptions!$D$87,AND(R19=0,P19&gt;=Assumptions!$D$88)),"SWITCH OFF",IF(W19&gt;=Assumptions!$D$86,"CUT 50%",IF(W19&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
+        <f aca="false">IF(D19=0,"Free – monitor quality",IF(F19=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P19&lt;Assumptions!$D$83,Q19&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W19&gt;=Assumptions!$D$87,AND(R19=0,P19&gt;=Assumptions!$D$88,Q19&gt;=Assumptions!$D$84)),"SWITCH OFF",IF(W19&gt;=Assumptions!$D$86,"CUT 50%",IF(W19&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
+      </c>
+      <c r="Y19" s="15"/>
+      <c r="Z19" s="41" t="str">
+        <f aca="false">IF(Y19&gt;0,P19/Y19,"")</f>
+        <v/>
+      </c>
+      <c r="AA19" s="32" t="n">
+        <f aca="false">Channels!U19</f>
+        <v>0.28828125</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19868,8 +20047,17 @@
         <v>1</v>
       </c>
       <c r="X20" s="2" t="str">
-        <f aca="false">IF(D20=0,"Free – monitor quality",IF(F20=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P20&lt;Assumptions!$D$83,Q20&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W20&gt;=Assumptions!$D$87,AND(R20=0,P20&gt;=Assumptions!$D$88)),"SWITCH OFF",IF(W20&gt;=Assumptions!$D$86,"CUT 50%",IF(W20&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
+        <f aca="false">IF(D20=0,"Free – monitor quality",IF(F20=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P20&lt;Assumptions!$D$83,Q20&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W20&gt;=Assumptions!$D$87,AND(R20=0,P20&gt;=Assumptions!$D$88,Q20&gt;=Assumptions!$D$84)),"SWITCH OFF",IF(W20&gt;=Assumptions!$D$86,"CUT 50%",IF(W20&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
+      </c>
+      <c r="Y20" s="15"/>
+      <c r="Z20" s="41" t="str">
+        <f aca="false">IF(Y20&gt;0,P20/Y20,"")</f>
+        <v/>
+      </c>
+      <c r="AA20" s="32" t="n">
+        <f aca="false">Channels!U20</f>
+        <v>0.339760044642857</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19891,11 +20079,11 @@
       </c>
       <c r="E21" s="30" t="n">
         <f aca="false">Channels!I21</f>
-        <v>0.1775</v>
+        <v>0.175</v>
       </c>
       <c r="F21" s="41" t="n">
         <f aca="false">Channels!O21</f>
-        <v>1008.45070422535</v>
+        <v>1022.85714285714</v>
       </c>
       <c r="G21" s="18"/>
       <c r="H21" s="15"/>
@@ -19928,19 +20116,28 @@
       </c>
       <c r="U21" s="30" t="n">
         <f aca="false">IF(AND(OR(P21&gt;=Assumptions!$D$83,Q21&gt;=Assumptions!$D$84),R21&gt;0),R21/Q21,E21)</f>
-        <v>0.1775</v>
+        <v>0.175</v>
       </c>
       <c r="V21" s="41" t="n">
         <f aca="false">IF(U21&gt;0,IF(AND(OR(P21&gt;=Assumptions!$D$83,Q21&gt;=Assumptions!$D$84),Q21&gt;0),S21,D21)/U21,0)</f>
-        <v>1008.45070422535</v>
+        <v>1022.85714285714</v>
       </c>
       <c r="W21" s="52" t="n">
         <f aca="false">IF(F21&gt;0,V21/F21,"")</f>
         <v>1</v>
       </c>
       <c r="X21" s="2" t="str">
-        <f aca="false">IF(D21=0,"Free – monitor quality",IF(F21=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P21&lt;Assumptions!$D$83,Q21&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W21&gt;=Assumptions!$D$87,AND(R21=0,P21&gt;=Assumptions!$D$88)),"SWITCH OFF",IF(W21&gt;=Assumptions!$D$86,"CUT 50%",IF(W21&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
+        <f aca="false">IF(D21=0,"Free – monitor quality",IF(F21=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P21&lt;Assumptions!$D$83,Q21&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W21&gt;=Assumptions!$D$87,AND(R21=0,P21&gt;=Assumptions!$D$88,Q21&gt;=Assumptions!$D$84)),"SWITCH OFF",IF(W21&gt;=Assumptions!$D$86,"CUT 50%",IF(W21&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
+      </c>
+      <c r="Y21" s="15"/>
+      <c r="Z21" s="41" t="str">
+        <f aca="false">IF(Y21&gt;0,P21/Y21,"")</f>
+        <v/>
+      </c>
+      <c r="AA21" s="32" t="n">
+        <f aca="false">Channels!U21</f>
+        <v>0.230970670391061</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19962,11 +20159,11 @@
       </c>
       <c r="E22" s="30" t="n">
         <f aca="false">Channels!I22</f>
-        <v>0.1775</v>
+        <v>0.175</v>
       </c>
       <c r="F22" s="41" t="n">
         <f aca="false">Channels!O22</f>
-        <v>1008.45070422535</v>
+        <v>1022.85714285714</v>
       </c>
       <c r="G22" s="18"/>
       <c r="H22" s="15"/>
@@ -19999,19 +20196,28 @@
       </c>
       <c r="U22" s="30" t="n">
         <f aca="false">IF(AND(OR(P22&gt;=Assumptions!$D$83,Q22&gt;=Assumptions!$D$84),R22&gt;0),R22/Q22,E22)</f>
-        <v>0.1775</v>
+        <v>0.175</v>
       </c>
       <c r="V22" s="41" t="n">
         <f aca="false">IF(U22&gt;0,IF(AND(OR(P22&gt;=Assumptions!$D$83,Q22&gt;=Assumptions!$D$84),Q22&gt;0),S22,D22)/U22,0)</f>
-        <v>1008.45070422535</v>
+        <v>1022.85714285714</v>
       </c>
       <c r="W22" s="52" t="n">
         <f aca="false">IF(F22&gt;0,V22/F22,"")</f>
         <v>1</v>
       </c>
       <c r="X22" s="2" t="str">
-        <f aca="false">IF(D22=0,"Free – monitor quality",IF(F22=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P22&lt;Assumptions!$D$83,Q22&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W22&gt;=Assumptions!$D$87,AND(R22=0,P22&gt;=Assumptions!$D$88)),"SWITCH OFF",IF(W22&gt;=Assumptions!$D$86,"CUT 50%",IF(W22&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
+        <f aca="false">IF(D22=0,"Free – monitor quality",IF(F22=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P22&lt;Assumptions!$D$83,Q22&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W22&gt;=Assumptions!$D$87,AND(R22=0,P22&gt;=Assumptions!$D$88,Q22&gt;=Assumptions!$D$84)),"SWITCH OFF",IF(W22&gt;=Assumptions!$D$86,"CUT 50%",IF(W22&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
+      </c>
+      <c r="Y22" s="15"/>
+      <c r="Z22" s="41" t="str">
+        <f aca="false">IF(Y22&gt;0,P22/Y22,"")</f>
+        <v/>
+      </c>
+      <c r="AA22" s="32" t="n">
+        <f aca="false">Channels!U22</f>
+        <v>0.272215432960894</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20033,11 +20239,11 @@
       </c>
       <c r="E23" s="30" t="n">
         <f aca="false">Channels!I23</f>
-        <v>0.1775</v>
+        <v>0.175</v>
       </c>
       <c r="F23" s="41" t="n">
         <f aca="false">Channels!O23</f>
-        <v>1008.45070422535</v>
+        <v>1022.85714285714</v>
       </c>
       <c r="G23" s="18"/>
       <c r="H23" s="15"/>
@@ -20070,19 +20276,28 @@
       </c>
       <c r="U23" s="30" t="n">
         <f aca="false">IF(AND(OR(P23&gt;=Assumptions!$D$83,Q23&gt;=Assumptions!$D$84),R23&gt;0),R23/Q23,E23)</f>
-        <v>0.1775</v>
+        <v>0.175</v>
       </c>
       <c r="V23" s="41" t="n">
         <f aca="false">IF(U23&gt;0,IF(AND(OR(P23&gt;=Assumptions!$D$83,Q23&gt;=Assumptions!$D$84),Q23&gt;0),S23,D23)/U23,0)</f>
-        <v>1008.45070422535</v>
+        <v>1022.85714285714</v>
       </c>
       <c r="W23" s="52" t="n">
         <f aca="false">IF(F23&gt;0,V23/F23,"")</f>
         <v>1</v>
       </c>
       <c r="X23" s="2" t="str">
-        <f aca="false">IF(D23=0,"Free – monitor quality",IF(F23=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P23&lt;Assumptions!$D$83,Q23&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W23&gt;=Assumptions!$D$87,AND(R23=0,P23&gt;=Assumptions!$D$88)),"SWITCH OFF",IF(W23&gt;=Assumptions!$D$86,"CUT 50%",IF(W23&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
+        <f aca="false">IF(D23=0,"Free – monitor quality",IF(F23=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P23&lt;Assumptions!$D$83,Q23&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W23&gt;=Assumptions!$D$87,AND(R23=0,P23&gt;=Assumptions!$D$88,Q23&gt;=Assumptions!$D$84)),"SWITCH OFF",IF(W23&gt;=Assumptions!$D$86,"CUT 50%",IF(W23&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
+      </c>
+      <c r="Y23" s="15"/>
+      <c r="Z23" s="41" t="str">
+        <f aca="false">IF(Y23&gt;0,P23/Y23,"")</f>
+        <v/>
+      </c>
+      <c r="AA23" s="32" t="n">
+        <f aca="false">Channels!U23</f>
+        <v>0.207873603351955</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20104,11 +20319,11 @@
       </c>
       <c r="E24" s="30" t="n">
         <f aca="false">Channels!I24</f>
-        <v>0.1633</v>
+        <v>0.161</v>
       </c>
       <c r="F24" s="41" t="n">
         <f aca="false">Channels!O24</f>
-        <v>1096.14206981017</v>
+        <v>1111.80124223602</v>
       </c>
       <c r="G24" s="18"/>
       <c r="H24" s="15"/>
@@ -20141,19 +20356,28 @@
       </c>
       <c r="U24" s="30" t="n">
         <f aca="false">IF(AND(OR(P24&gt;=Assumptions!$D$83,Q24&gt;=Assumptions!$D$84),R24&gt;0),R24/Q24,E24)</f>
-        <v>0.1633</v>
+        <v>0.161</v>
       </c>
       <c r="V24" s="41" t="n">
         <f aca="false">IF(U24&gt;0,IF(AND(OR(P24&gt;=Assumptions!$D$83,Q24&gt;=Assumptions!$D$84),Q24&gt;0),S24,D24)/U24,0)</f>
-        <v>1096.14206981017</v>
+        <v>1111.80124223602</v>
       </c>
       <c r="W24" s="52" t="n">
         <f aca="false">IF(F24&gt;0,V24/F24,"")</f>
         <v>1</v>
       </c>
       <c r="X24" s="2" t="str">
-        <f aca="false">IF(D24=0,"Free – monitor quality",IF(F24=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P24&lt;Assumptions!$D$83,Q24&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W24&gt;=Assumptions!$D$87,AND(R24=0,P24&gt;=Assumptions!$D$88)),"SWITCH OFF",IF(W24&gt;=Assumptions!$D$86,"CUT 50%",IF(W24&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
+        <f aca="false">IF(D24=0,"Free – monitor quality",IF(F24=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P24&lt;Assumptions!$D$83,Q24&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W24&gt;=Assumptions!$D$87,AND(R24=0,P24&gt;=Assumptions!$D$88,Q24&gt;=Assumptions!$D$84)),"SWITCH OFF",IF(W24&gt;=Assumptions!$D$86,"CUT 50%",IF(W24&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
+      </c>
+      <c r="Y24" s="15"/>
+      <c r="Z24" s="41" t="str">
+        <f aca="false">IF(Y24&gt;0,P24/Y24,"")</f>
+        <v/>
+      </c>
+      <c r="AA24" s="32" t="n">
+        <f aca="false">Channels!U24</f>
+        <v>0.160550279329609</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20223,8 +20447,17 @@
         <v>1</v>
       </c>
       <c r="X25" s="2" t="str">
-        <f aca="false">IF(D25=0,"Free – monitor quality",IF(F25=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P25&lt;Assumptions!$D$83,Q25&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W25&gt;=Assumptions!$D$87,AND(R25=0,P25&gt;=Assumptions!$D$88)),"SWITCH OFF",IF(W25&gt;=Assumptions!$D$86,"CUT 50%",IF(W25&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
+        <f aca="false">IF(D25=0,"Free – monitor quality",IF(F25=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P25&lt;Assumptions!$D$83,Q25&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W25&gt;=Assumptions!$D$87,AND(R25=0,P25&gt;=Assumptions!$D$88,Q25&gt;=Assumptions!$D$84)),"SWITCH OFF",IF(W25&gt;=Assumptions!$D$86,"CUT 50%",IF(W25&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
+      </c>
+      <c r="Y25" s="15"/>
+      <c r="Z25" s="41" t="str">
+        <f aca="false">IF(Y25&gt;0,P25/Y25,"")</f>
+        <v/>
+      </c>
+      <c r="AA25" s="32" t="n">
+        <f aca="false">Channels!U25</f>
+        <v>1.412775</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20294,8 +20527,17 @@
         <v>1</v>
       </c>
       <c r="X26" s="2" t="str">
-        <f aca="false">IF(D26=0,"Free – monitor quality",IF(F26=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P26&lt;Assumptions!$D$83,Q26&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W26&gt;=Assumptions!$D$87,AND(R26=0,P26&gt;=Assumptions!$D$88)),"SWITCH OFF",IF(W26&gt;=Assumptions!$D$86,"CUT 50%",IF(W26&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
+        <f aca="false">IF(D26=0,"Free – monitor quality",IF(F26=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P26&lt;Assumptions!$D$83,Q26&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W26&gt;=Assumptions!$D$87,AND(R26=0,P26&gt;=Assumptions!$D$88,Q26&gt;=Assumptions!$D$84)),"SWITCH OFF",IF(W26&gt;=Assumptions!$D$86,"CUT 50%",IF(W26&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
+      </c>
+      <c r="Y26" s="15"/>
+      <c r="Z26" s="41" t="str">
+        <f aca="false">IF(Y26&gt;0,P26/Y26,"")</f>
+        <v/>
+      </c>
+      <c r="AA26" s="32" t="n">
+        <f aca="false">Channels!U26</f>
+        <v>1.946835</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20365,8 +20607,17 @@
         <v>1</v>
       </c>
       <c r="X27" s="2" t="str">
-        <f aca="false">IF(D27=0,"Free – monitor quality",IF(F27=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P27&lt;Assumptions!$D$83,Q27&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W27&gt;=Assumptions!$D$87,AND(R27=0,P27&gt;=Assumptions!$D$88)),"SWITCH OFF",IF(W27&gt;=Assumptions!$D$86,"CUT 50%",IF(W27&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
+        <f aca="false">IF(D27=0,"Free – monitor quality",IF(F27=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P27&lt;Assumptions!$D$83,Q27&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W27&gt;=Assumptions!$D$87,AND(R27=0,P27&gt;=Assumptions!$D$88,Q27&gt;=Assumptions!$D$84)),"SWITCH OFF",IF(W27&gt;=Assumptions!$D$86,"CUT 50%",IF(W27&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
+      </c>
+      <c r="Y27" s="15"/>
+      <c r="Z27" s="41" t="str">
+        <f aca="false">IF(Y27&gt;0,P27/Y27,"")</f>
+        <v/>
+      </c>
+      <c r="AA27" s="32" t="n">
+        <f aca="false">Channels!U27</f>
+        <v>0.743337</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20436,8 +20687,17 @@
         <v>1</v>
       </c>
       <c r="X28" s="2" t="str">
-        <f aca="false">IF(D28=0,"Free – monitor quality",IF(F28=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P28&lt;Assumptions!$D$83,Q28&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W28&gt;=Assumptions!$D$87,AND(R28=0,P28&gt;=Assumptions!$D$88)),"SWITCH OFF",IF(W28&gt;=Assumptions!$D$86,"CUT 50%",IF(W28&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
+        <f aca="false">IF(D28=0,"Free – monitor quality",IF(F28=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P28&lt;Assumptions!$D$83,Q28&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W28&gt;=Assumptions!$D$87,AND(R28=0,P28&gt;=Assumptions!$D$88,Q28&gt;=Assumptions!$D$84)),"SWITCH OFF",IF(W28&gt;=Assumptions!$D$86,"CUT 50%",IF(W28&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
+      </c>
+      <c r="Y28" s="15"/>
+      <c r="Z28" s="41" t="str">
+        <f aca="false">IF(Y28&gt;0,P28/Y28,"")</f>
+        <v/>
+      </c>
+      <c r="AA28" s="32" t="n">
+        <f aca="false">Channels!U28</f>
+        <v>0.525504</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20507,8 +20767,17 @@
         <v>1</v>
       </c>
       <c r="X29" s="2" t="str">
-        <f aca="false">IF(D29=0,"Free – monitor quality",IF(F29=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P29&lt;Assumptions!$D$83,Q29&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W29&gt;=Assumptions!$D$87,AND(R29=0,P29&gt;=Assumptions!$D$88)),"SWITCH OFF",IF(W29&gt;=Assumptions!$D$86,"CUT 50%",IF(W29&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
+        <f aca="false">IF(D29=0,"Free – monitor quality",IF(F29=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P29&lt;Assumptions!$D$83,Q29&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W29&gt;=Assumptions!$D$87,AND(R29=0,P29&gt;=Assumptions!$D$88,Q29&gt;=Assumptions!$D$84)),"SWITCH OFF",IF(W29&gt;=Assumptions!$D$86,"CUT 50%",IF(W29&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
+      </c>
+      <c r="Y29" s="15"/>
+      <c r="Z29" s="41" t="str">
+        <f aca="false">IF(Y29&gt;0,P29/Y29,"")</f>
+        <v/>
+      </c>
+      <c r="AA29" s="32" t="n">
+        <f aca="false">Channels!U29</f>
+        <v>3.26025</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20578,8 +20847,17 @@
         <v>1</v>
       </c>
       <c r="X30" s="2" t="str">
-        <f aca="false">IF(D30=0,"Free – monitor quality",IF(F30=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P30&lt;Assumptions!$D$83,Q30&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W30&gt;=Assumptions!$D$87,AND(R30=0,P30&gt;=Assumptions!$D$88)),"SWITCH OFF",IF(W30&gt;=Assumptions!$D$86,"CUT 50%",IF(W30&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
+        <f aca="false">IF(D30=0,"Free – monitor quality",IF(F30=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P30&lt;Assumptions!$D$83,Q30&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W30&gt;=Assumptions!$D$87,AND(R30=0,P30&gt;=Assumptions!$D$88,Q30&gt;=Assumptions!$D$84)),"SWITCH OFF",IF(W30&gt;=Assumptions!$D$86,"CUT 50%",IF(W30&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
+      </c>
+      <c r="Y30" s="15"/>
+      <c r="Z30" s="41" t="str">
+        <f aca="false">IF(Y30&gt;0,P30/Y30,"")</f>
+        <v/>
+      </c>
+      <c r="AA30" s="32" t="n">
+        <f aca="false">Channels!U30</f>
+        <v>4.99516875</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20649,8 +20927,17 @@
         <v>1</v>
       </c>
       <c r="X31" s="2" t="str">
-        <f aca="false">IF(D31=0,"Free – monitor quality",IF(F31=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P31&lt;Assumptions!$D$83,Q31&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W31&gt;=Assumptions!$D$87,AND(R31=0,P31&gt;=Assumptions!$D$88)),"SWITCH OFF",IF(W31&gt;=Assumptions!$D$86,"CUT 50%",IF(W31&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
+        <f aca="false">IF(D31=0,"Free – monitor quality",IF(F31=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P31&lt;Assumptions!$D$83,Q31&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W31&gt;=Assumptions!$D$87,AND(R31=0,P31&gt;=Assumptions!$D$88,Q31&gt;=Assumptions!$D$84)),"SWITCH OFF",IF(W31&gt;=Assumptions!$D$86,"CUT 50%",IF(W31&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
+      </c>
+      <c r="Y31" s="15"/>
+      <c r="Z31" s="41" t="str">
+        <f aca="false">IF(Y31&gt;0,P31/Y31,"")</f>
+        <v/>
+      </c>
+      <c r="AA31" s="32" t="n">
+        <f aca="false">Channels!U31</f>
+        <v>1.61382375</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20720,8 +21007,17 @@
         <v>1</v>
       </c>
       <c r="X32" s="2" t="str">
-        <f aca="false">IF(D32=0,"Free – monitor quality",IF(F32=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P32&lt;Assumptions!$D$83,Q32&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W32&gt;=Assumptions!$D$87,AND(R32=0,P32&gt;=Assumptions!$D$88)),"SWITCH OFF",IF(W32&gt;=Assumptions!$D$86,"CUT 50%",IF(W32&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
+        <f aca="false">IF(D32=0,"Free – monitor quality",IF(F32=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P32&lt;Assumptions!$D$83,Q32&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W32&gt;=Assumptions!$D$87,AND(R32=0,P32&gt;=Assumptions!$D$88,Q32&gt;=Assumptions!$D$84)),"SWITCH OFF",IF(W32&gt;=Assumptions!$D$86,"CUT 50%",IF(W32&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
+      </c>
+      <c r="Y32" s="15"/>
+      <c r="Z32" s="41" t="str">
+        <f aca="false">IF(Y32&gt;0,P32/Y32,"")</f>
+        <v/>
+      </c>
+      <c r="AA32" s="32" t="n">
+        <f aca="false">Channels!U32</f>
+        <v>1.108485</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20791,8 +21087,17 @@
         <v>1</v>
       </c>
       <c r="X33" s="2" t="str">
-        <f aca="false">IF(D33=0,"Free – monitor quality",IF(F33=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P33&lt;Assumptions!$D$83,Q33&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W33&gt;=Assumptions!$D$87,AND(R33=0,P33&gt;=Assumptions!$D$88)),"SWITCH OFF",IF(W33&gt;=Assumptions!$D$86,"CUT 50%",IF(W33&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
+        <f aca="false">IF(D33=0,"Free – monitor quality",IF(F33=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P33&lt;Assumptions!$D$83,Q33&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W33&gt;=Assumptions!$D$87,AND(R33=0,P33&gt;=Assumptions!$D$88,Q33&gt;=Assumptions!$D$84)),"SWITCH OFF",IF(W33&gt;=Assumptions!$D$86,"CUT 50%",IF(W33&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
+      </c>
+      <c r="Y33" s="15"/>
+      <c r="Z33" s="41" t="str">
+        <f aca="false">IF(Y33&gt;0,P33/Y33,"")</f>
+        <v/>
+      </c>
+      <c r="AA33" s="32" t="n">
+        <f aca="false">Channels!U33</f>
+        <v>8.36325</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20862,8 +21167,17 @@
         <v>1</v>
       </c>
       <c r="X34" s="2" t="str">
-        <f aca="false">IF(D34=0,"Free – monitor quality",IF(F34=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P34&lt;Assumptions!$D$83,Q34&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W34&gt;=Assumptions!$D$87,AND(R34=0,P34&gt;=Assumptions!$D$88)),"SWITCH OFF",IF(W34&gt;=Assumptions!$D$86,"CUT 50%",IF(W34&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
+        <f aca="false">IF(D34=0,"Free – monitor quality",IF(F34=0,"SWITCH OFF – plan expects no qualified applicants",IF(AND(P34&lt;Assumptions!$D$83,Q34&lt;Assumptions!$D$84),"Wait – too little data",IF(OR(W34&gt;=Assumptions!$D$87,AND(R34=0,P34&gt;=Assumptions!$D$88,Q34&gt;=Assumptions!$D$84)),"SWITCH OFF",IF(W34&gt;=Assumptions!$D$86,"CUT 50%",IF(W34&lt;=Assumptions!$D$85,"ADD +"&amp;TEXT(Assumptions!$D$96,"0%")&amp;" (if slots free)","HOLD"))))))</f>
         <v>Wait – too little data</v>
+      </c>
+      <c r="Y34" s="15"/>
+      <c r="Z34" s="41" t="str">
+        <f aca="false">IF(Y34&gt;0,P34/Y34,"")</f>
+        <v/>
+      </c>
+      <c r="AA34" s="32" t="n">
+        <f aca="false">Channels!U34</f>
+        <v>18</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20918,10 +21232,18 @@
         <f aca="false">SUM(R5:R34)</f>
         <v>0</v>
       </c>
+      <c r="Y35" s="33" t="n">
+        <f aca="false">SUM(Y5:Y34)</f>
+        <v>0</v>
+      </c>
+      <c r="AA35" s="35" t="n">
+        <f aca="false">SUM(AA5:AA34)</f>
+        <v>100</v>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="28" t="s">
-        <v>751</v>
+        <v>754</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -20930,46 +21252,46 @@
         <v>312</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>752</v>
+        <v>755</v>
       </c>
       <c r="D39" s="12" t="s">
-        <v>753</v>
+        <v>756</v>
       </c>
       <c r="E39" s="12" t="s">
-        <v>754</v>
+        <v>757</v>
       </c>
       <c r="F39" s="12" t="s">
-        <v>755</v>
+        <v>758</v>
       </c>
       <c r="G39" s="12" t="s">
-        <v>756</v>
+        <v>759</v>
       </c>
       <c r="H39" s="12" t="s">
-        <v>757</v>
+        <v>760</v>
       </c>
       <c r="I39" s="12" t="s">
-        <v>758</v>
+        <v>761</v>
       </c>
       <c r="J39" s="12" t="s">
-        <v>759</v>
+        <v>762</v>
       </c>
       <c r="K39" s="12" t="s">
-        <v>760</v>
+        <v>763</v>
       </c>
       <c r="L39" s="12" t="s">
-        <v>761</v>
+        <v>764</v>
       </c>
       <c r="M39" s="12" t="s">
-        <v>762</v>
+        <v>765</v>
       </c>
       <c r="N39" s="12" t="s">
-        <v>763</v>
+        <v>766</v>
       </c>
       <c r="O39" s="12" t="s">
         <v>47</v>
       </c>
       <c r="P39" s="12" t="s">
-        <v>764</v>
+        <v>767</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21199,7 +21521,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="9" t="s">
-        <v>765</v>
+        <v>768</v>
       </c>
       <c r="B46" s="9"/>
       <c r="C46" s="9"/>

</xml_diff>

<commit_message>
Weekly plan paces I2/I3 from their go-live dates (inputs I2L, I3L), shares re-solved; supply-check attribution corrected
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V2NJtrYy3bzNxqKeiRXJfY
</commit_message>
<xml_diff>
--- a/operation_uptime/Operation_Uptime_Model.xlsx
+++ b/operation_uptime/Operation_Uptime_Model.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1473" uniqueCount="773">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1498" uniqueCount="792">
   <si>
     <t xml:space="preserve">Operation Uptime — model summary (hypothetical Tesla Giga Berlin maintenance hiring)</t>
   </si>
@@ -938,7 +938,7 @@
     <t xml:space="preserve">Maintenance trades as share of production occupations</t>
   </si>
   <si>
-    <t xml:space="preserve">BA employment, Germany: maintenance codes 2513 + 2625 + 2611 + 2612 + supervisors 2519 + 2619 + 2629 (536,520) ÷ production occupations 21–29 (6,850,263) = 7.8%. https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-d-0-202512-xlsx.xlsx?__blob=publicationFile</t>
+    <t xml:space="preserve">BA employment, Germany: maintenance codes 2513 + 2625 + 2611 + 2612 + supervisors 2519 + 2619 + 2629 (536,520) ÷ production occupations 21–29 (6,850,263) = 7.8%. Also applied to Polish industry for the I3 supply check (my estimate; an upper bound). https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-d-0-202512-xlsx.xlsx?__blob=publicationFile</t>
   </si>
   <si>
     <t xml:space="preserve">TURN</t>
@@ -1322,6 +1322,24 @@
     <t xml:space="preserve">Translation at the German statutory rate per line (JVEG). https://www.gesetze-im-internet.de/jveg/__11.html</t>
   </si>
   <si>
+    <t xml:space="preserve">I2L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I2: days from campaign start to go-live (ads, quiz, German copy)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Setup plan: copy and quiz written in 2 days, client profile sign-off, live Fri 23 Oct.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I3L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I3: days from campaign start to go-live (translation, freelancer hired)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Setup plan: Polish translation and hiring the freelancer take a week, live Tue 27 Oct.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Part 1 — Funnel by role (work back from openings)</t>
   </si>
   <si>
@@ -2123,34 +2141,73 @@
     <t xml:space="preserve">Supervisor share before re-scaling (useful days only)</t>
   </si>
   <si>
+    <t xml:space="preserve">I2 share (from go-live)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I3 share (from go-live)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I2 share before re-scaling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I3 share before re-scaling</t>
+  </si>
+  <si>
     <t xml:space="preserve">Weak channels are cut from Mon 2 Nov; tests are judged by Mon 9 Nov; the reserve is released only from week 3, on the Tracker rules.</t>
   </si>
   <si>
     <t xml:space="preserve">Helper totals</t>
   </si>
   <si>
+    <t xml:space="preserve">Late launches (paced from their go-live dates, cols AB–AE)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Spreadable media E/M/A (after tests, excl. rediscovery)</t>
   </si>
   <si>
+    <t xml:space="preserve">I2 media €</t>
+  </si>
+  <si>
     <t xml:space="preserve">Spreadable media Supervisors (after tests, excl. rediscovery)</t>
   </si>
   <si>
+    <t xml:space="preserve">I2 applications</t>
+  </si>
+  <si>
     <t xml:space="preserve">StepStone ads (all roles)</t>
   </si>
   <si>
+    <t xml:space="preserve">I2 qualified</t>
+  </si>
+  <si>
     <t xml:space="preserve">Referral bonuses E/M/A</t>
   </si>
   <si>
+    <t xml:space="preserve">I2 hires</t>
+  </si>
+  <si>
     <t xml:space="preserve">Referral bonuses Supervisors</t>
   </si>
   <si>
+    <t xml:space="preserve">I3 media €</t>
+  </si>
+  <si>
     <t xml:space="preserve">Test tranches (all roles)</t>
   </si>
   <si>
+    <t xml:space="preserve">I3 applications</t>
+  </si>
+  <si>
     <t xml:space="preserve">Test qualified E/M/A</t>
   </si>
   <si>
+    <t xml:space="preserve">I3 qualified</t>
+  </si>
+  <si>
     <t xml:space="preserve">Test qualified Supervisors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I3 hires</t>
   </si>
   <si>
     <t xml:space="preserve">Test applications E/M/A</t>
@@ -3147,7 +3204,7 @@
         <v>16</v>
       </c>
       <c r="C19" s="8" t="str">
-        <f aca="false">IF(((Assumptions!$D$10&lt;0)+(Assumptions!$D$10&gt;1)+(Assumptions!$D$52&lt;0)+(Assumptions!$D$52&gt;1)+(Assumptions!$D$50&lt;0)+(Assumptions!$D$50&gt;1)+(Assumptions!$D$64&lt;0)+(Assumptions!$D$64&gt;1)+(Assumptions!$D$155&lt;0)+(Assumptions!$D$155&gt;1)+(Assumptions!$D$156&lt;0)+(Assumptions!$D$156&gt;1)+(Assumptions!$D$161&lt;0)+(Assumptions!$D$161&gt;1)+(Assumptions!$D$166&lt;0)+(Assumptions!$D$166&gt;1)+(Assumptions!$D$168&lt;0)+(Assumptions!$D$168&gt;1)+(Assumptions!$D$172&lt;0)+(Assumptions!$D$172&gt;1)+(Assumptions!$D$93&lt;0)+(Assumptions!$D$93&gt;1)+(Assumptions!$D$94&lt;0)+(Assumptions!$D$94&gt;1)+(Assumptions!$D$95&lt;0)+(Assumptions!$D$95&gt;1)+(Assumptions!$D$89&lt;0)+(Assumptions!$D$89&gt;1)+(Assumptions!$D$91&lt;0)+(Assumptions!$D$91&gt;1)+(Assumptions!$D$29&lt;0)+(Assumptions!$D$29&gt;1)+(Assumptions!$D$30&lt;0)+(Assumptions!$D$30&gt;1)+(Assumptions!$D$31&lt;0)+(Assumptions!$D$31&gt;1)+(Assumptions!$D$32&lt;0)+(Assumptions!$D$32&gt;1)+(Assumptions!$D$33&lt;0)+(Assumptions!$D$33&gt;1)+(Assumptions!$D$34&lt;0)+(Assumptions!$D$34&gt;1)+(Assumptions!$D$35&lt;0)+(Assumptions!$D$35&gt;1)+(Assumptions!$D$36&lt;0)+(Assumptions!$D$36&gt;1)+(Assumptions!$D$37&lt;0)+(Assumptions!$D$37&gt;1)+(Assumptions!$D$38&lt;0)+(Assumptions!$D$38&gt;1)+(Assumptions!$D$39&lt;0)+(Assumptions!$D$39&gt;1)+(Assumptions!$D$40&lt;0)+(Assumptions!$D$40&gt;1)+(Assumptions!$D$41&lt;0)+(Assumptions!$D$41&gt;1)+(Assumptions!$D$42&lt;0)+(Assumptions!$D$42&gt;1)+(Assumptions!$D$43&lt;0)+(Assumptions!$D$43&gt;1)+(Assumptions!$D$44&lt;0)+(Assumptions!$D$44&gt;1)+(Assumptions!$D$53&lt;0)+(Assumptions!$D$53&gt;1)+(Assumptions!$D$54&lt;0)+(Assumptions!$D$54&gt;1)+(Assumptions!$D$55&lt;0)+(Assumptions!$D$55&gt;1)+(Assumptions!$D$56&lt;0)+(Assumptions!$D$56&gt;1)+(Assumptions!$D$57&lt;0)+(Assumptions!$D$57&gt;1)+(Assumptions!$D$58&lt;0)+(Assumptions!$D$58&gt;1)+(Assumptions!$D$59&lt;0)+(Assumptions!$D$59&gt;1)+(Assumptions!$D$60&lt;0)+(Assumptions!$D$60&gt;1)+(Assumptions!$D$61&lt;0)+(Assumptions!$D$61&gt;1)+(Assumptions!$D$62&lt;0)+(Assumptions!$D$62&gt;1)+(Assumptions!$D$63&lt;0)+(Assumptions!$D$63&gt;1)+(Assumptions!$D$72&lt;0)+(Assumptions!$D$72&gt;1)+(Assumptions!$D$73&lt;0)+(Assumptions!$D$73&gt;1)+(Assumptions!$D$74&lt;0)+(Assumptions!$D$74&gt;1)+(Assumptions!$D$75&lt;0)+(Assumptions!$D$75&gt;1)+(Assumptions!$D$96&lt;0)+(Assumptions!$D$96&gt;1)+(Assumptions!$D$99&lt;0)+(Assumptions!$D$99&gt;1)+(Assumptions!$D$100&lt;0)+(Assumptions!$D$100&gt;1)+(Assumptions!$D$101&lt;0)+(Assumptions!$D$101&gt;1)+(Assumptions!$D$102&lt;0)+(Assumptions!$D$102&gt;1)+(Assumptions!$D$108&lt;0)+(Assumptions!$D$108&gt;1)+(Assumptions!$D$109&lt;0)+(Assumptions!$D$109&gt;1)+(Assumptions!$D$110&lt;0)+(Assumptions!$D$110&gt;1)+(Assumptions!$D$111&lt;0)+(Assumptions!$D$111&gt;1)+(Assumptions!$D$112&lt;0)+(Assumptions!$D$112&gt;1)+(Assumptions!$D$113&lt;0)+(Assumptions!$D$113&gt;1)+(Assumptions!$D$115&lt;0)+(Assumptions!$D$115&gt;1)+(Assumptions!$D$121&lt;0)+(Assumptions!$D$121&gt;1)+(Assumptions!$D$122&lt;0)+(Assumptions!$D$122&gt;1)+(Assumptions!$D$123&lt;0)+(Assumptions!$D$123&gt;1))+((Assumptions!$D$9&lt;0)+(Assumptions!$D$11&lt;0)+(Assumptions!$D$12&lt;0)+(Assumptions!$D$13&lt;0)+(Assumptions!$D$14&lt;0)+(Assumptions!$D$15&lt;0)+(Assumptions!$D$19&lt;0)+(Assumptions!$D$21&lt;0)+(Assumptions!$D$22&lt;0)+(Assumptions!$D$23&lt;0)+(Assumptions!$D$24&lt;0)+(Assumptions!$D$25&lt;0)+(Assumptions!$D$49&lt;0)+(Assumptions!$D$51&lt;0)+(Assumptions!$D$68&lt;0)+(Assumptions!$D$69&lt;0)+(Assumptions!$D$70&lt;0)+(Assumptions!$D$71&lt;0)+(Assumptions!$D$76&lt;0)+(Assumptions!$D$77&lt;0)+(Assumptions!$D$78&lt;0)+(Assumptions!$D$79&lt;0)+(Assumptions!$D$83&lt;0)+(Assumptions!$D$84&lt;0)+(Assumptions!$D$85&lt;0)+(Assumptions!$D$86&lt;0)+(Assumptions!$D$87&lt;0)+(Assumptions!$D$88&lt;0)+(Assumptions!$D$90&lt;0)+(Assumptions!$D$92&lt;0)+(Assumptions!$D$97&lt;0)+(Assumptions!$D$98&lt;0)+(Assumptions!$D$103&lt;0)+(Assumptions!$D$114&lt;0)+(Assumptions!$D$116&lt;0)+(Assumptions!$D$117&lt;0)+(Assumptions!$D$118&lt;0)+(Assumptions!$D$119&lt;0)+(Assumptions!$D$120&lt;0)+(Assumptions!$D$124&lt;0)+(Assumptions!$D$151&lt;0)+(Assumptions!$D$152&lt;0)+(Assumptions!$D$153&lt;0)+(Assumptions!$D$154&lt;0)+(Assumptions!$D$157&lt;0)+(Assumptions!$D$158&lt;0)+(Assumptions!$D$159&lt;0)+(Assumptions!$D$160&lt;0)+(Assumptions!$D$162&lt;0)+(Assumptions!$D$163&lt;0)+(Assumptions!$D$164&lt;0)+(Assumptions!$D$165&lt;0)+(Assumptions!$D$167&lt;0)+(Assumptions!$D$169&lt;0)+(Assumptions!$D$170&lt;0)+(Assumptions!$D$171&lt;0)+(Assumptions!$D$173&lt;0)+(Assumptions!$D$174&lt;0)+(Assumptions!$D$175&lt;0)+(Assumptions!$D$176&lt;0)+(Assumptions!$D$177&lt;0))+((INT(Assumptions!$D$19)&lt;&gt;Assumptions!$D$19)+(INT(Assumptions!$D$21)&lt;&gt;Assumptions!$D$21)+(INT(Assumptions!$D$22)&lt;&gt;Assumptions!$D$22)+(INT(Assumptions!$D$23)&lt;&gt;Assumptions!$D$23)+(INT(Assumptions!$D$24)&lt;&gt;Assumptions!$D$24)+(INT(Assumptions!$D$25)&lt;&gt;Assumptions!$D$25))+SUMPRODUCT((Assumptions!$E$128:$E$147&lt;0)+(Assumptions!$G$128:$G$147&lt;0)+(Assumptions!$G$128:$G$147&gt;1)+(Assumptions!$H$128:$H$147&lt;0)+(Assumptions!$I$128:$I$147&lt;0)+(Assumptions!$J$128:$J$147&lt;0)+(Assumptions!$F$128:$F$147&lt;0)+((Assumptions!$D$128:$D$147="CPC")*(Assumptions!$F$128:$F$147&gt;1)))+(Assumptions!$D$48&lt;0)+(Assumptions!$D$48&gt;=1)+(Assumptions!$D$20&lt;Assumptions!$D$7)+(Assumptions!$D$20&gt;Assumptions!$D$8)+(Assumptions!$D$8&lt;=Assumptions!$D$7)+(Assumptions!$D$91&gt;=Assumptions!$D$89)+(Assumptions!$D$92&lt;Assumptions!$D$90)=0,"✓ all inputs valid","✗ invalid input: "&amp;IF(((Assumptions!$D$10&lt;0)+(Assumptions!$D$10&gt;1)+(Assumptions!$D$52&lt;0)+(Assumptions!$D$52&gt;1)+(Assumptions!$D$50&lt;0)+(Assumptions!$D$50&gt;1)+(Assumptions!$D$64&lt;0)+(Assumptions!$D$64&gt;1)+(Assumptions!$D$155&lt;0)+(Assumptions!$D$155&gt;1)+(Assumptions!$D$156&lt;0)+(Assumptions!$D$156&gt;1)+(Assumptions!$D$161&lt;0)+(Assumptions!$D$161&gt;1)+(Assumptions!$D$166&lt;0)+(Assumptions!$D$166&gt;1)+(Assumptions!$D$168&lt;0)+(Assumptions!$D$168&gt;1)+(Assumptions!$D$172&lt;0)+(Assumptions!$D$172&gt;1)+(Assumptions!$D$93&lt;0)+(Assumptions!$D$93&gt;1)+(Assumptions!$D$94&lt;0)+(Assumptions!$D$94&gt;1)+(Assumptions!$D$95&lt;0)+(Assumptions!$D$95&gt;1)+(Assumptions!$D$89&lt;0)+(Assumptions!$D$89&gt;1)+(Assumptions!$D$91&lt;0)+(Assumptions!$D$91&gt;1)+(Assumptions!$D$29&lt;0)+(Assumptions!$D$29&gt;1)+(Assumptions!$D$30&lt;0)+(Assumptions!$D$30&gt;1)+(Assumptions!$D$31&lt;0)+(Assumptions!$D$31&gt;1)+(Assumptions!$D$32&lt;0)+(Assumptions!$D$32&gt;1)+(Assumptions!$D$33&lt;0)+(Assumptions!$D$33&gt;1)+(Assumptions!$D$34&lt;0)+(Assumptions!$D$34&gt;1)+(Assumptions!$D$35&lt;0)+(Assumptions!$D$35&gt;1)+(Assumptions!$D$36&lt;0)+(Assumptions!$D$36&gt;1)+(Assumptions!$D$37&lt;0)+(Assumptions!$D$37&gt;1)+(Assumptions!$D$38&lt;0)+(Assumptions!$D$38&gt;1)+(Assumptions!$D$39&lt;0)+(Assumptions!$D$39&gt;1)+(Assumptions!$D$40&lt;0)+(Assumptions!$D$40&gt;1)+(Assumptions!$D$41&lt;0)+(Assumptions!$D$41&gt;1)+(Assumptions!$D$42&lt;0)+(Assumptions!$D$42&gt;1)+(Assumptions!$D$43&lt;0)+(Assumptions!$D$43&gt;1)+(Assumptions!$D$44&lt;0)+(Assumptions!$D$44&gt;1)+(Assumptions!$D$53&lt;0)+(Assumptions!$D$53&gt;1)+(Assumptions!$D$54&lt;0)+(Assumptions!$D$54&gt;1)+(Assumptions!$D$55&lt;0)+(Assumptions!$D$55&gt;1)+(Assumptions!$D$56&lt;0)+(Assumptions!$D$56&gt;1)+(Assumptions!$D$57&lt;0)+(Assumptions!$D$57&gt;1)+(Assumptions!$D$58&lt;0)+(Assumptions!$D$58&gt;1)+(Assumptions!$D$59&lt;0)+(Assumptions!$D$59&gt;1)+(Assumptions!$D$60&lt;0)+(Assumptions!$D$60&gt;1)+(Assumptions!$D$61&lt;0)+(Assumptions!$D$61&gt;1)+(Assumptions!$D$62&lt;0)+(Assumptions!$D$62&gt;1)+(Assumptions!$D$63&lt;0)+(Assumptions!$D$63&gt;1)+(Assumptions!$D$72&lt;0)+(Assumptions!$D$72&gt;1)+(Assumptions!$D$73&lt;0)+(Assumptions!$D$73&gt;1)+(Assumptions!$D$74&lt;0)+(Assumptions!$D$74&gt;1)+(Assumptions!$D$75&lt;0)+(Assumptions!$D$75&gt;1)+(Assumptions!$D$96&lt;0)+(Assumptions!$D$96&gt;1)+(Assumptions!$D$99&lt;0)+(Assumptions!$D$99&gt;1)+(Assumptions!$D$100&lt;0)+(Assumptions!$D$100&gt;1)+(Assumptions!$D$101&lt;0)+(Assumptions!$D$101&gt;1)+(Assumptions!$D$102&lt;0)+(Assumptions!$D$102&gt;1)+(Assumptions!$D$108&lt;0)+(Assumptions!$D$108&gt;1)+(Assumptions!$D$109&lt;0)+(Assumptions!$D$109&gt;1)+(Assumptions!$D$110&lt;0)+(Assumptions!$D$110&gt;1)+(Assumptions!$D$111&lt;0)+(Assumptions!$D$111&gt;1)+(Assumptions!$D$112&lt;0)+(Assumptions!$D$112&gt;1)+(Assumptions!$D$113&lt;0)+(Assumptions!$D$113&gt;1)+(Assumptions!$D$115&lt;0)+(Assumptions!$D$115&gt;1)+(Assumptions!$D$121&lt;0)+(Assumptions!$D$121&gt;1)+(Assumptions!$D$122&lt;0)+(Assumptions!$D$122&gt;1)+(Assumptions!$D$123&lt;0)+(Assumptions!$D$123&gt;1))&gt;0,"a share/rate is outside 0–100%; ","")&amp;IF(((Assumptions!$D$9&lt;0)+(Assumptions!$D$11&lt;0)+(Assumptions!$D$12&lt;0)+(Assumptions!$D$13&lt;0)+(Assumptions!$D$14&lt;0)+(Assumptions!$D$15&lt;0)+(Assumptions!$D$19&lt;0)+(Assumptions!$D$21&lt;0)+(Assumptions!$D$22&lt;0)+(Assumptions!$D$23&lt;0)+(Assumptions!$D$24&lt;0)+(Assumptions!$D$25&lt;0)+(Assumptions!$D$49&lt;0)+(Assumptions!$D$51&lt;0)+(Assumptions!$D$68&lt;0)+(Assumptions!$D$69&lt;0)+(Assumptions!$D$70&lt;0)+(Assumptions!$D$71&lt;0)+(Assumptions!$D$76&lt;0)+(Assumptions!$D$77&lt;0)+(Assumptions!$D$78&lt;0)+(Assumptions!$D$79&lt;0)+(Assumptions!$D$83&lt;0)+(Assumptions!$D$84&lt;0)+(Assumptions!$D$85&lt;0)+(Assumptions!$D$86&lt;0)+(Assumptions!$D$87&lt;0)+(Assumptions!$D$88&lt;0)+(Assumptions!$D$90&lt;0)+(Assumptions!$D$92&lt;0)+(Assumptions!$D$97&lt;0)+(Assumptions!$D$98&lt;0)+(Assumptions!$D$103&lt;0)+(Assumptions!$D$114&lt;0)+(Assumptions!$D$116&lt;0)+(Assumptions!$D$117&lt;0)+(Assumptions!$D$118&lt;0)+(Assumptions!$D$119&lt;0)+(Assumptions!$D$120&lt;0)+(Assumptions!$D$124&lt;0)+(Assumptions!$D$151&lt;0)+(Assumptions!$D$152&lt;0)+(Assumptions!$D$153&lt;0)+(Assumptions!$D$154&lt;0)+(Assumptions!$D$157&lt;0)+(Assumptions!$D$158&lt;0)+(Assumptions!$D$159&lt;0)+(Assumptions!$D$160&lt;0)+(Assumptions!$D$162&lt;0)+(Assumptions!$D$163&lt;0)+(Assumptions!$D$164&lt;0)+(Assumptions!$D$165&lt;0)+(Assumptions!$D$167&lt;0)+(Assumptions!$D$169&lt;0)+(Assumptions!$D$170&lt;0)+(Assumptions!$D$171&lt;0)+(Assumptions!$D$173&lt;0)+(Assumptions!$D$174&lt;0)+(Assumptions!$D$175&lt;0)+(Assumptions!$D$176&lt;0)+(Assumptions!$D$177&lt;0))&gt;0,"a count, cost or day value is negative; ","")&amp;IF(((INT(Assumptions!$D$19)&lt;&gt;Assumptions!$D$19)+(INT(Assumptions!$D$21)&lt;&gt;Assumptions!$D$21)+(INT(Assumptions!$D$22)&lt;&gt;Assumptions!$D$22)+(INT(Assumptions!$D$23)&lt;&gt;Assumptions!$D$23)+(INT(Assumptions!$D$24)&lt;&gt;Assumptions!$D$24)+(INT(Assumptions!$D$25)&lt;&gt;Assumptions!$D$25))&gt;0,"day inputs (T0, T2–T6) must be whole days; ","")&amp;IF(SUMPRODUCT((Assumptions!$E$128:$E$147&lt;0)+(Assumptions!$G$128:$G$147&lt;0)+(Assumptions!$G$128:$G$147&gt;1)+(Assumptions!$H$128:$H$147&lt;0)+(Assumptions!$I$128:$I$147&lt;0)+(Assumptions!$J$128:$J$147&lt;0)+(Assumptions!$F$128:$F$147&lt;0)+((Assumptions!$D$128:$D$147="CPC")*(Assumptions!$F$128:$F$147&gt;1)))&gt;0,"a channel input (Assumptions §7) is out of range; ","")&amp;IF(OR(Assumptions!$D$48&lt;0,Assumptions!$D$48&gt;=1),"reserve share must be 0–99%; ","")&amp;IF(OR(Assumptions!$D$20&lt;Assumptions!$D$7,Assumptions!$D$20&gt;Assumptions!$D$8),"last signing date must fall inside the campaign; ","")&amp;IF(Assumptions!$D$8&lt;=Assumptions!$D$7,"campaign end must be after its start; ","")&amp;IF(OR(Assumptions!$D$91&gt;=Assumptions!$D$89,Assumptions!$D$92&lt;Assumptions!$D$90),"initiative kill thresholds must sit below pass thresholds (TK1 &lt; TP1, TK2 ≥ TP2); ",""))</f>
+        <f aca="false">IF(((Assumptions!$D$10&lt;0)+(Assumptions!$D$10&gt;1)+(Assumptions!$D$52&lt;0)+(Assumptions!$D$52&gt;1)+(Assumptions!$D$50&lt;0)+(Assumptions!$D$50&gt;1)+(Assumptions!$D$64&lt;0)+(Assumptions!$D$64&gt;1)+(Assumptions!$D$155&lt;0)+(Assumptions!$D$155&gt;1)+(Assumptions!$D$156&lt;0)+(Assumptions!$D$156&gt;1)+(Assumptions!$D$161&lt;0)+(Assumptions!$D$161&gt;1)+(Assumptions!$D$166&lt;0)+(Assumptions!$D$166&gt;1)+(Assumptions!$D$168&lt;0)+(Assumptions!$D$168&gt;1)+(Assumptions!$D$172&lt;0)+(Assumptions!$D$172&gt;1)+(Assumptions!$D$93&lt;0)+(Assumptions!$D$93&gt;1)+(Assumptions!$D$94&lt;0)+(Assumptions!$D$94&gt;1)+(Assumptions!$D$95&lt;0)+(Assumptions!$D$95&gt;1)+(Assumptions!$D$89&lt;0)+(Assumptions!$D$89&gt;1)+(Assumptions!$D$91&lt;0)+(Assumptions!$D$91&gt;1)+(Assumptions!$D$29&lt;0)+(Assumptions!$D$29&gt;1)+(Assumptions!$D$30&lt;0)+(Assumptions!$D$30&gt;1)+(Assumptions!$D$31&lt;0)+(Assumptions!$D$31&gt;1)+(Assumptions!$D$32&lt;0)+(Assumptions!$D$32&gt;1)+(Assumptions!$D$33&lt;0)+(Assumptions!$D$33&gt;1)+(Assumptions!$D$34&lt;0)+(Assumptions!$D$34&gt;1)+(Assumptions!$D$35&lt;0)+(Assumptions!$D$35&gt;1)+(Assumptions!$D$36&lt;0)+(Assumptions!$D$36&gt;1)+(Assumptions!$D$37&lt;0)+(Assumptions!$D$37&gt;1)+(Assumptions!$D$38&lt;0)+(Assumptions!$D$38&gt;1)+(Assumptions!$D$39&lt;0)+(Assumptions!$D$39&gt;1)+(Assumptions!$D$40&lt;0)+(Assumptions!$D$40&gt;1)+(Assumptions!$D$41&lt;0)+(Assumptions!$D$41&gt;1)+(Assumptions!$D$42&lt;0)+(Assumptions!$D$42&gt;1)+(Assumptions!$D$43&lt;0)+(Assumptions!$D$43&gt;1)+(Assumptions!$D$44&lt;0)+(Assumptions!$D$44&gt;1)+(Assumptions!$D$53&lt;0)+(Assumptions!$D$53&gt;1)+(Assumptions!$D$54&lt;0)+(Assumptions!$D$54&gt;1)+(Assumptions!$D$55&lt;0)+(Assumptions!$D$55&gt;1)+(Assumptions!$D$56&lt;0)+(Assumptions!$D$56&gt;1)+(Assumptions!$D$57&lt;0)+(Assumptions!$D$57&gt;1)+(Assumptions!$D$58&lt;0)+(Assumptions!$D$58&gt;1)+(Assumptions!$D$59&lt;0)+(Assumptions!$D$59&gt;1)+(Assumptions!$D$60&lt;0)+(Assumptions!$D$60&gt;1)+(Assumptions!$D$61&lt;0)+(Assumptions!$D$61&gt;1)+(Assumptions!$D$62&lt;0)+(Assumptions!$D$62&gt;1)+(Assumptions!$D$63&lt;0)+(Assumptions!$D$63&gt;1)+(Assumptions!$D$72&lt;0)+(Assumptions!$D$72&gt;1)+(Assumptions!$D$73&lt;0)+(Assumptions!$D$73&gt;1)+(Assumptions!$D$74&lt;0)+(Assumptions!$D$74&gt;1)+(Assumptions!$D$75&lt;0)+(Assumptions!$D$75&gt;1)+(Assumptions!$D$96&lt;0)+(Assumptions!$D$96&gt;1)+(Assumptions!$D$99&lt;0)+(Assumptions!$D$99&gt;1)+(Assumptions!$D$100&lt;0)+(Assumptions!$D$100&gt;1)+(Assumptions!$D$101&lt;0)+(Assumptions!$D$101&gt;1)+(Assumptions!$D$102&lt;0)+(Assumptions!$D$102&gt;1)+(Assumptions!$D$108&lt;0)+(Assumptions!$D$108&gt;1)+(Assumptions!$D$109&lt;0)+(Assumptions!$D$109&gt;1)+(Assumptions!$D$110&lt;0)+(Assumptions!$D$110&gt;1)+(Assumptions!$D$111&lt;0)+(Assumptions!$D$111&gt;1)+(Assumptions!$D$112&lt;0)+(Assumptions!$D$112&gt;1)+(Assumptions!$D$113&lt;0)+(Assumptions!$D$113&gt;1)+(Assumptions!$D$115&lt;0)+(Assumptions!$D$115&gt;1)+(Assumptions!$D$121&lt;0)+(Assumptions!$D$121&gt;1)+(Assumptions!$D$122&lt;0)+(Assumptions!$D$122&gt;1)+(Assumptions!$D$123&lt;0)+(Assumptions!$D$123&gt;1))+((Assumptions!$D$9&lt;0)+(Assumptions!$D$11&lt;0)+(Assumptions!$D$12&lt;0)+(Assumptions!$D$13&lt;0)+(Assumptions!$D$14&lt;0)+(Assumptions!$D$15&lt;0)+(Assumptions!$D$19&lt;0)+(Assumptions!$D$21&lt;0)+(Assumptions!$D$22&lt;0)+(Assumptions!$D$23&lt;0)+(Assumptions!$D$24&lt;0)+(Assumptions!$D$25&lt;0)+(Assumptions!$D$49&lt;0)+(Assumptions!$D$51&lt;0)+(Assumptions!$D$68&lt;0)+(Assumptions!$D$69&lt;0)+(Assumptions!$D$70&lt;0)+(Assumptions!$D$71&lt;0)+(Assumptions!$D$76&lt;0)+(Assumptions!$D$77&lt;0)+(Assumptions!$D$78&lt;0)+(Assumptions!$D$79&lt;0)+(Assumptions!$D$83&lt;0)+(Assumptions!$D$84&lt;0)+(Assumptions!$D$85&lt;0)+(Assumptions!$D$86&lt;0)+(Assumptions!$D$87&lt;0)+(Assumptions!$D$88&lt;0)+(Assumptions!$D$90&lt;0)+(Assumptions!$D$92&lt;0)+(Assumptions!$D$97&lt;0)+(Assumptions!$D$98&lt;0)+(Assumptions!$D$103&lt;0)+(Assumptions!$D$114&lt;0)+(Assumptions!$D$116&lt;0)+(Assumptions!$D$117&lt;0)+(Assumptions!$D$118&lt;0)+(Assumptions!$D$119&lt;0)+(Assumptions!$D$120&lt;0)+(Assumptions!$D$124&lt;0)+(Assumptions!$D$151&lt;0)+(Assumptions!$D$152&lt;0)+(Assumptions!$D$153&lt;0)+(Assumptions!$D$154&lt;0)+(Assumptions!$D$157&lt;0)+(Assumptions!$D$158&lt;0)+(Assumptions!$D$159&lt;0)+(Assumptions!$D$160&lt;0)+(Assumptions!$D$162&lt;0)+(Assumptions!$D$163&lt;0)+(Assumptions!$D$164&lt;0)+(Assumptions!$D$165&lt;0)+(Assumptions!$D$167&lt;0)+(Assumptions!$D$169&lt;0)+(Assumptions!$D$170&lt;0)+(Assumptions!$D$171&lt;0)+(Assumptions!$D$173&lt;0)+(Assumptions!$D$174&lt;0)+(Assumptions!$D$175&lt;0)+(Assumptions!$D$176&lt;0)+(Assumptions!$D$177&lt;0)+(Assumptions!$D$178&lt;0)+(Assumptions!$D$179&lt;0))+((INT(Assumptions!$D$19)&lt;&gt;Assumptions!$D$19)+(INT(Assumptions!$D$21)&lt;&gt;Assumptions!$D$21)+(INT(Assumptions!$D$22)&lt;&gt;Assumptions!$D$22)+(INT(Assumptions!$D$23)&lt;&gt;Assumptions!$D$23)+(INT(Assumptions!$D$24)&lt;&gt;Assumptions!$D$24)+(INT(Assumptions!$D$25)&lt;&gt;Assumptions!$D$25))+SUMPRODUCT((Assumptions!$E$128:$E$147&lt;0)+(Assumptions!$G$128:$G$147&lt;0)+(Assumptions!$G$128:$G$147&gt;1)+(Assumptions!$H$128:$H$147&lt;0)+(Assumptions!$I$128:$I$147&lt;0)+(Assumptions!$J$128:$J$147&lt;0)+(Assumptions!$F$128:$F$147&lt;0)+((Assumptions!$D$128:$D$147="CPC")*(Assumptions!$F$128:$F$147&gt;1)))+(Assumptions!$D$48&lt;0)+(Assumptions!$D$48&gt;=1)+(Assumptions!$D$20&lt;Assumptions!$D$7)+(Assumptions!$D$20&gt;Assumptions!$D$8)+(Assumptions!$D$8&lt;=Assumptions!$D$7)+(Assumptions!$D$91&gt;=Assumptions!$D$89)+(Assumptions!$D$92&lt;Assumptions!$D$90)=0,"✓ all inputs valid","✗ invalid input: "&amp;IF(((Assumptions!$D$10&lt;0)+(Assumptions!$D$10&gt;1)+(Assumptions!$D$52&lt;0)+(Assumptions!$D$52&gt;1)+(Assumptions!$D$50&lt;0)+(Assumptions!$D$50&gt;1)+(Assumptions!$D$64&lt;0)+(Assumptions!$D$64&gt;1)+(Assumptions!$D$155&lt;0)+(Assumptions!$D$155&gt;1)+(Assumptions!$D$156&lt;0)+(Assumptions!$D$156&gt;1)+(Assumptions!$D$161&lt;0)+(Assumptions!$D$161&gt;1)+(Assumptions!$D$166&lt;0)+(Assumptions!$D$166&gt;1)+(Assumptions!$D$168&lt;0)+(Assumptions!$D$168&gt;1)+(Assumptions!$D$172&lt;0)+(Assumptions!$D$172&gt;1)+(Assumptions!$D$93&lt;0)+(Assumptions!$D$93&gt;1)+(Assumptions!$D$94&lt;0)+(Assumptions!$D$94&gt;1)+(Assumptions!$D$95&lt;0)+(Assumptions!$D$95&gt;1)+(Assumptions!$D$89&lt;0)+(Assumptions!$D$89&gt;1)+(Assumptions!$D$91&lt;0)+(Assumptions!$D$91&gt;1)+(Assumptions!$D$29&lt;0)+(Assumptions!$D$29&gt;1)+(Assumptions!$D$30&lt;0)+(Assumptions!$D$30&gt;1)+(Assumptions!$D$31&lt;0)+(Assumptions!$D$31&gt;1)+(Assumptions!$D$32&lt;0)+(Assumptions!$D$32&gt;1)+(Assumptions!$D$33&lt;0)+(Assumptions!$D$33&gt;1)+(Assumptions!$D$34&lt;0)+(Assumptions!$D$34&gt;1)+(Assumptions!$D$35&lt;0)+(Assumptions!$D$35&gt;1)+(Assumptions!$D$36&lt;0)+(Assumptions!$D$36&gt;1)+(Assumptions!$D$37&lt;0)+(Assumptions!$D$37&gt;1)+(Assumptions!$D$38&lt;0)+(Assumptions!$D$38&gt;1)+(Assumptions!$D$39&lt;0)+(Assumptions!$D$39&gt;1)+(Assumptions!$D$40&lt;0)+(Assumptions!$D$40&gt;1)+(Assumptions!$D$41&lt;0)+(Assumptions!$D$41&gt;1)+(Assumptions!$D$42&lt;0)+(Assumptions!$D$42&gt;1)+(Assumptions!$D$43&lt;0)+(Assumptions!$D$43&gt;1)+(Assumptions!$D$44&lt;0)+(Assumptions!$D$44&gt;1)+(Assumptions!$D$53&lt;0)+(Assumptions!$D$53&gt;1)+(Assumptions!$D$54&lt;0)+(Assumptions!$D$54&gt;1)+(Assumptions!$D$55&lt;0)+(Assumptions!$D$55&gt;1)+(Assumptions!$D$56&lt;0)+(Assumptions!$D$56&gt;1)+(Assumptions!$D$57&lt;0)+(Assumptions!$D$57&gt;1)+(Assumptions!$D$58&lt;0)+(Assumptions!$D$58&gt;1)+(Assumptions!$D$59&lt;0)+(Assumptions!$D$59&gt;1)+(Assumptions!$D$60&lt;0)+(Assumptions!$D$60&gt;1)+(Assumptions!$D$61&lt;0)+(Assumptions!$D$61&gt;1)+(Assumptions!$D$62&lt;0)+(Assumptions!$D$62&gt;1)+(Assumptions!$D$63&lt;0)+(Assumptions!$D$63&gt;1)+(Assumptions!$D$72&lt;0)+(Assumptions!$D$72&gt;1)+(Assumptions!$D$73&lt;0)+(Assumptions!$D$73&gt;1)+(Assumptions!$D$74&lt;0)+(Assumptions!$D$74&gt;1)+(Assumptions!$D$75&lt;0)+(Assumptions!$D$75&gt;1)+(Assumptions!$D$96&lt;0)+(Assumptions!$D$96&gt;1)+(Assumptions!$D$99&lt;0)+(Assumptions!$D$99&gt;1)+(Assumptions!$D$100&lt;0)+(Assumptions!$D$100&gt;1)+(Assumptions!$D$101&lt;0)+(Assumptions!$D$101&gt;1)+(Assumptions!$D$102&lt;0)+(Assumptions!$D$102&gt;1)+(Assumptions!$D$108&lt;0)+(Assumptions!$D$108&gt;1)+(Assumptions!$D$109&lt;0)+(Assumptions!$D$109&gt;1)+(Assumptions!$D$110&lt;0)+(Assumptions!$D$110&gt;1)+(Assumptions!$D$111&lt;0)+(Assumptions!$D$111&gt;1)+(Assumptions!$D$112&lt;0)+(Assumptions!$D$112&gt;1)+(Assumptions!$D$113&lt;0)+(Assumptions!$D$113&gt;1)+(Assumptions!$D$115&lt;0)+(Assumptions!$D$115&gt;1)+(Assumptions!$D$121&lt;0)+(Assumptions!$D$121&gt;1)+(Assumptions!$D$122&lt;0)+(Assumptions!$D$122&gt;1)+(Assumptions!$D$123&lt;0)+(Assumptions!$D$123&gt;1))&gt;0,"a share/rate is outside 0–100%; ","")&amp;IF(((Assumptions!$D$9&lt;0)+(Assumptions!$D$11&lt;0)+(Assumptions!$D$12&lt;0)+(Assumptions!$D$13&lt;0)+(Assumptions!$D$14&lt;0)+(Assumptions!$D$15&lt;0)+(Assumptions!$D$19&lt;0)+(Assumptions!$D$21&lt;0)+(Assumptions!$D$22&lt;0)+(Assumptions!$D$23&lt;0)+(Assumptions!$D$24&lt;0)+(Assumptions!$D$25&lt;0)+(Assumptions!$D$49&lt;0)+(Assumptions!$D$51&lt;0)+(Assumptions!$D$68&lt;0)+(Assumptions!$D$69&lt;0)+(Assumptions!$D$70&lt;0)+(Assumptions!$D$71&lt;0)+(Assumptions!$D$76&lt;0)+(Assumptions!$D$77&lt;0)+(Assumptions!$D$78&lt;0)+(Assumptions!$D$79&lt;0)+(Assumptions!$D$83&lt;0)+(Assumptions!$D$84&lt;0)+(Assumptions!$D$85&lt;0)+(Assumptions!$D$86&lt;0)+(Assumptions!$D$87&lt;0)+(Assumptions!$D$88&lt;0)+(Assumptions!$D$90&lt;0)+(Assumptions!$D$92&lt;0)+(Assumptions!$D$97&lt;0)+(Assumptions!$D$98&lt;0)+(Assumptions!$D$103&lt;0)+(Assumptions!$D$114&lt;0)+(Assumptions!$D$116&lt;0)+(Assumptions!$D$117&lt;0)+(Assumptions!$D$118&lt;0)+(Assumptions!$D$119&lt;0)+(Assumptions!$D$120&lt;0)+(Assumptions!$D$124&lt;0)+(Assumptions!$D$151&lt;0)+(Assumptions!$D$152&lt;0)+(Assumptions!$D$153&lt;0)+(Assumptions!$D$154&lt;0)+(Assumptions!$D$157&lt;0)+(Assumptions!$D$158&lt;0)+(Assumptions!$D$159&lt;0)+(Assumptions!$D$160&lt;0)+(Assumptions!$D$162&lt;0)+(Assumptions!$D$163&lt;0)+(Assumptions!$D$164&lt;0)+(Assumptions!$D$165&lt;0)+(Assumptions!$D$167&lt;0)+(Assumptions!$D$169&lt;0)+(Assumptions!$D$170&lt;0)+(Assumptions!$D$171&lt;0)+(Assumptions!$D$173&lt;0)+(Assumptions!$D$174&lt;0)+(Assumptions!$D$175&lt;0)+(Assumptions!$D$176&lt;0)+(Assumptions!$D$177&lt;0)+(Assumptions!$D$178&lt;0)+(Assumptions!$D$179&lt;0))&gt;0,"a count, cost or day value is negative; ","")&amp;IF(((INT(Assumptions!$D$19)&lt;&gt;Assumptions!$D$19)+(INT(Assumptions!$D$21)&lt;&gt;Assumptions!$D$21)+(INT(Assumptions!$D$22)&lt;&gt;Assumptions!$D$22)+(INT(Assumptions!$D$23)&lt;&gt;Assumptions!$D$23)+(INT(Assumptions!$D$24)&lt;&gt;Assumptions!$D$24)+(INT(Assumptions!$D$25)&lt;&gt;Assumptions!$D$25))&gt;0,"day inputs (T0, T2–T6) must be whole days; ","")&amp;IF(SUMPRODUCT((Assumptions!$E$128:$E$147&lt;0)+(Assumptions!$G$128:$G$147&lt;0)+(Assumptions!$G$128:$G$147&gt;1)+(Assumptions!$H$128:$H$147&lt;0)+(Assumptions!$I$128:$I$147&lt;0)+(Assumptions!$J$128:$J$147&lt;0)+(Assumptions!$F$128:$F$147&lt;0)+((Assumptions!$D$128:$D$147="CPC")*(Assumptions!$F$128:$F$147&gt;1)))&gt;0,"a channel input (Assumptions §7) is out of range; ","")&amp;IF(OR(Assumptions!$D$48&lt;0,Assumptions!$D$48&gt;=1),"reserve share must be 0–99%; ","")&amp;IF(OR(Assumptions!$D$20&lt;Assumptions!$D$7,Assumptions!$D$20&gt;Assumptions!$D$8),"last signing date must fall inside the campaign; ","")&amp;IF(Assumptions!$D$8&lt;=Assumptions!$D$7,"campaign end must be after its start; ","")&amp;IF(OR(Assumptions!$D$91&gt;=Assumptions!$D$89,Assumptions!$D$92&lt;Assumptions!$D$90),"initiative kill thresholds must sit below pass thresholds (TK1 &lt; TP1, TK2 ≥ TP2); ",""))</f>
         <v>✓ all inputs valid</v>
       </c>
     </row>
@@ -3198,7 +3255,7 @@
     <tabColor rgb="FFFFC000"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L177"/>
+  <dimension ref="A1:L179"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
@@ -4222,7 +4279,7 @@
         <v>131</v>
       </c>
       <c r="D53" s="16" t="n">
-        <v>0.25</v>
+        <v>0.316</v>
       </c>
       <c r="E53" s="2" t="s">
         <v>44</v>
@@ -4245,7 +4302,7 @@
         <v>131</v>
       </c>
       <c r="D54" s="16" t="n">
-        <v>0.145</v>
+        <v>0.131</v>
       </c>
       <c r="E54" s="2" t="s">
         <v>44</v>
@@ -4268,7 +4325,7 @@
         <v>131</v>
       </c>
       <c r="D55" s="16" t="n">
-        <v>0.18</v>
+        <v>0.161</v>
       </c>
       <c r="E55" s="2" t="s">
         <v>44</v>
@@ -4291,7 +4348,7 @@
         <v>131</v>
       </c>
       <c r="D56" s="16" t="n">
-        <v>0.185</v>
+        <v>0.17</v>
       </c>
       <c r="E56" s="2" t="s">
         <v>44</v>
@@ -4314,7 +4371,7 @@
         <v>131</v>
       </c>
       <c r="D57" s="16" t="n">
-        <v>0.215</v>
+        <v>0.195</v>
       </c>
       <c r="E57" s="2" t="s">
         <v>44</v>
@@ -4337,7 +4394,7 @@
         <v>131</v>
       </c>
       <c r="D58" s="16" t="n">
-        <v>0.025</v>
+        <v>0.027</v>
       </c>
       <c r="E58" s="2" t="s">
         <v>44</v>
@@ -7225,6 +7282,52 @@
       </c>
       <c r="G177" s="17" t="s">
         <v>430</v>
+      </c>
+    </row>
+    <row r="178" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A178" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="B178" s="13" t="s">
+        <v>432</v>
+      </c>
+      <c r="C178" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="D178" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="E178" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="F178" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="G178" s="13" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="179" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A179" s="2" t="s">
+        <v>434</v>
+      </c>
+      <c r="B179" s="13" t="s">
+        <v>435</v>
+      </c>
+      <c r="C179" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D179" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="E179" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="F179" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="G179" s="13" t="s">
+        <v>436</v>
       </c>
     </row>
   </sheetData>
@@ -7245,7 +7348,7 @@
       <formula1>DATE(2026,10,20)</formula1>
       <formula2>DATE(2026,12,31)</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" error="Enter a whole number of days (0 or more)." errorStyle="stop" errorTitle="Whole days" operator="greaterThanOrEqual" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D19 D21:D25 D119" type="whole">
+    <dataValidation allowBlank="false" error="Enter a whole number of days (0 or more)." errorStyle="stop" errorTitle="Whole days" operator="greaterThanOrEqual" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D19 D21:D25 D119 D178:D179" type="whole">
       <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -7299,7 +7402,7 @@
     <hyperlink ref="G118" r:id="rId46" display="Redline 2024–26: mean 29.5 qualified applications per Elektroniker campaign (11 campaigns). https://redline-grow.de/bewerbungen-pro-stelle"/>
     <hyperlink ref="G119" r:id="rId47" display="A StepStone ad runs 30 days. https://www.stepstone.de/e-recruiting/stellenanzeige-aufgeben/"/>
     <hyperlink ref="G120" r:id="rId48" display="Plant headcount (Electrek, March 2026). https://electrek.co/2026/03/04/tesla-giga-berlin-ig-metall-union-vote-collapse/"/>
-    <hyperlink ref="G121" r:id="rId49" display="BA employment, Germany: maintenance codes 2513 + 2625 + 2611 + 2612 + supervisors 2519 + 2619 + 2629 (536,520) ÷ production occupations 21–29 (6,850,263) = 7.8%. https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-d-0-202512-xlsx.xlsx?__blob=publicationFile"/>
+    <hyperlink ref="G121" r:id="rId49" display="BA employment, Germany: maintenance codes 2513 + 2625 + 2611 + 2612 + supervisors 2519 + 2619 + 2629 (536,520) ÷ production occupations 21–29 (6,850,263) = 7.8%. Also applied to Polish industry for the I3 supply check (my estimate; an upper bound). https://statistik.arbeitsagentur.de/Statistikdaten/Detail/202512/iiia6/beschaeftigung-sozbe-bo-heft/bo-heft-d-0-202512-xlsx.xlsx?__blob=publicationFile"/>
     <hyperlink ref="G122" r:id="rId50" display="IAB-Betriebspanel Brandenburg: ~6% of jobs ended in the first half of 2024 → ~12% a year. https://mweke.brandenburg.de/media/bb1.a.3814.de/Betriebspanel%20Brandenburg%202024%20-%20final.pdf"/>
     <hyperlink ref="G123" r:id="rId51" display="Referrals bring ~11% of hires (CareerPlug 2025). https://www.careerplug.com/wp-content/uploads/2025/04/Recruiting-Metrics-Report.pdf"/>
     <hyperlink ref="G124" r:id="rId52" display="Eurostat lfst_r_lfe2en2, 2025: Lubuskie (PL43) 97.0k + Zachodniopomorskie (PL42) 140.5k employed in industry B–E (https://ec.europa.eu/eurostat/databrowser/view/lfst_r_lfe2en2/default/table)."/>
@@ -7366,12 +7469,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>431</v>
+        <v>437</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>432</v>
+        <v>438</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7382,46 +7485,46 @@
         <v>47</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>433</v>
+        <v>439</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>434</v>
+        <v>440</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>435</v>
+        <v>441</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>436</v>
+        <v>442</v>
       </c>
       <c r="G4" s="12" t="s">
-        <v>437</v>
+        <v>443</v>
       </c>
       <c r="H4" s="12" t="s">
-        <v>438</v>
+        <v>444</v>
       </c>
       <c r="I4" s="12" t="s">
-        <v>439</v>
+        <v>445</v>
       </c>
       <c r="J4" s="12" t="s">
-        <v>440</v>
+        <v>446</v>
       </c>
       <c r="K4" s="12" t="s">
-        <v>441</v>
+        <v>447</v>
       </c>
       <c r="L4" s="12" t="s">
-        <v>442</v>
+        <v>448</v>
       </c>
       <c r="M4" s="12" t="s">
-        <v>443</v>
+        <v>449</v>
       </c>
       <c r="N4" s="12" t="s">
-        <v>444</v>
+        <v>450</v>
       </c>
       <c r="O4" s="12" t="s">
-        <v>445</v>
+        <v>451</v>
       </c>
       <c r="P4" s="12" t="s">
-        <v>446</v>
+        <v>452</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7686,7 +7789,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="28" t="s">
-        <v>447</v>
+        <v>453</v>
       </c>
       <c r="B9" s="33" t="n">
         <f aca="false">SUM(B5:B8)</f>
@@ -7731,17 +7834,17 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>448</v>
+        <v>454</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="28" t="s">
-        <v>449</v>
+        <v>455</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>450</v>
+        <v>456</v>
       </c>
       <c r="B13" s="36" t="n">
         <f aca="false">Assumptions!$D$7+Assumptions!$D$19</f>
@@ -7750,7 +7853,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>451</v>
+        <v>457</v>
       </c>
       <c r="B14" s="36" t="n">
         <f aca="false">Assumptions!$D$20</f>
@@ -7759,7 +7862,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>452</v>
+        <v>458</v>
       </c>
       <c r="B15" s="29" t="n">
         <f aca="false">Assumptions!$D$22+Assumptions!$D$23+Assumptions!$D$24</f>
@@ -7768,7 +7871,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>453</v>
+        <v>459</v>
       </c>
       <c r="B16" s="29" t="n">
         <f aca="false">B15+Assumptions!$D$25</f>
@@ -7777,7 +7880,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>454</v>
+        <v>460</v>
       </c>
       <c r="B17" s="36" t="n">
         <f aca="false">B14-B15</f>
@@ -7786,7 +7889,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>455</v>
+        <v>461</v>
       </c>
       <c r="B18" s="36" t="n">
         <f aca="false">B14-B16</f>
@@ -7813,7 +7916,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>456</v>
+        <v>462</v>
       </c>
       <c r="B21" s="29" t="n">
         <f aca="false">MAX(0,B17-B13+1)</f>
@@ -7831,7 +7934,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>457</v>
+        <v>463</v>
       </c>
       <c r="B23" s="29" t="n">
         <f aca="false">O9</f>
@@ -7853,7 +7956,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>458</v>
+        <v>464</v>
       </c>
       <c r="B25" s="31" t="n">
         <f aca="false">IF(O9&gt;0,Channels!U35/O9,0)</f>
@@ -7862,19 +7965,19 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>459</v>
+        <v>465</v>
       </c>
       <c r="B26" s="38" t="n">
         <f aca="false">B22*B25</f>
         <v>102.049737036446</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>460</v>
+        <v>466</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="28" t="s">
-        <v>461</v>
+        <v>467</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7885,34 +7988,34 @@
         <v>47</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>462</v>
+        <v>468</v>
       </c>
       <c r="D29" s="12" t="s">
-        <v>463</v>
+        <v>469</v>
       </c>
       <c r="E29" s="12" t="s">
-        <v>464</v>
+        <v>470</v>
       </c>
       <c r="F29" s="12" t="s">
-        <v>465</v>
+        <v>471</v>
       </c>
       <c r="G29" s="12" t="s">
-        <v>466</v>
+        <v>472</v>
       </c>
       <c r="H29" s="12" t="s">
-        <v>467</v>
+        <v>473</v>
       </c>
       <c r="I29" s="12" t="s">
-        <v>468</v>
+        <v>474</v>
       </c>
       <c r="J29" s="12" t="s">
-        <v>469</v>
+        <v>475</v>
       </c>
       <c r="K29" s="12" t="s">
-        <v>470</v>
+        <v>476</v>
       </c>
       <c r="L29" s="12" t="s">
-        <v>471</v>
+        <v>477</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7948,10 +8051,10 @@
         <v>2271.6049382716</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>472</v>
+        <v>478</v>
       </c>
       <c r="J30" s="2" t="s">
-        <v>473</v>
+        <v>479</v>
       </c>
       <c r="K30" s="40" t="n">
         <f aca="false">IF(B30&gt;0,(D30-SUMIFS(Channels!$N:$N,Channels!$A:$A,"I2-E",Channels!$C:$C,A30))/B30,0)</f>
@@ -7995,10 +8098,10 @@
         <v>1927.42237186682</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>474</v>
+        <v>480</v>
       </c>
       <c r="J31" s="2" t="s">
-        <v>475</v>
+        <v>481</v>
       </c>
       <c r="K31" s="40" t="n">
         <f aca="false">IF(B31&gt;0,(D31-SUMIFS(Channels!$N:$N,Channels!$A:$A,"I2-E",Channels!$C:$C,A31))/B31,0)</f>
@@ -8042,10 +8145,10 @@
         <v>1504.99706055262</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>472</v>
+        <v>478</v>
       </c>
       <c r="J32" s="2" t="s">
-        <v>475</v>
+        <v>481</v>
       </c>
       <c r="K32" s="40" t="n">
         <f aca="false">IF(B32&gt;0,(D32-SUMIFS(Channels!$N:$N,Channels!$A:$A,"I2-E",Channels!$C:$C,A32))/B32,0)</f>
@@ -8089,10 +8192,10 @@
         <v>1948.60552916819</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>472</v>
+        <v>478</v>
       </c>
       <c r="J33" s="2" t="s">
-        <v>475</v>
+        <v>481</v>
       </c>
       <c r="K33" s="40" t="n">
         <f aca="false">IF(B33&gt;0,(D33-SUMIFS(Channels!$N:$N,Channels!$A:$A,"I2-E",Channels!$C:$C,A33))/B33,0)</f>
@@ -8144,12 +8247,12 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="28" t="s">
-        <v>476</v>
+        <v>482</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
-        <v>477</v>
+        <v>483</v>
       </c>
       <c r="B40" s="30" t="n">
         <f aca="false">Assumptions!$D$64</f>
@@ -8158,33 +8261,33 @@
     </row>
     <row r="41" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="12" t="s">
-        <v>478</v>
+        <v>484</v>
       </c>
       <c r="B41" s="12" t="s">
-        <v>479</v>
+        <v>485</v>
       </c>
       <c r="C41" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D41" s="12" t="s">
-        <v>480</v>
+        <v>486</v>
       </c>
       <c r="E41" s="12" t="s">
-        <v>481</v>
+        <v>487</v>
       </c>
       <c r="F41" s="12" t="s">
-        <v>482</v>
+        <v>488</v>
       </c>
       <c r="G41" s="12" t="s">
-        <v>483</v>
+        <v>489</v>
       </c>
       <c r="H41" s="12" t="s">
-        <v>484</v>
+        <v>490</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="13" t="s">
-        <v>485</v>
+        <v>491</v>
       </c>
       <c r="B42" s="29" t="n">
         <f aca="false">O9</f>
@@ -8211,12 +8314,12 @@
         <v>0</v>
       </c>
       <c r="H42" s="13" t="s">
-        <v>486</v>
+        <v>492</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="13" t="s">
-        <v>487</v>
+        <v>493</v>
       </c>
       <c r="B43" s="29" t="n">
         <f aca="false">O9/(1-$B$40)</f>
@@ -8243,12 +8346,12 @@
         <v>0.428571428571429</v>
       </c>
       <c r="H43" s="13" t="s">
-        <v>488</v>
+        <v>494</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="13" t="s">
-        <v>489</v>
+        <v>495</v>
       </c>
       <c r="B44" s="29" t="n">
         <f aca="false">O9/(1-$B$40)</f>
@@ -8275,12 +8378,12 @@
         <v>0.428571428571429</v>
       </c>
       <c r="H44" s="13" t="s">
-        <v>490</v>
+        <v>496</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="13" t="s">
-        <v>491</v>
+        <v>497</v>
       </c>
       <c r="B45" s="29" t="n">
         <f aca="false">O9</f>
@@ -8307,12 +8410,12 @@
         <v>0.428571428571429</v>
       </c>
       <c r="H45" s="13" t="s">
-        <v>492</v>
+        <v>498</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="13" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="B46" s="29" t="n">
         <f aca="false">O9</f>
@@ -8339,12 +8442,12 @@
         <v>0.3</v>
       </c>
       <c r="H46" s="13" t="s">
-        <v>494</v>
+        <v>500</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="13" t="s">
-        <v>495</v>
+        <v>501</v>
       </c>
       <c r="B47" s="29" t="n">
         <f aca="false">O9</f>
@@ -8371,12 +8474,12 @@
         <v>0</v>
       </c>
       <c r="H47" s="13" t="s">
-        <v>496</v>
+        <v>502</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="28" t="s">
-        <v>497</v>
+        <v>503</v>
       </c>
       <c r="D49" s="8" t="str">
         <f aca="false">INDEX(A43:A46,MATCH(MAX(E43:E46),E43:E46,0))</f>
@@ -8408,7 +8511,7 @@
     </row>
     <row r="54" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="1" t="s">
-        <v>498</v>
+        <v>504</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8416,34 +8519,34 @@
         <v>316</v>
       </c>
       <c r="B57" s="12" t="s">
-        <v>499</v>
+        <v>505</v>
       </c>
       <c r="C57" s="12" t="s">
-        <v>500</v>
+        <v>506</v>
       </c>
       <c r="D57" s="12" t="s">
-        <v>501</v>
+        <v>507</v>
       </c>
       <c r="E57" s="12" t="s">
-        <v>502</v>
+        <v>508</v>
       </c>
       <c r="F57" s="12" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="G57" s="12" t="s">
-        <v>504</v>
+        <v>510</v>
       </c>
       <c r="H57" s="12" t="s">
-        <v>505</v>
+        <v>511</v>
       </c>
       <c r="I57" s="12" t="s">
-        <v>506</v>
+        <v>512</v>
       </c>
       <c r="J57" s="12" t="s">
-        <v>507</v>
+        <v>513</v>
       </c>
       <c r="K57" s="12" t="s">
-        <v>508</v>
+        <v>514</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8628,7 +8731,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="9" t="s">
-        <v>509</v>
+        <v>515</v>
       </c>
       <c r="B63" s="9"/>
       <c r="C63" s="9"/>
@@ -8688,22 +8791,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>510</v>
+        <v>516</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>511</v>
+        <v>517</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="28" t="s">
-        <v>512</v>
+        <v>518</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
-        <v>513</v>
+        <v>519</v>
       </c>
       <c r="B4" s="12" t="s">
         <v>48</v>
@@ -8718,12 +8821,12 @@
         <v>54</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>447</v>
+        <v>453</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>514</v>
+        <v>520</v>
       </c>
       <c r="B5" s="29" t="n">
         <f aca="false">Assumptions!$D$151</f>
@@ -8748,7 +8851,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>515</v>
+        <v>521</v>
       </c>
       <c r="B6" s="30" t="n">
         <f aca="false">Assumptions!$D$155</f>
@@ -8769,7 +8872,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>516</v>
+        <v>522</v>
       </c>
       <c r="B7" s="32" t="n">
         <f aca="false">B5*B6</f>
@@ -8794,7 +8897,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>517</v>
+        <v>523</v>
       </c>
       <c r="B8" s="30" t="n">
         <f aca="false">Assumptions!$D$156</f>
@@ -8815,7 +8918,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>518</v>
+        <v>524</v>
       </c>
       <c r="B9" s="31" t="n">
         <f aca="false">Funnel!$G$5*Assumptions!$D$164</f>
@@ -8836,7 +8939,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>519</v>
+        <v>525</v>
       </c>
       <c r="B10" s="41" t="n">
         <f aca="false">B5*Assumptions!$D$162</f>
@@ -8861,7 +8964,7 @@
     </row>
     <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>520</v>
+        <v>526</v>
       </c>
       <c r="B11" s="43" t="n">
         <f aca="false">IF(B7&gt;0,B10/B7,0)</f>
@@ -8886,7 +8989,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>521</v>
+        <v>527</v>
       </c>
       <c r="B12" s="32" t="n">
         <f aca="false">B7*B8*B9</f>
@@ -8911,7 +9014,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>522</v>
+        <v>528</v>
       </c>
       <c r="B13" s="32" t="n">
         <f aca="false">Assumptions!$D$157</f>
@@ -8936,7 +9039,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>523</v>
+        <v>529</v>
       </c>
       <c r="B14" s="30" t="n">
         <f aca="false">Assumptions!$D$161</f>
@@ -8957,7 +9060,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>524</v>
+        <v>530</v>
       </c>
       <c r="B15" s="32" t="n">
         <f aca="false">B13*B14*B9</f>
@@ -8982,7 +9085,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>525</v>
+        <v>531</v>
       </c>
       <c r="B16" s="41" t="n">
         <f aca="false">B15*Assumptions!$D$163</f>
@@ -9007,7 +9110,7 @@
     </row>
     <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="B17" s="43" t="n">
         <f aca="false">IF(B13&gt;0,B16/B13,0)</f>
@@ -9026,12 +9129,12 @@
         <v>123.165</v>
       </c>
       <c r="G17" s="13" t="s">
-        <v>527</v>
+        <v>533</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="B18" s="32" t="n">
         <f aca="false">B12+B15</f>
@@ -9056,7 +9159,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>529</v>
+        <v>535</v>
       </c>
       <c r="B19" s="41" t="n">
         <f aca="false">B10+B16</f>
@@ -9081,7 +9184,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>530</v>
+        <v>536</v>
       </c>
       <c r="B20" s="41" t="n">
         <f aca="false">IF(B18&gt;0,B19/B18,0)</f>
@@ -9106,12 +9209,12 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="28" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>532</v>
+        <v>538</v>
       </c>
       <c r="B24" s="29" t="n">
         <f aca="false">Assumptions!$D$165</f>
@@ -9120,7 +9223,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>533</v>
+        <v>539</v>
       </c>
       <c r="B25" s="31" t="n">
         <f aca="false">Assumptions!$D$166</f>
@@ -9129,7 +9232,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>534</v>
+        <v>540</v>
       </c>
       <c r="B26" s="29" t="n">
         <f aca="false">B24*B25</f>
@@ -9138,7 +9241,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>535</v>
+        <v>541</v>
       </c>
       <c r="B27" s="41" t="n">
         <f aca="false">Assumptions!$D$167</f>
@@ -9147,7 +9250,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>536</v>
+        <v>542</v>
       </c>
       <c r="B28" s="30" t="n">
         <f aca="false">Assumptions!$D$168</f>
@@ -9156,7 +9259,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>537</v>
+        <v>543</v>
       </c>
       <c r="B29" s="32" t="n">
         <f aca="false">B26*B28</f>
@@ -9165,7 +9268,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>538</v>
+        <v>544</v>
       </c>
       <c r="B30" s="31" t="n">
         <f aca="false">Funnel!$G$5*Assumptions!$D$169</f>
@@ -9174,7 +9277,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="B31" s="32" t="n">
         <f aca="false">B29*B30</f>
@@ -9183,7 +9286,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>540</v>
+        <v>546</v>
       </c>
       <c r="B32" s="41" t="n">
         <f aca="false">B26*B27</f>
@@ -9192,7 +9295,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>541</v>
+        <v>547</v>
       </c>
       <c r="B33" s="41" t="n">
         <f aca="false">Assumptions!$D$170</f>
@@ -9201,7 +9304,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>542</v>
+        <v>548</v>
       </c>
       <c r="B34" s="41" t="n">
         <f aca="false">IF(B31&gt;0,(B32+B33)/B31,0)</f>
@@ -9210,12 +9313,12 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="28" t="s">
-        <v>543</v>
+        <v>549</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
-        <v>544</v>
+        <v>550</v>
       </c>
       <c r="B38" s="43" t="n">
         <f aca="false">B44+B45</f>
@@ -9224,7 +9327,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
-        <v>545</v>
+        <v>551</v>
       </c>
       <c r="B39" s="30" t="n">
         <f aca="false">Assumptions!$D$172</f>
@@ -9233,7 +9336,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
-        <v>534</v>
+        <v>540</v>
       </c>
       <c r="B40" s="29" t="n">
         <f aca="false">Assumptions!$D$173</f>
@@ -9242,7 +9345,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
-        <v>546</v>
+        <v>552</v>
       </c>
       <c r="B41" s="31" t="n">
         <f aca="false">Funnel!$G$6*Assumptions!$D$174</f>
@@ -9251,7 +9354,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="2" t="s">
-        <v>547</v>
+        <v>553</v>
       </c>
       <c r="B42" s="32" t="n">
         <f aca="false">Assumptions!$D$10*Assumptions!$D$12</f>
@@ -9260,7 +9363,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="B43" s="32" t="n">
         <f aca="false">MIN(B40*B39*B41,B42)</f>
@@ -9269,7 +9372,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="2" t="s">
-        <v>549</v>
+        <v>555</v>
       </c>
       <c r="B44" s="43" t="n">
         <f aca="false">Assumptions!$D$171</f>
@@ -9278,7 +9381,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="2" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="B45" s="43" t="n">
         <f aca="false">Assumptions!$D$175/60*Assumptions!$D$176</f>
@@ -9287,7 +9390,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="2" t="s">
-        <v>551</v>
+        <v>557</v>
       </c>
       <c r="B46" s="41" t="n">
         <f aca="false">Assumptions!$D$177</f>
@@ -9296,7 +9399,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="2" t="s">
-        <v>552</v>
+        <v>558</v>
       </c>
       <c r="B47" s="29" t="n">
         <f aca="false">IF(B41*B39&gt;0,B43/B41/B39,0)</f>
@@ -9305,7 +9408,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="2" t="s">
-        <v>553</v>
+        <v>559</v>
       </c>
       <c r="B48" s="41" t="n">
         <f aca="false">IF(B43&gt;0,(B47*B38+B46)/B43,0)</f>
@@ -9314,8 +9417,8 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="9" t="str">
-        <f aca="false">"Polish supply check: the border regions have ~"&amp;TEXT(Assumptions!$D$124*Assumptions!$D$121,"#,##0")&amp;" maintenance-type workers ("&amp;TEXT(Assumptions!$D$124,"#,##0")&amp;" industry workers × "&amp;TEXT(Assumptions!$D$121,"0.0%")&amp;", Eurostat 2025). The plan needs "&amp;TEXT(B47,"0")&amp;" applications = "&amp;TEXT(B47/(Assumptions!$D$124*Assumptions!$D$121),"0.0%")&amp;" of them, vs the "&amp;TEXT(Assumptions!$D$166,"0.0%")&amp;" response assumed for construction electricians (I2). So the corridor needs a stronger response (German pay is the pull); at I2’s rate it brings ~"&amp;TEXT(Assumptions!$D$124*Assumptions!$D$121*Assumptions!$D$166,"0")&amp;" applications. The 9 Nov test decides; if it fails, the budget rises (slide 7)."</f>
-        <v>Polish supply check: the border regions have ~18,525 maintenance-type workers (237,500 industry workers × 7.8%, Eurostat 2025). The plan needs 346 applications = 1.9% of them, vs the 1.2% response assumed for construction electricians (I2). So the corridor needs a stronger response (German pay is the pull); at I2’s rate it brings ~219 applications. The 9 Nov test decides; if it fails, the budget rises (slide 7).</v>
+        <f aca="false">"Polish supply check: the border regions have ~"&amp;TEXT(Assumptions!$D$124*Assumptions!$D$121,"#,##0")&amp;" maintenance-type workers (Eurostat 2025: "&amp;TEXT(Assumptions!$D$124,"#,##0")&amp;" industry workers × the German BA maintenance share "&amp;TEXT(Assumptions!$D$121,"0.0%")&amp;", applied to Poland as my estimate; an upper bound, since whole regions and all industry staff are counted). The plan needs "&amp;TEXT(B47,"0")&amp;" applications = "&amp;TEXT(B47/(Assumptions!$D$124*Assumptions!$D$121),"0.0%")&amp;" of them, vs the "&amp;TEXT(Assumptions!$D$166,"0.0%")&amp;" response assumed for construction electricians (I2). So the corridor needs a stronger response (German pay is the pull); at I2’s rate it brings ~"&amp;TEXT(Assumptions!$D$124*Assumptions!$D$121*Assumptions!$D$166,"0")&amp;" applications. The 9 Nov test decides; if it fails, the budget rises (slide 7)."</f>
+        <v>Polish supply check: the border regions have ~18,525 maintenance-type workers (Eurostat 2025: 237,500 industry workers × the German BA maintenance share 7.8%, applied to Poland as my estimate; an upper bound, since whole regions and all industry staff are counted). The plan needs 346 applications = 1.9% of them, vs the 1.2% response assumed for construction electricians (I2). So the corridor needs a stronger response (German pay is the pull); at I2’s rate it brings ~219 applications. The 9 Nov test decides; if it fails, the budget rises (slide 7).</v>
       </c>
       <c r="B49" s="9"/>
       <c r="C49" s="9"/>
@@ -9337,50 +9440,50 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="28" t="s">
-        <v>554</v>
+        <v>560</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="12" t="s">
-        <v>555</v>
+        <v>561</v>
       </c>
       <c r="B52" s="12" t="s">
-        <v>556</v>
+        <v>562</v>
       </c>
       <c r="C52" s="12" t="s">
-        <v>557</v>
+        <v>563</v>
       </c>
       <c r="D52" s="12" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="E52" s="12" t="s">
-        <v>559</v>
+        <v>565</v>
       </c>
       <c r="F52" s="12" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="G52" s="12" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="H52" s="12" t="s">
-        <v>562</v>
+        <v>568</v>
       </c>
       <c r="I52" s="12" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="J52" s="12" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
       <c r="K52" s="12" t="s">
-        <v>565</v>
+        <v>571</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="28" t="s">
-        <v>566</v>
+        <v>572</v>
       </c>
       <c r="B53" s="13" t="s">
-        <v>567</v>
+        <v>573</v>
       </c>
       <c r="C53" s="30" t="n">
         <f aca="false">(Assumptions!$D$93+Assumptions!$D$94)</f>
@@ -9392,47 +9495,47 @@
       </c>
       <c r="E53" s="32" t="n">
         <f aca="false">(SUMIFS(Channels!$V:$V,Channels!$A:$A,"I1a-E")+SUMIFS(Channels!$V:$V,Channels!$A:$A,"I1a-M")+SUMIFS(Channels!$V:$V,Channels!$A:$A,"I1a-A")+SUMIFS(Channels!$V:$V,Channels!$A:$A,"I1a-S"))*(Assumptions!$D$93+Assumptions!$D$94)+(SUMIFS(Channels!$V:$V,Channels!$A:$A,"I1b-E")+SUMIFS(Channels!$V:$V,Channels!$A:$A,"I1b-M")+SUMIFS(Channels!$V:$V,Channels!$A:$A,"I1b-A")+SUMIFS(Channels!$V:$V,Channels!$A:$A,"I1b-S"))*(Weekly!$D$4+Weekly!$D$5)</f>
-        <v>22.9989</v>
+        <v>24.5433</v>
       </c>
       <c r="F53" s="2" t="s">
-        <v>568</v>
+        <v>574</v>
       </c>
       <c r="G53" s="29" t="n">
         <f aca="false">MAX(1,ROUNDDOWN(E53*Assumptions!$D$89,0))</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H53" s="2" t="s">
-        <v>569</v>
+        <v>575</v>
       </c>
       <c r="I53" s="29" t="n">
         <f aca="false">MIN(G53,MAX(1,ROUNDUP(E53*Assumptions!$D$91,0)))</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J53" s="2" t="s">
-        <v>569</v>
+        <v>575</v>
       </c>
       <c r="K53" s="13" t="s">
-        <v>570</v>
+        <v>576</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="28" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="B54" s="13" t="s">
-        <v>572</v>
+        <v>578</v>
       </c>
       <c r="C54" s="30" t="n">
-        <f aca="false">(Weekly!$D$4*4/7+Weekly!$D$5+Weekly!$D$6*3/7)</f>
-        <v>0.365</v>
+        <f aca="false">(Weekly!$AB$4+Weekly!$AB$5+Weekly!$AB$6*3/7)</f>
+        <v>0.440185062789161</v>
       </c>
       <c r="D54" s="41" t="n">
         <f aca="false">B33+SUMIFS(Channels!$X:$X,Channels!$A:$A,"I2-E")*C54</f>
-        <v>4817.88</v>
+        <v>5563.11434236616</v>
       </c>
       <c r="E54" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$V:$V,Channels!$A:$A,"I2-E")*C54</f>
-        <v>10.7675</v>
+        <v>12.9854593522802</v>
       </c>
       <c r="F54" s="41" t="n">
         <f aca="false">IF(B28&gt;0,B27/B28,0)</f>
@@ -9440,7 +9543,7 @@
       </c>
       <c r="G54" s="29" t="n">
         <f aca="false">MAX(1,ROUNDDOWN(E54*Assumptions!$D$89,0))</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H54" s="41" t="n">
         <f aca="false">ROUND(F54*Assumptions!$D$90/10,0)*10</f>
@@ -9455,27 +9558,27 @@
         <v>670</v>
       </c>
       <c r="K54" s="13" t="s">
-        <v>573</v>
+        <v>579</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="28" t="s">
-        <v>574</v>
+        <v>580</v>
       </c>
       <c r="B55" s="13" t="s">
-        <v>575</v>
+        <v>581</v>
       </c>
       <c r="C55" s="30" t="n">
-        <f aca="false">(Weekly!$D$5+Weekly!$D$6)</f>
-        <v>0.325</v>
+        <f aca="false">(Weekly!$AC$5+Weekly!$AC$6)</f>
+        <v>0.426900584795322</v>
       </c>
       <c r="D55" s="41" t="n">
         <f aca="false">B46+SUMIFS(Channels!$X:$X,Channels!$A:$A,"I3-M")*C55</f>
-        <v>2510.38961038961</v>
+        <v>3172.08171945014</v>
       </c>
       <c r="E55" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$V:$V,Channels!$A:$A,"I3-M")*C55</f>
-        <v>15.7575757575758</v>
+        <v>20.6982101718944</v>
       </c>
       <c r="F55" s="41" t="n">
         <f aca="false">IF(B39&gt;0,B38/B39,0)</f>
@@ -9483,7 +9586,7 @@
       </c>
       <c r="G55" s="29" t="n">
         <f aca="false">MAX(1,ROUNDDOWN(E55*Assumptions!$D$89,0))</f>
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="H55" s="41" t="n">
         <f aca="false">ROUND(F55*Assumptions!$D$90/10,0)*10</f>
@@ -9491,19 +9594,19 @@
       </c>
       <c r="I55" s="29" t="n">
         <f aca="false">MIN(G55,MAX(1,ROUNDUP(E55*Assumptions!$D$91,0)))</f>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J55" s="41" t="n">
         <f aca="false">MAX(H55,ROUND(F55*Assumptions!$D$92/10,0)*10)</f>
         <v>270</v>
       </c>
       <c r="K55" s="13" t="s">
-        <v>576</v>
+        <v>582</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="13" t="s">
-        <v>577</v>
+        <v>583</v>
       </c>
     </row>
   </sheetData>
@@ -9544,17 +9647,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>578</v>
+        <v>584</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="369.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="13" t="s">
-        <v>579</v>
+        <v>585</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="318.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="13" t="s">
-        <v>580</v>
+        <v>586</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9568,100 +9671,100 @@
         <v>316</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>581</v>
+        <v>587</v>
       </c>
       <c r="E4" s="12" t="s">
         <v>317</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>582</v>
+        <v>588</v>
       </c>
       <c r="G4" s="12" t="s">
-        <v>583</v>
+        <v>589</v>
       </c>
       <c r="H4" s="12" t="s">
-        <v>535</v>
+        <v>541</v>
       </c>
       <c r="I4" s="12" t="s">
         <v>320</v>
       </c>
       <c r="J4" s="12" t="s">
-        <v>534</v>
+        <v>540</v>
       </c>
       <c r="K4" s="12" t="s">
-        <v>584</v>
+        <v>590</v>
       </c>
       <c r="L4" s="12" t="s">
-        <v>437</v>
+        <v>443</v>
       </c>
       <c r="M4" s="12" t="s">
-        <v>585</v>
+        <v>591</v>
       </c>
       <c r="N4" s="12" t="s">
-        <v>586</v>
+        <v>592</v>
       </c>
       <c r="O4" s="12" t="s">
-        <v>587</v>
+        <v>593</v>
       </c>
       <c r="P4" s="12" t="s">
-        <v>588</v>
+        <v>594</v>
       </c>
       <c r="Q4" s="12" t="s">
-        <v>589</v>
+        <v>595</v>
       </c>
       <c r="R4" s="12" t="s">
-        <v>590</v>
+        <v>596</v>
       </c>
       <c r="S4" s="12" t="s">
-        <v>591</v>
+        <v>597</v>
       </c>
       <c r="T4" s="12" t="s">
-        <v>592</v>
+        <v>598</v>
       </c>
       <c r="U4" s="12" t="s">
-        <v>593</v>
+        <v>599</v>
       </c>
       <c r="V4" s="12" t="s">
-        <v>594</v>
+        <v>600</v>
       </c>
       <c r="W4" s="12" t="s">
-        <v>595</v>
+        <v>601</v>
       </c>
       <c r="X4" s="12" t="s">
-        <v>596</v>
+        <v>602</v>
       </c>
       <c r="Y4" s="12" t="s">
-        <v>597</v>
+        <v>603</v>
       </c>
       <c r="Z4" s="12" t="s">
-        <v>598</v>
+        <v>604</v>
       </c>
       <c r="AA4" s="12" t="s">
-        <v>599</v>
+        <v>605</v>
       </c>
       <c r="AB4" s="12" t="s">
-        <v>600</v>
+        <v>606</v>
       </c>
       <c r="AC4" s="12" t="s">
-        <v>601</v>
+        <v>607</v>
       </c>
       <c r="AD4" s="12" t="s">
-        <v>602</v>
+        <v>608</v>
       </c>
       <c r="AE4" s="12" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="AF4" s="12" t="s">
-        <v>604</v>
+        <v>610</v>
       </c>
       <c r="AG4" s="12" t="s">
-        <v>605</v>
+        <v>611</v>
       </c>
       <c r="AH4" s="12" t="s">
-        <v>606</v>
+        <v>612</v>
       </c>
       <c r="AI4" s="12" t="s">
-        <v>607</v>
+        <v>613</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12486,16 +12589,16 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>608</v>
+        <v>614</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>609</v>
+        <v>615</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>48</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>555</v>
+        <v>561</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>333</v>
@@ -12620,16 +12723,16 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>610</v>
+        <v>616</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>609</v>
+        <v>615</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>43</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>555</v>
+        <v>561</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>333</v>
@@ -12754,16 +12857,16 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>611</v>
+        <v>617</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>609</v>
+        <v>615</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>52</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>555</v>
+        <v>561</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>333</v>
@@ -12888,16 +12991,16 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>612</v>
+        <v>618</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>609</v>
+        <v>615</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>54</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>555</v>
+        <v>561</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>333</v>
@@ -13022,16 +13125,16 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>613</v>
+        <v>619</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>614</v>
+        <v>620</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>48</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>555</v>
+        <v>561</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>333</v>
@@ -13156,16 +13259,16 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>615</v>
+        <v>621</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>614</v>
+        <v>620</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>43</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>555</v>
+        <v>561</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>333</v>
@@ -13290,16 +13393,16 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>616</v>
+        <v>622</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>614</v>
+        <v>620</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>52</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>555</v>
+        <v>561</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>333</v>
@@ -13424,16 +13527,16 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>617</v>
+        <v>623</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>614</v>
+        <v>620</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>54</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>555</v>
+        <v>561</v>
       </c>
       <c r="E32" s="2" t="s">
         <v>333</v>
@@ -13558,16 +13661,16 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>618</v>
+        <v>624</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>619</v>
+        <v>625</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>48</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>555</v>
+        <v>561</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>333</v>
@@ -13692,16 +13795,16 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>620</v>
+        <v>626</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>621</v>
+        <v>627</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>43</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>555</v>
+        <v>561</v>
       </c>
       <c r="E34" s="2" t="s">
         <v>333</v>
@@ -13826,7 +13929,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="28" t="s">
-        <v>447</v>
+        <v>453</v>
       </c>
       <c r="J35" s="33" t="n">
         <f aca="false">SUM(J5:J34)</f>
@@ -13891,7 +13994,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="28" t="s">
-        <v>622</v>
+        <v>628</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13903,10 +14006,10 @@
         <v>47</v>
       </c>
       <c r="D38" s="12" t="s">
-        <v>623</v>
+        <v>629</v>
       </c>
       <c r="E38" s="12" t="s">
-        <v>624</v>
+        <v>630</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14005,7 +14108,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>625</v>
+        <v>631</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14016,7 +14119,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="2" t="s">
-        <v>626</v>
+        <v>632</v>
       </c>
       <c r="C4" s="41" t="n">
         <f aca="false">SUMIFS(Channels!X5:X34,Channels!D5:D34,"Channel")</f>
@@ -14025,7 +14128,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="2" t="s">
-        <v>627</v>
+        <v>633</v>
       </c>
       <c r="C5" s="41" t="n">
         <f aca="false">SUMIFS(Channels!X5:X34,Channels!D5:D34,"Initiative")</f>
@@ -14034,7 +14137,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="2" t="s">
-        <v>628</v>
+        <v>634</v>
       </c>
       <c r="C6" s="41" t="n">
         <f aca="false">Channels!Y35</f>
@@ -14043,7 +14146,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="2" t="s">
-        <v>629</v>
+        <v>635</v>
       </c>
       <c r="C7" s="41" t="n">
         <f aca="false">C4+C5+C6</f>
@@ -14052,7 +14155,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="2" t="s">
-        <v>630</v>
+        <v>636</v>
       </c>
       <c r="C8" s="41" t="n">
         <f aca="false">Channels!Z35</f>
@@ -14061,7 +14164,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="2" t="s">
-        <v>631</v>
+        <v>637</v>
       </c>
       <c r="C9" s="41" t="n">
         <f aca="false">C7</f>
@@ -14070,7 +14173,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="2" t="s">
-        <v>632</v>
+        <v>638</v>
       </c>
       <c r="C10" s="41" t="n">
         <f aca="false">IF(Assumptions!$D$48&lt;1,C9/(1-Assumptions!$D$48)*Assumptions!$D$48,0)</f>
@@ -14079,7 +14182,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="2" t="s">
-        <v>633</v>
+        <v>639</v>
       </c>
       <c r="C11" s="41" t="n">
         <f aca="false">C9+C10</f>
@@ -14088,7 +14191,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="28" t="s">
-        <v>634</v>
+        <v>640</v>
       </c>
       <c r="C12" s="4" t="n">
         <f aca="false">IF(Assumptions!$D$51&gt;0,ROUNDUP(C11/Assumptions!$D$51,0)*Assumptions!$D$51,C11)</f>
@@ -14097,7 +14200,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="2" t="s">
-        <v>635</v>
+        <v>641</v>
       </c>
       <c r="C13" s="46" t="n">
         <f aca="false">MIN(Channels!U35,Funnel!B26)</f>
@@ -14106,7 +14209,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="2" t="s">
-        <v>636</v>
+        <v>642</v>
       </c>
       <c r="C14" s="47" t="n">
         <f aca="false">IF(C13&gt;0,C9/C13,0)</f>
@@ -14115,7 +14218,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="2" t="s">
-        <v>637</v>
+        <v>643</v>
       </c>
       <c r="C15" s="41" t="n">
         <f aca="false">IF(C13&gt;0,C12/C13,0)</f>
@@ -14124,16 +14227,16 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="2" t="s">
-        <v>638</v>
+        <v>644</v>
       </c>
       <c r="C16" s="30" t="n">
         <f aca="false">IF(C12&gt;0,Weekly!N5/C12,0)</f>
-        <v>0.385951267678667</v>
+        <v>0.397471746280603</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="28" t="s">
-        <v>639</v>
+        <v>645</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14142,25 +14245,25 @@
         <v>316</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>640</v>
+        <v>646</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>597</v>
+        <v>603</v>
       </c>
       <c r="E20" s="12" t="s">
-        <v>641</v>
+        <v>647</v>
       </c>
       <c r="F20" s="12" t="s">
-        <v>599</v>
+        <v>605</v>
       </c>
       <c r="G20" s="12" t="s">
-        <v>642</v>
+        <v>648</v>
       </c>
       <c r="H20" s="12" t="s">
-        <v>643</v>
+        <v>649</v>
       </c>
       <c r="I20" s="12" t="s">
-        <v>644</v>
+        <v>650</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14297,7 +14400,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="28" t="s">
-        <v>447</v>
+        <v>453</v>
       </c>
       <c r="C25" s="42" t="n">
         <f aca="false">SUM(C21:C24)</f>
@@ -14330,7 +14433,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="28" t="s">
-        <v>645</v>
+        <v>651</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14339,16 +14442,16 @@
         <v>315</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>599</v>
+        <v>605</v>
       </c>
       <c r="D28" s="12" t="s">
-        <v>642</v>
+        <v>648</v>
       </c>
       <c r="E28" s="12" t="s">
-        <v>643</v>
+        <v>649</v>
       </c>
       <c r="F28" s="12" t="s">
-        <v>646</v>
+        <v>652</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14479,7 +14582,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="2" t="s">
-        <v>609</v>
+        <v>615</v>
       </c>
       <c r="C35" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$AA$5:$AA$34,Channels!$B$5:$B$34,B35)</f>
@@ -14500,7 +14603,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="2" t="s">
-        <v>614</v>
+        <v>620</v>
       </c>
       <c r="C36" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$AA$5:$AA$34,Channels!$B$5:$B$34,B36)</f>
@@ -14521,7 +14624,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="2" t="s">
-        <v>619</v>
+        <v>625</v>
       </c>
       <c r="C37" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$AA$5:$AA$34,Channels!$B$5:$B$34,B37)</f>
@@ -14542,7 +14645,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="2" t="s">
-        <v>621</v>
+        <v>627</v>
       </c>
       <c r="C38" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$AA$5:$AA$34,Channels!$B$5:$B$34,B38)</f>
@@ -14563,7 +14666,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="28" t="s">
-        <v>447</v>
+        <v>453</v>
       </c>
       <c r="C39" s="42" t="n">
         <f aca="false">SUM(C29:C38)</f>
@@ -14582,7 +14685,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="28" t="s">
-        <v>647</v>
+        <v>653</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14594,10 +14697,10 @@
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="12"/>
       <c r="B44" s="12" t="s">
-        <v>648</v>
+        <v>654</v>
       </c>
       <c r="C44" s="12" t="s">
-        <v>649</v>
+        <v>655</v>
       </c>
       <c r="D44" s="12" t="s">
         <v>48</v>
@@ -14612,10 +14715,10 @@
         <v>54</v>
       </c>
       <c r="H44" s="12" t="s">
-        <v>650</v>
+        <v>656</v>
       </c>
       <c r="I44" s="12" t="s">
-        <v>643</v>
+        <v>649</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14688,17 +14791,17 @@
     </row>
     <row r="49" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="1" t="s">
-        <v>651</v>
+        <v>657</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="2" t="s">
-        <v>652</v>
+        <v>658</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E51" s="28" t="s">
-        <v>653</v>
+        <v>659</v>
       </c>
       <c r="F51" s="48" t="n">
         <f aca="false">1</f>
@@ -14711,7 +14814,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E52" s="2" t="s">
-        <v>649</v>
+        <v>655</v>
       </c>
       <c r="F52" s="41" t="n">
         <f aca="false">Budget!$C$12*F51</f>
@@ -14724,7 +14827,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E53" s="2" t="s">
-        <v>654</v>
+        <v>660</v>
       </c>
       <c r="F53" s="41" t="n">
         <f aca="false">F52*(1-Assumptions!$D$48)</f>
@@ -14737,7 +14840,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E54" s="2" t="s">
-        <v>655</v>
+        <v>661</v>
       </c>
       <c r="F54" s="41" t="n">
         <f aca="false">MAX(0,Budget!$C$9-F53)</f>
@@ -14750,44 +14853,44 @@
     </row>
     <row r="55" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="12" t="s">
-        <v>656</v>
+        <v>662</v>
       </c>
       <c r="B55" s="12" t="s">
         <v>316</v>
       </c>
       <c r="C55" s="12" t="s">
-        <v>657</v>
+        <v>663</v>
       </c>
       <c r="D55" s="12" t="s">
-        <v>658</v>
+        <v>664</v>
       </c>
       <c r="E55" s="12" t="s">
-        <v>642</v>
+        <v>648</v>
       </c>
       <c r="F55" s="12" t="s">
-        <v>659</v>
+        <v>665</v>
       </c>
       <c r="G55" s="12" t="s">
-        <v>660</v>
+        <v>666</v>
       </c>
       <c r="H55" s="12"/>
       <c r="I55" s="12"/>
       <c r="J55" s="12" t="s">
-        <v>661</v>
+        <v>667</v>
       </c>
       <c r="K55" s="12" t="s">
-        <v>662</v>
+        <v>668</v>
       </c>
       <c r="L55" s="12"/>
       <c r="M55" s="12"/>
       <c r="N55" s="12" t="s">
-        <v>640</v>
+        <v>646</v>
       </c>
       <c r="O55" s="12" t="s">
-        <v>663</v>
+        <v>669</v>
       </c>
       <c r="P55" s="12" t="s">
-        <v>664</v>
+        <v>670</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
@@ -16292,7 +16395,7 @@
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E86" s="28" t="s">
-        <v>665</v>
+        <v>671</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16349,7 +16452,7 @@
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E91" s="28" t="s">
-        <v>447</v>
+        <v>453</v>
       </c>
       <c r="F91" s="35" t="n">
         <f aca="false">SUM(F87:F90)</f>
@@ -16362,7 +16465,7 @@
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E92" s="2" t="s">
-        <v>643</v>
+        <v>649</v>
       </c>
       <c r="F92" s="41" t="n">
         <f aca="false">IF(F91&gt;0,F52/F91,0)</f>
@@ -16375,7 +16478,7 @@
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E94" s="2" t="s">
-        <v>666</v>
+        <v>672</v>
       </c>
       <c r="F94" s="32" t="n">
         <f aca="false">SUM(O56:O85)</f>
@@ -16388,7 +16491,7 @@
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E95" s="2" t="s">
-        <v>667</v>
+        <v>673</v>
       </c>
       <c r="F95" s="30" t="n">
         <f aca="false">IF(F94&gt;0,MIN(1,Funnel!$B$22/F94),1)</f>
@@ -16401,7 +16504,7 @@
     </row>
     <row r="97" customFormat="false" ht="407.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="13" t="s">
-        <v>668</v>
+        <v>674</v>
       </c>
     </row>
   </sheetData>
@@ -16421,7 +16524,7 @@
     <tabColor rgb="FF8EA9DB"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AA55"/>
+  <dimension ref="A1:AE55"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="1"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
@@ -16434,95 +16537,107 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>669</v>
+        <v>675</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="344" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="13" t="s">
-        <v>670</v>
+        <v>676</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
-        <v>671</v>
+        <v>677</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>672</v>
+        <v>678</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>673</v>
+        <v>679</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>674</v>
+        <v>680</v>
       </c>
       <c r="E3" s="12" t="s">
-        <v>675</v>
+        <v>681</v>
       </c>
       <c r="F3" s="12" t="s">
-        <v>676</v>
+        <v>682</v>
       </c>
       <c r="G3" s="12" t="s">
-        <v>677</v>
+        <v>683</v>
       </c>
       <c r="H3" s="12" t="s">
-        <v>678</v>
+        <v>684</v>
       </c>
       <c r="I3" s="12" t="s">
-        <v>679</v>
+        <v>685</v>
       </c>
       <c r="J3" s="12" t="s">
-        <v>680</v>
+        <v>686</v>
       </c>
       <c r="K3" s="12" t="s">
-        <v>681</v>
+        <v>687</v>
       </c>
       <c r="L3" s="12" t="s">
-        <v>682</v>
+        <v>688</v>
       </c>
       <c r="M3" s="12" t="s">
-        <v>683</v>
+        <v>689</v>
       </c>
       <c r="N3" s="12" t="s">
-        <v>684</v>
+        <v>690</v>
       </c>
       <c r="O3" s="12" t="s">
-        <v>685</v>
+        <v>691</v>
       </c>
       <c r="P3" s="12" t="s">
-        <v>686</v>
+        <v>692</v>
       </c>
       <c r="Q3" s="12" t="s">
-        <v>687</v>
+        <v>693</v>
       </c>
       <c r="R3" s="12" t="s">
-        <v>688</v>
+        <v>694</v>
       </c>
       <c r="S3" s="12" t="s">
-        <v>689</v>
+        <v>695</v>
       </c>
       <c r="T3" s="12" t="s">
-        <v>690</v>
+        <v>696</v>
       </c>
       <c r="U3" s="12" t="s">
-        <v>691</v>
+        <v>697</v>
       </c>
       <c r="V3" s="12" t="s">
-        <v>692</v>
+        <v>698</v>
       </c>
       <c r="W3" s="12" t="s">
-        <v>693</v>
+        <v>699</v>
       </c>
       <c r="X3" s="12" t="s">
-        <v>694</v>
+        <v>700</v>
       </c>
       <c r="Y3" s="12" t="s">
-        <v>695</v>
+        <v>701</v>
       </c>
       <c r="Z3" s="49" t="s">
-        <v>696</v>
+        <v>702</v>
       </c>
       <c r="AA3" s="49" t="s">
-        <v>697</v>
+        <v>703</v>
+      </c>
+      <c r="AB3" s="49" t="s">
+        <v>704</v>
+      </c>
+      <c r="AC3" s="49" t="s">
+        <v>705</v>
+      </c>
+      <c r="AD3" s="49" t="s">
+        <v>706</v>
+      </c>
+      <c r="AE3" s="49" t="s">
+        <v>707</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16539,11 +16654,11 @@
       </c>
       <c r="D4" s="30" t="n">
         <f aca="false">IF(SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$19)*$Z$4:$Z$14)&gt;0,IF(B4&lt;=Funnel!$B$19,Z4,0)/SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$19)*$Z$4:$Z$14),0)</f>
-        <v>0.25</v>
+        <v>0.316</v>
       </c>
       <c r="E4" s="30" t="n">
         <f aca="false">IF(SUM($AA$4:$AA$14)&gt;0,AA4/SUM($AA$4:$AA$14),0)</f>
-        <v>0.31616982836495</v>
+        <v>0.392129055132069</v>
       </c>
       <c r="F4" s="30" t="n">
         <f aca="false">IF(A4-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($D$4:$D$14,A4-ROUNDUP(Funnel!$B$15/7,0)),0)</f>
@@ -16554,8 +16669,8 @@
         <v>0</v>
       </c>
       <c r="H4" s="41" t="n">
-        <f aca="false">$F$19*D4+$F$20*E4+$F$31*Y4</f>
-        <v>19548.5453738207</v>
+        <f aca="false">($F$19-$L$19-$L$23)*D4+$L$19*AB4+$L$23*AC4+$F$20*E4+$F$31*Y4</f>
+        <v>21493.923944841</v>
       </c>
       <c r="I4" s="41" t="n">
         <f aca="false">IF(A4=1,$F$21,0)</f>
@@ -16575,19 +16690,19 @@
       </c>
       <c r="M4" s="41" t="n">
         <f aca="false">SUM(H4:L4)</f>
-        <v>30544.5453738207</v>
+        <v>32489.923944841</v>
       </c>
       <c r="N4" s="41" t="n">
         <f aca="false">SUM($M$4:M4)</f>
-        <v>30544.5453738207</v>
+        <v>32489.923944841</v>
       </c>
       <c r="O4" s="29" t="n">
-        <f aca="false">(Funnel!$M$5+Funnel!$M$6+Funnel!$M$7-$F$27-$F$34)*D4+(Funnel!$M$8-$F$28-$F$35)*E4+($F$27+$F$28)*X4+($F$34+$F$35)*Y4</f>
-        <v>404.142980954988</v>
+        <f aca="false">(Funnel!$M$5+Funnel!$M$6+Funnel!$M$7-$F$27-$F$34-$L$20-$L$24)*D4+$L$20*AB4+$L$24*AC4+(Funnel!$M$8-$F$28-$F$35)*E4+($F$27+$F$28)*X4+($F$34+$F$35)*Y4</f>
+        <v>376.189537902275</v>
       </c>
       <c r="P4" s="29" t="n">
-        <f aca="false">(Funnel!$O$5+Funnel!$O$6+Funnel!$O$7-$F$25-$F$32)*D4+(Funnel!$O$8-$F$26-$F$33)*E4+($F$25+$F$26)*X4+($F$32+$F$33)*Y4</f>
-        <v>85.6310133800371</v>
+        <f aca="false">(Funnel!$O$5+Funnel!$O$6+Funnel!$O$7-$F$25-$F$32-$L$21-$L$25)*D4+$L$21*AB4+$L$25*AC4+(Funnel!$O$8-$F$26-$F$33)*E4+($F$25+$F$26)*X4+($F$32+$F$33)*Y4</f>
+        <v>86.1932888080734</v>
       </c>
       <c r="Q4" s="29" t="n">
         <f aca="false">Assumptions!$D$9*MAX(0,MIN(C4+Assumptions!$D$21,Funnel!$B$17)-MAX(IF(A4=1,Funnel!$B$13,B4+Assumptions!$D$21),Funnel!$B$13)+1)/7</f>
@@ -16595,14 +16710,14 @@
       </c>
       <c r="R4" s="30" t="n">
         <f aca="false">IF(Q4&gt;0,P4/Q4,IF(P4&gt;0,9.99,0))</f>
-        <v>0.990772055636793</v>
+        <v>0.997277721746304</v>
       </c>
       <c r="S4" s="2" t="str">
         <f aca="false">IF(P4&gt;Q4+0.5,"OVER "&amp;Assumptions!$D$9&amp;"/wk – pace down",IF(R4&gt;Assumptions!$D$102,"Full",IF(AND(Q4&gt;=Assumptions!$D$103,P4&lt;Assumptions!$D$103),"Under "&amp;Assumptions!$D$103&amp;" – release reserve","")))</f>
         <v>Full</v>
       </c>
       <c r="T4" s="32" t="n">
-        <f aca="false">$F$38*(F4*(Budget!$G$21+Budget!$G$22+Budget!$G$23-$F$29-$F$36)+IF(A4-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($X$4:$X$14,A4-ROUNDUP(Funnel!$B$15/7,0))*$F$29+INDEX($Y$4:$Y$14,A4-ROUNDUP(Funnel!$B$15/7,0))*$F$36,0))</f>
+        <f aca="false">$F$38*(F4*(Budget!$G$21+Budget!$G$22+Budget!$G$23-$F$29-$F$36-$L$22-$L$26)+IF(A4-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($X$4:$X$14,A4-ROUNDUP(Funnel!$B$15/7,0))*$F$29+INDEX($Y$4:$Y$14,A4-ROUNDUP(Funnel!$B$15/7,0))*$F$36+INDEX($AB$4:$AB$14,A4-ROUNDUP(Funnel!$B$15/7,0))*$L$22+INDEX($AC$4:$AC$14,A4-ROUNDUP(Funnel!$B$15/7,0))*$L$26,0))</f>
         <v>0</v>
       </c>
       <c r="U4" s="32" t="n">
@@ -16627,11 +16742,27 @@
       </c>
       <c r="Z4" s="30" t="n">
         <f aca="false">Assumptions!$D$53</f>
-        <v>0.25</v>
+        <v>0.316</v>
       </c>
       <c r="AA4" s="30" t="n">
         <f aca="false">D4*IF(MAX(0,MIN(C4,Funnel!$B$19)-B4+1)&gt;0,MAX(0,MIN(C4,Funnel!$B$20)-B4+1)/MAX(0,MIN(C4,Funnel!$B$19)-B4+1),0)</f>
-        <v>0.25</v>
+        <v>0.316</v>
+      </c>
+      <c r="AB4" s="30" t="n">
+        <f aca="false">IF(SUM($AD$4:$AD$14)&gt;0,AD4/SUM($AD$4:$AD$14),0)</f>
+        <v>0.208856576338401</v>
+      </c>
+      <c r="AC4" s="30" t="n">
+        <f aca="false">IF(SUM($AE$4:$AE$14)&gt;0,AE4/SUM($AE$4:$AE$14),0)</f>
+        <v>0</v>
+      </c>
+      <c r="AD4" s="30" t="n">
+        <f aca="false">D4*IF(MAX(0,MIN(C4,Funnel!$B$19)-B4+1)&gt;0,MAX(0,MIN(C4,Funnel!$B$19)-MAX(B4,Assumptions!$D$7+Assumptions!$D$178)+1)/MAX(0,MIN(C4,Funnel!$B$19)-B4+1),0)</f>
+        <v>0.180571428571429</v>
+      </c>
+      <c r="AE4" s="30" t="n">
+        <f aca="false">D4*IF(MAX(0,MIN(C4,Funnel!$B$19)-B4+1)&gt;0,MAX(0,MIN(C4,Funnel!$B$19)-MAX(B4,Assumptions!$D$7+Assumptions!$D$179)+1)/MAX(0,MIN(C4,Funnel!$B$19)-B4+1),0)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16648,11 +16779,11 @@
       </c>
       <c r="D5" s="30" t="n">
         <f aca="false">IF(SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$19)*$Z$4:$Z$14)&gt;0,IF(B5&lt;=Funnel!$B$19,Z5,0)/SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$19)*$Z$4:$Z$14),0)</f>
-        <v>0.145</v>
+        <v>0.131</v>
       </c>
       <c r="E5" s="30" t="n">
         <f aca="false">IF(SUM($AA$4:$AA$14)&gt;0,AA5/SUM($AA$4:$AA$14),0)</f>
-        <v>0.183378500451671</v>
+        <v>0.162559829817408</v>
       </c>
       <c r="F5" s="30" t="n">
         <f aca="false">IF(A5-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($D$4:$D$14,A5-ROUNDUP(Funnel!$B$15/7,0)),0)</f>
@@ -16663,8 +16794,8 @@
         <v>0</v>
       </c>
       <c r="H5" s="41" t="n">
-        <f aca="false">$F$19*D5+$F$20*E5+$F$31*Y5</f>
-        <v>11334.484916816</v>
+        <f aca="false">($F$19-$L$19-$L$23)*D5+$L$19*AB5+$L$23*AC5+$F$20*E5+$F$31*Y5</f>
+        <v>10800.3649745329</v>
       </c>
       <c r="I5" s="41" t="n">
         <f aca="false">IF(A5=1,$F$21,0)</f>
@@ -16684,19 +16815,19 @@
       </c>
       <c r="M5" s="41" t="n">
         <f aca="false">SUM(H5:L5)</f>
-        <v>16734.484916816</v>
+        <v>16200.3649745329</v>
       </c>
       <c r="N5" s="47" t="n">
         <f aca="false">SUM($M$4:M5)</f>
-        <v>47279.0302906367</v>
+        <v>48690.2889193739</v>
       </c>
       <c r="O5" s="29" t="n">
-        <f aca="false">(Funnel!$M$5+Funnel!$M$6+Funnel!$M$7-$F$27-$F$34)*D5+(Funnel!$M$8-$F$28-$F$35)*E5+($F$27+$F$28)*X5+($F$34+$F$35)*Y5</f>
-        <v>258.280538147827</v>
+        <f aca="false">(Funnel!$M$5+Funnel!$M$6+Funnel!$M$7-$F$27-$F$34-$L$20-$L$24)*D5+$L$20*AB5+$L$24*AC5+(Funnel!$M$8-$F$28-$F$35)*E5+($F$27+$F$28)*X5+($F$34+$F$35)*Y5</f>
+        <v>260.891023555101</v>
       </c>
       <c r="P5" s="29" t="n">
-        <f aca="false">(Funnel!$O$5+Funnel!$O$6+Funnel!$O$7-$F$25-$F$32)*D5+(Funnel!$O$8-$F$26-$F$33)*E5+($F$25+$F$26)*X5+($F$32+$F$33)*Y5</f>
-        <v>53.4170222057527</v>
+        <f aca="false">(Funnel!$O$5+Funnel!$O$6+Funnel!$O$7-$F$25-$F$32-$L$21-$L$25)*D5+$L$21*AB5+$L$25*AC5+(Funnel!$O$8-$F$26-$F$33)*E5+($F$25+$F$26)*X5+($F$32+$F$33)*Y5</f>
+        <v>52.7478476582212</v>
       </c>
       <c r="Q5" s="29" t="n">
         <f aca="false">Assumptions!$D$9*MAX(0,MIN(C5+Assumptions!$D$21,Funnel!$B$17)-MAX(IF(A5=1,Funnel!$B$13,B5+Assumptions!$D$21),Funnel!$B$13)+1)/7</f>
@@ -16704,14 +16835,14 @@
       </c>
       <c r="R5" s="30" t="n">
         <f aca="false">IF(Q5&gt;0,P5/Q5,IF(P5&gt;0,9.99,0))</f>
-        <v>0.97121858555914</v>
+        <v>0.959051775604022</v>
       </c>
       <c r="S5" s="2" t="str">
         <f aca="false">IF(P5&gt;Q5+0.5,"OVER "&amp;Assumptions!$D$9&amp;"/wk – pace down",IF(R5&gt;Assumptions!$D$102,"Full",IF(AND(Q5&gt;=Assumptions!$D$103,P5&lt;Assumptions!$D$103),"Under "&amp;Assumptions!$D$103&amp;" – release reserve","")))</f>
         <v>Full</v>
       </c>
       <c r="T5" s="32" t="n">
-        <f aca="false">$F$38*(F5*(Budget!$G$21+Budget!$G$22+Budget!$G$23-$F$29-$F$36)+IF(A5-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($X$4:$X$14,A5-ROUNDUP(Funnel!$B$15/7,0))*$F$29+INDEX($Y$4:$Y$14,A5-ROUNDUP(Funnel!$B$15/7,0))*$F$36,0))</f>
+        <f aca="false">$F$38*(F5*(Budget!$G$21+Budget!$G$22+Budget!$G$23-$F$29-$F$36-$L$22-$L$26)+IF(A5-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($X$4:$X$14,A5-ROUNDUP(Funnel!$B$15/7,0))*$F$29+INDEX($Y$4:$Y$14,A5-ROUNDUP(Funnel!$B$15/7,0))*$F$36+INDEX($AB$4:$AB$14,A5-ROUNDUP(Funnel!$B$15/7,0))*$L$22+INDEX($AC$4:$AC$14,A5-ROUNDUP(Funnel!$B$15/7,0))*$L$26,0))</f>
         <v>0</v>
       </c>
       <c r="U5" s="32" t="n">
@@ -16736,11 +16867,27 @@
       </c>
       <c r="Z5" s="30" t="n">
         <f aca="false">Assumptions!$D$54</f>
-        <v>0.145</v>
+        <v>0.131</v>
       </c>
       <c r="AA5" s="30" t="n">
         <f aca="false">D5*IF(MAX(0,MIN(C5,Funnel!$B$19)-B5+1)&gt;0,MAX(0,MIN(C5,Funnel!$B$20)-B5+1)/MAX(0,MIN(C5,Funnel!$B$19)-B5+1),0)</f>
-        <v>0.145</v>
+        <v>0.131</v>
+      </c>
+      <c r="AB5" s="30" t="n">
+        <f aca="false">IF(SUM($AD$4:$AD$14)&gt;0,AD5/SUM($AD$4:$AD$14),0)</f>
+        <v>0.151520158625248</v>
+      </c>
+      <c r="AC5" s="30" t="n">
+        <f aca="false">IF(SUM($AE$4:$AE$14)&gt;0,AE5/SUM($AE$4:$AE$14),0)</f>
+        <v>0.191520467836257</v>
+      </c>
+      <c r="AD5" s="30" t="n">
+        <f aca="false">D5*IF(MAX(0,MIN(C5,Funnel!$B$19)-B5+1)&gt;0,MAX(0,MIN(C5,Funnel!$B$19)-MAX(B5,Assumptions!$D$7+Assumptions!$D$178)+1)/MAX(0,MIN(C5,Funnel!$B$19)-B5+1),0)</f>
+        <v>0.131</v>
+      </c>
+      <c r="AE5" s="30" t="n">
+        <f aca="false">D5*IF(MAX(0,MIN(C5,Funnel!$B$19)-B5+1)&gt;0,MAX(0,MIN(C5,Funnel!$B$19)-MAX(B5,Assumptions!$D$7+Assumptions!$D$179)+1)/MAX(0,MIN(C5,Funnel!$B$19)-B5+1),0)</f>
+        <v>0.131</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16757,11 +16904,11 @@
       </c>
       <c r="D6" s="30" t="n">
         <f aca="false">IF(SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$19)*$Z$4:$Z$14)&gt;0,IF(B6&lt;=Funnel!$B$19,Z6,0)/SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$19)*$Z$4:$Z$14),0)</f>
-        <v>0.18</v>
+        <v>0.161</v>
       </c>
       <c r="E6" s="30" t="n">
         <f aca="false">IF(SUM($AA$4:$AA$14)&gt;0,AA6/SUM($AA$4:$AA$14),0)</f>
-        <v>0.227642276422764</v>
+        <v>0.199787271760326</v>
       </c>
       <c r="F6" s="30" t="n">
         <f aca="false">IF(A6-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($D$4:$D$14,A6-ROUNDUP(Funnel!$B$15/7,0)),0)</f>
@@ -16772,8 +16919,8 @@
         <v>0</v>
       </c>
       <c r="H6" s="41" t="n">
-        <f aca="false">$F$19*D6+$F$20*E6+$F$31*Y6</f>
-        <v>14054.5700691509</v>
+        <f aca="false">($F$19-$L$19-$L$23)*D6+$L$19*AB6+$L$23*AC6+$F$20*E6+$F$31*Y6</f>
+        <v>13258.1331061054</v>
       </c>
       <c r="I6" s="41" t="n">
         <f aca="false">IF(A6=1,$F$21,0)</f>
@@ -16793,19 +16940,19 @@
       </c>
       <c r="M6" s="41" t="n">
         <f aca="false">SUM(H6:L6)</f>
-        <v>14054.5700691509</v>
+        <v>13258.1331061054</v>
       </c>
       <c r="N6" s="41" t="n">
         <f aca="false">SUM($M$4:M6)</f>
-        <v>61333.6003597877</v>
+        <v>61948.4220254793</v>
       </c>
       <c r="O6" s="29" t="n">
-        <f aca="false">(Funnel!$M$5+Funnel!$M$6+Funnel!$M$7-$F$27-$F$34)*D6+(Funnel!$M$8-$F$28-$F$35)*E6+($F$27+$F$28)*X6+($F$34+$F$35)*Y6</f>
-        <v>262.993773874947</v>
+        <f aca="false">(Funnel!$M$5+Funnel!$M$6+Funnel!$M$7-$F$27-$F$34-$L$20-$L$24)*D6+$L$20*AB6+$L$24*AC6+(Funnel!$M$8-$F$28-$F$35)*E6+($F$27+$F$28)*X6+($F$34+$F$35)*Y6</f>
+        <v>263.608822740179</v>
       </c>
       <c r="P6" s="29" t="n">
-        <f aca="false">(Funnel!$O$5+Funnel!$O$6+Funnel!$O$7-$F$25-$F$32)*D6+(Funnel!$O$8-$F$26-$F$33)*E6+($F$25+$F$26)*X6+($F$32+$F$33)*Y6</f>
-        <v>54.0675635459762</v>
+        <f aca="false">(Funnel!$O$5+Funnel!$O$6+Funnel!$O$7-$F$25-$F$32-$L$21-$L$25)*D6+$L$21*AB6+$L$25*AC6+(Funnel!$O$8-$F$26-$F$33)*E6+($F$25+$F$26)*X6+($F$32+$F$33)*Y6</f>
+        <v>52.7201803898792</v>
       </c>
       <c r="Q6" s="29" t="n">
         <f aca="false">Assumptions!$D$9*MAX(0,MIN(C6+Assumptions!$D$21,Funnel!$B$17)-MAX(IF(A6=1,Funnel!$B$13,B6+Assumptions!$D$21),Funnel!$B$13)+1)/7</f>
@@ -16813,14 +16960,14 @@
       </c>
       <c r="R6" s="30" t="n">
         <f aca="false">IF(Q6&gt;0,P6/Q6,IF(P6&gt;0,9.99,0))</f>
-        <v>0.98304660992684</v>
+        <v>0.95854873436144</v>
       </c>
       <c r="S6" s="2" t="str">
         <f aca="false">IF(P6&gt;Q6+0.5,"OVER "&amp;Assumptions!$D$9&amp;"/wk – pace down",IF(R6&gt;Assumptions!$D$102,"Full",IF(AND(Q6&gt;=Assumptions!$D$103,P6&lt;Assumptions!$D$103),"Under "&amp;Assumptions!$D$103&amp;" – release reserve","")))</f>
         <v>Full</v>
       </c>
       <c r="T6" s="32" t="n">
-        <f aca="false">$F$38*(F6*(Budget!$G$21+Budget!$G$22+Budget!$G$23-$F$29-$F$36)+IF(A6-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($X$4:$X$14,A6-ROUNDUP(Funnel!$B$15/7,0))*$F$29+INDEX($Y$4:$Y$14,A6-ROUNDUP(Funnel!$B$15/7,0))*$F$36,0))</f>
+        <f aca="false">$F$38*(F6*(Budget!$G$21+Budget!$G$22+Budget!$G$23-$F$29-$F$36-$L$22-$L$26)+IF(A6-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($X$4:$X$14,A6-ROUNDUP(Funnel!$B$15/7,0))*$F$29+INDEX($Y$4:$Y$14,A6-ROUNDUP(Funnel!$B$15/7,0))*$F$36+INDEX($AB$4:$AB$14,A6-ROUNDUP(Funnel!$B$15/7,0))*$L$22+INDEX($AC$4:$AC$14,A6-ROUNDUP(Funnel!$B$15/7,0))*$L$26,0))</f>
         <v>0</v>
       </c>
       <c r="U6" s="32" t="n">
@@ -16845,11 +16992,27 @@
       </c>
       <c r="Z6" s="30" t="n">
         <f aca="false">Assumptions!$D$55</f>
-        <v>0.18</v>
+        <v>0.161</v>
       </c>
       <c r="AA6" s="30" t="n">
         <f aca="false">D6*IF(MAX(0,MIN(C6,Funnel!$B$19)-B6+1)&gt;0,MAX(0,MIN(C6,Funnel!$B$20)-B6+1)/MAX(0,MIN(C6,Funnel!$B$19)-B6+1),0)</f>
-        <v>0.18</v>
+        <v>0.161</v>
+      </c>
+      <c r="AB6" s="30" t="n">
+        <f aca="false">IF(SUM($AD$4:$AD$14)&gt;0,AD6/SUM($AD$4:$AD$14),0)</f>
+        <v>0.186219431592862</v>
+      </c>
+      <c r="AC6" s="30" t="n">
+        <f aca="false">IF(SUM($AE$4:$AE$14)&gt;0,AE6/SUM($AE$4:$AE$14),0)</f>
+        <v>0.235380116959064</v>
+      </c>
+      <c r="AD6" s="30" t="n">
+        <f aca="false">D6*IF(MAX(0,MIN(C6,Funnel!$B$19)-B6+1)&gt;0,MAX(0,MIN(C6,Funnel!$B$19)-MAX(B6,Assumptions!$D$7+Assumptions!$D$178)+1)/MAX(0,MIN(C6,Funnel!$B$19)-B6+1),0)</f>
+        <v>0.161</v>
+      </c>
+      <c r="AE6" s="30" t="n">
+        <f aca="false">D6*IF(MAX(0,MIN(C6,Funnel!$B$19)-B6+1)&gt;0,MAX(0,MIN(C6,Funnel!$B$19)-MAX(B6,Assumptions!$D$7+Assumptions!$D$179)+1)/MAX(0,MIN(C6,Funnel!$B$19)-B6+1),0)</f>
+        <v>0.161</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16866,23 +17029,23 @@
       </c>
       <c r="D7" s="30" t="n">
         <f aca="false">IF(SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$19)*$Z$4:$Z$14)&gt;0,IF(B7&lt;=Funnel!$B$19,Z7,0)/SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$19)*$Z$4:$Z$14),0)</f>
-        <v>0.185</v>
+        <v>0.17</v>
       </c>
       <c r="E7" s="30" t="n">
         <f aca="false">IF(SUM($AA$4:$AA$14)&gt;0,AA7/SUM($AA$4:$AA$14),0)</f>
-        <v>0.233965672990063</v>
+        <v>0.210955504343202</v>
       </c>
       <c r="F7" s="30" t="n">
         <f aca="false">IF(A7-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($D$4:$D$14,A7-ROUNDUP(Funnel!$B$15/7,0)),0)</f>
-        <v>0.25</v>
+        <v>0.316</v>
       </c>
       <c r="G7" s="30" t="n">
         <f aca="false">IF(A7-ROUNDUP(Funnel!$B$16/7,0)&gt;=1,INDEX($E$4:$E$14,A7-ROUNDUP(Funnel!$B$16/7,0)),0)</f>
         <v>0</v>
       </c>
       <c r="H7" s="41" t="n">
-        <f aca="false">$F$19*D7+$F$20*E7+$F$31*Y7</f>
-        <v>14437.8183766273</v>
+        <f aca="false">($F$19-$L$19-$L$23)*D7+$L$19*AB7+$L$23*AC7+$F$20*E7+$F$31*Y7</f>
+        <v>13991.9187455771</v>
       </c>
       <c r="I7" s="41" t="n">
         <f aca="false">IF(A7=1,$F$21,0)</f>
@@ -16890,7 +17053,7 @@
       </c>
       <c r="J7" s="41" t="n">
         <f aca="false">$F$22*F7+$F$23*G7</f>
-        <v>2467.310625</v>
+        <v>3118.68063</v>
       </c>
       <c r="K7" s="41" t="n">
         <f aca="false">IF(A7=1,Budget!$C$6,0)</f>
@@ -16902,19 +17065,19 @@
       </c>
       <c r="M7" s="41" t="n">
         <f aca="false">SUM(H7:L7)</f>
-        <v>16905.1290016273</v>
+        <v>17110.5993755771</v>
       </c>
       <c r="N7" s="41" t="n">
         <f aca="false">SUM($M$4:M7)</f>
-        <v>78238.729361415</v>
+        <v>79059.0214010564</v>
       </c>
       <c r="O7" s="29" t="n">
-        <f aca="false">(Funnel!$M$5+Funnel!$M$6+Funnel!$M$7-$F$27-$F$34)*D7+(Funnel!$M$8-$F$28-$F$35)*E7+($F$27+$F$28)*X7+($F$34+$F$35)*Y7</f>
-        <v>267.436589815917</v>
+        <f aca="false">(Funnel!$M$5+Funnel!$M$6+Funnel!$M$7-$F$27-$F$34-$L$20-$L$24)*D7+$L$20*AB7+$L$24*AC7+(Funnel!$M$8-$F$28-$F$35)*E7+($F$27+$F$28)*X7+($F$34+$F$35)*Y7</f>
+        <v>275.403825253605</v>
       </c>
       <c r="P7" s="29" t="n">
-        <f aca="false">(Funnel!$O$5+Funnel!$O$6+Funnel!$O$7-$F$25-$F$32)*D7+(Funnel!$O$8-$F$26-$F$33)*E7+($F$25+$F$26)*X7+($F$32+$F$33)*Y7</f>
-        <v>54.1381569778089</v>
+        <f aca="false">(Funnel!$O$5+Funnel!$O$6+Funnel!$O$7-$F$25-$F$32-$L$21-$L$25)*D7+$L$21*AB7+$L$25*AC7+(Funnel!$O$8-$F$26-$F$33)*E7+($F$25+$F$26)*X7+($F$32+$F$33)*Y7</f>
+        <v>54.1968240141581</v>
       </c>
       <c r="Q7" s="29" t="n">
         <f aca="false">Assumptions!$D$9*MAX(0,MIN(C7+Assumptions!$D$21,Funnel!$B$17)-MAX(IF(A7=1,Funnel!$B$13,B7+Assumptions!$D$21),Funnel!$B$13)+1)/7</f>
@@ -16922,15 +17085,15 @@
       </c>
       <c r="R7" s="30" t="n">
         <f aca="false">IF(Q7&gt;0,P7/Q7,IF(P7&gt;0,9.99,0))</f>
-        <v>0.984330126869253</v>
+        <v>0.985396800257421</v>
       </c>
       <c r="S7" s="2" t="str">
         <f aca="false">IF(P7&gt;Q7+0.5,"OVER "&amp;Assumptions!$D$9&amp;"/wk – pace down",IF(R7&gt;Assumptions!$D$102,"Full",IF(AND(Q7&gt;=Assumptions!$D$103,P7&lt;Assumptions!$D$103),"Under "&amp;Assumptions!$D$103&amp;" – release reserve","")))</f>
         <v>Full</v>
       </c>
       <c r="T7" s="32" t="n">
-        <f aca="false">$F$38*(F7*(Budget!$G$21+Budget!$G$22+Budget!$G$23-$F$29-$F$36)+IF(A7-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($X$4:$X$14,A7-ROUNDUP(Funnel!$B$15/7,0))*$F$29+INDEX($Y$4:$Y$14,A7-ROUNDUP(Funnel!$B$15/7,0))*$F$36,0))</f>
-        <v>24.3641121536279</v>
+        <f aca="false">$F$38*(F7*(Budget!$G$21+Budget!$G$22+Budget!$G$23-$F$29-$F$36-$L$22-$L$26)+IF(A7-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($X$4:$X$14,A7-ROUNDUP(Funnel!$B$15/7,0))*$F$29+INDEX($Y$4:$Y$14,A7-ROUNDUP(Funnel!$B$15/7,0))*$F$36+INDEX($AB$4:$AB$14,A7-ROUNDUP(Funnel!$B$15/7,0))*$L$22+INDEX($AC$4:$AC$14,A7-ROUNDUP(Funnel!$B$15/7,0))*$L$26,0))</f>
+        <v>23.2608949040937</v>
       </c>
       <c r="U7" s="32" t="n">
         <f aca="false">$F$38*(G7*(Budget!$G$24-$F$30-$F$37)+IF(A7-ROUNDUP(Funnel!$B$16/7,0)&gt;=1,INDEX($X$4:$X$14,A7-ROUNDUP(Funnel!$B$16/7,0))*$F$30+INDEX($Y$4:$Y$14,A7-ROUNDUP(Funnel!$B$16/7,0))*$F$37,0))</f>
@@ -16938,11 +17101,11 @@
       </c>
       <c r="V7" s="32" t="n">
         <f aca="false">T7+U7</f>
-        <v>24.3641121536279</v>
+        <v>23.2608949040937</v>
       </c>
       <c r="W7" s="32" t="n">
         <f aca="false">SUM($V$4:V7)</f>
-        <v>24.3641121536279</v>
+        <v>23.2608949040937</v>
       </c>
       <c r="X7" s="30" t="n">
         <f aca="false">IF(A7=1,Assumptions!$D$50,IF(A7=2,1-Assumptions!$D$50,0))</f>
@@ -16954,11 +17117,27 @@
       </c>
       <c r="Z7" s="30" t="n">
         <f aca="false">Assumptions!$D$56</f>
-        <v>0.185</v>
+        <v>0.17</v>
       </c>
       <c r="AA7" s="30" t="n">
         <f aca="false">D7*IF(MAX(0,MIN(C7,Funnel!$B$19)-B7+1)&gt;0,MAX(0,MIN(C7,Funnel!$B$20)-B7+1)/MAX(0,MIN(C7,Funnel!$B$19)-B7+1),0)</f>
-        <v>0.185</v>
+        <v>0.17</v>
+      </c>
+      <c r="AB7" s="30" t="n">
+        <f aca="false">IF(SUM($AD$4:$AD$14)&gt;0,AD7/SUM($AD$4:$AD$14),0)</f>
+        <v>0.196629213483146</v>
+      </c>
+      <c r="AC7" s="30" t="n">
+        <f aca="false">IF(SUM($AE$4:$AE$14)&gt;0,AE7/SUM($AE$4:$AE$14),0)</f>
+        <v>0.248538011695906</v>
+      </c>
+      <c r="AD7" s="30" t="n">
+        <f aca="false">D7*IF(MAX(0,MIN(C7,Funnel!$B$19)-B7+1)&gt;0,MAX(0,MIN(C7,Funnel!$B$19)-MAX(B7,Assumptions!$D$7+Assumptions!$D$178)+1)/MAX(0,MIN(C7,Funnel!$B$19)-B7+1),0)</f>
+        <v>0.17</v>
+      </c>
+      <c r="AE7" s="30" t="n">
+        <f aca="false">D7*IF(MAX(0,MIN(C7,Funnel!$B$19)-B7+1)&gt;0,MAX(0,MIN(C7,Funnel!$B$19)-MAX(B7,Assumptions!$D$7+Assumptions!$D$179)+1)/MAX(0,MIN(C7,Funnel!$B$19)-B7+1),0)</f>
+        <v>0.17</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16975,23 +17154,23 @@
       </c>
       <c r="D8" s="30" t="n">
         <f aca="false">IF(SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$19)*$Z$4:$Z$14)&gt;0,IF(B8&lt;=Funnel!$B$19,Z8,0)/SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$19)*$Z$4:$Z$14),0)</f>
-        <v>0.215</v>
+        <v>0.195</v>
       </c>
       <c r="E8" s="30" t="n">
         <f aca="false">IF(SUM($AA$4:$AA$14)&gt;0,AA8/SUM($AA$4:$AA$14),0)</f>
-        <v>0.038843721770551</v>
+        <v>0.0345683389469952</v>
       </c>
       <c r="F8" s="30" t="n">
         <f aca="false">IF(A8-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($D$4:$D$14,A8-ROUNDUP(Funnel!$B$15/7,0)),0)</f>
-        <v>0.145</v>
+        <v>0.131</v>
       </c>
       <c r="G8" s="30" t="n">
         <f aca="false">IF(A8-ROUNDUP(Funnel!$B$16/7,0)&gt;=1,INDEX($E$4:$E$14,A8-ROUNDUP(Funnel!$B$16/7,0)),0)</f>
-        <v>0.31616982836495</v>
+        <v>0.392129055132069</v>
       </c>
       <c r="H8" s="41" t="n">
-        <f aca="false">$F$19*D8+$F$20*E8+$F$31*Y8</f>
-        <v>13940.6975137465</v>
+        <f aca="false">($F$19-$L$19-$L$23)*D8+$L$19*AB8+$L$23*AC8+$F$20*E8+$F$31*Y8</f>
+        <v>13523.5759509396</v>
       </c>
       <c r="I8" s="41" t="n">
         <f aca="false">IF(A8=1,$F$21,0)</f>
@@ -16999,7 +17178,7 @@
       </c>
       <c r="J8" s="41" t="n">
         <f aca="false">$F$22*F8+$F$23*G8</f>
-        <v>1781.50967469512</v>
+        <v>1727.53994317807</v>
       </c>
       <c r="K8" s="41" t="n">
         <f aca="false">IF(A8=1,Budget!$C$6,0)</f>
@@ -17011,19 +17190,19 @@
       </c>
       <c r="M8" s="41" t="n">
         <f aca="false">SUM(H8:L8)</f>
-        <v>15722.2071884416</v>
+        <v>15251.1158941177</v>
       </c>
       <c r="N8" s="41" t="n">
         <f aca="false">SUM($M$4:M8)</f>
-        <v>93960.9365498566</v>
+        <v>94310.1372951741</v>
       </c>
       <c r="O8" s="29" t="n">
-        <f aca="false">(Funnel!$M$5+Funnel!$M$6+Funnel!$M$7-$F$27-$F$34)*D8+(Funnel!$M$8-$F$28-$F$35)*E8+($F$27+$F$28)*X8+($F$34+$F$35)*Y8</f>
-        <v>270.983393875365</v>
+        <f aca="false">(Funnel!$M$5+Funnel!$M$6+Funnel!$M$7-$F$27-$F$34-$L$20-$L$24)*D8+$L$20*AB8+$L$24*AC8+(Funnel!$M$8-$F$28-$F$35)*E8+($F$27+$F$28)*X8+($F$34+$F$35)*Y8</f>
+        <v>280.466076472631</v>
       </c>
       <c r="P8" s="29" t="n">
-        <f aca="false">(Funnel!$O$5+Funnel!$O$6+Funnel!$O$7-$F$25-$F$32)*D8+(Funnel!$O$8-$F$26-$F$33)*E8+($F$25+$F$26)*X8+($F$32+$F$33)*Y8</f>
-        <v>54.5398332456552</v>
+        <f aca="false">(Funnel!$O$5+Funnel!$O$6+Funnel!$O$7-$F$25-$F$32-$L$21-$L$25)*D8+$L$21*AB8+$L$25*AC8+(Funnel!$O$8-$F$26-$F$33)*E8+($F$25+$F$26)*X8+($F$32+$F$33)*Y8</f>
+        <v>54.7115391603946</v>
       </c>
       <c r="Q8" s="29" t="n">
         <f aca="false">Assumptions!$D$9*MAX(0,MIN(C8+Assumptions!$D$21,Funnel!$B$17)-MAX(IF(A8=1,Funnel!$B$13,B8+Assumptions!$D$21),Funnel!$B$13)+1)/7</f>
@@ -17031,27 +17210,27 @@
       </c>
       <c r="R8" s="30" t="n">
         <f aca="false">IF(Q8&gt;0,P8/Q8,IF(P8&gt;0,9.99,0))</f>
-        <v>0.991633331739186</v>
+        <v>0.99475525746172</v>
       </c>
       <c r="S8" s="2" t="str">
         <f aca="false">IF(P8&gt;Q8+0.5,"OVER "&amp;Assumptions!$D$9&amp;"/wk – pace down",IF(R8&gt;Assumptions!$D$102,"Full",IF(AND(Q8&gt;=Assumptions!$D$103,P8&lt;Assumptions!$D$103),"Under "&amp;Assumptions!$D$103&amp;" – release reserve","")))</f>
         <v>Full</v>
       </c>
       <c r="T8" s="32" t="n">
-        <f aca="false">$F$38*(F8*(Budget!$G$21+Budget!$G$22+Budget!$G$23-$F$29-$F$36)+IF(A8-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($X$4:$X$14,A8-ROUNDUP(Funnel!$B$15/7,0))*$F$29+INDEX($Y$4:$Y$14,A8-ROUNDUP(Funnel!$B$15/7,0))*$F$36,0))</f>
-        <v>14.9434387826712</v>
+        <f aca="false">$F$38*(F8*(Budget!$G$21+Budget!$G$22+Budget!$G$23-$F$29-$F$36-$L$22-$L$26)+IF(A8-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($X$4:$X$14,A8-ROUNDUP(Funnel!$B$15/7,0))*$F$29+INDEX($Y$4:$Y$14,A8-ROUNDUP(Funnel!$B$15/7,0))*$F$36+INDEX($AB$4:$AB$14,A8-ROUNDUP(Funnel!$B$15/7,0))*$L$22+INDEX($AC$4:$AC$14,A8-ROUNDUP(Funnel!$B$15/7,0))*$L$26,0))</f>
+        <v>15.0418178773517</v>
       </c>
       <c r="U8" s="32" t="n">
         <f aca="false">$F$38*(G8*(Budget!$G$24-$F$30-$F$37)+IF(A8-ROUNDUP(Funnel!$B$16/7,0)&gt;=1,INDEX($X$4:$X$14,A8-ROUNDUP(Funnel!$B$16/7,0))*$F$30+INDEX($Y$4:$Y$14,A8-ROUNDUP(Funnel!$B$16/7,0))*$F$37,0))</f>
-        <v>3.37581560318138</v>
+        <v>4.03662708146645</v>
       </c>
       <c r="V8" s="32" t="n">
         <f aca="false">T8+U8</f>
-        <v>18.3192543858526</v>
+        <v>19.0784449588182</v>
       </c>
       <c r="W8" s="32" t="n">
         <f aca="false">SUM($V$4:V8)</f>
-        <v>42.6833665394805</v>
+        <v>42.3393398629119</v>
       </c>
       <c r="X8" s="30" t="n">
         <f aca="false">IF(A8=1,Assumptions!$D$50,IF(A8=2,1-Assumptions!$D$50,0))</f>
@@ -17063,11 +17242,27 @@
       </c>
       <c r="Z8" s="30" t="n">
         <f aca="false">Assumptions!$D$57</f>
-        <v>0.215</v>
+        <v>0.195</v>
       </c>
       <c r="AA8" s="30" t="n">
         <f aca="false">D8*IF(MAX(0,MIN(C8,Funnel!$B$19)-B8+1)&gt;0,MAX(0,MIN(C8,Funnel!$B$20)-B8+1)/MAX(0,MIN(C8,Funnel!$B$19)-B8+1),0)</f>
-        <v>0.0307142857142857</v>
+        <v>0.0278571428571429</v>
+      </c>
+      <c r="AB8" s="30" t="n">
+        <f aca="false">IF(SUM($AD$4:$AD$14)&gt;0,AD8/SUM($AD$4:$AD$14),0)</f>
+        <v>0.225545274289491</v>
+      </c>
+      <c r="AC8" s="30" t="n">
+        <f aca="false">IF(SUM($AE$4:$AE$14)&gt;0,AE8/SUM($AE$4:$AE$14),0)</f>
+        <v>0.285087719298246</v>
+      </c>
+      <c r="AD8" s="30" t="n">
+        <f aca="false">D8*IF(MAX(0,MIN(C8,Funnel!$B$19)-B8+1)&gt;0,MAX(0,MIN(C8,Funnel!$B$19)-MAX(B8,Assumptions!$D$7+Assumptions!$D$178)+1)/MAX(0,MIN(C8,Funnel!$B$19)-B8+1),0)</f>
+        <v>0.195</v>
+      </c>
+      <c r="AE8" s="30" t="n">
+        <f aca="false">D8*IF(MAX(0,MIN(C8,Funnel!$B$19)-B8+1)&gt;0,MAX(0,MIN(C8,Funnel!$B$19)-MAX(B8,Assumptions!$D$7+Assumptions!$D$179)+1)/MAX(0,MIN(C8,Funnel!$B$19)-B8+1),0)</f>
+        <v>0.195</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17084,7 +17279,7 @@
       </c>
       <c r="D9" s="30" t="n">
         <f aca="false">IF(SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$19)*$Z$4:$Z$14)&gt;0,IF(B9&lt;=Funnel!$B$19,Z9,0)/SUMPRODUCT(($B$4:$B$14&lt;=Funnel!$B$19)*$Z$4:$Z$14),0)</f>
-        <v>0.025</v>
+        <v>0.027</v>
       </c>
       <c r="E9" s="30" t="n">
         <f aca="false">IF(SUM($AA$4:$AA$14)&gt;0,AA9/SUM($AA$4:$AA$14),0)</f>
@@ -17092,15 +17287,15 @@
       </c>
       <c r="F9" s="30" t="n">
         <f aca="false">IF(A9-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($D$4:$D$14,A9-ROUNDUP(Funnel!$B$15/7,0)),0)</f>
-        <v>0.18</v>
+        <v>0.161</v>
       </c>
       <c r="G9" s="30" t="n">
         <f aca="false">IF(A9-ROUNDUP(Funnel!$B$16/7,0)&gt;=1,INDEX($E$4:$E$14,A9-ROUNDUP(Funnel!$B$16/7,0)),0)</f>
-        <v>0.183378500451671</v>
+        <v>0.162559829817408</v>
       </c>
       <c r="H9" s="41" t="n">
-        <f aca="false">$F$19*D9+$F$20*E9+$F$31*Y9</f>
-        <v>1566.003805712</v>
+        <f aca="false">($F$19-$L$19-$L$23)*D9+$L$19*AB9+$L$23*AC9+$F$20*E9+$F$31*Y9</f>
+        <v>1814.20333387746</v>
       </c>
       <c r="I9" s="41" t="n">
         <f aca="false">IF(A9=1,$F$21,0)</f>
@@ -17108,7 +17303,7 @@
       </c>
       <c r="J9" s="41" t="n">
         <f aca="false">$F$22*F9+$F$23*G9</f>
-        <v>1979.73596707317</v>
+        <v>1769.14317545515</v>
       </c>
       <c r="K9" s="41" t="n">
         <f aca="false">IF(A9=1,Budget!$C$6,0)</f>
@@ -17120,19 +17315,19 @@
       </c>
       <c r="M9" s="41" t="n">
         <f aca="false">SUM(H9:L9)</f>
-        <v>3545.73977278518</v>
+        <v>3583.34650933261</v>
       </c>
       <c r="N9" s="41" t="n">
         <f aca="false">SUM($M$4:M9)</f>
-        <v>97506.6763226418</v>
+        <v>97893.4838045067</v>
       </c>
       <c r="O9" s="29" t="n">
-        <f aca="false">(Funnel!$M$5+Funnel!$M$6+Funnel!$M$7-$F$27-$F$34)*D9+(Funnel!$M$8-$F$28-$F$35)*E9+($F$27+$F$28)*X9+($F$34+$F$35)*Y9</f>
-        <v>30.7379665051514</v>
+        <f aca="false">(Funnel!$M$5+Funnel!$M$6+Funnel!$M$7-$F$27-$F$34-$L$20-$L$24)*D9+$L$20*AB9+$L$24*AC9+(Funnel!$M$8-$F$28-$F$35)*E9+($F$27+$F$28)*X9+($F$34+$F$35)*Y9</f>
+        <v>38.0159572504042</v>
       </c>
       <c r="P9" s="29" t="n">
-        <f aca="false">(Funnel!$O$5+Funnel!$O$6+Funnel!$O$7-$F$25-$F$32)*D9+(Funnel!$O$8-$F$26-$F$33)*E9+($F$25+$F$26)*X9+($F$32+$F$33)*Y9</f>
-        <v>6.17948672772832</v>
+        <f aca="false">(Funnel!$O$5+Funnel!$O$6+Funnel!$O$7-$F$25-$F$32-$L$21-$L$25)*D9+$L$21*AB9+$L$25*AC9+(Funnel!$O$8-$F$26-$F$33)*E9+($F$25+$F$26)*X9+($F$32+$F$33)*Y9</f>
+        <v>7.40339605223196</v>
       </c>
       <c r="Q9" s="29" t="n">
         <f aca="false">Assumptions!$D$9*MAX(0,MIN(C9+Assumptions!$D$21,Funnel!$B$17)-MAX(IF(A9=1,Funnel!$B$13,B9+Assumptions!$D$21),Funnel!$B$13)+1)/7</f>
@@ -17140,27 +17335,27 @@
       </c>
       <c r="R9" s="30" t="n">
         <f aca="false">IF(Q9&gt;0,P9/Q9,IF(P9&gt;0,9.99,0))</f>
-        <v>0.786480128983605</v>
+        <v>0.942250406647704</v>
       </c>
       <c r="S9" s="2" t="str">
         <f aca="false">IF(P9&gt;Q9+0.5,"OVER "&amp;Assumptions!$D$9&amp;"/wk – pace down",IF(R9&gt;Assumptions!$D$102,"Full",IF(AND(Q9&gt;=Assumptions!$D$103,P9&lt;Assumptions!$D$103),"Under "&amp;Assumptions!$D$103&amp;" – release reserve","")))</f>
-        <v/>
+        <v>Full</v>
       </c>
       <c r="T9" s="32" t="n">
-        <f aca="false">$F$38*(F9*(Budget!$G$21+Budget!$G$22+Budget!$G$23-$F$29-$F$36)+IF(A9-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($X$4:$X$14,A9-ROUNDUP(Funnel!$B$15/7,0))*$F$29+INDEX($Y$4:$Y$14,A9-ROUNDUP(Funnel!$B$15/7,0))*$F$36,0))</f>
-        <v>15.3990968656466</v>
+        <f aca="false">$F$38*(F9*(Budget!$G$21+Budget!$G$22+Budget!$G$23-$F$29-$F$36-$L$22-$L$26)+IF(A9-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($X$4:$X$14,A9-ROUNDUP(Funnel!$B$15/7,0))*$F$29+INDEX($Y$4:$Y$14,A9-ROUNDUP(Funnel!$B$15/7,0))*$F$36+INDEX($AB$4:$AB$14,A9-ROUNDUP(Funnel!$B$15/7,0))*$L$22+INDEX($AC$4:$AC$14,A9-ROUNDUP(Funnel!$B$15/7,0))*$L$26,0))</f>
+        <v>15.3710349309716</v>
       </c>
       <c r="U9" s="32" t="n">
         <f aca="false">$F$38*(G9*(Budget!$G$24-$F$30-$F$37)+IF(A9-ROUNDUP(Funnel!$B$16/7,0)&gt;=1,INDEX($X$4:$X$14,A9-ROUNDUP(Funnel!$B$16/7,0))*$F$30+INDEX($Y$4:$Y$14,A9-ROUNDUP(Funnel!$B$16/7,0))*$F$37,0))</f>
-        <v>2.2126720706385</v>
+        <v>2.03155889843711</v>
       </c>
       <c r="V9" s="32" t="n">
         <f aca="false">T9+U9</f>
-        <v>17.6117689362851</v>
+        <v>17.4025938294087</v>
       </c>
       <c r="W9" s="32" t="n">
         <f aca="false">SUM($V$4:V9)</f>
-        <v>60.2951354757655</v>
+        <v>59.7419336923206</v>
       </c>
       <c r="X9" s="30" t="n">
         <f aca="false">IF(A9=1,Assumptions!$D$50,IF(A9=2,1-Assumptions!$D$50,0))</f>
@@ -17172,11 +17367,27 @@
       </c>
       <c r="Z9" s="30" t="n">
         <f aca="false">Assumptions!$D$58</f>
-        <v>0.025</v>
+        <v>0.027</v>
       </c>
       <c r="AA9" s="30" t="n">
         <f aca="false">D9*IF(MAX(0,MIN(C9,Funnel!$B$19)-B9+1)&gt;0,MAX(0,MIN(C9,Funnel!$B$20)-B9+1)/MAX(0,MIN(C9,Funnel!$B$19)-B9+1),0)</f>
         <v>0</v>
+      </c>
+      <c r="AB9" s="30" t="n">
+        <f aca="false">IF(SUM($AD$4:$AD$14)&gt;0,AD9/SUM($AD$4:$AD$14),0)</f>
+        <v>0.0312293456708526</v>
+      </c>
+      <c r="AC9" s="30" t="n">
+        <f aca="false">IF(SUM($AE$4:$AE$14)&gt;0,AE9/SUM($AE$4:$AE$14),0)</f>
+        <v>0.0394736842105263</v>
+      </c>
+      <c r="AD9" s="30" t="n">
+        <f aca="false">D9*IF(MAX(0,MIN(C9,Funnel!$B$19)-B9+1)&gt;0,MAX(0,MIN(C9,Funnel!$B$19)-MAX(B9,Assumptions!$D$7+Assumptions!$D$178)+1)/MAX(0,MIN(C9,Funnel!$B$19)-B9+1),0)</f>
+        <v>0.027</v>
+      </c>
+      <c r="AE9" s="30" t="n">
+        <f aca="false">D9*IF(MAX(0,MIN(C9,Funnel!$B$19)-B9+1)&gt;0,MAX(0,MIN(C9,Funnel!$B$19)-MAX(B9,Assumptions!$D$7+Assumptions!$D$179)+1)/MAX(0,MIN(C9,Funnel!$B$19)-B9+1),0)</f>
+        <v>0.027</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17201,14 +17412,14 @@
       </c>
       <c r="F10" s="30" t="n">
         <f aca="false">IF(A10-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($D$4:$D$14,A10-ROUNDUP(Funnel!$B$15/7,0)),0)</f>
-        <v>0.185</v>
+        <v>0.17</v>
       </c>
       <c r="G10" s="30" t="n">
         <f aca="false">IF(A10-ROUNDUP(Funnel!$B$16/7,0)&gt;=1,INDEX($E$4:$E$14,A10-ROUNDUP(Funnel!$B$16/7,0)),0)</f>
-        <v>0.227642276422764</v>
+        <v>0.199787271760326</v>
       </c>
       <c r="H10" s="41" t="n">
-        <f aca="false">$F$19*D10+$F$20*E10+$F$31*Y10</f>
+        <f aca="false">($F$19-$L$19-$L$23)*D10+$L$19*AB10+$L$23*AC10+$F$20*E10+$F$31*Y10</f>
         <v>0</v>
       </c>
       <c r="I10" s="41" t="n">
@@ -17217,7 +17428,7 @@
       </c>
       <c r="J10" s="41" t="n">
         <f aca="false">$F$22*F10+$F$23*G10</f>
-        <v>2078.14791128049</v>
+        <v>1899.23241893725</v>
       </c>
       <c r="K10" s="41" t="n">
         <f aca="false">IF(A10=1,Budget!$C$6,0)</f>
@@ -17229,18 +17440,18 @@
       </c>
       <c r="M10" s="41" t="n">
         <f aca="false">SUM(H10:L10)</f>
-        <v>2078.14791128049</v>
+        <v>1899.23241893725</v>
       </c>
       <c r="N10" s="41" t="n">
         <f aca="false">SUM($M$4:M10)</f>
-        <v>99584.8242339222</v>
+        <v>99792.7162234439</v>
       </c>
       <c r="O10" s="29" t="n">
-        <f aca="false">(Funnel!$M$5+Funnel!$M$6+Funnel!$M$7-$F$27-$F$34)*D10+(Funnel!$M$8-$F$28-$F$35)*E10+($F$27+$F$28)*X10+($F$34+$F$35)*Y10</f>
+        <f aca="false">(Funnel!$M$5+Funnel!$M$6+Funnel!$M$7-$F$27-$F$34-$L$20-$L$24)*D10+$L$20*AB10+$L$24*AC10+(Funnel!$M$8-$F$28-$F$35)*E10+($F$27+$F$28)*X10+($F$34+$F$35)*Y10</f>
         <v>0</v>
       </c>
       <c r="P10" s="29" t="n">
-        <f aca="false">(Funnel!$O$5+Funnel!$O$6+Funnel!$O$7-$F$25-$F$32)*D10+(Funnel!$O$8-$F$26-$F$33)*E10+($F$25+$F$26)*X10+($F$32+$F$33)*Y10</f>
+        <f aca="false">(Funnel!$O$5+Funnel!$O$6+Funnel!$O$7-$F$25-$F$32-$L$21-$L$25)*D10+$L$21*AB10+$L$25*AC10+(Funnel!$O$8-$F$26-$F$33)*E10+($F$25+$F$26)*X10+($F$32+$F$33)*Y10</f>
         <v>0</v>
       </c>
       <c r="Q10" s="29" t="n">
@@ -17256,20 +17467,20 @@
         <v/>
       </c>
       <c r="T10" s="32" t="n">
-        <f aca="false">$F$38*(F10*(Budget!$G$21+Budget!$G$22+Budget!$G$23-$F$29-$F$36)+IF(A10-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($X$4:$X$14,A10-ROUNDUP(Funnel!$B$15/7,0))*$F$29+INDEX($Y$4:$Y$14,A10-ROUNDUP(Funnel!$B$15/7,0))*$F$36,0))</f>
-        <v>15.362988603859</v>
+        <f aca="false">$F$38*(F10*(Budget!$G$21+Budget!$G$22+Budget!$G$23-$F$29-$F$36-$L$22-$L$26)+IF(A10-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($X$4:$X$14,A10-ROUNDUP(Funnel!$B$15/7,0))*$F$29+INDEX($Y$4:$Y$14,A10-ROUNDUP(Funnel!$B$15/7,0))*$F$36+INDEX($AB$4:$AB$14,A10-ROUNDUP(Funnel!$B$15/7,0))*$L$22+INDEX($AC$4:$AC$14,A10-ROUNDUP(Funnel!$B$15/7,0))*$L$26,0))</f>
+        <v>15.753731859411</v>
       </c>
       <c r="U10" s="32" t="n">
         <f aca="false">$F$38*(G10*(Budget!$G$24-$F$30-$F$37)+IF(A10-ROUNDUP(Funnel!$B$16/7,0)&gt;=1,INDEX($X$4:$X$14,A10-ROUNDUP(Funnel!$B$16/7,0))*$F$30+INDEX($Y$4:$Y$14,A10-ROUNDUP(Funnel!$B$16/7,0))*$F$37,0))</f>
-        <v>2.03819196584367</v>
+        <v>1.79586581809263</v>
       </c>
       <c r="V10" s="32" t="n">
         <f aca="false">T10+U10</f>
-        <v>17.4011805697026</v>
+        <v>17.5495976775036</v>
       </c>
       <c r="W10" s="32" t="n">
         <f aca="false">SUM($V$4:V10)</f>
-        <v>77.6963160454681</v>
+        <v>77.2915313698242</v>
       </c>
       <c r="X10" s="30" t="n">
         <f aca="false">IF(A10=1,Assumptions!$D$50,IF(A10=2,1-Assumptions!$D$50,0))</f>
@@ -17285,6 +17496,22 @@
       </c>
       <c r="AA10" s="30" t="n">
         <f aca="false">D10*IF(MAX(0,MIN(C10,Funnel!$B$19)-B10+1)&gt;0,MAX(0,MIN(C10,Funnel!$B$20)-B10+1)/MAX(0,MIN(C10,Funnel!$B$19)-B10+1),0)</f>
+        <v>0</v>
+      </c>
+      <c r="AB10" s="30" t="n">
+        <f aca="false">IF(SUM($AD$4:$AD$14)&gt;0,AD10/SUM($AD$4:$AD$14),0)</f>
+        <v>0</v>
+      </c>
+      <c r="AC10" s="30" t="n">
+        <f aca="false">IF(SUM($AE$4:$AE$14)&gt;0,AE10/SUM($AE$4:$AE$14),0)</f>
+        <v>0</v>
+      </c>
+      <c r="AD10" s="30" t="n">
+        <f aca="false">D10*IF(MAX(0,MIN(C10,Funnel!$B$19)-B10+1)&gt;0,MAX(0,MIN(C10,Funnel!$B$19)-MAX(B10,Assumptions!$D$7+Assumptions!$D$178)+1)/MAX(0,MIN(C10,Funnel!$B$19)-B10+1),0)</f>
+        <v>0</v>
+      </c>
+      <c r="AE10" s="30" t="n">
+        <f aca="false">D10*IF(MAX(0,MIN(C10,Funnel!$B$19)-B10+1)&gt;0,MAX(0,MIN(C10,Funnel!$B$19)-MAX(B10,Assumptions!$D$7+Assumptions!$D$179)+1)/MAX(0,MIN(C10,Funnel!$B$19)-B10+1),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -17310,14 +17537,14 @@
       </c>
       <c r="F11" s="30" t="n">
         <f aca="false">IF(A11-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($D$4:$D$14,A11-ROUNDUP(Funnel!$B$15/7,0)),0)</f>
-        <v>0.215</v>
+        <v>0.195</v>
       </c>
       <c r="G11" s="30" t="n">
         <f aca="false">IF(A11-ROUNDUP(Funnel!$B$16/7,0)&gt;=1,INDEX($E$4:$E$14,A11-ROUNDUP(Funnel!$B$16/7,0)),0)</f>
-        <v>0.233965672990063</v>
+        <v>0.210955504343202</v>
       </c>
       <c r="H11" s="41" t="n">
-        <f aca="false">$F$19*D11+$F$20*E11+$F$31*Y11</f>
+        <f aca="false">($F$19-$L$19-$L$23)*D11+$L$19*AB11+$L$23*AC11+$F$20*E11+$F$31*Y11</f>
         <v>0</v>
       </c>
       <c r="I11" s="41" t="n">
@@ -17326,7 +17553,7 @@
       </c>
       <c r="J11" s="41" t="n">
         <f aca="false">$F$22*F11+$F$23*G11</f>
-        <v>2381.23457652439</v>
+        <v>2158.34329973187</v>
       </c>
       <c r="K11" s="41" t="n">
         <f aca="false">IF(A11=1,Budget!$C$6,0)</f>
@@ -17338,18 +17565,18 @@
       </c>
       <c r="M11" s="41" t="n">
         <f aca="false">SUM(H11:L11)</f>
-        <v>2381.23457652439</v>
+        <v>2158.34329973187</v>
       </c>
       <c r="N11" s="41" t="n">
         <f aca="false">SUM($M$4:M11)</f>
-        <v>101966.058810447</v>
+        <v>101951.059523176</v>
       </c>
       <c r="O11" s="29" t="n">
-        <f aca="false">(Funnel!$M$5+Funnel!$M$6+Funnel!$M$7-$F$27-$F$34)*D11+(Funnel!$M$8-$F$28-$F$35)*E11+($F$27+$F$28)*X11+($F$34+$F$35)*Y11</f>
+        <f aca="false">(Funnel!$M$5+Funnel!$M$6+Funnel!$M$7-$F$27-$F$34-$L$20-$L$24)*D11+$L$20*AB11+$L$24*AC11+(Funnel!$M$8-$F$28-$F$35)*E11+($F$27+$F$28)*X11+($F$34+$F$35)*Y11</f>
         <v>0</v>
       </c>
       <c r="P11" s="29" t="n">
-        <f aca="false">(Funnel!$O$5+Funnel!$O$6+Funnel!$O$7-$F$25-$F$32)*D11+(Funnel!$O$8-$F$26-$F$33)*E11+($F$25+$F$26)*X11+($F$32+$F$33)*Y11</f>
+        <f aca="false">(Funnel!$O$5+Funnel!$O$6+Funnel!$O$7-$F$25-$F$32-$L$21-$L$25)*D11+$L$21*AB11+$L$25*AC11+(Funnel!$O$8-$F$26-$F$33)*E11+($F$25+$F$26)*X11+($F$32+$F$33)*Y11</f>
         <v>0</v>
       </c>
       <c r="Q11" s="29" t="n">
@@ -17365,20 +17592,20 @@
         <v/>
       </c>
       <c r="T11" s="32" t="n">
-        <f aca="false">$F$38*(F11*(Budget!$G$21+Budget!$G$22+Budget!$G$23-$F$29-$F$36)+IF(A11-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($X$4:$X$14,A11-ROUNDUP(Funnel!$B$15/7,0))*$F$29+INDEX($Y$4:$Y$14,A11-ROUNDUP(Funnel!$B$15/7,0))*$F$36,0))</f>
-        <v>17.8542840531334</v>
+        <f aca="false">$F$38*(F11*(Budget!$G$21+Budget!$G$22+Budget!$G$23-$F$29-$F$36-$L$22-$L$26)+IF(A11-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($X$4:$X$14,A11-ROUNDUP(Funnel!$B$15/7,0))*$F$29+INDEX($Y$4:$Y$14,A11-ROUNDUP(Funnel!$B$15/7,0))*$F$36+INDEX($AB$4:$AB$14,A11-ROUNDUP(Funnel!$B$15/7,0))*$L$22+INDEX($AC$4:$AC$14,A11-ROUNDUP(Funnel!$B$15/7,0))*$L$26,0))</f>
+        <v>18.0704571328538</v>
       </c>
       <c r="U11" s="32" t="n">
         <f aca="false">$F$38*(G11*(Budget!$G$24-$F$30-$F$37)+IF(A11-ROUNDUP(Funnel!$B$16/7,0)&gt;=1,INDEX($X$4:$X$14,A11-ROUNDUP(Funnel!$B$16/7,0))*$F$30+INDEX($Y$4:$Y$14,A11-ROUNDUP(Funnel!$B$16/7,0))*$F$37,0))</f>
-        <v>2.03539726267266</v>
+        <v>1.83521903276862</v>
       </c>
       <c r="V11" s="32" t="n">
         <f aca="false">T11+U11</f>
-        <v>19.889681315806</v>
+        <v>19.9056761656224</v>
       </c>
       <c r="W11" s="32" t="n">
         <f aca="false">SUM($V$4:V11)</f>
-        <v>97.5859973612742</v>
+        <v>97.1972075354466</v>
       </c>
       <c r="X11" s="30" t="n">
         <f aca="false">IF(A11=1,Assumptions!$D$50,IF(A11=2,1-Assumptions!$D$50,0))</f>
@@ -17394,6 +17621,22 @@
       </c>
       <c r="AA11" s="30" t="n">
         <f aca="false">D11*IF(MAX(0,MIN(C11,Funnel!$B$19)-B11+1)&gt;0,MAX(0,MIN(C11,Funnel!$B$20)-B11+1)/MAX(0,MIN(C11,Funnel!$B$19)-B11+1),0)</f>
+        <v>0</v>
+      </c>
+      <c r="AB11" s="30" t="n">
+        <f aca="false">IF(SUM($AD$4:$AD$14)&gt;0,AD11/SUM($AD$4:$AD$14),0)</f>
+        <v>0</v>
+      </c>
+      <c r="AC11" s="30" t="n">
+        <f aca="false">IF(SUM($AE$4:$AE$14)&gt;0,AE11/SUM($AE$4:$AE$14),0)</f>
+        <v>0</v>
+      </c>
+      <c r="AD11" s="30" t="n">
+        <f aca="false">D11*IF(MAX(0,MIN(C11,Funnel!$B$19)-B11+1)&gt;0,MAX(0,MIN(C11,Funnel!$B$19)-MAX(B11,Assumptions!$D$7+Assumptions!$D$178)+1)/MAX(0,MIN(C11,Funnel!$B$19)-B11+1),0)</f>
+        <v>0</v>
+      </c>
+      <c r="AE11" s="30" t="n">
+        <f aca="false">D11*IF(MAX(0,MIN(C11,Funnel!$B$19)-B11+1)&gt;0,MAX(0,MIN(C11,Funnel!$B$19)-MAX(B11,Assumptions!$D$7+Assumptions!$D$179)+1)/MAX(0,MIN(C11,Funnel!$B$19)-B11+1),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -17419,14 +17662,14 @@
       </c>
       <c r="F12" s="30" t="n">
         <f aca="false">IF(A12-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($D$4:$D$14,A12-ROUNDUP(Funnel!$B$15/7,0)),0)</f>
-        <v>0.025</v>
+        <v>0.027</v>
       </c>
       <c r="G12" s="30" t="n">
         <f aca="false">IF(A12-ROUNDUP(Funnel!$B$16/7,0)&gt;=1,INDEX($E$4:$E$14,A12-ROUNDUP(Funnel!$B$16/7,0)),0)</f>
-        <v>0.038843721770551</v>
+        <v>0.0345683389469952</v>
       </c>
       <c r="H12" s="41" t="n">
-        <f aca="false">$F$19*D12+$F$20*E12+$F$31*Y12</f>
+        <f aca="false">($F$19-$L$19-$L$23)*D12+$L$19*AB12+$L$23*AC12+$F$20*E12+$F$31*Y12</f>
         <v>0</v>
       </c>
       <c r="I12" s="41" t="n">
@@ -17435,7 +17678,7 @@
       </c>
       <c r="J12" s="41" t="n">
         <f aca="false">$F$22*F12+$F$23*G12</f>
-        <v>289.788745426829</v>
+        <v>304.78803269766</v>
       </c>
       <c r="K12" s="41" t="n">
         <f aca="false">IF(A12=1,Budget!$C$6,0)</f>
@@ -17447,18 +17690,18 @@
       </c>
       <c r="M12" s="41" t="n">
         <f aca="false">SUM(H12:L12)</f>
-        <v>289.788745426829</v>
+        <v>304.78803269766</v>
       </c>
       <c r="N12" s="41" t="n">
         <f aca="false">SUM($M$4:M12)</f>
         <v>102255.847555873</v>
       </c>
       <c r="O12" s="29" t="n">
-        <f aca="false">(Funnel!$M$5+Funnel!$M$6+Funnel!$M$7-$F$27-$F$34)*D12+(Funnel!$M$8-$F$28-$F$35)*E12+($F$27+$F$28)*X12+($F$34+$F$35)*Y12</f>
+        <f aca="false">(Funnel!$M$5+Funnel!$M$6+Funnel!$M$7-$F$27-$F$34-$L$20-$L$24)*D12+$L$20*AB12+$L$24*AC12+(Funnel!$M$8-$F$28-$F$35)*E12+($F$27+$F$28)*X12+($F$34+$F$35)*Y12</f>
         <v>0</v>
       </c>
       <c r="P12" s="29" t="n">
-        <f aca="false">(Funnel!$O$5+Funnel!$O$6+Funnel!$O$7-$F$25-$F$32)*D12+(Funnel!$O$8-$F$26-$F$33)*E12+($F$25+$F$26)*X12+($F$32+$F$33)*Y12</f>
+        <f aca="false">(Funnel!$O$5+Funnel!$O$6+Funnel!$O$7-$F$25-$F$32-$L$21-$L$25)*D12+$L$21*AB12+$L$25*AC12+(Funnel!$O$8-$F$26-$F$33)*E12+($F$25+$F$26)*X12+($F$32+$F$33)*Y12</f>
         <v>0</v>
       </c>
       <c r="Q12" s="29" t="n">
@@ -17474,16 +17717,16 @@
         <v/>
       </c>
       <c r="T12" s="32" t="n">
-        <f aca="false">$F$38*(F12*(Budget!$G$21+Budget!$G$22+Budget!$G$23-$F$29-$F$36)+IF(A12-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($X$4:$X$14,A12-ROUNDUP(Funnel!$B$15/7,0))*$F$29+INDEX($Y$4:$Y$14,A12-ROUNDUP(Funnel!$B$15/7,0))*$F$36,0))</f>
-        <v>2.07607954106202</v>
+        <f aca="false">$F$38*(F12*(Budget!$G$21+Budget!$G$22+Budget!$G$23-$F$29-$F$36-$L$22-$L$26)+IF(A12-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($X$4:$X$14,A12-ROUNDUP(Funnel!$B$15/7,0))*$F$29+INDEX($Y$4:$Y$14,A12-ROUNDUP(Funnel!$B$15/7,0))*$F$36+INDEX($AB$4:$AB$14,A12-ROUNDUP(Funnel!$B$15/7,0))*$L$22+INDEX($AC$4:$AC$14,A12-ROUNDUP(Funnel!$B$15/7,0))*$L$26,0))</f>
+        <v>2.50206329531822</v>
       </c>
       <c r="U12" s="32" t="n">
         <f aca="false">$F$38*(G12*(Budget!$G$24-$F$30-$F$37)+IF(A12-ROUNDUP(Funnel!$B$16/7,0)&gt;=1,INDEX($X$4:$X$14,A12-ROUNDUP(Funnel!$B$16/7,0))*$F$30+INDEX($Y$4:$Y$14,A12-ROUNDUP(Funnel!$B$16/7,0))*$F$37,0))</f>
-        <v>0.3379230976638</v>
+        <v>0.300729169235193</v>
       </c>
       <c r="V12" s="32" t="n">
         <f aca="false">T12+U12</f>
-        <v>2.41400263872582</v>
+        <v>2.80279246455341</v>
       </c>
       <c r="W12" s="32" t="n">
         <f aca="false">SUM($V$4:V12)</f>
@@ -17505,6 +17748,22 @@
         <f aca="false">D12*IF(MAX(0,MIN(C12,Funnel!$B$19)-B12+1)&gt;0,MAX(0,MIN(C12,Funnel!$B$20)-B12+1)/MAX(0,MIN(C12,Funnel!$B$19)-B12+1),0)</f>
         <v>0</v>
       </c>
+      <c r="AB12" s="30" t="n">
+        <f aca="false">IF(SUM($AD$4:$AD$14)&gt;0,AD12/SUM($AD$4:$AD$14),0)</f>
+        <v>0</v>
+      </c>
+      <c r="AC12" s="30" t="n">
+        <f aca="false">IF(SUM($AE$4:$AE$14)&gt;0,AE12/SUM($AE$4:$AE$14),0)</f>
+        <v>0</v>
+      </c>
+      <c r="AD12" s="30" t="n">
+        <f aca="false">D12*IF(MAX(0,MIN(C12,Funnel!$B$19)-B12+1)&gt;0,MAX(0,MIN(C12,Funnel!$B$19)-MAX(B12,Assumptions!$D$7+Assumptions!$D$178)+1)/MAX(0,MIN(C12,Funnel!$B$19)-B12+1),0)</f>
+        <v>0</v>
+      </c>
+      <c r="AE12" s="30" t="n">
+        <f aca="false">D12*IF(MAX(0,MIN(C12,Funnel!$B$19)-B12+1)&gt;0,MAX(0,MIN(C12,Funnel!$B$19)-MAX(B12,Assumptions!$D$7+Assumptions!$D$179)+1)/MAX(0,MIN(C12,Funnel!$B$19)-B12+1),0)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="29" t="n">
@@ -17535,7 +17794,7 @@
         <v>0</v>
       </c>
       <c r="H13" s="41" t="n">
-        <f aca="false">$F$19*D13+$F$20*E13+$F$31*Y13</f>
+        <f aca="false">($F$19-$L$19-$L$23)*D13+$L$19*AB13+$L$23*AC13+$F$20*E13+$F$31*Y13</f>
         <v>0</v>
       </c>
       <c r="I13" s="41" t="n">
@@ -17563,11 +17822,11 @@
         <v>102255.847555873</v>
       </c>
       <c r="O13" s="29" t="n">
-        <f aca="false">(Funnel!$M$5+Funnel!$M$6+Funnel!$M$7-$F$27-$F$34)*D13+(Funnel!$M$8-$F$28-$F$35)*E13+($F$27+$F$28)*X13+($F$34+$F$35)*Y13</f>
+        <f aca="false">(Funnel!$M$5+Funnel!$M$6+Funnel!$M$7-$F$27-$F$34-$L$20-$L$24)*D13+$L$20*AB13+$L$24*AC13+(Funnel!$M$8-$F$28-$F$35)*E13+($F$27+$F$28)*X13+($F$34+$F$35)*Y13</f>
         <v>0</v>
       </c>
       <c r="P13" s="29" t="n">
-        <f aca="false">(Funnel!$O$5+Funnel!$O$6+Funnel!$O$7-$F$25-$F$32)*D13+(Funnel!$O$8-$F$26-$F$33)*E13+($F$25+$F$26)*X13+($F$32+$F$33)*Y13</f>
+        <f aca="false">(Funnel!$O$5+Funnel!$O$6+Funnel!$O$7-$F$25-$F$32-$L$21-$L$25)*D13+$L$21*AB13+$L$25*AC13+(Funnel!$O$8-$F$26-$F$33)*E13+($F$25+$F$26)*X13+($F$32+$F$33)*Y13</f>
         <v>0</v>
       </c>
       <c r="Q13" s="29" t="n">
@@ -17583,7 +17842,7 @@
         <v/>
       </c>
       <c r="T13" s="32" t="n">
-        <f aca="false">$F$38*(F13*(Budget!$G$21+Budget!$G$22+Budget!$G$23-$F$29-$F$36)+IF(A13-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($X$4:$X$14,A13-ROUNDUP(Funnel!$B$15/7,0))*$F$29+INDEX($Y$4:$Y$14,A13-ROUNDUP(Funnel!$B$15/7,0))*$F$36,0))</f>
+        <f aca="false">$F$38*(F13*(Budget!$G$21+Budget!$G$22+Budget!$G$23-$F$29-$F$36-$L$22-$L$26)+IF(A13-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($X$4:$X$14,A13-ROUNDUP(Funnel!$B$15/7,0))*$F$29+INDEX($Y$4:$Y$14,A13-ROUNDUP(Funnel!$B$15/7,0))*$F$36+INDEX($AB$4:$AB$14,A13-ROUNDUP(Funnel!$B$15/7,0))*$L$22+INDEX($AC$4:$AC$14,A13-ROUNDUP(Funnel!$B$15/7,0))*$L$26,0))</f>
         <v>0</v>
       </c>
       <c r="U13" s="32" t="n">
@@ -17614,6 +17873,22 @@
         <f aca="false">D13*IF(MAX(0,MIN(C13,Funnel!$B$19)-B13+1)&gt;0,MAX(0,MIN(C13,Funnel!$B$20)-B13+1)/MAX(0,MIN(C13,Funnel!$B$19)-B13+1),0)</f>
         <v>0</v>
       </c>
+      <c r="AB13" s="30" t="n">
+        <f aca="false">IF(SUM($AD$4:$AD$14)&gt;0,AD13/SUM($AD$4:$AD$14),0)</f>
+        <v>0</v>
+      </c>
+      <c r="AC13" s="30" t="n">
+        <f aca="false">IF(SUM($AE$4:$AE$14)&gt;0,AE13/SUM($AE$4:$AE$14),0)</f>
+        <v>0</v>
+      </c>
+      <c r="AD13" s="30" t="n">
+        <f aca="false">D13*IF(MAX(0,MIN(C13,Funnel!$B$19)-B13+1)&gt;0,MAX(0,MIN(C13,Funnel!$B$19)-MAX(B13,Assumptions!$D$7+Assumptions!$D$178)+1)/MAX(0,MIN(C13,Funnel!$B$19)-B13+1),0)</f>
+        <v>0</v>
+      </c>
+      <c r="AE13" s="30" t="n">
+        <f aca="false">D13*IF(MAX(0,MIN(C13,Funnel!$B$19)-B13+1)&gt;0,MAX(0,MIN(C13,Funnel!$B$19)-MAX(B13,Assumptions!$D$7+Assumptions!$D$179)+1)/MAX(0,MIN(C13,Funnel!$B$19)-B13+1),0)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="29" t="n">
@@ -17644,7 +17919,7 @@
         <v>0</v>
       </c>
       <c r="H14" s="41" t="n">
-        <f aca="false">$F$19*D14+$F$20*E14+$F$31*Y14</f>
+        <f aca="false">($F$19-$L$19-$L$23)*D14+$L$19*AB14+$L$23*AC14+$F$20*E14+$F$31*Y14</f>
         <v>0</v>
       </c>
       <c r="I14" s="41" t="n">
@@ -17672,11 +17947,11 @@
         <v>102255.847555873</v>
       </c>
       <c r="O14" s="29" t="n">
-        <f aca="false">(Funnel!$M$5+Funnel!$M$6+Funnel!$M$7-$F$27-$F$34)*D14+(Funnel!$M$8-$F$28-$F$35)*E14+($F$27+$F$28)*X14+($F$34+$F$35)*Y14</f>
+        <f aca="false">(Funnel!$M$5+Funnel!$M$6+Funnel!$M$7-$F$27-$F$34-$L$20-$L$24)*D14+$L$20*AB14+$L$24*AC14+(Funnel!$M$8-$F$28-$F$35)*E14+($F$27+$F$28)*X14+($F$34+$F$35)*Y14</f>
         <v>0</v>
       </c>
       <c r="P14" s="29" t="n">
-        <f aca="false">(Funnel!$O$5+Funnel!$O$6+Funnel!$O$7-$F$25-$F$32)*D14+(Funnel!$O$8-$F$26-$F$33)*E14+($F$25+$F$26)*X14+($F$32+$F$33)*Y14</f>
+        <f aca="false">(Funnel!$O$5+Funnel!$O$6+Funnel!$O$7-$F$25-$F$32-$L$21-$L$25)*D14+$L$21*AB14+$L$25*AC14+(Funnel!$O$8-$F$26-$F$33)*E14+($F$25+$F$26)*X14+($F$32+$F$33)*Y14</f>
         <v>0</v>
       </c>
       <c r="Q14" s="29" t="n">
@@ -17692,7 +17967,7 @@
         <v/>
       </c>
       <c r="T14" s="32" t="n">
-        <f aca="false">$F$38*(F14*(Budget!$G$21+Budget!$G$22+Budget!$G$23-$F$29-$F$36)+IF(A14-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($X$4:$X$14,A14-ROUNDUP(Funnel!$B$15/7,0))*$F$29+INDEX($Y$4:$Y$14,A14-ROUNDUP(Funnel!$B$15/7,0))*$F$36,0))</f>
+        <f aca="false">$F$38*(F14*(Budget!$G$21+Budget!$G$22+Budget!$G$23-$F$29-$F$36-$L$22-$L$26)+IF(A14-ROUNDUP(Funnel!$B$15/7,0)&gt;=1,INDEX($X$4:$X$14,A14-ROUNDUP(Funnel!$B$15/7,0))*$F$29+INDEX($Y$4:$Y$14,A14-ROUNDUP(Funnel!$B$15/7,0))*$F$36+INDEX($AB$4:$AB$14,A14-ROUNDUP(Funnel!$B$15/7,0))*$L$22+INDEX($AC$4:$AC$14,A14-ROUNDUP(Funnel!$B$15/7,0))*$L$26,0))</f>
         <v>0</v>
       </c>
       <c r="U14" s="32" t="n">
@@ -17723,10 +17998,26 @@
         <f aca="false">D14*IF(MAX(0,MIN(C14,Funnel!$B$19)-B14+1)&gt;0,MAX(0,MIN(C14,Funnel!$B$20)-B14+1)/MAX(0,MIN(C14,Funnel!$B$19)-B14+1),0)</f>
         <v>0</v>
       </c>
+      <c r="AB14" s="30" t="n">
+        <f aca="false">IF(SUM($AD$4:$AD$14)&gt;0,AD14/SUM($AD$4:$AD$14),0)</f>
+        <v>0</v>
+      </c>
+      <c r="AC14" s="30" t="n">
+        <f aca="false">IF(SUM($AE$4:$AE$14)&gt;0,AE14/SUM($AE$4:$AE$14),0)</f>
+        <v>0</v>
+      </c>
+      <c r="AD14" s="30" t="n">
+        <f aca="false">D14*IF(MAX(0,MIN(C14,Funnel!$B$19)-B14+1)&gt;0,MAX(0,MIN(C14,Funnel!$B$19)-MAX(B14,Assumptions!$D$7+Assumptions!$D$178)+1)/MAX(0,MIN(C14,Funnel!$B$19)-B14+1),0)</f>
+        <v>0</v>
+      </c>
+      <c r="AE14" s="30" t="n">
+        <f aca="false">D14*IF(MAX(0,MIN(C14,Funnel!$B$19)-B14+1)&gt;0,MAX(0,MIN(C14,Funnel!$B$19)-MAX(B14,Assumptions!$D$7+Assumptions!$D$179)+1)/MAX(0,MIN(C14,Funnel!$B$19)-B14+1),0)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="28" t="s">
-        <v>447</v>
+        <v>453</v>
       </c>
       <c r="D15" s="51" t="n">
         <f aca="false">SUM(D4:D14)</f>
@@ -17811,7 +18102,7 @@
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="s">
-        <v>698</v>
+        <v>708</v>
       </c>
       <c r="B16" s="9"/>
       <c r="C16" s="9"/>
@@ -17863,84 +18154,143 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="28" t="s">
-        <v>699</v>
+        <v>709</v>
+      </c>
+      <c r="H18" s="28" t="s">
+        <v>710</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="2" t="s">
-        <v>700</v>
+        <v>711</v>
       </c>
       <c r="F19" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot",Channels!$B$5:$B$34,"&lt;&gt;I1b Employee referral sprint (bonus on hire)",Channels!$B$5:$B$34,"&lt;&gt;I1a Talent rediscovery (past applicants in ATS)")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
         <v>62640.1522284802</v>
       </c>
+      <c r="H19" s="2" t="s">
+        <v>712</v>
+      </c>
+      <c r="L19" s="41" t="n">
+        <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,"I2 Handwerk → Industrie (construction electricians)")</f>
+        <v>9912</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="2" t="s">
-        <v>701</v>
+        <v>713</v>
       </c>
       <c r="F20" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot",Channels!$B$5:$B$34,"&lt;&gt;I1b Employee referral sprint (bonus on hire)",Channels!$B$5:$B$34,"&lt;&gt;I1a Talent rediscovery (past applicants in ATS)")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$C$5:$C$34,"Supervisors")</f>
         <v>12178.6678273933</v>
       </c>
+      <c r="H20" s="2" t="s">
+        <v>714</v>
+      </c>
+      <c r="L20" s="32" t="n">
+        <f aca="false">SUMIFS(Channels!$W$5:$W$34,Channels!$B$5:$B$34,"I2 Handwerk → Industrie (construction electricians)")</f>
+        <v>118</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="2" t="s">
-        <v>702</v>
+        <v>715</v>
       </c>
       <c r="F21" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$E$5:$E$34,"Slot")</f>
         <v>5796</v>
       </c>
+      <c r="H21" s="2" t="s">
+        <v>716</v>
+      </c>
+      <c r="L21" s="32" t="n">
+        <f aca="false">SUMIFS(Channels!$V$5:$V$34,Channels!$B$5:$B$34,"I2 Handwerk → Industrie (construction electricians)")</f>
+        <v>29.5</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="2" t="s">
-        <v>703</v>
+        <v>717</v>
       </c>
       <c r="F22" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,"I1b Employee referral sprint (bonus on hire)",Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
         <v>9869.2425</v>
       </c>
+      <c r="H22" s="2" t="s">
+        <v>718</v>
+      </c>
+      <c r="L22" s="32" t="n">
+        <f aca="false">SUMIFS(Channels!$U$5:$U$34,Channels!$B$5:$B$34,"I2 Handwerk → Industrie (construction electricians)")</f>
+        <v>8.36325</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="2" t="s">
-        <v>704</v>
+        <v>719</v>
       </c>
       <c r="F23" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,"I1b Employee referral sprint (bonus on hire)",Channels!$C$5:$C$34,"Supervisors")</f>
         <v>1108.485</v>
       </c>
+      <c r="H23" s="2" t="s">
+        <v>720</v>
+      </c>
+      <c r="L23" s="41" t="n">
+        <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,"I3 Polish border corridor + PL pre-screener")</f>
+        <v>6493.50649350649</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="2" t="s">
-        <v>705</v>
+        <v>721</v>
       </c>
       <c r="F24" s="41" t="n">
         <f aca="false">SUM(Channels!$Z$5:$Z$34)</f>
         <v>9000</v>
       </c>
+      <c r="H24" s="2" t="s">
+        <v>722</v>
+      </c>
+      <c r="L24" s="32" t="n">
+        <f aca="false">SUMIFS(Channels!$W$5:$W$34,Channels!$B$5:$B$34,"I3 Polish border corridor + PL pre-screener")</f>
+        <v>346.320346320346</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="2" t="s">
-        <v>706</v>
+        <v>723</v>
       </c>
       <c r="F25" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$AF$5:$AF$34,Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
         <v>8.9323002511364</v>
       </c>
+      <c r="H25" s="2" t="s">
+        <v>724</v>
+      </c>
+      <c r="L25" s="32" t="n">
+        <f aca="false">SUMIFS(Channels!$V$5:$V$34,Channels!$B$5:$B$34,"I3 Polish border corridor + PL pre-screener")</f>
+        <v>48.4848484848485</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="2" t="s">
-        <v>707</v>
+        <v>725</v>
       </c>
       <c r="F26" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$AF$5:$AF$34,Channels!$C$5:$C$34,"Supervisors")</f>
         <v>3.25605421987231</v>
       </c>
+      <c r="H26" s="2" t="s">
+        <v>726</v>
+      </c>
+      <c r="L26" s="32" t="n">
+        <f aca="false">SUMIFS(Channels!$U$5:$U$34,Channels!$B$5:$B$34,"I3 Polish border corridor + PL pre-screener")</f>
+        <v>18</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="2" t="s">
-        <v>708</v>
+        <v>727</v>
       </c>
       <c r="F27" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$AE$5:$AE$34,Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
@@ -17949,7 +18299,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="2" t="s">
-        <v>709</v>
+        <v>728</v>
       </c>
       <c r="F28" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$AE$5:$AE$34,Channels!$C$5:$C$34,"Supervisors")</f>
@@ -17958,7 +18308,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="2" t="s">
-        <v>710</v>
+        <v>729</v>
       </c>
       <c r="F29" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$AG$5:$AG$34,Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
@@ -17967,7 +18317,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="2" t="s">
-        <v>711</v>
+        <v>730</v>
       </c>
       <c r="F30" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$AG$5:$AG$34,Channels!$C$5:$C$34,"Supervisors")</f>
@@ -17976,7 +18326,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="2" t="s">
-        <v>712</v>
+        <v>731</v>
       </c>
       <c r="F31" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)")</f>
@@ -17985,7 +18335,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="2" t="s">
-        <v>713</v>
+        <v>732</v>
       </c>
       <c r="F32" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$V$5:$V$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)",Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
@@ -17994,7 +18344,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="2" t="s">
-        <v>714</v>
+        <v>733</v>
       </c>
       <c r="F33" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$V$5:$V$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)",Channels!$C$5:$C$34,"Supervisors")</f>
@@ -18003,7 +18353,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="2" t="s">
-        <v>715</v>
+        <v>734</v>
       </c>
       <c r="F34" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$W$5:$W$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)",Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
@@ -18012,7 +18362,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="2" t="s">
-        <v>716</v>
+        <v>735</v>
       </c>
       <c r="F35" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$W$5:$W$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)",Channels!$C$5:$C$34,"Supervisors")</f>
@@ -18021,7 +18371,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="2" t="s">
-        <v>717</v>
+        <v>736</v>
       </c>
       <c r="F36" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$U$5:$U$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)",Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
@@ -18030,7 +18380,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="2" t="s">
-        <v>718</v>
+        <v>737</v>
       </c>
       <c r="F37" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$U$5:$U$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)",Channels!$C$5:$C$34,"Supervisors")</f>
@@ -18039,7 +18389,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="2" t="s">
-        <v>719</v>
+        <v>738</v>
       </c>
       <c r="F38" s="30" t="n">
         <f aca="false">IF(Funnel!B23&gt;0,MIN(1,Funnel!B22/Funnel!B23),1)</f>
@@ -18048,7 +18398,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="28" t="s">
-        <v>720</v>
+        <v>739</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18057,40 +18407,40 @@
         <v>315</v>
       </c>
       <c r="C43" s="12" t="s">
-        <v>721</v>
+        <v>740</v>
       </c>
       <c r="D43" s="12" t="s">
-        <v>722</v>
+        <v>741</v>
       </c>
       <c r="E43" s="12" t="s">
-        <v>723</v>
+        <v>742</v>
       </c>
       <c r="F43" s="12" t="s">
-        <v>724</v>
+        <v>743</v>
       </c>
       <c r="G43" s="12" t="s">
-        <v>725</v>
+        <v>744</v>
       </c>
       <c r="H43" s="12" t="s">
-        <v>726</v>
+        <v>745</v>
       </c>
       <c r="I43" s="12" t="s">
-        <v>727</v>
+        <v>746</v>
       </c>
       <c r="J43" s="12" t="s">
-        <v>728</v>
+        <v>747</v>
       </c>
       <c r="K43" s="12" t="s">
-        <v>729</v>
+        <v>748</v>
       </c>
       <c r="L43" s="12" t="s">
-        <v>730</v>
+        <v>749</v>
       </c>
       <c r="M43" s="12" t="s">
-        <v>731</v>
+        <v>750</v>
       </c>
       <c r="N43" s="12" t="s">
-        <v>447</v>
+        <v>453</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18154,27 +18504,27 @@
       </c>
       <c r="C45" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$4+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"Supervisors"))*$E$4+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45)*$X$4+SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$E$5:$E$34,"Slot")+SUMIFS(Channels!$Y$5:$Y$34,Channels!$B$5:$B$34,$B45)</f>
-        <v>9368.64932274326</v>
+        <v>11525.1727439475</v>
       </c>
       <c r="D45" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$5+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"Supervisors"))*$E$5+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45)*$X$5</f>
-        <v>6537.81660719109</v>
+        <v>6080.37224511747</v>
       </c>
       <c r="E45" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$6+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"Supervisors"))*$E$6+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45)*$X$6</f>
-        <v>5881.42751237515</v>
+        <v>5260.61016384666</v>
       </c>
       <c r="F45" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$7+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"Supervisors"))*$E$7+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45)*$X$7</f>
-        <v>6044.80049883001</v>
+        <v>5554.68153946542</v>
       </c>
       <c r="G45" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$8+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"Supervisors"))*$E$8+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45)*$X$8</f>
-        <v>7025.0384175592</v>
+        <v>6371.54647173974</v>
       </c>
       <c r="H45" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$9+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"Supervisors"))*$E$9+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45)*$X$9</f>
-        <v>816.864932274326</v>
+        <v>882.214126856272</v>
       </c>
       <c r="I45" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$10+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45,Channels!$C$5:$C$34,"Supervisors"))*$E$10+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B45)*$X$10</f>
@@ -18262,27 +18612,27 @@
       </c>
       <c r="C47" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$4+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"Supervisors"))*$E$4+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47)*$X$4+SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$E$5:$E$34,"Slot")+SUMIFS(Channels!$Y$5:$Y$34,Channels!$B$5:$B$34,$B47)</f>
-        <v>7840.53942770084</v>
+        <v>9660.58481622726</v>
       </c>
       <c r="D47" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$5+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"Supervisors"))*$E$5+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47)*$X$5</f>
-        <v>5099.51286806649</v>
+        <v>4656.12851558788</v>
       </c>
       <c r="E47" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$6+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"Supervisors"))*$E$6+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47)*$X$6</f>
-        <v>5213.1883879446</v>
+        <v>4616.31061839427</v>
       </c>
       <c r="F47" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$7+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"Supervisors"))*$E$7+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47)*$X$7</f>
-        <v>5357.99917649862</v>
+        <v>4874.36524923618</v>
       </c>
       <c r="G47" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$8+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"Supervisors"))*$E$8+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47)*$X$8</f>
-        <v>3388.47520008336</v>
+        <v>3065.20576396032</v>
       </c>
       <c r="H47" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$9+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"Supervisors"))*$E$9+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47)*$X$9</f>
-        <v>339.001211100016</v>
+        <v>366.121307988017</v>
       </c>
       <c r="I47" s="41" t="n">
         <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$10+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47,Channels!$C$5:$C$34,"Supervisors"))*$E$10+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B47)*$X$10</f>
@@ -18490,27 +18840,27 @@
       </c>
       <c r="F51" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B51,Channels!$C$5:$C$34,"&lt;&gt;Supervisors")*$F$7+SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B51,Channels!$C$5:$C$34,"Supervisors")*$G$7</f>
-        <v>2467.310625</v>
+        <v>3118.68063</v>
       </c>
       <c r="G51" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B51,Channels!$C$5:$C$34,"&lt;&gt;Supervisors")*$F$8+SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B51,Channels!$C$5:$C$34,"Supervisors")*$G$8</f>
-        <v>1781.50967469512</v>
+        <v>1727.53994317807</v>
       </c>
       <c r="H51" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B51,Channels!$C$5:$C$34,"&lt;&gt;Supervisors")*$F$9+SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B51,Channels!$C$5:$C$34,"Supervisors")*$G$9</f>
-        <v>1979.73596707317</v>
+        <v>1769.14317545515</v>
       </c>
       <c r="I51" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B51,Channels!$C$5:$C$34,"&lt;&gt;Supervisors")*$F$10+SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B51,Channels!$C$5:$C$34,"Supervisors")*$G$10</f>
-        <v>2078.14791128049</v>
+        <v>1899.23241893725</v>
       </c>
       <c r="J51" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B51,Channels!$C$5:$C$34,"&lt;&gt;Supervisors")*$F$11+SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B51,Channels!$C$5:$C$34,"Supervisors")*$G$11</f>
-        <v>2381.23457652439</v>
+        <v>2158.34329973187</v>
       </c>
       <c r="K51" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B51,Channels!$C$5:$C$34,"&lt;&gt;Supervisors")*$F$12+SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B51,Channels!$C$5:$C$34,"Supervisors")*$G$12</f>
-        <v>289.788745426829</v>
+        <v>304.78803269766</v>
       </c>
       <c r="L51" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B51,Channels!$C$5:$C$34,"&lt;&gt;Supervisors")*$F$13+SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B51,Channels!$C$5:$C$34,"Supervisors")*$G$13</f>
@@ -18531,47 +18881,47 @@
         <v>I2 Handwerk → Industrie (construction electricians)</v>
       </c>
       <c r="C52" s="41" t="n">
-        <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$4+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"Supervisors"))*$E$4+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52)*$X$4+SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52,Channels!$E$5:$E$34,"Slot")+SUMIFS(Channels!$Y$5:$Y$34,Channels!$B$5:$B$34,$B52)</f>
-        <v>3678</v>
+        <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52)*$AB$4+SUMIFS(Channels!$Y$5:$Y$34,Channels!$B$5:$B$34,$B52)</f>
+        <v>3270.18638466623</v>
       </c>
       <c r="D52" s="41" t="n">
-        <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$5+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"Supervisors"))*$E$5+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52)*$X$5</f>
-        <v>1437.24</v>
+        <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52)*$AB$5</f>
+        <v>1501.86781229346</v>
       </c>
       <c r="E52" s="41" t="n">
-        <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$6+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"Supervisors"))*$E$6+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52)*$X$6</f>
-        <v>1784.16</v>
+        <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52)*$AB$6</f>
+        <v>1845.80700594845</v>
       </c>
       <c r="F52" s="41" t="n">
-        <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$7+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"Supervisors"))*$E$7+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52)*$X$7</f>
-        <v>1833.72</v>
+        <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52)*$AB$7</f>
+        <v>1948.98876404494</v>
       </c>
       <c r="G52" s="41" t="n">
-        <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$8+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"Supervisors"))*$E$8+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52)*$X$8</f>
-        <v>2131.08</v>
+        <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52)*$AB$8</f>
+        <v>2235.60475875744</v>
       </c>
       <c r="H52" s="41" t="n">
-        <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$9+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"Supervisors"))*$E$9+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52)*$X$9</f>
-        <v>247.8</v>
+        <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52)*$AB$9</f>
+        <v>309.545274289491</v>
       </c>
       <c r="I52" s="41" t="n">
-        <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$10+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"Supervisors"))*$E$10+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52)*$X$10</f>
+        <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52)*$AB$10</f>
         <v>0</v>
       </c>
       <c r="J52" s="41" t="n">
-        <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$11+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"Supervisors"))*$E$11+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52)*$X$11</f>
+        <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52)*$AB$11</f>
         <v>0</v>
       </c>
       <c r="K52" s="41" t="n">
-        <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$12+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"Supervisors"))*$E$12+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52)*$X$12</f>
+        <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52)*$AB$12</f>
         <v>0</v>
       </c>
       <c r="L52" s="41" t="n">
-        <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$13+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"Supervisors"))*$E$13+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52)*$X$13</f>
+        <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52)*$AB$13</f>
         <v>0</v>
       </c>
       <c r="M52" s="41" t="n">
-        <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$14+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52,Channels!$C$5:$C$34,"Supervisors"))*$E$14+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B52)*$X$14</f>
+        <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B52)*$AB$14</f>
         <v>0</v>
       </c>
       <c r="N52" s="42" t="n">
@@ -18585,47 +18935,47 @@
         <v>I3 Polish border corridor + PL pre-screener</v>
       </c>
       <c r="C53" s="41" t="n">
-        <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$4+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"Supervisors"))*$E$4+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53)*$X$4+SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53,Channels!$E$5:$E$34,"Slot")+SUMIFS(Channels!$Y$5:$Y$34,Channels!$B$5:$B$34,$B53)</f>
-        <v>2023.37662337662</v>
+        <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53)*$AC$4+SUMIFS(Channels!$Y$5:$Y$34,Channels!$B$5:$B$34,$B53)</f>
+        <v>400</v>
       </c>
       <c r="D53" s="41" t="n">
-        <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$5+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"Supervisors"))*$E$5+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53)*$X$5</f>
-        <v>941.558441558441</v>
+        <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53)*$AC$5</f>
+        <v>1243.63940153414</v>
       </c>
       <c r="E53" s="41" t="n">
-        <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$6+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"Supervisors"))*$E$6+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53)*$X$6</f>
-        <v>1168.83116883117</v>
+        <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53)*$AC$6</f>
+        <v>1528.442317916</v>
       </c>
       <c r="F53" s="41" t="n">
-        <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$7+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"Supervisors"))*$E$7+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53)*$X$7</f>
-        <v>1201.2987012987</v>
+        <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53)*$AC$7</f>
+        <v>1613.88319283056</v>
       </c>
       <c r="G53" s="41" t="n">
-        <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$8+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"Supervisors"))*$E$8+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53)*$X$8</f>
-        <v>1396.1038961039</v>
+        <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53)*$AC$8</f>
+        <v>1851.21895648211</v>
       </c>
       <c r="H53" s="41" t="n">
-        <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$9+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"Supervisors"))*$E$9+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53)*$X$9</f>
-        <v>162.337662337662</v>
+        <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53)*$AC$9</f>
+        <v>256.322624743677</v>
       </c>
       <c r="I53" s="41" t="n">
-        <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$10+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"Supervisors"))*$E$10+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53)*$X$10</f>
+        <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53)*$AC$10</f>
         <v>0</v>
       </c>
       <c r="J53" s="41" t="n">
-        <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$11+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"Supervisors"))*$E$11+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53)*$X$11</f>
+        <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53)*$AC$11</f>
         <v>0</v>
       </c>
       <c r="K53" s="41" t="n">
-        <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$12+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"Supervisors"))*$E$12+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53)*$X$12</f>
+        <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53)*$AC$12</f>
         <v>0</v>
       </c>
       <c r="L53" s="41" t="n">
-        <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$13+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"Supervisors"))*$E$13+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53)*$X$13</f>
+        <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53)*$AC$13</f>
         <v>0</v>
       </c>
       <c r="M53" s="41" t="n">
-        <f aca="false">(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"&lt;&gt;Supervisors"))*$D$14+(SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53,Channels!$C$5:$C$34,"Supervisors"))*$E$14+SUMIFS(Channels!$Z$5:$Z$34,Channels!$B$5:$B$34,$B53)*$X$14</f>
+        <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,$B53)*$AC$14</f>
         <v>0</v>
       </c>
       <c r="N53" s="42" t="n">
@@ -18635,43 +18985,43 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B54" s="28" t="s">
-        <v>447</v>
+        <v>453</v>
       </c>
       <c r="C54" s="42" t="n">
         <f aca="false">SUM(C44:C53)</f>
-        <v>30544.5453738207</v>
+        <v>32489.923944841</v>
       </c>
       <c r="D54" s="42" t="n">
         <f aca="false">SUM(D44:D53)</f>
-        <v>16734.484916816</v>
+        <v>16200.3649745329</v>
       </c>
       <c r="E54" s="42" t="n">
         <f aca="false">SUM(E44:E53)</f>
-        <v>14054.5700691509</v>
+        <v>13258.1331061054</v>
       </c>
       <c r="F54" s="42" t="n">
         <f aca="false">SUM(F44:F53)</f>
-        <v>16905.1290016273</v>
+        <v>17110.5993755771</v>
       </c>
       <c r="G54" s="42" t="n">
         <f aca="false">SUM(G44:G53)</f>
-        <v>15722.2071884416</v>
+        <v>15251.1158941177</v>
       </c>
       <c r="H54" s="42" t="n">
         <f aca="false">SUM(H44:H53)</f>
-        <v>3545.73977278518</v>
+        <v>3583.34650933261</v>
       </c>
       <c r="I54" s="42" t="n">
         <f aca="false">SUM(I44:I53)</f>
-        <v>2078.14791128049</v>
+        <v>1899.23241893725</v>
       </c>
       <c r="J54" s="42" t="n">
         <f aca="false">SUM(J44:J53)</f>
-        <v>2381.23457652439</v>
+        <v>2158.34329973187</v>
       </c>
       <c r="K54" s="42" t="n">
         <f aca="false">SUM(K44:K53)</f>
-        <v>289.788745426829</v>
+        <v>304.78803269766</v>
       </c>
       <c r="L54" s="42" t="n">
         <f aca="false">SUM(L44:L53)</f>
@@ -18725,12 +19075,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>732</v>
+        <v>751</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>733</v>
+        <v>752</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18744,76 +19094,76 @@
         <v>316</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>734</v>
+        <v>753</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>735</v>
+        <v>754</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>736</v>
+        <v>755</v>
       </c>
       <c r="G4" s="12" t="s">
-        <v>737</v>
+        <v>756</v>
       </c>
       <c r="H4" s="12" t="s">
-        <v>738</v>
+        <v>757</v>
       </c>
       <c r="I4" s="12" t="s">
-        <v>739</v>
+        <v>758</v>
       </c>
       <c r="J4" s="12" t="s">
-        <v>740</v>
+        <v>759</v>
       </c>
       <c r="K4" s="12" t="s">
-        <v>741</v>
+        <v>760</v>
       </c>
       <c r="L4" s="12" t="s">
-        <v>742</v>
+        <v>761</v>
       </c>
       <c r="M4" s="12" t="s">
-        <v>743</v>
+        <v>762</v>
       </c>
       <c r="N4" s="12" t="s">
-        <v>744</v>
+        <v>763</v>
       </c>
       <c r="O4" s="12" t="s">
-        <v>745</v>
+        <v>764</v>
       </c>
       <c r="P4" s="12" t="s">
-        <v>746</v>
+        <v>765</v>
       </c>
       <c r="Q4" s="12" t="s">
-        <v>747</v>
+        <v>766</v>
       </c>
       <c r="R4" s="12" t="s">
-        <v>748</v>
+        <v>767</v>
       </c>
       <c r="S4" s="12" t="s">
-        <v>749</v>
+        <v>768</v>
       </c>
       <c r="T4" s="12" t="s">
-        <v>750</v>
+        <v>769</v>
       </c>
       <c r="U4" s="12" t="s">
-        <v>751</v>
+        <v>770</v>
       </c>
       <c r="V4" s="12" t="s">
-        <v>752</v>
+        <v>771</v>
       </c>
       <c r="W4" s="12" t="s">
-        <v>753</v>
+        <v>772</v>
       </c>
       <c r="X4" s="12" t="s">
-        <v>754</v>
+        <v>773</v>
       </c>
       <c r="Y4" s="12" t="s">
-        <v>755</v>
+        <v>774</v>
       </c>
       <c r="Z4" s="12" t="s">
-        <v>756</v>
+        <v>775</v>
       </c>
       <c r="AA4" s="12" t="s">
-        <v>757</v>
+        <v>776</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21218,7 +21568,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="28" t="s">
-        <v>447</v>
+        <v>453</v>
       </c>
       <c r="G35" s="42" t="n">
         <f aca="false">SUM(G5:G34)</f>
@@ -21279,7 +21629,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="28" t="s">
-        <v>758</v>
+        <v>777</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -21288,46 +21638,46 @@
         <v>316</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>759</v>
+        <v>778</v>
       </c>
       <c r="D39" s="12" t="s">
-        <v>760</v>
+        <v>779</v>
       </c>
       <c r="E39" s="12" t="s">
-        <v>761</v>
+        <v>780</v>
       </c>
       <c r="F39" s="12" t="s">
-        <v>762</v>
+        <v>781</v>
       </c>
       <c r="G39" s="12" t="s">
-        <v>763</v>
+        <v>782</v>
       </c>
       <c r="H39" s="12" t="s">
-        <v>764</v>
+        <v>783</v>
       </c>
       <c r="I39" s="12" t="s">
-        <v>765</v>
+        <v>784</v>
       </c>
       <c r="J39" s="12" t="s">
-        <v>766</v>
+        <v>785</v>
       </c>
       <c r="K39" s="12" t="s">
-        <v>767</v>
+        <v>786</v>
       </c>
       <c r="L39" s="12" t="s">
-        <v>768</v>
+        <v>787</v>
       </c>
       <c r="M39" s="12" t="s">
-        <v>769</v>
+        <v>788</v>
       </c>
       <c r="N39" s="12" t="s">
-        <v>770</v>
+        <v>789</v>
       </c>
       <c r="O39" s="12" t="s">
         <v>47</v>
       </c>
       <c r="P39" s="12" t="s">
-        <v>771</v>
+        <v>790</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21516,7 +21866,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="28" t="s">
-        <v>447</v>
+        <v>453</v>
       </c>
       <c r="C44" s="35" t="n">
         <f aca="false">SUM(C40:C43)</f>
@@ -21557,7 +21907,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="9" t="s">
-        <v>772</v>
+        <v>791</v>
       </c>
       <c r="B46" s="9"/>
       <c r="C46" s="9"/>

</xml_diff>

<commit_message>
Go-live pacing fallback for typed shares that leave no week after launch (edge case)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V2NJtrYy3bzNxqKeiRXJfY
</commit_message>
<xml_diff>
--- a/operation_uptime/Operation_Uptime_Model.xlsx
+++ b/operation_uptime/Operation_Uptime_Model.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1498" uniqueCount="792">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1500" uniqueCount="794">
   <si>
     <t xml:space="preserve">Operation Uptime — model summary (hypothetical Tesla Giga Berlin maintenance hiring)</t>
   </si>
@@ -2151,6 +2151,12 @@
   </si>
   <si>
     <t xml:space="preserve">I3 share before re-scaling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I2 live days (fallback)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I3 live days (fallback)</t>
   </si>
   <si>
     <t xml:space="preserve">Weak channels are cut from Mon 2 Nov; tests are judged by Mon 9 Nov; the reserve is released only from week 3, on the Tracker rules.</t>
@@ -16524,7 +16530,7 @@
     <tabColor rgb="FF8EA9DB"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AE55"/>
+  <dimension ref="A1:AG55"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="1"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
@@ -16639,6 +16645,12 @@
       <c r="AE3" s="49" t="s">
         <v>707</v>
       </c>
+      <c r="AF3" s="49" t="s">
+        <v>708</v>
+      </c>
+      <c r="AG3" s="49" t="s">
+        <v>709</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="29" t="n">
@@ -16749,11 +16761,11 @@
         <v>0.316</v>
       </c>
       <c r="AB4" s="30" t="n">
-        <f aca="false">IF(SUM($AD$4:$AD$14)&gt;0,AD4/SUM($AD$4:$AD$14),0)</f>
+        <f aca="false">IF(SUM($AD$4:$AD$14)&gt;0,AD4/SUM($AD$4:$AD$14),IF(SUM($AF$4:$AF$14)&gt;0,AF4/SUM($AF$4:$AF$14),0))</f>
         <v>0.208856576338401</v>
       </c>
       <c r="AC4" s="30" t="n">
-        <f aca="false">IF(SUM($AE$4:$AE$14)&gt;0,AE4/SUM($AE$4:$AE$14),0)</f>
+        <f aca="false">IF(SUM($AE$4:$AE$14)&gt;0,AE4/SUM($AE$4:$AE$14),IF(SUM($AG$4:$AG$14)&gt;0,AG4/SUM($AG$4:$AG$14),0))</f>
         <v>0</v>
       </c>
       <c r="AD4" s="30" t="n">
@@ -16764,6 +16776,14 @@
         <f aca="false">D4*IF(MAX(0,MIN(C4,Funnel!$B$19)-B4+1)&gt;0,MAX(0,MIN(C4,Funnel!$B$19)-MAX(B4,Assumptions!$D$7+Assumptions!$D$179)+1)/MAX(0,MIN(C4,Funnel!$B$19)-B4+1),0)</f>
         <v>0</v>
       </c>
+      <c r="AF4" s="29" t="n">
+        <f aca="false">MAX(0,MIN(C4,Funnel!$B$19)-MAX(B4,Assumptions!$D$7+Assumptions!$D$178)+1)</f>
+        <v>4</v>
+      </c>
+      <c r="AG4" s="29" t="n">
+        <f aca="false">MAX(0,MIN(C4,Funnel!$B$19)-MAX(B4,Assumptions!$D$7+Assumptions!$D$179)+1)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="29" t="n">
@@ -16874,11 +16894,11 @@
         <v>0.131</v>
       </c>
       <c r="AB5" s="30" t="n">
-        <f aca="false">IF(SUM($AD$4:$AD$14)&gt;0,AD5/SUM($AD$4:$AD$14),0)</f>
+        <f aca="false">IF(SUM($AD$4:$AD$14)&gt;0,AD5/SUM($AD$4:$AD$14),IF(SUM($AF$4:$AF$14)&gt;0,AF5/SUM($AF$4:$AF$14),0))</f>
         <v>0.151520158625248</v>
       </c>
       <c r="AC5" s="30" t="n">
-        <f aca="false">IF(SUM($AE$4:$AE$14)&gt;0,AE5/SUM($AE$4:$AE$14),0)</f>
+        <f aca="false">IF(SUM($AE$4:$AE$14)&gt;0,AE5/SUM($AE$4:$AE$14),IF(SUM($AG$4:$AG$14)&gt;0,AG5/SUM($AG$4:$AG$14),0))</f>
         <v>0.191520467836257</v>
       </c>
       <c r="AD5" s="30" t="n">
@@ -16889,6 +16909,14 @@
         <f aca="false">D5*IF(MAX(0,MIN(C5,Funnel!$B$19)-B5+1)&gt;0,MAX(0,MIN(C5,Funnel!$B$19)-MAX(B5,Assumptions!$D$7+Assumptions!$D$179)+1)/MAX(0,MIN(C5,Funnel!$B$19)-B5+1),0)</f>
         <v>0.131</v>
       </c>
+      <c r="AF5" s="29" t="n">
+        <f aca="false">MAX(0,MIN(C5,Funnel!$B$19)-MAX(B5,Assumptions!$D$7+Assumptions!$D$178)+1)</f>
+        <v>7</v>
+      </c>
+      <c r="AG5" s="29" t="n">
+        <f aca="false">MAX(0,MIN(C5,Funnel!$B$19)-MAX(B5,Assumptions!$D$7+Assumptions!$D$179)+1)</f>
+        <v>7</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="29" t="n">
@@ -16999,11 +17027,11 @@
         <v>0.161</v>
       </c>
       <c r="AB6" s="30" t="n">
-        <f aca="false">IF(SUM($AD$4:$AD$14)&gt;0,AD6/SUM($AD$4:$AD$14),0)</f>
+        <f aca="false">IF(SUM($AD$4:$AD$14)&gt;0,AD6/SUM($AD$4:$AD$14),IF(SUM($AF$4:$AF$14)&gt;0,AF6/SUM($AF$4:$AF$14),0))</f>
         <v>0.186219431592862</v>
       </c>
       <c r="AC6" s="30" t="n">
-        <f aca="false">IF(SUM($AE$4:$AE$14)&gt;0,AE6/SUM($AE$4:$AE$14),0)</f>
+        <f aca="false">IF(SUM($AE$4:$AE$14)&gt;0,AE6/SUM($AE$4:$AE$14),IF(SUM($AG$4:$AG$14)&gt;0,AG6/SUM($AG$4:$AG$14),0))</f>
         <v>0.235380116959064</v>
       </c>
       <c r="AD6" s="30" t="n">
@@ -17014,6 +17042,14 @@
         <f aca="false">D6*IF(MAX(0,MIN(C6,Funnel!$B$19)-B6+1)&gt;0,MAX(0,MIN(C6,Funnel!$B$19)-MAX(B6,Assumptions!$D$7+Assumptions!$D$179)+1)/MAX(0,MIN(C6,Funnel!$B$19)-B6+1),0)</f>
         <v>0.161</v>
       </c>
+      <c r="AF6" s="29" t="n">
+        <f aca="false">MAX(0,MIN(C6,Funnel!$B$19)-MAX(B6,Assumptions!$D$7+Assumptions!$D$178)+1)</f>
+        <v>7</v>
+      </c>
+      <c r="AG6" s="29" t="n">
+        <f aca="false">MAX(0,MIN(C6,Funnel!$B$19)-MAX(B6,Assumptions!$D$7+Assumptions!$D$179)+1)</f>
+        <v>7</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="29" t="n">
@@ -17124,11 +17160,11 @@
         <v>0.17</v>
       </c>
       <c r="AB7" s="30" t="n">
-        <f aca="false">IF(SUM($AD$4:$AD$14)&gt;0,AD7/SUM($AD$4:$AD$14),0)</f>
+        <f aca="false">IF(SUM($AD$4:$AD$14)&gt;0,AD7/SUM($AD$4:$AD$14),IF(SUM($AF$4:$AF$14)&gt;0,AF7/SUM($AF$4:$AF$14),0))</f>
         <v>0.196629213483146</v>
       </c>
       <c r="AC7" s="30" t="n">
-        <f aca="false">IF(SUM($AE$4:$AE$14)&gt;0,AE7/SUM($AE$4:$AE$14),0)</f>
+        <f aca="false">IF(SUM($AE$4:$AE$14)&gt;0,AE7/SUM($AE$4:$AE$14),IF(SUM($AG$4:$AG$14)&gt;0,AG7/SUM($AG$4:$AG$14),0))</f>
         <v>0.248538011695906</v>
       </c>
       <c r="AD7" s="30" t="n">
@@ -17139,6 +17175,14 @@
         <f aca="false">D7*IF(MAX(0,MIN(C7,Funnel!$B$19)-B7+1)&gt;0,MAX(0,MIN(C7,Funnel!$B$19)-MAX(B7,Assumptions!$D$7+Assumptions!$D$179)+1)/MAX(0,MIN(C7,Funnel!$B$19)-B7+1),0)</f>
         <v>0.17</v>
       </c>
+      <c r="AF7" s="29" t="n">
+        <f aca="false">MAX(0,MIN(C7,Funnel!$B$19)-MAX(B7,Assumptions!$D$7+Assumptions!$D$178)+1)</f>
+        <v>7</v>
+      </c>
+      <c r="AG7" s="29" t="n">
+        <f aca="false">MAX(0,MIN(C7,Funnel!$B$19)-MAX(B7,Assumptions!$D$7+Assumptions!$D$179)+1)</f>
+        <v>7</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="29" t="n">
@@ -17249,11 +17293,11 @@
         <v>0.0278571428571429</v>
       </c>
       <c r="AB8" s="30" t="n">
-        <f aca="false">IF(SUM($AD$4:$AD$14)&gt;0,AD8/SUM($AD$4:$AD$14),0)</f>
+        <f aca="false">IF(SUM($AD$4:$AD$14)&gt;0,AD8/SUM($AD$4:$AD$14),IF(SUM($AF$4:$AF$14)&gt;0,AF8/SUM($AF$4:$AF$14),0))</f>
         <v>0.225545274289491</v>
       </c>
       <c r="AC8" s="30" t="n">
-        <f aca="false">IF(SUM($AE$4:$AE$14)&gt;0,AE8/SUM($AE$4:$AE$14),0)</f>
+        <f aca="false">IF(SUM($AE$4:$AE$14)&gt;0,AE8/SUM($AE$4:$AE$14),IF(SUM($AG$4:$AG$14)&gt;0,AG8/SUM($AG$4:$AG$14),0))</f>
         <v>0.285087719298246</v>
       </c>
       <c r="AD8" s="30" t="n">
@@ -17264,6 +17308,14 @@
         <f aca="false">D8*IF(MAX(0,MIN(C8,Funnel!$B$19)-B8+1)&gt;0,MAX(0,MIN(C8,Funnel!$B$19)-MAX(B8,Assumptions!$D$7+Assumptions!$D$179)+1)/MAX(0,MIN(C8,Funnel!$B$19)-B8+1),0)</f>
         <v>0.195</v>
       </c>
+      <c r="AF8" s="29" t="n">
+        <f aca="false">MAX(0,MIN(C8,Funnel!$B$19)-MAX(B8,Assumptions!$D$7+Assumptions!$D$178)+1)</f>
+        <v>7</v>
+      </c>
+      <c r="AG8" s="29" t="n">
+        <f aca="false">MAX(0,MIN(C8,Funnel!$B$19)-MAX(B8,Assumptions!$D$7+Assumptions!$D$179)+1)</f>
+        <v>7</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="29" t="n">
@@ -17374,11 +17426,11 @@
         <v>0</v>
       </c>
       <c r="AB9" s="30" t="n">
-        <f aca="false">IF(SUM($AD$4:$AD$14)&gt;0,AD9/SUM($AD$4:$AD$14),0)</f>
+        <f aca="false">IF(SUM($AD$4:$AD$14)&gt;0,AD9/SUM($AD$4:$AD$14),IF(SUM($AF$4:$AF$14)&gt;0,AF9/SUM($AF$4:$AF$14),0))</f>
         <v>0.0312293456708526</v>
       </c>
       <c r="AC9" s="30" t="n">
-        <f aca="false">IF(SUM($AE$4:$AE$14)&gt;0,AE9/SUM($AE$4:$AE$14),0)</f>
+        <f aca="false">IF(SUM($AE$4:$AE$14)&gt;0,AE9/SUM($AE$4:$AE$14),IF(SUM($AG$4:$AG$14)&gt;0,AG9/SUM($AG$4:$AG$14),0))</f>
         <v>0.0394736842105263</v>
       </c>
       <c r="AD9" s="30" t="n">
@@ -17389,6 +17441,14 @@
         <f aca="false">D9*IF(MAX(0,MIN(C9,Funnel!$B$19)-B9+1)&gt;0,MAX(0,MIN(C9,Funnel!$B$19)-MAX(B9,Assumptions!$D$7+Assumptions!$D$179)+1)/MAX(0,MIN(C9,Funnel!$B$19)-B9+1),0)</f>
         <v>0.027</v>
       </c>
+      <c r="AF9" s="29" t="n">
+        <f aca="false">MAX(0,MIN(C9,Funnel!$B$19)-MAX(B9,Assumptions!$D$7+Assumptions!$D$178)+1)</f>
+        <v>1</v>
+      </c>
+      <c r="AG9" s="29" t="n">
+        <f aca="false">MAX(0,MIN(C9,Funnel!$B$19)-MAX(B9,Assumptions!$D$7+Assumptions!$D$179)+1)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="29" t="n">
@@ -17499,11 +17559,11 @@
         <v>0</v>
       </c>
       <c r="AB10" s="30" t="n">
-        <f aca="false">IF(SUM($AD$4:$AD$14)&gt;0,AD10/SUM($AD$4:$AD$14),0)</f>
+        <f aca="false">IF(SUM($AD$4:$AD$14)&gt;0,AD10/SUM($AD$4:$AD$14),IF(SUM($AF$4:$AF$14)&gt;0,AF10/SUM($AF$4:$AF$14),0))</f>
         <v>0</v>
       </c>
       <c r="AC10" s="30" t="n">
-        <f aca="false">IF(SUM($AE$4:$AE$14)&gt;0,AE10/SUM($AE$4:$AE$14),0)</f>
+        <f aca="false">IF(SUM($AE$4:$AE$14)&gt;0,AE10/SUM($AE$4:$AE$14),IF(SUM($AG$4:$AG$14)&gt;0,AG10/SUM($AG$4:$AG$14),0))</f>
         <v>0</v>
       </c>
       <c r="AD10" s="30" t="n">
@@ -17512,6 +17572,14 @@
       </c>
       <c r="AE10" s="30" t="n">
         <f aca="false">D10*IF(MAX(0,MIN(C10,Funnel!$B$19)-B10+1)&gt;0,MAX(0,MIN(C10,Funnel!$B$19)-MAX(B10,Assumptions!$D$7+Assumptions!$D$179)+1)/MAX(0,MIN(C10,Funnel!$B$19)-B10+1),0)</f>
+        <v>0</v>
+      </c>
+      <c r="AF10" s="29" t="n">
+        <f aca="false">MAX(0,MIN(C10,Funnel!$B$19)-MAX(B10,Assumptions!$D$7+Assumptions!$D$178)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="AG10" s="29" t="n">
+        <f aca="false">MAX(0,MIN(C10,Funnel!$B$19)-MAX(B10,Assumptions!$D$7+Assumptions!$D$179)+1)</f>
         <v>0</v>
       </c>
     </row>
@@ -17624,11 +17692,11 @@
         <v>0</v>
       </c>
       <c r="AB11" s="30" t="n">
-        <f aca="false">IF(SUM($AD$4:$AD$14)&gt;0,AD11/SUM($AD$4:$AD$14),0)</f>
+        <f aca="false">IF(SUM($AD$4:$AD$14)&gt;0,AD11/SUM($AD$4:$AD$14),IF(SUM($AF$4:$AF$14)&gt;0,AF11/SUM($AF$4:$AF$14),0))</f>
         <v>0</v>
       </c>
       <c r="AC11" s="30" t="n">
-        <f aca="false">IF(SUM($AE$4:$AE$14)&gt;0,AE11/SUM($AE$4:$AE$14),0)</f>
+        <f aca="false">IF(SUM($AE$4:$AE$14)&gt;0,AE11/SUM($AE$4:$AE$14),IF(SUM($AG$4:$AG$14)&gt;0,AG11/SUM($AG$4:$AG$14),0))</f>
         <v>0</v>
       </c>
       <c r="AD11" s="30" t="n">
@@ -17637,6 +17705,14 @@
       </c>
       <c r="AE11" s="30" t="n">
         <f aca="false">D11*IF(MAX(0,MIN(C11,Funnel!$B$19)-B11+1)&gt;0,MAX(0,MIN(C11,Funnel!$B$19)-MAX(B11,Assumptions!$D$7+Assumptions!$D$179)+1)/MAX(0,MIN(C11,Funnel!$B$19)-B11+1),0)</f>
+        <v>0</v>
+      </c>
+      <c r="AF11" s="29" t="n">
+        <f aca="false">MAX(0,MIN(C11,Funnel!$B$19)-MAX(B11,Assumptions!$D$7+Assumptions!$D$178)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="AG11" s="29" t="n">
+        <f aca="false">MAX(0,MIN(C11,Funnel!$B$19)-MAX(B11,Assumptions!$D$7+Assumptions!$D$179)+1)</f>
         <v>0</v>
       </c>
     </row>
@@ -17749,11 +17825,11 @@
         <v>0</v>
       </c>
       <c r="AB12" s="30" t="n">
-        <f aca="false">IF(SUM($AD$4:$AD$14)&gt;0,AD12/SUM($AD$4:$AD$14),0)</f>
+        <f aca="false">IF(SUM($AD$4:$AD$14)&gt;0,AD12/SUM($AD$4:$AD$14),IF(SUM($AF$4:$AF$14)&gt;0,AF12/SUM($AF$4:$AF$14),0))</f>
         <v>0</v>
       </c>
       <c r="AC12" s="30" t="n">
-        <f aca="false">IF(SUM($AE$4:$AE$14)&gt;0,AE12/SUM($AE$4:$AE$14),0)</f>
+        <f aca="false">IF(SUM($AE$4:$AE$14)&gt;0,AE12/SUM($AE$4:$AE$14),IF(SUM($AG$4:$AG$14)&gt;0,AG12/SUM($AG$4:$AG$14),0))</f>
         <v>0</v>
       </c>
       <c r="AD12" s="30" t="n">
@@ -17762,6 +17838,14 @@
       </c>
       <c r="AE12" s="30" t="n">
         <f aca="false">D12*IF(MAX(0,MIN(C12,Funnel!$B$19)-B12+1)&gt;0,MAX(0,MIN(C12,Funnel!$B$19)-MAX(B12,Assumptions!$D$7+Assumptions!$D$179)+1)/MAX(0,MIN(C12,Funnel!$B$19)-B12+1),0)</f>
+        <v>0</v>
+      </c>
+      <c r="AF12" s="29" t="n">
+        <f aca="false">MAX(0,MIN(C12,Funnel!$B$19)-MAX(B12,Assumptions!$D$7+Assumptions!$D$178)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="AG12" s="29" t="n">
+        <f aca="false">MAX(0,MIN(C12,Funnel!$B$19)-MAX(B12,Assumptions!$D$7+Assumptions!$D$179)+1)</f>
         <v>0</v>
       </c>
     </row>
@@ -17874,11 +17958,11 @@
         <v>0</v>
       </c>
       <c r="AB13" s="30" t="n">
-        <f aca="false">IF(SUM($AD$4:$AD$14)&gt;0,AD13/SUM($AD$4:$AD$14),0)</f>
+        <f aca="false">IF(SUM($AD$4:$AD$14)&gt;0,AD13/SUM($AD$4:$AD$14),IF(SUM($AF$4:$AF$14)&gt;0,AF13/SUM($AF$4:$AF$14),0))</f>
         <v>0</v>
       </c>
       <c r="AC13" s="30" t="n">
-        <f aca="false">IF(SUM($AE$4:$AE$14)&gt;0,AE13/SUM($AE$4:$AE$14),0)</f>
+        <f aca="false">IF(SUM($AE$4:$AE$14)&gt;0,AE13/SUM($AE$4:$AE$14),IF(SUM($AG$4:$AG$14)&gt;0,AG13/SUM($AG$4:$AG$14),0))</f>
         <v>0</v>
       </c>
       <c r="AD13" s="30" t="n">
@@ -17887,6 +17971,14 @@
       </c>
       <c r="AE13" s="30" t="n">
         <f aca="false">D13*IF(MAX(0,MIN(C13,Funnel!$B$19)-B13+1)&gt;0,MAX(0,MIN(C13,Funnel!$B$19)-MAX(B13,Assumptions!$D$7+Assumptions!$D$179)+1)/MAX(0,MIN(C13,Funnel!$B$19)-B13+1),0)</f>
+        <v>0</v>
+      </c>
+      <c r="AF13" s="29" t="n">
+        <f aca="false">MAX(0,MIN(C13,Funnel!$B$19)-MAX(B13,Assumptions!$D$7+Assumptions!$D$178)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="AG13" s="29" t="n">
+        <f aca="false">MAX(0,MIN(C13,Funnel!$B$19)-MAX(B13,Assumptions!$D$7+Assumptions!$D$179)+1)</f>
         <v>0</v>
       </c>
     </row>
@@ -17999,11 +18091,11 @@
         <v>0</v>
       </c>
       <c r="AB14" s="30" t="n">
-        <f aca="false">IF(SUM($AD$4:$AD$14)&gt;0,AD14/SUM($AD$4:$AD$14),0)</f>
+        <f aca="false">IF(SUM($AD$4:$AD$14)&gt;0,AD14/SUM($AD$4:$AD$14),IF(SUM($AF$4:$AF$14)&gt;0,AF14/SUM($AF$4:$AF$14),0))</f>
         <v>0</v>
       </c>
       <c r="AC14" s="30" t="n">
-        <f aca="false">IF(SUM($AE$4:$AE$14)&gt;0,AE14/SUM($AE$4:$AE$14),0)</f>
+        <f aca="false">IF(SUM($AE$4:$AE$14)&gt;0,AE14/SUM($AE$4:$AE$14),IF(SUM($AG$4:$AG$14)&gt;0,AG14/SUM($AG$4:$AG$14),0))</f>
         <v>0</v>
       </c>
       <c r="AD14" s="30" t="n">
@@ -18012,6 +18104,14 @@
       </c>
       <c r="AE14" s="30" t="n">
         <f aca="false">D14*IF(MAX(0,MIN(C14,Funnel!$B$19)-B14+1)&gt;0,MAX(0,MIN(C14,Funnel!$B$19)-MAX(B14,Assumptions!$D$7+Assumptions!$D$179)+1)/MAX(0,MIN(C14,Funnel!$B$19)-B14+1),0)</f>
+        <v>0</v>
+      </c>
+      <c r="AF14" s="29" t="n">
+        <f aca="false">MAX(0,MIN(C14,Funnel!$B$19)-MAX(B14,Assumptions!$D$7+Assumptions!$D$178)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="AG14" s="29" t="n">
+        <f aca="false">MAX(0,MIN(C14,Funnel!$B$19)-MAX(B14,Assumptions!$D$7+Assumptions!$D$179)+1)</f>
         <v>0</v>
       </c>
     </row>
@@ -18102,7 +18202,7 @@
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="B16" s="9"/>
       <c r="C16" s="9"/>
@@ -18154,22 +18254,22 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="28" t="s">
-        <v>709</v>
+        <v>711</v>
       </c>
       <c r="H18" s="28" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="2" t="s">
-        <v>711</v>
+        <v>713</v>
       </c>
       <c r="F19" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot",Channels!$B$5:$B$34,"&lt;&gt;I1b Employee referral sprint (bonus on hire)",Channels!$B$5:$B$34,"&lt;&gt;I1a Talent rediscovery (past applicants in ATS)")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
         <v>62640.1522284802</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>712</v>
+        <v>714</v>
       </c>
       <c r="L19" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,"I2 Handwerk → Industrie (construction electricians)")</f>
@@ -18178,14 +18278,14 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="2" t="s">
-        <v>713</v>
+        <v>715</v>
       </c>
       <c r="F20" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot",Channels!$B$5:$B$34,"&lt;&gt;I1b Employee referral sprint (bonus on hire)",Channels!$B$5:$B$34,"&lt;&gt;I1a Talent rediscovery (past applicants in ATS)")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$C$5:$C$34,"Supervisors")</f>
         <v>12178.6678273933</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>714</v>
+        <v>716</v>
       </c>
       <c r="L20" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$W$5:$W$34,Channels!$B$5:$B$34,"I2 Handwerk → Industrie (construction electricians)")</f>
@@ -18194,14 +18294,14 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="2" t="s">
-        <v>715</v>
+        <v>717</v>
       </c>
       <c r="F21" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$E$5:$E$34,"Slot")</f>
         <v>5796</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>716</v>
+        <v>718</v>
       </c>
       <c r="L21" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$V$5:$V$34,Channels!$B$5:$B$34,"I2 Handwerk → Industrie (construction electricians)")</f>
@@ -18210,14 +18310,14 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="2" t="s">
-        <v>717</v>
+        <v>719</v>
       </c>
       <c r="F22" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,"I1b Employee referral sprint (bonus on hire)",Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
         <v>9869.2425</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>718</v>
+        <v>720</v>
       </c>
       <c r="L22" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$U$5:$U$34,Channels!$B$5:$B$34,"I2 Handwerk → Industrie (construction electricians)")</f>
@@ -18226,14 +18326,14 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="2" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
       <c r="F23" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,"I1b Employee referral sprint (bonus on hire)",Channels!$C$5:$C$34,"Supervisors")</f>
         <v>1108.485</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
       <c r="L23" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,"I3 Polish border corridor + PL pre-screener")</f>
@@ -18242,14 +18342,14 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="2" t="s">
-        <v>721</v>
+        <v>723</v>
       </c>
       <c r="F24" s="41" t="n">
         <f aca="false">SUM(Channels!$Z$5:$Z$34)</f>
         <v>9000</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>722</v>
+        <v>724</v>
       </c>
       <c r="L24" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$W$5:$W$34,Channels!$B$5:$B$34,"I3 Polish border corridor + PL pre-screener")</f>
@@ -18258,14 +18358,14 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="2" t="s">
-        <v>723</v>
+        <v>725</v>
       </c>
       <c r="F25" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$AF$5:$AF$34,Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
         <v>8.9323002511364</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>724</v>
+        <v>726</v>
       </c>
       <c r="L25" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$V$5:$V$34,Channels!$B$5:$B$34,"I3 Polish border corridor + PL pre-screener")</f>
@@ -18274,14 +18374,14 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="2" t="s">
-        <v>725</v>
+        <v>727</v>
       </c>
       <c r="F26" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$AF$5:$AF$34,Channels!$C$5:$C$34,"Supervisors")</f>
         <v>3.25605421987231</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>726</v>
+        <v>728</v>
       </c>
       <c r="L26" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$U$5:$U$34,Channels!$B$5:$B$34,"I3 Polish border corridor + PL pre-screener")</f>
@@ -18290,7 +18390,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="2" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
       <c r="F27" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$AE$5:$AE$34,Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
@@ -18299,7 +18399,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="2" t="s">
-        <v>728</v>
+        <v>730</v>
       </c>
       <c r="F28" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$AE$5:$AE$34,Channels!$C$5:$C$34,"Supervisors")</f>
@@ -18308,7 +18408,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="2" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
       <c r="F29" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$AG$5:$AG$34,Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
@@ -18317,7 +18417,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="2" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="F30" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$AG$5:$AG$34,Channels!$C$5:$C$34,"Supervisors")</f>
@@ -18326,7 +18426,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="2" t="s">
-        <v>731</v>
+        <v>733</v>
       </c>
       <c r="F31" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)")</f>
@@ -18335,7 +18435,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="2" t="s">
-        <v>732</v>
+        <v>734</v>
       </c>
       <c r="F32" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$V$5:$V$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)",Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
@@ -18344,7 +18444,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="2" t="s">
-        <v>733</v>
+        <v>735</v>
       </c>
       <c r="F33" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$V$5:$V$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)",Channels!$C$5:$C$34,"Supervisors")</f>
@@ -18353,7 +18453,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="2" t="s">
-        <v>734</v>
+        <v>736</v>
       </c>
       <c r="F34" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$W$5:$W$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)",Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
@@ -18362,7 +18462,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="2" t="s">
-        <v>735</v>
+        <v>737</v>
       </c>
       <c r="F35" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$W$5:$W$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)",Channels!$C$5:$C$34,"Supervisors")</f>
@@ -18371,7 +18471,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="2" t="s">
-        <v>736</v>
+        <v>738</v>
       </c>
       <c r="F36" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$U$5:$U$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)",Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
@@ -18380,7 +18480,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="2" t="s">
-        <v>737</v>
+        <v>739</v>
       </c>
       <c r="F37" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$U$5:$U$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)",Channels!$C$5:$C$34,"Supervisors")</f>
@@ -18389,7 +18489,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="2" t="s">
-        <v>738</v>
+        <v>740</v>
       </c>
       <c r="F38" s="30" t="n">
         <f aca="false">IF(Funnel!B23&gt;0,MIN(1,Funnel!B22/Funnel!B23),1)</f>
@@ -18398,7 +18498,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="28" t="s">
-        <v>739</v>
+        <v>741</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18407,37 +18507,37 @@
         <v>315</v>
       </c>
       <c r="C43" s="12" t="s">
-        <v>740</v>
+        <v>742</v>
       </c>
       <c r="D43" s="12" t="s">
-        <v>741</v>
+        <v>743</v>
       </c>
       <c r="E43" s="12" t="s">
-        <v>742</v>
+        <v>744</v>
       </c>
       <c r="F43" s="12" t="s">
-        <v>743</v>
+        <v>745</v>
       </c>
       <c r="G43" s="12" t="s">
-        <v>744</v>
+        <v>746</v>
       </c>
       <c r="H43" s="12" t="s">
-        <v>745</v>
+        <v>747</v>
       </c>
       <c r="I43" s="12" t="s">
-        <v>746</v>
+        <v>748</v>
       </c>
       <c r="J43" s="12" t="s">
-        <v>747</v>
+        <v>749</v>
       </c>
       <c r="K43" s="12" t="s">
-        <v>748</v>
+        <v>750</v>
       </c>
       <c r="L43" s="12" t="s">
-        <v>749</v>
+        <v>751</v>
       </c>
       <c r="M43" s="12" t="s">
-        <v>750</v>
+        <v>752</v>
       </c>
       <c r="N43" s="12" t="s">
         <v>453</v>
@@ -19075,12 +19175,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>751</v>
+        <v>753</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>752</v>
+        <v>754</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -19094,76 +19194,76 @@
         <v>316</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>753</v>
+        <v>755</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>755</v>
+        <v>757</v>
       </c>
       <c r="G4" s="12" t="s">
-        <v>756</v>
+        <v>758</v>
       </c>
       <c r="H4" s="12" t="s">
-        <v>757</v>
+        <v>759</v>
       </c>
       <c r="I4" s="12" t="s">
-        <v>758</v>
+        <v>760</v>
       </c>
       <c r="J4" s="12" t="s">
-        <v>759</v>
+        <v>761</v>
       </c>
       <c r="K4" s="12" t="s">
-        <v>760</v>
+        <v>762</v>
       </c>
       <c r="L4" s="12" t="s">
-        <v>761</v>
+        <v>763</v>
       </c>
       <c r="M4" s="12" t="s">
-        <v>762</v>
+        <v>764</v>
       </c>
       <c r="N4" s="12" t="s">
-        <v>763</v>
+        <v>765</v>
       </c>
       <c r="O4" s="12" t="s">
-        <v>764</v>
+        <v>766</v>
       </c>
       <c r="P4" s="12" t="s">
-        <v>765</v>
+        <v>767</v>
       </c>
       <c r="Q4" s="12" t="s">
-        <v>766</v>
+        <v>768</v>
       </c>
       <c r="R4" s="12" t="s">
-        <v>767</v>
+        <v>769</v>
       </c>
       <c r="S4" s="12" t="s">
-        <v>768</v>
+        <v>770</v>
       </c>
       <c r="T4" s="12" t="s">
-        <v>769</v>
+        <v>771</v>
       </c>
       <c r="U4" s="12" t="s">
-        <v>770</v>
+        <v>772</v>
       </c>
       <c r="V4" s="12" t="s">
-        <v>771</v>
+        <v>773</v>
       </c>
       <c r="W4" s="12" t="s">
-        <v>772</v>
+        <v>774</v>
       </c>
       <c r="X4" s="12" t="s">
-        <v>773</v>
+        <v>775</v>
       </c>
       <c r="Y4" s="12" t="s">
-        <v>774</v>
+        <v>776</v>
       </c>
       <c r="Z4" s="12" t="s">
-        <v>775</v>
+        <v>777</v>
       </c>
       <c r="AA4" s="12" t="s">
-        <v>776</v>
+        <v>778</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21629,7 +21729,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="28" t="s">
-        <v>777</v>
+        <v>779</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -21638,46 +21738,46 @@
         <v>316</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>778</v>
+        <v>780</v>
       </c>
       <c r="D39" s="12" t="s">
-        <v>779</v>
+        <v>781</v>
       </c>
       <c r="E39" s="12" t="s">
-        <v>780</v>
+        <v>782</v>
       </c>
       <c r="F39" s="12" t="s">
-        <v>781</v>
+        <v>783</v>
       </c>
       <c r="G39" s="12" t="s">
-        <v>782</v>
+        <v>784</v>
       </c>
       <c r="H39" s="12" t="s">
-        <v>783</v>
+        <v>785</v>
       </c>
       <c r="I39" s="12" t="s">
-        <v>784</v>
+        <v>786</v>
       </c>
       <c r="J39" s="12" t="s">
-        <v>785</v>
+        <v>787</v>
       </c>
       <c r="K39" s="12" t="s">
-        <v>786</v>
+        <v>788</v>
       </c>
       <c r="L39" s="12" t="s">
-        <v>787</v>
+        <v>789</v>
       </c>
       <c r="M39" s="12" t="s">
-        <v>788</v>
+        <v>790</v>
       </c>
       <c r="N39" s="12" t="s">
-        <v>789</v>
+        <v>791</v>
       </c>
       <c r="O39" s="12" t="s">
         <v>47</v>
       </c>
       <c r="P39" s="12" t="s">
-        <v>790</v>
+        <v>792</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21907,7 +22007,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="9" t="s">
-        <v>791</v>
+        <v>793</v>
       </c>
       <c r="B46" s="9"/>
       <c r="C46" s="9"/>

</xml_diff>

<commit_message>
README describes the current tests and sources; TP1/TK1 wording matches the rounding
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V2NJtrYy3bzNxqKeiRXJfY
</commit_message>
<xml_diff>
--- a/operation_uptime/Operation_Uptime_Model.xlsx
+++ b/operation_uptime/Operation_Uptime_Model.xlsx
@@ -632,13 +632,13 @@
     <t xml:space="preserve">TP1</t>
   </si>
   <si>
-    <t xml:space="preserve">Initiative test: PASS needs at least this share of planned qualified in the window</t>
+    <t xml:space="preserve">Initiative test: PASS needs about this share of planned qualified in the window (rounded down)</t>
   </si>
   <si>
     <t xml:space="preserve">Initiatives</t>
   </si>
   <si>
-    <t xml:space="preserve">Two-week test passes if at least 60% of the planned qualified applicants arrive.</t>
+    <t xml:space="preserve">Two-week test passes at about 60% of the planned qualified applicants (rounded down to a whole person, so 54–58% at the current plan).</t>
   </si>
   <si>
     <t xml:space="preserve">TP2</t>
@@ -656,7 +656,7 @@
     <t xml:space="preserve">Initiative test: KILL if qualified below this share of plan</t>
   </si>
   <si>
-    <t xml:space="preserve">Kill the initiative if fewer than 30% of the planned qualified arrive.</t>
+    <t xml:space="preserve">Kill the initiative if fewer than about 30% of the planned qualified arrive (rounded up to a whole person).</t>
   </si>
   <si>
     <t xml:space="preserve">TK2</t>

</xml_diff>

<commit_message>
Evaluator fixes: T2/T3 and StepStone volume as own estimates, IAB 25% quoted exactly, bridge-course row, empty-export downside on slide 7, sensitivity column label, signing-lag note; AI note as executive summary
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V2NJtrYy3bzNxqKeiRXJfY
</commit_message>
<xml_diff>
--- a/operation_uptime/Operation_Uptime_Model.xlsx
+++ b/operation_uptime/Operation_Uptime_Model.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1512" uniqueCount="800">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1518" uniqueCount="804">
   <si>
     <t xml:space="preserve">Operation Uptime — model summary (hypothetical Tesla Giga Berlin maintenance hiring)</t>
   </si>
@@ -242,7 +242,7 @@
     <t xml:space="preserve">Researched</t>
   </si>
   <si>
-    <t xml:space="preserve">Global median: 6 days to review an application (SmartRecruiters 2025, Germany edition; German processes run longer, so this assumes the client keeps pace). https://ta.smartrecruiters.com/rs/664-NIC-529/images/Germany%20Recruiting%20Benchmarks%202025%20Report%20DE.pdf</t>
+    <t xml:space="preserve">Own estimate: SmartRecruiters 2025 global median is 6 days to review (Germany 8); I assume the client keeps the global pace, an ask. Slide 1 shows the German-pace downside (~92 hires). https://ta.smartrecruiters.com/rs/664-NIC-529/images/Germany%20Recruiting%20Benchmarks%202025%20Report%20DE.pdf</t>
   </si>
   <si>
     <t xml:space="preserve">T3</t>
@@ -251,7 +251,7 @@
     <t xml:space="preserve">Days: recruiter assessment → technical interview/test done</t>
   </si>
   <si>
-    <t xml:space="preserve">Global median: 14 days from application to interview, minus the 6 above (SmartRecruiters 2025, Germany edition). https://ta.smartrecruiters.com/rs/664-NIC-529/images/Germany%20Recruiting%20Benchmarks%202025%20Report%20DE.pdf</t>
+    <t xml:space="preserve">Own estimate: global median 14 days application → interview minus the 6 above (Germany 20 − 8 = 12); same commitment as T2. https://ta.smartrecruiters.com/rs/664-NIC-529/images/Germany%20Recruiting%20Benchmarks%202025%20Report%20DE.pdf</t>
   </si>
   <si>
     <t xml:space="preserve">T4</t>
@@ -290,7 +290,7 @@
     <t xml:space="preserve">Application → qualified (baseline, all channels)</t>
   </si>
   <si>
-    <t xml:space="preserve">About 1 in 4 applications is suitable in production jobs; 23% for specialist roles (IAB 2026). https://iab-forum.de/iab-stellenerhebung-2-2026-fast-drei-von-vier-bewerbungen-sind-aus-betrieblicher-sicht-ungeeignet/</t>
+    <t xml:space="preserve">IAB 2026 chart: production jobs get 12 applications per vacancy, 3 suitable (25%); 28% across all jobs; 23% for specialist roles. https://iab-forum.de/iab-stellenerhebung-2-2026-fast-drei-von-vier-bewerbungen-sind-aus-betrieblicher-sicht-ungeeignet/</t>
   </si>
   <si>
     <t xml:space="preserve">QM</t>
@@ -1070,7 +1070,7 @@
     <t xml:space="preserve">Slot</t>
   </si>
   <si>
-    <t xml:space="preserve">From €1,449 per 30-day ad (StepStone price list); HR teams get ~12 applications per vacancy on average (StepStone), used as applications per ad. https://www.stepstone.de/e-recruiting/stellenanzeige-aufgeben/ https://www.stepstone.de/e-recruiting/hr-wissen/recruiting/bewerberqualitaet-steigern</t>
+    <t xml:space="preserve">Own estimate: from €1,449 per 30-day ad (StepStone price list); StepStone says HR teams get ~12 applications per vacancy across all channels, used here as applications per ad. https://www.stepstone.de/e-recruiting/stellenanzeige-aufgeben/ https://www.stepstone.de/e-recruiting/hr-wissen/recruiting/bewerberqualitaet-steigern</t>
   </si>
   <si>
     <t xml:space="preserve">C10</t>
@@ -1340,6 +1340,18 @@
     <t xml:space="preserve">Translation at the German statutory rate per line (JVEG). https://www.gesetze-im-internet.de/jveg/__11.html</t>
   </si>
   <si>
+    <t xml:space="preserve">I2W</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I2: bridge course after signing (weeks, run by the client's maintenance trainers)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">weeks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2–4 weeks to cover the PLC/industrial gap; onboarding time paid as salary, so outside the campaign budget. Client names a trainer by 23 Oct.</t>
+  </si>
+  <si>
     <t xml:space="preserve">I2L</t>
   </si>
   <si>
@@ -1511,7 +1523,7 @@
     <t xml:space="preserve">Hires lost vs 100</t>
   </si>
   <si>
-    <t xml:space="preserve">Paid media needed (€, lower bound: same channels, caps ignored)</t>
+    <t xml:space="preserve">Spend needed (€, approx.: all variable spend scaled, channel caps ignored)</t>
   </si>
   <si>
     <t xml:space="preserve">Change in media</t>
@@ -2075,7 +2087,7 @@
     <t xml:space="preserve">Week-by-week plan: cash out, qualified flow vs 55/week, signatures</t>
   </si>
   <si>
-    <t xml:space="preserve">Cash by week: tests in weeks 1–2, StepStone ads and set-up in week 1, media by the weekly shares, referral bonuses when people sign.</t>
+    <t xml:space="preserve">Cash by week: tests in weeks 1–2, StepStone ads and set-up in week 1, media by the weekly shares, referral bonuses when people sign (signatures land ~24 days after application, rounded to whole weeks).</t>
   </si>
   <si>
     <t xml:space="preserve">Week</t>
@@ -3228,7 +3240,7 @@
         <v>16</v>
       </c>
       <c r="C19" s="8" t="str">
-        <f aca="false">IF(((Assumptions!$D$10&lt;0)+(Assumptions!$D$10&gt;1)+(Assumptions!$D$52&lt;0)+(Assumptions!$D$52&gt;1)+(Assumptions!$D$50&lt;0)+(Assumptions!$D$50&gt;1)+(Assumptions!$D$64&lt;0)+(Assumptions!$D$64&gt;1)+(Assumptions!$D$157&lt;0)+(Assumptions!$D$157&gt;1)+(Assumptions!$D$158&lt;0)+(Assumptions!$D$158&gt;1)+(Assumptions!$D$163&lt;0)+(Assumptions!$D$163&gt;1)+(Assumptions!$D$168&lt;0)+(Assumptions!$D$168&gt;1)+(Assumptions!$D$170&lt;0)+(Assumptions!$D$170&gt;1)+(Assumptions!$D$174&lt;0)+(Assumptions!$D$174&gt;1)+(Assumptions!$D$93&lt;0)+(Assumptions!$D$93&gt;1)+(Assumptions!$D$94&lt;0)+(Assumptions!$D$94&gt;1)+(Assumptions!$D$95&lt;0)+(Assumptions!$D$95&gt;1)+(Assumptions!$D$89&lt;0)+(Assumptions!$D$89&gt;1)+(Assumptions!$D$91&lt;0)+(Assumptions!$D$91&gt;1)+(Assumptions!$D$29&lt;0)+(Assumptions!$D$29&gt;1)+(Assumptions!$D$30&lt;0)+(Assumptions!$D$30&gt;1)+(Assumptions!$D$31&lt;0)+(Assumptions!$D$31&gt;1)+(Assumptions!$D$32&lt;0)+(Assumptions!$D$32&gt;1)+(Assumptions!$D$33&lt;0)+(Assumptions!$D$33&gt;1)+(Assumptions!$D$34&lt;0)+(Assumptions!$D$34&gt;1)+(Assumptions!$D$35&lt;0)+(Assumptions!$D$35&gt;1)+(Assumptions!$D$36&lt;0)+(Assumptions!$D$36&gt;1)+(Assumptions!$D$37&lt;0)+(Assumptions!$D$37&gt;1)+(Assumptions!$D$38&lt;0)+(Assumptions!$D$38&gt;1)+(Assumptions!$D$39&lt;0)+(Assumptions!$D$39&gt;1)+(Assumptions!$D$40&lt;0)+(Assumptions!$D$40&gt;1)+(Assumptions!$D$41&lt;0)+(Assumptions!$D$41&gt;1)+(Assumptions!$D$42&lt;0)+(Assumptions!$D$42&gt;1)+(Assumptions!$D$43&lt;0)+(Assumptions!$D$43&gt;1)+(Assumptions!$D$44&lt;0)+(Assumptions!$D$44&gt;1)+(Assumptions!$D$53&lt;0)+(Assumptions!$D$53&gt;1)+(Assumptions!$D$54&lt;0)+(Assumptions!$D$54&gt;1)+(Assumptions!$D$55&lt;0)+(Assumptions!$D$55&gt;1)+(Assumptions!$D$56&lt;0)+(Assumptions!$D$56&gt;1)+(Assumptions!$D$57&lt;0)+(Assumptions!$D$57&gt;1)+(Assumptions!$D$58&lt;0)+(Assumptions!$D$58&gt;1)+(Assumptions!$D$59&lt;0)+(Assumptions!$D$59&gt;1)+(Assumptions!$D$60&lt;0)+(Assumptions!$D$60&gt;1)+(Assumptions!$D$61&lt;0)+(Assumptions!$D$61&gt;1)+(Assumptions!$D$62&lt;0)+(Assumptions!$D$62&gt;1)+(Assumptions!$D$63&lt;0)+(Assumptions!$D$63&gt;1)+(Assumptions!$D$72&lt;0)+(Assumptions!$D$72&gt;1)+(Assumptions!$D$73&lt;0)+(Assumptions!$D$73&gt;1)+(Assumptions!$D$74&lt;0)+(Assumptions!$D$74&gt;1)+(Assumptions!$D$75&lt;0)+(Assumptions!$D$75&gt;1)+(Assumptions!$D$96&lt;0)+(Assumptions!$D$96&gt;1)+(Assumptions!$D$99&lt;0)+(Assumptions!$D$99&gt;1)+(Assumptions!$D$100&lt;0)+(Assumptions!$D$100&gt;1)+(Assumptions!$D$101&lt;0)+(Assumptions!$D$101&gt;1)+(Assumptions!$D$102&lt;0)+(Assumptions!$D$102&gt;1)+(Assumptions!$D$108&lt;0)+(Assumptions!$D$108&gt;1)+(Assumptions!$D$109&lt;0)+(Assumptions!$D$109&gt;1)+(Assumptions!$D$110&lt;0)+(Assumptions!$D$110&gt;1)+(Assumptions!$D$111&lt;0)+(Assumptions!$D$111&gt;1)+(Assumptions!$D$112&lt;0)+(Assumptions!$D$112&gt;1)+(Assumptions!$D$113&lt;0)+(Assumptions!$D$113&gt;1)+(Assumptions!$D$115&lt;0)+(Assumptions!$D$115&gt;1)+(Assumptions!$D$121&lt;0)+(Assumptions!$D$121&gt;1)+(Assumptions!$D$122&lt;0)+(Assumptions!$D$122&gt;1)+(Assumptions!$D$123&lt;0)+(Assumptions!$D$123&gt;1))+((Assumptions!$D$9&lt;0)+(Assumptions!$D$11&lt;0)+(Assumptions!$D$12&lt;0)+(Assumptions!$D$13&lt;0)+(Assumptions!$D$14&lt;0)+(Assumptions!$D$15&lt;0)+(Assumptions!$D$19&lt;0)+(Assumptions!$D$21&lt;0)+(Assumptions!$D$22&lt;0)+(Assumptions!$D$23&lt;0)+(Assumptions!$D$24&lt;0)+(Assumptions!$D$25&lt;0)+(Assumptions!$D$49&lt;0)+(Assumptions!$D$51&lt;0)+(Assumptions!$D$68&lt;0)+(Assumptions!$D$69&lt;0)+(Assumptions!$D$70&lt;0)+(Assumptions!$D$71&lt;0)+(Assumptions!$D$76&lt;0)+(Assumptions!$D$77&lt;0)+(Assumptions!$D$78&lt;0)+(Assumptions!$D$79&lt;0)+(Assumptions!$D$83&lt;0)+(Assumptions!$D$84&lt;0)+(Assumptions!$D$85&lt;0)+(Assumptions!$D$86&lt;0)+(Assumptions!$D$87&lt;0)+(Assumptions!$D$88&lt;0)+(Assumptions!$D$90&lt;0)+(Assumptions!$D$92&lt;0)+(Assumptions!$D$97&lt;0)+(Assumptions!$D$98&lt;0)+(Assumptions!$D$103&lt;0)+(Assumptions!$D$114&lt;0)+(Assumptions!$D$116&lt;0)+(Assumptions!$D$117&lt;0)+(Assumptions!$D$118&lt;0)+(Assumptions!$D$119&lt;0)+(Assumptions!$D$120&lt;0)+(Assumptions!$D$124&lt;0)+(Assumptions!$D$125&lt;0)+(Assumptions!$D$126&lt;0)+(Assumptions!$D$153&lt;0)+(Assumptions!$D$154&lt;0)+(Assumptions!$D$155&lt;0)+(Assumptions!$D$156&lt;0)+(Assumptions!$D$159&lt;0)+(Assumptions!$D$160&lt;0)+(Assumptions!$D$161&lt;0)+(Assumptions!$D$162&lt;0)+(Assumptions!$D$164&lt;0)+(Assumptions!$D$165&lt;0)+(Assumptions!$D$166&lt;0)+(Assumptions!$D$167&lt;0)+(Assumptions!$D$169&lt;0)+(Assumptions!$D$171&lt;0)+(Assumptions!$D$172&lt;0)+(Assumptions!$D$173&lt;0)+(Assumptions!$D$175&lt;0)+(Assumptions!$D$176&lt;0)+(Assumptions!$D$177&lt;0)+(Assumptions!$D$178&lt;0)+(Assumptions!$D$179&lt;0)+(Assumptions!$D$180&lt;0)+(Assumptions!$D$181&lt;0))+((INT(Assumptions!$D$19)&lt;&gt;Assumptions!$D$19)+(INT(Assumptions!$D$21)&lt;&gt;Assumptions!$D$21)+(INT(Assumptions!$D$22)&lt;&gt;Assumptions!$D$22)+(INT(Assumptions!$D$23)&lt;&gt;Assumptions!$D$23)+(INT(Assumptions!$D$24)&lt;&gt;Assumptions!$D$24)+(INT(Assumptions!$D$25)&lt;&gt;Assumptions!$D$25))+SUMPRODUCT((Assumptions!$E$130:$E$149&lt;0)+(Assumptions!$G$130:$G$149&lt;0)+(Assumptions!$G$130:$G$149&gt;1)+(Assumptions!$H$130:$H$149&lt;0)+(Assumptions!$I$130:$I$149&lt;0)+(Assumptions!$J$130:$J$149&lt;0)+(Assumptions!$F$130:$F$149&lt;0)+((Assumptions!$D$130:$D$149="CPC")*(Assumptions!$F$130:$F$149&gt;1)))+(Assumptions!$D$48&lt;0)+(Assumptions!$D$48&gt;=1)+(Assumptions!$D$20&lt;Assumptions!$D$7)+(Assumptions!$D$20&gt;Assumptions!$D$8)+(Assumptions!$D$8&lt;=Assumptions!$D$7)+(Assumptions!$D$91&gt;=Assumptions!$D$89)+(Assumptions!$D$92&lt;Assumptions!$D$90)=0,"✓ all inputs valid","✗ invalid input: "&amp;IF(((Assumptions!$D$10&lt;0)+(Assumptions!$D$10&gt;1)+(Assumptions!$D$52&lt;0)+(Assumptions!$D$52&gt;1)+(Assumptions!$D$50&lt;0)+(Assumptions!$D$50&gt;1)+(Assumptions!$D$64&lt;0)+(Assumptions!$D$64&gt;1)+(Assumptions!$D$157&lt;0)+(Assumptions!$D$157&gt;1)+(Assumptions!$D$158&lt;0)+(Assumptions!$D$158&gt;1)+(Assumptions!$D$163&lt;0)+(Assumptions!$D$163&gt;1)+(Assumptions!$D$168&lt;0)+(Assumptions!$D$168&gt;1)+(Assumptions!$D$170&lt;0)+(Assumptions!$D$170&gt;1)+(Assumptions!$D$174&lt;0)+(Assumptions!$D$174&gt;1)+(Assumptions!$D$93&lt;0)+(Assumptions!$D$93&gt;1)+(Assumptions!$D$94&lt;0)+(Assumptions!$D$94&gt;1)+(Assumptions!$D$95&lt;0)+(Assumptions!$D$95&gt;1)+(Assumptions!$D$89&lt;0)+(Assumptions!$D$89&gt;1)+(Assumptions!$D$91&lt;0)+(Assumptions!$D$91&gt;1)+(Assumptions!$D$29&lt;0)+(Assumptions!$D$29&gt;1)+(Assumptions!$D$30&lt;0)+(Assumptions!$D$30&gt;1)+(Assumptions!$D$31&lt;0)+(Assumptions!$D$31&gt;1)+(Assumptions!$D$32&lt;0)+(Assumptions!$D$32&gt;1)+(Assumptions!$D$33&lt;0)+(Assumptions!$D$33&gt;1)+(Assumptions!$D$34&lt;0)+(Assumptions!$D$34&gt;1)+(Assumptions!$D$35&lt;0)+(Assumptions!$D$35&gt;1)+(Assumptions!$D$36&lt;0)+(Assumptions!$D$36&gt;1)+(Assumptions!$D$37&lt;0)+(Assumptions!$D$37&gt;1)+(Assumptions!$D$38&lt;0)+(Assumptions!$D$38&gt;1)+(Assumptions!$D$39&lt;0)+(Assumptions!$D$39&gt;1)+(Assumptions!$D$40&lt;0)+(Assumptions!$D$40&gt;1)+(Assumptions!$D$41&lt;0)+(Assumptions!$D$41&gt;1)+(Assumptions!$D$42&lt;0)+(Assumptions!$D$42&gt;1)+(Assumptions!$D$43&lt;0)+(Assumptions!$D$43&gt;1)+(Assumptions!$D$44&lt;0)+(Assumptions!$D$44&gt;1)+(Assumptions!$D$53&lt;0)+(Assumptions!$D$53&gt;1)+(Assumptions!$D$54&lt;0)+(Assumptions!$D$54&gt;1)+(Assumptions!$D$55&lt;0)+(Assumptions!$D$55&gt;1)+(Assumptions!$D$56&lt;0)+(Assumptions!$D$56&gt;1)+(Assumptions!$D$57&lt;0)+(Assumptions!$D$57&gt;1)+(Assumptions!$D$58&lt;0)+(Assumptions!$D$58&gt;1)+(Assumptions!$D$59&lt;0)+(Assumptions!$D$59&gt;1)+(Assumptions!$D$60&lt;0)+(Assumptions!$D$60&gt;1)+(Assumptions!$D$61&lt;0)+(Assumptions!$D$61&gt;1)+(Assumptions!$D$62&lt;0)+(Assumptions!$D$62&gt;1)+(Assumptions!$D$63&lt;0)+(Assumptions!$D$63&gt;1)+(Assumptions!$D$72&lt;0)+(Assumptions!$D$72&gt;1)+(Assumptions!$D$73&lt;0)+(Assumptions!$D$73&gt;1)+(Assumptions!$D$74&lt;0)+(Assumptions!$D$74&gt;1)+(Assumptions!$D$75&lt;0)+(Assumptions!$D$75&gt;1)+(Assumptions!$D$96&lt;0)+(Assumptions!$D$96&gt;1)+(Assumptions!$D$99&lt;0)+(Assumptions!$D$99&gt;1)+(Assumptions!$D$100&lt;0)+(Assumptions!$D$100&gt;1)+(Assumptions!$D$101&lt;0)+(Assumptions!$D$101&gt;1)+(Assumptions!$D$102&lt;0)+(Assumptions!$D$102&gt;1)+(Assumptions!$D$108&lt;0)+(Assumptions!$D$108&gt;1)+(Assumptions!$D$109&lt;0)+(Assumptions!$D$109&gt;1)+(Assumptions!$D$110&lt;0)+(Assumptions!$D$110&gt;1)+(Assumptions!$D$111&lt;0)+(Assumptions!$D$111&gt;1)+(Assumptions!$D$112&lt;0)+(Assumptions!$D$112&gt;1)+(Assumptions!$D$113&lt;0)+(Assumptions!$D$113&gt;1)+(Assumptions!$D$115&lt;0)+(Assumptions!$D$115&gt;1)+(Assumptions!$D$121&lt;0)+(Assumptions!$D$121&gt;1)+(Assumptions!$D$122&lt;0)+(Assumptions!$D$122&gt;1)+(Assumptions!$D$123&lt;0)+(Assumptions!$D$123&gt;1))&gt;0,"a share/rate is outside 0–100%; ","")&amp;IF(((Assumptions!$D$9&lt;0)+(Assumptions!$D$11&lt;0)+(Assumptions!$D$12&lt;0)+(Assumptions!$D$13&lt;0)+(Assumptions!$D$14&lt;0)+(Assumptions!$D$15&lt;0)+(Assumptions!$D$19&lt;0)+(Assumptions!$D$21&lt;0)+(Assumptions!$D$22&lt;0)+(Assumptions!$D$23&lt;0)+(Assumptions!$D$24&lt;0)+(Assumptions!$D$25&lt;0)+(Assumptions!$D$49&lt;0)+(Assumptions!$D$51&lt;0)+(Assumptions!$D$68&lt;0)+(Assumptions!$D$69&lt;0)+(Assumptions!$D$70&lt;0)+(Assumptions!$D$71&lt;0)+(Assumptions!$D$76&lt;0)+(Assumptions!$D$77&lt;0)+(Assumptions!$D$78&lt;0)+(Assumptions!$D$79&lt;0)+(Assumptions!$D$83&lt;0)+(Assumptions!$D$84&lt;0)+(Assumptions!$D$85&lt;0)+(Assumptions!$D$86&lt;0)+(Assumptions!$D$87&lt;0)+(Assumptions!$D$88&lt;0)+(Assumptions!$D$90&lt;0)+(Assumptions!$D$92&lt;0)+(Assumptions!$D$97&lt;0)+(Assumptions!$D$98&lt;0)+(Assumptions!$D$103&lt;0)+(Assumptions!$D$114&lt;0)+(Assumptions!$D$116&lt;0)+(Assumptions!$D$117&lt;0)+(Assumptions!$D$118&lt;0)+(Assumptions!$D$119&lt;0)+(Assumptions!$D$120&lt;0)+(Assumptions!$D$124&lt;0)+(Assumptions!$D$125&lt;0)+(Assumptions!$D$126&lt;0)+(Assumptions!$D$153&lt;0)+(Assumptions!$D$154&lt;0)+(Assumptions!$D$155&lt;0)+(Assumptions!$D$156&lt;0)+(Assumptions!$D$159&lt;0)+(Assumptions!$D$160&lt;0)+(Assumptions!$D$161&lt;0)+(Assumptions!$D$162&lt;0)+(Assumptions!$D$164&lt;0)+(Assumptions!$D$165&lt;0)+(Assumptions!$D$166&lt;0)+(Assumptions!$D$167&lt;0)+(Assumptions!$D$169&lt;0)+(Assumptions!$D$171&lt;0)+(Assumptions!$D$172&lt;0)+(Assumptions!$D$173&lt;0)+(Assumptions!$D$175&lt;0)+(Assumptions!$D$176&lt;0)+(Assumptions!$D$177&lt;0)+(Assumptions!$D$178&lt;0)+(Assumptions!$D$179&lt;0)+(Assumptions!$D$180&lt;0)+(Assumptions!$D$181&lt;0))&gt;0,"a count, cost or day value is negative; ","")&amp;IF(((INT(Assumptions!$D$19)&lt;&gt;Assumptions!$D$19)+(INT(Assumptions!$D$21)&lt;&gt;Assumptions!$D$21)+(INT(Assumptions!$D$22)&lt;&gt;Assumptions!$D$22)+(INT(Assumptions!$D$23)&lt;&gt;Assumptions!$D$23)+(INT(Assumptions!$D$24)&lt;&gt;Assumptions!$D$24)+(INT(Assumptions!$D$25)&lt;&gt;Assumptions!$D$25))&gt;0,"day inputs (T0, T2–T6) must be whole days; ","")&amp;IF(SUMPRODUCT((Assumptions!$E$130:$E$149&lt;0)+(Assumptions!$G$130:$G$149&lt;0)+(Assumptions!$G$130:$G$149&gt;1)+(Assumptions!$H$130:$H$149&lt;0)+(Assumptions!$I$130:$I$149&lt;0)+(Assumptions!$J$130:$J$149&lt;0)+(Assumptions!$F$130:$F$149&lt;0)+((Assumptions!$D$130:$D$149="CPC")*(Assumptions!$F$130:$F$149&gt;1)))&gt;0,"a channel input (Assumptions §7) is out of range; ","")&amp;IF(OR(Assumptions!$D$48&lt;0,Assumptions!$D$48&gt;=1),"reserve share must be 0–99%; ","")&amp;IF(OR(Assumptions!$D$20&lt;Assumptions!$D$7,Assumptions!$D$20&gt;Assumptions!$D$8),"last signing date must fall inside the campaign; ","")&amp;IF(Assumptions!$D$8&lt;=Assumptions!$D$7,"campaign end must be after its start; ","")&amp;IF(OR(Assumptions!$D$91&gt;=Assumptions!$D$89,Assumptions!$D$92&lt;Assumptions!$D$90),"initiative kill thresholds must sit below pass thresholds (TK1 &lt; TP1, TK2 ≥ TP2); ",""))</f>
+        <f aca="false">IF(((Assumptions!$D$10&lt;0)+(Assumptions!$D$10&gt;1)+(Assumptions!$D$52&lt;0)+(Assumptions!$D$52&gt;1)+(Assumptions!$D$50&lt;0)+(Assumptions!$D$50&gt;1)+(Assumptions!$D$64&lt;0)+(Assumptions!$D$64&gt;1)+(Assumptions!$D$157&lt;0)+(Assumptions!$D$157&gt;1)+(Assumptions!$D$158&lt;0)+(Assumptions!$D$158&gt;1)+(Assumptions!$D$163&lt;0)+(Assumptions!$D$163&gt;1)+(Assumptions!$D$168&lt;0)+(Assumptions!$D$168&gt;1)+(Assumptions!$D$170&lt;0)+(Assumptions!$D$170&gt;1)+(Assumptions!$D$174&lt;0)+(Assumptions!$D$174&gt;1)+(Assumptions!$D$93&lt;0)+(Assumptions!$D$93&gt;1)+(Assumptions!$D$94&lt;0)+(Assumptions!$D$94&gt;1)+(Assumptions!$D$95&lt;0)+(Assumptions!$D$95&gt;1)+(Assumptions!$D$89&lt;0)+(Assumptions!$D$89&gt;1)+(Assumptions!$D$91&lt;0)+(Assumptions!$D$91&gt;1)+(Assumptions!$D$29&lt;0)+(Assumptions!$D$29&gt;1)+(Assumptions!$D$30&lt;0)+(Assumptions!$D$30&gt;1)+(Assumptions!$D$31&lt;0)+(Assumptions!$D$31&gt;1)+(Assumptions!$D$32&lt;0)+(Assumptions!$D$32&gt;1)+(Assumptions!$D$33&lt;0)+(Assumptions!$D$33&gt;1)+(Assumptions!$D$34&lt;0)+(Assumptions!$D$34&gt;1)+(Assumptions!$D$35&lt;0)+(Assumptions!$D$35&gt;1)+(Assumptions!$D$36&lt;0)+(Assumptions!$D$36&gt;1)+(Assumptions!$D$37&lt;0)+(Assumptions!$D$37&gt;1)+(Assumptions!$D$38&lt;0)+(Assumptions!$D$38&gt;1)+(Assumptions!$D$39&lt;0)+(Assumptions!$D$39&gt;1)+(Assumptions!$D$40&lt;0)+(Assumptions!$D$40&gt;1)+(Assumptions!$D$41&lt;0)+(Assumptions!$D$41&gt;1)+(Assumptions!$D$42&lt;0)+(Assumptions!$D$42&gt;1)+(Assumptions!$D$43&lt;0)+(Assumptions!$D$43&gt;1)+(Assumptions!$D$44&lt;0)+(Assumptions!$D$44&gt;1)+(Assumptions!$D$53&lt;0)+(Assumptions!$D$53&gt;1)+(Assumptions!$D$54&lt;0)+(Assumptions!$D$54&gt;1)+(Assumptions!$D$55&lt;0)+(Assumptions!$D$55&gt;1)+(Assumptions!$D$56&lt;0)+(Assumptions!$D$56&gt;1)+(Assumptions!$D$57&lt;0)+(Assumptions!$D$57&gt;1)+(Assumptions!$D$58&lt;0)+(Assumptions!$D$58&gt;1)+(Assumptions!$D$59&lt;0)+(Assumptions!$D$59&gt;1)+(Assumptions!$D$60&lt;0)+(Assumptions!$D$60&gt;1)+(Assumptions!$D$61&lt;0)+(Assumptions!$D$61&gt;1)+(Assumptions!$D$62&lt;0)+(Assumptions!$D$62&gt;1)+(Assumptions!$D$63&lt;0)+(Assumptions!$D$63&gt;1)+(Assumptions!$D$72&lt;0)+(Assumptions!$D$72&gt;1)+(Assumptions!$D$73&lt;0)+(Assumptions!$D$73&gt;1)+(Assumptions!$D$74&lt;0)+(Assumptions!$D$74&gt;1)+(Assumptions!$D$75&lt;0)+(Assumptions!$D$75&gt;1)+(Assumptions!$D$96&lt;0)+(Assumptions!$D$96&gt;1)+(Assumptions!$D$99&lt;0)+(Assumptions!$D$99&gt;1)+(Assumptions!$D$100&lt;0)+(Assumptions!$D$100&gt;1)+(Assumptions!$D$101&lt;0)+(Assumptions!$D$101&gt;1)+(Assumptions!$D$102&lt;0)+(Assumptions!$D$102&gt;1)+(Assumptions!$D$108&lt;0)+(Assumptions!$D$108&gt;1)+(Assumptions!$D$109&lt;0)+(Assumptions!$D$109&gt;1)+(Assumptions!$D$110&lt;0)+(Assumptions!$D$110&gt;1)+(Assumptions!$D$111&lt;0)+(Assumptions!$D$111&gt;1)+(Assumptions!$D$112&lt;0)+(Assumptions!$D$112&gt;1)+(Assumptions!$D$113&lt;0)+(Assumptions!$D$113&gt;1)+(Assumptions!$D$115&lt;0)+(Assumptions!$D$115&gt;1)+(Assumptions!$D$121&lt;0)+(Assumptions!$D$121&gt;1)+(Assumptions!$D$122&lt;0)+(Assumptions!$D$122&gt;1)+(Assumptions!$D$123&lt;0)+(Assumptions!$D$123&gt;1))+((Assumptions!$D$9&lt;0)+(Assumptions!$D$11&lt;0)+(Assumptions!$D$12&lt;0)+(Assumptions!$D$13&lt;0)+(Assumptions!$D$14&lt;0)+(Assumptions!$D$15&lt;0)+(Assumptions!$D$19&lt;0)+(Assumptions!$D$21&lt;0)+(Assumptions!$D$22&lt;0)+(Assumptions!$D$23&lt;0)+(Assumptions!$D$24&lt;0)+(Assumptions!$D$25&lt;0)+(Assumptions!$D$49&lt;0)+(Assumptions!$D$51&lt;0)+(Assumptions!$D$68&lt;0)+(Assumptions!$D$69&lt;0)+(Assumptions!$D$70&lt;0)+(Assumptions!$D$71&lt;0)+(Assumptions!$D$76&lt;0)+(Assumptions!$D$77&lt;0)+(Assumptions!$D$78&lt;0)+(Assumptions!$D$79&lt;0)+(Assumptions!$D$83&lt;0)+(Assumptions!$D$84&lt;0)+(Assumptions!$D$85&lt;0)+(Assumptions!$D$86&lt;0)+(Assumptions!$D$87&lt;0)+(Assumptions!$D$88&lt;0)+(Assumptions!$D$90&lt;0)+(Assumptions!$D$92&lt;0)+(Assumptions!$D$97&lt;0)+(Assumptions!$D$98&lt;0)+(Assumptions!$D$103&lt;0)+(Assumptions!$D$114&lt;0)+(Assumptions!$D$116&lt;0)+(Assumptions!$D$117&lt;0)+(Assumptions!$D$118&lt;0)+(Assumptions!$D$119&lt;0)+(Assumptions!$D$120&lt;0)+(Assumptions!$D$124&lt;0)+(Assumptions!$D$125&lt;0)+(Assumptions!$D$126&lt;0)+(Assumptions!$D$153&lt;0)+(Assumptions!$D$154&lt;0)+(Assumptions!$D$155&lt;0)+(Assumptions!$D$156&lt;0)+(Assumptions!$D$159&lt;0)+(Assumptions!$D$160&lt;0)+(Assumptions!$D$161&lt;0)+(Assumptions!$D$162&lt;0)+(Assumptions!$D$164&lt;0)+(Assumptions!$D$165&lt;0)+(Assumptions!$D$166&lt;0)+(Assumptions!$D$167&lt;0)+(Assumptions!$D$169&lt;0)+(Assumptions!$D$171&lt;0)+(Assumptions!$D$172&lt;0)+(Assumptions!$D$173&lt;0)+(Assumptions!$D$175&lt;0)+(Assumptions!$D$176&lt;0)+(Assumptions!$D$177&lt;0)+(Assumptions!$D$178&lt;0)+(Assumptions!$D$179&lt;0)+(Assumptions!$D$180&lt;0)+(Assumptions!$D$181&lt;0)+(Assumptions!$D$182&lt;0))+((INT(Assumptions!$D$19)&lt;&gt;Assumptions!$D$19)+(INT(Assumptions!$D$21)&lt;&gt;Assumptions!$D$21)+(INT(Assumptions!$D$22)&lt;&gt;Assumptions!$D$22)+(INT(Assumptions!$D$23)&lt;&gt;Assumptions!$D$23)+(INT(Assumptions!$D$24)&lt;&gt;Assumptions!$D$24)+(INT(Assumptions!$D$25)&lt;&gt;Assumptions!$D$25))+SUMPRODUCT((Assumptions!$E$130:$E$149&lt;0)+(Assumptions!$G$130:$G$149&lt;0)+(Assumptions!$G$130:$G$149&gt;1)+(Assumptions!$H$130:$H$149&lt;0)+(Assumptions!$I$130:$I$149&lt;0)+(Assumptions!$J$130:$J$149&lt;0)+(Assumptions!$F$130:$F$149&lt;0)+((Assumptions!$D$130:$D$149="CPC")*(Assumptions!$F$130:$F$149&gt;1)))+(Assumptions!$D$48&lt;0)+(Assumptions!$D$48&gt;=1)+(Assumptions!$D$20&lt;Assumptions!$D$7)+(Assumptions!$D$20&gt;Assumptions!$D$8)+(Assumptions!$D$8&lt;=Assumptions!$D$7)+(Assumptions!$D$91&gt;=Assumptions!$D$89)+(Assumptions!$D$92&lt;Assumptions!$D$90)=0,"✓ all inputs valid","✗ invalid input: "&amp;IF(((Assumptions!$D$10&lt;0)+(Assumptions!$D$10&gt;1)+(Assumptions!$D$52&lt;0)+(Assumptions!$D$52&gt;1)+(Assumptions!$D$50&lt;0)+(Assumptions!$D$50&gt;1)+(Assumptions!$D$64&lt;0)+(Assumptions!$D$64&gt;1)+(Assumptions!$D$157&lt;0)+(Assumptions!$D$157&gt;1)+(Assumptions!$D$158&lt;0)+(Assumptions!$D$158&gt;1)+(Assumptions!$D$163&lt;0)+(Assumptions!$D$163&gt;1)+(Assumptions!$D$168&lt;0)+(Assumptions!$D$168&gt;1)+(Assumptions!$D$170&lt;0)+(Assumptions!$D$170&gt;1)+(Assumptions!$D$174&lt;0)+(Assumptions!$D$174&gt;1)+(Assumptions!$D$93&lt;0)+(Assumptions!$D$93&gt;1)+(Assumptions!$D$94&lt;0)+(Assumptions!$D$94&gt;1)+(Assumptions!$D$95&lt;0)+(Assumptions!$D$95&gt;1)+(Assumptions!$D$89&lt;0)+(Assumptions!$D$89&gt;1)+(Assumptions!$D$91&lt;0)+(Assumptions!$D$91&gt;1)+(Assumptions!$D$29&lt;0)+(Assumptions!$D$29&gt;1)+(Assumptions!$D$30&lt;0)+(Assumptions!$D$30&gt;1)+(Assumptions!$D$31&lt;0)+(Assumptions!$D$31&gt;1)+(Assumptions!$D$32&lt;0)+(Assumptions!$D$32&gt;1)+(Assumptions!$D$33&lt;0)+(Assumptions!$D$33&gt;1)+(Assumptions!$D$34&lt;0)+(Assumptions!$D$34&gt;1)+(Assumptions!$D$35&lt;0)+(Assumptions!$D$35&gt;1)+(Assumptions!$D$36&lt;0)+(Assumptions!$D$36&gt;1)+(Assumptions!$D$37&lt;0)+(Assumptions!$D$37&gt;1)+(Assumptions!$D$38&lt;0)+(Assumptions!$D$38&gt;1)+(Assumptions!$D$39&lt;0)+(Assumptions!$D$39&gt;1)+(Assumptions!$D$40&lt;0)+(Assumptions!$D$40&gt;1)+(Assumptions!$D$41&lt;0)+(Assumptions!$D$41&gt;1)+(Assumptions!$D$42&lt;0)+(Assumptions!$D$42&gt;1)+(Assumptions!$D$43&lt;0)+(Assumptions!$D$43&gt;1)+(Assumptions!$D$44&lt;0)+(Assumptions!$D$44&gt;1)+(Assumptions!$D$53&lt;0)+(Assumptions!$D$53&gt;1)+(Assumptions!$D$54&lt;0)+(Assumptions!$D$54&gt;1)+(Assumptions!$D$55&lt;0)+(Assumptions!$D$55&gt;1)+(Assumptions!$D$56&lt;0)+(Assumptions!$D$56&gt;1)+(Assumptions!$D$57&lt;0)+(Assumptions!$D$57&gt;1)+(Assumptions!$D$58&lt;0)+(Assumptions!$D$58&gt;1)+(Assumptions!$D$59&lt;0)+(Assumptions!$D$59&gt;1)+(Assumptions!$D$60&lt;0)+(Assumptions!$D$60&gt;1)+(Assumptions!$D$61&lt;0)+(Assumptions!$D$61&gt;1)+(Assumptions!$D$62&lt;0)+(Assumptions!$D$62&gt;1)+(Assumptions!$D$63&lt;0)+(Assumptions!$D$63&gt;1)+(Assumptions!$D$72&lt;0)+(Assumptions!$D$72&gt;1)+(Assumptions!$D$73&lt;0)+(Assumptions!$D$73&gt;1)+(Assumptions!$D$74&lt;0)+(Assumptions!$D$74&gt;1)+(Assumptions!$D$75&lt;0)+(Assumptions!$D$75&gt;1)+(Assumptions!$D$96&lt;0)+(Assumptions!$D$96&gt;1)+(Assumptions!$D$99&lt;0)+(Assumptions!$D$99&gt;1)+(Assumptions!$D$100&lt;0)+(Assumptions!$D$100&gt;1)+(Assumptions!$D$101&lt;0)+(Assumptions!$D$101&gt;1)+(Assumptions!$D$102&lt;0)+(Assumptions!$D$102&gt;1)+(Assumptions!$D$108&lt;0)+(Assumptions!$D$108&gt;1)+(Assumptions!$D$109&lt;0)+(Assumptions!$D$109&gt;1)+(Assumptions!$D$110&lt;0)+(Assumptions!$D$110&gt;1)+(Assumptions!$D$111&lt;0)+(Assumptions!$D$111&gt;1)+(Assumptions!$D$112&lt;0)+(Assumptions!$D$112&gt;1)+(Assumptions!$D$113&lt;0)+(Assumptions!$D$113&gt;1)+(Assumptions!$D$115&lt;0)+(Assumptions!$D$115&gt;1)+(Assumptions!$D$121&lt;0)+(Assumptions!$D$121&gt;1)+(Assumptions!$D$122&lt;0)+(Assumptions!$D$122&gt;1)+(Assumptions!$D$123&lt;0)+(Assumptions!$D$123&gt;1))&gt;0,"a share/rate is outside 0–100%; ","")&amp;IF(((Assumptions!$D$9&lt;0)+(Assumptions!$D$11&lt;0)+(Assumptions!$D$12&lt;0)+(Assumptions!$D$13&lt;0)+(Assumptions!$D$14&lt;0)+(Assumptions!$D$15&lt;0)+(Assumptions!$D$19&lt;0)+(Assumptions!$D$21&lt;0)+(Assumptions!$D$22&lt;0)+(Assumptions!$D$23&lt;0)+(Assumptions!$D$24&lt;0)+(Assumptions!$D$25&lt;0)+(Assumptions!$D$49&lt;0)+(Assumptions!$D$51&lt;0)+(Assumptions!$D$68&lt;0)+(Assumptions!$D$69&lt;0)+(Assumptions!$D$70&lt;0)+(Assumptions!$D$71&lt;0)+(Assumptions!$D$76&lt;0)+(Assumptions!$D$77&lt;0)+(Assumptions!$D$78&lt;0)+(Assumptions!$D$79&lt;0)+(Assumptions!$D$83&lt;0)+(Assumptions!$D$84&lt;0)+(Assumptions!$D$85&lt;0)+(Assumptions!$D$86&lt;0)+(Assumptions!$D$87&lt;0)+(Assumptions!$D$88&lt;0)+(Assumptions!$D$90&lt;0)+(Assumptions!$D$92&lt;0)+(Assumptions!$D$97&lt;0)+(Assumptions!$D$98&lt;0)+(Assumptions!$D$103&lt;0)+(Assumptions!$D$114&lt;0)+(Assumptions!$D$116&lt;0)+(Assumptions!$D$117&lt;0)+(Assumptions!$D$118&lt;0)+(Assumptions!$D$119&lt;0)+(Assumptions!$D$120&lt;0)+(Assumptions!$D$124&lt;0)+(Assumptions!$D$125&lt;0)+(Assumptions!$D$126&lt;0)+(Assumptions!$D$153&lt;0)+(Assumptions!$D$154&lt;0)+(Assumptions!$D$155&lt;0)+(Assumptions!$D$156&lt;0)+(Assumptions!$D$159&lt;0)+(Assumptions!$D$160&lt;0)+(Assumptions!$D$161&lt;0)+(Assumptions!$D$162&lt;0)+(Assumptions!$D$164&lt;0)+(Assumptions!$D$165&lt;0)+(Assumptions!$D$166&lt;0)+(Assumptions!$D$167&lt;0)+(Assumptions!$D$169&lt;0)+(Assumptions!$D$171&lt;0)+(Assumptions!$D$172&lt;0)+(Assumptions!$D$173&lt;0)+(Assumptions!$D$175&lt;0)+(Assumptions!$D$176&lt;0)+(Assumptions!$D$177&lt;0)+(Assumptions!$D$178&lt;0)+(Assumptions!$D$179&lt;0)+(Assumptions!$D$180&lt;0)+(Assumptions!$D$181&lt;0)+(Assumptions!$D$182&lt;0))&gt;0,"a count, cost or day value is negative; ","")&amp;IF(((INT(Assumptions!$D$19)&lt;&gt;Assumptions!$D$19)+(INT(Assumptions!$D$21)&lt;&gt;Assumptions!$D$21)+(INT(Assumptions!$D$22)&lt;&gt;Assumptions!$D$22)+(INT(Assumptions!$D$23)&lt;&gt;Assumptions!$D$23)+(INT(Assumptions!$D$24)&lt;&gt;Assumptions!$D$24)+(INT(Assumptions!$D$25)&lt;&gt;Assumptions!$D$25))&gt;0,"day inputs (T0, T2–T6) must be whole days; ","")&amp;IF(SUMPRODUCT((Assumptions!$E$130:$E$149&lt;0)+(Assumptions!$G$130:$G$149&lt;0)+(Assumptions!$G$130:$G$149&gt;1)+(Assumptions!$H$130:$H$149&lt;0)+(Assumptions!$I$130:$I$149&lt;0)+(Assumptions!$J$130:$J$149&lt;0)+(Assumptions!$F$130:$F$149&lt;0)+((Assumptions!$D$130:$D$149="CPC")*(Assumptions!$F$130:$F$149&gt;1)))&gt;0,"a channel input (Assumptions §7) is out of range; ","")&amp;IF(OR(Assumptions!$D$48&lt;0,Assumptions!$D$48&gt;=1),"reserve share must be 0–99%; ","")&amp;IF(OR(Assumptions!$D$20&lt;Assumptions!$D$7,Assumptions!$D$20&gt;Assumptions!$D$8),"last signing date must fall inside the campaign; ","")&amp;IF(Assumptions!$D$8&lt;=Assumptions!$D$7,"campaign end must be after its start; ","")&amp;IF(OR(Assumptions!$D$91&gt;=Assumptions!$D$89,Assumptions!$D$92&lt;Assumptions!$D$90),"initiative kill thresholds must sit below pass thresholds (TK1 &lt; TP1, TK2 ≥ TP2); ",""))</f>
         <v>✓ all inputs valid</v>
       </c>
     </row>
@@ -3279,7 +3291,7 @@
     <tabColor rgb="FFFFC000"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L181"/>
+  <dimension ref="A1:L182"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
@@ -3666,7 +3678,7 @@
         <v>62</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="G22" s="17" t="s">
         <v>74</v>
@@ -6258,7 +6270,7 @@
         <v>0</v>
       </c>
       <c r="K138" s="2" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="L138" s="17" t="s">
         <v>347</v>
@@ -6298,7 +6310,7 @@
         <v>0</v>
       </c>
       <c r="K139" s="2" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="L139" s="17" t="s">
         <v>347</v>
@@ -6338,7 +6350,7 @@
         <v>0</v>
       </c>
       <c r="K140" s="2" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="L140" s="17" t="s">
         <v>347</v>
@@ -6378,7 +6390,7 @@
         <v>0</v>
       </c>
       <c r="K141" s="2" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="L141" s="17" t="s">
         <v>347</v>
@@ -7368,27 +7380,27 @@
         <v>3</v>
       </c>
       <c r="E180" s="2" t="s">
-        <v>62</v>
+        <v>439</v>
       </c>
       <c r="F180" s="2" t="s">
         <v>63</v>
       </c>
       <c r="G180" s="13" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
     </row>
     <row r="181" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A181" s="2" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="B181" s="13" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="C181" s="2" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="D181" s="15" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E181" s="2" t="s">
         <v>62</v>
@@ -7397,7 +7409,30 @@
         <v>63</v>
       </c>
       <c r="G181" s="13" t="s">
-        <v>442</v>
+        <v>443</v>
+      </c>
+    </row>
+    <row r="182" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A182" s="2" t="s">
+        <v>444</v>
+      </c>
+      <c r="B182" s="13" t="s">
+        <v>445</v>
+      </c>
+      <c r="C182" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D182" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="E182" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="F182" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="G182" s="13" t="s">
+        <v>446</v>
       </c>
     </row>
   </sheetData>
@@ -7410,7 +7445,7 @@
       <formula1>0</formula1>
       <formula2>0.99</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" error="Enter a number ≥ 0." errorStyle="stop" errorTitle="Out of range" operator="greaterThanOrEqual" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D9 D11:D15 D49 D51 D68:D71 D76:D79 D83:D88 D90 D92 D97:D98 D103 D108:D110 D114 D116:D118 D120 D124:D126 E130:F149 H130:J149 D153:D156 D159:D162 D164:D167 D169 D171:D173 D175:D179" type="decimal">
+    <dataValidation allowBlank="false" error="Enter a number ≥ 0." errorStyle="stop" errorTitle="Out of range" operator="greaterThanOrEqual" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D9 D11:D15 D49 D51 D68:D71 D76:D79 D83:D88 D90 D92 D97:D98 D103 D108:D110 D114 D116:D118 D120 D124:D126 E130:F149 H130:J149 D153:D156 D159:D162 D164:D167 D169 D171:D173 D175:D180" type="decimal">
       <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -7418,7 +7453,7 @@
       <formula1>DATE(2026,10,20)</formula1>
       <formula2>DATE(2026,12,31)</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" error="Enter a whole number of days (0 or more)." errorStyle="stop" errorTitle="Whole days" operator="greaterThanOrEqual" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D19 D21:D25 D119 D180:D181" type="whole">
+    <dataValidation allowBlank="false" error="Enter a whole number of days (0 or more)." errorStyle="stop" errorTitle="Whole days" operator="greaterThanOrEqual" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D19 D21:D25 D119 D181:D182" type="whole">
       <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -7427,13 +7462,13 @@
     <hyperlink ref="G10" r:id="rId1" display="From the brief. Polish hires need no work permit (EU free movement) and are insured and taxed in Germany. https://www.make-it-in-germany.com/en/working-in-germany/information-eu-citizens/print"/>
     <hyperlink ref="G15" r:id="rId2" display="From the brief, so I plan no foreign-trained electricians. Worth raising: for employees the trade is not legally regulated, which could open this route. https://www.anerkennung-in-deutschland.de/en/interest/finder/profession/62/profile"/>
     <hyperlink ref="G20" r:id="rId3" display="My choice: the last Friday before Christmas. Indeed job searches fall to 45% below the 1–15 Dec average over the holidays (Indeed Hiring Lab). https://hiringlab.indeed.com/de/blog/2025/02/17/der-stellenmarkt-startet-unausgewogen-in-das-neue-jahr/"/>
-    <hyperlink ref="G21" r:id="rId4" display="Global median: 6 days to review an application (SmartRecruiters 2025, Germany edition; German processes run longer, so this assumes the client keeps pace). https://ta.smartrecruiters.com/rs/664-NIC-529/images/Germany%20Recruiting%20Benchmarks%202025%20Report%20DE.pdf"/>
-    <hyperlink ref="G22" r:id="rId5" display="Global median: 14 days from application to interview, minus the 6 above (SmartRecruiters 2025, Germany edition). https://ta.smartrecruiters.com/rs/664-NIC-529/images/Germany%20Recruiting%20Benchmarks%202025%20Report%20DE.pdf"/>
+    <hyperlink ref="G21" r:id="rId4" display="Own estimate: SmartRecruiters 2025 global median is 6 days to review (Germany 8); I assume the client keeps the global pace, an ask. Slide 1 shows the German-pace downside (~92 hires). https://ta.smartrecruiters.com/rs/664-NIC-529/images/Germany%20Recruiting%20Benchmarks%202025%20Report%20DE.pdf"/>
+    <hyperlink ref="G22" r:id="rId5" display="Own estimate: global median 14 days application → interview minus the 6 above (Germany 20 − 8 = 12); same commitment as T2. https://ta.smartrecruiters.com/rs/664-NIC-529/images/Germany%20Recruiting%20Benchmarks%202025%20Report%20DE.pdf"/>
     <hyperlink ref="G24" r:id="rId6" display="One-week offer validity; candidates take ~9 days on average to decide (NACE 2025). https://www.naceweb.org/talent-acquisition/trends-and-predictions/employers-make-more-offers-as-student-acceptance-rate-rises-response-time-shortens"/>
-    <hyperlink ref="G29" r:id="rId7" display="About 1 in 4 applications is suitable in production jobs; 23% for specialist roles (IAB 2026). https://iab-forum.de/iab-stellenerhebung-2-2026-fast-drei-von-vier-bewerbungen-sind-aus-betrieblicher-sicht-ungeeignet/"/>
-    <hyperlink ref="G30" r:id="rId8" display="About 1 in 4 applications is suitable in production jobs; 23% for specialist roles (IAB 2026). https://iab-forum.de/iab-stellenerhebung-2-2026-fast-drei-von-vier-bewerbungen-sind-aus-betrieblicher-sicht-ungeeignet/"/>
-    <hyperlink ref="G31" r:id="rId9" display="About 1 in 4 applications is suitable in production jobs; 23% for specialist roles (IAB 2026). https://iab-forum.de/iab-stellenerhebung-2-2026-fast-drei-von-vier-bewerbungen-sind-aus-betrieblicher-sicht-ungeeignet/"/>
-    <hyperlink ref="G32" r:id="rId10" display="About 1 in 4 applications is suitable in production jobs; 23% for specialist roles (IAB 2026). https://iab-forum.de/iab-stellenerhebung-2-2026-fast-drei-von-vier-bewerbungen-sind-aus-betrieblicher-sicht-ungeeignet/"/>
+    <hyperlink ref="G29" r:id="rId7" display="IAB 2026 chart: production jobs get 12 applications per vacancy, 3 suitable (25%); 28% across all jobs; 23% for specialist roles. https://iab-forum.de/iab-stellenerhebung-2-2026-fast-drei-von-vier-bewerbungen-sind-aus-betrieblicher-sicht-ungeeignet/"/>
+    <hyperlink ref="G30" r:id="rId8" display="IAB 2026 chart: production jobs get 12 applications per vacancy, 3 suitable (25%); 28% across all jobs; 23% for specialist roles. https://iab-forum.de/iab-stellenerhebung-2-2026-fast-drei-von-vier-bewerbungen-sind-aus-betrieblicher-sicht-ungeeignet/"/>
+    <hyperlink ref="G31" r:id="rId9" display="IAB 2026 chart: production jobs get 12 applications per vacancy, 3 suitable (25%); 28% across all jobs; 23% for specialist roles. https://iab-forum.de/iab-stellenerhebung-2-2026-fast-drei-von-vier-bewerbungen-sind-aus-betrieblicher-sicht-ungeeignet/"/>
+    <hyperlink ref="G32" r:id="rId10" display="IAB 2026 chart: production jobs get 12 applications per vacancy, 3 suitable (25%); 28% across all jobs; 23% for specialist roles. https://iab-forum.de/iab-stellenerhebung-2-2026-fast-drei-von-vier-bewerbungen-sind-aus-betrieblicher-sicht-ungeeignet/"/>
     <hyperlink ref="G33" r:id="rId11" display="Gem 2025: ~35% of candidates brought onsite get offers (mostly US tech). Set higher (50%) because only pre-qualified people reach this step. https://lp.gem.com/rs/972-IVV-330/images/2025%20Recruiting%20Benchmarks%20-%20Gem.pdf"/>
     <hyperlink ref="G34" r:id="rId12" display="Gem 2025: ~35% of onsite candidates get offers. Set at 55%: most common trade, the assessment is routine for it. https://lp.gem.com/rs/972-IVV-330/images/2025%20Recruiting%20Benchmarks%20-%20Gem.pdf"/>
     <hyperlink ref="G35" r:id="rId13" display="Gem 2025: ~35% of onsite candidates get offers. Set at 45%: PLC skills are tested hard. https://lp.gem.com/rs/972-IVV-330/images/2025%20Recruiting%20Benchmarks%20-%20Gem.pdf"/>
@@ -7486,10 +7521,10 @@
     <hyperlink ref="L135" r:id="rId60" display="Indeed's CPA median is €161 in TalentBait's DACH 2024–26 dataset (2,549 channel-campaigns across all channels), used as the programmatic proxy. Volume capped by Indeed's reach. https://www.talentbait.de/recruiting-kanaele-uebersicht/"/>
     <hyperlink ref="L136" r:id="rId61" display="Indeed's CPA median is €161 in TalentBait's DACH 2024–26 dataset (2,549 channel-campaigns across all channels), used as the programmatic proxy. Volume capped by Indeed's reach. https://www.talentbait.de/recruiting-kanaele-uebersicht/"/>
     <hyperlink ref="L137" r:id="rId62" display="Indeed's CPA median is €161 in TalentBait's DACH 2024–26 dataset (2,549 channel-campaigns across all channels), used as the programmatic proxy. Volume capped by Indeed's reach. https://www.talentbait.de/recruiting-kanaele-uebersicht/"/>
-    <hyperlink ref="L138" r:id="rId63" display="From €1,449 per 30-day ad (StepStone price list); HR teams get ~12 applications per vacancy on average (StepStone), used as applications per ad. https://www.stepstone.de/e-recruiting/stellenanzeige-aufgeben/ https://www.stepstone.de/e-recruiting/hr-wissen/recruiting/bewerberqualitaet-steigern"/>
-    <hyperlink ref="L139" r:id="rId64" display="From €1,449 per 30-day ad (StepStone price list); HR teams get ~12 applications per vacancy on average (StepStone), used as applications per ad. https://www.stepstone.de/e-recruiting/stellenanzeige-aufgeben/ https://www.stepstone.de/e-recruiting/hr-wissen/recruiting/bewerberqualitaet-steigern"/>
-    <hyperlink ref="L140" r:id="rId65" display="From €1,449 per 30-day ad (StepStone price list); HR teams get ~12 applications per vacancy on average (StepStone), used as applications per ad. https://www.stepstone.de/e-recruiting/stellenanzeige-aufgeben/ https://www.stepstone.de/e-recruiting/hr-wissen/recruiting/bewerberqualitaet-steigern"/>
-    <hyperlink ref="L141" r:id="rId66" display="From €1,449 per 30-day ad (StepStone price list); HR teams get ~12 applications per vacancy on average (StepStone), used as applications per ad. https://www.stepstone.de/e-recruiting/stellenanzeige-aufgeben/ https://www.stepstone.de/e-recruiting/hr-wissen/recruiting/bewerberqualitaet-steigern"/>
+    <hyperlink ref="L138" r:id="rId63" display="Own estimate: from €1,449 per 30-day ad (StepStone price list); StepStone says HR teams get ~12 applications per vacancy across all channels, used here as applications per ad. https://www.stepstone.de/e-recruiting/stellenanzeige-aufgeben/ https://www.stepstone.de/e-recruiting/hr-wissen/recruiting/bewerberqualitaet-steigern"/>
+    <hyperlink ref="L139" r:id="rId64" display="Own estimate: from €1,449 per 30-day ad (StepStone price list); StepStone says HR teams get ~12 applications per vacancy across all channels, used here as applications per ad. https://www.stepstone.de/e-recruiting/stellenanzeige-aufgeben/ https://www.stepstone.de/e-recruiting/hr-wissen/recruiting/bewerberqualitaet-steigern"/>
+    <hyperlink ref="L140" r:id="rId65" display="Own estimate: from €1,449 per 30-day ad (StepStone price list); StepStone says HR teams get ~12 applications per vacancy across all channels, used here as applications per ad. https://www.stepstone.de/e-recruiting/stellenanzeige-aufgeben/ https://www.stepstone.de/e-recruiting/hr-wissen/recruiting/bewerberqualitaet-steigern"/>
+    <hyperlink ref="L141" r:id="rId66" display="Own estimate: from €1,449 per 30-day ad (StepStone price list); StepStone says HR teams get ~12 applications per vacancy across all channels, used here as applications per ad. https://www.stepstone.de/e-recruiting/stellenanzeige-aufgeben/ https://www.stepstone.de/e-recruiting/hr-wissen/recruiting/bewerberqualitaet-steigern"/>
     <hyperlink ref="L142" r:id="rId67" display="DACH median €96 per application (TalentBait). Used only for automation and supervisors. https://www.talentbait.de/recruiting-kanaele-uebersicht/"/>
     <hyperlink ref="L143" r:id="rId68" display="DACH median €96 per application (TalentBait). Used only for automation and supervisors. https://www.talentbait.de/recruiting-kanaele-uebersicht/"/>
     <hyperlink ref="L144" r:id="rId69" display="Own estimate: TalentBait's example ad shows ~€84 per application for trades (its measured averages: €52 raw, €104 per qualified); volume from Redline campaign data. https://www.talentbait.de/social-media-recruiting"/>
@@ -7541,12 +7576,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>443</v>
+        <v>447</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>444</v>
+        <v>448</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7557,46 +7592,46 @@
         <v>47</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>445</v>
+        <v>449</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>446</v>
+        <v>450</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
       <c r="G4" s="12" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="H4" s="12" t="s">
-        <v>450</v>
+        <v>454</v>
       </c>
       <c r="I4" s="12" t="s">
-        <v>451</v>
+        <v>455</v>
       </c>
       <c r="J4" s="12" t="s">
-        <v>452</v>
+        <v>456</v>
       </c>
       <c r="K4" s="12" t="s">
-        <v>453</v>
+        <v>457</v>
       </c>
       <c r="L4" s="12" t="s">
-        <v>454</v>
+        <v>458</v>
       </c>
       <c r="M4" s="12" t="s">
-        <v>455</v>
+        <v>459</v>
       </c>
       <c r="N4" s="12" t="s">
-        <v>456</v>
+        <v>460</v>
       </c>
       <c r="O4" s="12" t="s">
-        <v>457</v>
+        <v>461</v>
       </c>
       <c r="P4" s="12" t="s">
-        <v>458</v>
+        <v>462</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7861,7 +7896,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="28" t="s">
-        <v>459</v>
+        <v>463</v>
       </c>
       <c r="B9" s="33" t="n">
         <f aca="false">SUM(B5:B8)</f>
@@ -7906,17 +7941,17 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="28" t="s">
-        <v>461</v>
+        <v>465</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>462</v>
+        <v>466</v>
       </c>
       <c r="B13" s="36" t="n">
         <f aca="false">Assumptions!$D$7+Assumptions!$D$19</f>
@@ -7925,7 +7960,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>463</v>
+        <v>467</v>
       </c>
       <c r="B14" s="36" t="n">
         <f aca="false">Assumptions!$D$20</f>
@@ -7934,7 +7969,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>464</v>
+        <v>468</v>
       </c>
       <c r="B15" s="29" t="n">
         <f aca="false">Assumptions!$D$22+Assumptions!$D$23+Assumptions!$D$24</f>
@@ -7943,7 +7978,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>465</v>
+        <v>469</v>
       </c>
       <c r="B16" s="29" t="n">
         <f aca="false">B15+Assumptions!$D$25</f>
@@ -7952,7 +7987,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>466</v>
+        <v>470</v>
       </c>
       <c r="B17" s="36" t="n">
         <f aca="false">B14-B15</f>
@@ -7961,7 +7996,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>467</v>
+        <v>471</v>
       </c>
       <c r="B18" s="36" t="n">
         <f aca="false">B14-B16</f>
@@ -7988,7 +8023,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>468</v>
+        <v>472</v>
       </c>
       <c r="B21" s="29" t="n">
         <f aca="false">MAX(0,B17-B13+1)</f>
@@ -8006,7 +8041,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>469</v>
+        <v>473</v>
       </c>
       <c r="B23" s="29" t="n">
         <f aca="false">O9</f>
@@ -8028,7 +8063,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>470</v>
+        <v>474</v>
       </c>
       <c r="B25" s="31" t="n">
         <f aca="false">IF(O9&gt;0,Channels!U35/O9,0)</f>
@@ -8037,19 +8072,19 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>471</v>
+        <v>475</v>
       </c>
       <c r="B26" s="38" t="n">
         <f aca="false">B22*B25</f>
         <v>102.049737036446</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>472</v>
+        <v>476</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="28" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8060,34 +8095,34 @@
         <v>47</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>474</v>
+        <v>478</v>
       </c>
       <c r="D29" s="12" t="s">
-        <v>475</v>
+        <v>479</v>
       </c>
       <c r="E29" s="12" t="s">
-        <v>476</v>
+        <v>480</v>
       </c>
       <c r="F29" s="12" t="s">
-        <v>477</v>
+        <v>481</v>
       </c>
       <c r="G29" s="12" t="s">
-        <v>478</v>
+        <v>482</v>
       </c>
       <c r="H29" s="12" t="s">
-        <v>479</v>
+        <v>483</v>
       </c>
       <c r="I29" s="12" t="s">
-        <v>480</v>
+        <v>484</v>
       </c>
       <c r="J29" s="12" t="s">
-        <v>481</v>
+        <v>485</v>
       </c>
       <c r="K29" s="12" t="s">
-        <v>482</v>
+        <v>486</v>
       </c>
       <c r="L29" s="12" t="s">
-        <v>483</v>
+        <v>487</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8123,10 +8158,10 @@
         <v>2271.6049382716</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>484</v>
+        <v>488</v>
       </c>
       <c r="J30" s="2" t="s">
-        <v>485</v>
+        <v>489</v>
       </c>
       <c r="K30" s="40" t="n">
         <f aca="false">IF(B30&gt;0,(D30-SUMIFS(Channels!$N:$N,Channels!$A:$A,"I2-E",Channels!$C:$C,A30))/B30,0)</f>
@@ -8170,10 +8205,10 @@
         <v>1927.42237186682</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>486</v>
+        <v>490</v>
       </c>
       <c r="J31" s="2" t="s">
-        <v>487</v>
+        <v>491</v>
       </c>
       <c r="K31" s="40" t="n">
         <f aca="false">IF(B31&gt;0,(D31-SUMIFS(Channels!$N:$N,Channels!$A:$A,"I2-E",Channels!$C:$C,A31))/B31,0)</f>
@@ -8217,10 +8252,10 @@
         <v>1504.99706055262</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>484</v>
+        <v>488</v>
       </c>
       <c r="J32" s="2" t="s">
-        <v>487</v>
+        <v>491</v>
       </c>
       <c r="K32" s="40" t="n">
         <f aca="false">IF(B32&gt;0,(D32-SUMIFS(Channels!$N:$N,Channels!$A:$A,"I2-E",Channels!$C:$C,A32))/B32,0)</f>
@@ -8264,10 +8299,10 @@
         <v>1948.60552916819</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>484</v>
+        <v>488</v>
       </c>
       <c r="J33" s="2" t="s">
-        <v>487</v>
+        <v>491</v>
       </c>
       <c r="K33" s="40" t="n">
         <f aca="false">IF(B33&gt;0,(D33-SUMIFS(Channels!$N:$N,Channels!$A:$A,"I2-E",Channels!$C:$C,A33))/B33,0)</f>
@@ -8319,12 +8354,12 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="28" t="s">
-        <v>488</v>
+        <v>492</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
-        <v>489</v>
+        <v>493</v>
       </c>
       <c r="B40" s="30" t="n">
         <f aca="false">Assumptions!$D$64</f>
@@ -8333,33 +8368,33 @@
     </row>
     <row r="41" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="12" t="s">
-        <v>490</v>
+        <v>494</v>
       </c>
       <c r="B41" s="12" t="s">
-        <v>491</v>
+        <v>495</v>
       </c>
       <c r="C41" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D41" s="12" t="s">
-        <v>492</v>
+        <v>496</v>
       </c>
       <c r="E41" s="12" t="s">
-        <v>493</v>
+        <v>497</v>
       </c>
       <c r="F41" s="12" t="s">
-        <v>494</v>
+        <v>498</v>
       </c>
       <c r="G41" s="12" t="s">
-        <v>495</v>
+        <v>499</v>
       </c>
       <c r="H41" s="12" t="s">
-        <v>496</v>
+        <v>500</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="13" t="s">
-        <v>497</v>
+        <v>501</v>
       </c>
       <c r="B42" s="29" t="n">
         <f aca="false">O9</f>
@@ -8386,12 +8421,12 @@
         <v>0</v>
       </c>
       <c r="H42" s="13" t="s">
-        <v>498</v>
+        <v>502</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="13" t="s">
-        <v>499</v>
+        <v>503</v>
       </c>
       <c r="B43" s="29" t="n">
         <f aca="false">O9/(1-$B$40)</f>
@@ -8418,12 +8453,12 @@
         <v>0.428571428571429</v>
       </c>
       <c r="H43" s="13" t="s">
-        <v>500</v>
+        <v>504</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="13" t="s">
-        <v>501</v>
+        <v>505</v>
       </c>
       <c r="B44" s="29" t="n">
         <f aca="false">O9/(1-$B$40)</f>
@@ -8450,12 +8485,12 @@
         <v>0.428571428571429</v>
       </c>
       <c r="H44" s="13" t="s">
-        <v>502</v>
+        <v>506</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="13" t="s">
-        <v>503</v>
+        <v>507</v>
       </c>
       <c r="B45" s="29" t="n">
         <f aca="false">O9</f>
@@ -8482,12 +8517,12 @@
         <v>0.428571428571429</v>
       </c>
       <c r="H45" s="13" t="s">
-        <v>504</v>
+        <v>508</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="13" t="s">
-        <v>505</v>
+        <v>509</v>
       </c>
       <c r="B46" s="29" t="n">
         <f aca="false">O9</f>
@@ -8514,12 +8549,12 @@
         <v>0.3</v>
       </c>
       <c r="H46" s="13" t="s">
-        <v>506</v>
+        <v>510</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="13" t="s">
-        <v>507</v>
+        <v>511</v>
       </c>
       <c r="B47" s="29" t="n">
         <f aca="false">O9</f>
@@ -8546,12 +8581,12 @@
         <v>0</v>
       </c>
       <c r="H47" s="13" t="s">
-        <v>508</v>
+        <v>512</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="28" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="D49" s="8" t="str">
         <f aca="false">INDEX(A43:A46,MATCH(MAX(E43:E46),E43:E46,0))</f>
@@ -8583,7 +8618,7 @@
     </row>
     <row r="54" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="1" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8591,34 +8626,34 @@
         <v>322</v>
       </c>
       <c r="B57" s="12" t="s">
-        <v>511</v>
+        <v>515</v>
       </c>
       <c r="C57" s="12" t="s">
-        <v>512</v>
+        <v>516</v>
       </c>
       <c r="D57" s="12" t="s">
-        <v>513</v>
+        <v>517</v>
       </c>
       <c r="E57" s="12" t="s">
-        <v>514</v>
+        <v>518</v>
       </c>
       <c r="F57" s="12" t="s">
-        <v>515</v>
+        <v>519</v>
       </c>
       <c r="G57" s="12" t="s">
-        <v>516</v>
+        <v>520</v>
       </c>
       <c r="H57" s="12" t="s">
-        <v>517</v>
+        <v>521</v>
       </c>
       <c r="I57" s="12" t="s">
-        <v>518</v>
+        <v>522</v>
       </c>
       <c r="J57" s="12" t="s">
-        <v>519</v>
+        <v>523</v>
       </c>
       <c r="K57" s="12" t="s">
-        <v>520</v>
+        <v>524</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8803,7 +8838,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="9" t="s">
-        <v>521</v>
+        <v>525</v>
       </c>
       <c r="B63" s="9"/>
       <c r="C63" s="9"/>
@@ -8863,22 +8898,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>522</v>
+        <v>526</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>523</v>
+        <v>527</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="28" t="s">
-        <v>524</v>
+        <v>528</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
-        <v>525</v>
+        <v>529</v>
       </c>
       <c r="B4" s="12" t="s">
         <v>48</v>
@@ -8893,12 +8928,12 @@
         <v>54</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>459</v>
+        <v>463</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>526</v>
+        <v>530</v>
       </c>
       <c r="B5" s="29" t="n">
         <f aca="false">Assumptions!$D$153</f>
@@ -8923,7 +8958,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>527</v>
+        <v>531</v>
       </c>
       <c r="B6" s="30" t="n">
         <f aca="false">Assumptions!$D$157</f>
@@ -8944,7 +8979,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>528</v>
+        <v>532</v>
       </c>
       <c r="B7" s="32" t="n">
         <f aca="false">B5*B6</f>
@@ -8969,7 +9004,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>529</v>
+        <v>533</v>
       </c>
       <c r="B8" s="30" t="n">
         <f aca="false">Assumptions!$D$158</f>
@@ -8990,7 +9025,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>530</v>
+        <v>534</v>
       </c>
       <c r="B9" s="31" t="n">
         <f aca="false">Funnel!$G$5*Assumptions!$D$166</f>
@@ -9011,7 +9046,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>531</v>
+        <v>535</v>
       </c>
       <c r="B10" s="41" t="n">
         <f aca="false">B5*Assumptions!$D$164</f>
@@ -9036,7 +9071,7 @@
     </row>
     <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>532</v>
+        <v>536</v>
       </c>
       <c r="B11" s="43" t="n">
         <f aca="false">IF(B7&gt;0,B10/B7,0)</f>
@@ -9061,7 +9096,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>533</v>
+        <v>537</v>
       </c>
       <c r="B12" s="32" t="n">
         <f aca="false">B7*B8*B9</f>
@@ -9086,7 +9121,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>534</v>
+        <v>538</v>
       </c>
       <c r="B13" s="32" t="n">
         <f aca="false">Assumptions!$D$159</f>
@@ -9111,7 +9146,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="B14" s="30" t="n">
         <f aca="false">Assumptions!$D$163</f>
@@ -9132,7 +9167,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>536</v>
+        <v>540</v>
       </c>
       <c r="B15" s="32" t="n">
         <f aca="false">B13*B14*B9</f>
@@ -9157,7 +9192,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>537</v>
+        <v>541</v>
       </c>
       <c r="B16" s="41" t="n">
         <f aca="false">B15*Assumptions!$D$165</f>
@@ -9182,7 +9217,7 @@
     </row>
     <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>538</v>
+        <v>542</v>
       </c>
       <c r="B17" s="43" t="n">
         <f aca="false">IF(B13&gt;0,B16/B13,0)</f>
@@ -9201,12 +9236,12 @@
         <v>123.165</v>
       </c>
       <c r="G17" s="13" t="s">
-        <v>539</v>
+        <v>543</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>540</v>
+        <v>544</v>
       </c>
       <c r="B18" s="32" t="n">
         <f aca="false">B12+B15</f>
@@ -9231,7 +9266,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>541</v>
+        <v>545</v>
       </c>
       <c r="B19" s="41" t="n">
         <f aca="false">B10+B16</f>
@@ -9256,7 +9291,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>542</v>
+        <v>546</v>
       </c>
       <c r="B20" s="41" t="n">
         <f aca="false">IF(B18&gt;0,B19/B18,0)</f>
@@ -9281,12 +9316,12 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="28" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>544</v>
+        <v>548</v>
       </c>
       <c r="B24" s="29" t="n">
         <f aca="false">Assumptions!$D$167</f>
@@ -9295,7 +9330,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>545</v>
+        <v>549</v>
       </c>
       <c r="B25" s="31" t="n">
         <f aca="false">Assumptions!$D$168</f>
@@ -9304,7 +9339,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>546</v>
+        <v>550</v>
       </c>
       <c r="B26" s="29" t="n">
         <f aca="false">B24*B25</f>
@@ -9313,7 +9348,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>547</v>
+        <v>551</v>
       </c>
       <c r="B27" s="41" t="n">
         <f aca="false">Assumptions!$D$169</f>
@@ -9322,7 +9357,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>548</v>
+        <v>552</v>
       </c>
       <c r="B28" s="30" t="n">
         <f aca="false">Assumptions!$D$170</f>
@@ -9331,7 +9366,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>549</v>
+        <v>553</v>
       </c>
       <c r="B29" s="32" t="n">
         <f aca="false">B26*B28</f>
@@ -9340,7 +9375,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>550</v>
+        <v>554</v>
       </c>
       <c r="B30" s="31" t="n">
         <f aca="false">Funnel!$G$5*Assumptions!$D$171</f>
@@ -9349,7 +9384,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>551</v>
+        <v>555</v>
       </c>
       <c r="B31" s="32" t="n">
         <f aca="false">B29*B30</f>
@@ -9358,7 +9393,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>552</v>
+        <v>556</v>
       </c>
       <c r="B32" s="41" t="n">
         <f aca="false">B26*B27</f>
@@ -9367,7 +9402,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>553</v>
+        <v>557</v>
       </c>
       <c r="B33" s="41" t="n">
         <f aca="false">Assumptions!$D$172</f>
@@ -9376,7 +9411,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="B34" s="41" t="n">
         <f aca="false">IF(B31&gt;0,(B32+B33)/B31,0)</f>
@@ -9385,12 +9420,12 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="28" t="s">
-        <v>555</v>
+        <v>559</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="B38" s="43" t="n">
         <f aca="false">B44+B45</f>
@@ -9399,7 +9434,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
-        <v>557</v>
+        <v>561</v>
       </c>
       <c r="B39" s="30" t="n">
         <f aca="false">Assumptions!$D$174</f>
@@ -9408,7 +9443,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
-        <v>546</v>
+        <v>550</v>
       </c>
       <c r="B40" s="29" t="n">
         <f aca="false">Assumptions!$D$175</f>
@@ -9417,7 +9452,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
-        <v>558</v>
+        <v>562</v>
       </c>
       <c r="B41" s="31" t="n">
         <f aca="false">Funnel!$G$6*Assumptions!$D$176</f>
@@ -9426,7 +9461,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="2" t="s">
-        <v>559</v>
+        <v>563</v>
       </c>
       <c r="B42" s="32" t="n">
         <f aca="false">Assumptions!$D$10*Assumptions!$D$12</f>
@@ -9435,7 +9470,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
-        <v>560</v>
+        <v>564</v>
       </c>
       <c r="B43" s="32" t="n">
         <f aca="false">MIN(B40*B39*B41,B42)</f>
@@ -9444,7 +9479,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="2" t="s">
-        <v>561</v>
+        <v>565</v>
       </c>
       <c r="B44" s="43" t="n">
         <f aca="false">Assumptions!$D$173</f>
@@ -9453,7 +9488,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="2" t="s">
-        <v>562</v>
+        <v>566</v>
       </c>
       <c r="B45" s="43" t="n">
         <f aca="false">Assumptions!$D$177/60*Assumptions!$D$178</f>
@@ -9462,7 +9497,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="2" t="s">
-        <v>563</v>
+        <v>567</v>
       </c>
       <c r="B46" s="41" t="n">
         <f aca="false">Assumptions!$D$179</f>
@@ -9471,7 +9506,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="2" t="s">
-        <v>564</v>
+        <v>568</v>
       </c>
       <c r="B47" s="29" t="n">
         <f aca="false">IF(B41*B39&gt;0,B43/B41/B39,0)</f>
@@ -9480,7 +9515,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="2" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
       <c r="B48" s="41" t="n">
         <f aca="false">IF(B43&gt;0,(B47*B38+B46)/B43,0)</f>
@@ -9512,50 +9547,50 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="28" t="s">
-        <v>566</v>
+        <v>570</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="12" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="B52" s="12" t="s">
-        <v>568</v>
+        <v>572</v>
       </c>
       <c r="C52" s="12" t="s">
-        <v>569</v>
+        <v>573</v>
       </c>
       <c r="D52" s="12" t="s">
-        <v>570</v>
+        <v>574</v>
       </c>
       <c r="E52" s="12" t="s">
-        <v>571</v>
+        <v>575</v>
       </c>
       <c r="F52" s="12" t="s">
-        <v>572</v>
+        <v>576</v>
       </c>
       <c r="G52" s="12" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="H52" s="12" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="I52" s="12" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="J52" s="12" t="s">
-        <v>576</v>
+        <v>580</v>
       </c>
       <c r="K52" s="12" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="28" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="B53" s="13" t="s">
-        <v>579</v>
+        <v>583</v>
       </c>
       <c r="C53" s="30" t="n">
         <f aca="false">(Assumptions!$D$93+Assumptions!$D$94)</f>
@@ -9570,32 +9605,32 @@
         <v>24.5433</v>
       </c>
       <c r="F53" s="2" t="s">
-        <v>580</v>
+        <v>584</v>
       </c>
       <c r="G53" s="29" t="n">
         <f aca="false">MAX(1,ROUNDDOWN(E53*Assumptions!$D$89,0))</f>
         <v>14</v>
       </c>
       <c r="H53" s="2" t="s">
-        <v>581</v>
+        <v>585</v>
       </c>
       <c r="I53" s="29" t="n">
         <f aca="false">MIN(G53,MAX(1,ROUNDUP(E53*Assumptions!$D$91,0)))</f>
         <v>8</v>
       </c>
       <c r="J53" s="2" t="s">
-        <v>581</v>
+        <v>585</v>
       </c>
       <c r="K53" s="13" t="s">
-        <v>582</v>
+        <v>586</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="28" t="s">
-        <v>583</v>
+        <v>587</v>
       </c>
       <c r="B54" s="13" t="s">
-        <v>584</v>
+        <v>588</v>
       </c>
       <c r="C54" s="30" t="n">
         <f aca="false">(Weekly!$AB$4+Weekly!$AB$5+Weekly!$AB$6*3/7)</f>
@@ -9630,15 +9665,15 @@
         <v>670</v>
       </c>
       <c r="K54" s="13" t="s">
-        <v>585</v>
+        <v>589</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="28" t="s">
-        <v>586</v>
+        <v>590</v>
       </c>
       <c r="B55" s="13" t="s">
-        <v>587</v>
+        <v>591</v>
       </c>
       <c r="C55" s="30" t="n">
         <f aca="false">(Weekly!$AC$5+Weekly!$AC$6)</f>
@@ -9673,12 +9708,12 @@
         <v>270</v>
       </c>
       <c r="K55" s="13" t="s">
-        <v>588</v>
+        <v>592</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="13" t="s">
-        <v>589</v>
+        <v>593</v>
       </c>
     </row>
   </sheetData>
@@ -9719,17 +9754,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>590</v>
+        <v>594</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="369.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="13" t="s">
-        <v>591</v>
+        <v>595</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="318.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="13" t="s">
-        <v>592</v>
+        <v>596</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9743,100 +9778,100 @@
         <v>322</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>593</v>
+        <v>597</v>
       </c>
       <c r="E4" s="12" t="s">
         <v>323</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>594</v>
+        <v>598</v>
       </c>
       <c r="G4" s="12" t="s">
-        <v>595</v>
+        <v>599</v>
       </c>
       <c r="H4" s="12" t="s">
-        <v>547</v>
+        <v>551</v>
       </c>
       <c r="I4" s="12" t="s">
         <v>326</v>
       </c>
       <c r="J4" s="12" t="s">
-        <v>546</v>
+        <v>550</v>
       </c>
       <c r="K4" s="12" t="s">
-        <v>596</v>
+        <v>600</v>
       </c>
       <c r="L4" s="12" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="M4" s="12" t="s">
-        <v>597</v>
+        <v>601</v>
       </c>
       <c r="N4" s="12" t="s">
-        <v>598</v>
+        <v>602</v>
       </c>
       <c r="O4" s="12" t="s">
-        <v>599</v>
+        <v>603</v>
       </c>
       <c r="P4" s="12" t="s">
-        <v>600</v>
+        <v>604</v>
       </c>
       <c r="Q4" s="12" t="s">
-        <v>601</v>
+        <v>605</v>
       </c>
       <c r="R4" s="12" t="s">
-        <v>602</v>
+        <v>606</v>
       </c>
       <c r="S4" s="12" t="s">
-        <v>603</v>
+        <v>607</v>
       </c>
       <c r="T4" s="12" t="s">
-        <v>604</v>
+        <v>608</v>
       </c>
       <c r="U4" s="12" t="s">
-        <v>605</v>
+        <v>609</v>
       </c>
       <c r="V4" s="12" t="s">
-        <v>606</v>
+        <v>610</v>
       </c>
       <c r="W4" s="12" t="s">
-        <v>607</v>
+        <v>611</v>
       </c>
       <c r="X4" s="12" t="s">
-        <v>608</v>
+        <v>612</v>
       </c>
       <c r="Y4" s="12" t="s">
-        <v>609</v>
+        <v>613</v>
       </c>
       <c r="Z4" s="12" t="s">
-        <v>610</v>
+        <v>614</v>
       </c>
       <c r="AA4" s="12" t="s">
-        <v>611</v>
+        <v>615</v>
       </c>
       <c r="AB4" s="12" t="s">
-        <v>612</v>
+        <v>616</v>
       </c>
       <c r="AC4" s="12" t="s">
-        <v>613</v>
+        <v>617</v>
       </c>
       <c r="AD4" s="12" t="s">
-        <v>614</v>
+        <v>618</v>
       </c>
       <c r="AE4" s="12" t="s">
-        <v>615</v>
+        <v>619</v>
       </c>
       <c r="AF4" s="12" t="s">
-        <v>616</v>
+        <v>620</v>
       </c>
       <c r="AG4" s="12" t="s">
-        <v>617</v>
+        <v>621</v>
       </c>
       <c r="AH4" s="12" t="s">
-        <v>618</v>
+        <v>622</v>
       </c>
       <c r="AI4" s="12" t="s">
-        <v>619</v>
+        <v>623</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12661,16 +12696,16 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>620</v>
+        <v>624</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>621</v>
+        <v>625</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>48</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>339</v>
@@ -12795,16 +12830,16 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>622</v>
+        <v>626</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>621</v>
+        <v>625</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>43</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>339</v>
@@ -12929,16 +12964,16 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>623</v>
+        <v>627</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>621</v>
+        <v>625</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>52</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>339</v>
@@ -13063,16 +13098,16 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>624</v>
+        <v>628</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>621</v>
+        <v>625</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>54</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>339</v>
@@ -13197,16 +13232,16 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>625</v>
+        <v>629</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>626</v>
+        <v>630</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>48</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>339</v>
@@ -13331,16 +13366,16 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>627</v>
+        <v>631</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>626</v>
+        <v>630</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>43</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>339</v>
@@ -13465,16 +13500,16 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>628</v>
+        <v>632</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>626</v>
+        <v>630</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>52</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>339</v>
@@ -13599,16 +13634,16 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>629</v>
+        <v>633</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>626</v>
+        <v>630</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>54</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="E32" s="2" t="s">
         <v>339</v>
@@ -13733,16 +13768,16 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>630</v>
+        <v>634</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>631</v>
+        <v>635</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>48</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>339</v>
@@ -13867,16 +13902,16 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>632</v>
+        <v>636</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>633</v>
+        <v>637</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>43</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="E34" s="2" t="s">
         <v>339</v>
@@ -14001,7 +14036,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="28" t="s">
-        <v>459</v>
+        <v>463</v>
       </c>
       <c r="J35" s="33" t="n">
         <f aca="false">SUM(J5:J34)</f>
@@ -14066,7 +14101,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="28" t="s">
-        <v>634</v>
+        <v>638</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14078,10 +14113,10 @@
         <v>47</v>
       </c>
       <c r="D38" s="12" t="s">
-        <v>635</v>
+        <v>639</v>
       </c>
       <c r="E38" s="12" t="s">
-        <v>636</v>
+        <v>640</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14180,7 +14215,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>637</v>
+        <v>641</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14191,7 +14226,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="2" t="s">
-        <v>638</v>
+        <v>642</v>
       </c>
       <c r="C4" s="41" t="n">
         <f aca="false">SUMIFS(Channels!X5:X34,Channels!D5:D34,"Channel")</f>
@@ -14200,7 +14235,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="2" t="s">
-        <v>639</v>
+        <v>643</v>
       </c>
       <c r="C5" s="41" t="n">
         <f aca="false">SUMIFS(Channels!X5:X34,Channels!D5:D34,"Initiative")</f>
@@ -14209,7 +14244,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="2" t="s">
-        <v>640</v>
+        <v>644</v>
       </c>
       <c r="C6" s="41" t="n">
         <f aca="false">Channels!Y35</f>
@@ -14218,7 +14253,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="2" t="s">
-        <v>641</v>
+        <v>645</v>
       </c>
       <c r="C7" s="41" t="n">
         <f aca="false">C4+C5+C6</f>
@@ -14227,7 +14262,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="2" t="s">
-        <v>642</v>
+        <v>646</v>
       </c>
       <c r="C8" s="41" t="n">
         <f aca="false">Channels!Z35</f>
@@ -14236,7 +14271,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="2" t="s">
-        <v>643</v>
+        <v>647</v>
       </c>
       <c r="C9" s="41" t="n">
         <f aca="false">C7</f>
@@ -14245,7 +14280,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="2" t="s">
-        <v>644</v>
+        <v>648</v>
       </c>
       <c r="C10" s="41" t="n">
         <f aca="false">IF(Assumptions!$D$48&lt;1,C9/(1-Assumptions!$D$48)*Assumptions!$D$48,0)</f>
@@ -14254,7 +14289,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="2" t="s">
-        <v>645</v>
+        <v>649</v>
       </c>
       <c r="C11" s="41" t="n">
         <f aca="false">C9+C10</f>
@@ -14263,7 +14298,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="28" t="s">
-        <v>646</v>
+        <v>650</v>
       </c>
       <c r="C12" s="4" t="n">
         <f aca="false">IF(Assumptions!$D$51&gt;0,ROUNDUP(C11/Assumptions!$D$51,0)*Assumptions!$D$51,C11)</f>
@@ -14272,7 +14307,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="2" t="s">
-        <v>647</v>
+        <v>651</v>
       </c>
       <c r="C13" s="46" t="n">
         <f aca="false">MIN(Channels!U35,Funnel!B26)</f>
@@ -14281,7 +14316,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="2" t="s">
-        <v>648</v>
+        <v>652</v>
       </c>
       <c r="C14" s="47" t="n">
         <f aca="false">IF(C13&gt;0,C9/C13,0)</f>
@@ -14290,7 +14325,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="2" t="s">
-        <v>649</v>
+        <v>653</v>
       </c>
       <c r="C15" s="41" t="n">
         <f aca="false">IF(C13&gt;0,C12/C13,0)</f>
@@ -14299,7 +14334,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="2" t="s">
-        <v>650</v>
+        <v>654</v>
       </c>
       <c r="C16" s="30" t="n">
         <f aca="false">IF(C12&gt;0,Weekly!N5/C12,0)</f>
@@ -14308,7 +14343,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="28" t="s">
-        <v>651</v>
+        <v>655</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14317,25 +14352,25 @@
         <v>322</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>652</v>
+        <v>656</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>609</v>
+        <v>613</v>
       </c>
       <c r="E20" s="12" t="s">
-        <v>653</v>
+        <v>657</v>
       </c>
       <c r="F20" s="12" t="s">
-        <v>611</v>
+        <v>615</v>
       </c>
       <c r="G20" s="12" t="s">
-        <v>654</v>
+        <v>658</v>
       </c>
       <c r="H20" s="12" t="s">
-        <v>655</v>
+        <v>659</v>
       </c>
       <c r="I20" s="12" t="s">
-        <v>656</v>
+        <v>660</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14472,7 +14507,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="28" t="s">
-        <v>459</v>
+        <v>463</v>
       </c>
       <c r="C25" s="42" t="n">
         <f aca="false">SUM(C21:C24)</f>
@@ -14505,7 +14540,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="28" t="s">
-        <v>657</v>
+        <v>661</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14514,16 +14549,16 @@
         <v>321</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>611</v>
+        <v>615</v>
       </c>
       <c r="D28" s="12" t="s">
-        <v>654</v>
+        <v>658</v>
       </c>
       <c r="E28" s="12" t="s">
-        <v>655</v>
+        <v>659</v>
       </c>
       <c r="F28" s="12" t="s">
-        <v>658</v>
+        <v>662</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14654,7 +14689,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="2" t="s">
-        <v>621</v>
+        <v>625</v>
       </c>
       <c r="C35" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$AA$5:$AA$34,Channels!$B$5:$B$34,B35)</f>
@@ -14675,7 +14710,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="2" t="s">
-        <v>626</v>
+        <v>630</v>
       </c>
       <c r="C36" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$AA$5:$AA$34,Channels!$B$5:$B$34,B36)</f>
@@ -14696,7 +14731,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="2" t="s">
-        <v>631</v>
+        <v>635</v>
       </c>
       <c r="C37" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$AA$5:$AA$34,Channels!$B$5:$B$34,B37)</f>
@@ -14717,7 +14752,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="2" t="s">
-        <v>633</v>
+        <v>637</v>
       </c>
       <c r="C38" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$AA$5:$AA$34,Channels!$B$5:$B$34,B38)</f>
@@ -14738,7 +14773,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="28" t="s">
-        <v>459</v>
+        <v>463</v>
       </c>
       <c r="C39" s="42" t="n">
         <f aca="false">SUM(C29:C38)</f>
@@ -14757,7 +14792,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="28" t="s">
-        <v>659</v>
+        <v>663</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14769,10 +14804,10 @@
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="12"/>
       <c r="B44" s="12" t="s">
-        <v>660</v>
+        <v>664</v>
       </c>
       <c r="C44" s="12" t="s">
-        <v>661</v>
+        <v>665</v>
       </c>
       <c r="D44" s="12" t="s">
         <v>48</v>
@@ -14787,10 +14822,10 @@
         <v>54</v>
       </c>
       <c r="H44" s="12" t="s">
-        <v>662</v>
+        <v>666</v>
       </c>
       <c r="I44" s="12" t="s">
-        <v>655</v>
+        <v>659</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14863,17 +14898,17 @@
     </row>
     <row r="49" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="1" t="s">
-        <v>663</v>
+        <v>667</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="2" t="s">
-        <v>664</v>
+        <v>668</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E51" s="28" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="F51" s="48" t="n">
         <f aca="false">1</f>
@@ -14886,7 +14921,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E52" s="2" t="s">
-        <v>661</v>
+        <v>665</v>
       </c>
       <c r="F52" s="41" t="n">
         <f aca="false">Budget!$C$12*F51</f>
@@ -14899,7 +14934,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E53" s="2" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="F53" s="41" t="n">
         <f aca="false">F52*(1-Assumptions!$D$48)</f>
@@ -14912,7 +14947,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E54" s="2" t="s">
-        <v>667</v>
+        <v>671</v>
       </c>
       <c r="F54" s="41" t="n">
         <f aca="false">MAX(0,Budget!$C$9-F53)</f>
@@ -14925,44 +14960,44 @@
     </row>
     <row r="55" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="12" t="s">
-        <v>668</v>
+        <v>672</v>
       </c>
       <c r="B55" s="12" t="s">
         <v>322</v>
       </c>
       <c r="C55" s="12" t="s">
-        <v>669</v>
+        <v>673</v>
       </c>
       <c r="D55" s="12" t="s">
-        <v>670</v>
+        <v>674</v>
       </c>
       <c r="E55" s="12" t="s">
-        <v>654</v>
+        <v>658</v>
       </c>
       <c r="F55" s="12" t="s">
-        <v>671</v>
+        <v>675</v>
       </c>
       <c r="G55" s="12" t="s">
-        <v>672</v>
+        <v>676</v>
       </c>
       <c r="H55" s="12"/>
       <c r="I55" s="12"/>
       <c r="J55" s="12" t="s">
-        <v>673</v>
+        <v>677</v>
       </c>
       <c r="K55" s="12" t="s">
-        <v>674</v>
+        <v>678</v>
       </c>
       <c r="L55" s="12"/>
       <c r="M55" s="12"/>
       <c r="N55" s="12" t="s">
-        <v>652</v>
+        <v>656</v>
       </c>
       <c r="O55" s="12" t="s">
-        <v>675</v>
+        <v>679</v>
       </c>
       <c r="P55" s="12" t="s">
-        <v>676</v>
+        <v>680</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="1" collapsed="false">
@@ -16467,7 +16502,7 @@
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E86" s="28" t="s">
-        <v>677</v>
+        <v>681</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16524,7 +16559,7 @@
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E91" s="28" t="s">
-        <v>459</v>
+        <v>463</v>
       </c>
       <c r="F91" s="35" t="n">
         <f aca="false">SUM(F87:F90)</f>
@@ -16537,7 +16572,7 @@
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E92" s="2" t="s">
-        <v>655</v>
+        <v>659</v>
       </c>
       <c r="F92" s="41" t="n">
         <f aca="false">IF(F91&gt;0,F52/F91,0)</f>
@@ -16550,7 +16585,7 @@
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E94" s="2" t="s">
-        <v>678</v>
+        <v>682</v>
       </c>
       <c r="F94" s="32" t="n">
         <f aca="false">SUM(O56:O85)</f>
@@ -16563,7 +16598,7 @@
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E95" s="2" t="s">
-        <v>679</v>
+        <v>683</v>
       </c>
       <c r="F95" s="30" t="n">
         <f aca="false">IF(F94&gt;0,MIN(1,Funnel!$B$22/F94),1)</f>
@@ -16576,7 +16611,7 @@
     </row>
     <row r="97" customFormat="false" ht="407.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="13" t="s">
-        <v>680</v>
+        <v>684</v>
       </c>
     </row>
   </sheetData>
@@ -16609,113 +16644,113 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>681</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="344" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>685</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="508.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="13" t="s">
-        <v>682</v>
+        <v>686</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
-        <v>683</v>
+        <v>687</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>684</v>
+        <v>688</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>685</v>
+        <v>689</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>686</v>
+        <v>690</v>
       </c>
       <c r="E3" s="12" t="s">
-        <v>687</v>
+        <v>691</v>
       </c>
       <c r="F3" s="12" t="s">
-        <v>688</v>
+        <v>692</v>
       </c>
       <c r="G3" s="12" t="s">
-        <v>689</v>
+        <v>693</v>
       </c>
       <c r="H3" s="12" t="s">
-        <v>690</v>
+        <v>694</v>
       </c>
       <c r="I3" s="12" t="s">
-        <v>691</v>
+        <v>695</v>
       </c>
       <c r="J3" s="12" t="s">
-        <v>692</v>
+        <v>696</v>
       </c>
       <c r="K3" s="12" t="s">
-        <v>693</v>
+        <v>697</v>
       </c>
       <c r="L3" s="12" t="s">
-        <v>694</v>
+        <v>698</v>
       </c>
       <c r="M3" s="12" t="s">
-        <v>695</v>
+        <v>699</v>
       </c>
       <c r="N3" s="12" t="s">
-        <v>696</v>
+        <v>700</v>
       </c>
       <c r="O3" s="12" t="s">
-        <v>697</v>
+        <v>701</v>
       </c>
       <c r="P3" s="12" t="s">
-        <v>698</v>
+        <v>702</v>
       </c>
       <c r="Q3" s="12" t="s">
-        <v>699</v>
+        <v>703</v>
       </c>
       <c r="R3" s="12" t="s">
-        <v>700</v>
+        <v>704</v>
       </c>
       <c r="S3" s="12" t="s">
-        <v>701</v>
+        <v>705</v>
       </c>
       <c r="T3" s="12" t="s">
-        <v>702</v>
+        <v>706</v>
       </c>
       <c r="U3" s="12" t="s">
-        <v>703</v>
+        <v>707</v>
       </c>
       <c r="V3" s="12" t="s">
-        <v>704</v>
+        <v>708</v>
       </c>
       <c r="W3" s="12" t="s">
-        <v>705</v>
+        <v>709</v>
       </c>
       <c r="X3" s="12" t="s">
-        <v>706</v>
+        <v>710</v>
       </c>
       <c r="Y3" s="12" t="s">
-        <v>707</v>
+        <v>711</v>
       </c>
       <c r="Z3" s="49" t="s">
-        <v>708</v>
+        <v>712</v>
       </c>
       <c r="AA3" s="49" t="s">
-        <v>709</v>
+        <v>713</v>
       </c>
       <c r="AB3" s="49" t="s">
-        <v>710</v>
+        <v>714</v>
       </c>
       <c r="AC3" s="49" t="s">
-        <v>711</v>
+        <v>715</v>
       </c>
       <c r="AD3" s="49" t="s">
-        <v>712</v>
+        <v>716</v>
       </c>
       <c r="AE3" s="49" t="s">
-        <v>713</v>
+        <v>717</v>
       </c>
       <c r="AF3" s="49" t="s">
-        <v>714</v>
+        <v>718</v>
       </c>
       <c r="AG3" s="49" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16835,19 +16870,19 @@
         <v>0</v>
       </c>
       <c r="AD4" s="30" t="n">
-        <f aca="false">D4*IF(MAX(0,MIN(C4,Funnel!$B$19)-B4+1)&gt;0,MAX(0,MIN(C4,Funnel!$B$19)-MAX(B4,Assumptions!$D$7+Assumptions!$D$180)+1)/MAX(0,MIN(C4,Funnel!$B$19)-B4+1),0)</f>
+        <f aca="false">D4*IF(MAX(0,MIN(C4,Funnel!$B$19)-B4+1)&gt;0,MAX(0,MIN(C4,Funnel!$B$19)-MAX(B4,Assumptions!$D$7+Assumptions!$D$181)+1)/MAX(0,MIN(C4,Funnel!$B$19)-B4+1),0)</f>
         <v>0.180571428571429</v>
       </c>
       <c r="AE4" s="30" t="n">
-        <f aca="false">D4*IF(MAX(0,MIN(C4,Funnel!$B$19)-B4+1)&gt;0,MAX(0,MIN(C4,Funnel!$B$19)-MAX(B4,Assumptions!$D$7+Assumptions!$D$181)+1)/MAX(0,MIN(C4,Funnel!$B$19)-B4+1),0)</f>
+        <f aca="false">D4*IF(MAX(0,MIN(C4,Funnel!$B$19)-B4+1)&gt;0,MAX(0,MIN(C4,Funnel!$B$19)-MAX(B4,Assumptions!$D$7+Assumptions!$D$182)+1)/MAX(0,MIN(C4,Funnel!$B$19)-B4+1),0)</f>
         <v>0</v>
       </c>
       <c r="AF4" s="29" t="n">
-        <f aca="false">MAX(0,MIN(C4,Funnel!$B$19)-MAX(B4,Assumptions!$D$7+Assumptions!$D$180)+1)</f>
+        <f aca="false">MAX(0,MIN(C4,Funnel!$B$19)-MAX(B4,Assumptions!$D$7+Assumptions!$D$181)+1)</f>
         <v>4</v>
       </c>
       <c r="AG4" s="29" t="n">
-        <f aca="false">MAX(0,MIN(C4,Funnel!$B$19)-MAX(B4,Assumptions!$D$7+Assumptions!$D$181)+1)</f>
+        <f aca="false">MAX(0,MIN(C4,Funnel!$B$19)-MAX(B4,Assumptions!$D$7+Assumptions!$D$182)+1)</f>
         <v>0</v>
       </c>
     </row>
@@ -16968,19 +17003,19 @@
         <v>0.191520467836257</v>
       </c>
       <c r="AD5" s="30" t="n">
-        <f aca="false">D5*IF(MAX(0,MIN(C5,Funnel!$B$19)-B5+1)&gt;0,MAX(0,MIN(C5,Funnel!$B$19)-MAX(B5,Assumptions!$D$7+Assumptions!$D$180)+1)/MAX(0,MIN(C5,Funnel!$B$19)-B5+1),0)</f>
-        <v>0.131</v>
-      </c>
-      <c r="AE5" s="30" t="n">
         <f aca="false">D5*IF(MAX(0,MIN(C5,Funnel!$B$19)-B5+1)&gt;0,MAX(0,MIN(C5,Funnel!$B$19)-MAX(B5,Assumptions!$D$7+Assumptions!$D$181)+1)/MAX(0,MIN(C5,Funnel!$B$19)-B5+1),0)</f>
         <v>0.131</v>
       </c>
+      <c r="AE5" s="30" t="n">
+        <f aca="false">D5*IF(MAX(0,MIN(C5,Funnel!$B$19)-B5+1)&gt;0,MAX(0,MIN(C5,Funnel!$B$19)-MAX(B5,Assumptions!$D$7+Assumptions!$D$182)+1)/MAX(0,MIN(C5,Funnel!$B$19)-B5+1),0)</f>
+        <v>0.131</v>
+      </c>
       <c r="AF5" s="29" t="n">
-        <f aca="false">MAX(0,MIN(C5,Funnel!$B$19)-MAX(B5,Assumptions!$D$7+Assumptions!$D$180)+1)</f>
+        <f aca="false">MAX(0,MIN(C5,Funnel!$B$19)-MAX(B5,Assumptions!$D$7+Assumptions!$D$181)+1)</f>
         <v>7</v>
       </c>
       <c r="AG5" s="29" t="n">
-        <f aca="false">MAX(0,MIN(C5,Funnel!$B$19)-MAX(B5,Assumptions!$D$7+Assumptions!$D$181)+1)</f>
+        <f aca="false">MAX(0,MIN(C5,Funnel!$B$19)-MAX(B5,Assumptions!$D$7+Assumptions!$D$182)+1)</f>
         <v>7</v>
       </c>
     </row>
@@ -17101,19 +17136,19 @@
         <v>0.235380116959064</v>
       </c>
       <c r="AD6" s="30" t="n">
-        <f aca="false">D6*IF(MAX(0,MIN(C6,Funnel!$B$19)-B6+1)&gt;0,MAX(0,MIN(C6,Funnel!$B$19)-MAX(B6,Assumptions!$D$7+Assumptions!$D$180)+1)/MAX(0,MIN(C6,Funnel!$B$19)-B6+1),0)</f>
-        <v>0.161</v>
-      </c>
-      <c r="AE6" s="30" t="n">
         <f aca="false">D6*IF(MAX(0,MIN(C6,Funnel!$B$19)-B6+1)&gt;0,MAX(0,MIN(C6,Funnel!$B$19)-MAX(B6,Assumptions!$D$7+Assumptions!$D$181)+1)/MAX(0,MIN(C6,Funnel!$B$19)-B6+1),0)</f>
         <v>0.161</v>
       </c>
+      <c r="AE6" s="30" t="n">
+        <f aca="false">D6*IF(MAX(0,MIN(C6,Funnel!$B$19)-B6+1)&gt;0,MAX(0,MIN(C6,Funnel!$B$19)-MAX(B6,Assumptions!$D$7+Assumptions!$D$182)+1)/MAX(0,MIN(C6,Funnel!$B$19)-B6+1),0)</f>
+        <v>0.161</v>
+      </c>
       <c r="AF6" s="29" t="n">
-        <f aca="false">MAX(0,MIN(C6,Funnel!$B$19)-MAX(B6,Assumptions!$D$7+Assumptions!$D$180)+1)</f>
+        <f aca="false">MAX(0,MIN(C6,Funnel!$B$19)-MAX(B6,Assumptions!$D$7+Assumptions!$D$181)+1)</f>
         <v>7</v>
       </c>
       <c r="AG6" s="29" t="n">
-        <f aca="false">MAX(0,MIN(C6,Funnel!$B$19)-MAX(B6,Assumptions!$D$7+Assumptions!$D$181)+1)</f>
+        <f aca="false">MAX(0,MIN(C6,Funnel!$B$19)-MAX(B6,Assumptions!$D$7+Assumptions!$D$182)+1)</f>
         <v>7</v>
       </c>
     </row>
@@ -17234,19 +17269,19 @@
         <v>0.248538011695906</v>
       </c>
       <c r="AD7" s="30" t="n">
-        <f aca="false">D7*IF(MAX(0,MIN(C7,Funnel!$B$19)-B7+1)&gt;0,MAX(0,MIN(C7,Funnel!$B$19)-MAX(B7,Assumptions!$D$7+Assumptions!$D$180)+1)/MAX(0,MIN(C7,Funnel!$B$19)-B7+1),0)</f>
-        <v>0.17</v>
-      </c>
-      <c r="AE7" s="30" t="n">
         <f aca="false">D7*IF(MAX(0,MIN(C7,Funnel!$B$19)-B7+1)&gt;0,MAX(0,MIN(C7,Funnel!$B$19)-MAX(B7,Assumptions!$D$7+Assumptions!$D$181)+1)/MAX(0,MIN(C7,Funnel!$B$19)-B7+1),0)</f>
         <v>0.17</v>
       </c>
+      <c r="AE7" s="30" t="n">
+        <f aca="false">D7*IF(MAX(0,MIN(C7,Funnel!$B$19)-B7+1)&gt;0,MAX(0,MIN(C7,Funnel!$B$19)-MAX(B7,Assumptions!$D$7+Assumptions!$D$182)+1)/MAX(0,MIN(C7,Funnel!$B$19)-B7+1),0)</f>
+        <v>0.17</v>
+      </c>
       <c r="AF7" s="29" t="n">
-        <f aca="false">MAX(0,MIN(C7,Funnel!$B$19)-MAX(B7,Assumptions!$D$7+Assumptions!$D$180)+1)</f>
+        <f aca="false">MAX(0,MIN(C7,Funnel!$B$19)-MAX(B7,Assumptions!$D$7+Assumptions!$D$181)+1)</f>
         <v>7</v>
       </c>
       <c r="AG7" s="29" t="n">
-        <f aca="false">MAX(0,MIN(C7,Funnel!$B$19)-MAX(B7,Assumptions!$D$7+Assumptions!$D$181)+1)</f>
+        <f aca="false">MAX(0,MIN(C7,Funnel!$B$19)-MAX(B7,Assumptions!$D$7+Assumptions!$D$182)+1)</f>
         <v>7</v>
       </c>
     </row>
@@ -17367,19 +17402,19 @@
         <v>0.285087719298246</v>
       </c>
       <c r="AD8" s="30" t="n">
-        <f aca="false">D8*IF(MAX(0,MIN(C8,Funnel!$B$19)-B8+1)&gt;0,MAX(0,MIN(C8,Funnel!$B$19)-MAX(B8,Assumptions!$D$7+Assumptions!$D$180)+1)/MAX(0,MIN(C8,Funnel!$B$19)-B8+1),0)</f>
-        <v>0.195</v>
-      </c>
-      <c r="AE8" s="30" t="n">
         <f aca="false">D8*IF(MAX(0,MIN(C8,Funnel!$B$19)-B8+1)&gt;0,MAX(0,MIN(C8,Funnel!$B$19)-MAX(B8,Assumptions!$D$7+Assumptions!$D$181)+1)/MAX(0,MIN(C8,Funnel!$B$19)-B8+1),0)</f>
         <v>0.195</v>
       </c>
+      <c r="AE8" s="30" t="n">
+        <f aca="false">D8*IF(MAX(0,MIN(C8,Funnel!$B$19)-B8+1)&gt;0,MAX(0,MIN(C8,Funnel!$B$19)-MAX(B8,Assumptions!$D$7+Assumptions!$D$182)+1)/MAX(0,MIN(C8,Funnel!$B$19)-B8+1),0)</f>
+        <v>0.195</v>
+      </c>
       <c r="AF8" s="29" t="n">
-        <f aca="false">MAX(0,MIN(C8,Funnel!$B$19)-MAX(B8,Assumptions!$D$7+Assumptions!$D$180)+1)</f>
+        <f aca="false">MAX(0,MIN(C8,Funnel!$B$19)-MAX(B8,Assumptions!$D$7+Assumptions!$D$181)+1)</f>
         <v>7</v>
       </c>
       <c r="AG8" s="29" t="n">
-        <f aca="false">MAX(0,MIN(C8,Funnel!$B$19)-MAX(B8,Assumptions!$D$7+Assumptions!$D$181)+1)</f>
+        <f aca="false">MAX(0,MIN(C8,Funnel!$B$19)-MAX(B8,Assumptions!$D$7+Assumptions!$D$182)+1)</f>
         <v>7</v>
       </c>
     </row>
@@ -17500,19 +17535,19 @@
         <v>0.0394736842105263</v>
       </c>
       <c r="AD9" s="30" t="n">
-        <f aca="false">D9*IF(MAX(0,MIN(C9,Funnel!$B$19)-B9+1)&gt;0,MAX(0,MIN(C9,Funnel!$B$19)-MAX(B9,Assumptions!$D$7+Assumptions!$D$180)+1)/MAX(0,MIN(C9,Funnel!$B$19)-B9+1),0)</f>
-        <v>0.027</v>
-      </c>
-      <c r="AE9" s="30" t="n">
         <f aca="false">D9*IF(MAX(0,MIN(C9,Funnel!$B$19)-B9+1)&gt;0,MAX(0,MIN(C9,Funnel!$B$19)-MAX(B9,Assumptions!$D$7+Assumptions!$D$181)+1)/MAX(0,MIN(C9,Funnel!$B$19)-B9+1),0)</f>
         <v>0.027</v>
       </c>
+      <c r="AE9" s="30" t="n">
+        <f aca="false">D9*IF(MAX(0,MIN(C9,Funnel!$B$19)-B9+1)&gt;0,MAX(0,MIN(C9,Funnel!$B$19)-MAX(B9,Assumptions!$D$7+Assumptions!$D$182)+1)/MAX(0,MIN(C9,Funnel!$B$19)-B9+1),0)</f>
+        <v>0.027</v>
+      </c>
       <c r="AF9" s="29" t="n">
-        <f aca="false">MAX(0,MIN(C9,Funnel!$B$19)-MAX(B9,Assumptions!$D$7+Assumptions!$D$180)+1)</f>
+        <f aca="false">MAX(0,MIN(C9,Funnel!$B$19)-MAX(B9,Assumptions!$D$7+Assumptions!$D$181)+1)</f>
         <v>1</v>
       </c>
       <c r="AG9" s="29" t="n">
-        <f aca="false">MAX(0,MIN(C9,Funnel!$B$19)-MAX(B9,Assumptions!$D$7+Assumptions!$D$181)+1)</f>
+        <f aca="false">MAX(0,MIN(C9,Funnel!$B$19)-MAX(B9,Assumptions!$D$7+Assumptions!$D$182)+1)</f>
         <v>1</v>
       </c>
     </row>
@@ -17633,19 +17668,19 @@
         <v>0</v>
       </c>
       <c r="AD10" s="30" t="n">
-        <f aca="false">D10*IF(MAX(0,MIN(C10,Funnel!$B$19)-B10+1)&gt;0,MAX(0,MIN(C10,Funnel!$B$19)-MAX(B10,Assumptions!$D$7+Assumptions!$D$180)+1)/MAX(0,MIN(C10,Funnel!$B$19)-B10+1),0)</f>
+        <f aca="false">D10*IF(MAX(0,MIN(C10,Funnel!$B$19)-B10+1)&gt;0,MAX(0,MIN(C10,Funnel!$B$19)-MAX(B10,Assumptions!$D$7+Assumptions!$D$181)+1)/MAX(0,MIN(C10,Funnel!$B$19)-B10+1),0)</f>
         <v>0</v>
       </c>
       <c r="AE10" s="30" t="n">
-        <f aca="false">D10*IF(MAX(0,MIN(C10,Funnel!$B$19)-B10+1)&gt;0,MAX(0,MIN(C10,Funnel!$B$19)-MAX(B10,Assumptions!$D$7+Assumptions!$D$181)+1)/MAX(0,MIN(C10,Funnel!$B$19)-B10+1),0)</f>
+        <f aca="false">D10*IF(MAX(0,MIN(C10,Funnel!$B$19)-B10+1)&gt;0,MAX(0,MIN(C10,Funnel!$B$19)-MAX(B10,Assumptions!$D$7+Assumptions!$D$182)+1)/MAX(0,MIN(C10,Funnel!$B$19)-B10+1),0)</f>
         <v>0</v>
       </c>
       <c r="AF10" s="29" t="n">
-        <f aca="false">MAX(0,MIN(C10,Funnel!$B$19)-MAX(B10,Assumptions!$D$7+Assumptions!$D$180)+1)</f>
+        <f aca="false">MAX(0,MIN(C10,Funnel!$B$19)-MAX(B10,Assumptions!$D$7+Assumptions!$D$181)+1)</f>
         <v>0</v>
       </c>
       <c r="AG10" s="29" t="n">
-        <f aca="false">MAX(0,MIN(C10,Funnel!$B$19)-MAX(B10,Assumptions!$D$7+Assumptions!$D$181)+1)</f>
+        <f aca="false">MAX(0,MIN(C10,Funnel!$B$19)-MAX(B10,Assumptions!$D$7+Assumptions!$D$182)+1)</f>
         <v>0</v>
       </c>
     </row>
@@ -17766,19 +17801,19 @@
         <v>0</v>
       </c>
       <c r="AD11" s="30" t="n">
-        <f aca="false">D11*IF(MAX(0,MIN(C11,Funnel!$B$19)-B11+1)&gt;0,MAX(0,MIN(C11,Funnel!$B$19)-MAX(B11,Assumptions!$D$7+Assumptions!$D$180)+1)/MAX(0,MIN(C11,Funnel!$B$19)-B11+1),0)</f>
+        <f aca="false">D11*IF(MAX(0,MIN(C11,Funnel!$B$19)-B11+1)&gt;0,MAX(0,MIN(C11,Funnel!$B$19)-MAX(B11,Assumptions!$D$7+Assumptions!$D$181)+1)/MAX(0,MIN(C11,Funnel!$B$19)-B11+1),0)</f>
         <v>0</v>
       </c>
       <c r="AE11" s="30" t="n">
-        <f aca="false">D11*IF(MAX(0,MIN(C11,Funnel!$B$19)-B11+1)&gt;0,MAX(0,MIN(C11,Funnel!$B$19)-MAX(B11,Assumptions!$D$7+Assumptions!$D$181)+1)/MAX(0,MIN(C11,Funnel!$B$19)-B11+1),0)</f>
+        <f aca="false">D11*IF(MAX(0,MIN(C11,Funnel!$B$19)-B11+1)&gt;0,MAX(0,MIN(C11,Funnel!$B$19)-MAX(B11,Assumptions!$D$7+Assumptions!$D$182)+1)/MAX(0,MIN(C11,Funnel!$B$19)-B11+1),0)</f>
         <v>0</v>
       </c>
       <c r="AF11" s="29" t="n">
-        <f aca="false">MAX(0,MIN(C11,Funnel!$B$19)-MAX(B11,Assumptions!$D$7+Assumptions!$D$180)+1)</f>
+        <f aca="false">MAX(0,MIN(C11,Funnel!$B$19)-MAX(B11,Assumptions!$D$7+Assumptions!$D$181)+1)</f>
         <v>0</v>
       </c>
       <c r="AG11" s="29" t="n">
-        <f aca="false">MAX(0,MIN(C11,Funnel!$B$19)-MAX(B11,Assumptions!$D$7+Assumptions!$D$181)+1)</f>
+        <f aca="false">MAX(0,MIN(C11,Funnel!$B$19)-MAX(B11,Assumptions!$D$7+Assumptions!$D$182)+1)</f>
         <v>0</v>
       </c>
     </row>
@@ -17899,19 +17934,19 @@
         <v>0</v>
       </c>
       <c r="AD12" s="30" t="n">
-        <f aca="false">D12*IF(MAX(0,MIN(C12,Funnel!$B$19)-B12+1)&gt;0,MAX(0,MIN(C12,Funnel!$B$19)-MAX(B12,Assumptions!$D$7+Assumptions!$D$180)+1)/MAX(0,MIN(C12,Funnel!$B$19)-B12+1),0)</f>
+        <f aca="false">D12*IF(MAX(0,MIN(C12,Funnel!$B$19)-B12+1)&gt;0,MAX(0,MIN(C12,Funnel!$B$19)-MAX(B12,Assumptions!$D$7+Assumptions!$D$181)+1)/MAX(0,MIN(C12,Funnel!$B$19)-B12+1),0)</f>
         <v>0</v>
       </c>
       <c r="AE12" s="30" t="n">
-        <f aca="false">D12*IF(MAX(0,MIN(C12,Funnel!$B$19)-B12+1)&gt;0,MAX(0,MIN(C12,Funnel!$B$19)-MAX(B12,Assumptions!$D$7+Assumptions!$D$181)+1)/MAX(0,MIN(C12,Funnel!$B$19)-B12+1),0)</f>
+        <f aca="false">D12*IF(MAX(0,MIN(C12,Funnel!$B$19)-B12+1)&gt;0,MAX(0,MIN(C12,Funnel!$B$19)-MAX(B12,Assumptions!$D$7+Assumptions!$D$182)+1)/MAX(0,MIN(C12,Funnel!$B$19)-B12+1),0)</f>
         <v>0</v>
       </c>
       <c r="AF12" s="29" t="n">
-        <f aca="false">MAX(0,MIN(C12,Funnel!$B$19)-MAX(B12,Assumptions!$D$7+Assumptions!$D$180)+1)</f>
+        <f aca="false">MAX(0,MIN(C12,Funnel!$B$19)-MAX(B12,Assumptions!$D$7+Assumptions!$D$181)+1)</f>
         <v>0</v>
       </c>
       <c r="AG12" s="29" t="n">
-        <f aca="false">MAX(0,MIN(C12,Funnel!$B$19)-MAX(B12,Assumptions!$D$7+Assumptions!$D$181)+1)</f>
+        <f aca="false">MAX(0,MIN(C12,Funnel!$B$19)-MAX(B12,Assumptions!$D$7+Assumptions!$D$182)+1)</f>
         <v>0</v>
       </c>
     </row>
@@ -18032,19 +18067,19 @@
         <v>0</v>
       </c>
       <c r="AD13" s="30" t="n">
-        <f aca="false">D13*IF(MAX(0,MIN(C13,Funnel!$B$19)-B13+1)&gt;0,MAX(0,MIN(C13,Funnel!$B$19)-MAX(B13,Assumptions!$D$7+Assumptions!$D$180)+1)/MAX(0,MIN(C13,Funnel!$B$19)-B13+1),0)</f>
+        <f aca="false">D13*IF(MAX(0,MIN(C13,Funnel!$B$19)-B13+1)&gt;0,MAX(0,MIN(C13,Funnel!$B$19)-MAX(B13,Assumptions!$D$7+Assumptions!$D$181)+1)/MAX(0,MIN(C13,Funnel!$B$19)-B13+1),0)</f>
         <v>0</v>
       </c>
       <c r="AE13" s="30" t="n">
-        <f aca="false">D13*IF(MAX(0,MIN(C13,Funnel!$B$19)-B13+1)&gt;0,MAX(0,MIN(C13,Funnel!$B$19)-MAX(B13,Assumptions!$D$7+Assumptions!$D$181)+1)/MAX(0,MIN(C13,Funnel!$B$19)-B13+1),0)</f>
+        <f aca="false">D13*IF(MAX(0,MIN(C13,Funnel!$B$19)-B13+1)&gt;0,MAX(0,MIN(C13,Funnel!$B$19)-MAX(B13,Assumptions!$D$7+Assumptions!$D$182)+1)/MAX(0,MIN(C13,Funnel!$B$19)-B13+1),0)</f>
         <v>0</v>
       </c>
       <c r="AF13" s="29" t="n">
-        <f aca="false">MAX(0,MIN(C13,Funnel!$B$19)-MAX(B13,Assumptions!$D$7+Assumptions!$D$180)+1)</f>
+        <f aca="false">MAX(0,MIN(C13,Funnel!$B$19)-MAX(B13,Assumptions!$D$7+Assumptions!$D$181)+1)</f>
         <v>0</v>
       </c>
       <c r="AG13" s="29" t="n">
-        <f aca="false">MAX(0,MIN(C13,Funnel!$B$19)-MAX(B13,Assumptions!$D$7+Assumptions!$D$181)+1)</f>
+        <f aca="false">MAX(0,MIN(C13,Funnel!$B$19)-MAX(B13,Assumptions!$D$7+Assumptions!$D$182)+1)</f>
         <v>0</v>
       </c>
     </row>
@@ -18165,25 +18200,25 @@
         <v>0</v>
       </c>
       <c r="AD14" s="30" t="n">
-        <f aca="false">D14*IF(MAX(0,MIN(C14,Funnel!$B$19)-B14+1)&gt;0,MAX(0,MIN(C14,Funnel!$B$19)-MAX(B14,Assumptions!$D$7+Assumptions!$D$180)+1)/MAX(0,MIN(C14,Funnel!$B$19)-B14+1),0)</f>
+        <f aca="false">D14*IF(MAX(0,MIN(C14,Funnel!$B$19)-B14+1)&gt;0,MAX(0,MIN(C14,Funnel!$B$19)-MAX(B14,Assumptions!$D$7+Assumptions!$D$181)+1)/MAX(0,MIN(C14,Funnel!$B$19)-B14+1),0)</f>
         <v>0</v>
       </c>
       <c r="AE14" s="30" t="n">
-        <f aca="false">D14*IF(MAX(0,MIN(C14,Funnel!$B$19)-B14+1)&gt;0,MAX(0,MIN(C14,Funnel!$B$19)-MAX(B14,Assumptions!$D$7+Assumptions!$D$181)+1)/MAX(0,MIN(C14,Funnel!$B$19)-B14+1),0)</f>
+        <f aca="false">D14*IF(MAX(0,MIN(C14,Funnel!$B$19)-B14+1)&gt;0,MAX(0,MIN(C14,Funnel!$B$19)-MAX(B14,Assumptions!$D$7+Assumptions!$D$182)+1)/MAX(0,MIN(C14,Funnel!$B$19)-B14+1),0)</f>
         <v>0</v>
       </c>
       <c r="AF14" s="29" t="n">
-        <f aca="false">MAX(0,MIN(C14,Funnel!$B$19)-MAX(B14,Assumptions!$D$7+Assumptions!$D$180)+1)</f>
+        <f aca="false">MAX(0,MIN(C14,Funnel!$B$19)-MAX(B14,Assumptions!$D$7+Assumptions!$D$181)+1)</f>
         <v>0</v>
       </c>
       <c r="AG14" s="29" t="n">
-        <f aca="false">MAX(0,MIN(C14,Funnel!$B$19)-MAX(B14,Assumptions!$D$7+Assumptions!$D$181)+1)</f>
+        <f aca="false">MAX(0,MIN(C14,Funnel!$B$19)-MAX(B14,Assumptions!$D$7+Assumptions!$D$182)+1)</f>
         <v>0</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="28" t="s">
-        <v>459</v>
+        <v>463</v>
       </c>
       <c r="D15" s="51" t="n">
         <f aca="false">SUM(D4:D14)</f>
@@ -18268,7 +18303,7 @@
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="B16" s="9"/>
       <c r="C16" s="9"/>
@@ -18320,22 +18355,22 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="28" t="s">
-        <v>717</v>
+        <v>721</v>
       </c>
       <c r="H18" s="28" t="s">
-        <v>718</v>
+        <v>722</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="2" t="s">
-        <v>719</v>
+        <v>723</v>
       </c>
       <c r="F19" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$C$5:$C$34,"&lt;&gt;Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot",Channels!$B$5:$B$34,"&lt;&gt;I1b Employee referral sprint (bonus on hire)",Channels!$B$5:$B$34,"&lt;&gt;I1a Talent rediscovery (past applicants in ATS)")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
         <v>62640.1522284802</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>720</v>
+        <v>724</v>
       </c>
       <c r="L19" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,"I2 Handwerk → Industrie (construction electricians)")</f>
@@ -18344,14 +18379,14 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="2" t="s">
-        <v>721</v>
+        <v>725</v>
       </c>
       <c r="F20" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$C$5:$C$34,"Supervisors",Channels!$E$5:$E$34,"&lt;&gt;Slot",Channels!$B$5:$B$34,"&lt;&gt;I1b Employee referral sprint (bonus on hire)",Channels!$B$5:$B$34,"&lt;&gt;I1a Talent rediscovery (past applicants in ATS)")-SUMIFS(Channels!$Z$5:$Z$34,Channels!$C$5:$C$34,"Supervisors")</f>
         <v>12178.6678273933</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>722</v>
+        <v>726</v>
       </c>
       <c r="L20" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$W$5:$W$34,Channels!$B$5:$B$34,"I2 Handwerk → Industrie (construction electricians)")</f>
@@ -18360,14 +18395,14 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="2" t="s">
-        <v>723</v>
+        <v>727</v>
       </c>
       <c r="F21" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$E$5:$E$34,"Slot")</f>
         <v>5796</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>724</v>
+        <v>728</v>
       </c>
       <c r="L21" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$V$5:$V$34,Channels!$B$5:$B$34,"I2 Handwerk → Industrie (construction electricians)")</f>
@@ -18376,14 +18411,14 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="2" t="s">
-        <v>725</v>
+        <v>729</v>
       </c>
       <c r="F22" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,"I1b Employee referral sprint (bonus on hire)",Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
         <v>9869.2425</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>726</v>
+        <v>730</v>
       </c>
       <c r="L22" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$U$5:$U$34,Channels!$B$5:$B$34,"I2 Handwerk → Industrie (construction electricians)")</f>
@@ -18392,14 +18427,14 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="2" t="s">
-        <v>727</v>
+        <v>731</v>
       </c>
       <c r="F23" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,"I1b Employee referral sprint (bonus on hire)",Channels!$C$5:$C$34,"Supervisors")</f>
         <v>1108.485</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>728</v>
+        <v>732</v>
       </c>
       <c r="L23" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,"I3 Polish border corridor + PL pre-screener")</f>
@@ -18408,14 +18443,14 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="2" t="s">
-        <v>729</v>
+        <v>733</v>
       </c>
       <c r="F24" s="41" t="n">
         <f aca="false">SUM(Channels!$Z$5:$Z$34)</f>
         <v>9000</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>730</v>
+        <v>734</v>
       </c>
       <c r="L24" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$W$5:$W$34,Channels!$B$5:$B$34,"I3 Polish border corridor + PL pre-screener")</f>
@@ -18424,14 +18459,14 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="2" t="s">
-        <v>731</v>
+        <v>735</v>
       </c>
       <c r="F25" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$AF$5:$AF$34,Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
         <v>8.9323002511364</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>732</v>
+        <v>736</v>
       </c>
       <c r="L25" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$V$5:$V$34,Channels!$B$5:$B$34,"I3 Polish border corridor + PL pre-screener")</f>
@@ -18440,14 +18475,14 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="2" t="s">
-        <v>733</v>
+        <v>737</v>
       </c>
       <c r="F26" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$AF$5:$AF$34,Channels!$C$5:$C$34,"Supervisors")</f>
         <v>3.25605421987231</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>734</v>
+        <v>738</v>
       </c>
       <c r="L26" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$U$5:$U$34,Channels!$B$5:$B$34,"I3 Polish border corridor + PL pre-screener")</f>
@@ -18456,7 +18491,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="2" t="s">
-        <v>735</v>
+        <v>739</v>
       </c>
       <c r="F27" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$AE$5:$AE$34,Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
@@ -18465,7 +18500,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="2" t="s">
-        <v>736</v>
+        <v>740</v>
       </c>
       <c r="F28" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$AE$5:$AE$34,Channels!$C$5:$C$34,"Supervisors")</f>
@@ -18474,7 +18509,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="2" t="s">
-        <v>737</v>
+        <v>741</v>
       </c>
       <c r="F29" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$AG$5:$AG$34,Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
@@ -18483,7 +18518,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="2" t="s">
-        <v>738</v>
+        <v>742</v>
       </c>
       <c r="F30" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$AG$5:$AG$34,Channels!$C$5:$C$34,"Supervisors")</f>
@@ -18492,7 +18527,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="2" t="s">
-        <v>739</v>
+        <v>743</v>
       </c>
       <c r="F31" s="41" t="n">
         <f aca="false">SUMIFS(Channels!$X$5:$X$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)")</f>
@@ -18501,7 +18536,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="2" t="s">
-        <v>740</v>
+        <v>744</v>
       </c>
       <c r="F32" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$V$5:$V$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)",Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
@@ -18510,7 +18545,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="2" t="s">
-        <v>741</v>
+        <v>745</v>
       </c>
       <c r="F33" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$V$5:$V$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)",Channels!$C$5:$C$34,"Supervisors")</f>
@@ -18519,7 +18554,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="2" t="s">
-        <v>742</v>
+        <v>746</v>
       </c>
       <c r="F34" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$W$5:$W$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)",Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
@@ -18528,7 +18563,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="2" t="s">
-        <v>743</v>
+        <v>747</v>
       </c>
       <c r="F35" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$W$5:$W$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)",Channels!$C$5:$C$34,"Supervisors")</f>
@@ -18537,7 +18572,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="2" t="s">
-        <v>744</v>
+        <v>748</v>
       </c>
       <c r="F36" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$U$5:$U$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)",Channels!$C$5:$C$34,"&lt;&gt;Supervisors")</f>
@@ -18546,7 +18581,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="2" t="s">
-        <v>745</v>
+        <v>749</v>
       </c>
       <c r="F37" s="32" t="n">
         <f aca="false">SUMIFS(Channels!$U$5:$U$34,Channels!$B$5:$B$34,"I1a Talent rediscovery (past applicants in ATS)",Channels!$C$5:$C$34,"Supervisors")</f>
@@ -18555,7 +18590,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="2" t="s">
-        <v>746</v>
+        <v>750</v>
       </c>
       <c r="F38" s="30" t="n">
         <f aca="false">IF(Funnel!B23&gt;0,MIN(1,Funnel!B22/Funnel!B23),1)</f>
@@ -18564,7 +18599,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="28" t="s">
-        <v>747</v>
+        <v>751</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18573,40 +18608,40 @@
         <v>321</v>
       </c>
       <c r="C43" s="12" t="s">
-        <v>748</v>
+        <v>752</v>
       </c>
       <c r="D43" s="12" t="s">
-        <v>749</v>
+        <v>753</v>
       </c>
       <c r="E43" s="12" t="s">
-        <v>750</v>
+        <v>754</v>
       </c>
       <c r="F43" s="12" t="s">
-        <v>751</v>
+        <v>755</v>
       </c>
       <c r="G43" s="12" t="s">
-        <v>752</v>
+        <v>756</v>
       </c>
       <c r="H43" s="12" t="s">
-        <v>753</v>
+        <v>757</v>
       </c>
       <c r="I43" s="12" t="s">
-        <v>754</v>
+        <v>758</v>
       </c>
       <c r="J43" s="12" t="s">
-        <v>755</v>
+        <v>759</v>
       </c>
       <c r="K43" s="12" t="s">
-        <v>756</v>
+        <v>760</v>
       </c>
       <c r="L43" s="12" t="s">
-        <v>757</v>
+        <v>761</v>
       </c>
       <c r="M43" s="12" t="s">
-        <v>758</v>
+        <v>762</v>
       </c>
       <c r="N43" s="12" t="s">
-        <v>459</v>
+        <v>463</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19151,7 +19186,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B54" s="28" t="s">
-        <v>459</v>
+        <v>463</v>
       </c>
       <c r="C54" s="42" t="n">
         <f aca="false">SUM(C44:C53)</f>
@@ -19241,12 +19276,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>759</v>
+        <v>763</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>760</v>
+        <v>764</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -19260,76 +19295,76 @@
         <v>322</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>761</v>
+        <v>765</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>762</v>
+        <v>766</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>763</v>
+        <v>767</v>
       </c>
       <c r="G4" s="12" t="s">
-        <v>764</v>
+        <v>768</v>
       </c>
       <c r="H4" s="12" t="s">
-        <v>765</v>
+        <v>769</v>
       </c>
       <c r="I4" s="12" t="s">
-        <v>766</v>
+        <v>770</v>
       </c>
       <c r="J4" s="12" t="s">
-        <v>767</v>
+        <v>771</v>
       </c>
       <c r="K4" s="12" t="s">
-        <v>768</v>
+        <v>772</v>
       </c>
       <c r="L4" s="12" t="s">
-        <v>769</v>
+        <v>773</v>
       </c>
       <c r="M4" s="12" t="s">
-        <v>770</v>
+        <v>774</v>
       </c>
       <c r="N4" s="12" t="s">
-        <v>771</v>
+        <v>775</v>
       </c>
       <c r="O4" s="12" t="s">
-        <v>772</v>
+        <v>776</v>
       </c>
       <c r="P4" s="12" t="s">
-        <v>773</v>
+        <v>777</v>
       </c>
       <c r="Q4" s="12" t="s">
-        <v>774</v>
+        <v>778</v>
       </c>
       <c r="R4" s="12" t="s">
-        <v>775</v>
+        <v>779</v>
       </c>
       <c r="S4" s="12" t="s">
-        <v>776</v>
+        <v>780</v>
       </c>
       <c r="T4" s="12" t="s">
-        <v>777</v>
+        <v>781</v>
       </c>
       <c r="U4" s="12" t="s">
-        <v>778</v>
+        <v>782</v>
       </c>
       <c r="V4" s="12" t="s">
-        <v>779</v>
+        <v>783</v>
       </c>
       <c r="W4" s="12" t="s">
-        <v>780</v>
+        <v>784</v>
       </c>
       <c r="X4" s="12" t="s">
-        <v>781</v>
+        <v>785</v>
       </c>
       <c r="Y4" s="12" t="s">
-        <v>782</v>
+        <v>786</v>
       </c>
       <c r="Z4" s="12" t="s">
-        <v>783</v>
+        <v>787</v>
       </c>
       <c r="AA4" s="12" t="s">
-        <v>784</v>
+        <v>788</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21734,7 +21769,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="28" t="s">
-        <v>459</v>
+        <v>463</v>
       </c>
       <c r="G35" s="42" t="n">
         <f aca="false">SUM(G5:G34)</f>
@@ -21795,7 +21830,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="28" t="s">
-        <v>785</v>
+        <v>789</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -21804,46 +21839,46 @@
         <v>322</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>786</v>
+        <v>790</v>
       </c>
       <c r="D39" s="12" t="s">
-        <v>787</v>
+        <v>791</v>
       </c>
       <c r="E39" s="12" t="s">
-        <v>788</v>
+        <v>792</v>
       </c>
       <c r="F39" s="12" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="G39" s="12" t="s">
-        <v>790</v>
+        <v>794</v>
       </c>
       <c r="H39" s="12" t="s">
-        <v>791</v>
+        <v>795</v>
       </c>
       <c r="I39" s="12" t="s">
-        <v>792</v>
+        <v>796</v>
       </c>
       <c r="J39" s="12" t="s">
-        <v>793</v>
+        <v>797</v>
       </c>
       <c r="K39" s="12" t="s">
-        <v>794</v>
+        <v>798</v>
       </c>
       <c r="L39" s="12" t="s">
-        <v>795</v>
+        <v>799</v>
       </c>
       <c r="M39" s="12" t="s">
-        <v>796</v>
+        <v>800</v>
       </c>
       <c r="N39" s="12" t="s">
-        <v>797</v>
+        <v>801</v>
       </c>
       <c r="O39" s="12" t="s">
         <v>47</v>
       </c>
       <c r="P39" s="12" t="s">
-        <v>798</v>
+        <v>802</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22032,7 +22067,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="28" t="s">
-        <v>459</v>
+        <v>463</v>
       </c>
       <c r="C44" s="35" t="n">
         <f aca="false">SUM(C40:C43)</f>
@@ -22073,7 +22108,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="9" t="s">
-        <v>799</v>
+        <v>803</v>
       </c>
       <c r="B46" s="9"/>
       <c r="C46" s="9"/>

</xml_diff>

<commit_message>
Final evaluator points: T2 label matches note, referral downside on slide 7, bridge-course trainer time stated; Q&A figures aligned
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V2NJtrYy3bzNxqKeiRXJfY
</commit_message>
<xml_diff>
--- a/operation_uptime/Operation_Uptime_Model.xlsx
+++ b/operation_uptime/Operation_Uptime_Model.xlsx
@@ -239,57 +239,57 @@
     <t xml:space="preserve">Days: application → recruiter assessment of a qualified applicant</t>
   </si>
   <si>
+    <t xml:space="preserve">Own estimate: SmartRecruiters 2025 global median is 6 days to review (Germany 8); I assume the client keeps the global pace, an ask. Slide 1 shows the German-pace downside (~92 hires). https://ta.smartrecruiters.com/rs/664-NIC-529/images/Germany%20Recruiting%20Benchmarks%202025%20Report%20DE.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Days: recruiter assessment → technical interview/test done</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Own estimate: global median 14 days application → interview minus the 6 above (Germany 20 − 8 = 12); same commitment as T2. https://ta.smartrecruiters.com/rs/664-NIC-529/images/Germany%20Recruiting%20Benchmarks%202025%20Report%20DE.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Days: interview → written offer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">My ask to the client: written offer within 3 days of the interview. No public benchmark exists for this step.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Days: offer → signed contract</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One-week offer validity; candidates take ~9 days on average to decide (NACE 2025). https://www.naceweb.org/talent-acquisition/trends-and-predictions/employers-make-more-offers-as-student-acceptance-rate-rises-response-time-shortens</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extra days for supervisors (second round with plant management)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Supervisors have one extra round with plant management (about a week).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Funnel rates by role (Part 1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Application → qualified (baseline, all channels)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Researched</t>
   </si>
   <si>
-    <t xml:space="preserve">Own estimate: SmartRecruiters 2025 global median is 6 days to review (Germany 8); I assume the client keeps the global pace, an ask. Slide 1 shows the German-pace downside (~92 hires). https://ta.smartrecruiters.com/rs/664-NIC-529/images/Germany%20Recruiting%20Benchmarks%202025%20Report%20DE.pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Days: recruiter assessment → technical interview/test done</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Own estimate: global median 14 days application → interview minus the 6 above (Germany 20 − 8 = 12); same commitment as T2. https://ta.smartrecruiters.com/rs/664-NIC-529/images/Germany%20Recruiting%20Benchmarks%202025%20Report%20DE.pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Days: interview → written offer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">My ask to the client: written offer within 3 working days. No public benchmark exists for this step.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Days: offer → signed contract</t>
-  </si>
-  <si>
-    <t xml:space="preserve">One-week offer validity; candidates take ~9 days on average to decide (NACE 2025). https://www.naceweb.org/talent-acquisition/trends-and-predictions/employers-make-more-offers-as-student-acceptance-rate-rises-response-time-shortens</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Extra days for supervisors (second round with plant management)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Supervisors have one extra round with plant management (about a week).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. Funnel rates by role (Part 1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">QE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Application → qualified (baseline, all channels)</t>
-  </si>
-  <si>
     <t xml:space="preserve">IAB 2026 chart: production jobs get 12 applications per vacancy, 3 suitable (25%); 28% across all jobs; 23% for specialist roles. https://iab-forum.de/iab-stellenerhebung-2-2026-fast-drei-von-vier-bewerbungen-sind-aus-betrieblicher-sicht-ungeeignet/</t>
   </si>
   <si>
@@ -1349,7 +1349,7 @@
     <t xml:space="preserve">weeks</t>
   </si>
   <si>
-    <t xml:space="preserve">2–4 weeks to cover the PLC/industrial gap; onboarding time paid as salary, so outside the campaign budget. Client names a trainer by 23 Oct.</t>
+    <t xml:space="preserve">Own estimate: 2–4 weeks to cover the PLC/industrial gap; one client trainer for the ~8-person cohort ≈ 15 person-days (3 weeks × 5), client-funded onboarding outside the campaign budget.</t>
   </si>
   <si>
     <t xml:space="preserve">I2L</t>
@@ -3655,18 +3655,18 @@
         <v>62</v>
       </c>
       <c r="F21" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="G21" s="17" t="s">
         <v>70</v>
-      </c>
-      <c r="G21" s="17" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B22" s="13" t="s">
         <v>72</v>
-      </c>
-      <c r="B22" s="13" t="s">
-        <v>73</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>31</v>
@@ -3681,15 +3681,15 @@
         <v>63</v>
       </c>
       <c r="G22" s="17" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="2" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2" t="s">
+      <c r="B23" s="13" t="s">
         <v>75</v>
-      </c>
-      <c r="B23" s="13" t="s">
-        <v>76</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>31</v>
@@ -3704,15 +3704,15 @@
         <v>63</v>
       </c>
       <c r="G23" s="13" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B24" s="13" t="s">
         <v>78</v>
-      </c>
-      <c r="B24" s="13" t="s">
-        <v>79</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>31</v>
@@ -3727,15 +3727,15 @@
         <v>63</v>
       </c>
       <c r="G24" s="17" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B25" s="13" t="s">
         <v>81</v>
-      </c>
-      <c r="B25" s="13" t="s">
-        <v>82</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>54</v>
@@ -3750,12 +3750,12 @@
         <v>63</v>
       </c>
       <c r="G25" s="13" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="10" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B27" s="11"/>
       <c r="C27" s="11"/>
@@ -3789,10 +3789,10 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B29" s="13" t="s">
         <v>85</v>
-      </c>
-      <c r="B29" s="13" t="s">
-        <v>86</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>48</v>
@@ -3804,7 +3804,7 @@
         <v>44</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="G29" s="17" t="s">
         <v>87</v>
@@ -3815,7 +3815,7 @@
         <v>88</v>
       </c>
       <c r="B30" s="13" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>43</v>
@@ -3827,7 +3827,7 @@
         <v>44</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="G30" s="17" t="s">
         <v>87</v>
@@ -3838,7 +3838,7 @@
         <v>89</v>
       </c>
       <c r="B31" s="13" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>52</v>
@@ -3850,7 +3850,7 @@
         <v>44</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="G31" s="17" t="s">
         <v>87</v>
@@ -3861,7 +3861,7 @@
         <v>90</v>
       </c>
       <c r="B32" s="13" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>54</v>
@@ -3873,7 +3873,7 @@
         <v>44</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="G32" s="17" t="s">
         <v>87</v>
@@ -4723,7 +4723,7 @@
         <v>44</v>
       </c>
       <c r="F72" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="G72" s="17" t="s">
         <v>169</v>
@@ -4746,7 +4746,7 @@
         <v>44</v>
       </c>
       <c r="F73" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="G73" s="17" t="s">
         <v>169</v>
@@ -4769,7 +4769,7 @@
         <v>44</v>
       </c>
       <c r="F74" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="G74" s="17" t="s">
         <v>169</v>
@@ -4792,7 +4792,7 @@
         <v>44</v>
       </c>
       <c r="F75" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="G75" s="17" t="s">
         <v>169</v>
@@ -5458,7 +5458,7 @@
         <v>256</v>
       </c>
       <c r="F108" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="G108" s="17" t="s">
         <v>257</v>
@@ -5481,7 +5481,7 @@
         <v>256</v>
       </c>
       <c r="F109" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="G109" s="17" t="s">
         <v>260</v>
@@ -5504,7 +5504,7 @@
         <v>256</v>
       </c>
       <c r="F110" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="G110" s="17" t="s">
         <v>263</v>
@@ -5527,7 +5527,7 @@
         <v>44</v>
       </c>
       <c r="F111" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="G111" s="17" t="s">
         <v>266</v>
@@ -5550,7 +5550,7 @@
         <v>44</v>
       </c>
       <c r="F112" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="G112" s="17" t="s">
         <v>269</v>
@@ -5573,7 +5573,7 @@
         <v>44</v>
       </c>
       <c r="F113" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="G113" s="17" t="s">
         <v>272</v>
@@ -5596,7 +5596,7 @@
         <v>186</v>
       </c>
       <c r="F114" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="G114" s="17" t="s">
         <v>276</v>
@@ -5619,7 +5619,7 @@
         <v>44</v>
       </c>
       <c r="F115" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="G115" s="17" t="s">
         <v>279</v>
@@ -5642,7 +5642,7 @@
         <v>283</v>
       </c>
       <c r="F116" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="G116" s="17" t="s">
         <v>284</v>
@@ -5665,7 +5665,7 @@
         <v>283</v>
       </c>
       <c r="F117" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="G117" s="17" t="s">
         <v>288</v>
@@ -5688,7 +5688,7 @@
         <v>283</v>
       </c>
       <c r="F118" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="G118" s="17" t="s">
         <v>292</v>
@@ -5711,7 +5711,7 @@
         <v>62</v>
       </c>
       <c r="F119" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="G119" s="17" t="s">
         <v>296</v>
@@ -5734,7 +5734,7 @@
         <v>159</v>
       </c>
       <c r="F120" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="G120" s="17" t="s">
         <v>300</v>
@@ -5757,7 +5757,7 @@
         <v>44</v>
       </c>
       <c r="F121" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="G121" s="17" t="s">
         <v>303</v>
@@ -5780,7 +5780,7 @@
         <v>44</v>
       </c>
       <c r="F122" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="G122" s="17" t="s">
         <v>306</v>
@@ -5803,7 +5803,7 @@
         <v>44</v>
       </c>
       <c r="F123" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="G123" s="17" t="s">
         <v>309</v>
@@ -5826,7 +5826,7 @@
         <v>159</v>
       </c>
       <c r="F124" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="G124" s="17" t="s">
         <v>313</v>
@@ -5849,7 +5849,7 @@
         <v>159</v>
       </c>
       <c r="F125" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="G125" s="17" t="s">
         <v>316</v>
@@ -5872,7 +5872,7 @@
         <v>159</v>
       </c>
       <c r="F126" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="G126" s="17" t="s">
         <v>319</v>
@@ -5964,7 +5964,7 @@
         <v>0</v>
       </c>
       <c r="K130" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="L130" s="17" t="s">
         <v>333</v>
@@ -6002,7 +6002,7 @@
         <v>0</v>
       </c>
       <c r="K131" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="L131" s="17" t="s">
         <v>333</v>
@@ -6040,7 +6040,7 @@
         <v>0</v>
       </c>
       <c r="K132" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="L132" s="17" t="s">
         <v>333</v>
@@ -6078,7 +6078,7 @@
         <v>0</v>
       </c>
       <c r="K133" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="L133" s="17" t="s">
         <v>333</v>
@@ -6116,7 +6116,7 @@
         <v>0</v>
       </c>
       <c r="K134" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="L134" s="17" t="s">
         <v>340</v>
@@ -6154,7 +6154,7 @@
         <v>0</v>
       </c>
       <c r="K135" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="L135" s="17" t="s">
         <v>340</v>
@@ -6192,7 +6192,7 @@
         <v>0</v>
       </c>
       <c r="K136" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="L136" s="17" t="s">
         <v>340</v>
@@ -6230,7 +6230,7 @@
         <v>0</v>
       </c>
       <c r="K137" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="L137" s="17" t="s">
         <v>340</v>
@@ -6428,7 +6428,7 @@
         <v>0</v>
       </c>
       <c r="K142" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="L142" s="17" t="s">
         <v>353</v>
@@ -6466,7 +6466,7 @@
         <v>0</v>
       </c>
       <c r="K143" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="L143" s="17" t="s">
         <v>353</v>
@@ -6580,7 +6580,7 @@
         <v>0</v>
       </c>
       <c r="K146" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="L146" s="17" t="s">
         <v>361</v>
@@ -6618,7 +6618,7 @@
         <v>0</v>
       </c>
       <c r="K147" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="L147" s="17" t="s">
         <v>361</v>
@@ -6656,7 +6656,7 @@
         <v>0</v>
       </c>
       <c r="K148" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="L148" s="17" t="s">
         <v>361</v>
@@ -6694,7 +6694,7 @@
         <v>0</v>
       </c>
       <c r="K149" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="L149" s="17" t="s">
         <v>361</v>
@@ -7035,7 +7035,7 @@
         <v>119</v>
       </c>
       <c r="F165" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="G165" s="17" t="s">
         <v>393</v>
@@ -7314,7 +7314,7 @@
         <v>429</v>
       </c>
       <c r="F177" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="G177" s="17" t="s">
         <v>430</v>
@@ -7337,7 +7337,7 @@
         <v>119</v>
       </c>
       <c r="F178" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="G178" s="17" t="s">
         <v>433</v>

</xml_diff>

<commit_message>
Traceability: slide 4 cost basis stated, Talent CRM source in the model, I1 read date after its window
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V2NJtrYy3bzNxqKeiRXJfY
</commit_message>
<xml_diff>
--- a/operation_uptime/Operation_Uptime_Model.xlsx
+++ b/operation_uptime/Operation_Uptime_Model.xlsx
@@ -1808,7 +1808,7 @@
     <t xml:space="preserve">Also stop if far fewer than planned pass the language call. The freelancer is paid hourly, so stopping costs little.</t>
   </si>
   <si>
-    <t xml:space="preserve">Who does what is on deck slide 7. I2 and I3 are read on Mon 9 Nov, I1 on Mon 2 Nov.</t>
+    <t xml:space="preserve">Who does what is on deck slide 7. I2 and I3 are read on Mon 9 Nov, I1 on Wed 4 Nov (after its window closes on 3 Nov). Repeatable product: Joveo's Talent CRM already re-engages past applicants by email, SMS and WhatsApp (https://www.joveo.com/), so a consented past-applicant feed fits the same pipeline.</t>
   </si>
   <si>
     <t xml:space="preserve">Part 2 — Channel × role economics and allocation (cheapest cost-per-hire first, until each role's openings are covered)</t>
@@ -9711,7 +9711,7 @@
         <v>592</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="57" customFormat="false" ht="77.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="13" t="s">
         <v>593</v>
       </c>

</xml_diff>